<commit_message>
Update latest deduped XLSX
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,24 +482,24 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>The Princess of Wales dazzles in deeply personal Cartier earrings on Christmas Day - Tatler</t>
+          <t>Inside the Bullring's giant beauty hall featuring Dior, Gucci and Armani - Birmingham Live</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Thu, 25 Dec 2025 11:51:59 GMT</t>
+          <t>Fri, 26 Dec 2025 05:46:00 GMT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxNTE85eUQ4NTg3OXd3UHFiajNZanRZRXMyMXdKck1oaWVYRTF4d011NzBoVHROZ1R3RUY3VDJLVzk3NzhHajN5QWxwcU1yV1VtZW8wWFkxZHNKRi1lRVdQemlGc2EzOFc5ZDVLZjlzczVvUk9QbUd0b1lnNmMzRXZJeU5lTHFNSEhlSEhUOTBuRmk3UGJ4UzZTbXpPcXlfM2JzeG1FZlNaU0lkQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOTi05TWJfVEJRLVROTUN0anJrSlM1bkU4d0RfS2tZbVRjOFZHXzJEX3dnQ3N1OVpyOFZoZ1UxQjZmdldkZ2U3T0dVNnY4RTNLOGVZMGJVenRielRmR1UtWFZVaXZXeUhCUVdwOUVCZWlCYjFlT2RoYS1VckQxUmRwSk9Ed25kQjM0NFh2a0llOXQzN0VoTlVsZzhLcnJjQXVjQzJoaDN2dmNEM1XSAbABQVVfeXFMTnkwSEstdmU3c2ZGMWZEaHd6WmpzUS05YTZ3dkt5c0hnLWtQaExfVnFXY1dVRVZlQjF4b1JveklWenNsU1JhUDljejk2WjFlelJHWVV5WXFHOEdkYS0xNEYydi1FXy03UEVibXN5YXppb3NjbV8tcWxJczRWaHM2Vl9UNWE2OEpLc21fRk5FVmEwUjZEVEhoOTlqVTNyUWI0d0lqMXVYbTEwUlRVV0ZGdS0?oc=5</t>
         </is>
       </c>
       <c r="F2" t="n">
         <v>1</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>46016.49443287037</v>
+        <v>46017.24027777778</v>
       </c>
     </row>
     <row r="3">
@@ -515,24 +515,24 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Swedbank AB Acquires 25,000 Shares of Ralph Lauren Corporation $RL - MarketBeat</t>
+          <t>Kate Middleton Wears $4,000 Cartier Earrings on Christmas Morning in an Under-the-Radar Nod to Princess Diana - instyle.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Thu, 25 Dec 2025 11:23:19 GMT</t>
+          <t>Thu, 25 Dec 2025 17:57:56 GMT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxQWDU3a2hNNTdmUG13NjFFMWVNR1FsZ25OdFZJdjAydFhXVDVoU2dkTk44b3UtR3dhZDh0c2FlZ2lXQm9PMi1yYjFuaFlVVncwNE50SmNFZFBHQTBfYWtkZmtSbDBaaEZwbWpmdGVIRVR5NFZhMHAxV3FYZW1mVEZXeFBZblRaUXBDVE05dE9ZMTdnOWJTa1hTVHI5bWFVeFoxU1VlWjc5SVZNNUVTTEdoZTdvazJZMmgwb0xpMldIaWhNa0E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxNb0hzVWY0cERJOUl2WFdBb3pwSDRFRXU2U0hfYW45VkNWTHVvUXJuQXFVWDJqRTFZLTN0Q09Rd094M090cnppNHB4LW9RUUtmSUpOZXpkM1lSWElJSk80UmhHTEhjYWNiNEdDSmozaWZvVVk1WjdTWFNXbFgzNElJRkppaE10UllqcXh5eXF3aWg?oc=5</t>
         </is>
       </c>
       <c r="F3" t="n">
         <v>1</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>46016.47452546296</v>
+        <v>46016.74856481481</v>
       </c>
     </row>
     <row r="4">
@@ -548,816 +548,2895 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Cartier Resources (CVE:ECR) Trading Up 16.7% - Still a Buy? - MarketBeat</t>
+          <t>Percy Jackson: Dior Goodjohn on Clarisse's Quest, Annabeth Alliance - Bleeding Cool News</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Thu, 25 Dec 2025 11:19:15 GMT</t>
+          <t>Thu, 25 Dec 2025 21:37:03 GMT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxNckh6QldiR2E4eUtaZDVxTVFGaTZIZ1M0Z3Bia1haZTJsVnlHeXNnR3psS3RacS1ITldxV0VqSi1ZaTRUZVRpc2VINFZESU1zVzZLU0pLMmt0cmowUFRELUw5TVBEV0Q0d2NfT1AxX24zNGloNmFHTXZQRE9FUHlVTU9QMnlpbElTajkxUkdJeml1V1BvM1Nlc29vakRIbW9ibnVLc0FycFk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQamotTWI2enJKWWNZQUtidmtBUUl0NWRoTGdyNHNFOW4yZk5YOHV3SVdwYWN5cFBOTVRfYThxZG5mX25YdDFyS3Nzd0RrWC1HbU9uRHVxRUo1WTEzV21GdjByTmFxa0d4SUFjRFJNd21QVW1MYzJ1R3ZHWTZVaHFXUk5VUGk3dlZ0T2doaXdzN054V2RHLTZIdg?oc=5</t>
         </is>
       </c>
       <c r="F4" t="n">
         <v>1</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>46016.47170138889</v>
+        <v>46016.90072916666</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Value Retail</t>
+          <t>Brand search Google News and X - PROTEST</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("valueretail" OR "Value retail" OR "Bicester Collection")</t>
+          <t>("Gucci" OR "Ralph Lauren" OR "Dior" OR "Armani" OR "louis Vuitton" OR "Valentino" OR "Burberry" OR "dolce &amp; gabbana" OR "Polo Ralph Lauren" OR "Cartier" OR "Calvin Klein"  OR "Hilfiger" OR "Tommy H" OR "Timberland" OR "Prada" OR "Nike" OR "Balenciaga" OR "Canada Goose" ) AND ("protest")</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>The outlet shopping centre near Cambridgeshire perfect for Boxing Day bargains - Cambridge News</t>
+          <t>Maison Louis Vuitton Sanlitun: A fusion of tradition and modernity in architectural elegance - China Daily</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Thu, 25 Dec 2025 11:00:00 GMT</t>
+          <t>Fri, 26 Dec 2025 00:12:00 GMT</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxQTmJCdzlRVlY4VDN6OFpfSWExS0tSSXViSG1yUmZ5bFE2YUMyYWdWLUdQZXdQZl9VTU1IXzFNbE85dnZfMlBhQndFSWNWbzZzVWlYeWh2eE1DcTRfWnYxeHdWQU5NWWFLelUyT0RxN3dzN2FSRVhNV0ItcTVPbFF2MzJWbURnTm5BSi1fRzlHU2ZFSnI3b3puNDlFQXM5R2l3RjBPX0k1MVJ1QdIBqgFBVV95cUxQTmJCdzlRVlY4VDN6OFpfSWExS0tSSXViSG1yUmZ5bFE2YUMyYWdWLUdQZXdQZl9VTU1IXzFNbE85dnZfMlBhQndFSWNWbzZzVWlYeWh2eE1DcTRfWnYxeHdWQU5NWWFLelUyT0RxN3dzN2FSRVhNV0ItcTVPbFF2MzJWbURnTm5BSi1fRzlHU2ZFSnI3b3puNDlFQXM5R2l3RjBPX0k1MVJ1QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1qZUpCMXduNGZsT0R1SzV6UUgyblZOQTA1YVlUUkV6QVQxQkVOdy1qZnQ0OUxuWmdwZjQwRGUxS004RkowY3F6SHJxSWJEc1dsT2hjbjJVdE9PSDVOUHdKcnFhYmh6X0lMdVNEWHBKSTNxd0dsSnR0UGFSdlZSUQ?oc=5</t>
         </is>
       </c>
       <c r="F5" t="n">
         <v>1</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>46016.45833333334</v>
+        <v>46017.00833333333</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Value Retail</t>
+          <t>Brand search Google News and X - PROTEST</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>("valueretail" OR "Value retail" OR "Bicester Collection")</t>
+          <t>("Gucci" OR "Ralph Lauren" OR "Dior" OR "Armani" OR "louis Vuitton" OR "Valentino" OR "Burberry" OR "dolce &amp; gabbana" OR "Polo Ralph Lauren" OR "Cartier" OR "Calvin Klein"  OR "Hilfiger" OR "Tommy H" OR "Timberland" OR "Prada" OR "Nike" OR "Balenciaga" OR "Canada Goose" ) AND ("protest")</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Retail sector poised for rapid growth in 2026 - News Arena India</t>
+          <t>Giorgio Armani: Milano, per amore - www.upscalelivingmag.com</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Thu, 25 Dec 2025 10:39:23 GMT</t>
+          <t>Fri, 26 Dec 2025 02:39:57 GMT</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxNa2UyRUU0NU13b0pPNXpFQWU3cUtGY2hrcWhIclVYN2FNMzdOOEsza3hrSDE5aGdValRsaGV6c1NTS2s0M3hncFhucm5IMUN4MGs2YzQwVzEwc2FsMGo1Rk9MOEdDZ0YteWhqUVp4T2RQTkh4R25KQV96dWJ4TjhXVktYd3RHaTZnSkhmQkJOWQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxOVTVjdENOLXl5cHhseGdLMTdPcDZGUGlMY3ZvYXB1eWgyZnZJWlpGU0FjLW1oWjhXTjB1c25CMGd6em1OVm9jdkxQemdFZ0dFRjFjWU5CQ3ltNXZTbi1fa2xTTTAtSTZDQ3RKOEtIMHFOU255enFDbGNPZHVmSWVDQ1daZHVRdHl2X0xhSWJzR3g?oc=5</t>
         </is>
       </c>
       <c r="F6" t="n">
         <v>1</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>46016.44401620371</v>
+        <v>46017.11107638889</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BV Logistics Companies</t>
+          <t>Brand search Google News and X - PROTEST</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>("Dropit" OR "DHL" OR "UPS" OR "DPD" OR "Flight Logistics" OR "Fedex" OR "Amazon" OR "Royal Mail" OR "Parcelforce" OR "EVRI" ) AND ( "supply " OR  "delivery")</t>
+          <t>("Gucci" OR "Ralph Lauren" OR "Dior" OR "Armani" OR "louis Vuitton" OR "Valentino" OR "Burberry" OR "dolce &amp; gabbana" OR "Polo Ralph Lauren" OR "Cartier" OR "Calvin Klein"  OR "Hilfiger" OR "Tommy H" OR "Timberland" OR "Prada" OR "Nike" OR "Balenciaga" OR "Canada Goose" ) AND ("protest")</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>You Can Now Tip Your Amazon Delivery Driver for Christmas – at No Extra Cost - AOL.com</t>
+          <t>Cartier's Marlin Yuson on crafting the latest leather bags - Condé Nast Traveller Middle East</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Thu, 25 Dec 2025 11:32:03 GMT</t>
+          <t>Thu, 25 Dec 2025 21:00:00 GMT</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE8zRmpzQkY1LUpwSWlrdWpPUm9PZ2dRREdRdklMdkpzTDA4WGxfSUpWaU5SaUswaE1xODNnaU53V1BnTzlrcnppUTY0UTdJOWVqQndVTURvSVJaZlpIU3FkNDZBMzdFNGF0ZzNteDNjaFR0V1pWSjV2SklDSXYybUU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQaVJoMmc1ZVNMR3k3RFhEUEd2LVFicy1zaE00QXRqS2VvZm45UmtpSkgwOFNVYnloeVRTOXYwa1RNMW5KQUt2SDI2RTlDdG9JVGVLSHVOVlVFTXpnVUdETTZfbWtYUG1KOG1mWlFZaWdIN0NvUDhOcTNfNHo0ZmZJTlB5bkUwNzRDTHF1X0Q1ZTE4cVl4aXRnaA?oc=5</t>
         </is>
       </c>
       <c r="F7" t="n">
         <v>1</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>46016.48059027778</v>
+        <v>46016.875</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BV Logistics Companies</t>
+          <t>Brand search Google News and X - PROTEST</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>("Dropit" OR "DHL" OR "UPS" OR "DPD" OR "Flight Logistics" OR "Fedex" OR "Amazon" OR "Royal Mail" OR "Parcelforce" OR "EVRI" ) AND ( "supply " OR  "delivery")</t>
+          <t>("Gucci" OR "Ralph Lauren" OR "Dior" OR "Armani" OR "louis Vuitton" OR "Valentino" OR "Burberry" OR "dolce &amp; gabbana" OR "Polo Ralph Lauren" OR "Cartier" OR "Calvin Klein"  OR "Hilfiger" OR "Tommy H" OR "Timberland" OR "Prada" OR "Nike" OR "Balenciaga" OR "Canada Goose" ) AND ("protest")</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Why Swiggy, Zomato, Amazon delivery partners are on strike on Dec 25, 31 - Business Standard</t>
+          <t>Jonathan Anderson Gets Downright Whimsical for Dior Menswear Fall 2026 - Esquire Singapore</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Thu, 25 Dec 2025 09:32:13 GMT</t>
+          <t>Fri, 26 Dec 2025 04:03:56 GMT</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxQNDhFWFBkWXhrWktpcFNfSGdyMUlFaThsNXl3Z2NsZUs4bnc5X2JNVjhzMU1vQkN4VVB2a1Y4am5NbjdVVk1UZDl5dDAzMXRGajlHLVhiTlo5eUpibUg4U0VQOHdtV0Fmam9ENzJod09fSmdBVWRnUXNVVVhpVHlVZEtST1pwTXRSOW42SHp6eUp1Q25Qc3JsbjkzZGNTOS1oOGRFWlE4NGhrZkljQjB0MkdiOU04cVZNV1VqQi1IM1VZc0cyZnI2LVUtWS1JNUptOTRUZdIB2gFBVV95cUxNTVZlQk9CMGVtQThXZDZ5NWxLSkRtNDk5RE92dk5OblIzWGFqWndfOGYxbmE0VWNVbUJPb2FnVmVvSnU1SHJ4LVplQjVjNVVsU3F1UTdUQWllTUk2LUNLdTRYdWFWMkZXS09yc0Y1bnNWR3dqUUYzbmlqTWNILXRPVnVYR1F4cVBlMnJUdjhPNFBuOGJ2VHdrUUVHYjdoeFBqSFphSnRGckFmR3BJbmJBbE5iMTIxZzFuRl8zaHBCNjRlaWt2V1RpeVgxNk9PVGtJem84cmJVemViZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE11MEJDQjRFUTJ1aFhQckVCb21ScEV6eUhsem53REtCc05JNkluYjVoaWU1M3BtMEduNGxOUmZtamZVY1VhZHhaQ3FjTWs1SUNVQUNHLXlvNTRVNmhqOFUwRmtZdXIxZU1JeG9lV2hOV0xoQQ?oc=5</t>
         </is>
       </c>
       <c r="F8" t="n">
         <v>1</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>46016.39737268518</v>
+        <v>46017.16939814815</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>High Level City searches   Belgium English language</t>
+          <t>Brand search Google News and X - PROTEST</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>("brussels" OR "Maastricht" OR "Antwerp") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" OR "Retail crime")</t>
+          <t>("Gucci" OR "Ralph Lauren" OR "Dior" OR "Armani" OR "louis Vuitton" OR "Valentino" OR "Burberry" OR "dolce &amp; gabbana" OR "Polo Ralph Lauren" OR "Cartier" OR "Calvin Klein"  OR "Hilfiger" OR "Tommy H" OR "Timberland" OR "Prada" OR "Nike" OR "Balenciaga" OR "Canada Goose" ) AND ("protest")</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Individual seriously injured in Christmas Eve stabbing outside Brussels Stock Exchange - VRT</t>
+          <t>Burberry Group (LON:BRBY) Stock Price Passes Above Two Hundred Day Moving Average - What's Next? - MarketBeat</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Thu, 25 Dec 2025 08:39:56 GMT</t>
+          <t>Fri, 26 Dec 2025 05:40:52 GMT</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPelU1QUNTRmhiX196cGxvaUlMcUVBelg0aVJYdHdoTmZkcXkwQUxLc1AtcGVmZEcxWFFQRlVRa3F4RVZPblQwaUJDOWFfOUJGUV9zdHJiVF9obEE4d3dyR2NDUUY3TDJiQ1VZM0R2bFR2T1k5RUhVWmZHQ0VpWmlkcFZULUgzR2NvbXl5aTBmTGZGbGQtb3I0X2s0Uy1IZ29jaC1nb2NoNng?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxOVnV6Wm9TVU5vSTJ0Smp5MXZXU3MzX0dTR2ZjcThMOEhoRHJFYTIyTUQ5WWZJSXlWSWJDZEZwSkhZZmM1czNCWVdCRUZablVnMzhQNEZ5bktlSmNDc0liOWg1b3kyYUc0WHlJbGVNQVNGUnIwV0JCOVUwWmkyNWg5aWNQQlJLcFFhSjBoTDFpWVgxRHFZZlRZa2t6ZjlKUXhMRnd6MkxQVC1MZ0dJQ3pRSzlsMkNrU01lWXpmTlRHT05UNTJsbWtDQnhpSGktenM3VUlDSTB4Vl9GNHc?oc=5</t>
         </is>
       </c>
       <c r="F9" t="n">
         <v>1</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>46016.36106481482</v>
+        <v>46017.23671296296</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>High Level City searches   Germany, English Terms</t>
+          <t>Brand search Google News and X - PROTEST</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>( "Frankfurt" OR  "Cologne"  OR "Munich"  ) AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing"  OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat")</t>
+          <t>("Gucci" OR "Ralph Lauren" OR "Dior" OR "Armani" OR "louis Vuitton" OR "Valentino" OR "Burberry" OR "dolce &amp; gabbana" OR "Polo Ralph Lauren" OR "Cartier" OR "Calvin Klein"  OR "Hilfiger" OR "Tommy H" OR "Timberland" OR "Prada" OR "Nike" OR "Balenciaga" OR "Canada Goose" ) AND ("protest")</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Muller hails Bayern Munich whiz Karl: Just like Podolski - TribalFootball</t>
+          <t>Paris Haute Couture Week Spring/Summer 2026 Official Schedule and Participating Brands - ouispeakfashion.com</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Thu, 25 Dec 2025 11:47:30 GMT</t>
+          <t>Fri, 26 Dec 2025 04:59:00 GMT</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxNOXBuc25sdHNwVWRtcjFYUWJ5NjV5eDN6MVo1M0V1d3VxeUFNN1RGSmpWaGpZeHZrang5cndocy1PMzU0YlZxaUM3VWpSdFdqLThYS1FucmRfcTF6RWhGLUV3R29jZVVIM05BM2RUbVBsZUlMTDNTLVFPb196WXhGUmNJZkx5aTZBUXhGT1d0bDFtVzV0ZERkU3hvcG1QZkRPeGd5cjkzcUsxeVlfYVNnSXo3SkFBcUFUeDA1QTdxa3NkbmFkUEpfNVRCQWp1bjBPRmNVNzNBUDExQUgwYk84TTEyMA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE42T1ZJTFVFVjF3Ymd5NDZpRVlaeGFtVm4yMGhFLTFRbkVaR1o2X0R2M1JMSjN1eTBTaWgyNEFIN1ZMWDJ4d3hTd0JRUFZrVGtORUVNemJPWGhZcVpjemhTdlgtVGVOOGdTbWt1SVE3NFI4RmRBUjYzVXlwRVE?oc=5</t>
         </is>
       </c>
       <c r="F10" t="n">
         <v>1</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>46016.49131944445</v>
+        <v>46017.20763888889</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>High Level City searches   Germany, English Terms</t>
+          <t>Value Retail</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>( "Frankfurt" OR  "Cologne"  OR "Munich"  ) AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing"  OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat")</t>
+          <t>("valueretail" OR "Value retail" OR "Bicester Collection")</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Indo Farm Equipment Limited Inches Above Key Support — Safe to Hold - Options Trading Strategies &amp; Best Stocks For Explosive Growth - Bollywood Helpline</t>
+          <t>Indian Retail Sector Eyes Margin-Led Growth In 2026, Driven By Tier II &amp; III Cities Demand - Free Press Journal</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Thu, 25 Dec 2025 12:13:44 GMT</t>
+          <t>Fri, 26 Dec 2025 03:21:28 GMT</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQOE9DOVI3U2JLU0x3ZDlaX3RnYlk4LVJiV000UlZ0bTRoR20zdXZOS1ptMVNZTUp5OHhTVEt6VjktZkVqWnh5UzJuMzNJQzA0WWhzaTZpcE43blM0bDFBby1PeEpCMEc1ZVFRZzRsYW9icXdBSnlxRE5KekJtYlYzZGI2NnFmWHNRc2FkcUZWampEdTJtREQxU1p3UHRrZzBqUHlreWVLdXRuZnpjWUxj?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxNbGZVT1BGMUh1blZvZFktdlBfLURieDNaRmhFV0Vocm55WTk4UzYzdlktTkxZTEFLcEpYMDd4aGNMb2k4SFlwblltVm0zX2RWejN4V3lfeWQ2THJBU2N2ajBzRUxMb0NQSG93VUFoVmhBU25DN05YdnhCLXR3THBrdVlXSDZpYUVMZWZGOWh5VVhYVXN5WHUzN0JBMHljMEQwRHZLeDE2WFNlbmNnVUZoWFhVaEl1UU1OWXVLTzNqaHlUdGdDdFdKbjUwazHSAcwBQVVfeXFMTWxmVU9QRjFIdW5Wb2RZLXZQXy1EYngzWkZoRVdFaHJueVk5OFM2M3ZZLU5MWUxBS3BKWDA3eGhjTG9pOEhZcG5ZbVZtM19kVnozeFd5X3lkNkxyQVNjdmowc0VMTG9DUEhvd1VBaFZoQVNuQzdOWHZ4Qi10d0xwa3VZV0g2aWFFTGVmRjloeVVYWFVzeVh1MzdCQTB5YzBEMER2S3gxNlhTZW5jZ1VGaFhYVWhJdVFNTll1S08zamh5VHRnQ3RXSm41MGsx?oc=5</t>
         </is>
       </c>
       <c r="F11" t="n">
         <v>1</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>46016.50953703704</v>
+        <v>46017.13990740741</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Shoplifting UK</t>
+          <t>BV Logistics Companies</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>"shoplifting gang" OR "shoplifting trend" OR "pickpocket gang" OR "theft from person" OR "retail crime" OR "shop theft"</t>
+          <t>("Dropit" OR "DHL" OR "UPS" OR "DPD" OR "Flight Logistics" OR "Fedex" OR "Amazon" OR "Royal Mail" OR "Parcelforce" OR "EVRI" ) AND ( "supply " OR  "delivery")</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Extra police patrols across North Wales as part of Christmas crime crackdown - Wrexham.com</t>
+          <t>Royal Mail December 24: Christmas Delivery Delays Hit 92 Postcodes - Meyka</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Thu, 25 Dec 2025 11:03:27 GMT</t>
+          <t>Thu, 25 Dec 2025 17:09:13 GMT</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNTDh4SW81Vmk4WHdCZElTOFVuVEVuQnVRSVIxRlJDM2ItVGlMVWFYSldXWDRsQUZnTGowM2FXRUR0R3ljYkg0MHlQelJQaW1BQmU2cXl2am1SSE1sR0dxSWdDc3JkWlJ3VEllNmFoUS1YalZkRmVJMlpLSkYtSFJGb3hqVnBWZlVLcjI5NGZMN2xDUy1sVWF6ZlRXS3UxaFR5eFEzMnI3d3Y4MmVMTkhzTy1MWQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOc3hpVDE0VmVPNTh2XzdHbG1yUWg0dWl5eFVMdndnNW5UcnRHb01NMW9vbUdfanhfTVM3WlZJcFd0RFp4cG1uZ2doaXNHT29ib0dBUGRkV29uZ3RmN0E5d3g3ejBBZGFIWTBMWWwtb0VvcnZndWFrcDBrM1JuNVc1ZDR2MzFzdWF5Q284QnhvTUdtQno1Z0RLRDhn?oc=5</t>
         </is>
       </c>
       <c r="F12" t="n">
         <v>1</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>46016.46072916667</v>
+        <v>46016.7147337963</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Shoplifting UK</t>
+          <t>BV Logistics Companies</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>"shoplifting gang" OR "shoplifting trend" OR "pickpocket gang" OR "theft from person" OR "retail crime" OR "shop theft"</t>
+          <t>("Dropit" OR "DHL" OR "UPS" OR "DPD" OR "Flight Logistics" OR "Fedex" OR "Amazon" OR "Royal Mail" OR "Parcelforce" OR "EVRI" ) AND ( "supply " OR  "delivery")</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>PILFERING SPREE Bognor Regis Thieves Nabbed After Festive Spree - UK News in Pictures</t>
+          <t>Why Swiggy, Zomato, Amazon delivery partners are on strike on Christmas, New Year's Eve - MSN</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Thu, 25 Dec 2025 10:29:00 GMT</t>
+          <t>Thu, 25 Dec 2025 20:27:30 GMT</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxPYXhrUjVzRVoyZmdKYzhHTkUxcUpmbjdCTERoSEg4Qk9iY3ItMzN5MjRLYXEyWXNSaGJNUUkzTlNmeFFRSHluSWJSUm9jR2k1Z3QwcjFFaU15eDRWWlVNLWNxRWFhQTJ4cDN3QjcxclE1c0tnODZ2S3ZFUEVHLWhLRWNCRndsdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4wJBVV95cUxPYVFSVTVxOUN6QmhVYVVaSWlhOF94NFdWZ2ltQlp6a0hGd1BfM09qVTQwSEJLYmh0dUFndXRtYndyR3JtS1lmREVJSGNBYXJGVDBBYzdoVXJya0dZM003WFhEV3psOGVldDhaSFNUQ2gwcFRjYjdxLWh2aUtJSzAyMEZOT1VyVks0Vm5kVDlUUmRQOHZkZzJPdDRYcFA3RmdjY3lTejhERDlPam15RERSUVoyUjZxQ3ZuZlZrMTZTUDBpNEh4N2ZKOWtwbXVDT0Y4WnJ0X1Rma3NNZ0dPeUVtaE9icTE5TVFTZlhiV0k1Q2d0SWxvaExmb2JCalYzNUtCbXBjRjRvRGpySE1QM1RMM0hZUEpSd3FUdGc4WElTV0lINGhfZlUxZEhDUjhJV3BVWnlVVERuV19GWFdKTXFPYVVtUWNnMElLN0FFNktJVGFWaHJQMFVCTTNLSUI1SWJPMWdv?oc=5</t>
         </is>
       </c>
       <c r="F13" t="n">
         <v>1</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>46016.43680555555</v>
+        <v>46016.85243055555</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>High Level City searches   Spain, English   language</t>
+          <t>BV Logistics Companies</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>("Madrid" OR  "Barcelona")  AND ("Bomb" OR "explosion" OR "shooting" OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat")</t>
+          <t>("Dropit" OR "DHL" OR "UPS" OR "DPD" OR "Flight Logistics" OR "Fedex" OR "Amazon" OR "Royal Mail" OR "Parcelforce" OR "EVRI" ) AND ( "supply " OR  "delivery")</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>52-Year-Old Man Found Dead Under Rubble and 25 Injured in Explosion After Suspected Gas Leak - AOL.com</t>
+          <t>Discounts surpass Black Friday: Amazon starts Christmas campaign with guaranteed delivery until December 25th - Mix Vale</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Thu, 25 Dec 2025 10:50:21 GMT</t>
+          <t>Thu, 25 Dec 2025 18:12:46 GMT</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTFAzbnlId3JELUF1alowMVB1WmZlMjV5enNpbF94Xy1MaDZyM0J1MlF4RGRSd3h1ZW1pQ2ZCSWR2R05YbVM1LWc0OENLREUzdC1RaWwwNDhDRS1wcDBUM3NNekpUU1p0aEUtX2lmOHJpT0dDSlk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxOdWpzQkptU0xjUjBPVURmNlVGWlNfQ1ktSlMtM1dzdGFaWFFMRjFWRDdSNl9sUVRVdTNQTDNxZUg0OHQ3cE9zZm42VkVoeFFXMUN2TUtCSUFtYUZaNHFJU0MyUmhXTzVBRHVsOE1jejVLUVhJR0YyV0k3SHkzb1dRdW1hdnp2NVM1MDNES1FBelBDUS1WTTExQTIwUmE4VjBhVjRLNnpPZ3duZ0hRWXZLQjBMNUt5M2x6TEhnM05ORXVBTk5SSlBwS2lIWlVaSWJUUzNhblpyVUlzSGltbFNFd1Nfd1HSAeQBQVVfeXFMTnVqc0JKbVNMY1IwT1VEZjZVRlpTX0NZLUpTLTNXc3RhWlhRTEYxVkQ3UjZfbFFUVXUzUEwzcWVINDh0N3BPc2ZuNlZFaHhRVzFDdk1LQklBbWFGWjRxSVNDMlJoV081QUR1bDhNY3o1S1FYSUdGMldJN0h5M29XUXVtYXZ6djVTNTAzREtRQXpQQ1EtVk0xMUEyMFJhOFYwYVY0SzZ6T2d3bmdIUVl2S0IwTDVLeTNsekxIZzNOTkV1QU5OUkpQcEtpSFpVWkliVFMzYW5aclVJc0hpbWxTRXdTX3dR?oc=5</t>
         </is>
       </c>
       <c r="F14" t="n">
         <v>1</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>46016.45163194444</v>
+        <v>46016.75886574074</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>High Level City searches   Spain, English   language</t>
+          <t>BV Logistics Companies</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>("Madrid" OR  "Barcelona")  AND ("Bomb" OR "explosion" OR "shooting" OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat")</t>
+          <t>("Dropit" OR "DHL" OR "UPS" OR "DPD" OR "Flight Logistics" OR "Fedex" OR "Amazon" OR "Royal Mail" OR "Parcelforce" OR "EVRI" ) AND ( "supply " OR  "delivery")</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>South Korea, Japan, Spain, and Singapore Witness Explosive Surge in Chinese Independent Travelers – How Korean Airlines, Iberia, and Luxury Hotels Are Cashing In on the Gold Rush! - Travel And Tour World</t>
+          <t>Amazon 2025 Deep Dive: The $6B USPS Standoff and the AWS AI Pivot - FinancialContent</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Thu, 25 Dec 2025 10:57:33 GMT</t>
+          <t>Thu, 25 Dec 2025 14:41:00 GMT</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgJBVV95cUxObnNFdXdZdGR2Y1pUQkJKS0huTjZIbFBiOFRaTWMxZ3ZEQWlBeC1rcWdDQXNvMjhMSFlqTGM5SDVVblEzMk8ySFkzTkc3enVmaUIzTV9UYlh3UzR6endDWjRTVmpXdUFMcjk4U0VLZi1UMHU4TEx2blVpYzd6dEVjZjl6Nnp3OVpPUXBYQ2U3SGN1eWN4c3BSRmdiSDM4Q0xrMmx4dV8yNDE4eVN3dFJoMVFkekx2Z1VnekUxa3F5M2FxRjVMb05XcHBCS0I1Y2xhQW9RR3FLUnZZV3N2WEZSMTRYcnBrZHpZMmI3OVFIOTVPZUFKTFdvQVB5ZU1PaTRkTlNETjJCZGQ2RVNrRDZzekI0bldzakRHb2V6aEIzX0dCbklCQS1mNXRJUnVaTUJpTm4zbGZTaWFtdkRyZ3FNWVV3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxNUXBpdWl1V011UEJTMlBKZzZFU2FwaUs1WXl2NWZLSkktd2dJRUY1ajNsczZVRUJ4NVdpMjVqRUNpRjhqV3RSTi1TMFFHSlAxaExTbTBQdVhZb0Q3RW13ZnNnTjZDNVdzbVVlMkk1R0l4eU5wSGgwTmRsS0pWYUY3c2hYX1pmbEZfYWdlVzlmS2JtNXF6RHhreDJzT1ozQ2UxYmlEMEtDczBHM1NWSDB5SkVGc2ZHZ3VOb1dYaHlvNXFvYVZyRUo1LVpsZ1pzQjg0S0tTOXRKcw?oc=5</t>
         </is>
       </c>
       <c r="F15" t="n">
         <v>1</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>46016.45663194444</v>
+        <v>46016.61180555556</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>High Level City searches   Spain, English   language</t>
+          <t>BV Logistics Companies</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>("Madrid" OR  "Barcelona")  AND ("Bomb" OR "explosion" OR "shooting" OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat")</t>
+          <t>("Dropit" OR "DHL" OR "UPS" OR "DPD" OR "Flight Logistics" OR "Fedex" OR "Amazon" OR "Royal Mail" OR "Parcelforce" OR "EVRI" ) AND ( "supply " OR  "delivery")</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Rashford signals end to Man United partnership with move to Barcelona - CHOSUNBIZ - Chosunbiz</t>
+          <t>Interested in FedEx? Mark your calendars for June 1, 2026. - MSN</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Thu, 25 Dec 2025 11:58:00 GMT</t>
+          <t>Fri, 26 Dec 2025 05:19:31 GMT</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE5UcUJrRzlXOU5mTTd1QXVTZ2E4XzFkUHF5ZHA2d3ViRzhIXy1MWlpWSTEtVnozblNpMGt3eVF4T1c0SmdrdU9FSGxiZ0hacERnRGpfdjVGbHJQMnVMU3o3TXhqc3ZUcWhVOEV1Tkk2SFZic3BGU01fb00waXBYQkHSAZMBQVVfeXFMTzh5bGFCYjlhTHV6TU5Dd09SS2hKY2JxMDBZb1pnY21QQko2bFFEbUZyOG5nMml4Z3BDQ3RBZmRoZktfQlU5Ri00V3dESzBPMWk1eTFOMWktM1V6bWtjWXdYX19CTHpWQWJPeDN5S0VVc0VuTGppUjh0d09lbGdBTThxRmFBdHNhQ0lnRnRIamxtRlFv?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxPWUYtbDFzT0Z2MUYzWDBuOUtTN0FFWFVkU2QzcWVSYmtOczBFbkEwQl9ybXB4RllPX0RGYjdFZ09oVnEwRDBJX3FmSGNQT3NiaGhjVGlyTXhfMnFSbmFvSThFWFAtSkRxbmQ1RjA1a1NBTzNkcjRsYjk0MjFYUl9hcm9mTlRuQTJtTGE3Z0o5N3NJanFuRUFRTmViUlFRNk5kTXhsaWt5MXlCRDBtR1pMNGJVNlhGRUxWcGNOMUJOalFtLWpvVk9ZcUFoTVpSSkV6?oc=5</t>
         </is>
       </c>
       <c r="F16" t="n">
         <v>1</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>46016.49861111111</v>
+        <v>46017.22188657407</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>High Level City searches   Spain, English   language</t>
+          <t>BV Logistics Companies</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>("Madrid" OR  "Barcelona")  AND ("Bomb" OR "explosion" OR "shooting" OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat")</t>
+          <t>("Dropit" OR "DHL" OR "UPS" OR "DPD" OR "Flight Logistics" OR "Fedex" OR "Amazon" OR "Royal Mail" OR "Parcelforce" OR "EVRI" ) AND ( "supply " OR  "delivery")</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Xabi Alonso intent on recovering the best version of Real Madrid heavyweight - Madrid Universal</t>
+          <t>Swiggy, Eternal under pressure amid Amazon's quick commerce expansion says Macquarie — check downside - MSN</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Thu, 25 Dec 2025 13:07:30 GMT</t>
+          <t>Fri, 26 Dec 2025 05:15:28 GMT</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPNlhPTnFPTmpwX2Y0U09mSGtKR0RLdnVnNEFtbEhzeHZJQWRlenFwZTBHRWlpQlJuQTZrWVZLQ1B1dlF5eC1FQllWUFhieVlKZkVWYy1GR3ZuZjd4emJ2a1N5WW9RTTVHSlVZeWdIR1BzNHJWWU1BT3UzSTFoR0lQd29DU3h2eW1vR0Zjd3VfZGxpMEhJMkkxOURSTVd4Nnh0V293dXczX0I?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxOVG4xRGl4VFh2WjFkU3daTTZEMnBOd1JYTjVLS21OUWRVajNYSE9LOWVlT0h3QzZjRjRBOGJVdTktZzBSd1F1SFdoVlRVWVNvUEtSOWIyM3l4TU9fZVoza0p6ZlByaVgxejBfVzRqT1d6cHN3WC10Wmdvd0RIby0xaDZuank3R0pid0VUSEh5VDF6eFJDQ2VkTXZGNFlpYWVqZFlGeEJHYWJOUUFCMmZ4c1dNbTFlbDFrcUZ0bS1wekNTZGcwVE9qbUhWbGZuZlVrN1pfQVZEeG1STThjVF8xNUtyZjQ0Y0pOaTIxZVdOTENHUjF6VkNN?oc=5</t>
         </is>
       </c>
       <c r="F17" t="n">
         <v>1</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>46016.546875</v>
+        <v>46017.21907407408</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>High Level City searches   Spain, English   language</t>
+          <t>BV Logistics Companies</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>("Madrid" OR  "Barcelona")  AND ("Bomb" OR "explosion" OR "shooting" OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat")</t>
+          <t>("Dropit" OR "DHL" OR "UPS" OR "DPD" OR "Flight Logistics" OR "Fedex" OR "Amazon" OR "Royal Mail" OR "Parcelforce" OR "EVRI" ) AND ( "supply " OR  "delivery")</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Surprise! he leaves Saudi Arabia to play at the Bernabéu: he is better than Dani Ceballos - madrid-barcelona.com</t>
+          <t>Lucky Redditor scores $6,000 in free Samsung 9100 PRO SSDs after Amazon shipping blunder - Notebookcheck</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Thu, 25 Dec 2025 11:30:00 GMT</t>
+          <t>Thu, 25 Dec 2025 18:48:00 GMT</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxOOE9qS1hEdXRfY1d5bXpfWjlvdEdGVUloOEU4S3lDYTdfWEFIUlBnMEhRdlMxZ0laVWxMLW1KcDdsZHQyenFqX2piT3hIcnVWSnJ6R2c2QTVWN0JUdUoydE1ENXkzWk1JM1Y0ZE5NQ2p2Rk9EbmExYjFfQV9ETWNNeFpsSmMxNHNyWllEM0NKX1A5clJkT2ZIVDRtWjdrQk9pSHZtRlNCLXllZVdSQmtiMw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxNenE2anhHbVF2a2VTUEJENWpZeGhkODR0OUFBRGJkUHNweXR1eDdxYWxob3VaNGE2elpWOG5XUmhJMGR1RlJWbmNXWXRCUDZnSTVVcE5ETFNWUXlkSDZOUWpnSHRWblpZZmpxb19NeHZ1ZFJrdlk5MVB1Q1c2bzZUS2ZEVnd6Vk1VUTJONGNBS29ORjUxems1amNjUGNpcFJZSHRtbl9XOXdhT21FeUQ0Z0h0ZlZNYkI5aGxJaEF3M09yOWRnLTZIcXpHQUo?oc=5</t>
         </is>
       </c>
       <c r="F18" t="n">
         <v>1</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>46016.47916666666</v>
+        <v>46016.78333333333</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>High Level City searches   UK &amp; Ireland</t>
+          <t>BV Logistics Companies</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+          <t>("Dropit" OR "DHL" OR "UPS" OR "DPD" OR "Flight Logistics" OR "Fedex" OR "Amazon" OR "Royal Mail" OR "Parcelforce" OR "EVRI" ) AND ( "supply " OR  "delivery")</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Knife fight erupts on Tube platform in front of horrified passengers - London Evening Standard</t>
+          <t>Thailand Emerges as ASEAN's Premier Logistics Hub Amid Global Supply Chain Realignment - Nation Thailand</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Thu, 25 Dec 2025 09:37:07 GMT</t>
+          <t>Thu, 25 Dec 2025 23:31:00 GMT</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxPQ1NoTXVwV056cXBDZXRmT1BOWG1GVElPYzd6allIeFBrd2dkSEl6S3gwLV9FNXhlM3VMb2NzQVlRdUpaME1YNTRzSmVCWHFEb0FURmlvVGZ3WWlSMVl0eTVBWFhMTGFoVDNnV3VaYmk5R19DWGYzTDdTcU1RbDRiS2JFLWxVWmlTV0RGUGU5aUNlTEJvTkdXVFRUM0NBRGY2?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiZEFVX3lxTE1FeHMtZElyaml4NGcwSE9jOGdBM0J0NmxsSmREMXFFdHppSW9IMUluUzdGYU1nQk04S3ByYVdmSG1lU2pHUlJObEVweUNILUQ4eEdnQUZ4a1RoV0NUYXlrRmpaUFA?oc=5</t>
         </is>
       </c>
       <c r="F19" t="n">
         <v>1</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>46016.40077546296</v>
+        <v>46016.97986111111</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>High Level City searches   UK &amp; Ireland</t>
+          <t>BV Logistics Companies</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+          <t>("Dropit" OR "DHL" OR "UPS" OR "DPD" OR "Flight Logistics" OR "Fedex" OR "Amazon" OR "Royal Mail" OR "Parcelforce" OR "EVRI" ) AND ( "supply " OR  "delivery")</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Test your EastEnders knowledge with our iconic Christmas episodes quiz - My London</t>
+          <t>Where Will UPS Stock Be in 1 Year? - AOL.com</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Thu, 25 Dec 2025 11:54:25 GMT</t>
+          <t>Thu, 25 Dec 2025 14:31:04 GMT</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNYk5ucW5xOWFaeExlN0JxSjNHaVdBZTYxWDJZaDJDX01ISXdkbVoxRno1SE5IOFFtWEV5dURsOVlldFcwZy1IamVZemVjb3B2cUVyYk5PelVJVktwNjJLSU9XNUZMc1hmaXB1QzZrWkgyTFZROG1ZQlZjRENpT3ZTYWh1cWs0MFB0YmhqeHJSZTY4M200ZmdaM2RiUEFTa3Np0gGMAUFVX3lxTFBQbkJESHBPaGV2WjQ1UFhNa09lUXh5TFE5Tm9vak1DMFIzV04tTjhmZ2xaTkNXMFNEWDdDSmZfbkExN1VZRHZfNktCZ3NtcnpUb0NJLVBWdS0tNWVjUmx3VEdBUzh2allLNm5rNnNWcXRNVzNqc0lZdUtoY1ctS0xLV0dGLWh4Z1dqcUVz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1UUG5rVmlBcFV2VzBNRkFkdWJfX2dPNWgyOGhickVZbWlJWVpqQWxBNUdKeDJpVGxMalJIcEcwM3JvWlFwS0Q5SVR5ZE1mSUJFVFREY3Vyb3FobzdBcEROWnZHVUhzZkVxcnFUNA?oc=5</t>
         </is>
       </c>
       <c r="F20" t="n">
         <v>1</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>46016.49612268519</v>
+        <v>46016.60490740741</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>High Level City searches   UK &amp; Ireland</t>
+          <t>BV Logistics Companies</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+          <t>("Dropit" OR "DHL" OR "UPS" OR "DPD" OR "Flight Logistics" OR "Fedex" OR "Amazon" OR "Royal Mail" OR "Parcelforce" OR "EVRI" ) AND ( "supply " OR  "delivery")</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>25 chocolate bars that vanished from UK shelves that are seriously missed - My London</t>
+          <t>Is the post office open on Friday, Dec. 26? Does the mail run? - NJ.com</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Thu, 25 Dec 2025 09:05:53 GMT</t>
+          <t>Fri, 26 Dec 2025 06:18:30 GMT</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE5ZZjMyWVdCazVSUzBFZHRWaHhNOVR5X2V6QU9hS2dXRHp4LXcwRXJMdFVjZUtyZjRTZzd2SnVndDV2V05DLVFQLW1GVzItLThURGU1eFllTkxON2hvbjlMZFE3QnUtdm5zNE5wenk1MElrQ05nXzczMGtzdHkzelHSAYQBQVVfeXFMUGNvQk9RRXBFR0tpczQxaDBvT3Y5am9PbUlpMUlWNHFNcEt1R1BCQ3llcTZyLXh6M05wa19lci0zZmhlRjdxbE1xdUV4czZqZ1E0dGhlbEoteVhER1MwdXlkcEJNQUo5akR6emo5NGxNX1hBV0lWYWRkQS1VQkROOTRlS2hY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxOa2pEcDc1cVRhSTMzZ1BSOGZhVkdncEJfZm5MRUFra2xqSFRINTMxRU84am9JMkxJWWw3Q0w5TDc5YzhfaU50VzlkMUYybGVBM3ZoQkRmTF9rQ0pjc0k4MVl4UzJDSkJjY3RLcG51RklpMkVWTzF6ZUt3TV8tbFFnT1k4TG81Z9IBmgFBVV95cUxPVHdaanFuNzczb2NMUW9iV0M2bjBzUEFTbEZSQUctYk5NdFRHQ0w3UXZZN1ExRG1HYXZENWpJcWhxcFRHREpUSnBfckw0MzFmeUsxN2tjLXNvY3A2UTdVdU1SUnM5VU9rMDg5UC1PR1otN0J5aTdhcllFOHQ2dGJvWmstZXVubUk3S1hwSjFxN1JXaUxKbFNLSTlR?oc=5</t>
         </is>
       </c>
       <c r="F21" t="n">
         <v>1</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>46016.37908564815</v>
+        <v>46017.26284722222</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>High Level City searches   UK &amp; Ireland</t>
+          <t>BV Logistics Companies</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+          <t>("Dropit" OR "DHL" OR "UPS" OR "DPD" OR "Flight Logistics" OR "Fedex" OR "Amazon" OR "Royal Mail" OR "Parcelforce" OR "EVRI" ) AND ( "supply " OR  "delivery")</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Horror as construction labourer lynched by vicious gang on suspicion of being a migrant - Daily Express</t>
+          <t>Delivery workers haul more NYC packages than Santa Claus - Gothamist</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Thu, 25 Dec 2025 13:01:00 GMT</t>
+          <t>Thu, 25 Dec 2025 22:07:00 GMT</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxPZFhJUUNYU1JkZ1NrR3N4U0xpODUybjFXb2hfX08xNkNheDI4VEtzUUJ6S0VKbjZEZ2V0c012YndLUE91REx6UERLZEluVnRYVlFpMnJFdmtNekNNTmtTLUFSOFpZZ1dGTlNUVDVYT2djU0VCOFZFV29lekctQ1NqOUdFdWVhWllm0gGOAUFVX3lxTFBRenJOZFIwM2dOWTdIT09fdXo1VTFCTndkeHpBbDFkRTUyWlZ5SmU5SWhLeUplM1BRSFR3Rm1xY1M5OHNwTUVoMHFVckpUaFpyWTYxMDdEM05QQ1VGU0JJekR3NnZ2VFNrcUZYby1oTlRoSmRtcG5DMFc2OHcwTnpFdjlPbE0wa3R4MjhKUEE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxNWjNPblZNVEJ6LVQta21YU1BWamE1NlhzdzhWY1BtVzkxZmJLTDFMNHFkQXlzY2ZGWlQ4ZDN4YjJ3dkZVaEs5aUJ0WHlIYmRlanVralJGaGRLRHJRZ2ZPYnMtLV9ldmpldWFnUmZEQkx0a1E3TjQwUDZ6M0k5b2xzNDMxaWM1LXRKOVpj?oc=5</t>
         </is>
       </c>
       <c r="F22" t="n">
         <v>1</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>46016.54236111111</v>
+        <v>46016.92152777778</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>High Level City searches  France  English language</t>
+          <t>BV Logistics Companies</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>("Paris") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing"  OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+          <t>("Dropit" OR "DHL" OR "UPS" OR "DPD" OR "Flight Logistics" OR "Fedex" OR "Amazon" OR "Royal Mail" OR "Parcelforce" OR "EVRI" ) AND ( "supply " OR  "delivery")</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Major sports events in India 2026 - full schedule - Olympics.com</t>
+          <t>FedEx H-1B hiring sparks outrage amid firing of American employees, Indian-origin CEO faces heat, 'They are now awful' - MSN</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Thu, 25 Dec 2025 11:54:00 GMT</t>
+          <t>Thu, 25 Dec 2025 19:51:53 GMT</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxQc0RwX182RlFOVWtuXzRrRGJFYTZSdUsyYzhkYXJaYzRlV2UyT3VmMl8xU3lsaWtGX2ZRSlR0cWFfdnFqVXV3dEE2aTVDOHZvcEZXMl9ZYTZkRzBtRGl3YTdwZUhibS1vUzhCS0lPQ0djeDMyWFJXRDVMdmJ6a2JRckJWTG5mREVLMnBj?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirgNBVV95cUxOeHlPM3hoTW5jTzl2VURnSk9LZkNRTDlDYWFaZkZmdXo2Njhuc1ZrOXlwQzd0c2I0anMwMjhIN3R3dFAwQlBBMzVNcXVsdXRXU01NVllwdTJtNkswNFJSQWkzY0luS05zcFNIYkY4Y1I2aHo4eTRKMkFrbzVIckJlSjBHN2VnREkyc1VIeUVmRGtxLURBYjNNV2hkY3dqdlZpVkxQMmZURVUxVEV4ck92VXkzYTNuMFB4Rk9WeTBmek5IT0Zma0xGS1U0RnU4emhlaHl2b0oxd1k2dzVxczIyLXpqdk52ajR4OGtFdDBhdmtaSDg5Sktab0J4bVlqU01VeTlFOC13dUd3dnYzdFVHUVB2X2p1M1JGa3JQSjFuMDNVMGRMTUxsam5OWWZqTWZCdmdsNlFfRzJwQzdqbWloTjBNZU5sRHd4UEIyZzUyYU92OGZwdkM2Y0JqN1Y4SnNiMGJoU252aXlPQzZMSnk2cnd2OVd3WXlHcHNMR2xXLU5BUjFGZkpsemJWQmlTdXBkN0YxQm9UbXhlNDJxcFZRTmlyUGdLZWxWLUJFSS1B?oc=5</t>
         </is>
       </c>
       <c r="F23" t="n">
         <v>1</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>46016.49583333333</v>
+        <v>46016.82769675926</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>High Level City searches  France  English language</t>
+          <t>BV Logistics Companies</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>("Paris") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing"  OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+          <t>("Dropit" OR "DHL" OR "UPS" OR "DPD" OR "Flight Logistics" OR "Fedex" OR "Amazon" OR "Royal Mail" OR "Parcelforce" OR "EVRI" ) AND ( "supply " OR  "delivery")</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Kinetic Trust Limited Building a Base Near Support - Earnings Beat Highlights &amp; Budget Friendly Trading Strategies - Bollywood Helpline</t>
+          <t>Is Christmas Day a federal holiday? What stores are open? What to know - Cincinnati Enquirer</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Thu, 25 Dec 2025 08:38:37 GMT</t>
+          <t>Thu, 25 Dec 2025 14:47:00 GMT</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxQYU9uLW95VW95ZlRQNEVKUjRvRWVSaHlKdXJDdTd5blRaZFhtQWlrSnlTOWJHUUNyazdUN3NteFZQX2hXWDFYdVl0bnJVcEYwdUt4NTJIX3Y1ZlZGNDJoOUt4MEwtcE4tczc4Q0M3bVdvWTZ6d2hoOTlXT1NaTW9YZGhiWE0xTlY1SVhUS0JR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxQQW1KODloTFVYakxhU3pURTRiU0hiTHdtZTFrNXhXODFGczRGOGl5bGhHeFdRRFpDMXVRWVViblVNd0RmN290TG9XeEJLRUxyRGJ2V1Z1Q2xUZHlaV1dLNjRSR1lGWnBlWEc0TXJSNUs0Q1RGNW41VkVnV1ROTjVOZkplRjdwOHM3VUI3MGl3endfekExcjBNUlJnUXlCY090Sl9OV01QMEVadUZBRGlRREE3Y2w2Z1M5Z3c?oc=5</t>
         </is>
       </c>
       <c r="F24" t="n">
         <v>1</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>46016.36015046296</v>
+        <v>46016.61597222222</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>High Level City searches  France  English language</t>
+          <t>High Level City searches Belgium French language</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>("Paris") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing"  OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+          <t>("brussels" OR "Maastricht" OR "Antwerp" ) AND ("Bombe" OR "alerte à la bombe" OR "explosif" OR "colis sans surveillance" OR  "explosion" OR "colis suspect" OR "tournage" OR "poignarder")</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Is Autoline Industries Limited Forming a Consolidation Base - Market Sentiment Shifts &amp; Buy Sell Signal Notifications - Bollywood Helpline</t>
+          <t>Brussels unveils historic housing plan - financial-world.org</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Thu, 25 Dec 2025 11:49:30 GMT</t>
+          <t>Fri, 26 Dec 2025 01:00:50 GMT</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxPbS1kS1BuUXBFOWcxUE9UTHczUlI2ODNtSk02ZWpjTzB1UmpiSEMtaWd5T3doVk5jaXZjdmhDdlA5V2Z1VjdpMmQ4WGNMSXdwNG1ScFdLcUlqNURKaHNwc09JVXMyWXJVR0ZuSk1aWFlRbWJyQnNCTVQyRWMtU2lxemVYWkFmWGlIM3J2c2FZOE1RNzBLVmlQOHlXcTdld1FCMUx5cnZTTUpXRFNDMmc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxNZi16RVR5RGVNaGMzZktjMkI3azFRUndhc2NwYVlRTHphbGY5QnJqX196UmVQbDhaX0ExSGNmR3dWZS0zTHJWVWNlRHVYOVJ2aDlaS0trMm9rRmUwdWRIeGNZaFlaSVlVaWVkQ1BUWFAybTlEOHBTMU5ScVh6Y0ttWkgyLVdIYmJENFhGX21EeWt4LTJrYjNqdzV2ejJuZ9IBnAFBVV95cUxQSDlUVWFFMlZFZk1SOU9DVTlURWhLdHpHRjhtcFNxYW1ZLUFIamtEUDFUbGtybTBYV04xQWJFWllYS0kzaXh1WEUwNnhHVzJfQlFUZG82cnBNWVJTZWl6bXBZRE53eEVKN0gxMlBNYVdNeUFCZXZFRzZyWEZ1SURyVUMxLWw1MUVDYmJkcTdZMHJWZFR2dlprMkNWS0U?oc=5</t>
         </is>
       </c>
       <c r="F25" t="n">
         <v>1</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>46016.49270833333</v>
+        <v>46017.04224537037</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>High Level City searches   Belgium Dutch language</t>
+          <t>High Level City searches   Germany, English Terms</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Maastricht" OR "Antwerp") AND (bomb OR explosion OR shooting OR stabbing OR police OR evacuation OR "suspicious package" OR "unattended package" OR protest OR riot)</t>
+          <t>( "Frankfurt" OR  "Cologne"  OR "Munich"  ) AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing"  OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat")</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Man shot by police in the centre of Bruges, leaving him critically injured - The Brussels Times</t>
+          <t>Hinrunde Wrapped: Looking back on Bayern Munich’s first half - Bavarian Football Works</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Thu, 25 Dec 2025 09:02:03 GMT</t>
+          <t>Thu, 25 Dec 2025 15:30:00 GMT</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxObDZKVDladlB2QnR2cE5GejdBLWRtbTJLNVE1blFhOEtJaUtsWnVuWHBGYnA4cmJBSkVFWXNxVFprbGJsNGhURnJ4eGV2cUhEZjZodE9BSzVqTktTQXBWN1lXSlZma3FqOWI4TDVwMXVoN29CaDZVZnZnN3l2N0pCYW9MaWhMRWg5Sy1KQUFnaEhzeHp2YUdqbndtekNWOWVPUFR1Qno0aWpBaUR5Mi11RFJDdlhEeFIzYi0w?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxOazJXb3ZtQ01lOHpqZTRWbFJlZHEwNGJ2ZHZBYXZKWU1DTjNsUWhrRFdiOEU5Mkd5ek1TVVM3NFVIQlFyQ0x5anMwMFZnaE9ROHVCQ0ZaRnFJTVNpT0pQTFQ2OXIwX2pzMGxnYk1WQUY2TDBOZEp5YjF5OUdZZXg1UVpWTFVwbEZYMV96TTVqclYxbEtudHJiOEtqQXZ1eUZweE9QR1VPZVRwUGgtc1RqdDA0TzFKaWpuc19UOHlidjhxVDJVbzdV?oc=5</t>
         </is>
       </c>
       <c r="F26" t="n">
         <v>1</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>46016.37642361111</v>
+        <v>46016.64583333334</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>High Level City searches   Belgium Dutch language</t>
+          <t>High Level City searches   Germany, English Terms</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Maastricht" OR "Antwerp") AND (bomb OR explosion OR shooting OR stabbing OR police OR evacuation OR "suspicious package" OR "unattended package" OR protest OR riot)</t>
+          <t>( "Frankfurt" OR  "Cologne"  OR "Munich"  ) AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing"  OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat")</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Prison staff angered as government fails to act on overcrowding - belganewsagency.eu</t>
+          <t>Short Term Trend Reversal in Deep Polymers Limited Possible - Monthly Performance Summary &amp; Explosive Capital Growth - Bollywood Helpline</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Thu, 25 Dec 2025 11:41:00 GMT</t>
+          <t>Fri, 26 Dec 2025 00:16:57 GMT</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOa0JZczJ5VkVoMUZSUS13VnZGSVVzQjdqYzg2VFRtY3NHN0c2ZzEzWXRiUTNVOXQ3UU1VNHJDQ3NCa3J0elRqdzNoQmkxR3IyYXplOFZROF81OWhnVERBRVBieVBNcHVRclQzV1RERGhlYkxJc25mRXZxWXU1RU1Vb3NnYk5sQ0ZiXzMwSm42OFBhTjhOMTRzcWln?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxONGxXVUY0OEZfeFFrcEN1SjVuMkMwOVRuN1poZnU3eEEzOENrTldmM2JtV2FWZFphVnJSMTZrZk9XSzl0WVJXODAzSGl6emF1WDhfX09JTnlTOHFyd1lMcEd2ZGctVXRUY3phQnlhYmUzT19fX2V6WWdFc0V5Z0dtd3ptUEt3VFhIbF9UVElNTGpmaThMSU1IRUV3?oc=5</t>
         </is>
       </c>
       <c r="F27" t="n">
         <v>1</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>46016.48680555556</v>
+        <v>46017.01177083333</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Ireland / Kildare Protest Groups - Social Media</t>
+          <t>High Level City searches   Germany, English Terms</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>("Kildare" OR "Newbridge" OR "Celbridge") AND (protest OR demonstration OR activist OR police OR disruption)</t>
+          <t>( "Frankfurt" OR  "Cologne"  OR "Munich"  ) AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing"  OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat")</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>North Kildare RNLI Raises €117K to Fund New Lifeboat for Wexford - afloat.ie</t>
+          <t>Piccadily Agro Industries Limited (530305) Hits 52 Week High - Breakout Stock Watch &amp; Explosive Growth Opportunities - Bollywood Helpline</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Thu, 25 Dec 2025 12:17:56 GMT</t>
+          <t>Fri, 26 Dec 2025 04:29:26 GMT</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNeWwzN3NYYzMxMFBJSWlXcDBuOTFtS2NXZzA2VzI1Q0xrNG84NFdaX1d6NTZpWlNOckRpbTlScnlPVlliMUp3VHgwbmNJR1p3OG9KUHk0dDVEOE5yblNLVmlMZWp0T09icEpWZmV5X2NwbmZfNGZ1aXBZaHMtWlVTa3F1Y194emJCX1o0dUFEY3RUbzg1dDNzNXJ6R2FYcGhhdmFVX0dPQUEyZ1E2ckE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNZ05vWkVWOVhjbFBGejZxYkw0ZjAzQkpxV3ZzOTREYnA4TWp3bks1c1R6ZmRKMFFkWGNkMHg4b0ZGb2swM1NkX2QtbWtWYmpHaThfcUtGcklzS2pyX3JQSU83bU85emp5ZGUxTnFnT01MZkZoRmtnYnBDSTRGT2d2ZzUzM05jYXd6MVdSSjNoMmtNX1Z1VTJRZ1l1UEpzNU51cVgxbWV3?oc=5</t>
         </is>
       </c>
       <c r="F28" t="n">
         <v>1</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>46016.5124537037</v>
+        <v>46017.18710648148</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>XR and JSO Broad search</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>"Extinction Rebellion"</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>The impact of the Palestine solidarity movement - Red Flag (AU)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 01:26:12 GMT</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxNM2tCeDFiY3N2cGNfUjduWXdkWjd3Vi1zMmlhMlpsY2ZCbnlPU3FmTjZFZklBaGdlMkVCNUhvbTc0VXRFa0gtMmZLYlVISDh0RHROdDZnM21PQ0VIbTMyNjdGRHRFd0dFVHZYLV84M19OT0tIVElQQTk0dWxNS3Z5UURJY0w?oc=5</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>46017.05986111111</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Shoplifting UK</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>"shoplifting gang" OR "shoplifting trend" OR "pickpocket gang" OR "theft from person" OR "retail crime" OR "shop theft"</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>C.C. Citizens Police Academy Alumni Association responds to officer investigation - KRIS 6 News Corpus Christi</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 03:26:54 GMT</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxPZFpLbFZFRld0eDZ2Qy1ScWlOTkJ5bGt5aGo2OWhKbE5Md2xoMlk3dDV5eDh4ZGo5UFFSbndNUDRicW9zRWdGR1ptU3FfU0t3NTQzdk4yQnpuZEFXVHk4OW1SYlg4Nkd3VVhUTFBKSUhkOXMzdTVnbzU1UkhHbE1QYmR1QlpNOTZTNFIwQ01PYm1DRC1HcDVzUUMxbmFPZDVNY3dITFJpQzBIUTN0SC13WmpWNzdxa0hMYkllSzBnQnZodGc3YmpqWUJnX1FHcDh1UlN2Q19GRnEtRVR5MGtnS2o1RnJFQ1hLaEw0?oc=5</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>46017.14368055556</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Shoplifting UK</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>"shoplifting gang" OR "shoplifting trend" OR "pickpocket gang" OR "theft from person" OR "retail crime" OR "shop theft"</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>$400K shipment of live lobsters hijacked on way to Costco in possible ring of thieves - New York Post</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 19:56:00 GMT</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxON3VOVFpIeTUxREdqeUhZX193ekxoOHpFQ01hbWVWT2VpcXo0TXVmQURRTU9QMmhUclFvdmczSFhWSy1nYXlkQkZxcmNVM1N3a2M0bloyNWVWQm4tQ05QblU1bDBTdTRRQ1VzUVpvNEdBdHU3QWxqUW0wSjJhb3UycHdIN1Q0b2dzdXk5c0hPY2lWc3pzc05wY3FvOERLY0FWMDU1bVBISk10SGg1a0R5UlBqU2R0S1U?oc=5</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>46016.83055555556</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>High Level City searches   Spain, English   language</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>("Madrid" OR  "Barcelona")  AND ("Bomb" OR "explosion" OR "shooting" OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat")</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Fabrizio Romano Transfer News: Man Utd ONE TO WATCH, Barca PLAN, Glasner BOMB - FootballTransfers.com</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 07:59:00 GMT</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi5gFBVV95cUxOQmRKbzBENlRjT2t2VkdwU3dhajZGRFYxMmY2TkFsUUthcUUtNWtTRTJsNkhESTJZaXJjMG5PNGRWbEc5MkJtRlFYcnk2VWsyUnUyTnNVQlV2bUJMWXdqR0FQS29KXzJ6YW9JTHNCN1F0bzU3UEJULW1VUzVXRGdUbk9OVjBWSGdGbTFNNFJfTTJZUE5MS0tqcTh2Vmd2ZmlGanpBR1pORzNQOEZiZXQycU43YUstZmhpT3V3eFdySzBHbURLZ3QtNmVxMjNLelJvRGNyVHllcDZVSS1sWmZlaTAwSV9tUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>46017.33263888889</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>High Level City searches   Spain, English   language</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>("Madrid" OR  "Barcelona")  AND ("Bomb" OR "explosion" OR "shooting" OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat")</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Can KFin Technologies Limited (KFINTECH) Maintain Its Valuation - Emerging Market Stocks &amp; Capitalize on Stocks with Explosive Potential - Bollywood Helpline</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 00:11:20 GMT</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNOU9mbEdGbFBGbTlja2RpVUV1V01kZ2gzeWFMVnlTeHhKb2hNNWlOZDRkbWYzRVU1OHZ6SGNQbnhBMzhyVGN2VDBDWXFuZnh6czM4UTJMbktoVDRGZWRtU1R4eTRXbEVCQjVNdjF1RXJZV1JGbTVDUC1ldkR1aGNTZGFrT1A3eElEeWszbjhlVmhLQl9kOTJfcmtrMHRtQVE?oc=5</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>46017.00787037037</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>High Level City searches   Spain, English   language</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>("Madrid" OR  "Barcelona")  AND ("Bomb" OR "explosion" OR "shooting" OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat")</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Andreas Christensen and Marcus Rashford send Barcelona into Copa last 16 - IOL</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 03:26:45 GMT</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPU0o1WHA1OVFZTTQ4LVlaZWdnT3BZY0pteWowcHZLcVg1Ni13b0I2aWFGMHhoZFZianNiZlBVQWxvR0NicDFMSFI2c3VmS3VST1pkQkVFTTdBUlpFMjVZZDFqZFZoU3cxbnNPZGJSM1I5VjdfLWw1ejJKOU9QN2VTbWVldTVEWGRGbzFvSTlJY0xSbFdsZEw0QXFqbE9jdlBZODh0YWVkOWhLR1J2bHctTEtjSHpYUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>46017.14357638889</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>High Level City searches   Spain, English   language</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>("Madrid" OR  "Barcelona")  AND ("Bomb" OR "explosion" OR "shooting" OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat")</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Football transfer watch: Liverpool beats Real Madrid in the race to sign the ‘new Vinicius’: Report - lokmattimes.com</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 17:04:24 GMT</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOLXplSUczRlM5VVVaSThvdi1XVW5ieUw1dXJxd2ZPMmdwVFdMaC10X1FENHpJTmNpaW1uOFZDSVpnSk4wNW15X2RYWWlKbGpRWFhtc2tmTTZIbDRIVDRSU1FnbUh0OTFsQVBrdFU1a3VNUkNmWTE2c3hvVFVCSkNoSF9kZmVLUTI5VmxjdUdXVWRDVHBqWkplUEJYTm9oOGM5VHc3dHhBSGFtdnpxSWxKQ2g4NUNrYVBsSnNoTVUyZ09mR0pDSnlEcS1CbW5hNlpSNGpFU0t3M0bSAdgBQVVfeXFMTi16ZUlHM0ZTOVVVWkk4b3YtV1VuYnlMNXVycXdmTzJncFRXTGgtdF9RRDR6SU5jaWltbjhWQ0laZ0pOMDVteV9kWFlpSmxqUVhYbXNrZk02SGw0SFQ0UlNRZ21IdDkxbEFQa3RVNWt1TVJDZlkxNnN4b1RVQkpDaEhfZGZlS1EyOVZsY3VHV1VkQ1RwalpKZVBCWE5vaDhjOVR3N3R4QUhhbXZ6cUlsSkNoODVDa2FQbEpzaE1VMmdPZkdKQ0p5RHEtQm1uYTZaUjRqRVNLdzNG?oc=5</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>46016.71138888889</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>High Level City searches   Spain, English   language</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>("Madrid" OR  "Barcelona")  AND ("Bomb" OR "explosion" OR "shooting" OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat")</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Heatmap Data Shows High Activity in Remsons Industries Limited Sector - High Dividend Yield Stocks &amp; Explosive Capital Gains - Bollywood Helpline</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 02:31:54 GMT</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQUlJKV0dGbW5xdXdmR3NCcTJvSmlWdFNJQWg0RC1zcEpzbTBUMkJvNGp6dFprS0NKbll5WkhvLXdTMGVXWnlQbi0wbXlXWWJsQk92bTk5dTFmNWpUa1VpRmc0bWpsM1FRQzgyRzQ5RFBXR0J5NmxwNGJWOEpJb0NXdzQ1QkVCdDRYTHNfVHUtQlV3VjZwc3RSbi1hbGRmenR4cjJKZXJwbmNNZkpMMUJmdXhoLW5rU1VFTlIw?oc=5</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>46017.10548611111</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>High Level City searches   Spain, English   language</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>("Madrid" OR  "Barcelona")  AND ("Bomb" OR "explosion" OR "shooting" OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat")</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Would You Accumulate or Wait on The Ugar Sugar Works Limited (UGARSUGAR) - Stock Liquidity Analysis &amp; Outstanding Investment Returns - Bollywood Helpline</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 06:09:31 GMT</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPOTQxNDdCazJTU1g4Tzd4ekVGSWFCV2FLRmctMHZ1eFAtaGZOMVRsOS14Z05jMmxrSThmaWk1UTNPUFNtUjhQTkVJaDlRYnIzeUpnck5NQi1NdVF4bUVkWG5CcEswWDlxWnhvTi1pWF9YV1V2eVp5Wjl6OU9uLUJoM01NaDFzVFhVMzlMX1BXMEF0VENmbjJaNFpYM0NLUlV0SkRyVHdjNEFZQUE?oc=5</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>46017.2566087963</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>High Level City searches   Spain, English   language</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>("Madrid" OR  "Barcelona")  AND ("Bomb" OR "explosion" OR "shooting" OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat")</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>“Has been offered to” – Fabrizio Romano provides shock update on forgotten €44.5m Chelsea ace - chelsea.news</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 06:45:00 GMT</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTFBVU2RjOHA1LTRHQjZVMUtfOWVId002bkJsWmFkTUtIYTJHWGd3Z3JoWURnVmZtam5CMkNSVDNtV1NRM3ZKX1ZDMm8xdXFIMzBvNmZSUm5jb1FyQzB0MHdXUGJkU3BzekFWTGhjS2hDckg3MGtTUjRN0gF8QVVfeXFMT1dDNlo0TnViczNCV0xXOEd6WlpUMlZucVBrdHdYOWIza3JnRHlsUWQwUHhpUmpqbXBwa05KSXlNS1dhVVZKeUN3ZnlwRE81aTJrblhTS0xlZzlKbnZtNkxxQjdRdHBVVVZSSW9xTzJxZ3ZsZUhoT2ZtN2NVRQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>46017.28125</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>High Level City searches   Spain, English   language</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>("Madrid" OR  "Barcelona")  AND ("Bomb" OR "explosion" OR "shooting" OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat")</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Flamengo fans cry foul after defeat against PSG, Cherki “bomb” gets people talking in Spain - French Football Weekly</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 02:11:26 GMT</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxPYXZxWExDZDNJc1gzTFE2X2VYNktXZzlpSmhfTW1vNWFWZ2JBdk5Da0F4WllNcDJNLS1oSnZyV0lEWmFNRUx4Y19OWDZjUjlORnpBVDVwMGlpZ25qQUdWOUtCNWlyWFBzeXRxMXhBM1hQMkQ0d0Rrb01mdXZEZUItXzl3ZURxLTgtRy1GaXJOem9NRnBXa041bEVOdHFNZFBFWXVyd29jak1RLTVWZDdQX3dzT3haeTd0VGpmMnhxVnpIWmNJbWV4S1JlUjcxQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>46017.09127314815</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Local Town Searches Bicester and Kildare</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>(Kildare OR "Newbridge" OR "Bicester") AND ("protest" OR "boycott" OR "bomb" OR "shooting" OR "explosion" OR "stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Police hunt suspect following Bangor stabbing attack - kildare-nationalist.ie</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 15:25:35 GMT</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxQNFNaRk5qb2dMZDM1TkFIcEZrNnAzamtuQXBlN3JOVnJieFp4RG00cW9IVC1GQnFPeHFxRkVkYjZpOXFRZmNCWk9UaW10Wk9RbHM0UkpvdXVYci1lNXB1UG9sakpkN1hrU2owTE1HTGpGTEdsbXJfTWpESVZyWVdDTVlYSlEtekE0WXFhVV9SaUFJUnhhWjl4OVhubkUzTFJLUHAxTVhDd1JDVk9v?oc=5</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>46016.6427662037</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Village Search Bicester and Kildare</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>( "Bicester Village" OR "BicesterVillage"  OR "#BicesterVillage"  OR "Kildare Village" OR "KildareVillage" OR "#KildareVillage" )</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Discover the ultimate shop-and-relax treat with voco The Club’s €50 Kildare Village gift card and stay package - MSN</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 05:51:33 GMT</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi-gFBVV95cUxOY1cwd05RU2VQbmtzS3NmejlJN0Nhd1RUdjRmX3NjWXgyc0RqaXNnTUZhcVExRGNIQnJvamNxazJialBOWFpiUXp6d3ZMajJWaFFsY2FIOXlPRVlIOGlvN05zR2I3bnF0UVlNSFpnamJ4XzJac09LR3JFaWNVekcyU0IweVZVa1BUWVJQV2xrOFlYaFY2dWtoblBMY1ZOdlFTbkl6T2NKR1h4VlBYOHNYbGpmanN1VkVENHZ5LW9BWnM1WlFWZDVoZ0VHMldOSUtRTlNNcWJvWV9hak1FUVRQMFlHWEFNa1ZjaFNVMDFFckFtZDVHaS1fS2NB?oc=5</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>46017.24413194445</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>High Level City searches   UK &amp; Ireland</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>New Covent Garden bar inspired by New York's cocktail scene set to open in 2026 - Wimbledon Guardian</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 05:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOZFF6RDJsSHlmNVk3SEl3dGpEeF9OZjFHYTNPSjRESGp4WDZGdE5ET0pRb1lhODUxVjFfNXdlX1RCd3djSU5YVEJFR3BvMGRFRkdSMDhJd2VIellkU01UdlA5Q0xhSzFCT2UzWGk1M3I1U0FtWUZXQk1OOERneGxJR1F5OGRhS1VIZXNnWm5qeF90cDhvaHcxZzh0ZWdDcHRwdk1ibW5oN05ocTZkZFhaVDcyN2xFTmREeGhEZg?oc=5</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" s="2" t="n">
+        <v>46017.20833333334</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>High Level City searches   UK &amp; Ireland</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>'I'm a bin man - don't throw away your wrapping paper this Christmas' - My London</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 17:34:59 GMT</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE9BMUZibTcyc0doZ29ySFk1RElZa3Q0cHdRZjR4X1MzZG1kTER6dVJ1V0RkbmhLVVUxMnphbF81T3RvdDNMdUpWTzJfb1VwOGFuQm9penZpTGZoUWg5V0YtMXpJRExmS1hiSExta3R6a01tZmh10gF6QVVfeXFMTjZ6Q1VBRy1ZLUl3UkF3ZzRxakNYby01NEtqbTFpQUdoVzZVMm93RTNsS3JSMkZ2TDJ0dFdpci02YkxlRXVtRG94ZEJuUG1STXVhLTBqVWctLXFzaWtBb2o2QS03cGc5LTN5bXZqQkxuUnZUc19IdHZZVHc?oc=5</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" s="2" t="n">
+        <v>46016.73262731481</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>High Level City searches   UK &amp; Ireland</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Danielle Galligan selected for European Shooting Stars 2026 - MSN</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 03:24:52 GMT</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxOTGFtOEpiTE56SlZpVUxhTVBHUmJaYm9BOUlPNEJxU0tsVFhYNUpyM2dWU3ZsSFJ1MkpZNEJaeGkyQ0NFUWhvVGoycHBJU2pSRVVUNXpBTHRMblJYeWFUUkNSQ2t1VTNQMXNGMTVtb1pTZm5HMmVBYzJ3a3BxX1RlNnNPNUtoNjFjREFNSHJHR1BHcHRIZzc3ODFQajRYdDdORHQ2QThPVEN6V2NxaWhkbTl4NUVVZDN2U1E?oc=5</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>46017.14226851852</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>High Level City searches   UK &amp; Ireland</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Early Christmas morning shooting injures man on London Avenue in Gentilly - WDSU</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 15:02:00 GMT</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxQRDRVY19iS1JnemI1Z01yc2szblc1S3JubVpVSTdaMmExdmdVai01a3VTTllIWGxMbFVhZTVpX00yVUpMY3UxY0pRVEVhQmx6MFlkcTJGX253RF9pdmctVHpIbWh5UkpCUGRiNHFiT2stM3ZWeFdSYl9paGJzMnNudW5vOVROTnJpZ25Qd0I1M1dXa3ppRUdhZ2FGcTl2dVoxUUJISUJBMHZrNEt0MktsWTln?oc=5</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>1</v>
+      </c>
+      <c r="G45" s="2" t="n">
+        <v>46016.62638888889</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>High Level City searches   UK &amp; Ireland</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Michigan teen gets life in prison for Oxford High attack after wrenching statements: ‘I’ve done terrible things’ - nwitimes.com</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 16:45:59 GMT</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi7wFBVV95cUxOdzByTkdWdXdFa2h3eWxPSkFHMm84TmRKRTN3WGxBNFN5ZGY0RFFwM2VsMmxHS0VSM0FMa0poNFhKNENmbG9Pb0FkcTdPR25Vc3JKMkJ5TzZIbnVPazBEZ1doZ0FGLWUzYjdfcWRkckh0X052b2ZybW9CdVlxeWowaDlvSGJ6OWkzb0hJVTFwMWdQLURpWV92NGdsQnItbTRxTjNxVnNnNm1FTkd1emNJWTJ1eVIxcUxQN29XWmhQMUNIVS1Hb1FOeUpkaDk1QkxoU0hONWEtN0thTDM2aUxWS3pYMEM1NUNQMEZVSTdVTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>46016.69859953703</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>High Level City searches   UK &amp; Ireland</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Published on: 2025-12-25 21:18:12 - Bollywood Helpline</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 22:50:30 GMT</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxOUXgwdUZERVRDcjNYVEtNX2VBNjhDNFZrTkJQUG1Mc296SGhmNXFYRXkyeW44VVQ4c2F0ZUhNZ19vV0hraTV3MVdURFVNNFRGbkU0c0JuWFFMdHZYVV82ajNiY2xXRk1UYzJhRXJpaTAwWkIzRVR2clpNYmpDcDBpanFKaXVya2Z2Q0d0UXEyaW1nc244WXYxaklESlMwTm50U0tYN0ZOa2VIRVplS1dLcGlsMnFCMlhucXc?oc=5</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>46016.95173611111</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>High Level City searches   UK &amp; Ireland</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>‘Build a Bangla, we dream of’ - The Hans India</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 03:03:32 GMT</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxOS0FkQllzM3NmSVVzSXY4RDUta0VFckZsc2swWWRONldtbjE2OUZmYl9paXNXRV93aS1SZjh1Z21zVHJRM1VaNVYtQWYzNzFreEZBRUtnZDVsdjZ6WkpraEwzOS11NVlBVFVEalRfZkNCNmdmNDJsT3BVMHB2SlJSZ0gtekw2eGdT0gGIAUFVX3lxTE5LQWRCWXMzc2ZJVXNJdjhENS1rRUVyRmxzazBZZE42V21uMTY5RmZiX2lpc1dFX3dpLVJmOHVnbXNUclEzVVo1Vi1BZjM3MWt4RkFFS2dkNWx2NnpaSmtoTDM5LXU1WUFUVURqVF9mQ0I2Z2Y0MmxPcFUwcHZKUlJnSC16TDZ4Z1M?oc=5</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>46017.1274537037</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>High Level City searches   UK &amp; Ireland</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Hyderabad's RGIA gets bomb threat for Flynas flight; lands safely - irishsun.com</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 15:31:00 GMT</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOek1CclNaWXVrem9xZUZ1ckdENkxVWVVfRzdYM1JIVWVEbG1kZWIzQlUxUjE1aXEyUzJubHVsSG16OHdLRlpTWlhobW9JUnFVcnBQVlV4dngzVHY2aGlQak9EbVFQck02NHE4TjY0YzRncS1NRkxFYkdqNTNCa0R1TGNWMnZkcEpMMGZNZ3dOUWlkeEx0WV9fenJsOG1QdHpMUjBjRw?oc=5</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>1</v>
+      </c>
+      <c r="G49" s="2" t="n">
+        <v>46016.64652777778</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>High Level City searches   UK &amp; Ireland</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>The 5 best fish and chips in London according to reviews you need to visit - Tottenham Independent</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 05:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxNY3E2VTc3dFBUM1JidDU5MjRDd2FUTWhDVEpsQ2wtNEI2XzA1czVXWnpXa2NydVY3Sktpa1hISFNCa21RRENNU05ZLURyaS1qemNqNFlQaFBRR3VPVEVsT0Z0cU1Gb19SUnp4elRMazA2R216Z3ZjMEU2WHg4WEo0UmZIVERVMUlPeUNJSmpKUWNHa0JMbmZhazVmVVZSdGdCTThqUHUzYmE?oc=5</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>1</v>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>46017.20833333334</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>High Level City searches   UK &amp; Ireland</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Bromley women living longer than those in neighbouring boroughs - london-now.co.uk</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 05:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxNeXBYSU5XVWNocTlrU1hpZzVrRWhlcjJUN29xTzZfbWY1VXJzMExZR0YtcEdhMmFfeGJtcUdZTXJIMjBja01Ld0d4VzZKdGlhclRUa2RMOFVDZjUzcm9CSkZDSm9jdWFqZEVGVnVSVjA2blNFN1hTSEwyUXQtcTJBR0kzZC1vRWQ0WU5xNEl6OXdvS2p1ZXpabXlrbmNUd0xJdTRV?oc=5</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>46017.20833333334</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>High Level City searches   UK &amp; Ireland</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Businesses across Havering that we lost in 2025 - london-now.co.uk</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 07:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQeGw4b0dmQUwyT09PMU1waUlNTzJnODRhM25NVGR2bF84MDdYWHZWN0VTVkpVanNZOWwwZ1RvekFhd0tfNlNoTjVucGZFRGl1am9WekhGU1ZxYllFQTFYWTkteFFQdWJ2eXdrck44YUZabzE0WHR4SWZSUnlRQVRfbmZXaUZweXRrUDJCMkJMcFllUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>1</v>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>46017.29166666666</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>High Level City searches   UK &amp; Ireland</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>All the biggest developments coming to Southwark in 2026 - london-now.co.uk</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 05:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxOV3NjRFBjb1UxUEhqM3FXV2RGLUtielVGZEdqTi1SUnEzdnRXaDI1ZUVPTmZwOVVhUGlsbUNDMFFyd0huTnpzNk55TlhjRnFJX00tZ0FJLXRzb1lUejk0ZzctYkdPUS0zNmpFTzdWVWRiaUdZcGNFOVJNVVRvTWRUQkJDTnVlMkpwb05SblE1MFpWN3I2U05N?oc=5</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>1</v>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>46017.20833333334</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>High Level City searches   UK &amp; Ireland</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>New 'fantastic' shared ownership homes launched in Epping - london-now.co.uk</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 07:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOb1p1R2dDLUVGQWJ1aTRpSC1XaG5SdkVDaXdLbGVtaWZSVFBzVkRJOXF6QW5PUjhrLVNSaVFIQ0djWkg2aXR2TDZ2TkJRRHhaMjJxakdVYWFUNDJqeC1VbkRzaWZtX28taU4zVUQ2c1NvaVRDa0pFbFIxdVRaODlhLTFOUFhvc1p6dmlFamZRak1ndDYxd1l3ejg2WmJpLWY0ek5MQg?oc=5</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>46017.29166666666</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>High Level City searches   UK &amp; Ireland</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Vue Bromley to screen a packed Christmas weekend of classics and blockbusters - london-now.co.uk</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 05:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNS1FndnRnb2pITi1qblh5cEtUX0RhdE44S3ZES1EtRDE0Uk5IbE1tRjBIV29RdXVEWkpaNDlaNnRweWdSbV9iY1dZYzVYb1ZVemZpdkM0NnRyNllnazcyaXNkbU9EeHIxNXVMZmc0TENudVplSVpadGFOdElFYWdGQ3ZHbUhKa0plUGV4bGNjSWFjanpWSzFyNUVraXNoM3F6MEE?oc=5</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>1</v>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>46017.20833333334</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>High Level City searches   UK &amp; Ireland</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>UK snow maps show 13 counties to be hit as far south as London in Arctic blast - The Mirror</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 21:32:00 GMT</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE5RdDNWUmc1eTg3eHI1MmlFaEdQVzNLU3BuYzlLZmhtbW1qNXk2RVVKME1oNFBYNWZDWXpkdGJXdHF6d0gzWUlpVHBBSDdiT3h6akFJYjF4bEJFMVJkaXZnUmVjREVWdUc1S0x1d1FpMkFXRjBqX2FiTGRlONIBe0FVX3lxTE5RdDNWUmc1eTg3eHI1MmlFaEdQVzNLU3BuYzlLZmhtbW1qNXk2RVVKME1oNFBYNWZDWXpkdGJXdHF6d0gzWUlpVHBBSDdiT3h6akFJYjF4bEJFMVJkaXZnUmVjREVWdUc1S0x1d1FpMkFXRjBqX2FiTGRlOA?oc=5</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>1</v>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>46016.89722222222</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>High Level City searches   UK &amp; Ireland</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>UK faces 739-mile snow storm 'lasting two days' with 13cm set to settle - Birmingham Live</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 06:25:00 GMT</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxPLW42STFjN09zM1FxSm1EZzgzQUdrTFp5cV9tY0VvOXY3UFF2ZUFrR1hnbkJIbWVoeHBqNENGWERiVnM3YkZsLXRlNmxGZDRHQlhjNzJvWkloMms3dnhGSmczTmtPYm40RG90WHk0R0pxYXlQTkhPNl9kcDJ6QW9KajRHR0JIQzRrNko4WTBjaDg?oc=5</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>1</v>
+      </c>
+      <c r="G57" s="2" t="n">
+        <v>46017.26736111111</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>High Level City searches   UK &amp; Ireland</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>King Charles pays homage to Bondi heroes in Christmas speech - AFR</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 22:11:00 GMT</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxPNndTSEd2RHZORzl2eGlBMEpPY1NHcUdpVU1RZGttSkZmX1ZXZ0VuMHZmTExDdXhKVHZjMkFBbmZLTjVMd2VCVXBoQjBCVnVEeHc2SW9vSzlXQlR5SlVhaEtkNkM4RDFIWlZWTDEycmtBTTN1MFFpSm1tWE5aMi1TR2FYbjdjVlBOSjFzU282ZEZyZVFla2NvUWJ5aFhhemdnckpmVjM3UnNhRGpBM0E?oc=5</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>1</v>
+      </c>
+      <c r="G58" s="2" t="n">
+        <v>46016.92430555556</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>High Level City searches   UK &amp; Ireland</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Call the Midwife icon gives huge marriage update after moving out of family home - The Mirror</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 21:15:00 GMT</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxPYlhVTS0yQ3BMZ1hQS3pOZFNIa213VmdYZnlTOGxKVUZ2elZkMFdzQWEwM0F3cTI0ajFQV21BQWg5aGNVcHRUX2xXMVAwbmk2TG9YNmJObTZPbUJDV2kxSGo2cHRET2taelNZZVpwT1JlRnNVUnI3MXdfZmE3eEtpREUtMNIBgwFBVV95cUxPYlhVTS0yQ3BMZ1hQS3pOZFNIa213VmdYZnlTOGxKVUZ2elZkMFdzQWEwM0F3cTI0ajFQV21BQWg5aGNVcHRUX2xXMVAwbmk2TG9YNmJObTZPbUJDV2kxSGo2cHRET2taelNZZVpwT1JlRnNVUnI3MXdfZmE3eEtpREUtMA?oc=5</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" s="2" t="n">
+        <v>46016.88541666666</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>High Level City searches   UK &amp; Ireland</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Irrfan Khan’s health deteriorated while shooting Angrezi Medium, was in immense pain, reveals costume designer | Bollywood - Hindustan Times</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 03:18:09 GMT</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgJBVV95cUxQOGlRNDlIUlNGN0c1SUpfd1dxWnFLSmo5MzR5UDZqc2lPQkpPaGZGYXd6eTY5X1o2WEdhMEs5U1VXX0Fta2NaVmpyeTBpUzVtdlRpTE5FRFQwUU5IbkdMUXVfZGp1QnhpMEpfMHVvZGEzRWZ1aEgwOXU1NmRPR1VNOFRYZ1NnUV9MaFBlSkFnN3lmN3JEMjNETHdGYlI4Nl9oT1UyeDJZRjBQUnF1dndsb3l5WFZzVlNKQS10czR5SnRuQmNLbHdYT090a2RESk5hWTlWdFZwMC1HZ2V3bm5lc2lqdk56OXVxeFZBS2M2SWpJOWl2MzZkQ2dCaUpCcTM2dFpxSFBockNxT1BjSnJzYVJB0gGXAkFVX3lxTFA3MHhoaV9nbWFOR1lpRURxNUZFbHRqUWJNUWxTN0NSMjRZMnBiVVBKSW5KRWwzOENNdWFLOEdXci1FRWJZelk5ZjBybTgyV0hlcjB5VGNIWlAtODRqc0ZDeGlRQmFTRjB0YVcwc1VLYkdVanRfY2gxeUtfVW5UcnhaOTFXS1B5UnJUY21WQnFPWXZfMHMtdVF4NjFId1lpU0VWdGtkRVBzajBtdDc0YmtnN3hFUVJ6ZEhGZ01PeFdzZVBSZDd4SGVlc2xpT3RVUkJER2JLNk5OSWZrY2pST2VLWU01Y2RTbFNOd0x2ZGNkazRONF9pN2ZQSm1jdWtsR0tTczNITUd2UFhmNm1BUWhxUzFlSndYMA?oc=5</t>
+        </is>
+      </c>
+      <c r="F60" t="n">
+        <v>1</v>
+      </c>
+      <c r="G60" s="2" t="n">
+        <v>46017.13760416667</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>High Level City searches   UK &amp; Ireland</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Festive joy for parents as Christmas Day babies born at Ireland's maternity hospitals - Irish Mirror</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 14:42:26 GMT</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxNUlYwUV9TUGtfcjhKNFZxYi0tUlhSVVh3SWRiTWlkbU5EaUdhSlFLVnZuenRCVHN0N1RwTmxyWlRaQUdRNkhVS2dzblBUeUdmeTBsLVJ3Ym1aVVJkRnpkWGFuRVFHWU1rSXFsTk1uT2JJV3NSU2J3ekJZRVZUMkdGQWd4QWZGRkFEdktBVVB3UFhLUknSAZMBQVVfeXFMTVJWMFFfU1BrX3I4SjRWcWItLVJYUlVYd0lkYk1pZG1ORGlHYUpRS1Z2bnp0QlRzdDdUcE5sclpUWkFHUTZIVUtnc25QVHlHZnkwbC1Sd2JtWlVSZEZ6ZFhhbkVRR1lNa0lxbE5Nbk9iSVdzUlNid3pCWUVWVDJHRkFneEFmRkZBRHZLQVVQd1BYS1JJ?oc=5</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G61" s="2" t="n">
+        <v>46016.61280092593</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>High Level City searches   UK &amp; Ireland</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Bangladesh news highlights: Tarique Rahman meets Khaleda Zia after homecoming | World News - Hindustan Times</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 19:55:51 GMT</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxQdXFCNDYtTzRNWXNxbi1iNmdabkxZYTR3LXV6OXZtSXhsWTU0bXFNQS03UG1YQktpbzRHQktrZE5Lc1NBVVFJZEpGRWFjRFM3NU5XUUZrT3FBbVctY1hCZXJ5cmF6eWg0UXdfMDR1dVlHSENaZGM4bDVCWnNWV3dfdm5LWXJHMTBXVjktZ1cybk1MeU1tQXR4WVVDd2ZZYmlTaURDVWNwMTk5THhUaUU0NGxDVk1iYnVncnRTOS1JaThtbDd2SE8zdWpBUy1QQ2tNNE42YXdrX2swbHZxbTljNHdYR2hWMHZHZGFlWi1obXYwN3dn0gH6AUFVX3lxTE9ld1I0d0ZGQTZvSGllMktSUkVzZFg1eGQ5dm1GanNHVVhPSy1SQjEzeWZ1NGlNakJSczRFb2UtX05LUjNvQWRMMVhhdEFSRzNRb0FEVFFwTHNWaFhsRGR2N2IyY3VBZjNLVzI5VktOeG9lVEZCVlBkN0ZRdmpoNWJtR3RWTTFrSUlSdFRuVmNyYjZ6aS1PWlZ5QWVUUWVYelVoN1lKUm9iel93SG5wLU15STFQeFFrVUxscnZJX1ZybTc0eVJSUzBrNmFsT19ITkphQ21ma1pEem5XMVZ3cmowTjMyVFNLb0RzMmxYVEQwSGtBX0duZnNPd2c?oc=5</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>1</v>
+      </c>
+      <c r="G62" s="2" t="n">
+        <v>46016.83045138889</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>High Level City searches   UK &amp; Ireland</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Woman in her 80s dies on Christmas Day after 'serious assault' in UK market town - Daily Express</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 16:19:00 GMT</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxQbURheXYzRUZTSzVMc1pGdFRMbFE1SFZpQWppNFVvWDlWSDNsNVlSOUxPWmRsTU84VEFxRmdTbHhvS1VpYlp1Qks0RG5WUVNDY1JLb0FMUmMtQ3F1SXdXRmxJZVFnamU5NzlOOUJheWUtRXE0UVR6Z0V1bUJuWThKdzBweDhpQXFTMWdkZjBnZ0NWbGPSAZgBQVVfeXFMTUg5QjFwbDlKTTR6Qm1xTi1DNVpVYWdWeTFuLWQ3U1RYSGdUOWFOU21HdndjZUppbVpXbVJyNXlrZFNIakJCZVAxSXlMS1ExcDQzckw1LVAyeUs2MzZ4NGNtUXJ1VWttbE5pdlhuYmFOZV8wOGVQR2NuTDFlUWd4VGxIREY3MFJWOHdpUHpRQ2JHSlhhSzExeVY?oc=5</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G63" s="2" t="n">
+        <v>46016.67986111111</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>High Level City searches  France  English language</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>("Paris") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing"  OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>All Koreans want for Christmas is a better cake - Nation Thailand</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 02:07:00 GMT</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiZkFVX3lxTE8tQXhhT1BYcEhIVDJ6dkc1N3NPa0dUaEF4Z1g2cGRGVjRSc3BYVDBQTzZIQnk4eTVIc3M0TE1IME1NQnV4LUd4OVFzU2M4eTZmTEZIZi1fUW1RNGJucDQxMjRhMnhaUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>1</v>
+      </c>
+      <c r="G64" s="2" t="n">
+        <v>46017.08819444444</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>High Level City searches  France  English language</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>("Paris") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing"  OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Lily Collins On Her Struggles Filming Emily In Paris As New Mom - News18</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 04:55:04 GMT</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOa3AwMlRQTFpJcjNsVWpTaDg4bzVOWHhGZTllMFI1RWZfWlF0akNlX0d3NEkxeWFaamQ2ZjlXNVZUdnVZVDc3MTM0aUItOUhqUVhkdUo3ZEdxVDFvN1BoUEo5R1RSMC1HN2dzTEdkQ1lUVkdzSmZnV3ZCV3lrYWVhNjdyU3ZqSE5vS0diME4xVlA5cUQxNC1FTjM2QWhjZ2gyN1dqQ2xYazlhb0hPYXc0b3FaT0Q2cU0tcDA00gHAAUFVX3lxTE00MmhNLVVnbGFIcXhUR19qOUthenl5aWhENlZwWWliVlNfc20yYktQNGVyeWZVWUk3NURIYkZmdjZwcExfOVZ6cEFRVTBaUXpkX3ZZUi0xby12MV9zM2VPWUtZdWlQMWVON0MtY1c1Ql8xV2dzMHFETms1bjQxWE1GaWk3djZWUjk4Z0hNNDR5WnJ3RWU1NEp2cHAzZi1QZThVdWVscFFjTHRYN3N5U0ZnZi1hMEgzSlgzRk5QS1hCWg?oc=5</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>1</v>
+      </c>
+      <c r="G65" s="2" t="n">
+        <v>46017.20490740741</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>High Level City searches  France  English language</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>("Paris") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing"  OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>2025: Her Year – How Paris Olympics setback is fuelling boxer Preeti Pawar - The Indian Express</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 03:16:18 GMT</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQdDUtSUtrelB1S0c4OWxSSU85X1FWdUp6ZGJ2UXQ0ckhqbTY5REVuLU9PMnJGWjVCTUZFVGNGVl9YVW9aTjlndEJxRGNNcW9nNEI0ZTA5c3BkaVVHNVBEQzVOTHVqNVduN3FoaFk1bFdxWFp3dC1XbDBHZ19vcHNsUENGRnE2eXphQUUzTUJlcml2bzFKRGdhZWhDN3lHZ2xselE4d1ZEb09BLVNscEpGWmp5YzFnYllIbWww0gHCAUFVX3lxTE1YMjdINFdKVHM2Rm1hMlVjVHQ5TGJ4czhYekh1cXdLT2t4SWxJTTN3aURQbnNoWUhPUEdRY3otSDNGQWQ4a19ZU2k4WklBU1lEX3gwUThnRlFWVFQ3cGhhcFFMUlRUMkwxRUNNQTFtOXZCVmh3ZmxqMm5oMzZEV3E2X2laRk9teG1BcndaanZLOERsbXFjX3FkSzVwbGRkMGJxaWp3MHh5MVB1c0hhTW4wb3lydTEzc1BQMFZSYmVtaU1B?oc=5</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>1</v>
+      </c>
+      <c r="G66" s="2" t="n">
+        <v>46017.13631944444</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>High Level City searches  France  English language</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>("Paris") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing"  OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Zenith Drugs Ltd: Hidden Pharma Star Poised for Explosive Growth - Price Momentum Alerts &amp; Budget Friendly Portfolio Growth - Bollywood Helpline</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 04:07:01 GMT</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxQWXBrdXJxVWFrcGtuUk1aMklLRWJTQkFKSkpyQkl2YUw4bEVibWJPWnVQRC1YQWlEak1weEEwOVM3cFItZER2SWdtZmJhQjN5NmJJaXlzd3ZwRDFpb3RnTENQb2xUYjhTekg4b2wwT3JHODJUcGxoQU5lUGxwMlE5WE5uODBmZHBXREV1NnBLTlRDLXZvSVZrV08zY3dUVFZn?oc=5</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>1</v>
+      </c>
+      <c r="G67" s="2" t="n">
+        <v>46017.17153935185</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>High Level City searches  France  English language</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>("Paris") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing"  OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>SoCal mother and 2-year-old daughter who were living in car surprised with fully furnished apartment - ABC7 Los Angeles</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 18:25:46 GMT</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxORHYzWG1UcnItR1FBRXBsMHV0NnhCaDRXQmlrNmxTQXFJSEdMNFpMdElmb0pyUDNLVm1XLXhHRXRyVTN6SWwzeGNYZWNfTkp2VVdNSGR0eDd6a1J0SGZwa3Z2ZGs3Rng5SVYzbm9xbVZva2l4WFZiVWVZQzFVdGJQS3BGem1od0xta0xVbmgzY1Bhc3BYSWJ0WTRQOWVCTm5VQTJfQjYtalE1QUFGZVFZaWFrbU1vanPSAbwBQVVfeXFMT3FjT3JCazVVS2ZILW51dGE0ZTRHYzdBbGpoZlhHSUYwSWZ4b19RUzBSZDFaQjBJUng5emlaSXlkbTYxWjIxNHZDWUZOaVdwMFNlWUxtM202eGZiZXlYb1dVTFdzUmoyd2prLThmVndmY25hVXlWOHRwR1QxOFlaZkxVb0JXX1FNbTA5ZnFPMW1SMkJMdkVzSGNYT3RqdElDajYxLWxXVkZhZVlDS1N6bEdxTGZLdTRrcll0UnY?oc=5</t>
+        </is>
+      </c>
+      <c r="F68" t="n">
+        <v>1</v>
+      </c>
+      <c r="G68" s="2" t="n">
+        <v>46016.76789351852</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>High Level City searches  France  English language</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>("Paris") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing"  OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Following the Bondi attacks, a US rabbi’s plea to the Australian government - SBS Australia</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 05:04:48 GMT</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxQUjNYRlVOUWFfQTFsLUhzY2RrRG1qbUFLSE55WkFrLTNFeTZReTRwU0lvOVc1bFl4TDdaZUhzMjM0R3JZUEdvQ3JibzNlTG1weXZyYUw4bUZ5NDdiUnd2UnQ3c0hhNndsdnBPWXY5MjZMT2prR0tsTHR6bC1CUFF5RjVfanZidFFGTzNEUGVBSE8zQTlkOGJVUmdZRmhIUDVyZHMwYmVfMXdSMjRPazVDN1dlUXBrMFlBcWRHOGgxZVA4YWk4SE00Q2FDSnoyamR6ZF81WTR6TzY?oc=5</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>1</v>
+      </c>
+      <c r="G69" s="2" t="n">
+        <v>46017.21166666667</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>High Level City searches  France  English language</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>("Paris") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing"  OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Mehuli Ghosh Interview: Arjuna Award Nomination, Asian Games 2026, Road to LA28 and more - Sports News Portal</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 04:48:04 GMT</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQZXVDRlBXY1VtWHdvNUQwUWE4ZkM3ZnQxWjFnZm5IMGwwLXc2TFdldjllSWtEVV8yZ09DbXRkMkhYakxKcGtIR1d3bktPclNQeklLbllFOWNJY0JtTVRaWTh1NV9GNU1ITm9sSEdtbUY2OHpVNlRwb2pCZ2hWcmwxMV9XNTNEdW9FdUQ4OWY3SzZnSEV2ZFAxYjNSN2k4eXdMa00tZ2lKc3ZuRDjSAbMBQVVfeXFMTTR5OTJQTUJiM3Baa0lsUmlkc2tnNVJzQklhTzg0dHBGR2VOTjFDSXRFNlpJRFRFemQ2ZFM4ckNYZEJqX1kzME1TWXNDRDVMajd1QWV6QUsxUmxnQm5YYzBRWlhTRUtwNlNaaENsU3BuZHlqaDVnczBycFZjQXRpUWR0SVZ2SXFTMFJudmFpb2RkQmx6dkxTb0NjMWoyRlhvaU9KVHd0OUlRYVgybWdRc0RXeVU?oc=5</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>1</v>
+      </c>
+      <c r="G70" s="2" t="n">
+        <v>46017.2000462963</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>High Level City searches  France  English language</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>("Paris") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing"  OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Sentiment Tools Show Shift in Trader Mood on Mayank Cattle Food Limited - Bollywood Helpline</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 05:40:04 GMT</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNS2pkNHhqRVdHNENkWXRXNGdhZS1qMGlWcTNwbEE5MUlQb2RlLWZBdU1XMVh0eDlyMEtoSE1UVG80UGlDRjlKVXNJV3NERTlyRWtMNkR4cThPbUtMRExGT3B5N1liVDdPZjhwUVlmLVdHcUJqemlkRndGa0xQcUNIaEhXLWVqak5rRnNGUEd0UmwycmRtSW1OMlplZ2dKWkM4UkJISjN1dWl0Qm84MTFnelgwRzI?oc=5</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G71" s="2" t="n">
+        <v>46017.23615740741</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>High Level City searches  France  English language</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>("Paris") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing"  OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Used when: Market is flat or expected to stay in a range. - Dividend Aristocrats List &amp; Free Explosive Wealth Accumulation - Bollywood Helpline</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 23:32:47 GMT</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxPcGJsZkVRTHlkWUxkMzBiMnJFc29rbkUwVnJuOC1NUmg5SlRQTi1XTkszZ1I5czRQcXRLRUFwZWdCTlk2cDBkWTlBTW9FdVdQSTZueUtwZzRlLWJmOFc3U3NYeVl1ODFDSlNuaVRzakx6SW0wSDhHQ0VLbjBJNnFIYXFvNHp0UmZYb2hYOFQ4MENGcmZFZkZNR25nb0pEZ3E3aGc?oc=5</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>1</v>
+      </c>
+      <c r="G72" s="2" t="n">
+        <v>46016.98109953704</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>High Level City searches  France  English language</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>("Paris") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing"  OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Earnings Chart Overlay Points to Bafna Pharmaceuticals Limited Upside - Earnings Beat Highlights &amp; Free Rapid Return Acceleration - Bollywood Helpline</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 01:14:23 GMT</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPZ2VJRG40VUtCYVdSRkE0akxqTlBoVk5kZmhsZ21HNXJfUnBZendVNmdlWnBVY2NxLXlCMWgweUdYbEhObVl0OENlV0p1dEJNaVRZZUJFMmRpZDdUWWl5V201QUtxdjZVSllmVktFclZyVmowd2hoYWxaWVVZVFBkSkM1NDNJcTZKd3hXOVBKTVJNNXlmaFlMcG9xVDBtZnowMmVlTnYteWRMenhVRmNCOTZR?oc=5</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>1</v>
+      </c>
+      <c r="G73" s="2" t="n">
+        <v>46017.05165509259</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>High Level City searches  France  English language</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>("Paris") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing"  OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Is Sakuma Exports Limited Starting a New Uptrend - Retail Trading Trends &amp; Capitalize on Stocks with Explosive Potential - Bollywood Helpline</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 17:59:20 GMT</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOTFhmQ216UnppQV8zTlgyNkhRVm1Fd2ItdkZIYXUwZWd0ajUtV0NEb3VUdmlKU25PTkMzaEgyT2FwNkpnLWVlS0gtZkxBUWJrSWdlR0JBZ25mUW8yLXNNZzN2SS1uby1meU4wZkpKU2Nid0tqY2NEdldYNDA0TXMtT1JhbU9LMmFwZ2RNZzlFdl9STHdEaHc?oc=5</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>1</v>
+      </c>
+      <c r="G74" s="2" t="n">
+        <v>46016.74953703704</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>High Level City searches  France  English language</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>("Paris") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing"  OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Honeywell Automation India Limited (HONAUT) Announces Strategic Shift - Stock Liquidity Analysis &amp; High Yield Stock Picks - Bollywood Helpline</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 22:53:53 GMT</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOeUg0NUpqQ0NxQlNCVmhsV0lDR2pVNzVXdGoyRE52aGg3UnVTdkNFeVRjQlAta2duUW1adi1pb2tJNXhrX1BGa0s1U0NXdl9qWmpJOEdURE90UVFvYzVGb19WdVFWRmV0SFVLMlJDWFhaWE1oMlkxd2tlR0lkYjRBdU5iOTItTWdPc0NYWDlVbUM3czRmVV9wNXQ1UVQyMm40TTB4YjFPTDBsMkZtTGxUSnhaWXBWekZRLTgw?oc=5</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>1</v>
+      </c>
+      <c r="G75" s="2" t="n">
+        <v>46016.95408564815</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>High Level City searches  France  English language</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>("Paris") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing"  OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Pacific Industries Limited (523483) Expands into New Market - Volume Profile Analysis &amp; Interactive Charts for Smarter Trading - Bollywood Helpline</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 16:58:49 GMT</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxOMTg1YjRmdDg0alFIRG4tZ2JSeXhYbVlkellOWGxGVXZOMFF3UUFONE5aMlRRQzJjYVZkbXNNV1lleXdGeVdTM09DVGl4Q1dRenoxdElzbUdMbVdmcmJWVUU0TDlaRlJRcXZvcWlFaHhTMEd1bE9kbE4tYU05bG5iUEF3eTdRZXRoUHVrVm9QN3l4OUNZLVhaNjJUSTJKZVRQMGZTdHJ3WEdxbHgyVkE?oc=5</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>1</v>
+      </c>
+      <c r="G76" s="2" t="n">
+        <v>46016.70751157407</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>High Level City searches  France  English language</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>("Paris") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing"  OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Wyckoff Accumulation Phase Possible in Saboo Sodium Chloro Limited - Sector ETF Performance &amp; Rapid Portfolio Strategies - Bollywood Helpline</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 23:47:50 GMT</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxQQU8zR1g2Ulo1NWYxT1RJUnVjSm9BQ1NveFRMOG5LQ3hjd1FGNk1RRWotR25PbE84aDl2MUhZQjd1MUFCbXM0UGZIZzMxejRvcENMSC1VNTdiYldIUkVxWU9vWVFCMU8zZ2dCdU9WTWlUV0RkWDIyN3NCSXowTEZlOEVqa2oxUy1vbWlGRkhnd3VWVkdrbWt0WXFYTlJVOURvOTg0?oc=5</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>1</v>
+      </c>
+      <c r="G77" s="2" t="n">
+        <v>46016.99155092592</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>High Level City searches  France  English language</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>("Paris") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing"  OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>The Best Celebrity Memoirs To Add To Your TBR List -- Ranked By How Juicy They Are! - Perez Hilton</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 16:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiekFVX3lxTE1RTWZSYkdyNXk4LXN2OGRFOUpfdHFwQVJybWQ2eF9wTFB2TU85a1Y5UXdwV1pVcm1oQ1B0OENzMjlkbFpiVXpSTUczdC1lSldteE9rdU5lZWRjVnROVU1lQ0RxZVpVbnBYa3ZIdjFvVzFBYVVhZDlSY2ZR0gF_QVVfeXFMTnpDNVBXUHRFLWd0UlFjTW1ocmRzdkFkbFd2djlFVzdFRGlfeXNTLWFaQ1RERlJLa1JGYUZjZkNabVVENEFvX3hyVmxKVmdaVTYweHdwV2lfR2lBaG9hNUlvYmIyQ0ttc1djWjdPakk3SlpIOTk2UW1adHI2M0MyNA?oc=5</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>1</v>
+      </c>
+      <c r="G78" s="2" t="n">
+        <v>46016.66666666666</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>High Level City searches  France  English language</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>("Paris") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing"  OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Nanterre vs Paris – Preview &amp; Prediction (Dec. 26, 2025) - basketballsphere.com</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 15:35:34 GMT</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNSHF3cno1S19mNV9rMS1DUHVaRy1sNUhkSGp6YTNtZHhPaXMwWXpyNWNOMGlKOUhnZU81LWU3M192M3FVR2twbFFtYlNYMHg3RWdJb0RJdFlQTEtGcmhTZGtxVENVV3owNE81VmFzcGEzNkx4Zmg2M0ozRmRhMlZQZHJkZVhTazE2?oc=5</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>1</v>
+      </c>
+      <c r="G79" s="2" t="n">
+        <v>46016.64969907407</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>High Level City searches  France  French language</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>("Paris" ) AND ("Bombe" OR "alerte à la bombe" OR "explosion" OR "explosifs" OR "explosif" OR "explosive"  OR "colis sans surveillance"  OR "colis suspect" OR "tournage" OR "poignarder")</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Can Diligent Industries Limited (531153) Maintain Its Valuation - Market Correction Analysis &amp; Budget Friendly Growth - Bollywood Helpline</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 04:14:18 GMT</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQNUpGak5DNmRsd1EwYktSaWdQSjZyNEVIb1BUWVFDTTBBTzFlUHp0ekJKNURNU0ZiZk5BMVNETFBjSlR2WnZSOHpkMHJZVEVtZmhZTmxKTUhRY2hSeDdTR05hZ1h6RUFEaURveTVqMVZGYTRFN3lSTVVaMlItSWVCSkpkN0lRNnZhdjNsc0FyZ0N4ZzlzN0ItaDZGR0VpUS1Yc3BzZXNfZFZJZWVjTkRDWnVCRQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>1</v>
+      </c>
+      <c r="G80" s="2" t="n">
+        <v>46017.17659722222</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>High Level City searches  France  French language</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>("Paris" ) AND ("Bombe" OR "alerte à la bombe" OR "explosion" OR "explosifs" OR "explosif" OR "explosive"  OR "colis sans surveillance"  OR "colis suspect" OR "tournage" OR "poignarder")</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Can Traders Expect Breakout From IntraSoft Technologies Limited This Week - Dividend Reinvestment Plans &amp; Explosive Growth Opportunities - Bollywood Helpline</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 18:44:15 GMT</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNLUZac1dDajROVjZiaklmaXV4YVZTZ0RicXEwTW80U25Eb3V0OGJJVDF6ZWFSQVdkbXdNY1pkbmFvSXFvX2VYZC1iRU5oel9FLU9JTjdVMDNVbWVDMnJrYTJCdEh3SW9kVzdyYUNOTE90UFk1OVktOHBwckJPaEpYcXhDZlhKanhIRGtJc0JraGQxREdnMnRiM2hRYVhGNi1MMVFQSUpEVXg3MlNV?oc=5</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>1</v>
+      </c>
+      <c r="G81" s="2" t="n">
+        <v>46016.78072916667</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>High Level City searches  France  French language</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>("Paris" ) AND ("Bombe" OR "alerte à la bombe" OR "explosion" OR "explosifs" OR "explosif" OR "explosive"  OR "colis sans surveillance"  OR "colis suspect" OR "tournage" OR "poignarder")</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Oriental Hotels Limited (ORIENTHOT) vs yyy - Candlestick Trading Patterns &amp; Explosive Capital Gains - Bollywood Helpline</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 14:53:44 GMT</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxQSkM2NzBpWklnZVB2TF9CNXZfb3VxdTdTTWFBRUtnel9lTi12d0lvaUp5WVhTMDRMVlBoRldzOGh2VGgxLUhmM2l3dS1Ocl9STnlmX3MycXhlcjdGekpNZ2tSMzZpYTRfal8wbHRTTHJ0SjBNQ0Y4RDk0YXVidldncjk2M0Q3V1BmUjhlN2NB?oc=5</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>1</v>
+      </c>
+      <c r="G82" s="2" t="n">
+        <v>46016.62064814815</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>High Level City searches   Italy, English   language</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>("Milan" OR "Bologna") AND ("Bomb" OR "Bomb Threat" OR "explosion" OR "shooting" OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive")</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Not Antoine Semenyo: Top three Liverpool targets to replace Mohamed Salah - LiverpoolWorld</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 19:29:00 GMT</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxOdnZKNnUwejVEa1dzUHlWTlVFNkhvT1drTUVjSlB6dC1SNDNOYk9lelU1VUM0QXpETFlWc2stV1FCUWtiblVnYWhvRXdBa0tNWGVuSVZ6d2RvZVZLQ1JCbE5nak4tN3RCdnpnRlFmcUlGTFZ2MTVaWDVuYm5nMFpycTNudERYVXktbVRTek5RVVBWRm5FQk44dEg5OGI3eHl6V3QySTE1c0RDT0J6dzR6ZC1wMEVEdUU?oc=5</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>1</v>
+      </c>
+      <c r="G83" s="2" t="n">
+        <v>46016.81180555555</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>High Level City searches   Belgium Dutch language</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>("Brussels" OR "Maastricht" OR "Antwerp") AND (bomb OR explosion OR shooting OR stabbing OR police OR evacuation OR "suspicious package" OR "unattended package" OR protest OR riot)</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>From ports to streets: The spread of organised crime violence in Europe - belganewsagency.eu</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 06:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPVXNTdFRMcWtqeGp1NFItNXphNmQxZHlfdG4waHZYZlJ1SEEtZFMzQUdNTjlBUnAzcnhfYkhrZFJyMUtHM3IxZ1hZT3FaLWxxYklqQmdGRWhRQ1dIRzhUV3dNUlEwZ2tWZldMaG5pVk5zTmhLR2dkelhGNDVHM0R0UEFnUGxNRkUyejA5c1RkTVJpM1NYY1AxSTEtU09rRlpULUFZ?oc=5</t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>1</v>
+      </c>
+      <c r="G84" s="2" t="n">
+        <v>46017.25</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>High Level City searches   Belgium Dutch language</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>("Brussels" OR "Maastricht" OR "Antwerp") AND (bomb OR explosion OR shooting OR stabbing OR police OR evacuation OR "suspicious package" OR "unattended package" OR protest OR riot)</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Man shot by police in the centre of Bruges, leaving him critically injured - The Brussels Times</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 20:30:02 GMT</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQdmxGOW9IRkxJbUJielFaRHB0NWM2MkdRVzFsMjhYY1NyYzNWOVdwdlU1YXFBcy0tRllvVTRiZUFVbUlab1NhOHpJWFk5bTFnTENxVzBUcnpCWm9PcVNQOFVtbVFSRHJocUlCRXptY3lJV2Fla3F4b05aa0Y1bVltelBhNW9vRTBOY2dDTGZyWGQ1cGpEeFpiRmdwQUlKcWxmdmlTbC1oc2VPS1ZVb1k0bg?oc=5</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>1</v>
+      </c>
+      <c r="G85" s="2" t="n">
+        <v>46016.85418981482</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>High Level City searches   Belgium Dutch language</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>("Brussels" OR "Maastricht" OR "Antwerp") AND (bomb OR explosion OR shooting OR stabbing OR police OR evacuation OR "suspicious package" OR "unattended package" OR protest OR riot)</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Zelenskyy says he's open to creating demilitarized zone in Ukraine's industrial heartland - bastillepost.com</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Fri, 26 Dec 2025 00:25:55 GMT</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxNRWNITnBlRVg5N2IzWGlQUE1USTVGYU55TzdxZVp6VmhqaDdvMEgxTEdia3R6S3lkblZaYTVMSkctMXNKYzRjM2FRRU9ORnc3bUtlajlELV92OXRERHEzOUdITmRiWjVSb3RTM0FzbWtxZkhQeVFJelIyNVJCV1cyczBJT3BDblpWQ01yMnpxM0cyU3YzYm1XTkppREh2akpqZjV5ckh5NkdSa0RJNTVNd0FJWjJvcXhNSE5yNHVYRi04NENwdFpmbmI0bWlZV0dBTE5mYW13?oc=5</t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>1</v>
+      </c>
+      <c r="G86" s="2" t="n">
+        <v>46017.01799768519</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>High Level City searches   Belgium Dutch language</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>("Brussels" OR "Maastricht" OR "Antwerp") AND (bomb OR explosion OR shooting OR stabbing OR police OR evacuation OR "suspicious package" OR "unattended package" OR protest OR riot)</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Monika Kryemadhi: Brussels' number one condition, Edi Rama's departure - Balkanweb.com</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 17:20:25 GMT</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxPazNqYTJ1Y19EVFF2WDBZTmhNcGxMMmlFX0NLR0RkbWtKZVNzSWEwTmg5b1c4UVlEM0RLR1hCcTgxUTZELS11YWJ3UUdnNE5XZEFNUGNDQXI1SHdRdC1XTENpOFpJUXRTbnQ3ZEhxbThQdnZKRkI2d25oajhUR09MYzVaU1lMQ3VOUXlyU3p6b1R2NFhIZGllb3ZfOXRvQUZl?oc=5</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>1</v>
+      </c>
+      <c r="G87" s="2" t="n">
+        <v>46016.72251157407</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>High Level City searches   Belgium Dutch language</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>("Brussels" OR "Maastricht" OR "Antwerp") AND (bomb OR explosion OR shooting OR stabbing OR police OR evacuation OR "suspicious package" OR "unattended package" OR protest OR riot)</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>The European laws curbing big tech... and irking Trump - Kuwait Times</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 17:09:00 GMT</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxObm5VY2FYOHVDYWdERlFRRUduUk01LVVjUWljVVJHaVNnMllMNWFwQlpKZ2NUZUpUbmc2QnUxenk2YWRCby15U3pJVk1GemFTTV9UbmZlSkNBOURjaTh3STB2ME5DanFTVGptNmJMcVBFc1FxOElLSXVjbEpDRDNZX1kyMzcxX25WVWhqbXpTTkNrY2o5Q2ZlS0NpT185QnBSdWx0X9IBpAFBVV95cUxObm5VY2FYOHVDYWdERlFRRUduUk01LVVjUWljVVJHaVNnMllMNWFwQlpKZ2NUZUpUbmc2QnUxenk2YWRCby15U3pJVk1GemFTTV9UbmZlSkNBOURjaTh3STB2ME5DanFTVGptNmJMcVBFc1FxOElLSXVjbEpDRDNZX1kyMzcxX25WVWhqbXpTTkNrY2o5Q2ZlS0NpT185QnBSdWx0Xw?oc=5</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>1</v>
+      </c>
+      <c r="G88" s="2" t="n">
+        <v>46016.71458333333</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>High Level City searches   Belgium Dutch language</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>("Brussels" OR "Maastricht" OR "Antwerp") AND (bomb OR explosion OR shooting OR stabbing OR police OR evacuation OR "suspicious package" OR "unattended package" OR protest OR riot)</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>How the Art Nouveau soul of Brussels was saved - The Brussels Times</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 14:34:23 GMT</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPeFFrVVFBNTZseVpvc0VhSmQxRllRUHJsckNFRGpJZ3FYd01NaWY0Mm9Kd2VnbU43SmNvV2FvUVZYMEJ3QmQwLXdEdGR0VWVIUzR4ejZLalM0aTIycVFUQzhxYTJkUm9aOHBwUWVWNXBNLXViaG5iMVVLanRXQ1gxVnFhSFpWQ3QtT3NPcE1aRDhyU2l4YzU4?oc=5</t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>1</v>
+      </c>
+      <c r="G89" s="2" t="n">
+        <v>46016.60721064815</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Local Town Searches  Maasmechelen Dutch Terms</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (bomb OR explosion OR shooting OR stabbing OR police OR evacuation OR "suspicious package" OR "unattended package" OR protest OR boycott)</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Two men killed in separate Christmas Eve crashes in Zwartsluis and Maasdijk - NL Times</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 15:25:00 GMT</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxOaWY4cEhRaXBQNDhkTnlyMExXNXRScTNfZWtBelFTVGRvY2trMkJiay1ZcDRGejh5di1MdjR5WWhKdENvdmRYdzNsbmtHVVY3TGc3MGtuVlY0bTVobGduUVIyOVhYT1hvUjhCbmxzWWtRUHlWRGV6WWpXaWtqaXlHMjZUQXQzYUhrSTRuanRqYTdVY0hhY2c1QnV5Zw?oc=5</t>
+        </is>
+      </c>
+      <c r="F90" t="n">
+        <v>1</v>
+      </c>
+      <c r="G90" s="2" t="n">
+        <v>46016.64236111111</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Local Town Searches Wertheim German Terms</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Wurzburg" OR "Aschaffenburg") AND (bomb OR explosion OR shooting OR stabbing OR police OR evacuation OR "suspicious package" OR "unattended package" OR protest OR boycott)</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Wurzburg vs Trier – Preview &amp; Prediction (Dec. 26, 2025) - basketballsphere.com</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Thu, 25 Dec 2025 15:37:24 GMT</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxOVFd3SVlmbXRxeUpUdHVKc1FHdlZ3S3lzTEpSOU9Rc2preGs4MkdGQll2Nmk2ZFd6dGVVb1FNRzFlMmR3cmlyLWt1RFBFNDZ2XzRtQ2sxbWIycTFuU0JGbThpQ3diX1UxelNVTlByYXlEdlEtYThPYXFqbGJhUFNkTnBKcXV3a1Ri?oc=5</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>1</v>
+      </c>
+      <c r="G91" s="2" t="n">
+        <v>46016.65097222223</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-02-21 07:41 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K48"/>
+  <dimension ref="A1:K56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -590,32 +590,32 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Shoplifting UK</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>("shoplifting" OR "retail theft" OR "retail crime" OR "shop theft" OR "pickpocket") AND ("UK" OR "England" OR "Britain") AND ("gang" OR "organised" OR "trend" OR "rise" OR "survey" OR "report")</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>New survey names Doncaster as UK shoplifting hot spot - Doncaster Free Press</t>
+          <t>Steinhoff's Business Report: Adapting to Market Challenges - Studocu</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>New survey names Doncaster as UK shoplifting hot spot - Doncaster Free Press</t>
+          <t>Steinhoff's Business Report: Adapting to Market Challenges - Studocu</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 11:06:00 GMT</t>
+          <t>Fri, 20 Feb 2026 20:16:22 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxOa2ZMT1lMellVa1p4RDRyR0xhZnVzVjN2cE5RSjU4emY1ZzdyUVRoZDJJc0xkb2Z0MTFhZXpPdi1mS0hIN0prdTNoa2ZIcWpPVEljY1h4VWJyUVduUjk0ai13OW9iNEwteGptQVQ0V1hGRjV5eC0zMnAtMHFUbGxCeEw0MWxjLUJCczFFMklXaHp0M2pBZnI4ZWw5QjBRbFBjNXIyMVM2VlZaSm5MVUE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxOczUwYXFCX3dNZk9ZLUpWQjN0b2hTaDA1V0QwWjFIV2RmdUpmV1gzbmdJU1Q2OE9xNGduSDFpbEFQcG81bklHZGVXRTR4Mk5oUnRNRVlXM2VWSjFNZmUxRElUYVI0U3ZraTFBd05BX3BKMDZLaXl6aFBpSFVXWHFvVHpVdUY4ektSbkpsQkZManl4dXFJSFRIbXpPU1gxNjRQbF9mUHlDbEVoZzVtcUJ0cHZMejVITTZjN2F0RnFENWptMUJRajBOa3hxTE5lbFJPQW9GeHRXUTFPS2J6WUJVX2tBWXNOYS1xSGJ6N0VZb2lmc3NPVlNj?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -639,38 +639,38 @@
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46073.4625</v>
+        <v>46073.84469907408</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Politie opgeroepen voor schietpartij in Sint-Jans-Molenbeek - Nieuwsblad</t>
+          <t>GUNPOINT ROBBERY: Rs 12 Cr Gold Looted After Employees Tied Up in Assam’s Barpeta Road - NorthEast India24</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Police called for shooting in Sint-Jans-Molenbeek - Nieuwsblad</t>
+          <t>GUNPOINT ROBBERY: Rs 12 Cr Gold Looted After Employees Tied Up in Assam’s Barpeta Road - NorthEast India24</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 15:28:55 GMT</t>
+          <t>Fri, 20 Feb 2026 15:46:38 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOZ05fQW93OTZLWm51TDhlYXQ3WURtbDRNY1JXdjBQYWlQazRmZXF4SGtKUzBFbmRvQ2Z5c3E4S3d4TG54S3VyZ3FJZ0JBdVJIaXd6Y0kxY3BtV21tUjdmeW90X3hHcVhpcGZaMGl5VGhzdFFDRm82SnZSdUw2cy11QXpUYnB6Zl9mWkxsdHpJTVNHdGluMHRYUnd0bFRFRTR4ZnF6NjZkcHNValU3UEFSZVMyU0c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNZEE3cFZDZTF0aWNaOUc5WTFMUzRHcVUzNXJEbE1GdFE0S1hkUndPTnpGU19KNzdGZUZRWXpIOU1nclRkNDNGQ2VUVUpoQ1hjWmlibVdKeXIzQzljdnBzY1pHcWlWaVRVVHJLdHd3eHNOeHIzT0NTMG9KVjV0OUZaMGh0UmxLelVjWDhxN29CWWtfN0wzbjVfUFBKNlNLOERiSkw0UDVDdldVWjg5eUg1ZVI1Uks?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -680,52 +680,52 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46073.64508101852</v>
+        <v>46073.65738425926</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>"Overwinning voor alle overlevenden": familie Epstein-slachtoffer Virginia Giuffre reageert op arrestatie Andrew - VRT</t>
+          <t>The Best Hotels, Restaurants and Shops to Visit in the Cotswolds — the Hamptons of London - The Hollywood Reporter</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>"Victory for all survivors": Epstein victim Virginia Giuffre's family responds to Andrew's arrest - VRT</t>
+          <t>The Best Hotels, Restaurants and Shops to Visit in the Cotswolds — the Hamptons of London - The Hollywood Reporter</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 11:01:01 GMT</t>
+          <t>Sat, 21 Feb 2026 02:13:23 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxNMFBjUkoxZldtaEhqbmpmc0oyWlEteF95WWFIX1RmcEtqVi1mTXhsbmpBMVlNZUFaamo0N0NEbTRKZjMxdXFaeEk4Q2pCOWVsM2tOc21oTU5hejB2SkJHeGlBZnY5d2M3WURCWU4yTVFPcTRYcE02al9HSXVsRjhabWhpc1FOb0RmUUU2SWVudmg2NkFseVJjRzJ0a2RleFF5LThtQnU3MGwxazRwOXZB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxNMVBPdmNZZ3ByY0FYNVpyck1fS0NKT3pmN19mTTBjMGFOcy1adlpnZmVRYWVtU05kYndYMkpvNk9SOEluanVEZTYxRnNaeFVyQy1DemtLNGtKTFRSYVdYZ1VJdUx0NlBUVXY1UWtpSllTSE9QVUVYMWppLUlyZ0hTdzZ0UGFjOHRsZXBZSk5ReDM5UktWVHJGaWl0SjdxbS1Kc21qeU42azAzSVV1d1NEQTR4TVZKbDk3bzJBZllFX2c?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -735,52 +735,52 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46073.45903935185</v>
+        <v>46074.09262731481</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Shoplifting UK</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("shoplifting" OR "retail theft" OR "retail crime" OR "shop theft" OR "pickpocket") AND ("UK" OR "England" OR "Britain") AND ("gang" OR "organised" OR "trend" OR "rise" OR "survey" OR "report")</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Scooterrijder gooit zwaar vuurwerk onder de auto van Frans Theunisz: ‘Geen idee uit welke hoek dit komt’ - De Limburger</t>
+          <t>New survey names Doncaster as UK shoplifting hot spot - Doncaster Free Press</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Scooter rider throws heavy fireworks under Frans Theunisz's car: 'No idea where this came from' - De Limburger</t>
+          <t>New survey names Doncaster as UK shoplifting hot spot - Doncaster Free Press</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 12:07:28 GMT</t>
+          <t>Fri, 20 Feb 2026 11:06:00 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi7wFBVV95cUxPVTRGc1VJNk9UQlZVenZuamd1aG1CakdYQVZrb1FjUzJLazRiUFNtTFdtVjUwT0tlZnQzWUlZQnBVRUdabkE1WEpXb1pldzhjbV9JTGlmMzJ3ZHczYTFZNnJIUGJWVUIxOW9xOFJIaFNxQUFtNm9FbjZXeFRVLXgxUlMzSHRkNlBacnY2cUF0b3c3NFNwSjF4RFF4SWhLWE96VGtjTExYbUFvcEJHTzlvSzU4Yi1UWDVnUTd4aE0xZk9lSnVJd3hFZldkV3pBRnZkZTI5SjNaWjRWYTFzT1VpaFh0ZWZHSXV0MGE4QUNXQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxOa2ZMT1lMellVa1p4RDRyR0xhZnVzVjN2cE5RSjU4emY1ZzdyUVRoZDJJc0xkb2Z0MTFhZXpPdi1mS0hIN0prdTNoa2ZIcWpPVEljY1h4VWJyUVduUjk0ai13OW9iNEwteGptQVQ0V1hGRjV5eC0zMnAtMHFUbGxCeEw0MWxjLUJCczFFMklXaHp0M2pBZnI4ZWw5QjBRbFBjNXIyMVM2VlZaSm5MVUE?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -790,21 +790,21 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46073.50518518518</v>
+        <v>46073.4625</v>
       </c>
     </row>
     <row r="8">
@@ -820,22 +820,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Importverbod op Russische olie per schip vertraagd - Nieuwsblad Transport</t>
+          <t>Politie opgeroepen voor schietpartij in Sint-Jans-Molenbeek - Nieuwsblad</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Import ban on Russian oil by ship delayed - Nieuwsblad Transport</t>
+          <t>Police called for shooting in Sint-Jans-Molenbeek - Nieuwsblad</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 11:18:17 GMT</t>
+          <t>Fri, 20 Feb 2026 15:28:55 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxNZTVMSVdIUDhqZUVobFVoZ1pLdUJiVGlSRjhBSGcxSmdWWDJwZGdxOFdNeGpMZW1TVGllc1RfV2YyUnZaRzdyMEVDMkpaUW9GT1pvTkFpZUJwQ0JZVzRpS1pNdUJtd291dmMyMGZtTjNjLURzM0tkY2dfTEZ6YVFHbXBiZzY4WXk1V3dubF8zcTRYX0Vpbnkw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOZ05fQW93OTZLWm51TDhlYXQ3WURtbDRNY1JXdjBQYWlQazRmZXF4SGtKUzBFbmRvQ2Z5c3E4S3d4TG54S3VyZ3FJZ0JBdVJIaXd6Y0kxY3BtV21tUjdmeW90X3hHcVhpcGZaMGl5VGhzdFFDRm82SnZSdUw2cy11QXpUYnB6Zl9mWkxsdHpJTVNHdGluMHRYUnd0bFRFRTR4ZnF6NjZkcHNValU3UEFSZVMyU0c?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46073.47103009259</v>
+        <v>46073.64508101852</v>
       </c>
     </row>
     <row r="9">
@@ -875,22 +875,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Explosie bij bedrijfspand in Helmond: harde knal en veel schade - AD.nl</t>
+          <t>Cokeconflict tussen Bolle Jos en zijn oude rechterhand: ‘Heb zware materiaal daar, die overleven dit niet’ - AD.nl</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Explosion at business premises in Helmond: loud bang and a lot of damage - AD.nl</t>
+          <t>Coke conflict between Bolle Jos and his old right hand: 'I have heavy equipment there, they won't survive this' - AD.nl</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 09:42:00 GMT</t>
+          <t>Sat, 21 Feb 2026 06:22:00 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQdEN1aWVLUmtRb0wzcjNGWVhGT1pWQjU5eC1qX0dRUHhWTUV0dHAxaUlQb1ZEZ3AwSDFOSkJHUHdJQW9hR0lleFZ5QXY1b1JnOFFCQ1Rud0FNRjhFVUQxajJtSkNONHNvazlkeHNBbEpVM2VFbXgyYlhyZWc2Y2J5dWg4YTVlWDJBRUIwNnQzcTlrQmViYlIyb0I5Y180R2s?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxNYjA1ZTJNUHhLM1QwVXg2V2czM21tOFZFUGR3V0Y5bW9mQldYMEZCZHJfV2pXd0g0OUliTW9xcVU3cmVHN1g2Q2dieWVJd2tubG5HZEFxeUhONWwxYWgtX3R4R1loSmI3TXhPYmJBbV9FZzVGS2ZyVzZOZHQ0VDZWS1FTNUlGUm5YaXdjaUVGS01Tb09jWlplN1BtaVluN0dFVzh1bFkzZllXX0pfRzFOeHJCRmFBS19YckFPaEF2VFpPWjQ0bWN5VERUbTBNS0NhbHhmSFZuYTg?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -914,38 +914,38 @@
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46073.40416666667</v>
+        <v>46074.26527777778</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Turkey arrests European activists probing prison conditions - The Straits Times</t>
+          <t>Scooterrijder gooit zwaar vuurwerk onder de auto van Frans Theunisz: ‘Geen idee uit welke hoek dit komt’ - De Limburger</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Turkey arrests European activists probing prison conditions - The Straits Times</t>
+          <t>Scooter rider throws heavy fireworks under Frans Theunisz's car: 'No idea where this came from' - De Limburger</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 10:04:47 GMT</t>
+          <t>Fri, 20 Feb 2026 12:07:28 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOcVV3cGgtM0t5Nm5XbTFJbGR2N0Q1RHRhVmJ3VnJFTGhiUVN5bFJpWUUyNUxVLVEwVjF1elZ4WXdIVUVVWXVmcm1nelZXYV9FcEVBS3ZPeU92aDlmRko2eWI3WjZqRWxUeTlteVVvVDM3Y2ZlbkJWT2QtWFJNQ0paNUJDOTh2b1JaZVdOSVdsVndLbXVUNU0tTlBTUUdKUFF5TVdF?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7wFBVV95cUxPVTRGc1VJNk9UQlZVenZuamd1aG1CakdYQVZrb1FjUzJLazRiUFNtTFdtVjUwT0tlZnQzWUlZQnBVRUdabkE1WEpXb1pldzhjbV9JTGlmMzJ3ZHczYTFZNnJIUGJWVUIxOW9xOFJIaFNxQUFtNm9FbjZXeFRVLXgxUlMzSHRkNlBacnY2cUF0b3c3NFNwSjF4RFF4SWhLWE96VGtjTExYbUFvcEJHTzlvSzU4Yi1UWDVnUTd4aE0xZk9lSnVJd3hFZldkV3pBRnZkZTI5SjNaWjRWYTFzT1VpaFh0ZWZHSXV0MGE4QUNXQQ?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -955,7 +955,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -965,42 +965,42 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46073.41998842593</v>
+        <v>46073.50518518518</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>The student who was injured in the "Gjuta" hotel, the fiancée of a police officer, the lawyer, BLOWS the bomb: She lied to the boy about her age and origin! - Vox News Albania</t>
+          <t>Gheysens schiet uit krammen: bom ontploft bij Antwerp - VoetbalNieuws.be</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>The student who was injured in the "Gjuta" hotel, the fiancée of a police officer, the lawyer, BLOWS the bomb: She lied to the boy about her age and origin! - Vox News Albania</t>
+          <t>Gheysens shoots out of jams: bomb explodes near Antwerp - VoetbalNieuws.be</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 12:57:47 GMT</t>
+          <t>Fri, 20 Feb 2026 16:41:00 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQNkdQYmNiZjFHS0pDdmR0MEJkMkQxcGZRUlJZVzJPeEJBY1VoZWNabWN3NFdZM25Qb01iaWVVSVNyUlZUUXc3QmdPN2RvWFFkdlhDZU1rRjdRUF9kRV8xTy0xOE03SmhHUmdyLWdyclJaQXBEYUFlNl95eXR5Vy1WUmFHaHVDSlpNVUdwUnlSUWtKbl8xMU5wLWs5Q2V0bUhCdVBhaHBMR21JdlowUTNNVU4wNzh1Wk5ORjIw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxPdkR3UDd5RHNTR1VOVWVBdl9lV3ZLTVpnYThkWFcwWFVtQmFrVzhFcUhCZDN0dnhTTWtPcHV2UjdOY2ZFZnZRVjd6MGxEdE90dnBaSWg4MDlkZENVeEVUT2lsZUNRMDZUTVZnM2Q3ZTdIZ0tsYmtEV1J1OEttbWN3OVR3ZU1fOUhRdlhiVERWZmZsSUoxeVFBTQ?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1020,42 +1020,42 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46073.54012731482</v>
+        <v>46073.69513888889</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Un Belge détenu en France pour agression sexuelle sur un garçon de 13 ans extradé vers la Belgique - 7sur7.be</t>
+          <t>“Nu zweet hij wél”: dit schrijven Britse kranten over de arrestatie van ex-prins Andrew - Nieuwsblad</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Belgian detained in France for sexual assault on 13-year-old boy extradited to Belgium - 7sur7.be</t>
+          <t>“Now he is sweating”: this is what British newspapers write about the arrest of ex-Prince Andrew - Nieuwsblad</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 15:35:00 GMT</t>
+          <t>Fri, 20 Feb 2026 16:56:00 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxNWF9veDBvVHRlMy1ESVJ4MTFVUTJzSm5FeXB4RUExV01BaE9PaEdjMElYRE5wb2NlVFJsclV1U1A0R3BjN0pqb1NWeDI5T0IyNWFqV0VUZDhtZjZRSFMySXdoSDdHZEluMXA0bWp2MXZCVFkxUDc2Y2l4UWxRZDZybmU3YjRXdXN0MTNkTkxGQ3hweXJDV1JhdUhpM3lQNldib1RuajFPMjRualdMSlpRMC1DWWxQYkFFNU5CYXpNbzZrdnRCam1fN0U3ZEFzdGo2a2VhTjZrWEZNZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxOSzlCYWpUcFVINmw3bDNOWVNqUTVmV2ZrVjd4c2VFdHFSbTBVNWhtMWJwU2RFN25OSXlwNG1RZERoczdNLXFwWmpmd24yVDBnSk9PR3BZb2VCMFBDYUJlcWk5R2dGaHZMeTA4R184MjJrUk5ELWI1U2tVc2oxUnUwMFFSMGxzYU8yRl9mUDNNRXktVG40V0dtSFNjVUdqMDFYUEljd29yekcxRUZET0hLNDdQNDhkRUpUSkdRWDJiR2x2ei1PWWFLd0hTaFJDVGxwMnc?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1075,42 +1075,42 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46073.64930555555</v>
+        <v>46073.70555555556</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Des adolescents forcés à monter en voiture et dépouillés en périphérie bruxelloise : le véhicule retrouvé à Molenbeek - BruxellesToday</t>
+          <t>Importverbod op Russische olie per schip vertraagd - Nieuwsblad Transport</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Teenagers forced into a car and robbed on the outskirts of Brussels: the vehicle found in Molenbeek - BruxellesToday</t>
+          <t>Import ban on Russian oil by ship delayed - Nieuwsblad Transport</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 11:18:00 GMT</t>
+          <t>Fri, 20 Feb 2026 11:18:17 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNa1czMENlV0VNOUxwc3VuaXpucVNSdy1DYnM2WjZZNm9KN2MwVG1pWnBIRUVJc0ZJbThrVzVQVlBLejl0RDZ1RmZDVzdtcTBBYV9MQ2JPdFV2RElUbVpqQ2xCSmkyMjRMcGNQUHZtUl9HWWVMcDJtRTZSNnJFSHVGUWRMbG9QZnE5Nm4wWXBxNnpkZzlmODhmanNkUXZfM2Qw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxNZTVMSVdIUDhqZUVobFVoZ1pLdUJiVGlSRjhBSGcxSmdWWDJwZGdxOFdNeGpMZW1TVGllc1RfV2YyUnZaRzdyMEVDMkpaUW9GT1pvTkFpZUJwQ0JZVzRpS1pNdUJtd291dmMyMGZtTjNjLURzM0tkY2dfTEZ6YVFHbXBiZzY4WXk1V3dubF8zcTRYX0Vpbnkw?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1130,42 +1130,42 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46073.47083333333</v>
+        <v>46073.47103009259</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>#FrigoVide : les associations dénoncent l’explosion de la précarité alimentaire - tvcom.be</t>
+          <t>OpenAI overwoog Canadese politie te waarschuwen over latere schoolschutter maar greep toen niet in - Nieuwsblad</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>#FrigoVide: associations denounce the explosion of food insecurity - tvcom.be</t>
+          <t>OpenAI considered alerting Canadian police about later school shooter but did not intervene - Nieuwsblad</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 15:39:26 GMT</t>
+          <t>Sat, 21 Feb 2026 05:05:33 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOUWpKRFpFYlQ5ZTd6NFJfQXZlRnZhMVo0ZlFDMExaQkRldUEweDFNSWd2eFdBMDB1TGlzYk93MFRQR0ZJWVZsQ19yak04UmZlZFMwWDMyUllJUVB5d2R1WTJQT3dQS2NOMTN4TC1DeTMwM3FxWEFuQ09aeE5STWpiSGpUZmVtbzJILWx2aWFaZ3UtejV0cnRRUXRMdVFsYUJ1dGNuSWV3LVZyODg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxOeGxqcjFnVEVUeUFyRUFVWkhOb2Z3RE1OcExMR2tXeG9yNXJYVERveGpwSmZTNjBqRmdoVGFBZGR0YWtIenFuaWtZUC1qYzc2WHhMdjM1RXlFRDU1NUNRaldpd256TEN5YmVacmFPSlNXTThoenBadG5qUEZaakJ0cnZycmwzRXpBeTJxYzYtOFJHUF9sOXhENmFLRGM2cjFjTXJSLU9yVVUxa2ZlcEI3OWpvSzZhMHhlbWtWRkw3dmNtUmdCNzItaTVKTW5TUkZ4V3VjT2lBeXduajkwbE1WWk1sMHQ?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1185,42 +1185,42 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46073.65238425926</v>
+        <v>46074.2121875</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Un député québécois agressé à Bruxelles: “Triste que les villes européennes en soient rendues là” - 7sur7.be</t>
+          <t>Shots fired near metro station in Molenbeek - The Brussels Times</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>A Quebec MP attacked in Brussels: “Sad that European cities have reached this point” - 7sur7.be</t>
+          <t>Shots fired near metro station in Molenbeek - The Brussels Times</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 12:56:00 GMT</t>
+          <t>Sat, 21 Feb 2026 01:07:30 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxPeDFBWkdGenBYUkpaZXpzNVB4RzZJemNrTFlwbnpiUzRta0VpcjJUdGhhd0NuMWJjb25ZTFZBZGZhQ2c1VTQzNDVoVzhQYW84Z2k1cFY4R1FGWEpSSkxxQzdXQ2xaWU1Yajh0aG15TEtpLUpMVHRHUXdUd2d4eTZrWHdOZXpNNjJVMHFhV0t4ckdrR2dvOEJFY1RXR044d2ZYODhRYkpOUEJSQWxsTDdQejVaUkwxZFQ1aDNzUkNDaTBsczY1bUREbDNEQmpHMlFEUUZvRlpB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxPV0o2UTVpdFBzMTU3TFJPNjFCRGVickVXbG5EUW5haVlrWkJHLXNGcXpjSUJnek8wTkIxWVpFZ1gxcXRvM2doRHBBTFJOY2FSWGRwZFVCWnFzTHBiMk1BQVdVR0dkYVpQaTlBVEdmc042MW4wUTNVNnJEZ0JKdHc4MzFkM3dHTTVp?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1240,42 +1240,42 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46073.53888888889</v>
+        <v>46074.046875</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Un cycliste perd la vie après avoir été percuté par un camion à Kuurne - 7sur7.be</t>
+          <t>Turkey arrests European activists probing prison conditions - The Straits Times</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Cyclist dies after being hit by truck in Kuurne - 7sur7.be</t>
+          <t>Turkey arrests European activists probing prison conditions - The Straits Times</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 14:16:00 GMT</t>
+          <t>Fri, 20 Feb 2026 22:07:18 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxPRFNoR2lJX2FBOEFZcnlvN1NYTFgxemZoTG5KWVJETkdmb3kyY2FuUUlGQktvMXAtUlMyWGNHZWZ6RDc4WHY0REhVMTlHdnpzWHpMdUY3VmUyZUNibXVDTnl3S3ZscVZxQjhKTGpvWHFSNDlEUUIwM19lVk5hVm1BY2RMSHlhbFZDTVNoZDFjQ1hqZ3hnYlNSbU1vMjVWNlVnQ2ZoRGxWTlpZOUdYemV4SkhJQXI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOcVV3cGgtM0t5Nm5XbTFJbGR2N0Q1RHRhVmJ3VnJFTGhiUVN5bFJpWUUyNUxVLVEwVjF1elZ4WXdIVUVVWXVmcm1nelZXYV9FcEVBS3ZPeU92aDlmRko2eWI3WjZqRWxUeTlteVVvVDM3Y2ZlbkJWT2QtWFJNQ0paNUJDOTh2b1JaZVdOSVdsVndLbXVUNU0tTlBTUUdKUFF5TVdF?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1295,42 +1295,42 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46073.59444444445</v>
+        <v>46073.92173611111</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>TC Hasselt - Sept ans de prison pour des violences sexuelles sur ses deux belles-petites-filles - DHnet</t>
+          <t>Germany, partners prepare to send Ukraine additional PAC-3 interceptors - The New Voice of Ukraine</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>TC Hasselt - Seven years in prison for sexual violence against his two step-granddaughters - DHnet</t>
+          <t>Germany, partners prepare to send Ukraine additional PAC-3 interceptors - The New Voice of Ukraine</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 09:55:00 GMT</t>
+          <t>Fri, 20 Feb 2026 19:06:00 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxQaHF5Vnl2YUlleldpV0kzTDJZZEtSM2ZJT3pOaWw0aVFxUFpiTGxJaXQ4ajlNSFlibDllVUpHeWhCcnY1WE9DbEdsMzhWb1VXTVJ0MkVBTFZ1NVpONXczUjd2ellXSlRGRWsySFNjdmt4Q1VTU1NPcWVfOG81WEtJcjhlUjFBcDVXSWl5alNXbHlCSjFMeVZUNFZiNFNJamZCS2pVLUt6UVppblVVUjhLeUFfbV9CSUY3OUVrQllHcFRrZDlmVEI4UEpXZWhoYzcxbURqZVR0RnBuenVnb2xhbmVYX2k5QXRnVXRUaUotYjBjWTItZzBxQmNxM3NjRUdaLUE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxPa2d1RGR3b2xkU3UxYzRoWmNmTGpOTWpaajBwUDQ3UlFrdFVVckhYZ1JncEgyLTB1bXU4MjA0STF6TFE0VmZ2ZDhycG03d250VVdtTWJJQlFHcWJpN1ktTDJKWlJEWWVtZWRrSHBfNGtEMC0zdW05c0diTUxrVjBUcjB3WHA1TDY1S2hCSExJX3Jma19YRi16ctIBlAFBVV95cUxQLTZEZTJzSzNuc3dqcHJGbDZYVnNYWWxSdG1QLXB3TV94ZkxBSWdFaVdzYlUzYXUwOWItYmhsSXJ4RmtqS3dEdXFSQU1PaEFLRkxLV2I5N0IyRGQyVUVLQi0wUW4zUU5OX29nV3k3NHdSNGVma3o1TXBsTjFuV2V1ckdmUkRqR2dCNDdYejViSExpdzM4?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1350,42 +1350,42 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46073.41319444445</v>
+        <v>46073.79583333333</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>French PM says government intends to criminalize calls for any country’s destruction - The Times of Israel</t>
+          <t>Several Belgian teenagers abducted and robbed at knifepoint in stolen car - The Brussels Times</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>French PM says government intends to criminalize calls for any country’s destruction - The Times of Israel</t>
+          <t>Several Belgian teenagers abducted and robbed at knifepoint in stolen car - The Brussels Times</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 09:57:21 GMT</t>
+          <t>Fri, 20 Feb 2026 12:14:33 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPdHVVcjRxOUM5a2JxNUlFUjNPdG5iTTc2UDk1cFU1c1ZCd1ltODY4blN2UTdXcGYwN3ZSWXZyV3pFMXZTZWlRemlhTmVib2EtMmhlVHd2RGdNaWlvMmQ2clpBWUYyakE2R09aR1F6Mnk1MHNqV0FsVjlUWmZyWkJuVG03NmstTmIzVmxfQlZkdnNVZmR3N0JabFR3Z1ptOEtRQ1ROQ3huWlZuOHZFV21NeFRyWkVhMmxvOUVhTzdFZ2xJN0xYU0piZA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPNkJQRzUtRTNwSkt5RmdyUEZaUV9jOXhLTERWY2xUOXBZTlBQWDZjY0tTY2lOS1oyTFlKWEU4aFdjaXl1aVdDckxTVGRUWVdIaXJjN2NiQzlJU2xXenZlenY5UWtESllJNF9JSmNKRENMc0RvdzJVSHVzWFF3WVFiUVgtWFQ1MnR5cGktanRmRnhtVE1HcnFwV0htWERTZjMtTmI3cWp4aTg0ckxYVTNvWg?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1400,47 +1400,47 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46073.41482638889</v>
+        <v>46073.51010416666</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Hundreds of Belgians locked up in foreign prisons - The Brussels Times</t>
+          <t>The student who was injured in the "Gjuta" hotel, the fiancée of a police officer, the lawyer, BLOWS the bomb: She lied to the boy about her age and origin! - Vox News Albania</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Hundreds of Belgians locked up in foreign prisons - The Brussels Times</t>
+          <t>The student who was injured in the "Gjuta" hotel, the fiancée of a police officer, the lawyer, BLOWS the bomb: She lied to the boy about her age and origin! - Vox News Albania</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 12:13:13 GMT</t>
+          <t>Fri, 20 Feb 2026 12:57:47 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOM1dqd09VU1RVSjFaYnlfVzlYRmUzc0lWZXN0TVRmZDdOdmJzaTE5TmRxQ1VncHpGM3BJSFItLTVTSktKNDRjdFJEMVVsNHBtbUo1R1J3eFJhdnRhR05RMHk5MExTdGNENnROZ1g2NXREUFZjNU1pWFBEUE9zS3dlckYzSFdSbVhqa3lDTUNFZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQNkdQYmNiZjFHS0pDdmR0MEJkMkQxcGZRUlJZVzJPeEJBY1VoZWNabWN3NFdZM25Qb01iaWVVSVNyUlZUUXc3QmdPN2RvWFFkdlhDZU1rRjdRUF9kRV8xTy0xOE03SmhHUmdyLWdyclJaQXBEYUFlNl95eXR5Vy1WUmFHaHVDSlpNVUdwUnlSUWtKbl8xMU5wLWs5Q2V0bUhCdVBhaHBMR21JdlowUTNNVU4wNzh1Wk5ORjIw?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1455,47 +1455,47 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46073.50917824074</v>
+        <v>46073.54012731482</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Wertheim: 48 junge Beamte zu Polizeiobermeistern ernannt - Fränkische Nachrichten</t>
+          <t>Fusillade à proximité de la station Étangs Noirs - BruxellesToday</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Wertheim: 48 young officers appointed police chiefs - Fränkische Nachrichten</t>
+          <t>Shooting near Étangs Noirs station - BruxellesToday</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 11:00:00 GMT</t>
+          <t>Fri, 20 Feb 2026 15:34:29 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxOVmx1X1F5RFNnSlRmakZ1d2dxcmtYcnJQWFdSeVlKWVBCMzE0Y3d6b1VSVTRPN1l5LWZPa2NGX25Gb0ktUEVxaEFnYkpHc1pTTHl3WTkxMHhrRlVnazRPcE9JcE1OaExlRHhEZ2ZRYkN4TWRSakg5VFdodHAwV0pRSHI2TlRLU1dXZjNXVDVEVDNULXI3amZuX0FLVEFCTWVDX05VTG16bE1WYWtkRVBoVXFkbUxmYjdzSlhTMEhsRzBKTDBFTGc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxObV9GWTNXT0pnV2VZLW5zUGFTUDZ5UjEwaXlFZ2N6V2g4a2tLMjVyUGdXeXZRWmFwVURCYTJ1bnR2bnZVcEZTRHVmMmtoR2ZSaDFjcGVPWnRSLVFkQUpPTU82ZGx4MTBBWFR6elU3MTV6RXhyazI0ckdFXzJyQlNJS0RVOEU?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1505,52 +1505,52 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46073.45833333334</v>
+        <v>46073.64894675926</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+          <t>Un Belge détenu en France pour agression sexuelle sur un garçon de 13 ans extradé vers la Belgique - 7sur7.be</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+          <t>Belgian detained in France for sexual assault on 13-year-old boy extradited to Belgium - 7sur7.be</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 12:52:05 GMT</t>
+          <t>Fri, 20 Feb 2026 15:35:00 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE03RUZJdVVWTG5jTlA1R0dmc2YyQ3Z2S1ExYmhkN0FENFJGamUwenJsSFFPWGpKc3B2aFBaeHRYVDR3aWM1SXg0YWZFVDk0N3d4a0Jz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxNWF9veDBvVHRlMy1ESVJ4MTFVUTJzSm5FeXB4RUExV01BaE9PaEdjMElYRE5wb2NlVFJsclV1U1A0R3BjN0pqb1NWeDI5T0IyNWFqV0VUZDhtZjZRSFMySXdoSDdHZEluMXA0bWp2MXZCVFkxUDc2Y2l4UWxRZDZybmU3YjRXdXN0MTNkTkxGQ3hweXJDV1JhdUhpM3lQNldib1RuajFPMjRualdMSlpRMC1DWWxQYkFFNU5CYXpNbzZrdnRCam1fN0U3ZEFzdGo2a2VhTjZrWEZNZw?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1560,52 +1560,52 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46073.53616898148</v>
+        <v>46073.64930555555</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>​Ochsenfurt: E-Scooter-Fahrer mit fast drei Promille erwischt - Radio Gong Würzburg</t>
+          <t>Plainte pour atteinte à l’intégrité sexuelle d’une stagiaire contre Marc Uyttendaele : des étudian... - L-Post</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>​Ochsenfurt: E-scooter driver caught with almost three per mille - Radio Gong Würzburg</t>
+          <t>Complaint for violation of the sexual integrity of an intern against Marc Uyttendaele: students... - L-Post</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 15:15:00 GMT</t>
+          <t>Sat, 21 Feb 2026 00:04:19 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxPcmhQcUtxRGRzSmpkbEpwdmYwR2NzTWI5eXRDSzg2Sm1Cd3FuYXFaTmtvMzdWLWFRU1FXcVhDWXF2ZGcxT0ZETzFGeHZoWDdIY29zNjUwNndnLVp5M202cDRsNnFiRVpUQkRMZlJUN0VZeFpXZmt6N2FfWkdkQ0dSZ1Q5NmtmZXNYVnBUT3RQRExkMmZjQlc4TA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7wFBVV95cUxQeWRLOThYc195ZlAzSGNFX2ppSHVCQzMwRE0xUXBtaTRFa0xOR2M0M1EtOUpwdTFTLUtWeFgyMEt6eXpvNERHeGpubUpIaUZTTG9jSlZ1NEl0bTNSbnI0OHhBS0xoaTM2b201VW15ajFMSUZSRUl2Nmg1UlJwcHZobTY0U3JELTJwVmUxZW9MaTh0RHBKTDBJVlAzajdoTUJfQXYxR19hVHloa2ozbE9QZnUzbm1LUUtrUUFwMWNnRU1oaHpoaTl3X3F0cmtnQ2lRV05pT01SdVBtemt1UHJFT3FGeUpyamwwcXhoMy0tb9IB7wFBVV95cUxQeWRLOThYc195ZlAzSGNFX2ppSHVCQzMwRE0xUXBtaTRFa0xOR2M0M1EtOUpwdTFTLUtWeFgyMEt6eXpvNERHeGpubUpIaUZTTG9jSlZ1NEl0bTNSbnI0OHhBS0xoaTM2b201VW15ajFMSUZSRUl2Nmg1UlJwcHZobTY0U3JELTJwVmUxZW9MaTh0RHBKTDBJVlAzajdoTUJfQXYxR19hVHloa2ozbE9QZnUzbm1LUUtrUUFwMWNnRU1oaHpoaTl3X3F0cmtnQ2lRV05pT01SdVBtemt1UHJFT3FGeUpyamwwcXhoMy0tbw?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1615,52 +1615,52 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46073.63541666666</v>
+        <v>46074.00299768519</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Randersacker: Telefontrickbetrüger mit Arzt-Masche erfolgreich - Charivari Würzburg</t>
+          <t>Nouvelle stratégie de la Croix-Rouge de Flandre : « En cas de catastrophe majeure, il faudra pouvoir se débrouiller plus longtemps seul - De Standaard</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Randersacker: Telephone scammer with doctor scam successful - Charivari Würzburg</t>
+          <t>New strategy of the Flanders Red Cross: “In the event of a major disaster, we will need to be able to manage alone for longer - De Standaard</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 14:00:00 GMT</t>
+          <t>Fri, 20 Feb 2026 23:42:16 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxPMGh3SXFhTUFXXzVCVUQxa1UxSmNGSEhOZ1N6c2VOM0xabHk4a3I4QkwyQWNzaUl2V3VCc2VzZUNmTTFnX1J6TFhRR04zUXlMRDVJc0REZmFRLWZOV0hzMDNzbGtHd1RUYXE0dXVLbkdxOEJNR0dzLXJxOGR0eFpxeTlzdURxRHE2RmtQX0R0VDlOWXNJV0loNjd2cHRMZEVV?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwJBVV95cUxPTjhOa3haWkhPQ1ZxbTVXWUJ5N2dwVXRlTy1aXzhmcllfbnBCREM3bE43eHNRRFZnYlE1UkxBMUJnVzFhbjVHaXNoZmlERnFydWpySmM2MVJKX3Bnd2R1ZTNpSFBhbjRNSFA2TFRZNWZxYzRnYzNpM1lnZzhBRVExUTJHTW81bVQ5bk1mNFVxY2FYY0RsTEZRV3FjZDNxeGhqekU1X1hLUnZhcXZKaGlOeHpRZ2lJOG5uaFRuXy1yWVZlY2Z4aU9aei1LNTJmbU5EV2R1bjhQWEJ1dlNtRXN2b0puNF8xTVRtYkRtWHQza0J1Ykx4N3JoQ1N2TWNPWHg3TEhEcFB6SQ?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1670,52 +1670,52 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46073.58333333334</v>
+        <v>46073.98768518519</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Einbruch in Laufacher Fachgeschäft: Zeugen gesucht | Foto: Silas Stein - main-echo.de</t>
+          <t>#FrigoVide : les associations dénoncent l’explosion de la précarité alimentaire - tvcom.be</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Burglary in Laufach specialist store: Witnesses wanted | Photo: Silas Stein - main-echo.de</t>
+          <t>#FrigoVide: associations denounce the explosion of food insecurity - tvcom.be</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 10:31:21 GMT</t>
+          <t>Fri, 20 Feb 2026 15:39:26 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxNWmtnWnFmSm5hNWthTXJnQXFTSHA1aFdfNkZmQlFPQ0xPenNWMG1PMnpIbEVYblFlN0djMXBIOXZKVWtoRXFadkNrbE9zQnV3YnJ4RENiV1BDeHJkQUt3VkVGdmwxN0FqOTAteDY1ZlZKcVZkTV9OT2xQUTdWOERNU09RZ2lQelo3VkNsUGNfRXdtb1ZPOHFleGtLaDBzZF83TWpWbGQ2NlMxQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOUWpKRFpFYlQ5ZTd6NFJfQXZlRnZhMVo0ZlFDMExaQkRldUEweDFNSWd2eFdBMDB1TGlzYk93MFRQR0ZJWVZsQ19yak04UmZlZFMwWDMyUllJUVB5d2R1WTJQT3dQS2NOMTN4TC1DeTMwM3FxWEFuQ09aeE5STWpiSGpUZmVtbzJILWx2aWFaZ3UtejV0cnRRUXRMdVFsYUJ1dGNuSWV3LVZyODg?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1725,52 +1725,52 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46073.4384375</v>
+        <v>46073.65238425926</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Mobile Blitzer in Aschaffenburg aktuell am Freitag: Hier nimmt die Polizei am 20.02.2026 Raser ins Visier - News.de</t>
+          <t>Un député québécois agressé à Bruxelles: “Triste que les villes européennes en soient rendues là” - 7sur7.be</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Mobile speed cameras in Aschaffenburg currently on Friday: Here the police are targeting speeders on February 20th, 2026 - News.de</t>
+          <t>A Quebec MP attacked in Brussels: “Sad that European cities have reached this point” - 7sur7.be</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 13:15:45 GMT</t>
+          <t>Fri, 20 Feb 2026 12:56:00 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxQNkVuMENSQnJIdUE5ZUpFWWJRNHZVeEVXcHFMQVRwQ1hub2V0Q1VmdDZtS2hsSDQ1d2JiUjhrTW11bHZjWXcxQ0tfNmZpRUdYVHY3OTlzblhSMUVKNmU3THJFdXhNTTd1SGczbjdwbmJDWjNOLS1femx5UjJpUmR5NzNsN3EwWGI2Q3Frb2RESlNBcF9wcVM0WnN0QUdYQ2o2YXJQTDQ5ekJ5bEtFYjlxZlBkOGVUby1lbzFqbXJqMjNVdU5oMEZNZFRYNG5NY0txbFNrUTdNOWJmX1ZibzRtZkN1UC0wVzI2V0hua0pFcllSbFAtSVRn0gH8AUFVX3lxTE90amswVGNHQ01Odnl5TkpmNkQzd2laX3VMSXJjaXQzU3JRcGlfbnJfUi10LWlSM1JjM29KSWIyanFZWnNtcHN3Xy1KOHFIdWRRN2EwUERsWHVrZTZKaWc1bENIdHpGb1Ztb1pKNGNkeVZnQ2lnTi0tRWZlVERwNW5aWGhLOFVPMG8xWmF0OXYtd1QwLVJjaTdWU3hqRkIzV0pRSWk5eW5KelRnbE5IM1cwQ1hDQTBNWko3bS1kdkdPR3V1N09IVEpKRHNTNnhNUFdZUlBCM01oSlFIMlNBMG1SbzRxM1hIVjh5ZG9fNlJGdkU3TU41WXEwUG13SA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxPeDFBWkdGenBYUkpaZXpzNVB4RzZJemNrTFlwbnpiUzRta0VpcjJUdGhhd0NuMWJjb25ZTFZBZGZhQ2c1VTQzNDVoVzhQYW84Z2k1cFY4R1FGWEpSSkxxQzdXQ2xaWU1Yajh0aG15TEtpLUpMVHRHUXdUd2d4eTZrWHdOZXpNNjJVMHFhV0t4ckdrR2dvOEJFY1RXR044d2ZYODhRYkpOUEJSQWxsTDdQejVaUkwxZFQ1aDNzUkNDaTBsczY1bUREbDNEQmpHMlFEUUZvRlpB?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1780,52 +1780,52 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46073.55260416667</v>
+        <v>46073.53888888889</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Polizei-News Bamberg / Schweinfurt / Würzburg, 20.02.26: Zollamt Schweinfurt intensiviert Kampf gegen Schwarzarbeit 2025 - News.de</t>
+          <t>Accident entre une moto et un camion place Madou: deux personnes hospitalisées - BruxellesToday</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Police News Bamberg / Schweinfurt / Würzburg, February 20, 2026: Schweinfurt Customs Office intensifies the fight against undeclared work 2025 - News.de</t>
+          <t>Accident between a motorcycle and a truck at Madou Square: two people hospitalized - BruxellesToday</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 09:54:02 GMT</t>
+          <t>Fri, 20 Feb 2026 17:01:00 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPT0gzcXJvcDBRa3pZM3AxVzlTeldTSVU5aGVZSmMwclE3STQ1RTE3c2RXNW9abjg1QXY3ZTQ1UWs1ZVUxX0o1R1BITEdWYmVncXd5aXB0MnlrcG5YT29DS1JTQ3pnb2dBMEZ2RU1kUTV6THlBeXlUejJjTlV1cXpZS01YRUU2a0ZEWmtTdUJRQTQ5eFh3THEtU0RnOEdaV2dleUltLXpSaHRtZUxRdlFV0gG0AUFVX3lxTFB1WmM1eFdVSHVJTVVXN1F4dTRsRkpaaTVWTFZxVWVwMG1JdENPelhXVndjX01Gb3p1NndvblN5WjJPTWdUMG52eFcxOWxDenRSWnBvb0tCUllITTJyNmZDR2t0S2lqbnVnZ2dBMkhIRnBOLXNpbmZ2bnJ2b25IOEtoSmROUDlfajRpLW11Z01lTzUzS3VGZS1oTHZybmxBYkFXdmszQXdtRzJ0Z05lOHozNGFuSQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxOZVFQQzlPaFFsSjBwaVBickxVRmdtd0ZjZ3ZnbmtiT3U0cEgxblVZWmNFN2hfMnByT1pvQUItNEVtZ0dlMkMxRlFFX0dkdEUzM0lWdGtLX0VMQmNNczdtMGZoTnNvZ0RpQWdWNm9TREo2YU9fcVlocGpNeXFGM1ZHX1FvS0hhVVk?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1835,52 +1835,52 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46073.41252314814</v>
+        <v>46073.70902777778</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Polizeimeldung Bamberg, 20.02.2026: Einbrecher entkommen mit Tresor - News.de</t>
+          <t>Des adolescents embarqués en voiture puis dépouillés à Braine-l’Alleud et à Waterloo - 7sur7.be</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Police report Bamberg, February 20, 2026: Burglars escape with a safe - News.de</t>
+          <t>Teenagers taken by car then robbed in Braine-l’Alleud and Waterloo - 7sur7.be</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 11:35:02 GMT</t>
+          <t>Fri, 20 Feb 2026 11:18:00 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxQTDRVeGxRTzBmZ200OEl2d2huS2VhcFZvTWxucWc0VVhaQkJzak96dW51NEt3V2g3SC1INEZmWXdjbDBVbVRqeDl0NDBqYzJZSHV6Vllwa1NXbC1YRGRLWkpmbWFKdFBHSW5WWVFLQW1vb3hfeWIyY2R1bm5EUllUTkRtLW5iQ3phV3pNSjF0S3dyYS1XZzZkOTd6NG9UWFY1c3Qw0gGoAUFVX3lxTFBlLXFyeU1ONEpmNEV5bFpuQUV6V0lhazdlY21XUFpZaUpVUVFEUVBGbjItWEJaX3ZxWVZpSW1UczJCak9DNkxiMW9NTFhZeXhDUmR0R3M5WGFJbjQtUjN5TldKbkdZOVIyVTVKcUZJd2VHdjdBektOT2ltZ1VwREZDSmFqWVdKeXVBbEhZcGRZYXAzTjhDOW5wX1o2d05SU3RwOTdCSTk4Xw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxQdWZrakJRZHh6c1h0RzJHaWtoU0NCYkdmZlNsWWdlaEgxQTJ2ZUxfVUczU2c5MkxwNkM2NF9YY3pRek1NRUw4R0JCZlRWc0FORWxKdWh1dm1RRl9HbUVPMFVpbjZYZklhZVdtejVScnFWYjlKX05xTThIQWpUelRLZVp5cU1TR3Uzc3R1aGNzTWJVV3VDYXI1S2ZESG96bFN4Wkg5UEMzaTNkcXNNWmwwQVcxT0VnWlMySW04OU5DODFYYVNmZFE?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1890,52 +1890,52 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46073.48266203704</v>
+        <v>46073.47083333333</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Village Wertheim (fallback)</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Business of Healthcare Summit welcomes another packed house - Florida State University News</t>
+          <t>Un garçon de 10 ans meurt percuté par un tracteur dans une ferme en Flandre - 7sur7.be</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Business of Healthcare Summit welcomes another packed house - Florida State University News</t>
+          <t>A 10-year-old boy dies after being hit by a tractor on a farm in Flanders - 7sur7.be</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 15:22:25 GMT</t>
+          <t>Fri, 20 Feb 2026 16:34:00 GMT</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNb01GazY5VElxMXdSWmg3MnpPcFFIYy1pM1FzTFV6enF3SG81MzhFS0xPNzlDUzZCcm5aMXF6NzdEanlKRnpFbHBuNVJqSGN4MU1sUGIzYTZUWldieTF5UHhrQVdQbmZaT0pOOV9QYTZBbTFvdlc2dlVSaER0QVFGQ1Rpc2N3Tlh2WDFIUlZTM1VXYko5YVZZVk5jZlJMb1ExYWVpUnNhamRqUTdPUUIxaUJNNFpONXNU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOTEtfWklVd0F0cTVyenY3LTNHSlJqczhYM2EwVDdYRWtjQ2ZYVkZJVzFpNmNJbWhNOFB1NUlxLTluOEVEazRoM2o2SUF3WUpuV3c3X2JKdlVBdmFZdlE1WFhyZU84Y1lNLTA3Vk1hZ0l2VE9KTk9Fb1R1WmdVLUFuakZ4dkFFZmU2R2pxaGtPMVluOTY2dUhlRXpmb3ZEYzRMTW1HRUVHU2dsTW9ZTXpsbDRJOFc4Qlh1TGlZ?oc=5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1945,52 +1945,52 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K28" s="1" t="n">
-        <v>46073.64056712963</v>
+        <v>46073.69027777778</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Village Wertheim (fallback)</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>University of Florida expands study abroad with Antarctic expedition - Gainesville Sun</t>
+          <t>Verdachte gevat na crash bij politieachtervolging in Hasselt-Kortessem - MSN</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>University of Florida expands study abroad with Antarctic expedition - Gainesville Sun</t>
+          <t>Suspect caught after crash during police chase in Hasselt-Kortessem - MSN</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 10:02:00 GMT</t>
+          <t>Fri, 20 Feb 2026 09:17:18 GMT</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxPdkVfYlpLQ2ViMnBuUy1hUUtTYUhZbFhiUlNHeUJ2cEkzT3QtWEdBcHRDS2tnZ0dWSVBSZ2tGRnUtYjBHbnB5eVN1Z2gzWUtlZVNTZXR3UFZiZDBsQ1NaRWJlNEcyNHlUbWhiNDNlMjMtMjJkaHZKVWtOVGJ2OG9mZm1qWmVRWkFQaGRSaXlnSGM4NzhuSlkwcWplaTF2dXVHMGZjVHZzSWxtdW9ZWmtnNkpVQTVHZjlaMVRSQ0FKR0lWT01zcVROVi1nQnl1NV9NR2p3ZkI2X05Ua1k?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2gJBVV95cUxNV0VnTkp1dmVVT3pBOTNwdnU3dVhCUy14UTF4TXBPamttNjJfc212eWF6N1NMX2hlTS10Ullqckd6SjJUVlhkVV9yWTl3cW90U0UyYmtiSkJMM0xYcndpRElhbTZxTk9rNVhRSVRSZDNPQW5iaGw2YjhXSDVLWmpMaldWYWdrQWtxZ05SRmM0Y0JLNFJEclFObjFDTVN4SEk0UGgxX1NNUWRtdTNLZEdPWGxKVWpfaDVMZmVDSmVRVkZ4cnE5c3VEVGR3UThMVVFGZFpjdS03OENTdjM3Snd1TFFVY1R6ZTBHa29OaGllVlpJaWdNQWU5ck5lSWFmRW5seVo1cUhVTGxPVnNNcWtGNVdxbXhmNHlNNjc3cGxPV21reTZIeGQtWGl4SGlMRHFDRjVyTnZTOEgzS3kxSDFLbDJLWm1MX2NZYnZmdXpBaERsTDBTZncyaTR3?oc=5</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2000,52 +2000,52 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K29" s="1" t="n">
-        <v>46073.41805555556</v>
+        <v>46073.38701388889</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>Local Town Maasmechelen French</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Autobahn gesperrt: Getränkelaster rutscht in die Leitplanke – Unfall auf A93 - Augsburger Allgemeine</t>
+          <t>TC Hasselt - Sept ans de prison pour des violences sexuelles sur ses deux belles-petites-filles - La Libre.be</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Motorway closed: drinks truck slides into the guardrail - accident on A93 - Augsburger Allgemeine</t>
+          <t>TC Hasselt - Seven years in prison for sexual violence against his two step-granddaughters - La Libre.be</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 10:46:49 GMT</t>
+          <t>Fri, 20 Feb 2026 09:55:00 GMT</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxQb2RxcW1rQ0l1LWN0UnJ6c2RNXzdPdGJwbW9IWjlSN3czX1NaRE9LSGIyZ0JuRi1aWTFrVFBHTEdmaFdUZXZ3T3NRcmI3dHp3WkF6NGYxeUtjLS1XUlZROW5jcG0tS1lCdEFGZl9ibi1VLUFoSjFnS3pmc3E3VDdkS2JBNWRUX3hhU05qcThTM29hWTFXLW5temVmR0w0QzBsbWZKeFJtZnZlUjE2YVNPVXpMVWZWNlN4MHFFY0h1Z0lkX2VvVnhuNHBxTnV1dWxKR0NBZDcyQjVyRFVMM3NDRw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxOclBuU1RUenlOSXdkOXhpbFZkYndoLXF4aFAtUzFidUtabDlLemJ4bklOLTFMcWRKVk50VnRCaHZxOURvLTl1TTNuSm5CZFQxOHJfNFpqdVYybzRuR2RRS3QwbGVJdHhRWkZxWDhvancybUctWUdpTGNmZkpjclJSa1E5S1haTW93SWUxYURpS3plQ2wtTGxXaEc4d0RTQ3dfRFhOM296SGtMc0s1NU1HM19yeXRZYk5ic1RJOUQxdXRSQUVoY2dseGU3UGlaMlZaRkwwOG4wWmVxQi1fdm1Fa0lBWm51ek9XTnBvUUE3QmJhU1Bnc2pxLXdWX2lhcFpoNk5HVQ?oc=5</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2055,52 +2055,52 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K30" s="1" t="n">
-        <v>46073.44917824074</v>
+        <v>46073.41319444445</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>Local Town Maasmechelen French</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Bayern: Polizei- und Feuerwehrmeldungen am 20.02.2026 - Newsflash24</t>
+          <t>"Samedi 21 février, l’extrême droite marche dans les rues de Lyon, et nous continuerons à résister" - Politis.fr</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Bavaria: Police and fire brigade reports on February 20, 2026 - Newsflash24</t>
+          <t>“Saturday February 21, the far right marches in the streets of Lyon, and we will continue to resist” - Politis.fr</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 08:46:00 GMT</t>
+          <t>Fri, 20 Feb 2026 14:49:09 GMT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxQNmd1b2lTdTQwQ003YVZEc0RlQTFpRHBkcVUzNnU4OWlkOXpHbXRwZF9QUTEtU0FvWVoxQW40SUgxRzVIenoyLUdES3cyX2llYnBvOE1qRVByeDRXWTRTN2syT1IzbFJZSndCZlJManFkbjhVc3ByVV9BcVM1Y3dlUjlFdW02d0hOVW9nZnZPQnJZdXpTaU9r?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxPUEpJREtJZFcwTlZpcWRJNk9jLXR6aUU4aVBiejZ0cmwzX2NNcmF2M0V5S29uVHExMXI1RGZvUmRIWVZNZDlsY2tRTTBNNnNKU1EzX3FkdjBDOGJDaHRlSVJaeVRKTDRETVVaME5rRExuUE12N2lDdDR0ZEdGN3ZoaEtEWUQyek43b0xsU05XaU0xQVFlTFl6QkszRHVNcnh6em9fLU9DR1NVRjFWUnNSN1RIZFhPV2p3Mlk1NGI0OUs3Q2NNcFJ1QURCd1M4RmN5?oc=5</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2110,52 +2110,52 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K31" s="1" t="n">
-        <v>46073.36527777778</v>
+        <v>46073.61746527778</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Village Ingolstadt (fallback)</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>New attendance record! Remaining regular season games sold out - EHC Red Bull München</t>
+          <t>Jeugd Patro Eisden Maasmechelen vs RFC Liege Livescore,... - SportyTV</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>New attendance record! Remaining regular season games sold out - EHC Red Bull München</t>
+          <t>Youth Patro Eisden Maasmechelen vs RFC Liege Livescore,... - SportyTV</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 11:30:00 GMT</t>
+          <t>Fri, 20 Feb 2026 10:06:22 GMT</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPQmRWY0VOQzRiY3U1amZfOUIwSVplbGFjTkpXUGxfQ25IWjQtWlMyN1gwcmMtVm1LSnNBMzFGYnJaYklsMG1RdG15R2JBVWFXcHF3R1NGUmZGcHpUSGFnb0RhdUZVXzBCMlJKbWs1ODJ6WHY0Si1rMkRXZmVUaFZZU2lCZnNzUnhWdmQyaXkySmJ5R0l6QlBqV04wMTMtVHJKZW5oN05PT3RtZktCNWVyS2pYYUh0UGZ3RVE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxObldNLU5POXlqSFY5bzV5TGJ3Qy1qbEE0SlYxUk41YlZsNW9yOHhGMW9XdjE4aDZpVXd6bjNoV3lSMTFIUFBqSjdyWXdhb3Byd2RFZU9Vb2lJbklsRWRaQ1paampuV0doRmZieHZPU2hnSmFIeVJzajU3YjNqSVpXcXJiTWxqbWwxV2tlcll4SUIweGdmc3FjaGI1R0s?oc=5</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2179,38 +2179,38 @@
         </is>
       </c>
       <c r="K32" s="1" t="n">
-        <v>46073.47916666666</v>
+        <v>46073.42108796296</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Village Las Rozas La Roca (fallback)</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>("Las Rozas Village" OR "La Roca Village" OR "Las Rozas" OR "La Roca") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Surprising results: why more parents in Madrid are opting for gadget bans, making unexpected choices for the sake of family harmony - russpain.com</t>
+          <t>French PM says government intends to criminalize calls for any country’s destruction - The Times of Israel</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Surprising results: why more parents in Madrid are opting for gadget bans, making unexpected choices for the sake of family harmony - russpain.com</t>
+          <t>French PM says government intends to criminalize calls for any country’s destruction - The Times of Israel</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 09:18:53 GMT</t>
+          <t>Fri, 20 Feb 2026 09:57:21 GMT</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPekk2OFAwVk0tWG5ua3NUdkQzQXV0T1B1WHpraDZIckNOeWZ6dHpkMjRQc3JKb1pkSV9WMkltZkdzanVQV0VtNmRqRTBBNXI0TWNWRjY0SlpuUV9uTHFuaFctbEJ6cWRKYm1kc3hjejhTV1pXMU9hOV9GMVpYcERnc1VwWGRkakNqNl8tcENveENHeGFaZHZZWVZUalA1WHMtWXkwNGpaTGxUbTNwWXow?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPdHVVcjRxOUM5a2JxNUlFUjNPdG5iTTc2UDk1cFU1c1ZCd1ltODY4blN2UTdXcGYwN3ZSWXZyV3pFMXZTZWlRemlhTmVib2EtMmhlVHd2RGdNaWlvMmQ2clpBWUYyakE2R09aR1F6Mnk1MHNqV0FsVjlUWmZyWkJuVG03NmstTmIzVmxfQlZkdnNVZmR3N0JabFR3Z1ptOEtRQ1ROQ3huWlZuOHZFV21NeFRyWkVhMmxvOUVhTzdFZ2xJN0xYU0piZA?oc=5</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2234,38 +2234,38 @@
         </is>
       </c>
       <c r="K33" s="1" t="n">
-        <v>46073.38811342593</v>
+        <v>46073.41482638889</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Kildare woman who went on theft spree avoids jail - kildare-nationalist.ie</t>
+          <t>Hundreds of Belgians locked up in foreign prisons - The Brussels Times</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Kildare woman who went on theft spree avoids jail - kildare-nationalist.ie</t>
+          <t>Hundreds of Belgians locked up in foreign prisons - The Brussels Times</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 13:09:31 GMT</t>
+          <t>Fri, 20 Feb 2026 12:13:14 GMT</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxQclVHcWtrOEZBRVkwWmc1Zzc2VzRtYlJrek1hSnVnYzRUTjR6ejRJeGdhbnNtTXFGd2drdWctcFg1R01MOG5fY3ZBd2RMOUFSY2U0NktsQ0tnS2dMUE5OY1NyTmpLaTlGeHR4UExkdWNqMEZoLTZGbWEzcXVfSjl1YmVJazFiNEN3VVoxMC1DNXpGS1RQamhpZE5tM1N1T3BoY0RUakV2bXk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOM1dqd09VU1RVSjFaYnlfVzlYRmUzc0lWZXN0TVRmZDdOdmJzaTE5TmRxQ1VncHpGM3BJSFItLTVTSktKNDRjdFJEMVVsNHBtbUo1R1J3eFJhdnRhR05RMHk5MExTdGNENnROZ1g2NXREUFZjNU1pWFBEUE9zS3dlckYzSFdSbVhqa3lDTUNFZw?oc=5</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2289,38 +2289,38 @@
         </is>
       </c>
       <c r="K34" s="1" t="n">
-        <v>46073.54827546296</v>
+        <v>46073.50918981482</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>LATEST: Approval for new 50-bed care facility for Kildare - Kildare Now</t>
+          <t>Margot Robbie Stuns in Red Gown at Wuthering Heights Premiere - AOL.com</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>LATEST: Approval for new 50-bed care facility for Kildare - Kildare Now</t>
+          <t>Margot Robbie Stuns in Red Gown at Wuthering Heights Premiere - AOL.com</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 14:00:00 GMT</t>
+          <t>Fri, 20 Feb 2026 16:35:57 GMT</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPbExsSFlvZXFyanNuUkpoQzRGbDgtOHpleTd5Z05LVmdXSDM1SzJ2bFhLMG92RWZld1MzNEh3LUxIUEE0VEtWaGdLbVNDeExYa295cExfOWtRal85cGhKQi1XRWNnT00wS20zRTBaOHNuZmlBSGd5ZktrcmhwRHJOcXRJMEk1OU82WG9vektZU3JCcGpaR19OWnFSQmxlMUF0X1BsTmJQWjI4U290WmtDRjJR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE8waEpNdEZmMmtDMFhIVzRBZ0QteWtGc0JMUjRFT2hzUXNGa25Pa2FPNzRHSWtUZVVvcGNORnNvYjFVZ2dIeVBMNEs4dTBvdVhmYUt0UWx6T0RQR2daak9ZR2p2SFpZU3lRS2dNaXJ0M0pSMGM3bmcyeEJvT1Y?oc=5</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2344,38 +2344,38 @@
         </is>
       </c>
       <c r="K35" s="1" t="n">
-        <v>46073.58333333334</v>
+        <v>46073.69163194444</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>TEAM NEWS: Dublin LGFA Senior Panel is Announced for Kildare Clash - dublingaa.ie</t>
+          <t>Wertheim: 48 junge Beamte zu Polizeiobermeistern ernannt - Fränkische Nachrichten</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>TEAM NEWS: Dublin LGFA Senior Panel is Announced for Kildare Clash - dublingaa.ie</t>
+          <t>Wertheim: 48 young officers appointed police chiefs - Fränkische Nachrichten</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 12:05:44 GMT</t>
+          <t>Fri, 20 Feb 2026 11:00:00 GMT</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNMTd1bndiQlVXcTAtUjV3aHZ0ZE9McEV3VGp2Z0wwMF94b2Q5Z21uaWRTZFZXQzJOZVVOMjFJTkhmYzE2OVRqQmpwSXAtbDVRVG41bGRFVnlmU252TVdNTjlPa3NSdDdwaXFjMnFUU05RVXIxem9pQ1pkWlJzNUhFMjd3azNIdTlfeDVtTG1uRlRfYnU4SWZneWRGbw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxOVmx1X1F5RFNnSlRmakZ1d2dxcmtYcnJQWFdSeVlKWVBCMzE0Y3d6b1VSVTRPN1l5LWZPa2NGX25Gb0ktUEVxaEFnYkpHc1pTTHl3WTkxMHhrRlVnazRPcE9JcE1OaExlRHhEZ2ZRYkN4TWRSakg5VFdodHAwV0pRSHI2TlRLU1dXZjNXVDVEVDNULXI3amZuX0FLVEFCTWVDX05VTG16bE1WYWtkRVBoVXFkbUxmYjdzSlhTMEhsRzBKTDBFTGc?oc=5</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2385,52 +2385,52 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K36" s="1" t="n">
-        <v>46073.50398148148</v>
+        <v>46073.45833333334</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>A new spin on Irish mythology: Kildare-based author to launch his debut children's fantasy book - Kildare Now</t>
+          <t>​Lkr. Würzburg: Nach Einbrüchen in Kürnach und Gerbrunn – Zeugen gesucht - Charivari Würzburg</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>A new spin on Irish mythology: Kildare-based author to launch his debut children's fantasy book - Kildare Now</t>
+          <t>​Lkr. Würzburg: Witnesses wanted after break-ins in Kürnach and Gerbrunn - Charivari Würzburg</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 11:05:00 GMT</t>
+          <t>Fri, 20 Feb 2026 15:00:00 GMT</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxNNlQ4bXZjaGp1VG5KNjUxSFhzZFhVZXV2NDEzR3BqX3lVUS10NW9oYWx4bjRNYndyczhudXJ3NFhjWkNhcTlQOXNwQjBUMl96NGZqaGo3eUdqM3hxQlBBbDN3bTNhQVBlX0pTSnRhTUhSMVFVX2NEYmlDS3FzQ3hqTTBvQjBiTWpvblNva3YyTWthXy1NVDVOWnF3dTRtUlF6RlowNlpEOUVwOVZSR1dDdWo0SkpYcUpQeTBlM2VHbDNGQlp4OWZXVmYzVGNLOEVMQklTV2NyNkdVV1l1S1k1aUg2ZS0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQV2FjWFB5LVFqM0tJZm9pMkpqcThoaFFTWmt5V1JwUTYtT2RqejFFdF9XZTZOZmFubERuZEZBMGJKbWxFMHVNdDdWRVNBbDhBNXYydEZMRjZ4VGRtV0MtVWZBQzhhQnAyTkc1NzlpOUlORGptMFRkaVFwNjZ3RDJtTmNQbnI0eWsxSHhTdnNmTVh4eWxhTWo0a0FUcjUwOTBZZ0xjVm1FNks0YU0?oc=5</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2440,52 +2440,52 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K37" s="1" t="n">
-        <v>46073.46180555555</v>
+        <v>46073.625</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Kildare student represents county on Gaisce Youth Ambassador Panel - kildare-nationalist.ie</t>
+          <t>​Ochsenfurt: E-Scooter-Fahrer mit fast drei Promille erwischt - Charivari Würzburg</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Kildare student represents county on Gaisce Youth Ambassador Panel - kildare-nationalist.ie</t>
+          <t>​Ochsenfurt: E-scooter driver caught with almost three per mille - Charivari Würzburg</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 14:01:22 GMT</t>
+          <t>Fri, 20 Feb 2026 15:15:00 GMT</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxOd3lPbGJWMkdJdVdaR0FHU253VUQyYWtkMnV6UFVWWTB3QVpPN0hReV9LZ1NRWFpwRGZMWFRMN2JHdDNYTXBhM0JIVm14MmxqOTAwanMxb3gybkd5emd4XzBUSmdGQWFVZjItZXE4REg4Umd5bE9rOGxnd1Y1c0FlQXRselBoRkxkZGgzMUl5WGpxdUxRb3o3NkhqejI0UFAzU0xyR3liblJFUGw5MEh1WmxhU2d5OE9feHJvUFYzdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxONmFITnUybVNkanBFVkpVbU55VktuTUJRYzJacnlFdXA2X1ZvakdvMlo5RGxkZ2E0aDl4R2xsbVAwdUhPY2Jfclg2S0dIYU1OV0lWZkJSZ25iMVQ5ck5UX19lZlByeHlZSjVSY09VLTJYWHFObmZXbEtNVmlFUWRUZ0lxQ0FUMzVhWDRNbXl6RmRfVkNtMnZWb2tDSGg?oc=5</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2495,52 +2495,52 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K38" s="1" t="n">
-        <v>46073.58428240741</v>
+        <v>46073.63541666666</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Great news for Kildare house hunters! 24 new properties get green light - Kildare Now</t>
+          <t>Bad Neustadt: Person von Güterzug erfasst – Bahnstrecke war stundenlang gesperrt - Charivari Würzburg</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Great news for Kildare house hunters! 24 new properties get green light - Kildare Now</t>
+          <t>Bad Neustadt: Person hit by freight train - railway line was closed for hours - Charivari Würzburg</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 10:26:00 GMT</t>
+          <t>Fri, 20 Feb 2026 16:30:00 GMT</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOWHlfdkVaZnhqWkFoXzBNaURZcG5MX3cxamJNTzkwOThlQ2lmSEx2VzBVQVp6YWZjN19YX2lyY3Z1YTBNbWhMUWlLRUwtZjlJbGFGaG9iakFHdU5KVG9zZ3JjUDM3VVoyelhVVEo1Nm9ycThXQUk1bkdjR3oxSzI4d3BnUXlyc0RaQnlPN2lrZDFkRENwR3pYenZQNmMtMFdraldPb3liWmN2S3VrU2RlbGhQbDlJUndaaGhXckt2M3FLYWx1?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxNZ1BkcFp4Smw0OVB5M1hrbk5nWmp3ZHdWUWVMMGEzSjN1MjNUSDR2djNsd19kS0o3NTJtblg5Umw4R1lFOWYxRE83bGlHd3hjRU1XNlh3Q1pESndBNFdnTmV1T2VsM0xJcm1Ub0Z6cUNCTGdMVkh0blNhNk5fcjlNalk1aW5INmtPM3A2QUdnUG1seGoyMzVDX2JHLXEyY3hTd1pJQlZVWU9IMWkwMU4xb1pQZzJOQ1hSNHc?oc=5</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2550,52 +2550,52 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K39" s="1" t="n">
-        <v>46073.43472222222</v>
+        <v>46073.6875</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Bus stop between Newbridge and Naas is ‘a mud bath’, Kildare County Council is told - Kildare Now</t>
+          <t>Mobile Blitzer in Aschaffenburg aktuell am Freitag: Hier nimmt die Polizei am 20.02.2026 Raser ins Visier - News.de</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Bus stop between Newbridge and Naas is ‘a mud bath’, Kildare County Council is told - Kildare Now</t>
+          <t>Mobile speed cameras in Aschaffenburg currently on Friday: Here the police are targeting speeders on February 20th, 2026 - News.de</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 09:35:00 GMT</t>
+          <t>Fri, 20 Feb 2026 13:15:00 GMT</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxON2daWDdiY3FuQWdJcUNjRFJHQ1FlZ3luX0o5OGJaNDlfSlFRSVZVVi1yTVh6bVJXMUxPOENXMDZ5OWZUcmN0cjVPTjhKTEYwSjVfTHl6Y1ZPZVpLU2w2WmxxRHZ1RGw3LXF4Q2U5Tkx4QWdTX1ptY0VNRTZsd21KSWNWNHh6VkpDOVBXMlhIRDBRMmhmVFhFdmtKYlhpQzQzZV9yQ2U3ejhIaUQwWnppLVUxX3RCekdHRnc2NWx6QUpOOW9wbVltMFJVdkIwX1NSN2c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxQNkVuMENSQnJIdUE5ZUpFWWJRNHZVeEVXcHFMQVRwQ1hub2V0Q1VmdDZtS2hsSDQ1d2JiUjhrTW11bHZjWXcxQ0tfNmZpRUdYVHY3OTlzblhSMUVKNmU3THJFdXhNTTd1SGczbjdwbmJDWjNOLS1femx5UjJpUmR5NzNsN3EwWGI2Q3Frb2RESlNBcF9wcVM0WnN0QUdYQ2o2YXJQTDQ5ekJ5bEtFYjlxZlBkOGVUby1lbzFqbXJqMjNVdU5oMEZNZFRYNG5NY0txbFNrUTdNOWJmX1ZibzRtZkN1UC0wVzI2V0hua0pFcllSbFAtSVRn0gH8AUFVX3lxTE90amswVGNHQ01Odnl5TkpmNkQzd2laX3VMSXJjaXQzU3JRcGlfbnJfUi10LWlSM1JjM29KSWIyanFZWnNtcHN3Xy1KOHFIdWRRN2EwUERsWHVrZTZKaWc1bENIdHpGb1Ztb1pKNGNkeVZnQ2lnTi0tRWZlVERwNW5aWGhLOFVPMG8xWmF0OXYtd1QwLVJjaTdWU3hqRkIzV0pRSWk5eW5KelRnbE5IM1cwQ1hDQTBNWko3bS1kdkdPR3V1N09IVEpKRHNTNnhNUFdZUlBCM01oSlFIMlNBMG1SbzRxM1hIVjh5ZG9fNlJGdkU3TU41WXEwUG13SA?oc=5</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2605,52 +2605,52 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K40" s="1" t="n">
-        <v>46073.39930555555</v>
+        <v>46073.55208333334</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Kildare Death Notices for today: Friday, February 20 2026 - Kildare Now</t>
+          <t>Polizei-News Bamberg / Schweinfurt / Würzburg, 20.02.26: Zollamt Schweinfurt intensiviert Kampf gegen Schwarzarbeit 2025 - News.de</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Kildare Death Notices for today: Friday, February 20 2026 - Kildare Now</t>
+          <t>Police News Bamberg / Schweinfurt / Würzburg, February 20, 2026: Schweinfurt Customs Office intensifies the fight against undeclared work 2025 - News.de</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 10:00:00 GMT</t>
+          <t>Fri, 20 Feb 2026 09:54:02 GMT</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxNSTFFSkdXdUJsYWtmMHloQ1QyOUNQc3R2UngtM1VQZElxOWVzYm9BeGg4WTF2dkxIdGRKUWVUc25hdUZob3dOX25wSUxhcHJVM0ZsekVQRHBITjBxeHhpV2hRNXcyYkprRzJ6MUlpaUJ1SjhSUUgydmJoazg2MUhxRDFpcWdLZGhLNk1iZXpFb1N2R3R4eE9zMFVnbFpLSnRFNVJWc01tQ1kzX2s?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPT0gzcXJvcDBRa3pZM3AxVzlTeldTSVU5aGVZSmMwclE3STQ1RTE3c2RXNW9abjg1QXY3ZTQ1UWs1ZVUxX0o1R1BITEdWYmVncXd5aXB0MnlrcG5YT29DS1JTQ3pnb2dBMEZ2RU1kUTV6THlBeXlUejJjTlV1cXpZS01YRUU2a0ZEWmtTdUJRQTQ5eFh3THEtU0RnOEdaV2dleUltLXpSaHRtZUxRdlFV0gG0AUFVX3lxTFB1WmM1eFdVSHVJTVVXN1F4dTRsRkpaaTVWTFZxVWVwMG1JdENPelhXVndjX01Gb3p1NndvblN5WjJPTWdUMG52eFcxOWxDenRSWnBvb0tCUllITTJyNmZDR2t0S2lqbnVnZ2dBMkhIRnBOLXNpbmZ2bnJ2b25IOEtoSmROUDlfajRpLW11Z01lTzUzS3VGZS1oTHZybmxBYkFXdmszQXdtRzJ0Z05lOHozNGFuSQ?oc=5</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2660,52 +2660,52 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K41" s="1" t="n">
-        <v>46073.41666666666</v>
+        <v>46073.41252314814</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>‘Unprecedented’ demand for jewellery helps retail sales surge in January - Bicester Advertiser</t>
+          <t>Demo-Termine heute, 20.02.2026: Wo gibt's am Freitag Demos gegen AfD, Menschenhass und Rechtsruck? - News.de</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>‘Unprecedented’ demand for jewellery helps retail sales surge in January - Bicester Advertiser</t>
+          <t>Demo dates today, February 20th, 2026: Where will there be demos against AfD, misanthropy and the shift to the right on Friday? - News.de</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 13:31:56 GMT</t>
+          <t>Fri, 20 Feb 2026 13:25:00 GMT</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxPV2w4cTNCTFlMZlA5R3d4VklDNDVJVUJGWFVKSHlDVHVHYV9HQTRwLXd2SUFvckladTMwbzFlUHl0Y3g5M1FzM2NrLUxEWHg2TlNqRGZ0UXJic01oNTJrTWJ2OTliaHZZcnpta2haVkdIMkFMc1h2Z3FsTjRHekU2aUJ5S3A0VmlkOE9ia3BJdHZqRG5CbmR6MUt5ZVc0MzZrYk1vc3pkRzdGcVB4QmhjWGR5c3pTX2VsU09LNTJiOA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigwJBVV95cUxNWTdIQ1g4R3pnTEZCSHU0dFZnX3M2OURENy1obTNCUDBjQWFQa0VZTFZ5RWJoRFl5ajY0RGktdXBvOTZZbXo5QU4ya25BVlhKVjJHV1ZEM3pfR0dfc2NPRDAwMTJtcUt3cTlUZWlUZ3FvZEV1bUNaUERVeWxjWW5rMzFqSnY3LWVoa0ZyUFdJa09UamZlVUs3RHQ0c0JvemxJYzZWajBpNk1MSGVqNlYzY19rbi1YSGdFQ3ozMW9oNE5GbVBsOTRkNzUzeTRranhOY0w3RldDZGZNZHF1NUdyMFpiM3pvUWQ4S0JnSXpiTDhnbVVER2RWak1jNWZWY215TG5r0gGIAkFVX3lxTE1QblRoS0tQdEFtdVNHdzQ3YUIyb1pVOEFmeTk4NDRVb3RDNTVhYW1rVmN3RmlZd0NYeFpaVTR1VDhFakNuYWpLY0VzLURIM2VMUlI2aWNtS1VzUjRVZFkxV1IyQl9vNm1LdjdqWnVQZE0zOElnc082VDE1Vzd2UUhHcThnRm1sMzNyLXpyRTh4REdFWEptVTF1dmdFMVhKb2RUTGsxclR1WVhiYkY0dWV2ekhuTERlUkhUaExhOXNuQXNXWlVhRUNLVlUteWZpOE1mb3lpSXVHa01VY0lWeW9XSHA3UlV0b2RJRWlFVXJhU2o0QndFdlhUdGk4VWhZLWFGWXk2Z1hKNg?oc=5</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2715,52 +2715,52 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K42" s="1" t="n">
-        <v>46073.56384259259</v>
+        <v>46073.55902777778</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Riverbank Arts Centre and Kildare Jazz Festival announce Hayley Kavanagh as the 2026 Emerging Act - Kildare Now</t>
+          <t>Polizeimeldung Bamberg, 20.02.2026: Einbrecher entkommen mit Tresor - News.de</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Riverbank Arts Centre and Kildare Jazz Festival announce Hayley Kavanagh as the 2026 Emerging Act - Kildare Now</t>
+          <t>Police report Bamberg, February 20, 2026: Burglars escape with a safe - News.de</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 13:30:00 GMT</t>
+          <t>Fri, 20 Feb 2026 11:35:02 GMT</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxNT0xWZElNc1lMTS02WWIwU21RemFTUmpsYVEtSTdTc3NZdW1NQzdVTExzNzlWMExCU1dlajluQzZjZmItdlA4TlJ2T3JRSnZ4MXp1YW5VOTNTSnBTblJja3IyLURGV2pYY0RDdkRZX1QteFVJRHdZNDFuVHZVcmdzcmhKcUhhcTE1TzFtYk9aRGw0azZNMmdFZE9xRldYajFXVG1FN3NZSTVvYkV5c0ttMk9rOHVZS2o4Nk9PSkJvVjR1alE3dW1NZUItZW1aZW9INEJXdTg2bE0zcTFVc0k0a1Q0OTRIdWla?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxQTDRVeGxRTzBmZ200OEl2d2huS2VhcFZvTWxucWc0VVhaQkJzak96dW51NEt3V2g3SC1INEZmWXdjbDBVbVRqeDl0NDBqYzJZSHV6Vllwa1NXbC1YRGRLWkpmbWFKdFBHSW5WWVFLQW1vb3hfeWIyY2R1bm5EUllUTkRtLW5iQ3phV3pNSjF0S3dyYS1XZzZkOTd6NG9UWFY1c3Qw0gGoAUFVX3lxTFBlLXFyeU1ONEpmNEV5bFpuQUV6V0lhazdlY21XUFpZaUpVUVFEUVBGbjItWEJaX3ZxWVZpSW1UczJCak9DNkxiMW9NTFhZeXhDUmR0R3M5WGFJbjQtUjN5TldKbkdZOVIyVTVKcUZJd2VHdjdBektOT2ltZ1VwREZDSmFqWVdKeXVBbEhZcGRZYXAzTjhDOW5wX1o2d05SU3RwOTdCSTk4Xw?oc=5</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2770,52 +2770,52 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K43" s="1" t="n">
-        <v>46073.5625</v>
+        <v>46073.48266203704</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Village Wertheim (fallback)</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Cautious optimism expressed over Kildare bridge project - Kildare Now</t>
+          <t>Business of Healthcare Summit welcomes another packed house - Florida State University News</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Cautious optimism expressed over Kildare bridge project - Kildare Now</t>
+          <t>Business of Healthcare Summit welcomes another packed house - Florida State University News</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 15:05:00 GMT</t>
+          <t>Fri, 20 Feb 2026 15:22:25 GMT</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPVjJER2xhQ2VUa1owNjFaMWRKVnpFcnVoZ0N3UjVlcHhIWlJ3N0VyelU0WDZlNkdLMVlQX3ZvVkpiTnhELTBodGk5Sk9wQzR6eGxtQ3QtSVVXZlg0NGhqdkhSQlVaWU9laktQQ2JRNTl1RVRwQnlJX0lJS1QzQ2IwcmpSQ0h5UmVKR1Q4MGJYY19aRW5ZSHRGdGU0dDQ4a1J5RDhiOFZFMk5MOVF1QnFnRw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNb01GazY5VElxMXdSWmg3MnpPcFFIYy1pM1FzTFV6enF3SG81MzhFS0xPNzlDUzZCcm5aMXF6NzdEanlKRnpFbHBuNVJqSGN4MU1sUGIzYTZUWldieTF5UHhrQVdQbmZaT0pOOV9QYTZBbTFvdlc2dlVSaER0QVFGQ1Rpc2N3Tlh2WDFIUlZTM1VXYko5YVZZVk5jZlJMb1ExYWVpUnNhamRqUTdPUUIxaUJNNFpONXNU?oc=5</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2839,38 +2839,38 @@
         </is>
       </c>
       <c r="K44" s="1" t="n">
-        <v>46073.62847222222</v>
+        <v>46073.64056712963</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Village Wertheim (fallback)</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Sadness as long-standing Athy business to close - kildare-nationalist.ie</t>
+          <t>University of Florida expands study abroad with Antarctic expedition - Gainesville Sun</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Sadness as long-standing Athy business to close - kildare-nationalist.ie</t>
+          <t>University of Florida expands study abroad with Antarctic expedition - Gainesville Sun</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 14:24:33 GMT</t>
+          <t>Fri, 20 Feb 2026 10:02:00 GMT</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNVEN3ZVJBblhZYjJSVUlOUEl0cG91WGxRMGt1X2FtUEdEWXJfZkctREVMWHYxOF9Kd3pBMkNiTzA0NGlTNi1obnY1N3BQTjRieUxhMTRhSDNLTDVBWjNxdHpwUTZBQy15dTI0QTJ4eGh0alJ4Q05TZFplYkVnWTAwZGZCQkowbEo3ZnFReHdIR0Z1Unc2VDZnTld2V2VnQ2FHZ1VtRkVB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxPdkVfYlpLQ2ViMnBuUy1hUUtTYUhZbFhiUlNHeUJ2cEkzT3QtWEdBcHRDS2tnZ0dWSVBSZ2tGRnUtYjBHbnB5eVN1Z2gzWUtlZVNTZXR3UFZiZDBsQ1NaRWJlNEcyNHlUbWhiNDNlMjMtMjJkaHZKVWtOVGJ2OG9mZm1qWmVRWkFQaGRSaXlnSGM4NzhuSlkwcWplaTF2dXVHMGZjVHZzSWxtdW9ZWmtnNkpVQTVHZjlaMVRSQ0FKR0lWT01zcVROVi1nQnl1NV9NR2p3ZkI2X05Ua1k?oc=5</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2894,38 +2894,38 @@
         </is>
       </c>
       <c r="K45" s="1" t="n">
-        <v>46073.60038194444</v>
+        <v>46073.41805555556</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Plans granted for residential development in Athy, Kildare - Ireland Live</t>
+          <t>Autobahn gesperrt: Getränkelaster rutscht in die Leitplanke – Unfall auf A93 - Augsburger Allgemeine</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Plans granted for residential development in Athy, Kildare - Ireland Live</t>
+          <t>Motorway closed: drinks truck slides into the guardrail - accident on A93 - Augsburger Allgemeine</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 12:33:30 GMT</t>
+          <t>Fri, 20 Feb 2026 10:46:49 GMT</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPNVpadk9wS3hjS2dUTmp0dmJ2T0JLTlhiLUhybFk1X2RSS3FMU29ZZFc0VUNaODNRQVZqYjhYRVRtSDdycWFZNXMyUkI2X1c5ZEUzNGRkWjA1RWdReDZzQnA1U04tRGo4U3pLMkdEWFZlOXV4S1lYclNYRkMxTHdiY0NGeng3RmRaVGF2TlY3Z0tXaWpwUVhLRDVTOUZiREgxY1gwTnJBUlF3ZDNTSmNZTVdzSnBSdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxQb2RxcW1rQ0l1LWN0UnJ6c2RNXzdPdGJwbW9IWjlSN3czX1NaRE9LSGIyZ0JuRi1aWTFrVFBHTEdmaFdUZXZ3T3NRcmI3dHp3WkF6NGYxeUtjLS1XUlZROW5jcG0tS1lCdEFGZl9ibi1VLUFoSjFnS3pmc3E3VDdkS2JBNWRUX3hhU05qcThTM29hWTFXLW5temVmR0w0QzBsbWZKeFJtZnZlUjE2YVNPVXpMVWZWNlN4MHFFY0h1Z0lkX2VvVnhuNHBxTnV1dWxKR0NBZDcyQjVyRFVMM3NDRw?oc=5</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2935,52 +2935,52 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K46" s="1" t="n">
-        <v>46073.52326388889</v>
+        <v>46073.44917824074</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Home from home for Byrne’s first pro fight - kildare-nationalist.ie</t>
+          <t>Vollsperrung der A93 bei Wolnzach nach Sattelzug-Unfall mit Ladungs-Verlust - Pfaffenhofen Today</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Home from home for Byrne’s first pro fight - kildare-nationalist.ie</t>
+          <t>Complete closure of the A93 near Wolnzach after a tractor-trailer accident with loss of load - Pfaffenhofen Today</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 11:51:12 GMT</t>
+          <t>Fri, 20 Feb 2026 12:23:00 GMT</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOcFllajRWcUNjNkZLTjVZdGNSR21TR2VvYk5ISUlza3JlNEVsRGxmcWVOVm9nR3piZjVmc0djMS0yM0V4YTJjUmJKSEdHWEZqWTRrbm1EM21EWG0zRkY2QlI3bmZpcjRXdXBFQTEwenhuUi03aDFScmI3THRHcnpFM1BTNmhtTnJxMlpWaGltdXZna3h0cGJiVnE4X0ZQUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTFBmdXlwZFk1ckJ3R05ia2YwTVNwcm9xTzY4VTBpREN3REYxMUwzMzZ0SkFOeWpHQ25yR25mNWs5M2xvSzBXcV9uTHdLLUUwcmdieFJLS1JoMHBkbjdfTUN0N2tjV2tUU3c?oc=5</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2990,52 +2990,52 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K47" s="1" t="n">
-        <v>46073.49388888889</v>
+        <v>46073.51597222222</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Village Ingolstadt (fallback)</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>TII urged to discuss controversial Kildare cycleway project with councillors - Kildare Now</t>
+          <t>Why the Audi A6 e-tron makes me thankful for wing mirrors - evo.co.uk</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>TII urged to discuss controversial Kildare cycleway project with councillors - Kildare Now</t>
+          <t>Why the Audi A6 e-tron makes me thankful for wing mirrors - evo.co.uk</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 13:05:00 GMT</t>
+          <t>Fri, 20 Feb 2026 17:59:48 GMT</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOdzVpNUNBTVJnOUtlQ2NGUVBYaWxiXzZSeHZRbmptX3l2dFVacHBMYk8weldFcEFCaEVLTnlDamgzTkw2a1RwalJ2SkdnbGpJeW92Zy16UXByV1lWSXBhQ0Z6eG5ya18tNDYwblkwa0hVS1ZxYjBqX00tNjBNUnpCdDQ0VDVxbXhVWW91U05WRElHdFpySmY5SE53VnFGWm83RlNSY2pQNjlxYlBLMXJ3TWlRSm5BM3FoNHJZLWlLMXhBTTV1?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxQZDhCYURsaFYtb081ZzlCQ1ZyQzdnRHB3OGU1OEozWVVlTmMwbEVSanFlc0IteFlwdkVQa1hSU3FFVlVlNnAyd2RDZ2I2eW5PT2FPUTNiaWNuSTFaVXlUSEkwWXVETXJPSTc1Z2g0ckFoZ0lKRjd6QUlmeXQ2cjBKQVVheXRDTnl3cEJNOFpxYXVxMHZ5bmIyVXNpeTVRcTM3ZGJEMlZPSEJSUQ?oc=5</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3059,7 +3059,447 @@
         </is>
       </c>
       <c r="K48" s="1" t="n">
-        <v>46073.54513888889</v>
+        <v>46073.74986111111</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Village Ingolstadt (fallback)</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>New attendance record! Remaining regular season games sold out - EHC Red Bull München</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>New attendance record! Remaining regular season games sold out - EHC Red Bull München</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Fri, 20 Feb 2026 11:30:00 GMT</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPQmRWY0VOQzRiY3U1amZfOUIwSVplbGFjTkpXUGxfQ25IWjQtWlMyN1gwcmMtVm1LSnNBMzFGYnJaYklsMG1RdG15R2JBVWFXcHF3R1NGUmZGcHpUSGFnb0RhdUZVXzBCMlJKbWs1ODJ6WHY0Si1rMkRXZmVUaFZZU2lCZnNzUnhWdmQyaXkySmJ5R0l6QlBqV04wMTMtVHJKZW5oN05PT3RtZktCNWVyS2pYYUh0UGZ3RVE?oc=5</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K49" s="1" t="n">
+        <v>46073.47916666666</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Village Ingolstadt (fallback)</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>FC Ingolstadt 04 vs. TSV Havelse - Boxscore - Live Score - February 21, 2026 - FOX Sports</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>FC Ingolstadt 04 vs. TSV Havelse - Boxscore - Live Score - February 21, 2026 - FOX Sports</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Fri, 20 Feb 2026 11:37:50 GMT</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxPT3BDbXZudFp6N2FtcVBuSWpWQmhTTVNWRkNlbk9mVlRSLUYwTW8zTkJ0ekZRcDUtYlNMMWI3bERueTNIRms3YTA5LUhNX25DaGlxZDc1eTkxZjFLLV96bmdtb0g5bDU2NVc3c3lOQWdRYWcya3BEalJKQ0hKSnFBY0cwdkRBc1MyanNfSTBLaDVhTklTSVpiMms2RzNydDl2bXZ0LUVld0lMemZCQ29nbnZtUW4?oc=5</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K50" s="1" t="n">
+        <v>46073.48460648148</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Village Ingolstadt (fallback)</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>News: New Audi RS 5 PHEV: Up to 639PS/825Nm, 8-speed gearbox, quattro AWD - CarSifu</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>News: New Audi RS 5 PHEV: Up to 639PS/825Nm, 8-speed gearbox, quattro AWD - CarSifu</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Fri, 20 Feb 2026 09:08:29 GMT</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxOd3M4d3l4OHplRHNoNW1EYzBiVzkwNHRMcFh6RWRKRWFEUktLWXJQbzVab3dKSVFZSTYyMDVMZE0xenFEWUNWU201Tk85bXJudnlKOUdVaTlXS1puRmhybzVZa3BJcWpJN3NxNEFSUjhBZFFvcVNDYU03Z3pJMk15RTE1MURBLWUyYUwwQWVzdGtrS0tWX093?oc=5</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K51" s="1" t="n">
+        <v>46073.38089120371</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Village Las Rozas La Roca (fallback)</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>("Las Rozas Village" OR "La Roca Village" OR "Las Rozas" OR "La Roca") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Surprising results: why more parents in Madrid are opting for gadget bans, making unexpected choices for the sake of family harmony - russpain.com</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Surprising results: why more parents in Madrid are opting for gadget bans, making unexpected choices for the sake of family harmony - russpain.com</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Fri, 20 Feb 2026 09:18:53 GMT</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPekk2OFAwVk0tWG5ua3NUdkQzQXV0T1B1WHpraDZIckNOeWZ6dHpkMjRQc3JKb1pkSV9WMkltZkdzanVQV0VtNmRqRTBBNXI0TWNWRjY0SlpuUV9uTHFuaFctbEJ6cWRKYm1kc3hjejhTV1pXMU9hOV9GMVpYcERnc1VwWGRkakNqNl8tcENveENHeGFaZHZZWVZUalA1WHMtWXkwNGpaTGxUbTNwWXow?oc=5</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K52" s="1" t="n">
+        <v>46073.38811342593</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester outlet" OR "Kildare outlet")</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>See The Guests At An Exclusive Preview Of Kildare Village’s The Edit - The Gloss Magazine</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>See The Guests At An Exclusive Preview Of Kildare Village’s The Edit - The Gloss Magazine</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Fri, 20 Feb 2026 17:55:26 GMT</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOMkxfOWp5U1FDTThlcGN2UV9HUUV3SXp4NlppbE52Ym0ydGpNMTc3b2d5RnZmLVVfQUpiYVRIM1A3b1RWNGsxTUJGelRNeWNBZU9MU1ZDdmZaVzVkeFJ3Rk9zeDNSY09pbkd0QnFVaFFJSXdYVWw4NVQ5M0lqMkwweG9YNkF6RDJtcFdudG5EQXhYUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K53" s="1" t="n">
+        <v>46073.7468287037</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>High Level City France English</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>("Paris" OR "Île-de-France") AND "France" AND ("bomb threat" OR "suspicious package" OR "shooting" OR "stabbing" OR "terror attack" OR "police operation" OR evacuation) AND -Texas AND -"Paris, Texas" AND -film AND -movie AND -football AND -transfer</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Bomb threat in Paris as major landmarks evacuated by police - The Mirror</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Bomb threat in Paris as major landmarks evacuated by police - The Mirror</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Fri, 20 Feb 2026 21:57:21 GMT</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxORmk1NjhhUjlMSTNZOVJJb2luVGwwXzlNZVNhUFFMOU55VUs2cllsellWdENXUjNuSHBCRVZlY2p6X1paTVg4LVlHWlNzbnMzWllhWlJ0Sm1mSnNmQVZlZXdSdUdrdHBjWTVpMVI3cmp4LTZrQlQ1dUdhcFQ4NDlITmF1SnBfcm1nUkN30gGQAUFVX3lxTE13b1hBY3Bsb3luazcwcTIwWTRnM2lIN3VKX1RzZFNEbk8xVExIVWhyYXNqcS1EbjZoWUZhQ1JHREtyc2pLdnZkNGVORG1FbnNVMmtvUFFqS3lpd0pJdWFGc2p5QURxengwUUFsa29kVWpsbFdjc2VFbFNlMlpSNExNeVNmNGp3Y2h4a2NpazBaVA?oc=5</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>FR:en</t>
+        </is>
+      </c>
+      <c r="K54" s="1" t="n">
+        <v>46073.91482638889</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>High Level City France French</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>("Paris" OR "Île-de-France") AND ("alerte à la bombe" OR "colis suspect" OR "menace à la bombe" OR fusillade OR "attentat" OR "attaque au couteau" OR "opération de police" OR évacuation) AND -immobilier AND -"prix immobilier" AND -foot AND -transfert AND -Texas</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>INFO BFMTV. Tour Montparnasse et Sciences Po évacués après un signalement: levée de doute terminée, aucun engin explosif trouvé - BFM</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>INFO BFMTV. Tour Montparnasse and Sciences Po evacuated after a report: doubt cleared, no explosive device found - BFM</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Fri, 20 Feb 2026 19:22:16 GMT</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAJBVV95cUxNRDdZR2stLV9SN1dDaG9yTlUyN3VzUEpVa2VpVnc5ZXQtX1FoR0tVWDlpXzlhSW5xd1FDcVNBSzBPdGtwLWpnQ0RTRy1TcTUyRGFNbG5nM2RrSkdPZVU1Y0pKUFlsbG81SVdqaWZyaWdfVXlOVUxUNnhMN1VUbGtWX1lwTWM5ZmUyNXdHOVFlUy1DVFpQa3lvVW1mcTh3b0hYX3E5R0wtTW44N1M1bHhpX1V1MGFPVnd6bzZwdUVudjJmVGNhSjZ3NE1fQk94RTh1RG5DOXdseVZtb3hhbGNwckZXTlZBYXBfeGlsUlZhTHpvR3NyWXhJZW9acEZIaWtBa2psbTJSSG1sWkNS?oc=5</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>FR:fr</t>
+        </is>
+      </c>
+      <c r="K55" s="1" t="n">
+        <v>46073.80712962963</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>High Level City France French</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>("Paris" OR "Île-de-France") AND ("alerte à la bombe" OR "colis suspect" OR "menace à la bombe" OR fusillade OR "attentat" OR "attaque au couteau" OR "opération de police" OR évacuation) AND -immobilier AND -"prix immobilier" AND -foot AND -transfert AND -Texas</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Alertes à la bombe à Paris, Sciences Po et la tour Montparnasse évacués - 20 Minutes</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Bomb alerts in Paris, Sciences Po and the Montparnasse tower evacuated - 20 Minutes</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Fri, 20 Feb 2026 20:17:00 GMT</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOcVFrb1pIOGJKdlU1OGIzRHd5dnJsZXY0NVBWbE55RmJ1QU1uS0NqYy1ESXBpdER6OUtZZ0JQVVdUdm04SzEtaENGN0RaWExiV2FHSGpuVUlVOGtmTzRXcGpKTlVUSjdSMXN3aXMyUGk1OUp4Z2NwZWtRbnlrRTdjM256NDhNNDRZXy1Lbk0wOHAzTnlLOTZhTXBnd1N0VDE1cVJRUmhPZTN3Vi1kdlRjWU5HZjZBU2R1dzlkZmxlMFBxMHRzWEpQekV3Tm8xQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>FR:fr</t>
+        </is>
+      </c>
+      <c r="K56" s="1" t="n">
+        <v>46073.84513888889</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-02-23 08:02 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K42"/>
+  <dimension ref="A1:K64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,32 +480,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>London Marylebone Incident</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>("London Marylebone" OR "Marylebone station") AND (incident OR disruption OR closure OR police OR bomb OR explosion OR stabbing OR shooting OR "suspicious package")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Chiltern Railways to be disrupted by work on Tube - AOL.com</t>
+          <t>Europese dag van het slachtoffer: Linda getuigt na steekpartij in Veerle-Laakdal: "Ik sta sterker in het leven nu" - rtv.be</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Chiltern Railways to be disrupted by work on Tube - AOL.com</t>
+          <t>European Day of the Victim: Linda testifies after stabbing in Veerle-Laakdal: "I am stronger in life now" - rtv.be</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 22:32:35 GMT</t>
+          <t>Sun, 22 Feb 2026 14:02:35 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQOGNjVDdzNXFXVEZHMEFmaGdnaVZTN1UzZ0txV1BGYzc1dm5CLTg2dmEtSEdYSVBlN3drRUVGSmJrNmg4QWxkdUd3by0wN0ZIRVNJd3c2cDJqenFCTnNyWTJyZnlEUVZ4MWFaU3p5LUJXNzNRWEhBVEVjUTQ1U2o2aGJn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNLUxWTXZSNktaZVNZaFVhMlN0djhHazE0QVR0a0l0QTlLZUQ3a1ZUY1RyUFE3Wlc5aTZhN0ZXWmVFX3lXMWFqcUtESW1Pc3dOYVJVZTRsNnZXRVp1Z3ZmcUVpODJfWDVoc2YtODJjbVdRWEg5ZENRbHhnQkNZMURwNU1ZX2MxSVZDb2ZOYWZaTWlCUGI1RllSRkJ5ejJWZllBT3I2cU5UMWF1SUtJYWtyZkVVMW1sWnhH?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -515,21 +515,21 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46074.93929398148</v>
+        <v>46075.58512731481</v>
       </c>
     </row>
     <row r="3">
@@ -545,22 +545,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Schoten gelost in centrum Brussel, verdachten op de vlucht - BRUZZ</t>
+          <t>BBC tipt dit museum in Brussel bij ‘zes meest veelbelovende openingen ter wereld’: “Een absolute mijlpaal” - HLN</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Shots fired in the center of Brussels, suspects on the run - BRUZZ</t>
+          <t>BBC recommends this museum in Brussels among 'six most promising openings in the world': “An absolute milestone” - HLN</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 07:37:20 GMT</t>
+          <t>Sun, 22 Feb 2026 16:45:55 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxPWmo4U0ZjR3FRZk92dVJHZnhpUDBLY0hsMGc5SWhZblV0T0tfMllRNHEtLTZmZW1fZEg1dGE3NXFobHd1QjRMeUkxcW14YWM3R2JCa1E5RVg5SzZBenFmWi1pVkgtLVE0MXZ0dHdLVWZGZHc1cmxzQW0wY1hkRnFhU3NfMmpWb1B5N1VQWTJ1UndNcFRPbUx0Q0JOOFI0d0tQam4wNldB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxNbWtyZ29waXdQa2VEaV9MZWZyTlJtclVEc3g1bk1oNGZsTjdoLVpXcGZwRFgxbnN4aXJvSl9BUi0ya0xETFhiRm9nRXUzRE5jclcwVG8zcHpveXFla3JQaFUyLU1EMFV4eWRmYWpRSF9ENVhkcDA4NlQzUXk4MzRiZVN4aGk4QXBzSXI3WWVfVnRIRjk5M3hiVkgwUlg4c204R1NoWDNHRG9vYTRFYXhzbnBpQVdFUktBYmFwX0RxVDVWOS1MbE9iaXZZWWhORS1wV2RLTg?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46075.31759259259</v>
+        <v>46075.69855324074</v>
       </c>
     </row>
     <row r="4">
@@ -600,22 +600,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Explosief ontploft onder auto van volkszanger Frans Theunisz terwijl hij in Lanaken op het podium staat - HBVL</t>
+          <t>Ruben Van Gucht in shock: 'Bekentenis slaat in als een bom' - VoetbalNieuws.be</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Explosive exploded under the car of folk singer Frans Theunisz while he was on stage in Lanaken - HBVL</t>
+          <t>Ruben Van Gucht in shock: 'Confession hits like a bomb' - VoetbalNieuws.be</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 14:24:32 GMT</t>
+          <t>Sun, 22 Feb 2026 19:43:00 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxQSWlUQ2V3U012MWRWY0JOTGp0dlFiTVpoblhvUUk0NWJzdEt6aHJhcV94RElKX29NbG1xbmpLSlE1bXdxeW1RUFZCb0NLWExKNTJjU3R1WXBOclJNS2k5MktaOUVsOW9MTFpmVFNWSS1SbE9HQkQ3d2lFSWhLdnpPRC1oOEZqY0ZNMG1QSjR0a0tHLVFlemtYaUhpdERYN19NOEV5MEJ6S002bVZ2VjRnNnhvaklaMEJzSjVxc2JQUS1zMlRpMDc2Yml1LTVyYS00ZkJFazlQZFNhVVNta3FMbzYxU21WcWc4X2N2ZkdNYTM0dw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxQNTBkNjR2dWVMcWRqcEp5MmM0eHZSenlEOWVsejhsOXM2aDZsdHhKMlI5Vm16NHJreWM0MlA3WmQ3LW5WUTNxMVg0bS04dFFtYUdpbHNfT256QWhHM1kzVDQzS0ZtVjdQLTZlWjJvaTR3WjNDQWRzNEhyNzgxV3c5U0FpaUYxXy10alJUOFNCYk5GTWlTTlVVZkw5VFluM1lBVkE?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46075.60037037037</v>
+        <v>46075.82152777778</v>
       </c>
     </row>
     <row r="5">
@@ -655,22 +655,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Geen gewonden bij schietpartij op Anderlechtsesteenweg - Nieuwsblad</t>
+          <t>Explosief ontploft onder auto van volkszanger Frans Theunisz terwijl hij in Lanaken op het podium staat - Nieuwsblad</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>No injuries in shooting on Anderlechtsesteenweg - Nieuwsblad</t>
+          <t>Explosive exploded under the car of folk singer Frans Theunisz while he was on stage in Lanaken - Nieuwsblad</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 18:56:10 GMT</t>
+          <t>Sun, 22 Feb 2026 23:10:54 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxOb1owRUFnMEhDaHZROVZmd1R3alZTWHZFRlVIRmx5eHdQVDlBeXI4MXBWcUVuTl95OWIxcDRuTmxLMnNySWlDOENpMnMweHBYeTBEMkJnSnptU0ZjM0NXM2FTREtPSDNQY3l1dTZrZEJVQy1la1I2UmM0OVBicVBSWk14S0ZSaGJ3amVDM2otNGNBSlRPWGJhZFF3VGx0M1RhNXNKMUs5MlNvc0hmOVExMlRDdGtuZ3ZZ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-gFBVV95cUxPS1Fvczk4VGdrakpKT1VxdVNfZGNJZXc2LWt1dHF4S184U0MxNXdYME5xOVNzbG9oT05wWkVKQnhnZDJVUy1BT08xbWVfZ2NoWVc0TVpieDBtTEt2eF9BNjQzNG0tZDVKVnV5ZDRpRFh4b0t0TUlfUVMwckZoYkp3Nk84SzVVVnJDWjgxY0hLWGdFd1FEZ0NjYXQxNllySlhuekVQbW5qRHdMVGs3bTdRVzZpdHNqM2hKN2hRQmY1al9EUnNCTlBhVEkyVjU0LVhuYXJiVnBZaFFDTmhzM3FDcUxKckdxZ1d1T3VPQzJFUHg4Nk1LeFItNW5R?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46074.78900462963</v>
+        <v>46075.96590277777</v>
       </c>
     </row>
     <row r="6">
@@ -710,22 +710,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Prinses Catherine laat zich voor het eerst zien sinds arrestatie van Andrew - GVA</t>
+          <t>Hoe deden de voetbalclubs uit Tervuren het afgelopen weekend in hun reeks? - HLN</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Princess Catherine shows up for the first time since Andrew's arrest - GVA</t>
+          <t>How did the football clubs from Tervuren do in their series last weekend? - HLN</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 18:23:06 GMT</t>
+          <t>Sun, 22 Feb 2026 18:40:18 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPLUtNREZGT2ZldFIyQ2tUVzVfa05hSk41ZWJFQm9ReTI3TXY2aU4yMGpwQnJ6OXkwZ0hpdXVnV0lyaVpUM3N3bDZkcWhBOS03Q0ZxNnY3SWR4R2VEMmpwZjZIaGxjTGgyRDU4VjZQdFdfVVVER2hScnNaTUlCVzF2VlN6cEM4eFFYcDFma2pDMjhiMk1YVHh0cjdPREZrS1VzUk9UdHVSWFhOcFplbC1xMDNRRElkR05Hc3NRRQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxONS1jbXYyX0dkQ3JGVWViM29ndnp0dmZualdpMFBqbTR2NnpwdlJ6czlCbWdiTkV5emxzcEZHcjlRblFsM1lOX0lnX1pKa3NxNlFlMDBEV2J1VHhYSFljYTF0djZQZFdua0VPb2pHWjNfUEtYSTMtNm9PX1RfVnl3aVdGV0ExM2RxUVB2U29ybFN2blJRckZKRXVhdlZaZmZqdnNVVjZHNkJGcFQtLTRiRHdnYmduS1Iz?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46074.76604166667</v>
+        <v>46075.77798611111</v>
       </c>
     </row>
     <row r="7">
@@ -765,22 +765,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Chinees Nieuwjaar kleurt Antwerpen: leeuwen, luidruchtig geluk en veel traditie - VRT</t>
+          <t>Berlaen viert jubileum als singer-songwriter met dubbel concert in Knipperlicht: “Mijn tweede thuis” - Nieuwsblad</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Chinese New Year colors Antwerp: lions, noisy happiness and lots of tradition - VRT</t>
+          <t>Berlaen celebrates his anniversary as a singer-songwriter with a double concert in Knipperlicht: “My second home” - Nieuwsblad</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 16:56:15 GMT</t>
+          <t>Sun, 22 Feb 2026 10:22:36 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNMWNfbFZxeW5nZXY3VXZNblQ5aWJ4M3lBcWV0Y2tTcUdzWVNoaEJjZGcwTFg4bkJqSk4wY3QxbEdjMndlVURicjZhQnh2MDl5VHpCSzFCNENOQXBjOUJheU9XbzZ3SVEtczk4VENnVzJzMFhYcjdfVjhUSEpqMmRPMUk2cWQ1SEdPdHFEU3dDNi1Rb3dVMlRMMmZCQkJPUDRxZWFRT1B6OWZ6T050?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiAJBVV95cUxOQ2ZNRUx5elg4NGlsbTI4UUdMM0tZZVgtYXpvXzhuUEtkLWN0dHJjeTdjTjVNUDU3bGJfSHNkdkFMMF9FSTBCdEpYVWtuRUpYajBjWHQ1TncxekloMFU4QzA3cV9vUEZlai1qRTNWbHJUcVA4WFFMVi12UG5GWmtBVndlQmcyY3FjaFV2SUVvamhqYkttYjQxSnVkUHJ4ZzUxNG9xclVXVVkwczNIcmJ6NTRnVTJYZTVjM3kzeXlFc2pJaFA3RTltS2pnNk1OWU5sYXhFWjZiYjF0WVBsWTBqVnBQa0tQU0VVcnM2VXpjelFkZjRreExBb2lDS0pQcW1QU1BzZ1FDYzI?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -804,38 +804,38 @@
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46074.70572916666</v>
+        <v>46075.43236111111</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Ruben Van Gucht in shock: 'Bekentenis slaat in als een bom' - VoetbalNieuws.be</t>
+          <t>Explosion and Fire Reported on Container Ship MSC Giada III in Gulf of Finland - 112.ua</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Ruben Van Gucht in shock: 'Confession hits like a bomb' - VoetbalNieuws.be</t>
+          <t>Explosion and Fire Reported on Container Ship MSC Giada III in Gulf of Finland - 112.ua</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 13:46:40 GMT</t>
+          <t>Sun, 22 Feb 2026 20:17:56 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxQNTBkNjR2dWVMcWRqcEp5MmM0eHZSenlEOWVsejhsOXM2aDZsdHhKMlI5Vm16NHJreWM0MlA3WmQ3LW5WUTNxMVg0bS04dFFtYUdpbHNfT256QWhHM1kzVDQzS0ZtVjdQLTZlWjJvaTR3WjNDQWRzNEhyNzgxV3c5U0FpaUYxXy10alJUOFNCYk5GTWlTTlVVZkw5VFluM1lBVkE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOR1plTldVMXlJQTNVdkJ5YWlRNmJZU1VRZXlVb1Vpc2pad0plMEZxWkZXenRVcVVzRnk3OXlBb0JPUFhYUmx4Q2Z3LV9DbG00VmFsNnRKR1RNdjhZUER5a0FiYmdjNk5zdEFydWdZR29mbkl2bzByUHI0X3dDWUZoUUs2bW5wQ3ZReVpFVHJuRlRDODNHSzAxYTBn?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -855,42 +855,42 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46075.57407407407</v>
+        <v>46075.84578703704</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>In lijstje met Obama Center: BBC tipt Kanal-Centre Pompidou in Brussel bij “zes meest veelbelovende museumopeningen ter wereld” - HLN</t>
+          <t>Un homme de 79 ans tire des coups de feu sur une maison avant de se donner la mort à La Panne - 7sur7.be</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>In list with Obama Center: BBC recommends Kanal-Centre Pompidou in Brussels among “six most promising museum openings in the world” - HLN</t>
+          <t>A 79-year-old man fires shots at a house before killing himself in La Panne - 7sur7.be</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 09:03:57 GMT</t>
+          <t>Mon, 23 Feb 2026 06:29:00 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxPS18wMUl6RndXdjExZGZvZUx6N2IzQ3VKYXZvajZodkdJSi1wSnZLZ3VGcm1YM3NCSUF2bnhGenViTElvZDdLUjNwdnpWTGpXcWphdTlzakZtOE91UERQbmo5NDVUOFJLYkszc0s4eVVqaTFIYTlaVzJSWmlTSUtkTU9objhONDF0ckY0bk5GcW1haVVSVXljS2JLQWg5U3d0d1BLRi1FaTVaSzk0eDRaZHBlY3lPZDhUTzJMUDgxUlVvNFc4bVFEZVc3QWl0b2lBZndrNDNwdWZuWmlh?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxQaE1ZcmdIVzVhMVE3bkJxRXdkci1DN25Sa3VQczFQQjN2R2NvQU51S3JuaURxOGtHZ2RTREV5Wm1zT2JWWi1NWm1ydk91eUluWk5GWHpOeDNHZl9SVVJEVG9FVlNwak9mVFM1TVk2anc1WFdnY0RpeWYxZTlCTUhGejJiZ2pPd2lGd3NDaWx5QmZ6Vkh2VHFiTnRqWXhBNmdzN0k5RF9vR05DUHVWVFhYSXM4SWdPanlKa0VHLWdfNUNzSHk5S3ZzS2VUMjNaTnJWc1R3?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -910,42 +910,42 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46075.37774305556</v>
+        <v>46076.27013888889</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Ongeval met letsel op Wilhelminalaan in Valkenburg - AD.nl</t>
+          <t>Un bébé de 16 mois retrouvé sans vie à Berchem, le parquet ouvre une enquête - BruxellesToday</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Accident with injuries on Wilhelminalaan in Valkenburg - AD.nl</t>
+          <t>A 16-month-old baby found lifeless in Berchem, the prosecution opens an investigation - BruxellesToday</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 17:57:00 GMT</t>
+          <t>Sun, 22 Feb 2026 12:40:00 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxQanpMRjRySTZPcTQydFUxQjVXUzhuTXJBT0VxWHh3REpmNFlDY2M4MVh5aV9HQUpoSGRuQ19NMTRXVGIxMXU1c0xCbWZ1VmdpUG01LVR5Znp0NmFtMW9GcUlpODNrSEFVbW55WEZpTG90ekpSb1BhRmJzWGZLLXNNc0YwUDZNNHNJUGdmWV9fdDVBVkt2LVBZdmJMcjJyazZBMUs1dzJET1FWYjdNb1VGMXJR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTE0yMzAzNE9wYTFoTGJBLXdOWHpfRWJ5MUoxUGQxWHlMc09jQWZQY0l4Vm9FWlV0d2dRX2c2bWZTazRZRmg5cnZndmJzdmFXSi03eGhja0Y1NGR0TWIyeE5EcVN3T0RDUzdiYktDMERDZlJ6MTE4S2E0YQ?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -955,7 +955,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -965,42 +965,42 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46074.74791666667</v>
+        <v>46075.52777777778</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Berlaen viert jubileum als singer-songwriter met dubbel concert in Knipperlicht: “Mijn tweede thuis” - Nieuwsblad</t>
+          <t>Il a couru aux JO avant de combattre la bombe nucléaire : pourquoi l’histoire de Philip Noel-Baker dérange encore - Daily Geek Show</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Berlaen celebrates his anniversary as a singer-songwriter with a double concert in Knipperlicht: “My second home” - Nieuwsblad</t>
+          <t>He ran in the Olympics before fighting the nuclear bomb: why the story of Philip Noel-Baker is still disturbing - Daily Geek Show</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 10:22:36 GMT</t>
+          <t>Sun, 22 Feb 2026 20:31:00 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAJBVV95cUxOQ2ZNRUx5elg4NGlsbTI4UUdMM0tZZVgtYXpvXzhuUEtkLWN0dHJjeTdjTjVNUDU3bGJfSHNkdkFMMF9FSTBCdEpYVWtuRUpYajBjWHQ1TncxekloMFU4QzA3cV9vUEZlai1qRTNWbHJUcVA4WFFMVi12UG5GWmtBVndlQmcyY3FjaFV2SUVvamhqYkttYjQxSnVkUHJ4ZzUxNG9xclVXVVkwczNIcmJ6NTRnVTJYZTVjM3kzeXlFc2pJaFA3RTltS2pnNk1OWU5sYXhFWjZiYjF0WVBsWTBqVnBQa0tQU0VVcnM2VXpjelFkZjRreExBb2lDS0pQcW1QU1BzZ1FDYzI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiTEFVX3lxTE12aG1TZFZ1ZE43SkdRT1lfbTByMk1sS1NQQVAteEVGMWI0YmNpcWFtT0pwX1BXa3MtVm9UQ3dLbDhWaXZteXVVNTdGXzI?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1020,42 +1020,42 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46075.43236111111</v>
+        <v>46075.85486111111</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>American citizen killed by an immigration agent in Texas last year, records show - NBC 5 Dallas-Fort Worth</t>
+          <t>Une enquête ouverte après le décès suspect d’un bébé de 16 mois à Anvers - 7sur7.be</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>American citizen killed by an immigration agent in Texas last year, records show - NBC 5 Dallas-Fort Worth</t>
+          <t>An investigation opened after the suspicious death of a 16-month-old baby in Antwerp - 7sur7.be</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 18:07:53 GMT</t>
+          <t>Sun, 22 Feb 2026 13:04:00 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPQW54SkdIdzdMaXZsemJzZE1qTXRnV2c4cGdxSWFHdHRJOTROcGVjTlhWVzNBamJWNURMTHpWT00tVzQ2STNXb2JWTEZzbGlrVDdCWUVkMWxKSU1LTmwtdDRHaHUxMG9QMk9jUkMxV1REVlNvaDVvUUUwaVlmX3lRLXFIWUpCeUszSzZNNGxMMEphSkVBUVFKeDdodUxCVE1ibHVnX1k1c3BMbTDSAbMBQVVfeXFMTXRyXzRwa0F4cWVkNHFLUUN5b3pPa3VxdUZnQ3FSVjJCbTROaFVBbl9VT0V4SUZ4U0ZEMURfVjBKZDlnd1R5Y3FRUFdvak5kMDk0TDJzcWVyUVdUSzZmWGhoMUVHbU9LN2FzQVVja2ZvZUZIMVhubUdpX2xjZURIanplTHZHdjlJTXpGVU5XdUJFZDd1TWtDa21iTHRNM0d0R3NZZTBlVko3bFB3S3RUeEdJMFk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPWlNZaUs0UnI4bmNvaDFjUDdieDV5RUszU09Ud3NGTV9DT3p0cUtBOUxrd0h3LXBnQzJ6U1YxcE4za3EyUGJBUWtFOFRtaHdrX3JzU0pWVFpLSlhjU3pBTkdfUXVINVhtZUd2LXFXUWpJUjBhTjZKLUkzUS1vdy1jcWJjTkFscEVqUkQydTUwY1JHdFB5ZnhQOUktbXR5bW1rak9Hc0NsQVN3RXVrV3piZmt2MmZKZw?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1075,11 +1075,11 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46074.75547453704</v>
+        <v>46075.54444444444</v>
       </c>
     </row>
     <row r="13">
@@ -1095,22 +1095,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Fusillade rue d’Anderlecht à Bruxelles, les suspects en fuite - 7sur7.be</t>
+          <t>Agression sexuelle, contrats abusifs: une plainte secoue la finale de Miss Belgique 2026 - BruxellesToday</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Shooting on rue d'Anderlecht in Brussels, the suspects on the run - 7sur7.be</t>
+          <t>Sexual assault, abusive contracts: a complaint shakes up the Miss Belgium 2026 final - BruxellesToday</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 01:40:01 GMT</t>
+          <t>Sun, 22 Feb 2026 09:30:24 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxPUEVSV3R2eHFabUEwaHNXYVMzOUI1R0pGb2JWZXpEODljRDdIbTZlT1E2aUxLbldLUW1yVW40WktaXzYyQV9QQ2xuMm9QSXhrRnZjUldIRlJMV013dXNIcHNZb2lESDY3ZVJkQzExRExCR3VVZzFPcWFCVzhVX01uTmkzMkVxeUJCVlFyaUVadFRoMkg1VWdIdWVUM1ZoTEoy?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxNWDlJSDhHeGdmcjAwVGxLZU5LbXNtT2R2U3Y2cElYTm9GdUNmczVodkt5N2FDZXNBbFF5YkJCSjFFdXY3NzNEOTh4ZzY3US0yeThIaXMwOFVOeG9XeUxTYTFjVEh0VnEtODc5dTBkOUF2cXJ0cVlFMXZ5X0lYZTNNVWd3THd0ZEE?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1134,7 +1134,7 @@
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46075.06945601852</v>
+        <v>46075.39611111111</v>
       </c>
     </row>
     <row r="14">
@@ -1150,22 +1150,22 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Un bébé de 16 mois retrouvé sans vie à Berchem, le parquet ouvre une enquête - BruxellesToday</t>
+          <t>Grisaille et pluie pour la 2e semaine des vacances, une belle journée printanière mercredi - 7sur7.be</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>A 16-month-old baby found lifeless in Berchem, the prosecution opens an investigation - BruxellesToday</t>
+          <t>Gray and rain for the 2nd week of the holidays, a beautiful spring day Wednesday - 7sur7.be</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 12:40:00 GMT</t>
+          <t>Sun, 22 Feb 2026 11:52:00 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTE0yMzAzNE9wYTFoTGJBLXdOWHpfRWJ5MUoxUGQxWHlMc09jQWZQY0l4Vm9FWlV0d2dRX2c2bWZTazRZRmg5cnZndmJzdmFXSi03eGhja0Y1NGR0TWIyeE5EcVN3T0RDUzdiYktDMERDZlJ6MTE4S2E0YQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPY1NLZFc2MW8ySDZMNlo1LW1GQ0FRSG1jSjhrSHBrNmxtSmpELW15bkR0V0FfRnRzcVhTbXpqOWVieXlDNl9fVFEtUzFWWTRiVWJNcWRUMjZXcF9ZdXU2R19uendIajY5YkNOMG5ENzBZdlVKQnJ4OXpuSVBheHJPcGNkcVp3ZzByNUJoaWRVUUFlaHBqVnYwTXhSZGdfWG9nYmNvdzA0emVLa04wWmMyQUdlN21zODNyZlgyQUlGRUREZ084Z0ZxVg?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1189,38 +1189,38 @@
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46075.52777777778</v>
+        <v>46075.49444444444</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Grisaille et pluie pour la 2e semaine des vacances, une belle journée printanière mercredi - 7sur7.be</t>
+          <t>Moddervoetbal in Hasseltse derby: Torpedo ploeg van de stad na “fysieke uitputtingsslag” - HBVL</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Gray and rain for the 2nd week of the holidays, a beautiful spring day Wednesday - 7sur7.be</t>
+          <t>Mud football in Hasselt derby: Torpedo team of the city after “physical war of attrition” - HBVL</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 11:52:00 GMT</t>
+          <t>Mon, 23 Feb 2026 03:45:00 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPY1NLZFc2MW8ySDZMNlo1LW1GQ0FRSG1jSjhrSHBrNmxtSmpELW15bkR0V0FfRnRzcVhTbXpqOWVieXlDNl9fVFEtUzFWWTRiVWJNcWRUMjZXcF9ZdXU2R19uendIajY5YkNOMG5ENzBZdlVKQnJ4OXpuSVBheHJPcGNkcVp3ZzByNUJoaWRVUUFlaHBqVnYwTXhSZGdfWG9nYmNvdzA0emVLa04wWmMyQUdlN21zODNyZlgyQUlGRUREZ084Z0ZxVg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxOdnpuSXp0Vi1mZFlMU1d1YWlZZWJ6UDc4RnhrZURUcmstVDZjcmlGaFZBLUxYXzZja2ZxRDMwNEotMlc1MVpON2JSV1A5WXdId3ZZZ1l2ZnVLamFtVGxjeXp5cmFLZWFIVkJtZ0hxbkVFdFBoQVpubV9Gc1hFa2lPY1JhemhQMTkxWmZweS1uUkc2d2RJSXA1MWpTZFhKVjMzOHF4a2J1a3lsVkZqdjNwamFuLVY3cTI0ZkJ3OWI5em12Nm9uYURzcWNKRDM2WlU?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1240,42 +1240,42 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46075.49444444444</v>
+        <v>46076.15625</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Agression sexuelle, contrats abusifs: une plainte secoue la finale de Miss Belgique 2026 - BruxellesToday</t>
+          <t>Hasselt stuurt team op pad om hen te zoeken en gaat huis helpen houden na stijging aantal daklozen - Nieuwsblad</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Sexual assault, abusive contracts: a complaint shakes up the Miss Belgium 2026 final - BruxellesToday</t>
+          <t>Hasselt sends a team to look for them and will help keep the house after an increase in the number of homeless people - Nieuwsblad</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 09:30:24 GMT</t>
+          <t>Mon, 23 Feb 2026 05:07:57 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxNWDlJSDhHeGdmcjAwVGxLZU5LbXNtT2R2U3Y2cElYTm9GdUNmczVodkt5N2FDZXNBbFF5YkJCSjFFdXY3NzNEOTh4ZzY3US0yeThIaXMwOFVOeG9XeUxTYTFjVEh0VnEtODc5dTBkOUF2cXJ0cVlFMXZ5X0lYZTNNVWd3THd0ZEE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8wFBVV95cUxNa2U4QXlmQnlGUFNwOVltQ0lpbmtpQXhLMmVVSXB6Vzl1UVFDc2lybG1oRTdnek5pZXlwY1hnU2ZVLTFIUXhvbkdTRXFhaGM3dl9TVUN1SENQT0pRUjc3bkpMR2dqZXZZd0RZcWRGTXJoNFFNdXB6NThoWjNrdnJBMEdPTkIxNU4yNjhlLXkxVFZkMTdJVDVZVlh0TWlGVi1IUmg2Ny1abDV0cnR5bFc3YWJkdktnc2JLT3h5ZzZjb2MzS01TZS1odW83UFFhc3J1MzlvSzJpNnVkbTNFMXVEWXBHSFhVbmg1UWJqOGQwb2x2Y3M?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1295,42 +1295,42 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46075.39611111111</v>
+        <v>46076.21385416666</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>La justice alerte contre le phishing via de fausses applications: “Impossible de distinguer le vrai du faux” - 7sur7.be</t>
+          <t>“Dat zij vrijdag al een match hadden afgewerkt, speelde in ons voordeel”: Hasselt kegelt Lommel uit de beker - HBVL</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Justice warns against phishing via fake applications: “Impossible to distinguish real from fake” - 7sur7.be</t>
+          <t>“The fact that they had already completed a match on Friday played to our advantage”: Hasselt knocks Lommel out of the cup - HBVL</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 06:20:52 GMT</t>
+          <t>Mon, 23 Feb 2026 04:17:12 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxQOHpEb0RWNVpvS08zNmdON0xCMzUwN3VHZ21lcnFtS2syVEd6ZVAyNVJSdmduUy1vRVhpOUwtaV8xSksxVHA2UkNmRm4zQk5oMkpUVUplQzB4QU92SWRFTFNrQjZ6M0g3di1FeW1ZM1dXbmEweV9ISTRzZUR2ZUg5NVNabHdNajZRdE43bElzZVBodU5NUzl5OTZsMGJvam1fdTBVczE4RHc5UE9sd2NkdDFSNEdmNnF0X0ZLMUtzbllsZzhzbDhXVXB2UkF2S0RkN0FPcm1SaW9pNW93Z2c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxPMGFkeXA5YWFTakNwa2tOcHBEZFk0REpKck11RzFwS2J1Y2YxY0RYd2lBVTZVdVRzb3lGQjdaWUNyMk45cTJxNmJIYUpEbjZxTDJwVi1qMFZCc3pPcE9DcEtidnpBSm1hd2FJU3lXU1pzRk03NHdyaEdFblItQ3QwRjR6TzltU21pLW1PVU1GVy1PX3BrS1hnQkV1MG1uWUZuQnF4aHQtWHBVelYyT1poRDNwWC14VVdjMkI4a1IwSngwWk8zNVk2UWUxNno3LW1vVHFiWnhwdVl5N1E5U2p6bnZBYVhtR2FjcVp5Z1lR?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1350,11 +1350,11 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46075.26449074074</v>
+        <v>46076.17861111111</v>
       </c>
     </row>
     <row r="18">
@@ -1370,22 +1370,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Vakantiehuis voor mensen met beperking in Maasmechelen verliest half miljoen aan subsidies: toekomst onder druk - HLN</t>
+          <t>Eerste afdeling: leider Hasselt loopt verder uit, Diegem verliest degradatieduel - HLN</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Holiday home for people with disabilities in Maasmechelen loses half a million in subsidies: future under pressure - HLN</t>
+          <t>First division: leader Hasselt continues to lag, Diegem loses relegation match - HLN</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 10:53:39 GMT</t>
+          <t>Sun, 22 Feb 2026 21:23:33 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxPSGxqbkRqNVpYNWk4RFVLN0hzNmZWY0hXMmN4RnRPeW4yZzd2LXlMeEhOWTB4TnhOSTJPSUR6VFVFVkJjeV9VUUZ4MEd5SGY3OHJBVGt5Q1lSdzAwTkh2clBVV2lhYWUyNFlrYTRkVDBhRTRPdEVpU2ZKVFZWSDhndHV6YlpRN056LVVlVjgweFhUVFJfTGdMYldJQmhROUlxRVZsci1lbGczR3BtRUo4R0FsNElrWk5RM0dYb0pUaFJzWXNhOEUxaGJyQ2dCUW9FcjlfUWhNb1VBdzc3ekJscFZDSlk0S0U?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxQMGVLR2RfRkhGYmJUbzhMa184bWZHRUE3TS1QOUlzOTczVVZRc2pjRXJoQk5yd0VVWmRGMkwwaEU4SEprRGoxMHZDRmF3d1d5MkpaaG1hd0ZFQk9lelZPYnpzZnhSYTNTV0lCSlQ4eEsxRFZLVVVZZm9qckFLUjQtTVpFcG9relJRUXhQLXFYNGszY1ZqdDJoSmFGc1MzaHoxMmJBcExMV1BGTEdQZjlhYWJmc1NJZXN3Ukk3MDAxUVI2bEk?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1409,7 +1409,7 @@
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46075.45392361111</v>
+        <v>46075.89135416667</v>
       </c>
     </row>
     <row r="19">
@@ -1425,22 +1425,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>“Misschien hadden we die uppercut van vorige week wel nodig?”: Sporting Hasselt weet weer wat winnen is - HBVL</t>
+          <t>OVERZICHT 1STE AFDELING. Knokke en Roeselare nestelen zich in top vijf, ook Jong Cercle klopt aan de poort - Nieuwsblad</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>“Maybe we needed that uppercut from last week?”: Sporting Hasselt knows what winning is again - HBVL</t>
+          <t>OVERVIEW 1ST SECTION. Knokke and Roeselare are in the top five, Jong Cercle is also knocking at the gate - Nieuwsblad</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 10:54:56 GMT</t>
+          <t>Mon, 23 Feb 2026 04:18:00 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOY3o5T3d5emNMWXFhbW5Gdko0djNqZlhTSkZEVE1RQkp4U3hYN2xiQk1BU1FwWTZVelFrTjQ4Sm5tanBvZDcwanJUWDJrSjZrMk9mUWJwang0bC03bS15RVFQMEJBa0hJcGdIOFM0UEtVZWpZc1RqRVdxZlNBVklaVlJ5alRWWlNGSkpuTGRCZnlySTJ2bnBOZUZ4UGNCN1p2TWFYU21JelZBSHU4NHF1VS0wQkotNm12R25mTmpiLXRSeTZETWJzcWEwWWEwTHVPUzN2Y2NuN2xzTFNsakpkQ2FB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi9gFBVV95cUxOemJ4d0ZmcmdRaHptdXdVQjAtUVgxanZpZkRDTDBaY3dUZFNvNTFXbHdUMUxBdS1qclppLTJOcDNYMUNiU3BIZ2pMaFQ3UW85LUlzQjMyeks1WGtRcG0xQkZtR1pyM3ZqSHhzZ0RHNS1URFVNM0lldFYtRUJlMFVjUVp0SHJoUkJDQ0h3ZnM0TlVzaVp0aVNBVk9uMkN5bXpVd3E4SnVRdzVSOHN2SnNHOGFOYmVCNnNPdG9TLUhfczNVdjhKUWtTV3Y4VTh3UC1OYklYYmFtMUhLQnpnR3ZUR1Z0Zk13RE9MbnBfZlhqVDQ5OFdyd3c?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1464,7 +1464,7 @@
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46075.45481481482</v>
+        <v>46076.17916666667</v>
       </c>
     </row>
     <row r="20">
@@ -1480,22 +1480,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>KVK Tienen gaat in slotminuten van eerste helft onderuit tegen leider Sporting Hasselt: “Leuke ervaring om voor zoveel supporters te spelen” - Nieuwsblad</t>
+          <t>Cash geld en juwelen gestolen bij woninginbraak - HLN</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>KVK Tienen loses to leader Sporting Hasselt in the final minutes of the first half: “Nice experience to play in front of so many supporters” - Nieuwsblad</t>
+          <t>Cash and jewelry stolen during home burglary - HLN</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 13:09:58 GMT</t>
+          <t>Sun, 22 Feb 2026 22:15:08 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAJBVV95cUxNZS1oMU9NNV9iOUVyeG41eHo2dzV1cUdMekJLWmJLVmJyMVR6aW95U0VkTUw2bVRfalUwcEZMRkpZU0NjNEJQd2RXQjVvc19HdlI4bzRleGd4eUIxQTRoWVNmWjJXQmh6MDBPdDJwYWNiMmkxTzhfVXk1bDA0RmFEYU9PVl9adDZuamhJWDF2YmFCUE1KSU5IQzl5VnJhcnZUQkJvMXZKSS1UTVp0MEROYkVpNklwdlYtLXFocy1aTG9FRUQ4MHpSNnV5MXdfc3A3LWlOSEZwcFR6ODRiaVVFblpHMWdXLWhQRFJ2cjduRGFZSHZVZnBZWktLVFUyMlRaNmNfVVB1V0tKNmd4R0wyRDBIbGtvQlM4TVg2bWVmWTY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxPUGtqazY3d2Rrb20tcU5ZNnZsM0Z3R1h0V1l4WV9GYWp6QTNFZ0x1dV9CVzUxaE5zWkxmZ0h0cmd4YVRLbjJFeTVmSW93a0FpTTJKU2RGMUtzZE84ek9zRlpNOUpwdjJIWXZrMzhBNWo2dkZzaGl0VXkwZGEyUThqWEphY2FUODRNVk5tRTBn?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1519,7 +1519,7 @@
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46075.54858796296</v>
+        <v>46075.92717592593</v>
       </c>
     </row>
     <row r="21">
@@ -1535,22 +1535,22 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Hasselt verhoogt ambitie sociale woningbouw - TV Limburg</t>
+          <t>Gesprongen waterleiding langs fietspad Luikersteenweg zorgt even voor oponthoud in Wimmertingen - HBVL</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Hasselt increases ambition for social housing - TV Limburg</t>
+          <t>Burst water pipe along Luikersteenweg cycle path causes temporary delay in Wimmertingen - HBVL</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 17:21:48 GMT</t>
+          <t>Mon, 23 Feb 2026 07:05:40 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxONWFSbE8zTHl0VVBBdnlMU1oydWVHMGU0cXY0cWtqRXdqeld4dXMxa0tMWDhmbC1pZV9aMUYxZlJOQ2R6RTZlb1FPVWdiQndWQUVyQ1BiWGQweTN4bUtxR1BWOUtzb3hZa1l4MFp2Y0M2Z1ZWVF8xUkhJR2Z6ME5MSEln?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxQQjlqZkhUbHB0SVFCNFNOSGNLb2ZiSXlkanZlM0YyNXotOVR0VVRCaWpqamZtQ3pDMWJWbVJ6MWxpWXBuWGpOMWlpRkFUNkpmX29xYUoxOC1NLS12QnQ5R01yQVRNN0puSy10M1VSekZZRnRNQWk2SkxUX2NHZmhnRVV4a0NkNHNENWMtbUh3Vm54YjRFUDJ3bVZ1NG1MUzJzbjJuZ2NwOF9QMHl2Q3AzOWZ2VXE2WHQyZHI4dDlTQkRYWVF2NmtwMUgwZV9VXzlVUHdPSFRIYXU1RnZWQVFYbGtSWFZpVTg?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1574,7 +1574,7 @@
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46074.72347222222</v>
+        <v>46076.29560185185</v>
       </c>
     </row>
     <row r="22">
@@ -1590,22 +1590,22 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>De Lijn moet 35,5 miljoen euro besparen: deze buslijnen in Hasselt zijn bedreigd - HLN</t>
+          <t>Roger (87) heeft meer dan 210.000 luciferdoosjes van over de hele wereld: “Maar nog nooit één sigaret gerookt” - Nieuwsblad</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>De Lijn must save 35.5 million euros: these bus lines in Hasselt are threatened - HLN</t>
+          <t>Roger (87) has more than 210,000 matchboxes from all over the world: “But he has never smoked a single cigarette” - Nieuwsblad</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 07:33:32 GMT</t>
+          <t>Mon, 23 Feb 2026 01:00:00 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNSkgyWE83bXY1azFfX2NlZHFYaGNqT1JlNGotYmE0M3hTRHVzY3RFa3BPdEhXOWVnMGpWenBtTEJSSWNqUms4bTdsMHV3bDkxRDZNZEF2Z1V1MFFEVnFsYXYtazN1aWNRVjNOZGs0bG1PRjJVWEVDTjl1SWpnYUhhbWF1MkZEU0dJY1l0Zzd5bzRxbGk4bEhPdXhJYm5mam5CUXExOFFKck9DVEZoamtnMjR6NHpaM1k?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxPakp6SkhoSXdMdmEwbVBqMWo5X2hlaTBIbTRGaDFhaXNtZEJkaGdFY19GdUpnM1Jud0pJeVVEZE9WRVo4ZDZfZ3NVUk9sMFdhVnR2N1RQbWNTZ2N1Z211Z2xtOGlfcmxKdFlDeW9rQnRBdWwwb0t1TThFYXRURmtkV0w3Mm5NUzk4cVJnUFdadWpIcEtMeS1ZVjkybmtSX3FVeHJzTDctVWw4cFNFMDNiODJhX3Y0azBOSUFTTzZBX2RpTHJyWVR5S0RHVURQR28tY1U2V2FCVlhxYS03SGJ6TEdhdHZhTE5jTnVhSFdXbTgydlNXTUNzU0x6Z3Q?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1629,7 +1629,7 @@
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46075.3149537037</v>
+        <v>46076.04166666666</v>
       </c>
     </row>
     <row r="23">
@@ -1645,22 +1645,22 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Tafelschuimster teistert horecazaken in Eisden: “Serveer haar geen drank” - Nieuwsblad</t>
+          <t>Stefan Mertens, 56 jaar - HBVL</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Table skimmer plagues catering establishments in Eisden: “Don't serve her drinks” - Nieuwsblad</t>
+          <t>Stefan Mertens, 56 years old - HBVL</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 13:56:34 GMT</t>
+          <t>Mon, 23 Feb 2026 04:11:43 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxOLXR4Zm9rU1RXTFhMTFItYzc0Q1Z0RlBfNjFaMVUtNnhqTEI0T2ZCX2FlZ2dsa1RBNUdCTm53anl4QkVWWGNIOF81bl9BOWZiMV9RSnBZRVNtTzU3WmRDdkNXSjhmMk1xdUNxaVluTlNKdG9jdnY2Y1djUTN2bVEwTUNocTlmOHJFNXRrMUZKUzlyRVBqSTc2T0htMnBBcEY2ck01N2VnSThmNmxseHdiUnFlemQxa0RkMEZWNWgzR1RpcEwxZThLQkZNSGdCQWhrR3AyYQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE40Sjc1bFB1QWFTU1p0NlpnUEdCX3BVdmFlUXM4bVU0aEdLemc1WGlxa1JpZWhFUlhaLUo5TFNueEJZcDZIZ2xocWdyQ2VxNmZFXzNwRTVyY2p5S0U0YWp1UXBwQ1Z4UWFySUR6dDFnVkVJZDJyeGJLRVNxMV8ycW8?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1684,7 +1684,7 @@
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46075.58094907407</v>
+        <v>46076.17480324074</v>
       </c>
     </row>
     <row r="24">
@@ -1700,22 +1700,22 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Niet alleen biathlon op de Winterspelen, ook in Hasselt wordt gestreden om het BK - TV Limburg</t>
+          <t>Naar de supermarkt op zondag wordt steeds populairder: “Op zondag heb je veel meer tijd” - Nieuwsblad</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Not only biathlon at the Winter Games, the BK - TV Limburg is also being competed in Hasselt</t>
+          <t>Going to the supermarket on Sunday is becoming increasingly popular: “You have a lot more time on Sundays” - Nieuwsblad</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 17:30:42 GMT</t>
+          <t>Mon, 23 Feb 2026 00:39:12 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxON29teHZNZ1hxY1QyX3NYSG1TZ3JOY1pYUzVsLWtwSTJmUkFqOVF1blg3T2NNLWdtdXVPY2lZbGJhZWJtcElZOXNXcUhMSjhrRC1yMFhlQW5aV3JxbG5iZDNJai1HeTBraDNRT3M4LWJaVUp1em9ibkJ5WnlVUDJBY0JXbzl6X2ZjMmkxaDFIWjRzNHVZa0Jzd1p5Z01CaC1UVUV2NFhZRDJKUE04VkZnUHVmWQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOcC1XQjFOeXlDY1ZkdURFMG1HYnprcjZ0MEVMZkJKZ3NPYnAzYkVFbFdzSFR3RUxZNllEOGhfb2M0R2dWRUFUYmRiR05iMlE5cVEtWTJpazRCRVlpZFhjbHRPOWR6Uzc4VG5feXllMW9jTEVlU2QyYWRLR3RUUGNxZGlaaTFFQ1lEd092VnczM3pzazNkOU56Mld4eXpSRGo0YURXU3prV0FtTkU0aHpVelg5b0dFQlh5OWlRRVVaOTRMcDB4dU5PYnp3VU5CVExxNVQ2TDEyRzFqMDJPa0V0dkdR?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1739,7 +1739,7 @@
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46074.72965277778</v>
+        <v>46076.02722222222</v>
       </c>
     </row>
     <row r="25">
@@ -1755,22 +1755,22 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Honderden bezoekers wanen zich op de Olympische Winterspelen tijdens het BK virtueel biatlon: “Toch moeilijker dan op tv” - HLN</t>
+          <t>Buren zijn boos over natte tuinen en kelders door bouwprojecten in Godsheide: “We zijn het grondig beu” - HBVL</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Hundreds of visitors imagine themselves at the Winter Olympics during the BK virtual biathlon: “Still more difficult than on TV” - HLN</t>
+          <t>Neighbors are angry about wet gardens and cellars due to construction projects in Godsheide: “We are thoroughly fed up with it” - HBVL</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 13:45:43 GMT</t>
+          <t>Mon, 23 Feb 2026 00:48:08 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxQTEpNOUxzazNpeFFOMF9ETVhxZGZQcFZacVFmX2xySU5HZThCVlFSLVdQMzhKRU5aMTMyelc5ajJyeFhHNlFhV2NpY3JQaC1oUGh6VGxxT3BQdlktS2VPRk52dFNzWmN4N2NSRjI4SURyTEJ6cW9Na3YwV3V1RF9wNlVFS0sxWjhQQUZFYUMzRG9GYlJ4dlpPVVJkc01FbndCVmFvdVcyZHZHNnJLUHNwVXprclR6aUFvQS16TWhac3R6aEJXN2JMT2g3cjhMUzE5QWVucnl2dGY2Uzg4YWZFOGVQV1RpNXF5Z3dv?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxPLUZubFhyVVp2OGVJWkNIWGpSaW9QVndPRThSZjFZbkhienl0dFVkVF9XQzBDOEpySjMxWDlFZzFVdHl5RXYwUEwwcVROR2Fnd0pVNUMwRkhxWUdfcDl4eXFoMkRfT0xLem45VVZULTNKMkUwb1duUVJvWEU0Q3YwdHE0enVWMFJKODZuczVPY3Rxbi1zYlhwSEs0M1hWNjk1QUpUWjZkdGdZWEhSRFdiRThZZjhsaGVBSlJETHdmNHdYX2ZJb0JUdVFacGxzakNRV1U2OEZWTUdQNGJZN0o1REZLUkpwU3JLcUEzd0pn?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1794,7 +1794,7 @@
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46075.57341435185</v>
+        <v>46076.03342592593</v>
       </c>
     </row>
     <row r="26">
@@ -1810,22 +1810,22 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Loksbergen in spannend duel voorbij Juve Hasselt B - Nieuwsblad</t>
+          <t>Tafelschuimster teistert horecazaken in Eisden: “Serveer haar geen drank” - HBVL</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Loksbergen in exciting match over Juve Hasselt B - Nieuwsblad</t>
+          <t>Table skimmer plagues catering establishments in Eisden: “Don't serve her drinks” - HBVL</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 03:26:01 GMT</t>
+          <t>Sun, 22 Feb 2026 22:53:07 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQNDJZeXhHbk9WMzhoYXZuVXhIOW9VWlpCdUhmR0xaZ0hGcGlneWN6UWZWTmVSdm9Bc2xHdkhjbTVNajc2bHk1bk5nX2d2SGN6ck5ORjd3bEpXUWRXeGI5M3RESmRvMm90eGhyRHI1bk1BYXVBUFp2N1pTMzlIVDBPX19SNHlvczFFR1pKOXpIU0xwbW9FYXRGYjIzN2pIcV9JaVNiQWdaT0twMTNkMG16Wg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxPYWpfYndHRFVOdGNOMnJ2S1R0X1RYRFYzTDZSQWJFdlpzSU9TVnBwUWVSaUFweUZFUWJrQjd3V1BMQ2xfSUtUcENCYjRkVjFvd2huTE5yN3JPQVlnUlFzMTB3Yy0tdmFUd1I4NE84Zkh2dDBoekpjNHN1ckNINGZOTFFWcWlaVDRNNmYtQ0tlNzdzSWhwanlKYldZcVZHeTg5M3BxNjl4RGNYdEdjMkhyRHdGZDh3NnpucXNBMktTWDJHMURONlpLdm9HRHA?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1849,7 +1849,7 @@
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46075.14306712963</v>
+        <v>46075.95355324074</v>
       </c>
     </row>
     <row r="27">
@@ -1865,22 +1865,22 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Torpedo Hasselt B en E. Houthalen delen de punten - HBVL</t>
+          <t>Torpedo Hasselt wint uit van Kortessem, mede dankzij twee treffers Bijloos - HBVL</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Torpedo Hasselt B and E. Houthalen share the points - HBVL</t>
+          <t>Torpedo Hasselt wins against Kortessem, partly thanks to two hits Bijloos - HBVL</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 23:32:41 GMT</t>
+          <t>Sun, 22 Feb 2026 16:34:50 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxONDhpVVh2SUdFRnR1RHUzd0dXWlJSMFoxX3Z1UVRPSFhiNV82M3ZoYTJyMnF0aGY5bVlDUXcxTGswNlZVWnFmZUUtSS1lVnRWMlJEOTd2RXdNeFlyZTd3N2VBcDVxdWIwMEZidzdUbmM5RjljX0JON05MaTBHRElyRjhvYVZneTlaRUVWNzRfWWRvTlZ6Yjd3b2ktV1oySVd1YnJqZDg5dE11Zw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxNaWZsa3ZpUkhIYU41QUM1Sl9ueHkxV3R2UDZTSDVGMkVvYnRKX3lZVHl3blV3YzQ0Mm9OZGV4ZUt6QmQ4SklzNHFac01MaTNaS1ZNOXY3QWd2ME5OVXhQNHJockhtMWpZRm9ReXUxNmcyamZSR24wcHhkb2psMVFBeUpJSjdUaUxHdjZkTG9nMGQtRDJvOG0tUWNHQVByaU5kVWk0VTFTQzNyV19MRlRLcDVzekZGdmlNdS1NRUxTVlBRTmYtRG5QOTVR?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1904,7 +1904,7 @@
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46074.98103009259</v>
+        <v>46075.69085648148</v>
       </c>
     </row>
     <row r="28">
@@ -1920,22 +1920,22 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Cash en juwelen gestolen bij inbraak in Stevoort - HBVL</t>
+          <t>De prima reeks van Lanaken VV zet voort – tien nederlagen voor Herk Sp. - HBVL</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Cash and jewelry stolen during burglary in Stevoort - HBVL</t>
+          <t>Lanaken VV's excellent run continues - ten defeats for Herk Sp. - HBVL</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 11:09:32 GMT</t>
+          <t>Sun, 22 Feb 2026 17:15:06 GMT</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOZUVNeG1OdjFmeERwdnZVSk14cjJ5SEFUazh0cDY4TEpnNnd2V1ZKQy1ZdEwtV0V5ME8tSW9uV0xYaEt3WG9EQk9JVWVyQ3JZa0dXeGpkZ0puemZkRDBfdzNQZDJxTmdoUTM5UmM2Ul9UekNINXphTzlRa2pQTURHM3dtUFZhSEpPUF8wXzJfWXpIZHBIeW83aVVkdFY2WlByekVlRnY0VUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxPenBKZkhxY0RiOWF2ZVJCWHptQjUxNmJtSGRTLXFlSXNVVk4xcGVuRlp6eER5eGNTc0w4cnJnd1pfM2NXam5SZm1MeC0zdDQ1VjhQZkphWTZjaEtlMmVxd2I1Y01WY2xaZnczcHBDejlaVFlpZjAtbGU5VWVvT3BwXzZxcGNRUnRvQmdYZnhkN0JjVXp1ejk5WDZiV0ZSc0hTX3lELXBlcWF5Y09TX2JOUUZ6LWVzNDd1dWFNZVJWUEh0aVhqLXZRZXpCQQ?oc=5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1959,7 +1959,7 @@
         </is>
       </c>
       <c r="K28" s="1" t="n">
-        <v>46075.4649537037</v>
+        <v>46075.71881944445</v>
       </c>
     </row>
     <row r="29">
@@ -1975,22 +1975,22 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Sporting Hasselt wint de wedstrijd tegen KVK Tienen en beslist in de eerste helft - Nieuwsblad</t>
+          <t>Sporting Hasselt is al voor rust klaar met KVK Tienen: “Hier moesten we de punten niet komen halen” - Nieuwsblad</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Sporting Hasselt wins the match against KVK Tienen and decides in the first half - Nieuwsblad</t>
+          <t>Sporting Hasselt is done with KVK Tienen before half time: “We shouldn't have come here to get the points” - Nieuwsblad</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 23:23:01 GMT</t>
+          <t>Sun, 22 Feb 2026 16:03:00 GMT</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxQaFNlS2hMaUVLWkQxR1FQcVV1ZE5Bay1kT2J5ODRDazRZNkZ2a0JSZWQ0SUx6TzlQQ0VycFdvN015SVZNZi1HSXFmclk5c0ZfRWMzd2E5dUdQbHl3MHZJSzhveVZPcU0zVmxaaFRneXFfZDJma3BEWThtYjNrSnQzNmQxVUVObzBFZlZkb3lHTHpvSlltSHM2QTh4MF9BeVB2TThBXzBJNkpKQUhJR1R2TmdLRF9WTUdydjZ4TzRrMVJaRXFObE9rTXRlckh3OF9wYkcxUnRURnluQkti?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMioAJBVV95cUxNZS1oMU9NNV9iOUVyeG41eHo2dzV1cUdMekJLWmJLVmJyMVR6aW95U0VkTUw2bVRfalUwcEZMRkpZU0NjNEJQd2RXQjVvc19HdlI4bzRleGd4eUIxQTRoWVNmWjJXQmh6MDBPdDJwYWNiMmkxTzhfVXk1bDA0RmFEYU9PVl9adDZuamhJWDF2YmFCUE1KSU5IQzl5VnJhcnZUQkJvMXZKSS1UTVp0MEROYkVpNklwdlYtLXFocy1aTG9FRUQ4MHpSNnV5MXdfc3A3LWlOSEZwcFR6ODRiaVVFblpHMWdXLWhQRFJ2cjduRGFZSHZVZnBZWktLVFUyMlRaNmNfVVB1V0tKNmd4R0wyRDBIbGtvQlM4TVg2bWVmWTY?oc=5</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2014,7 +2014,7 @@
         </is>
       </c>
       <c r="K29" s="1" t="n">
-        <v>46074.97431712963</v>
+        <v>46075.66875</v>
       </c>
     </row>
     <row r="30">
@@ -2030,22 +2030,22 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Ongeslagen reeks van Lanaken VV B tot een einde gebracht na 2-0 tegen KMR Biesen B - HBVL</t>
+          <t>Taxi’s onder de loep bij politieactie in Limburg Regio Hoofdstad - HLN</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Undefeated series of Lanaken VV B ended after 2-0 against KMR Biesen B - HBVL</t>
+          <t>Taxis under scrutiny during police action in Limburg Capital Region - HLN</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 22:35:45 GMT</t>
+          <t>Sun, 22 Feb 2026 16:13:38 GMT</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi3wFBVV95cUxNR3RsNTM5cnR0ZFZXdHdTYnM4dXpTTTRZejRpMWdvUjgwSXUxblNmOFVwdTBIdEZFREYtQnpRMHNLSThiVjV0OTNpYkdZNy1tcXFpWU5qVkFRY3pxNlBWWGxiWVpCOWNrbjVZOFl0RHlFRkRwV2RCNW54OHFQeHRpb0pwSERuQkZmQTViOGpUVUp2ZmpHa1VjaUU3SkFOQTBELVMyX3FNU2tIV3ZBMUNadjVOUGhsdDVfeENYVm0tSk9oa2tHdTQtWjdnUF9qcHNFdVo5SGViR0VwbThiWURN?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxQaXRmNHdwVmRESmpGTklZSERKbWliSzB5aUVmMk1zQXpxM2o1M0NLbkxNZkFKaXhBeWJVTFdDM2Jqcm9IU0NObTFRSFAxaFo3dFBPUkNGQ1o1WTktYjhtb0hFLURhazJjVnNIdVdXNkJvaTgwVXlnQTZNZ2t2d2lrdDNieHhxRlgwNU9lTGt6NjllT2xwM05kQnExMlVqdXdxN1E?oc=5</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2069,7 +2069,7 @@
         </is>
       </c>
       <c r="K30" s="1" t="n">
-        <v>46074.94149305556</v>
+        <v>46075.67613425926</v>
       </c>
     </row>
     <row r="31">
@@ -2085,22 +2085,22 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Swinnen redt punt voor Juve Hasselt tegen Nieuwerkerken - HBVL</t>
+          <t>“Misschien hadden we die uppercut van vorige week wel nodig?”: Sporting Hasselt weet weer wat winnen is - HBVL</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Swinnen saves a point for Juve Hasselt against Nieuwerkerken - HBVL</t>
+          <t>“Maybe we needed that uppercut from last week?”: Sporting Hasselt knows what winning is again - HBVL</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 21:50:44 GMT</t>
+          <t>Sun, 22 Feb 2026 11:49:47 GMT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPcGdBZ3ZRTko2WHRaaFlOUUM4VE5KeG84amJuQUcxblBrcVVCelhZODd6TWtNU1NoQUFOdURNOHFjV0d5ZjUzdHU4NkwzaHZNSE9CbkdjTkU5SUtSaWgtekphSXN1NUotb0tETXJMYlRlLTA1N0RxUVpnVVdZV1JCb2tGM2MtMDhmZ294LUstXzhEVV9oT0xuckVBQTc0YlY2ZHJ0cUlwNHBsX3hVd2N6aEpB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOY3o5T3d5emNMWXFhbW5Gdko0djNqZlhTSkZEVE1RQkp4U3hYN2xiQk1BU1FwWTZVelFrTjQ4Sm5tanBvZDcwanJUWDJrSjZrMk9mUWJwang0bC03bS15RVFQMEJBa0hJcGdIOFM0UEtVZWpZc1RqRVdxZlNBVklaVlJ5alRWWlNGSkpuTGRCZnlySTJ2bnBOZUZ4UGNCN1p2TWFYU21JelZBSHU4NHF1VS0wQkotNm12R25mTmpiLXRSeTZETWJzcWEwWWEwTHVPUzN2Y2NuN2xzTFNsakpkQ2FB?oc=5</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2124,7 +2124,7 @@
         </is>
       </c>
       <c r="K31" s="1" t="n">
-        <v>46074.91023148148</v>
+        <v>46075.49290509259</v>
       </c>
     </row>
     <row r="32">
@@ -2140,22 +2140,22 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>De Spor herleeft: Is Erik Van Looy de geheime redder? - VoetbalNieuws.be</t>
+          <t>Vakantiehuis voor mensen met beperking in Maasmechelen verliest half miljoen aan subsidies: toekomst onder druk - HLN</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>De Spor revives: Is Erik Van Looy the secret savior? - VoetbalNieuws.be</t>
+          <t>Holiday home for people with disabilities in Maasmechelen loses half a million in subsidies: future under pressure - HLN</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 10:45:00 GMT</t>
+          <t>Sun, 22 Feb 2026 10:53:39 GMT</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxOaGhEQlBKWGZsbElpQkZBZl95czJqVXVacmFxWFhpSFVHOXBYRGdnYnY0RkdIUTdoN0dTY04yUHJtdlB0amcteGdoSTFmOWljX3NoVkozTW53ZkYwZFRyMkJ2NGQ4S0lDSGlWM2tDQzdOY21jOWRnY1BEaHptZUZQSGpLdGdWeW9KSzM1WmFWX2NKSUNKMUFkcG11VQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxPSGxqbkRqNVpYNWk4RFVLN0hzNmZWY0hXMmN4RnRPeW4yZzd2LXlMeEhOWTB4TnhOSTJPSUR6VFVFVkJjeV9VUUZ4MEd5SGY3OHJBVGt5Q1lSdzAwTkh2clBVV2lhYWUyNFlrYTRkVDBhRTRPdEVpU2ZKVFZWSDhndHV6YlpRN056LVVlVjgweFhUVFJfTGdMYldJQmhROUlxRVZsci1lbGczR3BtRUo4R0FsNElrWk5RM0dYb0pUaFJzWXNhOEUxaGJyQ2dCUW9FcjlfUWhNb1VBdzc3ekJscFZDSlk0S0U?oc=5</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2179,38 +2179,38 @@
         </is>
       </c>
       <c r="K32" s="1" t="n">
-        <v>46075.44791666666</v>
+        <v>46075.45392361111</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Devant New York, Londres et Berlin : cette ville belge est une référence du street art mondial - RTL Info</t>
+          <t>LIVE. Erop en erover, Torpedo draait de rollen om in Hasseltse derby tegen Kortessem - HBVL</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Ahead of New York, London and Berlin: this Belgian city is a reference in global street art - RTL Info</t>
+          <t>LIVE. On and on, Torpedo turns the tables in the Hasselt derby against Kortessem - HBVL</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 18:30:00 GMT</t>
+          <t>Sun, 22 Feb 2026 14:30:00 GMT</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxQeHFWdUhraEVFWEpncWVmUUR5b3ViTU9kN29PYzNJeXV5TjB0U0Vyc0t1UDRpUlhJejhULTN5eWJWcnNQd2drbnJZVFJFdDg1YlVZdVd5Z3EzXzQwVVdfaHBsZkRXd3FfTXpxU193bHBjM2wtdjNDSnRmMmNnYnpCYUFYR09KcHdtcEY4T210Z2R0OXh0Ym1ZVGlzdWsybXVZanFxX0MySjZaOFhBeDdQckJ2M0xlTkFybVA1VnRJUHJMeU9MMmdIMGxoNzU2Q0dmdjZEZkc1V0cydlFtakE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxOdmt2ZmlPYldiQjNsM2hoU3Npd2RQSWFXQUxmQTgwVHRxbXNwbnVBcm4zUG5qRTFhcU5nSnA4OVVxS2NXYjFwV2stNEw5UldRQy1mYWN4Z0c5endfdWFYWUZyRDdJZlRfcGh6Q0pHWkZoWU14VE5VcEx3UzItYzM0T0hVVmZ0eHNkdmNZZU5RU01CRWFOSHA1TGR4THlCVDF2YW8wVkdISGxKRVA4YUlMNzdPQ2NudHFkQ0lfekFyc0k4MFBZa2diTHh5SVE?oc=5</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2220,7 +2220,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2230,17 +2230,17 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K33" s="1" t="n">
-        <v>46074.77083333334</v>
+        <v>46075.60416666666</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2250,22 +2250,22 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Cultural Compass: Illumination at Atomium, exploration of nature and historical opera - belganewsagency.eu</t>
+          <t>VOLLEYBAL. Ontdek hier alle opstellingen van dit weekend - HBVL</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Cultural Compass: Illumination at Atomium, exploration of nature and historical opera - belganewsagency.eu</t>
+          <t>VOLLEY-BALL. Discover all the lineups of this weekend here - HBVL</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 07:00:00 GMT</t>
+          <t>Sun, 22 Feb 2026 21:17:59 GMT</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOY3U5LTUtNXZGTG5qbHJmby1mR1dpOXJGVTF0aUI1NHBkYVZ6Skg1ZWRxWDZhRU00ek1aMzlvbTZwazAtcU5LZDNDM2I1NUl3MnlLUVRIUjdoVXZTYjZqWDNGRG5aQVVTNDFiZ0h6UDRHY2tSLVFGdkQ4Rzh4dVQ5T2h3UWNta0k3MHNqNnFBbi1SaHd6ZmVEVnk0YWN2Tm1URTBYeEp4X2taRW85Z1VMZUN0aEg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPSGtOeUQxT1pyempNTVpvZnMwQTR0N2F3cDgwdWtDMVBVUzVUb2ZsaFZGWmx3ODVvaml0S2V1Uml5U0lEaUFjQklYdmRCb0NpMnRzYzhNTksza3BxYTJtQUJmV2d6T21RdzBJUWJuVDFaem5GakpGS05vQmNmNTIxVDB3QlRmRG9ZZkZjWTZfZzN1My1waTBnZHo4bmRXd1pZUURmU1g5QndBTEc2WEM1Mnc5YkpMbkdIdUxR?oc=5</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2275,27 +2275,27 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K34" s="1" t="n">
-        <v>46075.29166666666</v>
+        <v>46075.88748842593</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2305,22 +2305,22 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Margot Robbie Stuns in Red Gown at Wuthering Heights Premiere - AOL.com</t>
+          <t>Challenger Pro League : Renversant au Patro Maasmechelen, Beveren acte (déjà) sa montée en Jupiler Pro League - DHnet</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Margot Robbie Stuns in Red Gown at Wuthering Heights Premiere - AOL.com</t>
+          <t>Challenger Pro League: Stunning at Patro Maasmechelen, Beveren (already) marks its rise in Jupiler Pro League - DHnet</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 09:11:18 GMT</t>
+          <t>Sun, 22 Feb 2026 17:31:00 GMT</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE8waEpNdEZmMmtDMFhIVzRBZ0QteWtGc0JMUjRFT2hzUXNGa25Pa2FPNzRHSWtUZVVvcGNORnNvYjFVZ2dIeVBMNEs4dTBvdVhmYUt0UWx6T0RQR2daak9ZR2p2SFpZU3lRS2dNaXJ0M0pSMGM3bmcyeEJvT1Y?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinAJBVV95cUxOMlhPQzRIdU1oWjk2ZXgtQmpiQmowckwwY256b2pINDRDb01YVlhZakJyYmJiWFpFdEVxZ0FxY1pESDNRbGNLQ3VKSzJwXzVDNU8wZDhBYXFTaGZSTHpzdEU2T2QwNTUxdWYxcS01WUw0M3BSYXNUaWFucXZhUFVvSlBYYkFaeUM2Y1FDVkhsYWdBTzhoSVFkYV9LNjlCWFQ3U0JXaGVQWEd4VjgwdjVvbndxTmo4OTlwTUdMQkdwbXdIb0RzZWpTVUxtV2xPMFRObWI1d1RuNmVrMFJTZXhUeGZNMTNKYXdMSF9lTGRHaEFoLTJieC11eVBGWDN5SUZFVlZ0Z29IeFgtSEVUWjU4YkpJZWxNYjdVZUNGRw?oc=5</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2330,27 +2330,27 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K35" s="1" t="n">
-        <v>46075.38284722222</v>
+        <v>46075.72986111111</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2360,22 +2360,22 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Sparkx Antwerp or Pairi Daiza Edenya: Which Belgian Mega Attraction Is Really Worth Your Time and Money in 2026? - Travel And Tour World</t>
+          <t>Toujours invaincu, coach de 33 ans : le premier promu en JPL vit une saison impressionnante - Walfoot.be</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Sparkx Antwerp or Pairi Daiza Edenya: Which Belgian Mega Attraction Is Really Worth Your Time and Money in 2026? - Travel And Tour World</t>
+          <t>Still undefeated, 33-year-old coach: the first promoted to JPL is having an impressive season - Walfoot.be</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 08:55:43 GMT</t>
+          <t>Sun, 22 Feb 2026 21:26:00 GMT</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxOTURZdURLM2hrTHotVTREVkg3RVdJRTFwdlpRWE9faEpydkxPLUVqTktyN2hsR3J2a2hxNUdkTFJZRlRRbk1EOUNEVFppbVFhX1pIYkhSY01kUWpwZUlucGE5OHloNjF6blRoQ3RRN0EzYncwMXVnNGJCdHpOYk5zN0xhRU9XUDhlNldjeTFwckt3Qm1JZkVCV056c0ZRd0xiNW1sU1dScVRXaTFwSGpoWS03bm9fU0RwN1lManNDSlkwUl8yOEVnZ1lVNUFCb2xqS2daUnlDMjdaTzQxeUxnalhqRHB3UDRyOEJlcnhqV0k?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxPUm1aUHIzYkdJcldqSDFGdGJnV2dhR2ptNXpyb2Q3cmw2WnhJVEpHNGhycTU3Qng0MFozcThHdUFwbF91WjI2Rl9JT0dLUHpPX1k0VG5Vc0VrZWU2X1ZNZi1JalJ6dHZDSE8wNXJuMm03cUxHNjRBZHpna19tc1FhQnNISHJHbUZjTTNWZDUtVGFOTmtzNUx2NzZ6V2M4WFVQQkF0S0RUNk9DTmNMWGtaXzhQeHFGeXUzRFdwNlJEYXF1ajdocnhr0gHMAUFVX3lxTE5RSHcwUHQ5dWY5Rmk0RkRWSUhBSEdEMnJXTWh2bWIzYTY4N3hmWnZocm42cE9SaUNfb3d6Y3FsNkdPQUpLbUduMXB1WGRRNTFrc0NzVHdZYm5vaTRUOXdWYUhPczVHLTJYZDM1ajRrVWEzcldycExJdWNiWElhSXhmN1A3MnU2SUNTWk1Ta3VrdVA0cUlZSlZibGJGcWV3VHE0Q0tVZWZRTEQtdjllandwNFQwM09feDlabG1aMHBjWEdhNVBjYUlLQ3d2SQ?oc=5</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2385,52 +2385,52 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K36" s="1" t="n">
-        <v>46075.37202546297</v>
+        <v>46075.89305555556</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Lkr: Aschaffenburg: Nach Sturz: Radfahrer als mutmaßlicher Fahrraddieb entlarvt - Radio Gong Würzburg</t>
+          <t>Hippisme. He And Me drivé par Eric Raffin vainqueur du Prix de Paris - Ouest-France</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>District: Aschaffenburg: After a fall: cyclist exposed as suspected bicycle thief - Radio Gong Würzburg</t>
+          <t>Horse riding. He And Me driven by Eric Raffin winner of the Prix de Paris - Ouest-France</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 12:24:00 GMT</t>
+          <t>Sun, 22 Feb 2026 15:42:10 GMT</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxNb05tZ05NYVlVdmx5SmVWdXc3eERabUhHVEdyZjNFZ0V1S3BqMU5qNFBZN21rdmk0RTRiUHVOaUYzUWU0YV92NDJGZ2VJU0ZFVFNNNkVWSXFNRWJZNl8wNGJWVVlBdVI0ZlJTeEZzeWgtVXE1WTVYVmU3TmhwMzVhcVJFSjRIY202dThjYjNrWm5HRzIzZG1PQk5SdFFVUl9Zd1BFaWlLNmtBLTVRWTNCMA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxQX3ZXcjVDbzRNblZfdE5yeDVDb0xKb1RGSnRhZ0J0Tk11akhzb0pCQzE1bUNEOU9mSTQ3N1Z3Mm5Ud2szV2M4b0hIT1BxR3djeUJyQ1JWak5PaHV1SFpvRVotQ2U0RFJXbDVhRWhJRnZXdzREMXFiM0FoN2gxQlZwbTBKQTZ2ZFBBZUpLNHkwX0xaNzdXdWh5UmE4MWkweVpaSVZzSUlvTEtybmlUb2NERkdhSERNeHJrQ2NZaDhzNE5zN0JNWjlOX0pMNnA1ejVGY19ZeFM3Ym9mZmlZNmR1OA?oc=5</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2440,52 +2440,52 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K37" s="1" t="n">
-        <v>46075.51666666667</v>
+        <v>46075.65428240741</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Gestürzter Fahrradfahrer in Bessenbach als Dieb entlarvt | Foto: Bernd Setnik (dpa) - main-echo.de</t>
+          <t>Le Beerschot se loupe à la dernière minute : Beveren exulte et valide sa montée en Pro League - Walfoot.be</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Fallen cyclist in Bessenbach exposed as a thief | Photo: Bernd Setnik (dpa) - main-echo.de</t>
+          <t>The Beerschot misses out at the last minute: Beveren exults and validates his rise to the Pro League - Walfoot.be</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 09:20:03 GMT</t>
+          <t>Sun, 22 Feb 2026 17:20:00 GMT</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOaTZKZlVndVE3SGxUYlJRRnV4S2pSSm85SERZNEc3RWx6c2R2MW90YVZaVlVxcFU4S2tqeFcyRVBPVXFvQlhxSzJXZXBWd1J2c0VmSzdBbHdJRE5zcm42Z2VrRnBLWEI2bjA4MUpPZmE3QUQzRW14RXN0QUM4Q012eEtyQVJGZTZ6bDVIY0NVSUZzRTZNU29XWmRBeG9hYzVfY0tDMGEtencwYlZRMVZlaXpqTQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOMjM1SmJwVkRCWkx0aWwxVUpnYTA1dTcyMlpWTElWSTlQc1NGcHNaajRPTk9wVGxOMXl4clhJSWx2Z01XUXdPeFpCa3ZpT2c1T0pMam9GdG9jeDZENWlUWUt1cEV0SGozLTZDdmNaTWtaX3VaalRpd19jVHJyQmx6dlZIeDVhV09KSHN3NFllQmtaMElOWGVIcnFPVTd4QnFoUm9Wc09rbWpURXVYWkU4clRTQTJiNWxvVGlKSHJPN0VaSmxIOG5LUFJsVdIB0AFBVV95cUxQQmd0R2haLW1QSEM5WG4wVVZ1UFc4RWpVRFdka0pQQXM0QnVjMmVfQkdUSE5iejVKMmtFRHZ0dEJLWHk1VXJTeWNhVmJ0VTZEZWZoRy03aDJVQ2F3NlFfMnlTSFdZRHFvSW8yQkh4dG5HelFXNndaalZsYmJFS3dvSW9lTE5BMm1Ga3BlQ0VONUtjcno1Q25qaWxQak9oWG55VUpZMjV6U0ItdW9SMjJBcnRIM05tTllLMThMYXBkQmVIT0cyNl9kRXRSM1d5VHlI?oc=5</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2495,52 +2495,52 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K38" s="1" t="n">
-        <v>46075.38892361111</v>
+        <v>46075.72222222222</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>A3 bei Frankfurt gleicht nach Unfall Trümmerfeld – Mehrere Schwerverletzte - Frankfurter Rundschau</t>
+          <t>« Mon grand-père est fier de moi parce que je reprends le flambeau » : Gwenaëlle, 19 ans, candidate au service militaire - Ouest-France</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>A3 near Frankfurt resembles a field of rubble after accident - several seriously injured - Frankfurter Rundschau</t>
+          <t>“My grandfather is proud of me because I am taking up the torch”: Gwenaëlle, 19, candidate for military service - Ouest-France</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 09:35:00 GMT</t>
+          <t>Sun, 22 Feb 2026 11:07:25 GMT</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQRTlnZEV6ckd5ZE91N2JkT09DbEtvaXFJSG42c0lHOFk0blpOTXVDdXFwT2JRWHJjYjd2dFR2OFRxWmpac09FSGpHcHItM2xRdGlQQTFmWW9iRWpwcXBYbDFNaW1Td3lRVlJOVDZMSXdQSDVpb0dGSkdaRnNNQnFSU0lEemtoei1HeUNOQ0RZV2tZSlZwTFMyX3Nnc2Y5TWlqbWlvdnpvTC1LZmpFMTZBVjZVcXRLdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitwJBVV95cUxPeXl3QTFDbzFpMDFsZGVYUG0xX0M5VW9QRDRMWVBNS1pBUVhCUFFmbUZ4cllPanNKVlpmcVk4b3MyVGdXUUdQRjVrWHpmVnBkTkN6cUtkTVpqQWZoeGRPa0xZNzRZekVrTmRrMUdpdl9OT0kzQW56VDlNVEh1aElkOUhfYTZqQUVCRHFMWVVlV3dSWnE4QUthNFp1VXh5clZ1RFBfYko1ek9EMTRTcE12NVFEQWJYX3NsQlVDQ3dWNjU4TG5mSzFTUkxpSGdMTGpJN1VEUWJYal8tMDlJMDE1WGFjSHlibzZtam45WmR0Rjd6c0ppN2RoWExpSUpWUGV0V2tZR3o3dERBT3Zzcllva1pZOExkVC1EMHlXUjdzenNaZDlyLXE4LUhpMzluUVoxNlhmbXA2Yw?oc=5</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2550,52 +2550,52 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K39" s="1" t="n">
-        <v>46075.39930555555</v>
+        <v>46075.46348379629</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Mobile Blitzer in Wertheim aktuell am Sonntag: Fuß vom Gas! Blitzer am 22.02.2026 - News.de</t>
+          <t>Sparkx Antwerp or Pairi Daiza Edenya: Which Belgian Mega Attraction Is Really Worth Your Time and Money in 2026? - Travel And Tour World</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Mobile speed cameras in Wertheim currently on Sunday: Take your foot off the gas! Speed ​​cameras on February 22, 2026 - News.de</t>
+          <t>Sparkx Antwerp or Pairi Daiza Edenya: Which Belgian Mega Attraction Is Really Worth Your Time and Money in 2026? - Travel And Tour World</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 09:28:15 GMT</t>
+          <t>Sun, 22 Feb 2026 08:55:43 GMT</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingJBVV95cUxQS3NPNWtUalRJSHBfajA4X1FTQURMaUlRY08xMVUtX0FHY3FBbkc1ZktaMGlSRVZDMUdWMm5tanFCdjUtdC1UUjNHM1M4WVBYUU9vRFd3VXQ4TDhKSTliQzdtblpFZ2hOdWVCMVZsanVyT0ZKeE9ZTEswbHh3ODNWUlZYLXBjdUo0SVd6VjVYbWU5V190c0dBdG9NalJOMnhiVXBLYzJMSUFnNzdtSlNKMU9Db1htaFhBMl9PVHp2MW55OGczVFBHaUFTYk9uTndxWnIwYTVod25PcU9kUjRYRjRBVG5MNkw4THNFeF9YcGpRb2R2UWZHTW41aEVjZXFCUXVHaE4zLXRlZmRkMzhNWHR1dkNLN1dQWDhOREF30gGjAkFVX3lxTFBZM01kM0F6R3pYcVplVWhxaVNQM0xGYUM0bFdDQVJCaU44MzZzRlNwSlNEUnU5eTJUZFdJT3I1M0EyenVVR2xfSVRMd2JRaWZTZUFRdFE0TXY5NUNMMjUwYzNiNERwQnRRYjFlZXhsSGVPUWdBZ0I5em9aMG84VkxjN0tmaFNSVXRaQlQySEN1ejZDT2VMUDRFR2dTMHYxTzVRcGI2VTBuVkw3d3F6SWtQRGZqcnhGdTVoSTVJTlNWYUtCaHEzbmdaUnVfMlFOUTJNRlNNTjlPTmxDSE9HemhOZDM5aUFuWl9CX004MmRzQVpubm9Ub0Fhb0dkYUp4OTl2eFhsZkxPbnNYblQydFo0WEpQSTdaeWFyQXdad0tMbnFYdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxOTURZdURLM2hrTHotVTREVkg3RVdJRTFwdlpRWE9faEpydkxPLUVqTktyN2hsR3J2a2hxNUdkTFJZRlRRbk1EOUNEVFppbVFhX1pIYkhSY01kUWpwZUlucGE5OHloNjF6blRoQ3RRN0EzYncwMXVnNGJCdHpOYk5zN0xhRU9XUDhlNldjeTFwckt3Qm1JZkVCV056c0ZRd0xiNW1sU1dScVRXaTFwSGpoWS03bm9fU0RwN1lManNDSlkwUl8yOEVnZ1lVNUFCb2xqS2daUnlDMjdaTzQxeUxnalhqRHB3UDRyOEJlcnhqV0k?oc=5</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2605,21 +2605,21 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K40" s="1" t="n">
-        <v>46075.39461805556</v>
+        <v>46075.37202546297</v>
       </c>
     </row>
     <row r="41">
@@ -2635,22 +2635,22 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Demo-Termine heute, 22.02.2026: Hier gibt's am Sonntag Demos gegen AfD, Menschenhass und Rechtsruck - News.de</t>
+          <t>Lkr. Würzburg: Zwei Einbrüche im Landkreis - Charivari Würzburg</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Demo dates today, February 22nd, 2026: Here on Sunday there will be demos against AfD, misanthropy and the shift to the right - News.de</t>
+          <t>District of Würzburg: Two burglaries in the district - Charivari Würzburg</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 03:10:00 GMT</t>
+          <t>Sun, 22 Feb 2026 15:57:00 GMT</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxPbjg1bHBjNUY3b3BoMEZlQ2FyeU44dE53WVVQYXFKdk5iMDJGYnhyOGdGZ3oxeHFHMUJDTUxEWXRIczl6SVcxTlZ6WHctR2FRMThndTdLUnQydFotNW04WHV6TFBJN2FiMlRkWVBFdjFGcnYtcEFvb080WWk5eXJOSGNDam5aMTZGd3dBRXB3NGdjaTEzajZwTmNBZDJvd2lBTlUyeUtIXzd5ZURhdlJ3a2ZrOW1xNEl6eUhJTnc2eG9nU3ZrU3BfTWEwNWdDUTZqalRoNFNBY0dkOHppWWxrU1IwbHBROS1jNDV3T2ppaFgzZVBGaE8xam5EdXhxUXVrcklySNIBigJBVV95cUxPOFFPVE5JQmROaVRiTGNpQ0NQOXM0VGdNOC1PeE93Z2FnVDM3VDIxZFNnT1lvNWtIajhLQ2Zsam1JRUhUTkZQOVpabTFHM3ZYbThnR2Vic1F0TjBRZ3h2SmQxZTBRVlVEQTFwX0tQSTJ0THNkZzhSdFdmQkNpdFhtam1YLTZneVNmMnA3TXlYYkNpR0ttZklsOUpkUW9JY0VnWGVJNWk3dlY3cThubVZFZG4zOFFjVHhBZ0N3aDFCeHJVaTByQVZBQTd6NkwtUGl4MlB6RWI3TC1nQjZFOGt2b2tvUzU5WTZ5d1pWY2VqVnJ3Qmc1MWwtNk9PcjFIc09wSUF2R0xLTUhRZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxOcjNiSF9HSFJ0Nk90elM4RFEtdVBGdFZBU2FBTjhJUjVxR2pMMGJVNlhCZE1MQ2VjbVYtaExGS1lURGcwSTRkb21iQnlrUjZBcFU1eGNvaVRjZkZrRUJHNGFhYlpaaTVoSE1pNG9wbU53d1dIS1lQNVE5dmZtZHNFb0REZkJjQQ?oc=5</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2674,62 +2674,1272 @@
         </is>
       </c>
       <c r="K41" s="1" t="n">
-        <v>46075.13194444445</v>
+        <v>46075.66458333333</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Gestürzter Fahrradfahrer in Bessenbach als Dieb entlarvt | Foto: Bernd Setnik (dpa) - main-echo.de</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Fallen cyclist in Bessenbach exposed as a thief | Photo: Bernd Setnik (dpa) - main-echo.de</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 09:20:03 GMT</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOaTZKZlVndVE3SGxUYlJRRnV4S2pSSm85SERZNEc3RWx6c2R2MW90YVZaVlVxcFU4S2tqeFcyRVBPVXFvQlhxSzJXZXBWd1J2c0VmSzdBbHdJRE5zcm42Z2VrRnBLWEI2bjA4MUpPZmE3QUQzRW14RXN0QUM4Q012eEtyQVJGZTZ6bDVIY0NVSUZzRTZNU29XWmRBeG9hYzVfY0tDMGEtencwYlZRMVZlaXpqTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K42" s="1" t="n">
+        <v>46075.38892361111</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>A3 bei Frankfurt gleicht nach Unfall Trümmerfeld – Mehrere Schwerverletzte - Frankfurter Rundschau</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>A3 near Frankfurt resembles a field of rubble after accident - several seriously injured - Frankfurter Rundschau</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 09:35:00 GMT</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQRTlnZEV6ckd5ZE91N2JkT09DbEtvaXFJSG42c0lHOFk0blpOTXVDdXFwT2JRWHJjYjd2dFR2OFRxWmpac09FSGpHcHItM2xRdGlQQTFmWW9iRWpwcXBYbDFNaW1Td3lRVlJOVDZMSXdQSDVpb0dGSkdaRnNNQnFSU0lEemtoei1HeUNOQ0RZV2tZSlZwTFMyX3Nnc2Y5TWlqbWlvdnpvTC1LZmpFMTZBVjZVcXRLdw?oc=5</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K43" s="1" t="n">
+        <v>46075.39930555555</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Lkr. Bad Kissingen: Wohnhaus stand in Vollbrand - Charivari Würzburg</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>District of Bad Kissingen: Residential building was completely on fire - Charivari Würzburg</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 11:35:00 GMT</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxObEFzQ0Vub0JLRk1SdUhxNjJnV0xTSEFOWjdlRVFyYnpob1ZZYnZyaEtvRks5dC1GN2poVG5aczg1SGRmRWIzbTducWZOZ1poX1lYeUdaWTFfbENPSHp5MFEzczludVJwa2tpTnU5dEJ5MjNWMm1WWkZlTFFYMzZxYTgyV3Y4b1BwYkE?oc=5</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K44" s="1" t="n">
+        <v>46075.48263888889</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Demo-Termine heute, 23.02.2026: Hier gibt's am Montag Demos gegen AfD, Menschenhass und Rechtsruck - News.de</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Demo dates today, February 23rd, 2026: Here on Monday there will be demos against AfD, misanthropy and the shift to the right - News.de</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Mon, 23 Feb 2026 06:09:00 GMT</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwJBVV95cUxNcEw4UEFXTE9LZ3BUZHVRb0JhdDNVaTdaYUszLUdBam1CREwwRFN5NlUzUEdnYVZtN0dINC0xbTRudW5DSFR2QlY2QjhDVm5JMXJaN2F5SE5ubmMwWEZibXBFZ2tGM0c3dFZObV9FVGQ4dDlDam5GeDYzc09qWjJLdDBnMTdjTFJaamdheE1tX0FtaGt5WUkxdFVkZ0RXSWc2T2dlU3U0eXlhR2FhS2cxVU92OXVZcmpoUGs3allvX2h2S2s0ZWd1WW4yVGprekR2WUk1d2JPeEhhWFBnbHF1MG9xckV6dVppVEZKdnZvU05IQVRNdEZ0dGY0TDVoNmhrQ2tB0gGIAkFVX3lxTE1rWXg1LXplU3B4SGpfSG5LLXdwV0pGbEROYW5VUlJxWGRVVW9oZjgwY3djOENybFlTRDJMTUFmcVEtRmgwRGRNLV9vUWZ4M0tuenh1X190STlLX2FET09idW9Bak1JTFRtN2ZCM2NjeU9ZZElLY1A2V1Q4clNHZnhMR0NZVmFQMkpRUW1pckZuWnBNYmxicVpDZVNiMktDWUtVcHF4RGEycm5kOHN6dUJmMVdxdktDVTJLNzVsYm9vY1ZMOWh2YTRLdFcxRGFmZl9WdjNrRGR0c255SzB3R2pZZ1FTZUJlWWNHUWxwaTBmSEdYaTFXaFlRR3pEVDh5ZVJ2Y2cya1k2Sg?oc=5</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K45" s="1" t="n">
+        <v>46076.25625</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Mobile Blitzer in Wertheim aktuell am Sonntag: Fuß vom Gas! Blitzer am 22.02.2026 - News.de</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Mobile speed cameras in Wertheim currently on Sunday: Take your foot off the gas! Speed ​​cameras on February 22, 2026 - News.de</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 09:28:15 GMT</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingJBVV95cUxQS3NPNWtUalRJSHBfajA4X1FTQURMaUlRY08xMVUtX0FHY3FBbkc1ZktaMGlSRVZDMUdWMm5tanFCdjUtdC1UUjNHM1M4WVBYUU9vRFd3VXQ4TDhKSTliQzdtblpFZ2hOdWVCMVZsanVyT0ZKeE9ZTEswbHh3ODNWUlZYLXBjdUo0SVd6VjVYbWU5V190c0dBdG9NalJOMnhiVXBLYzJMSUFnNzdtSlNKMU9Db1htaFhBMl9PVHp2MW55OGczVFBHaUFTYk9uTndxWnIwYTVod25PcU9kUjRYRjRBVG5MNkw4THNFeF9YcGpRb2R2UWZHTW41aEVjZXFCUXVHaE4zLXRlZmRkMzhNWHR1dkNLN1dQWDhOREF30gGjAkFVX3lxTFBZM01kM0F6R3pYcVplVWhxaVNQM0xGYUM0bFdDQVJCaU44MzZzRlNwSlNEUnU5eTJUZFdJT3I1M0EyenVVR2xfSVRMd2JRaWZTZUFRdFE0TXY5NUNMMjUwYzNiNERwQnRRYjFlZXhsSGVPUWdBZ0I5em9aMG84VkxjN0tmaFNSVXRaQlQySEN1ejZDT2VMUDRFR2dTMHYxTzVRcGI2VTBuVkw3d3F6SWtQRGZqcnhGdTVoSTVJTlNWYUtCaHEzbmdaUnVfMlFOUTJNRlNNTjlPTmxDSE9HemhOZDM5aUFuWl9CX004MmRzQVpubm9Ub0Fhb0dkYUp4OTl2eFhsZkxPbnNYblQydFo0WEpQSTdaeWFyQXdad0tMbnFYdw?oc=5</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K46" s="1" t="n">
+        <v>46075.39461805556</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
           <t>Village Wertheim (fallback)</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>What is going on with the new FSU College of Business? - FSView &amp; Florida Flambeau</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>What is going on with the new FSU College of Business? - FSView &amp; Florida Flambeau</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E47" t="inlineStr">
         <is>
           <t>Sun, 22 Feb 2026 14:01:00 GMT</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F47" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOdGhlNk5VS041eFZaNXlCZElIOTNxVHpsbEVuLTVETEN5SzROZXVpc2NEX0tjdW9UQlBUR3RUY2JYWjBZWUsyOWgxaUFwWWJoWlBOYm53Tl9OakN5czlGanZLbEMzX3VWTkt6ZW1OdEdPb1ZMUEF5V0k3QTJsLUtPT090eElobUFBWnR4MVR3SjRWd1BMOUpIQU1nY180dTFPOWVBUTJ2MW5RRm8xaWV6Y3JqRQ?oc=5</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
         <is>
           <t>en-GB</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="I47" t="inlineStr">
         <is>
           <t>GB</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="J47" t="inlineStr">
         <is>
           <t>GB:en</t>
         </is>
       </c>
-      <c r="K42" s="1" t="n">
+      <c r="K47" s="1" t="n">
         <v>46075.58402777778</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Village Ingolstadt (fallback)</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Audi RS 5: A tonne (actually several) of talent - Motoringnz</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Audi RS 5: A tonne (actually several) of talent - Motoringnz</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 20:59:44 GMT</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxNS2Z2ZDJ2cE43aWEyaEFvclJ2WG53ZkJzTk9TMHdfa2dGSDBYZWlrUkcxRnRBaUV0NjZVZkExNFRZR3cwUWdURlhMcVRPRkhIdHd0dlpfWi1ib2hnWndCQlZwYl9LMlYwaTg1dTZWQ1h4bFZjSHNDWml2QmxySXhSZ3J1Q3NPamVHRU1tUkk2Zw?oc=5</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K48" s="1" t="n">
+        <v>46075.87481481482</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Village Las Rozas La Roca (fallback)</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>("Las Rozas Village" OR "La Roca Village" OR "Las Rozas" OR "La Roca") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Spain: Las Rozas Black Demons rally past Zaragoza Hurricanes in second-half thriller - American Football International</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Spain: Las Rozas Black Demons rally past Zaragoza Hurricanes in second-half thriller - American Football International</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Mon, 23 Feb 2026 05:45:33 GMT</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxPcGUwMFYxdHY2dEZ6TXR6aFk2MlowaVV5bElVem9WRDBobjRld2wzR3dmWHBqZjBIVFdWQXVrWGM2VE4xSERvcnBTc3ltNFVCeEJlSXFMd2pIQ3kxMHIwWXFReU1KSnMtZGx6LUpFSE1iUzlXN1lUNGJfVnZPclVhM0ItN2h1SnVVNU9renpfVmlpTEJvMnhERElrR1JVZkdZeGRYV0ZKcjVuOC0xNGhrbXdsWjQtWHZtNHIxS3dJMm1TS0F1ZDB6TTZ4STl1dzTSAc8BQVVfeXFMT3BlMDBWMXR2NnRGek10emhZNjJaMGlVeWxJVXpvVkQwaG40ZXdsM0d3ZlhwamYwSFRXVkF1a1hjNlROMUhEb3JwU3N5bTRVQnhCZUlxTHdqSEN5MTByMFlxUXlNSkpzLWRsei1KRUhNYlM5VzdZVDRiX1Z2T3JVYTNCLTdodUp1VTVPa3p6X1ZpaUxCbzJ4RERJa0dSVWZHWXhkWFdGSnI1bjgtMTRoa213bFo0LVh2bTRyMUt3STJtU0tBdWQwek02eEk5dXc0?oc=5</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K49" s="1" t="n">
+        <v>46076.23996527777</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Village Las Rozas La Roca (fallback)</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>("Las Rozas Village" OR "La Roca Village" OR "Las Rozas" OR "La Roca") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Spain’s luxury mansions: where global buyers are investing - Idealista</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Spain’s luxury mansions: where global buyers are investing - Idealista</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Mon, 23 Feb 2026 07:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNR0luNkFMMjRNcGU0TWllT1gyZ0w5VzhVU3ZjLWlqaHkwUEpXLWxjSEV0MS00MF9iTXJBNGtmTlVpWHNGQkd1ZFhMQnJIUEdUZkQyQW1UTlFxWGd6RzFOTzFsdXo0cGpKeEN6SGtNRUJ0anZ4QlA1QWN5TzcxNnROS3E3NDBfeGduUjl4bmJ1d1JlZEV4Qk1lRjFaQXhGRm1CTGlEQzJ0Mk9MR3BmUGNueUdBaVJoV3ZfTTlhbjJia2U5Q0tkb3hsZ1BTV1c3S0xUbDZJ0gHYAUFVX3lxTFBHd2NDN1YxWHVRZjQ5aDlhV1oyejc5WkxsdUlSbFJVNF9VVG5nUV9Ud2RXMGhYWVFVX1NWV29LUDlrTGVUd0pPQ0FmOGlQamtndVk5b1cwUEZZTm9vdWZmb1NFOEZmR08xNXVXb0tOVlVkd1p1Z2JHQWZVS2txeXhRX1pJVEtoejgzMjcxbHo5dl9DbWRmNWM3WWNsT1pMczZna21oM0tfaHVCcTN6ak5jTkxjMmkwc1lTTHNBVU9fWmYyZFQwaEUwd3l6V25JRU9NbkMxZVA5QQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K50" s="1" t="n">
+        <v>46076.29166666666</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare (fallback)</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Bicester Motion announces two new senior appointments - Yahoo News UK</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Bicester Motion announces two new senior appointments - Yahoo News UK</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 13:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxNcFpYbFZXdUdYdzNvdl9od1RuMUdpWm9yMmhrUGs3dW1YMUVNenIyLVFMcnJiaGR3czhfTXM2TGh6ZUNvLUtjVDlqd1d6NmE5S2lWbS1Gc2dacEdjcmlBM2JFN1lRZU9pY3lGSzJYMTBIVE1pTEk4OGVqUzVnbWJ5aVFKRQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K51" s="1" t="n">
+        <v>46075.54166666666</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare (fallback)</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Search operation underway in Kildare after reports person entered water - Irish Mirror</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Search operation underway in Kildare after reports person entered water - Irish Mirror</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 22:37:31 GMT</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNR0FNY0lDUjkxYTVDbjNBVFBEclA5cVpETmRzaHhqc2Y5VTMxMXBOeXJpOENFb3FqWFBUeVJpbW9CSUVsS1QtVDlIR0JZbFJRc011aVJJOWFmRUxEbGxob24telZKWFlVZGctcXlsM0Qya2h1MXFRQnVEZThoYy1WTGZqLVN5djZIakZqSU9tSjE3S0RIUGfSAZsBQVVfeXFMUHhNb1lyLS1qMkk5R3RibzdCWUJHNkEwOUdHZGRUOHFVb1VOal83VTNHWl9Pek1hVnRyMWNjVHJUcnEtYldjdFZCc3N1aDdNVTk2UjQyQVVFWGNLSUFaOERaQXJxSktHaW9XR0kzLVlQY1FOb25INm04eDlvUWs5cjlOTmdGVG81QzNVQTYxbVBLQ3ZlZFNNMnJqc0k?oc=5</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K52" s="1" t="n">
+        <v>46075.94271990741</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare (fallback)</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>McDonald’s drive-thru causing traffic jams in Kildare town - kildare-nationalist.ie</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>McDonald’s drive-thru causing traffic jams in Kildare town - kildare-nationalist.ie</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 20:01:39 GMT</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOWElKdEpWUmpFTWczS2l5LWFob2pDaGdpbUJyWFM5elFGajFkQ21UM3hyeHc4NXJnZ2x3ZW1vdThhVVRjVW9jbXhjWHZ3YTRFQlpXY1VqQVdINFdLM3NvWmxOZ3pwZWNCLVB1MlVrYU11WExvWlY1YnZlbEVzcUw5RUhCUXJTekRMV2hBS2RJX3A0ZFRjQnlrTE40NjNBNnlQTE53ZTdEbWQ1RXNrTVE2RG1QVQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K53" s="1" t="n">
+        <v>46075.83447916667</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare (fallback)</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Former husband 'does not accept he is divorced', woman tells Kildare court - Kildare Now</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Former husband 'does not accept he is divorced', woman tells Kildare court - Kildare Now</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 15:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxQWmxiZWhLcV93VXNZcWFrQ3UxM29xVnJnNEVSZW9qVFdqc2dJY0xmd0d0SGZ4WHR3eWEtRmwzbnZUNi0yNmpnVTB3LXpRalpGOWZldmZOYjJkR3NQODdTY2FWU0xOSHVYWG5NWlBnRHduS1l1T05fZ1Q5Q1hrTUJ4czRPMFRvUWo5NWNubmVJNk9QLXNpMFZoaVRpeFBZT0x0RUVOcVFoSllnWVNlLTctLXpRRTJ5cl9ZemlDc2FoZEI2VTJVSlE?oc=5</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K54" s="1" t="n">
+        <v>46075.625</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare (fallback)</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Poor Kildare give way to Cavan - Leinster Leader</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Poor Kildare give way to Cavan - Leinster Leader</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 16:59:27 GMT</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxQVml5ZlNRaEhfTi1WbEpTcC1VS3lGZnZyaDBPS2pPdWdRVFF6NXE2LWtwWHlCZENmSjM3bDhiMkE0NlN3OGJ3RHpreEswMUgyd0VKbk9qNEpnSjFjYWk4NTlVRGtHSlBQRjA2ZGRVaFE4YUFyY3JhaHN5LXYtNk11OVNhb0NvLWVib3c?oc=5</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K55" s="1" t="n">
+        <v>46075.70795138889</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare (fallback)</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>LGFA - Dubs secure victory over Kildare - dublingaa.ie</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>LGFA - Dubs secure victory over Kildare - dublingaa.ie</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 17:24:44 GMT</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE0tWDdBeWpTdkNBZVhiRXNuc3ZrcGQ4RHZpbzRGd0M0WTZzNDBVWUk0T2RsZWR4M3hSTWJZYUFZdzBFTF9yTzNfX08yN2Q1R21VYk1DYmdtTk1QaDd4MzBxNjdMYkk0Y18zbjhraC1LNXNUSTBzeFE?oc=5</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K56" s="1" t="n">
+        <v>46075.72550925926</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare (fallback)</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>UPDATED: Search in Athy stood down this evening - kildare-nationalist.ie</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>UPDATED: Search in Athy stood down this evening - kildare-nationalist.ie</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 20:52:30 GMT</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxQZ0xWSkpYbVB2eGwxQVF1UzdtT2VBQUo2NHZGV19iTmVjaEtZZmFZcEp2cjAwaFJlTkFvejdsS0FFcTlTYVAzUml2TW5hUUEwT3FGMklWMWgwNTVoVzFwckdkWFVUQzJlMmdNaHFqTXdHVmh4VDJZY1BGeWRoQ0VVbHR2RC0ycWRIV0xzaENzcGRJa3dwTnFhSlJ6dVc2TWxNeWpHUw?oc=5</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K57" s="1" t="n">
+        <v>46075.86979166666</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare (fallback)</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Emergency response in Athy following report of person in river - kildare-nationalist.ie</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Emergency response in Athy following report of person in river - kildare-nationalist.ie</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 14:16:14 GMT</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPZDJjWllad1pFWWp4UG9may1DV19rZEtISlpNTEZaSjU0Vm85ZUFOUW5rbExLdzRIY1JreWkyN3ZlOGVjTVQyc1ZhbVd0aVFGbGtoSDdhdldENTBNVmVpSlJyQXNwbUlLMEJ1aWpFNk90aGtFUWJsMEpEUDgwQUZLVkc5empYSkctbkFOdkZkczRVQTJrZE9razBGbElabjEza2t2bGdEMWk3alA2TjUtQ3IzVl9fS1Vab0E?oc=5</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K58" s="1" t="n">
+        <v>46075.59460648148</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare (fallback)</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Kildare sucked back into relegation dogfight after dismal display in Cavan - kildare-nationalist.ie</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Kildare sucked back into relegation dogfight after dismal display in Cavan - kildare-nationalist.ie</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 21:31:41 GMT</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxQSnZwWEF3a2xxcGNSYXhhcFBIN1pnOHJ3TDlIY3BIeEdvX0R3WmZCVUJaem9WRmR0bVdqMHBsU1JvbGVsRUcxZDZMdGlyc2pvN1Y1SkEwMVE2NzNqNE1OTkIwSnBlSURnWWdpZ3d4OTRsMTAxV1JWUHprRUVKNXoxTG93TE9vMm45V2h4SjJ3R242Z1o4Y0pQcUU0NVVJNGhSWmszeXNWVHA1ZldGNTVFUDNzRVVPQ2x1Zl9rLVJpVERfRWZ5YlNwR2ZR?oc=5</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K59" s="1" t="n">
+        <v>46075.89700231481</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare (fallback)</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Deirdre’s murder, hiding bodies &amp; ‘never find DNA’ claim…Prisoner reveals sick Larry Murphy’s ‘detailed’ boasts in jail - The Irish Sun</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Deirdre’s murder, hiding bodies &amp; ‘never find DNA’ claim…Prisoner reveals sick Larry Murphy’s ‘detailed’ boasts in jail - The Irish Sun</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 08:03:37 GMT</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxOeEZPYUEwOVZqWTdndzVRcHlLUGttakxOWkxVNnU0RlllYXNBVHptcDJ1RUtYcjI5MzJDeWdTT1ZrVnZFS202cEZyRG1Qek9QRG9tMk8yazVOanQ3MXNJOXY3OFF6bzU2aXZEd05ENTBBa2JKMGhkTmthSk9BT1VXcHJyVmN1ZzFFVkE?oc=5</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K60" s="1" t="n">
+        <v>46075.33584490741</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare (fallback)</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>GALLERY: Naas RFC President's Dinner at well-known Kildare hotel - Kildare Now</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>GALLERY: Naas RFC President's Dinner at well-known Kildare hotel - Kildare Now</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 09:05:00 GMT</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxNRl90ZnFUdnhLY2JBcGtZR2lTNWRfQWljR2E0a25iMDlnQkxZYlNqN0pDdVdYYWgxc0RSWkRCU1dKaGlSZUx2XzNjT0Fud2hoeXhKT19QeUQzTkJ3Y2c5R3dLM3ROcGNSNFV3cnRVaHBwNmRtbVZSbGZpLVlZSVdiZWxwd2lvWHV1c0lXeGZwaFNBMzdpUmxIcTU0dUhkczJ2VG9wZG1mWVpWd1lvSk9PSWVVem9pU0dpUWJQa3NpS1hzbDFJM2xB?oc=5</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K61" s="1" t="n">
+        <v>46075.37847222222</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare (fallback)</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>All you need to know about the February 2026 Local Property Tax allocations for the Kildare-Newbridge Municipal District - Kildare Now</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>All you need to know about the February 2026 Local Property Tax allocations for the Kildare-Newbridge Municipal District - Kildare Now</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 17:05:00 GMT</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihwJBVV95cUxQdUlQZ01sYVdUQk5TZllvV2hVZVFlb3p4WHNueDd2RENsTTkxMDFWVGdGWVlrNjFwdnRwdEVFRHEzWFVjRGZyVXBmd3Y0dENTWFF5WXh4OGtDcFdIUW1kbE95U1VDa2RrSnc5UUd4MGtoYmw1N2tmcFlJUzhKemxyU3FwQUxsUHZOZkV1a21uOUVPWkhvLUpCYmt3aWVBdnV6TXRySzlVbk5Cb2JqYm51M2VxVnhDZTRCQTdBa1duVlF1Q0Zrdkg5WHhjZExWNVdGcnk4cmNIRnJSLTFVdEYxd3hMM2U5cHVOVzRTOHExVktPaWQwckdnYmFmZ3NSWHVBZmxiTU5sVQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K62" s="1" t="n">
+        <v>46075.71180555555</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare (fallback)</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>GALLERY: Mable Lyons' 105th birthday celebration in Kill Village, Kildare - Leinster Leader</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>GALLERY: Mable Lyons' 105th birthday celebration in Kill Village, Kildare - Leinster Leader</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 11:04:14 GMT</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxNM0dVSHhHaGZlOXgtSjUxd0tCWkpJRllLbXVxamh4OG1ZT18wSkdMZy1MQ2ZNY0F6STVraDRnSkxYOEo3YVF3TDR4bS1vN2w2ZTBpcWc1SXJGUGE4VUx6SzJCVy1IeGVYQlcxUWNHVE9RQmlPM1hoeDN0RE1jX2Znc0NTRW9VYTg5UW1LVV9aUElLdEdNWTd0bmZSazI5RFgxLXRhVUd3QmhycnRGQ1RjNFNlcVQxZW5wSG5TTEgwbG5aQmw0azN6OEozR3c2cmQzTnVuTA?oc=5</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K63" s="1" t="n">
+        <v>46075.46127314815</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Village Fidenza (fallback)</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>("Fidenza Village" OR "Fidenza") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Fulgor Fidenza - Nuova Pallacanestro Vigevano: 89 - 94 tabellino campionato di Basket: Serie B Nazionale Girone A - basketmarche.it</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Fulgor Fidenza - Nuova Pallacanestro Vigevano: 89 - 94 Basketball championship scoreboard: National Serie B Group A - basketmarche.it</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Mon, 23 Feb 2026 03:57:00 GMT</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxPVklxcUQyVFRfaXl4bmRWYWFubU9hZkNfRzFyYTVaamx1aDRrN1IyOER1cDZrcWV3QVdnVFlaQjQybnZ3SHRLVTBZdXFpeHJudkJsOC1ONWs2ZEZaNXNCd2N6WkQwa0J4SS1RMjdNS3AtZ0t6c3NKU0UyYkZieUtEeUYyd0RJZHpBOVJpV09ybkRpZXJ0dEJERHF0b1FMcVBVYndvQXZSanl3ejQ3ckhJSlZjYUxMNzkyVnJaR3NKeXhqSi1nVzZZdHZTeGJfeHVfUWdIWElMV1Bwdw?oc=5</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K64" s="1" t="n">
+        <v>46076.16458333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-02-24 07:58 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K49"/>
+  <dimension ref="A1:K61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,32 +480,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>London Marylebone Incident</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>("London Marylebone" OR "Marylebone station") AND (incident OR disruption OR closure OR police OR bomb OR explosion OR stabbing OR shooting OR "suspicious package")</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Chiltern Railways to be disrupted by work on Tube - AOL.com</t>
+          <t>REVIEW: 'It's longevity speaks for itself' Shan Shui at Bicester Village continues to prove its mettle - Ox In A Box</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Chiltern Railways to be disrupted by work on Tube - AOL.com</t>
+          <t>REVIEW: 'It's longevity speaks for itself' Shan Shui at Bicester Village continues to prove its mettle - Ox In A Box</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 08:35:59 GMT</t>
+          <t>Tue, 24 Feb 2026 06:00:00 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQOGNjVDdzNXFXVEZHMEFmaGdnaVZTN1UzZ0txV1BGYzc1dm5CLTg2dmEtSEdYSVBlN3drRUVGSmJrNmg4QWxkdUd3by0wN0ZIRVNJd3c2cDJqenFCTnNyWTJyZnlEUVZ4MWFaU3p5LUJXNzNRWEhBVEVjUTQ1U2o2aGJn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxQNHhwYkgyd1ZmTnNNLVZCd3otNHlNa2VLRHhuYlN0VDZlQlk2Y1M2WFVLSUNJUDhVQW0yclppd01lNTU1N0JyUGhGb2ZfZ1hnWFJmUEhkZnZTd2Z3RW1ZbmFZeDBZMXlUTnVOWkFjbmdsdGx2TXEySDF3bF8yZVJTb3pvNVhVczVoTXdDbnBWSU14bTdyNW5GSW9zVEg5RU9FYlloWnltSkZtVURCT0JWNUdnQ0NlaUN3UEkyenZXNA?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -529,38 +529,38 @@
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46076.35832175926</v>
+        <v>46077.25</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Hof van beroep buigt zich over wrakingsverzoeken in zaak-Costa: “Mijn cliënt gelooft niet meer in een eerlijk proces” - HBVL</t>
+          <t>'Disgusting' bins and rubbish at Oxfordshire Sainsbury's condemned - Oxford Mail</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Court of Appeal considers requests for recusal in Costa case: “My client no longer believes in a fair trial” - HBVL</t>
+          <t>'Disgusting' bins and rubbish at Oxfordshire Sainsbury's condemned - Oxford Mail</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 11:23:00 GMT</t>
+          <t>Tue, 24 Feb 2026 05:00:00 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijgJBVV95cUxQNlh2cU1lN1puZmpfZl9TblJvbVRMOWtxMU5QNzZ2aDloSXNOZHFQUHN0ZW81SzJlcnZxaXJSSzFoUWNNY2pJbThxVk5lRm8yMWRWcHhTTEtick1DLXN1WVBLZmdISXJJSWJ3WDBNNVJSRHVWOHJuZUF4dUZMLS1YaV9rdVB5cFBHRGpac1duQm0wQURWenlGN3F1Yl9yRW5yOUVmdWhrejhSSENKa2lfdURpRW9PaVp3VlFEb2hjbk9veUN5X1VtWFRWSDRTTmZFYm95YlJrSTRIWHNmQ1lvak8xQ2w0MjdCY2NheUVqMUZ3azY0Y0c4TW1rRGNqbUtaX1hJSUU1aU1WWE9IZVE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOdXNXbzM5M1gwd1ZmUm5VWHdqYVZ4T0swWVNoaDlxaEk3dFNzWUxmODBnQklwNF9JOERhckV0RGVmNTF3aF9xcVVEQ3M2TzRORDBNVXJtcDdpeHV6ekVaMEVsWTUtVUZ2N2Y3THFrUmJMaVFMT29nNFNic2V5MmUwZ2pYUkc1dkhaakE1WjdkVFpQU2p1NFdpLUd3?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -570,52 +570,52 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46076.47430555556</v>
+        <v>46077.20833333334</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Ruben Van Gucht in shock: 'Bekentenis slaat in als een bom' - VoetbalNieuws.be</t>
+          <t>Rising UK Engagement with Chinese Automakers and Asia-Pacific Industry - IDTechEx</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Ruben Van Gucht in shock: 'Confession hits like a bomb' - VoetbalNieuws.be</t>
+          <t>Rising UK Engagement with Chinese Automakers and Asia-Pacific Industry - IDTechEx</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 19:43:00 GMT</t>
+          <t>Tue, 24 Feb 2026 04:33:36 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxQNTBkNjR2dWVMcWRqcEp5MmM0eHZSenlEOWVsejhsOXM2aDZsdHhKMlI5Vm16NHJreWM0MlA3WmQ3LW5WUTNxMVg0bS04dFFtYUdpbHNfT256QWhHM1kzVDQzS0ZtVjdQLTZlWjJvaTR3WjNDQWRzNEhyNzgxV3c5U0FpaUYxXy10alJUOFNCYk5GTWlTTlVVZkw5VFluM1lBVkE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPeDRlc29GOWdqOVQwYm5ZLS1BYUhHbXE4ZWFLOEp3ZEp2NU9kSHF2LVFyZmN5WW5Vb3lnWDdCRTUtZkY5REQ5ZVNNd29MRHZKdmVMRzFUcHZNTFhNN1VvZUVvcGQ3UHFibWRENE1mZG5EcTB1ODZlT2ZNYVA5dDJZeGhJUVgtUGZZeFo5T003V1ItUmR2b294YzVESUhzUVEzeG55TWVVY2JSaDhKeFBUSklzSURvZW5nNUNkcjFR?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -625,52 +625,52 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46075.82152777778</v>
+        <v>46077.19</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Explosief ontploft onder auto van volkszanger Frans Theunisz terwijl hij in Lanaken op het podium staat - Nieuwsblad</t>
+          <t>Changes announced for Oxford Tube services to and from London - Oxford Mail</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Explosive exploded under the car of folk singer Frans Theunisz while he was on stage in Lanaken - Nieuwsblad</t>
+          <t>Changes announced for Oxford Tube services to and from London - Oxford Mail</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 23:10:54 GMT</t>
+          <t>Tue, 24 Feb 2026 07:29:15 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-gFBVV95cUxPS1Fvczk4VGdrakpKT1VxdVNfZGNJZXc2LWt1dHF4S184U0MxNXdYME5xOVNzbG9oT05wWkVKQnhnZDJVUy1BT08xbWVfZ2NoWVc0TVpieDBtTEt2eF9BNjQzNG0tZDVKVnV5ZDRpRFh4b0t0TUlfUVMwckZoYkp3Nk84SzVVVnJDWjgxY0hLWGdFd1FEZ0NjYXQxNllySlhuekVQbW5qRHdMVGs3bTdRVzZpdHNqM2hKN2hRQmY1al9EUnNCTlBhVEkyVjU0LVhuYXJiVnBZaFFDTmhzM3FDcUxKckdxZ1d1T3VPQzJFUHg4Nk1LeFItNW5R?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxPaTRYa2NPSkxzZE1UWjRJSjU3eXZ3TkZka3VXdGd0YndMdHpscHJzSmJ6cWRRTGhNM2plYjFDX1hJeS00T1FMMGtnc3BsaEN1SmZ1dVYzSUFqc3pwTmtDSG12LWlRY3dkcXBxVTFUUjlubGs1dFhLMG9weGZYelhKcmZCYTQ5T1NoX292cHBWdGN4Zw?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -680,52 +680,52 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46075.96590277777</v>
+        <v>46077.31197916667</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Israel faces an internal time bomb - www.israelhayom.com</t>
+          <t>One of the UK’s biggest villages to become a new town – with cosy pubs and historic canal - The Sun</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Israel faces an internal time bomb - www.israelhayom.com</t>
+          <t>One of the UK’s biggest villages to become a new town – with cosy pubs and historic canal - The Sun</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 10:42:43 GMT</t>
+          <t>Mon, 23 Feb 2026 15:11:00 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE9UT1ZXandBRVdxaS1sbDVUNnVsVkhieWpMenNQLXlWZWxULWx0dUtUWHVDQUJpaWFzQUF0OFJBMHpRVXczTWxMVV9LWUhuSmUycFk0OVVqSWhQSVgzckVWcHBfQzhkcnYteC1VdGpiczd6cUMtZEFGeG93Zmc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxQTFdPODFXLUpCeFczUnFia3EtVG9wRmExQUV3cUppMmFkWEQ3Z1RzZFBHZVMxRl8yNThsc1JTajdfQjdzWmg2T2VSeDlSd1NWVWFjMmlxLXBaZ2dqVEhiR2FrMFhSTWV1dUNtbDF6SWpSZmtBRC1TWnh5Ykt1MDVESW5mR0U?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -740,47 +740,47 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46076.44633101852</v>
+        <v>46076.63263888889</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Shoplifting UK</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("shoplifting" OR "retail theft" OR "retail crime" OR "shop theft" OR "pickpocket") AND ("UK" OR "England" OR "Britain") AND ("gang" OR "organised" OR "trend" OR "rise" OR "survey" OR "report")</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Air Force One fleet to be repainted in Trump colours - Travel Tomorrow</t>
+          <t>Organised Retail Crime Surges in UK Costing Billions Annually - streamlinefeed.co.ke</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Air Force One fleet to be repainted in Trump colours - Travel Tomorrow</t>
+          <t>Organised Retail Crime Surges in UK Costing Billions Annually - streamlinefeed.co.ke</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 10:16:17 GMT</t>
+          <t>Tue, 24 Feb 2026 06:52:41 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxOeEwwd2VzTFZKaTJyblhmQXJONW9sNjVubTVtTmpEZjN1SW1XWXB4Qk9sMHNBZEhmdzh5OXZ3VUVhVUpGTWZsMTM1cTFuZ2VFQ0FjajlpejZwb3VrTllqY2NKWV85R3dmV0pBcUNrcFpDYmlzakpQTnotZmM5QXlBbHJaS2xGUEU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxQYXAwZGpoTUZsSlVHOUpRbDl3OUsycnA1RkEwNE9IdHE1S3FiZEhZbXdwcENSa3dSTEE4aDZIVTB6ZXJWZWx4LXN2N25WWUJrNzcySnlkV0dxWlhsQUI4aHUxalJ5LXhGSG1HeVZPMjRwWWE5Ykt1TUN1dFNZQVZDTXB0ZkVmbGFuNU5weEVZckJud0lRVkZZ?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -795,47 +795,47 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46076.42797453704</v>
+        <v>46077.28658564815</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>London Marylebone Incident (fallback)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("London Marylebone" OR "Marylebone station")</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Germany’s ruling CDU wants to stop Gaza payments via UNRWA - Brussels Signal</t>
+          <t>Farewell tour for 50-year-old trains raises £20,000 for charity - Chiltern Railways News</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Germany’s ruling CDU wants to stop Gaza payments via UNRWA - Brussels Signal</t>
+          <t>Farewell tour for 50-year-old trains raises £20,000 for charity - Chiltern Railways News</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 13:37:46 GMT</t>
+          <t>Mon, 23 Feb 2026 12:36:24 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxONTJpaS1CY1VFdHlVY0NtVzhNdTJmMG4wOHdydnY5MlM3bHVTZ2RRcVlzZ0dmX3JxdVEzNHFmM1VjWXZQOVlHVzdKU1I4TUMzeDJfZTAyNTJOVDgwcElQXzJfZzI0UFVZWGs3ZFdxMmlmNlF0N0pGa0pSY1hLWEw3WXFoVGx1WXFIaFZIeHM5VnVIVDNsMlFF?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxOOHVqT3VMZy1qWEJUZDQ3dU9nSWZnSmp1UDZmYjkzNlczRnpYRzJwWjRtWEdjNVF5TG55RUdPX2tuTjJEMWFWWG91T0dtVERUZTdQa2U4SmlaNGxfTlJtejg4Wjg5LWNTak1oVE9PNEhLM2lOVGxRZnVUT3Rmemd0SXhvbzBCTkx3bDBXdjVqS0V3TGdOUXI0N1UxZDg5bFRHWDZha28yc3ZCdnNj?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -850,47 +850,47 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46076.56789351852</v>
+        <v>46076.52527777778</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>London Marylebone Incident (fallback)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("London Marylebone" OR "Marylebone station")</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>"A deal is a deal": EU demands US to honour its trade commitments amid tariff uncertainty - lokmattimes.com</t>
+          <t>Chiltern to use four Mk 5A sets until late-summer - modernrailways.com</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>"A deal is a deal": EU demands US to honour its trade commitments amid tariff uncertainty - lokmattimes.com</t>
+          <t>Chiltern to use four Mk 5A sets until late-summer - modernrailways.com</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 04:53:47 GMT</t>
+          <t>Mon, 23 Feb 2026 12:00:00 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQSEt2eExmVkxGQ2hINXRmaTdwYXJ5NnhmdVNOM2ZSdGlHb1dxaVdyMGpaYnBWWTVmVVd0WXh5SnVkaVdfdU5RMkh3TGVxVlFSS253MkNLZjM0NXZzQWlSeGQtQWN1ZW1SaUdfd0w3eEtqT1RwWThzb2tfWUNFdEV0NmYzUTRIQ3JuN1JENmZUSWgyMy1JZDNsYzlQQ3FXTXJvRnR1VmJ1VHRHVVd4dldqaDRZY2V5OTdtRzRobWhpdFhkYzdVWTVF0gHOAUFVX3lxTE9KUnZzY2U3d3A4eHBpY3ZXV0RiWkhEWFl0M2VkUUExNW1DOTM3WE94RjZtMUxod0U0UFdKRmZ1RUVLTzJhUEV1NFNkX1ZMTFhtTkVvaWlyWVJNenlLdjQ5ZkVpYXhaWmF4V0ZFRzV1X0Nnbks0NmZsVFNpOTJWVlJiSTZnVEIyT2Q4ZncwSngzNE5INTZGQkJha0I0R3ZvMzk1WDE3YS1nUy1jYm42UjBYbkt3amRvdEVHTmN4bFVYV3NWbGtkOXA4ZmpwV3RB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOblRHV1pybVdYR1lYOUYwVTEteFIyYVZiYXd4bzFTc21UMDlnZFJLWklDU0FValplQ0RndTJNTjV0cm1sZG5jUFpWTzE3a3huRTV3YWRiSkZpcWwwNDhPQ3I1WFlxanhUNlZuNy1RYjUyNVA5Zk92aHJ0aUd5WXlhdVFONFI2RjBQZVR0NGpn?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -905,47 +905,47 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46076.2040162037</v>
+        <v>46076.5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Ukrainian oil pipeline "Odesa-Brody" may replace Russian "Druzhba" - Online.UA</t>
+          <t>Valse bommelding aan Grote Synagoge in Brussel: omgeving en tramverkeer tijdlang afgesloten - HLN</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Ukrainian oil pipeline "Odesa-Brody" may replace Russian "Druzhba" - Online.UA</t>
+          <t>False bomb threat to Great Synagogue in Brussels: area and tram traffic closed for a while - HLN</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 20:08:33 GMT</t>
+          <t>Mon, 23 Feb 2026 19:18:38 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNZlBCeEZXakZ5VVBhQWpxMEpCVzFtTm9CYlZ2emxsaXhUci1GUXRybGp0T2ZKRDJNYmFXYjFNZDRSS3NTLXBrRnVfS3RLRndzcFNTUU9rVGFmM3ZnV3hFbGNUN0JMVHRjSnpqWkVSWDFrS2pQa1JjeFZzN3luS2pqS1U3REhERHQ3dV9WUGVZeWl6Q014Sk5EenVfaGY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxNWTVCY1dETU45MTMzQ1l4YXhSaVQyWjhjQjRtd1E0OEdMNllTQnZ5SlJiN2Rod3JUaTlMMTU3bGM2U01jSkJuUkpCUlExQXl3MUFFcE1acFdpRVY4MnQtcVdoZW5zSHlGZDBIRWlGQTFtLWd6RzJraG9iWWd2RHdJSktMYkRfaWFBN3prOUFTQTZyS1F6OUdfOWs3RzFqSzlGRF9LbDFsUG5LM1pyOGxSbWJKamItVXRmMTM0UW5EbXlmeWc3eFE?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -955,7 +955,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -965,42 +965,42 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46075.83927083333</v>
+        <v>46076.80460648148</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Explosion and Fire Reported on Container Ship MSC Giada III in Gulf of Finland - 112.ua</t>
+          <t>Vals bomalarm aan Grote Synagoge in Brussel: “Volgens eerste elementen weer zogenaamde grap” - Nieuwsblad</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Explosion and Fire Reported on Container Ship MSC Giada III in Gulf of Finland - 112.ua</t>
+          <t>False bomb alarm at Great Synagogue in Brussels: “According to first elements, another so-called joke” - Nieuwsblad</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 20:17:56 GMT</t>
+          <t>Tue, 24 Feb 2026 03:20:00 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOR1plTldVMXlJQTNVdkJ5YWlRNmJZU1VRZXlVb1Vpc2pad0plMEZxWkZXenRVcVVzRnk3OXlBb0JPUFhYUmx4Q2Z3LV9DbG00VmFsNnRKR1RNdjhZUER5a0FiYmdjNk5zdEFydWdZR29mbkl2bzByUHI0X3dDWUZoUUs2bW5wQ3ZReVpFVHJuRlRDODNHSzAxYTBn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxPLVNGa1QzTEV5X253bFc0c0pCX0NmNVphY2tGVHJkN3BjS2tyd3BHSmo4cGtsY09FaTR5NjhKNU9Dd01rQjY1c0wwZUFQWVdlTlBSTjFMcDZaenRISzJqTUlTNTJmOFAzbVF0Ti14Vjl5aXZlNkhmSWM5NkNKcjlwNUxTWHJOUnBuQU01Q2tIUmVjdkhTd1V3S1F5dWNwd3NxQ0d2WTFwNlI3aVV5MjR6X3gxQVRRRmVmekllYTdoUUYxeG10cTRqb2hyZkI1eEtOMGRlLTllTmVUY2JPRFlXQUhYdEdIWnc?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1020,42 +1020,42 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46075.84578703704</v>
+        <v>46077.13888888889</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Un homme de 79 ans tire des coups de feu sur une maison avant de se donner la mort à La Panne - 7sur7.be</t>
+          <t>Vals bomalarm aan Grote Synagoge - BRUZZ</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>A 79-year-old man fires shots at a house before killing himself in La Panne - 7sur7.be</t>
+          <t>False bomb alarm at Great Synagogue - BRUZZ</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 06:29:00 GMT</t>
+          <t>Mon, 23 Feb 2026 18:42:22 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxQaE1ZcmdIVzVhMVE3bkJxRXdkci1DN25Sa3VQczFQQjN2R2NvQU51S3JuaURxOGtHZ2RTREV5Wm1zT2JWWi1NWm1ydk91eUluWk5GWHpOeDNHZl9SVVJEVG9FVlNwak9mVFM1TVk2anc1WFdnY0RpeWYxZTlCTUhGejJiZ2pPd2lGd3NDaWx5QmZ6Vkh2VHFiTnRqWXhBNmdzN0k5RF9vR05DUHVWVFhYSXM4SWdPanlKa0VHLWdfNUNzSHk5S3ZzS2VUMjNaTnJWc1R3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNUmhvam1VWGcxVmZOSEEwLXh4cHp0ZzBPa0dpR3dxRzJpcGFzRnY3Ylc5TlRPZVllcExRbnpBT0NhSVdiRUY5em1MZGFsdk1CcmVvQVphUkVxMG5nS29BT3FCWW1QWGN1QzVuT1lTVC1wZ0tSUmZQSTI4RjdHdmZYMkR0ZzlFb2dU?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1075,42 +1075,42 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46076.27013888889</v>
+        <v>46076.7794212963</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Marc Uyttendaele ne donnera plus cours à l’ULB après un “geste inapproprié” envers une stagiaire - 7sur7.be</t>
+          <t>‘Spion van Poetin’ opgepakt in Brussel: zakenman zou militaire technologie aan Rusland leveren - De Morgen</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Marc Uyttendaele will no longer teach at ULB after an “inappropriate gesture” towards a trainee - 7sur7.be</t>
+          <t>'Putin's spy' arrested in Brussels: businessman allegedly supplies military technology to Russia - De Morgen</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 10:32:00 GMT</t>
+          <t>Tue, 24 Feb 2026 02:00:07 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxQZzFuWjJVUFozaFJYUWEydER4aXlOX1ZILTZnNDFoY1VXaGY5UExQQktYcDlBa3hjZVNaZHJFYVRTWFJxeTM3dnJqTWlocGhIOHlBUlBzOW14emRnRlZ0a2JldXZQckVBcVgyajRIY0xEVGQ3cy1uQkhaQ3pNNlhublRzNUJwaXd1Z3BHN1ZseXhYbjNtTWFYbFFXdU5rR09OZTBLd0JxLWU0UGhuWFM4ZVpRcExHanNNQ2FQQ1ZYNkNJQkFEcVhiUmRaUkg2Z00?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQODlCWFZTUFlFb01fd2dRN05EWTBuT3YzVEN6YUhDWnRnR1FfN3Y5NjdXcWJaUGtjSzZ3bkJpWGFLVkd5VEpHNzF6ZElHSC1RUGZFZlRGZUkxTHJ2MXBJOWlVMkI1aUJGX2VqeEdHU2ZWUzhqMFJFNkxuSXgzcWFSR1Z0dmxrTUJmdmpacVZnTEplVDItbUp5WHoxbkFlcnRGYmVka1dMbGt1Wk5GeTZkb3Jma0swcDhJSkdiRy15bFNMQlFwV2hJNVBnOVk?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1130,42 +1130,42 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46076.43888888889</v>
+        <v>46077.08341435185</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Tajani à Bruxelles pour le Conseil des affaires étrangères : Rassurez les entreprises concernant les droits de douane ; les guerres commerciales sont inutiles. - Agenzia Nova</t>
+          <t>Papa zet zoontje af op school in Antwerpen. Wat later vliegen de kogels in het rond: “Hij zou 50 miljoen euro aan drugs hebben gestolen” - pzc.nl</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Tajani in Brussels for the Foreign Affairs Council: Reassure businesses about customs duties; trade wars are unnecessary. - Agenzia Nova</t>
+          <t>Dad drops off son at school in Antwerp. A little later the bullets start flying: “He allegedly stole 50 million euros in drugs” - pzc.nl</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 06:20:13 GMT</t>
+          <t>Tue, 24 Feb 2026 04:35:00 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAJBVV95cUxPdWVlY25DdEpZUGhvdF9ZZ0JPeGFzVl9sdEFfT2FaT1N6ZzFWWDJwNkh6bEtONXYxM2FlNHBKdTF1UXFEc09LVDI3V3RoLW9qdTdDWWpUMWItdzVOLXpyNkN2WUdUOE5QWjk3cnEwMlhKWmFZNTdjU0Y4M1FKUzZlODFmbkF6T1hTU3RnaWN4cHQxenI1RDNVRVBVcWJLcWs4YkJ3NmUxcHljbEJ3cVpOelpxVEE4S3F3dFQySE1CRU9xZnN5cHhRRVFhTTNrTUd2dVc0ejNzdUM5blUxVjBfa1dlYkJXTWplWVFKVWxXRUpQNWNicE1IZ3VPTUl5S1BJRmMzQ2QtNEZ3MWhBZDlPeW1KTUpMLVQ1b3JDLUphR1gxWFBi?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxOR3ZBTk1uT2pkY0thS0FZNWZFbjR2c2gxWkhBUEgtZExhc0ptdHU3RHk3Z2tCNUZVYjVIbExCd1BMUXRkQnlZeTVLMVRZNllzQmlwaEZOc29kVG5venNocmlsa09wd2ZScGJWSEdCd0t1SnBlQnB4VDNzaTNTaGUtemN3el9DWFB0OEJnb0p1M1ZuRXd2bDRkUnVLajNtbGVsbGNfTGUzLTFObGpuRDhJNWhrUEZFV2JpXzFxeXRCeXluSEpXTDZOVlZKOVlVTWJ6TDBFZm80V2dvZHB5WWhudExNN3ZIbzFsMXdSeU4xc21jWWN6eGhGRFFad0JuYlQ4?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1185,42 +1185,42 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46076.26403935185</v>
+        <v>46077.19097222222</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Accusée de harcèlement, Elisabeth Degryse réagit: “Ces cris et jets de signataires ne figurent pas dans la plainte” - 7sur7.be</t>
+          <t>Tiener móét van ‘Zero’ naar Antwerpen rijden... Wat later woedt brand bij juwelier en krijgen hotelgasten rook binnen - HLN</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Accused of harassment, Elisabeth Degryse reacts: “These cries and throws of signatories do not appear in the complaint” - 7sur7.be</t>
+          <t>Teenager has to drive from 'Zero' to Antwerp... A little later, a fire rages at a jeweler and hotel guests ingest smoke - HLN</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 14:09:00 GMT</t>
+          <t>Tue, 24 Feb 2026 04:36:58 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5gFBVV95cUxNdE1zQmdaVE4xOWlKZE9memxWRldLYjZwaG9acmZPME8zOXk2ZE1xZXBlX1loaV9oeTJmdnJuWVVYcnZIaXhUNklkaml4YkNaakVqaW5UZWZ3WEt0blVmZVdqQ3lfVlNKTEdCMUU3TGppdl9jMHh0MXUyOGFETHk1YTdQN2pOd0JVeFBRbnZwQjlib0dBUFBRQkUwQnZFQVA0YzZYbGxibW1XWVJNNTBBWkpzVU1JRzYwN1oyMW1RTGZteHJ4eE9va09taHduMm1vbW1Sal84cUJQMjk0Y1Q1OVB0Rk1YZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5gFBVV95cUxQX21rWDN5aHZDUzI2X1hIb1JxaDRVRXlEYlhMaGt2Uld4RjIwWGhDWWl4aVZsTVBlMndIVUZ2UFg1WUhGM0tMVXJTc3N3cFctUWJVNl9QNHRmWXpRWHowTkljR2dtNnhFSHJaY04zS01WYl83Y0gzcG5famVkOUs0TGJWZlpTX201U2hvOEdPVmFCNVNpV1pxb2VkallKbEtfc3Z2NGEwdmRZSmxObEVDQXAyM0ZPeWpORXhWMUJNOGo4UDZDQ0dheDBCY3ktYlVVblNHQ2VGalpTZVNWZzRfQmtkaVEyQQ?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1240,42 +1240,42 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46076.58958333333</v>
+        <v>46077.19233796297</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Il a couru aux JO avant de combattre la bombe nucléaire : pourquoi l’histoire de Philip Noel-Baker dérange encore - Daily Geek Show</t>
+          <t>Hof van beroep buigt zich over wrakingsverzoeken in zaak-Costa: “Mijn cliënt gelooft niet meer in een eerlijk proces” - HBVL</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>He ran in the Olympics before fighting the nuclear bomb: why the story of Philip Noel-Baker is still disturbing - Daily Geek Show</t>
+          <t>Court of Appeal considers requests for recusal in Costa case: “My client no longer believes in a fair trial” - HBVL</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 20:31:00 GMT</t>
+          <t>Mon, 23 Feb 2026 19:23:00 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiTEFVX3lxTE12aG1TZFZ1ZE43SkdRT1lfbTByMk1sS1NQQVAteEVGMWI0YmNpcWFtT0pwX1BXa3MtVm9UQ3dLbDhWaXZteXVVNTdGXzI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijgJBVV95cUxQNlh2cU1lN1puZmpfZl9TblJvbVRMOWtxMU5QNzZ2aDloSXNOZHFQUHN0ZW81SzJlcnZxaXJSSzFoUWNNY2pJbThxVk5lRm8yMWRWcHhTTEtick1DLXN1WVBLZmdISXJJSWJ3WDBNNVJSRHVWOHJuZUF4dUZMLS1YaV9rdVB5cFBHRGpac1duQm0wQURWenlGN3F1Yl9yRW5yOUVmdWhrejhSSENKa2lfdURpRW9PaVp3VlFEb2hjbk9veUN5X1VtWFRWSDRTTmZFYm95YlJrSTRIWHNmQ1lvak8xQ2w0MjdCY2NheUVqMUZ3azY0Y0c4TW1rRGNqbUtaX1hJSUU1aU1WWE9IZVE?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1295,42 +1295,42 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46075.85486111111</v>
+        <v>46076.80763888889</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>220 oproepen in één weekend voor Politiezone - De Internetgazet</t>
+          <t>Oefening Snelleresponsteam (SRT) levert indrukwekkende beelden op - GVA</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>220 calls in one weekend for Police Zone - De Internetgazet</t>
+          <t>Rapid Response Team (SRT) exercise produces impressive images - GVA</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 09:41:10 GMT</t>
+          <t>Mon, 23 Feb 2026 15:23:01 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxNYTBpdElMU1JKTjk3LXFvdXg0aG1LWVd4S1RZaEtXS3FfdzdCU0ZSQnE2NWJjX3JwU3VVNnlPRU9SN1VqTUtqYm9ON0FGVUY4STdEaFdWUno1WGxfTzRNc21wX3JkdUZ4c2p5LWZBVjhWcnRpXzVLekJaLXhyQnItY0NhcVo?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxPbDZkSXpSOUlTSzA1SWtYdTZFUVZpaTN3UFAzdzZUQkplNEk1SkFvSEx1dWpweWdvdFA0VlBYcDJ3VzYwZFR4bnpjUzZkTllXOTA5c0YxS284bTBfS2ZFa3RZVmQ0cnZyMmdmTk1mc1NuUWNVc2p2QV9haTNyRXl2THIxZFoxQ2hnRXY0eHA3eUYyWng4cUJhMkwtakpxdy1XM1VxUGlYR3llcnBHcHBlUHFVYkctNlN4NTFpWVlBYjJMeEotUm51V21oVktmbV9SSFQtX2RR?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1354,38 +1354,38 @@
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46076.40358796297</v>
+        <v>46076.64098379629</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Challenger Pro League : Renversant au Patro Maasmechelen, Beveren acte (déjà) sa montée en Jupiler Pro League - DHnet</t>
+          <t>Notoire drugsbaron ‘Flash’ gelinkt aan granaataanslag in Knokke-Heist - Nieuwsblad</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Challenger Pro League: Stunning at Patro Maasmechelen, Beveren (already) marks its rise in Jupiler Pro League - DHnet</t>
+          <t>Notorious drug lord 'Flash' linked to grenade attack in Knokke-Heist - Nieuwsblad</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 17:31:00 GMT</t>
+          <t>Tue, 24 Feb 2026 01:45:00 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinAJBVV95cUxOMlhPQzRIdU1oWjk2ZXgtQmpiQmowckwwY256b2pINDRDb01YVlhZakJyYmJiWFpFdEVxZ0FxY1pESDNRbGNLQ3VKSzJwXzVDNU8wZDhBYXFTaGZSTHpzdEU2T2QwNTUxdWYxcS01WUw0M3BSYXNUaWFucXZhUFVvSlBYYkFaeUM2Y1FDVkhsYWdBTzhoSVFkYV9LNjlCWFQ3U0JXaGVQWEd4VjgwdjVvbndxTmo4OTlwTUdMQkdwbXdIb0RzZWpTVUxtV2xPMFRObWI1d1RuNmVrMFJTZXhUeGZNMTNKYXdMSF9lTGRHaEFoLTJieC11eVBGWDN5SUZFVlZ0Z29IeFgtSEVUWjU4YkpJZWxNYjdVZUNGRw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-AFBVV95cUxOREMtU3Z3Q2ZUQmh2dTJKWHB5SDFYVklncFk0ZE1fUGRWUnJyUjN1OUktTGh1a29ma0ZFdFZYWENEQ3NwQUNrNEYwcW1JREdkTF9HaWlRR2pfOU04eHBXQXlHOFZKVUs3dzBvaFEyZll3eGNJUklvOFl1a0E0bnAybHFOT29YaGQyS21nUFYtd2c4VGVkZ19fb2FjQ2RtS29HZXdsLXp5R3F5RHh6VnFoTld6VTNOc3RXWlJ6dmhlTUJiTzRCTEpRVDBQdmxxYU1XbFhSdFJBTUNDLVQ0Y2Q0Qm5UTDdOekNqLWVGV2hlUWc0RVcwM0lnaQ?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1395,7 +1395,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1405,42 +1405,42 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46075.72986111111</v>
+        <v>46077.07291666666</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Beveren a fêté sa montée sur la pelouse de Patro : la réaction de Stijn Stijnen a surpris tout le monde - Walfoot.be</t>
+          <t>Oplettende voorbijganger helpt politie inbreker te klissen op lijnbus richting Antwerpen - HLN</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Beveren celebrated his rise on the Patro pitch: Stijn Stijnen's reaction surprised everyone - Walfoot.be</t>
+          <t>Attentive passerby helps police catch burglar on scheduled bus to Antwerp - HLN</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 12:00:00 GMT</t>
+          <t>Tue, 24 Feb 2026 01:58:36 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOMFZUdHIwV2NXVUVCZ2JjRVJ0d2Q2Q2ZOWUw1OFB5ZV9GNkt6eVNSS1h6RjhDbGtrNFg3eUhOU2NROWlxMkZ2ZVVxbTBaQ1dPTXZLYmMwcFVRaHNLOEdPVmZFYkptVWJxWDZiTGRlZjVPaHJTWGJ2UnhLaklhcW1TenlRd0FTUGZRZEtCdUoxUkFHNHpZamVYMGFSNFVyaDI2RUItaE5KeVN1dEZfQTRJNkdZUXp1TS1lRFNDUXVDZjhVZmRiTWsyVnlreUoyekVSUG5wWHVheVbSAd4BQVVfeXFMT2R1OWxYLVlQVHkxTkJOOFVTdVV4ZHA2Q2RiQXRpblVQdGV2Nlh2Q2xBMnBqSWxCaW43Y2ZKcTdIbWRDdEY2ZHVlN2NhRFNsaThCX0hpMDhsaXQ2U2lIZ1lWUGNvRTNndkJvWUUteXg1WWFIdnRXbGFhVC02aVc1RmtLdHU2dVd3RDliSHpndEg0ZzJyQXhacEl3LU05Mk5WWjZZUUdKRDVuS3IzN3NzdFQwX3VnbmctMV9QQWxtOElPT2Y1bFJXSFdKVTdvb3BibXFXQ25lLThqVW1CX0p3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPSVVWMEZtMTZNTVN3YnZYTjhHMGl5blBYNVVoZ2pTOWVzYlhKMm1hVkZRUWtmNEVIcWdRalJteGJuR3VSSU9IWEhUNTQ5aG9GWDBfYUNpb0dZdll4c2NJRTlCTXlIUDFNSkFMTWtQZ0I2SUU1b1Z1TGNhUzlUTWZ4dVlvd0lEQ0c0ZFVfbGZJellkNkFfSGdhU2pTSExLcUFod1JxMEZuVlE0UjExQnRQTHdQM1dTTUp4YldiazRYTmxTaVE?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1450,7 +1450,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,42 +1460,42 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46076.5</v>
+        <v>46077.08236111111</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Toujours invaincu, coach de 33 ans : le premier promu en JPL vit une saison impressionnante - Walfoot.be</t>
+          <t>Jonge ondernemers lanceren app die Antwerps nachtleven bundelt: “Handig overzicht in plaats van onoverzichtelijke waas” - HLN</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Still undefeated, 33-year-old coach: the first to be promoted to JPL is having an impressive season - Walfoot.be</t>
+          <t>Young entrepreneurs launch app that bundles Antwerp nightlife: “Handy overview instead of a confusing blur” - HLN</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 21:26:00 GMT</t>
+          <t>Tue, 24 Feb 2026 07:01:06 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxPUm1aUHIzYkdJcldqSDFGdGJnV2dhR2ptNXpyb2Q3cmw2WnhJVEpHNGhycTU3Qng0MFozcThHdUFwbF91WjI2Rl9JT0dLUHpPX1k0VG5Vc0VrZWU2X1ZNZi1JalJ6dHZDSE8wNXJuMm03cUxHNjRBZHpna19tc1FhQnNISHJHbUZjTTNWZDUtVGFOTmtzNUx2NzZ6V2M4WFVQQkF0S0RUNk9DTmNMWGtaXzhQeHFGeXUzRFdwNlJEYXF1ajdocnhr0gHMAUFVX3lxTE5RSHcwUHQ5dWY5Rmk0RkRWSUhBSEdEMnJXTWh2bWIzYTY4N3hmWnZocm42cE9SaUNfb3d6Y3FsNkdPQUpLbUduMXB1WGRRNTFrc0NzVHdZYm5vaTRUOXdWYUhPczVHLTJYZDM1ajRrVWEzcldycExJdWNiWElhSXhmN1A3MnU2SUNTWk1Ta3VrdVA0cUlZSlZibGJGcWV3VHE0Q0tVZWZRTEQtdjllandwNFQwM09feDlabG1aMHBjWEdhNVBjYUlLQ3d2SQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxNMkRPZ0ZtVEpRMHVSYTZGMDhqY1RYRzZIck0zQjE4MzM5UmRmdE1VUFpPSWJZR0ZCOTI0Y0kxQXc5VTVIejNuQzJQOXdhRThUc1NqWTBPajFnelFuUjZ4VzdPUmpLaDg2TmtMSU1FTWZzRGtsWjJsWGlrQW45Z041Y0d1UXotNzVHcUd5ZDhwYjJ1SUt3WXhibGtSZ2gzYkFoaTFvM3diYWlCYnVyc1hMczIzOGk2UHlkNWMxa25zRGF0VEdHNVBMNXpWYkxrR3AwYUlZbHA4eld3WVNXVkNkR0xIamI4ZVZQdXFB?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1515,42 +1515,42 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46075.89305555556</v>
+        <v>46077.29243055556</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Cambriolage au musée du Louvre : Rachida Dati finalement auditionnée à huis clos par l’Assemblée nationale - Ouest-France</t>
+          <t>“Ontruimd wegens zeer hoge CO-waarden”: burgemeester Els van Doesburg laat vier shishabars tijdelijk sluiten - HLN</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Burglary at the Louvre Museum: Rachida Dati finally heard behind closed doors by the National Assembly - Ouest-France</t>
+          <t>“Evacuated due to very high CO values”: Mayor Els van Doesburg temporarily closes four shisha bars - HLN</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 14:01:49 GMT</t>
+          <t>Mon, 23 Feb 2026 16:39:31 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimwJBVV95cUxNZmw4eWxPU2NZRUF6aHJSSmZFYWx2STRHd1dSZFJSNVQwNXBzcFlSYlpWendqN2NKVmY5YWp4OW9rLV9IVVJhMzFJTG9USmRtTTR2ZnNTOGVzYzd3T3docUI3MTllcW03MVhHZ0NPTDVHN094OG5pLUdrbkNPRXpqajFEWFZDQTFGaFdLbU56akZYSENfem5qUGVDVGdtdmRTSjM2NHdfZ3ppZHNkbDh4N1E2R1h6V0o0bVpWSHF0RXlfbmdfVDI5cFFoUmFVZnFUY1VRTmgtNngyMHFIaVhYYWRNQ0tGQThxQXVBOUdfVGVZSlNwR0lUaklzc2pWa2hTanJRTnhjeGIwYmhNN2ZvZk53QVVua0pHeUxn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxNY1BNank2aWc2R0RzV3ZpdUw4eVFYZTBwS2xrSVRHbERueXlIY3lTSGs5MFNVTkZnUVJpWXhnWE9vSC1FU3BUWkFFT2NuSVlzcHo4S29NYXJESENlQ19uMEVFdU1jTERFQjVvV1VGM2lGREZyTHRDUDZYdkZ2amVtSUJ5dlMxNUVpcS1jZTNma3ZmRnFkQ3NrLVNOdVlJVGZBQ0x2SWc5bVVKVFdKcjlVZ1pWSV84YU53elQxM09JcE5yeF9Ub2tFeW1DRGFaeVlmalhpaEpRU04xbXlW?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1560,7 +1560,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1570,42 +1570,42 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46076.58459490741</v>
+        <v>46076.6941087963</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Le Beerschot se loupe à la dernière minute : Beveren exulte et valide sa montée en Pro League - Walfoot.be</t>
+          <t>Expo met juwelen start eind deze maand in DIVA: “Toont hoe we kijken, waarderen en betekenis geven” - HLN</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>The Beerschot misses out at the last minute: Beveren exults and validates his rise to the Pro League - Walfoot.be</t>
+          <t>Expo with jewelry starts at the end of this month in DIVA: “Shows how we look, appreciate and give meaning” - HLN</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 17:20:00 GMT</t>
+          <t>Mon, 23 Feb 2026 19:13:33 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOMjM1SmJwVkRCWkx0aWwxVUpnYTA1dTcyMlpWTElWSTlQc1NGcHNaajRPTk9wVGxOMXl4clhJSWx2Z01XUXdPeFpCa3ZpT2c1T0pMam9GdG9jeDZENWlUWUt1cEV0SGozLTZDdmNaTWtaX3VaalRpd19jVHJyQmx6dlZIeDVhV09KSHN3NFllQmtaMElOWGVIcnFPVTd4QnFoUm9Wc09rbWpURXVYWkU4clRTQTJiNWxvVGlKSHJPN0VaSmxIOG5LUFJsVdIB0AFBVV95cUxQQmd0R2haLW1QSEM5WG4wVVZ1UFc4RWpVRFdka0pQQXM0QnVjMmVfQkdUSE5iejVKMmtFRHZ0dEJLWHk1VXJTeWNhVmJ0VTZEZWZoRy03aDJVQ2F3NlFfMnlTSFdZRHFvSW8yQkh4dG5HelFXNndaalZsYmJFS3dvSW9lTE5BMm1Ga3BlQ0VONUtjcno1Q25qaWxQak9oWG55VUpZMjV6U0ItdW9SMjJBcnRIM05tTllLMThMYXBkQmVIT0cyNl9kRXRSM1d5VHlI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxNaEtQeEJXd3g1aGZjNlZLampULUliUnNwUWIwMnpEdFhMdGozRWVTTzYtREpYNDlQVFdseElRb1JRMFV2Z2pXMEV0YnM5dGJaUzc3NzljQWxJdXFQd19NeVNxS0tBeUlLcjdEcGlQeFdsV1BoWThXcHhxV3Y1bndubjVlQ2VJcXFUTGJzMzNodUpPb2IzdVNDWjQ5aFE1S3ZLWFFBZ2ZuSThvU3hjODh1Rmc1eEJOdElDSUpnYk1zWEhPWXJTRXZZbWJ4dmRLOFU?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1615,7 +1615,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1625,42 +1625,42 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46075.72222222222</v>
+        <v>46076.80107638889</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>SA Winger Fires Beveren To Promotion In Belgium - iDiski Times</t>
+          <t>Modeketen IKKS in België failliet verklaard, tientallen banen op de tocht in Brussel - HLN</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>SA Winger Fires Beveren To Promotion In Belgium - iDiski Times</t>
+          <t>Fashion chain IKKS declared bankrupt in Belgium, dozens of jobs at risk in Brussels - HLN</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 10:35:28 GMT</t>
+          <t>Mon, 23 Feb 2026 17:13:38 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPS3ktRHpRekdhell6bG9ZVUdNeXhoQ2loT2RYMHl6eWNPNVFqd1p5Yk1wbGtPZGpzeGtkN0J3MGwtWVZhUm92NUFHSTk1bzR5WTlOTDgtbkZKWkpNbmgyUzFPS2ZJQXF4UnhRaGlwRW9jZldLNWdvU0FuOVdLVXMwMkJRaHlaVGdhUGZUY0YzX2V2Qkdrb0s5bHFB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQSWhmNWVoTlRWSHN4Q0RaVTBVT1FxYXRIa1RuVG15cjdsS0Rsa2VXNFpCWW1xU2tTZEFlRGVfUkYzM056YWJ2RVlFZ0FnN3lzYkNWUDlwd0h6ZVl1VHhORzVrU2JaOTYyVWllbEJsalYxeWZzZENPX3k1RS02YWFzWGpMeTBYTVdyVFNZcFJtWUdYQzBzcHpLaHowYkhnR0RwOVNmNFhFZGRZcXJ2ODVQYXJvTWtjTFdnb3huRQ?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1670,52 +1670,52 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46076.4412962963</v>
+        <v>46076.71780092592</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Würzburg: Nach Angriff am Hauptbahnhof – Polizei sucht Zeugen - Radio Gong Würzburg</t>
+          <t>VUB lanceert app ‘Moment’ om onveiligheidsgevoel in Brussel in kaart te brengen - HLN</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Würzburg: After the attack at the main train station – police are looking for witnesses - Radio Gong Würzburg</t>
+          <t>VUB launches app 'Moment' to map feelings of insecurity in Brussels - HLN</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 14:30:00 GMT</t>
+          <t>Mon, 23 Feb 2026 11:38:38 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxNUk1fcXRlQzR0TUx0eFZ4Rk1TMTBnQ2Z5RjJjeU02bGVXczhsQ0lfblVYOGJWRXRueExfZThlbTM2Smo3T25UQWs1TTNrZVRySUl6cl92NjJ1cktxVzltTTZmZGtJWXJVSWNWSmlDZVpYZFZiS1Q1WVgzRXFZbVBOT3lOUHlIbS1rMTBjQzNFNFhQdXFwLUNTZA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxPQ1RuNGMzWE1TNWZhc0xaOHI0STZsOXJzWW5EMW5rV1FMdzFWR1FqSHdEU0hNYm9wbXBaZkQyUzlzMm56M2tFQzRhWTdlWnBOMEFhanJIWFVVRGhiakF6SnpYWFpfeDgxTlktMUxlZ1hpeUVlMFc2NkFCSWphZVljWHFPMktpTW9tbWJwZ01UQ1htR2x0dVdsSDFvV1JORXh5TGdIcjBGVFVsUjlkSENZZXJ6VnQ?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1725,52 +1725,52 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46076.60416666666</v>
+        <v>46076.48516203704</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Schüsse in Kahl am Main – Polizei nimmt 19-Jährigen fest - Fränkische Nachrichten</t>
+          <t>Bommelding bij Grote Synagoge in Brussel zorgt voor kort oponthoud - P-magazine</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Shots in Kahl am Main – police arrest 19-year-old - Fränkische Nachrichten</t>
+          <t>Bomb threat at Great Synagogue in Brussels causes short delay - P-magazine</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 13:35:00 GMT</t>
+          <t>Mon, 23 Feb 2026 19:28:46 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxQdktzWkJUVTRINDl3TGRPNzVZUmJPYXRkWXlDbFJ1YUNMSWp6OUhNM1lrOGlHT3hiRm5OUXh5YTQzdk9aNDNMMERHTkNWMWQtYTZfdG5GdGRtSE92RE9DZkZ0N205d0FGUkx3N0VnV2haWkJVam5yN2xzTVc0RTl4TDRTUVdoTWNCeW0tbkkxU1VER0ZOZ0NMWFdzeUJ0ZWVOdjNqNXlqTXhFcDQwbnF2UW1WSHN5aUstTXlseWlGdkR3QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxNT3c3X25ZLW1HMjlMQ0VDZjZ1RFFvNjFRZ0tSdkJ1TEFlY3RWMnh0c2p0cmVCemVpSGdxU0ZNckVsbEVoUVFiT1BnTmc1bTdSSk56SFN5bU1PNHNFVFhka19saDJGV2wtb0lkNlhTMHZiTUowaEdvY1FQMjkzX3M4NFN1ZGJUT0NyZl94ZDkzaGtveVFYQ0lubXJ5RndqZXZBZWVB?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1780,52 +1780,52 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46076.56597222222</v>
+        <v>46076.81164351852</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Demo-Termine heute, 23.02.2026: Hier gibt's am Montag Demos gegen AfD, Menschenhass und Rechtsruck - News.de</t>
+          <t>Lijnbus belandt in gracht bij Pervijze: geen gewonden - P-magazine</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Demo dates today, February 23rd, 2026: Here on Monday there will be demos against AfD, misanthropy and the shift to the right - News.de</t>
+          <t>Lijnbus ends up in a canal near Pervijze: no injuries - P-magazine</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 06:09:00 GMT</t>
+          <t>Mon, 23 Feb 2026 21:03:59 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigwJBVV95cUxNcEw4UEFXTE9LZ3BUZHVRb0JhdDNVaTdaYUszLUdBam1CREwwRFN5NlUzUEdnYVZtN0dINC0xbTRudW5DSFR2QlY2QjhDVm5JMXJaN2F5SE5ubmMwWEZibXBFZ2tGM0c3dFZObV9FVGQ4dDlDam5GeDYzc09qWjJLdDBnMTdjTFJaamdheE1tX0FtaGt5WUkxdFVkZ0RXSWc2T2dlU3U0eXlhR2FhS2cxVU92OXVZcmpoUGs3allvX2h2S2s0ZWd1WW4yVGprekR2WUk1d2JPeEhhWFBnbHF1MG9xckV6dVppVEZKdnZvU05IQVRNdEZ0dGY0TDVoNmhrQ2tB0gGIAkFVX3lxTE1rWXg1LXplU3B4SGpfSG5LLXdwV0pGbEROYW5VUlJxWGRVVW9oZjgwY3djOENybFlTRDJMTUFmcVEtRmgwRGRNLV9vUWZ4M0tuenh1X190STlLX2FET09idW9Bak1JTFRtN2ZCM2NjeU9ZZElLY1A2V1Q4clNHZnhMR0NZVmFQMkpRUW1pckZuWnBNYmxicVpDZVNiMktDWUtVcHF4RGEycm5kOHN6dUJmMVdxdktDVTJLNzVsYm9vY1ZMOWh2YTRLdFcxRGFmZl9WdjNrRGR0c255SzB3R2pZZ1FTZUJlWWNHUWxwaTBmSEdYaTFXaFlRR3pEVDh5ZVJ2Y2cya1k2Sg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxNTHhwSmNYRHNtX1ZYal9wM04yYWhsQ3dYaGhPVzhiUGttV0lORnNzVkZNLWFiR3hxLXQ2QkhUMldCTmN2X3RYWlQ1V29ZR0lQeHc1NHlQT1BhNlZuMFRiU1hnQkpPQW1qeUl1aUhLelEweDRIS2l6TTRSeHhLdG8wRDRJblRGaWJ0bVk2V1NhZno?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1835,52 +1835,52 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46076.25625</v>
+        <v>46076.8777662037</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Würzburg Hbf: Mann greift mehrere Personen mit Messer an - New-Facts.eu</t>
+          <t>Obus ontdekt in Kortrijk tijdens graafwerken - P-magazine</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Würzburg Hbf: Man attacks several people with a knife - New-Facts.eu</t>
+          <t>Obus discovered in Kortrijk during excavation works - P-magazine</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 09:36:08 GMT</t>
+          <t>Mon, 23 Feb 2026 15:53:08 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxOM24zMzhrM2czdEk2MmF1TzJoSTdKNzZnZURodkdsRVFMZTIzakE2RDNTYWI3Wll6MzNNNUNsUDdsX09reEVwMF9nTGt6YzFaVkl4TnBfUzBvRzRKVGctdXpUUS1LTkJGMW1id1VFWFNsNm9ZT0FTMHM5LXA5MURHNnB5S1lPalRReDNtMWJOMTc0M1pUR05qN0tTckVhZS1Fa2ZpdElCaVlZMXUxaW93S3NFaEJHVGNuU1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxOSUc3UDRUeWljYlBzM1hETXpDTXZTekJ2SERQQlRMNE83RW51b3h3ZnVOdlBreXBqdUdRTTNxVF9RanlfTmNMaGpPb0oxc2E5Q09WU0k1NlpHckVpU0ptcHZjYnloRUFnTzF5X1R5bTlDQzRheG1LSWFWYzd1MGh6YllmZmRLdw?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1890,52 +1890,52 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46076.40009259259</v>
+        <v>46076.66189814815</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Village Ingolstadt (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Audi RS 5: A tonne (actually several) of talent - Motoringnz</t>
+          <t>Israel faces an internal time bomb - www.israelhayom.com</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Audi RS 5: A tonne (actually several) of talent - Motoringnz</t>
+          <t>Israel faces an internal time bomb - www.israelhayom.com</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 20:59:44 GMT</t>
+          <t>Mon, 23 Feb 2026 10:42:43 GMT</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxNS2Z2ZDJ2cE43aWEyaEFvclJ2WG53ZkJzTk9TMHdfa2dGSDBYZWlrUkcxRnRBaUV0NjZVZkExNFRZR3cwUWdURlhMcVRPRkhIdHd0dlpfWi1ib2hnWndCQlZwYl9LMlYwaTg1dTZWQ1h4bFZjSHNDWml2QmxySXhSZ3J1Q3NPamVHRU1tUkk2Zw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE9UT1ZXandBRVdxaS1sbDVUNnVsVkhieWpMenNQLXlWZWxULWx0dUtUWHVDQUJpaWFzQUF0OFJBMHpRVXczTWxMVV9LWUhuSmUycFk0OVVqSWhQSVgzckVWcHBfQzhkcnYteC1VdGpiczd6cUMtZEFGeG93Zmc?oc=5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1950,47 +1950,47 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K28" s="1" t="n">
-        <v>46075.87481481482</v>
+        <v>46076.44633101852</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Village Ingolstadt (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Lamborghini Technology Boss To Head Audi R&amp;D - AutoSpies.com</t>
+          <t>Hungary Blocks EU’s 20th Russia Sanctions as Oil Row Sparks Explosive Brussels Showdown - The Times of India</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Lamborghini Technology Boss To Head Audi R&amp;D - AutoSpies.com</t>
+          <t>Hungary Blocks EU’s 20th Russia Sanctions as Oil Row Sparks Explosive Brussels Showdown - The Times of India</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 13:01:28 GMT</t>
+          <t>Mon, 23 Feb 2026 17:55:34 GMT</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTE4zU1R5OU1XNHpNbXhaWHY3N0hFdFRKNTl1UTJnQU5fc1prNUw2VjU1QTlCcUp5d3BFcGNsc2VjaTBOalEtX2N6RHFXZVFUcnNkZGZBWVdmSXRYZFNxRjhSaGtrdjQ4cndUbVljMWVn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxOTlJDdnZJcUhhajNFWEtvMldrV0NBVDlQbThJYXI2MVBCbktZNWQ4dEtWVEc1bW9KT0RkRTFGcENzamNHQXd2STBjMVRQc1N5S3pvdHJ1TGFjeTc0STZMZ0t4MFY5RGJuNnowc3ZFcDRaV1VZQkNqNWF1Q21hcEcyc1VqTi05SUl0eF9nQ1lYYlFoQXNuWjdsM3c5TnNUeGliX3dvLUdwSWk0YzY0eENTb3hhNDJFN3VBMHZpRlViQ0lrcVkzLUFXS1BGdzNyZkd2ZDBMdzdEU1JSOUxHV0ZsdGZHRU9LSGl3SHpRQnd4RW5YdS1Udlp5S19jVdIBgAJBVV95cUxQSno4aUl4RDNXXzh6UXNFdWJyMHh3SkJzbEd5NFI4ZE5PRFRHWE10ZllZXzNVam1LdXZWYnBaeU9PYkJvcks2VXRLeEZlRFR0VFp1N21XZVdiMGZXaGszMER3OERaR0hHbDREYndvQ0ROdmFEa0l1dkFxemVRNkJBOGtNVFNWQjJpeW5DWjFneTBBMDlQbjlOVXRBanNybjNMR2ZZQkRyM1lRUDNHV0YtT3pYbVAwbTNuX1BBckZRa3RfeHd1SHhlOVZheldMTzh4eEZuWkZWa2VTWXNfaDV0TWx5a2lqcm4zZmhDaFpEQ09PMXhlYnRVRDJqRXNQdERG?oc=5</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2005,47 +2005,47 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K29" s="1" t="n">
-        <v>46076.54268518519</v>
+        <v>46076.7469212963</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Village Las Rozas La Roca (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>("Las Rozas Village" OR "La Roca Village" OR "Las Rozas" OR "La Roca") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Spain: Las Rozas Black Demons rally past Zaragoza Hurricanes in second-half thriller - American Football International</t>
+          <t>Germany’s ruling CDU wants to stop Gaza payments via UNRWA - Brussels Signal</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Spain: Las Rozas Black Demons rally past Zaragoza Hurricanes in second-half thriller - American Football International</t>
+          <t>Germany’s ruling CDU wants to stop Gaza payments via UNRWA - Brussels Signal</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 05:45:33 GMT</t>
+          <t>Mon, 23 Feb 2026 13:37:46 GMT</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxPcGUwMFYxdHY2dEZ6TXR6aFk2MlowaVV5bElVem9WRDBobjRld2wzR3dmWHBqZjBIVFdWQXVrWGM2VE4xSERvcnBTc3ltNFVCeEJlSXFMd2pIQ3kxMHIwWXFReU1KSnMtZGx6LUpFSE1iUzlXN1lUNGJfVnZPclVhM0ItN2h1SnVVNU9renpfVmlpTEJvMnhERElrR1JVZkdZeGRYV0ZKcjVuOC0xNGhrbXdsWjQtWHZtNHIxS3dJMm1TS0F1ZDB6TTZ4STl1dzTSAc8BQVVfeXFMT3BlMDBWMXR2NnRGek10emhZNjJaMGlVeWxJVXpvVkQwaG40ZXdsM0d3ZlhwamYwSFRXVkF1a1hjNlROMUhEb3JwU3N5bTRVQnhCZUlxTHdqSEN5MTByMFlxUXlNSkpzLWRsei1KRUhNYlM5VzdZVDRiX1Z2T3JVYTNCLTdodUp1VTVPa3p6X1ZpaUxCbzJ4RERJa0dSVWZHWXhkWFdGSnI1bjgtMTRoa213bFo0LVh2bTRyMUt3STJtU0tBdWQwek02eEk5dXc0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxONTJpaS1CY1VFdHlVY0NtVzhNdTJmMG4wOHdydnY5MlM3bHVTZ2RRcVlzZ0dmX3JxdVEzNHFmM1VjWXZQOVlHVzdKU1I4TUMzeDJfZTAyNTJOVDgwcElQXzJfZzI0UFVZWGs3ZFdxMmlmNlF0N0pGa0pSY1hLWEw3WXFoVGx1WXFIaFZIeHM5VnVIVDNsMlFF?oc=5</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2060,47 +2060,47 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K30" s="1" t="n">
-        <v>46076.23996527777</v>
+        <v>46076.56789351852</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Village Las Rozas La Roca (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>("Las Rozas Village" OR "La Roca Village" OR "Las Rozas" OR "La Roca") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Spain’s luxury mansions: where global buyers are investing - Idealista</t>
+          <t>EU adds eight Russian officials to human rights sanctions list - The Straits Times</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Spain’s luxury mansions: where global buyers are investing - Idealista</t>
+          <t>EU adds eight Russian officials to human rights sanctions list - The Straits Times</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 07:00:00 GMT</t>
+          <t>Mon, 23 Feb 2026 15:16:00 GMT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxQR3djQzdWMVh1UWY0OWg5YVdaMno3OVpMbHVJUmxSVTRfVVRuZ1FfVHdkVzBoWFlRVV9TVldvS1A5a0xlVHdKT0NBZjhpUGprZ3VZOW9XMFBGWU5vb3VmZm9TRThGZkdPMTV1V29LTlZVZHdadWdiR0FmVUtrcXl4UV9aSVRLaHo4MzI3MWx6OXZfQ21kZjVjN1ljbE9aTHM2Z2ttaDNLX2h1QnEzempOY05MYzJpMHNZU0xzQVVPX1pmMmRUMGhFMHd5elduSUVPTW5DMWVQOUHSAdgBQVVfeXFMUEd3Y0M3VjFYdVFmNDloOWFXWjJ6NzlaTGx1SVJsUlU0X1VUbmdRX1R3ZFcwaFhZUVVfU1ZXb0tQOWtMZVR3Sk9DQWY4aVBqa2d1WTlvVzBQRllOb291ZmZvU0U4RmZHTzE1dVdvS05WVWR3WnVnYkdBZlVLa3F5eFFfWklUS2h6ODMyNzFsejl2X0NtZGY1YzdZY2xPWkxzNmdrbWgzS19odUJxM3pqTmNOTGMyaTBzWVNMc0FVT19aZjJkVDBoRTB3eXpXbklFT01uQzFlUDlB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxQTU1vZDZ1QWVmS3RBUktpb3I4a3pkN1FFaGtkRkl3U0FKOUVQUF9Ec0VmVld3ZHJXQ3B6aGpZS3dxU3hzdms4Y2w5cGZWZGw5UlZmenVlRl9ZdkZidEd2OFUtRll3UlFIbXAzTGpUeVNhZUZlVUlBbUp2azdxYnROMDRFYmRYOFhVLTNMd3pWQXhmaUg2Qk9LNDdxd3BxM3BqelAtSVctWXNPVzRETmZySFZLcjdDcEpDR3BOTnJ4X1l1dw?oc=5</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2115,47 +2115,47 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K31" s="1" t="n">
-        <v>46076.29166666666</v>
+        <v>46076.63611111111</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Tributes paid to Kildare couple killed in road collision - kildare-nationalist.ie</t>
+          <t>Nadezhda Neynski and Mark Rutte discussed the changing security environment and transatlantic relations - fakti.bg</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Tributes paid to Kildare couple killed in road collision - kildare-nationalist.ie</t>
+          <t>Nadezhda Neynski and Mark Rutte discussed the changing security environment and transatlantic relations - fakti.bg</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 12:14:14 GMT</t>
+          <t>Tue, 24 Feb 2026 02:44:00 GMT</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxQYXB4b3ZvUklCZkNkMjdEaDRwN2FrN0JaaXJNQXpzV2tybENnb1ZjX2kyQUl2NU4yNUlTT1RXcXpTVVRIQktyTlpWUFNmMFFKX2pSR1B1WWUzMDkweGZoUWE4ZHkySlYzVUtRdFExUm1aTjNkcFdZY3IxNkxCV2k4VHc3a2EwUGtVajNBZWstc1ZDaXpkZUh0RG80dlV2eHg5OW8zc3pFRTBjLXFGeS1xdkR3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxPN1ZLQW9wZnR3UzM4bzVkNWZhbW1NS2g3WHRucjQ5RC1YZHNncWhzZ05VUWdOLWNSRnJhZ3FaMTlWVzRxLUhhTnBMYlh2VWF3V3dtSDBfaDNMdkZmN3JaaTdQUHhmQ0MwYVpLQmtTeVJzNjUwWEJVVUNpRmJsbnNzQjB2dFFUVktmREF2UEpSRm1XYmlPaWd5X3YxNGRVeWdoQUZlOEdjZmZMc09XaG9KMFN1ZEwxN1I2RHR3Y3JnMFk0aHYtaE9vYlFIMkxIU2NFeE9FVDNDU2c?oc=5</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2170,47 +2170,47 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K32" s="1" t="n">
-        <v>46076.50988425926</v>
+        <v>46077.11388888889</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Kildare workers being forced to give up right to work remotely - Cllr - Kildare Now</t>
+          <t>Fire breaks out after explosion at Baku flower shop - Latest news from Azerbaijan</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Kildare workers being forced to give up right to work remotely - Cllr - Kildare Now</t>
+          <t>Fire breaks out after explosion at Baku flower shop - Latest news from Azerbaijan</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 12:30:00 GMT</t>
+          <t>Mon, 23 Feb 2026 10:27:55 GMT</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxQYTFHcVRLbTdXdW45dWlLR3l6ZkpCS0RtZVVDd2M1dGprU1ltY3Y3UXVjemlqLW9PNkw2Mm91eDdsU3liZTYzX3hPSXZYSEpsZG04dTFrREFaY3EtVlU3TG5YVFRfT2JSd2FDSlIybmNKN2ZfZ0NCazdpenZEdXhvS0RIYkExVzVxZWFQNFFHbmc0dHZtUUVVRFJ1SEFnbzZHT2hwOXg3ZnRQTl9FS1lnN29B?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE1GUmdfSEw4Y0xPQnNwazNxWEY0cm56RjZIOWZ0R0lFVVZtanZuRXBOWUNZUWVURWdGaE9peWlud0NwZFYxbUhzTDZLcGxsM3pEWm9WM2ttbm9uczJkVzVEdTNFNm83NXFSQW1LSTBxeF9YLVRYUVZodmN3WFQ?oc=5</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2225,47 +2225,47 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K33" s="1" t="n">
-        <v>46076.52083333334</v>
+        <v>46076.43605324074</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Search operation underway in Kildare after reports person entered water - Irish Mirror</t>
+          <t>La Grande Synagogue de Bruxelles visée par une fausse alerte à la bombe - BruxellesToday</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Search operation underway in Kildare after reports person entered water - Irish Mirror</t>
+          <t>The Great Synagogue of Brussels targeted by a false bomb threat - BruxellesToday</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 17:56:34 GMT</t>
+          <t>Mon, 23 Feb 2026 18:51:00 GMT</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNR0FNY0lDUjkxYTVDbjNBVFBEclA5cVpETmRzaHhqc2Y5VTMxMXBOeXJpOENFb3FqWFBUeVJpbW9CSUVsS1QtVDlIR0JZbFJRc011aVJJOWFmRUxEbGxob24telZKWFlVZGctcXlsM0Qya2h1MXFRQnVEZThoYy1WTGZqLVN5djZIakZqSU9tSjE3S0RIUGfSAZsBQVVfeXFMUHhNb1lyLS1qMkk5R3RibzdCWUJHNkEwOUdHZGRUOHFVb1VOal83VTNHWl9Pek1hVnRyMWNjVHJUcnEtYldjdFZCc3N1aDdNVTk2UjQyQVVFWGNLSUFaOERaQXJxSktHaW9XR0kzLVlQY1FOb25INm04eDlvUWs5cjlOTmdGVG81QzNVQTYxbVBLQ3ZlZFNNMnJqc0k?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE5nRUxDNnpMb3JkTzgwMHV5YmVnMkY0M3JZWGIxMjhvNFBlTnQyXzBmdHFSU2x3LU5DTWw1Tm5sdjdSRDFSWVd5dmkyVWVOQzVMYkZwUWV5X3BhSmxXUTI1Qkp6aF9Wb2lnUHNQZjRqcjZ4MWFKWHc?oc=5</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2275,52 +2275,52 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K34" s="1" t="n">
-        <v>46075.74761574074</v>
+        <v>46076.78541666667</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Search continues in Kildare along the Barrow - kildare-nationalist.ie</t>
+          <t>Trafic de stupéfiants à Montignies-sur-Sambre: Un individu arrêté - Télésambre</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Search continues in Kildare along the Barrow - kildare-nationalist.ie</t>
+          <t>Drug trafficking in Montignies-sur-Sambre: An individual arrested - Télésambre</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 12:34:17 GMT</t>
+          <t>Mon, 23 Feb 2026 15:16:10 GMT</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxPQ0ZHNG9EZklpZHFCNEs3ZEJUOVpTM25ENmZKdEg5LWNQLWVuM2ZsWXZUZlRYQzRzb1cxQlRUVnUwZF85eFlvYm44Qklvb0RmcTJqMHNjU012VEVJY3J1M2RFZ2V4em1HUFlEZUN2TzZ0cDVZNHV4QzROaEJrWkwwMDd2QnlScVBWUW5VektiSlgta3kxVkdxLW5OYUV0eG9FcWc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNSXp2bmZ5TlN5YkZZLTBhalF5SmRHRGd4Mk50dWZZdW82WngwNXVXTDNSUXdfdWZET2t1dlNCcjZLTVdOY01DYTBQaVMzY3draDBabE13cHlYZ0xJeGNwYlhGdkNLU0JkMGZvSW5xZGZxX0FWLWtFRmF6N0R0TFlhdFVnZXNPczVNUG9zT0ZYMUl6TlFUQ09SbHFPeUZ2SFk?oc=5</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2330,52 +2330,52 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K35" s="1" t="n">
-        <v>46076.52380787037</v>
+        <v>46076.63622685185</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>LGFA - Dubs secure victory over Kildare - dublingaa.ie</t>
+          <t>PostNL va installer des distributeurs automatiques de colis en Belgique - 7sur7.be</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>LGFA - Dubs secure victory over Kildare - dublingaa.ie</t>
+          <t>PostNL to install parcel vending machines in Belgium - 7sur7.be</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 17:24:44 GMT</t>
+          <t>Mon, 23 Feb 2026 09:39:00 GMT</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE0tWDdBeWpTdkNBZVhiRXNuc3ZrcGQ4RHZpbzRGd0M0WTZzNDBVWUk0T2RsZWR4M3hSTWJZYUFZdzBFTF9yTzNfX08yN2Q1R21VYk1DYmdtTk1QaDd4MzBxNjdMYkk0Y18zbjhraC1LNXNUSTBzeFE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQUXVDZWdDN1M5TnNNUXptdEQ4UWFzdnRCcmVOZ1U3QnpaYzZkTGpybXlaTHRKV2s4eUF2YnNTbEU1MjIta0YwSTdaSXcyRHA5M0ZuU3lMY3FsU19VVWdwNGpwVjdYQjBPYzAwRXJNY191UU9oSmNsQ3k3N3ZRRjFKN2pEcjhHTDNhdzllYkVFYXhHQ3hoMjhvNmdBTWxnY0M2emk1b09QQUxSZk5ITGJsRQ?oc=5</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2385,52 +2385,52 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K36" s="1" t="n">
-        <v>46075.72550925926</v>
+        <v>46076.40208333333</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Former husband 'does not accept he is divorced', woman tells Kildare court - Kildare Now</t>
+          <t>Elisabeth Degryse répond aux accusations de harcèlement: “Ces cris et jets de signataires ne figurent pas dans la plainte” - 7sur7.be</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Former husband 'does not accept he is divorced', woman tells Kildare court - Kildare Now</t>
+          <t>Elisabeth Degryse responds to accusations of harassment: “These cries and throwing of signatories do not appear in the complaint” - 7sur7.be</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 15:00:00 GMT</t>
+          <t>Mon, 23 Feb 2026 14:09:00 GMT</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxQWmxiZWhLcV93VXNZcWFrQ3UxM29xVnJnNEVSZW9qVFdqc2dJY0xmd0d0SGZ4WHR3eWEtRmwzbnZUNi0yNmpnVTB3LXpRalpGOWZldmZOYjJkR3NQODdTY2FWU0xOSHVYWG5NWlBnRHduS1l1T05fZ1Q5Q1hrTUJ4czRPMFRvUWo5NWNubmVJNk9QLXNpMFZoaVRpeFBZT0x0RUVOcVFoSllnWVNlLTctLXpRRTJ5cl9ZemlDc2FoZEI2VTJVSlE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxNSWJoWVlHOGJFNi03b2w5Y1p6UmxvSndnOF9pTHBZOVBMZnNoN2RweXBoN0hKamlQSFZFSklRNUY3NGp4aktrUDExbjBObDQ5ZkoyeGliZTcyMC1iZTJYTE05eEZMbUVmb2lEWmpxb3RhRlo5cVRHbjJtTVRkR2JBeDRxc29veThvdWRDaUZjcER5WEM3QTZyNWZHanZjbjBVb244bC1KUmNMU1VYVXVVNndRU1ZBUC1xdFJhTlowa3ZoeTBjU0FaemVVdzNoelhaektaUTZrSVZ2QmNzRHNXN0o2LUwwT0xQY1FUbnJEN1E?oc=5</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2440,52 +2440,52 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K37" s="1" t="n">
-        <v>46075.625</v>
+        <v>46076.58958333333</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Poor Kildare give way to Cavan in dismal affair - Kildare Live Leinster Leader</t>
+          <t>Marc Uyttendaele ne donnera plus cours à l’ULB après un “geste inapproprié” envers une stagiaire - 7sur7.be</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Poor Kildare give way to Cavan in dismal affair - Kildare Live Leinster Leader</t>
+          <t>Marc Uyttendaele will no longer teach at ULB after an “inappropriate gesture” towards a trainee - 7sur7.be</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 16:59:27 GMT</t>
+          <t>Mon, 23 Feb 2026 10:32:00 GMT</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxQVml5ZlNRaEhfTi1WbEpTcC1VS3lGZnZyaDBPS2pPdWdRVFF6NXE2LWtwWHlCZENmSjM3bDhiMkE0NlN3OGJ3RHpreEswMUgyd0VKbk9qNEpnSjFjYWk4NTlVRGtHSlBQRjA2ZGRVaFE4YUFyY3JhaHN5LXYtNk11OVNhb0NvLWVib3c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxQZzFuWjJVUFozaFJYUWEydER4aXlOX1ZILTZnNDFoY1VXaGY5UExQQktYcDlBa3hjZVNaZHJFYVRTWFJxeTM3dnJqTWlocGhIOHlBUlBzOW14emRnRlZ0a2JldXZQckVBcVgyajRIY0xEVGQ3cy1uQkhaQ3pNNlhublRzNUJwaXd1Z3BHN1ZseXhYbjNtTWFYbFFXdU5rR09OZTBLd0JxLWU0UGhuWFM4ZVpRcExHanNNQ2FQQ1ZYNkNJQkFEcVhiUmRaUkg2Z00?oc=5</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2495,52 +2495,52 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K38" s="1" t="n">
-        <v>46075.70795138889</v>
+        <v>46076.43888888889</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Driver fined after filming garda incident in Kildare - kildare-nationalist.ie</t>
+          <t>Opnieuw laadkabels gestolen, nu in Maasmechelen en Lanaken - VRT</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Driver fined after filming garda incident in Kildare - kildare-nationalist.ie</t>
+          <t>Charging cables stolen again, now in Maasmechelen and Lanaken - VRT</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 07:03:36 GMT</t>
+          <t>Mon, 23 Feb 2026 16:16:31 GMT</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNT0F6MzV3LUtGWGx6Q1Y2bUExeU1ydEN1empwRnFYQTN2T2t6b0swb1V3c0I0MEM0QUZlX3NnWGJpYTB4endTNmNRelUwa29FY2xIaDc3SFNBd0xnSWhlS1NPT21NU0cxVUdMZFdtcTF3TEtKdFFJWGpuR0ItQno1TEw2U0NqdFJvbV8yWmRoeGJxa0xNTUxQUHFFSWYyVXZ6bjVYWkI4dDR2R1o0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQLXpEcnVvUUFXZTVvb0o3cEl0bG8taUR5R3ZmT1RybVhhNDBXeHFaNHZ3TWlabXpySzljU3JiTTlPc09uaElITUlISDhBTERBcW10ZEdvV3otMG4xZm50R1IzOEpzX05sVzVMb3VwMGNyenk0MWNIYlY3andhSWpNdWQ4d3NNTlowbGZDV0FXYTNLRHc4RjdaczdLaTJiRG8?oc=5</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2550,52 +2550,52 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K39" s="1" t="n">
-        <v>46076.29416666667</v>
+        <v>46076.67813657408</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>McDonald’s drive-thru causing traffic jams in Kildare town - kildare-nationalist.ie</t>
+          <t>Vakantiehuis Fabiola in Maasmechelen voor kinderen met een beperking krijgt toch nog 1 jaar subsidies van Vlaanderen - VRT</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>McDonald’s drive-thru causing traffic jams in Kildare town - kildare-nationalist.ie</t>
+          <t>Holiday home Fabiola in Maasmechelen for children with disabilities will still receive subsidies from Flanders for 1 year - VRT</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 20:01:39 GMT</t>
+          <t>Tue, 24 Feb 2026 07:52:45 GMT</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOWElKdEpWUmpFTWczS2l5LWFob2pDaGdpbUJyWFM5elFGajFkQ21UM3hyeHc4NXJnZ2x3ZW1vdThhVVRjVW9jbXhjWHZ3YTRFQlpXY1VqQVdINFdLM3NvWmxOZ3pwZWNCLVB1MlVrYU11WExvWlY1YnZlbEVzcUw5RUhCUXJTekRMV2hBS2RJX3A0ZFRjQnlrTE40NjNBNnlQTE53ZTdEbWQ1RXNrTVE2RG1QVQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE5OenpKUkhrQ1AxTlBhUlRETGdRSFpRaVJKOW9TelBUUXdpU01tdmEwZ0VFM2dvR05IaFViZkVWM0YxLVlwU2ZETUxJbld6c3NrTm1DU1Z1SWlzZG9PNWFyZEJMSEVyX2hCY1BIa1RGaHdtQi1OQU9pR3ozdw?oc=5</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2605,52 +2605,52 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K40" s="1" t="n">
-        <v>46075.83447916667</v>
+        <v>46077.32829861111</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Kildare sucked back into relegation dogfight after dismal display in Cavan - kildare-nationalist.ie</t>
+          <t>Filipijnse oud-president Rodrigo Duterte staat terecht voor Internationaal Strafhof - MSN</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Kildare sucked back into relegation dogfight after dismal display in Cavan - kildare-nationalist.ie</t>
+          <t>Former Philippine President Rodrigo Duterte is on trial before the International Criminal Court - MSN</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 21:31:41 GMT</t>
+          <t>Mon, 23 Feb 2026 23:49:19 GMT</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxQSnZwWEF3a2xxcGNSYXhhcFBIN1pnOHJ3TDlIY3BIeEdvX0R3WmZCVUJaem9WRmR0bVdqMHBsU1JvbGVsRUcxZDZMdGlyc2pvN1Y1SkEwMVE2NzNqNE1OTkIwSnBlSURnWWdpZ3d4OTRsMTAxV1JWUHprRUVKNXoxTG93TE9vMm45V2h4SjJ3R242Z1o4Y0pQcUU0NVVJNGhSWmszeXNWVHA1ZldGNTVFUDNzRVVPQ2x1Zl9rLVJpVERfRWZ5YlNwR2ZR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxQSlN1U2R4azRIVFo0b0lNbUhzbjBDWFJpemk0eFIxcDN0NF81bXgxS2U0dDZUb1ExdThSVXhJd1hyQmZvVGtYNHpNVTNfTXR3WEprc1N6cUk0WGZkeXVpVVRsR0FwS0RyLUtXV2w3TWVCU1hidGJFRXN2X0hNcG1LSUl5SmNodUNib2M1NHRyWC1kTzNBNGxhR0hDcUNXcmlaM0t6ZlNhVXphcFFOajY4RDlpSjlBN3VHOURfYUhVYnJUNzdNbFRsT2ptZXdQeWdCX08zeDFDWkR6LUtZWVljSlRzaS1HSnlZdjFlbDBhdll6Zw?oc=5</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2660,52 +2660,52 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K41" s="1" t="n">
-        <v>46075.89700231481</v>
+        <v>46076.99258101852</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Pair sentenced for drug dealing and having an unlicenced air rifle - Oxford Mail</t>
+          <t>220 oproepen in één weekend voor Politiezone - De Internetgazet</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Pair sentenced for drug dealing and having an unlicenced air rifle - Oxford Mail</t>
+          <t>220 calls in one weekend for Police Zone - De Internetgazet</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 05:00:00 GMT</t>
+          <t>Mon, 23 Feb 2026 09:41:10 GMT</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxNTHVNSDlCQ0ZlMUZwZTBKM2llc0hOR1lnRUc5blhOOWd2amxLYm01WlpReFF1cmpfU19CN3l3NGdmZ1VDRjJfSmhVazZISVB3ZDhWbk1aVHNEbGl6Y0tTUGVhQkwwR3BBcHQzWFJsdHgyay1QQ1JqUnFoSm1EM2JaM0ZiblRWUG5BRmtQclByN3ktNlFpaWdJ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxNYTBpdElMU1JKTjk3LXFvdXg0aG1LWVd4S1RZaEtXS3FfdzdCU0ZSQnE2NWJjX3JwU3VVNnlPRU9SN1VqTUtqYm9ON0FGVUY4STdEaFdWUno1WGxfTzRNc21wX3JkdUZ4c2p5LWZBVjhWcnRpXzVLekJaLXhyQnItY0NhcVo?oc=5</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2715,52 +2715,52 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K42" s="1" t="n">
-        <v>46076.20833333334</v>
+        <v>46076.40358796297</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Road in Kildare ‘is like a patchwork quilt’, local rep claims - Kildare Now</t>
+          <t>Beveren a fêté sa montée sur la pelouse de Patro : la réaction de Stijn Stijnen a surpris tout le monde - Walfoot.be</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Road in Kildare ‘is like a patchwork quilt’, local rep claims - Kildare Now</t>
+          <t>Beveren celebrated his rise on the Patro pitch: Stijn Stijnen's reaction surprised everyone - Walfoot.be</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 13:05:00 GMT</t>
+          <t>Mon, 23 Feb 2026 12:00:00 GMT</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQc0NBaUFXZlFwVlEtZnBFS3RlZF9walhsUHFLY1U1Vjl5ZTFsTGFSUGQzcHhGeHVyMDFWWEloUVMtSld3X1Z2VTIxS20xUGV0elE0c042TjMtSUxiUU9HcDdoSHozN1JrZ0ZtNzhXaVVJelplOWdmOWZXNFl4UFBKQVRDNVVvU1hQQTV1MXdYZ1Jzc0V1MjR5R1NrYlctbE10YlJSXzYzZWtVbDRjZlF3TkxoeGg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOMFZUdHIwV2NXVUVCZ2JjRVJ0d2Q2Q2ZOWUw1OFB5ZV9GNkt6eVNSS1h6RjhDbGtrNFg3eUhOU2NROWlxMkZ2ZVVxbTBaQ1dPTXZLYmMwcFVRaHNLOEdPVmZFYkptVWJxWDZiTGRlZjVPaHJTWGJ2UnhLaklhcW1TenlRd0FTUGZRZEtCdUoxUkFHNHpZamVYMGFSNFVyaDI2RUItaE5KeVN1dEZfQTRJNkdZUXp1TS1lRFNDUXVDZjhVZmRiTWsyVnlreUoyekVSUG5wWHVheVbSAd4BQVVfeXFMT2R1OWxYLVlQVHkxTkJOOFVTdVV4ZHA2Q2RiQXRpblVQdGV2Nlh2Q2xBMnBqSWxCaW43Y2ZKcTdIbWRDdEY2ZHVlN2NhRFNsaThCX0hpMDhsaXQ2U2lIZ1lWUGNvRTNndkJvWUUteXg1WWFIdnRXbGFhVC02aVc1RmtLdHU2dVd3RDliSHpndEg0ZzJyQXhacEl3LU05Mk5WWjZZUUdKRDVuS3IzN3NzdFQwX3VnbmctMV9QQWxtOElPT2Y1bFJXSFdKVTdvb3BibXFXQ25lLThqVW1CX0p3?oc=5</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2770,52 +2770,52 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K43" s="1" t="n">
-        <v>46076.54513888889</v>
+        <v>46076.5</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Claim that independent bookshop in Kildare is suffering because of parking dilemma - Kildare Now</t>
+          <t>SA Winger Fires Beveren To Promotion In Belgium - iDiski Times</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Claim that independent bookshop in Kildare is suffering because of parking dilemma - Kildare Now</t>
+          <t>SA Winger Fires Beveren To Promotion In Belgium - iDiski Times</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 11:05:00 GMT</t>
+          <t>Mon, 23 Feb 2026 10:35:28 GMT</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxPTmVXT0ZBZG5sWE8xMk5IeFpPeFhHNUY5OHljdC1NX0ZUNV9fVGpIS094SS1QbGh3SEREc0hNcEh4MFZxYVE1UWxoaFBVWENPTk1XbHo3Yk1wWkpEdUNMLUFDalpZZzkxa1QzbWhiZVg4Zl9sNkhOTk5ZbUhPYl9zZ1A3RWVqY1ZyUmZPeE0wQnB3MnJSTC1XZ25GQTYxaDY1bGxzTzVfdlg1Y1R1OGVwSVBFdDBtc0p3cDFfdXlUdnFaY0x2cHBhRFVtZXltcmwwSHBRUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPS3ktRHpRekdhell6bG9ZVUdNeXhoQ2loT2RYMHl6eWNPNVFqd1p5Yk1wbGtPZGpzeGtkN0J3MGwtWVZhUm92NUFHSTk1bzR5WTlOTDgtbkZKWkpNbmgyUzFPS2ZJQXF4UnhRaGlwRW9jZldLNWdvU0FuOVdLVXMwMkJRaHlaVGdhUGZUY0YzX2V2Qkdrb0s5bHFB?oc=5</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2839,38 +2839,38 @@
         </is>
       </c>
       <c r="K44" s="1" t="n">
-        <v>46076.46180555555</v>
+        <v>46076.4412962963</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>LATEST: Attractive apartments planned for this town in Kildare - Kildare Now</t>
+          <t>Würzburg: Nach Angriff am Hauptbahnhof – Polizei sucht Zeugen - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>LATEST: Attractive apartments planned for this town in Kildare - Kildare Now</t>
+          <t>Würzburg: After the attack at the main train station – police are looking for witnesses - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 10:30:00 GMT</t>
+          <t>Mon, 23 Feb 2026 14:30:00 GMT</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNQUc3VkZBTTBTMjdpdm8yWEhlWjl6Q1JDUzA3XzFNQW5BQTE2WVlPb2pRVkdRNEZNTXpBSU0wSmVsMklXTXlOX0Z0STVtYUVPOVkzb01TUlJRY3k4cTd6VloybzhzUXA5V3ZKaUhWOFhCV1FkcW1vUW1BNFo4bUxkbTZQSHRrS0VybFRKSXFEaDMtVXZwbnAyRE12WU1rTnVtNUt4U1ZzOG9OZVhjTUNmLWhXaEhvUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxNUk1fcXRlQzR0TUx0eFZ4Rk1TMTBnQ2Z5RjJjeU02bGVXczhsQ0lfblVYOGJWRXRueExfZThlbTM2Smo3T25UQWs1TTNrZVRySUl6cl92NjJ1cktxVzltTTZmZGtJWXJVSWNWSmlDZVpYZFZiS1Q1WVgzRXFZbVBOT3lOUHlIbS1rMTBjQzNFNFhQdXFwLUNTZA?oc=5</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2880,52 +2880,52 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K45" s="1" t="n">
-        <v>46076.4375</v>
+        <v>46076.60416666666</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Kildare woman locked herself and children into bedroom after partner broke into her home, court told - Kildare Now</t>
+          <t>Reichenberg: Frontalzusammenstoß auf der B19 bei Würzburg: Zwei Autofahrerinnen schwer verletzt - Main-Post</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Kildare woman locked herself and children into bedroom after partner broke into her home, court told - Kildare Now</t>
+          <t>Reichenberg: Head-on collision on the B19 near Würzburg: Two drivers seriously injured - Main-Post</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 13:47:00 GMT</t>
+          <t>Mon, 23 Feb 2026 20:00:00 GMT</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxONjl3Z1A5Ti1kcno5SkFmWlVJX3doZUVPMWQ3ZndrUHdfaDhUUENHTGdYQjJHRmExTjFVQlpnV29NV0puc0wyNXRzWklXMXI0OHZTdG1qbWdRSzhyZXROT3dGajNHeFltblJyS2Q0Z2JKMV9EdjI1dmVUWFJCZXNZSFpmMXFoZmFBcGppOV8yRE1QdnRiRkF2V2NUVkdVdHhpcUFDMlVSSGxXTXpLbmVIb2RYVjU5OTB2WXFRb2VHalR6cUlsd0tWU2NlWEkyYXZ5WThWMGNxTUFiM3gtLS1WTXBTRGRWMFo0dTJZ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxON0VPNERZb21RaF8xWTQtUzVObjNuUUw5LXpNbEVyOGtLQ3I2eWc2STlOUEd2OTU3UUVMNlVhNlRvTGFSQmxvb181ZkxJNzFtQXI5NGoxZHJPZ0gtbUVBd0l6Wm96UjREZ3JnV3dfNjYyQklGWVlSUTVLRjZrRE5mU3E5dVFaNU5WdE0yblAxWHIzR1hJdU1JVFEyZnEyMFVneGhHTl9UVF8zYnZPTVM2bTQtT3l1RUg4WFc2WHhVekMxVTZCRmo4eXA5THhKRzRibTE1UkpFaGJqYW1qaXhZZ3VJcFpVYUVrNGh6Qkc2NDQyS19FMFItR2E4V3k?oc=5</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2935,52 +2935,52 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K46" s="1" t="n">
-        <v>46076.57430555556</v>
+        <v>46076.83333333334</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Dowling 'immensely proud' of his Kildare side after close-run battle with Clare - Kildare Now</t>
+          <t>Schüsse in Kahl: Polizei nimmt 19-Jährigen fest | Foto: Oliver Killig (dpa-Zentralbild) - main-echo.de</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Dowling 'immensely proud' of his Kildare side after close-run battle with Clare - Kildare Now</t>
+          <t>Shots in Kahl: Police arrest 19-year-old | Photo: Oliver Killig (dpa-Zentralbild) - main-echo.de</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 12:00:00 GMT</t>
+          <t>Mon, 23 Feb 2026 11:01:41 GMT</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxPcE1iMWVSLWRYTzZrdW12eDNBRFJDVHktTXE2aDFrSDR3S1BLNm9xc2VaUGdGWE9FX25kVDhwckZSdkJWWHhFNHJHT0VETUROaHlhZ1RHUjlZaTNRZHF5V1c2NHdNU1NGN3VlMjhUTk5hZjU2YUJiUnctZVFrYnNUTUEzSkNPT25mQVRIU0w4ZXM4VmhtaGtXeThwOXN5OHZPNnJJTzJLcmZ4RUtCakN6X2tNbktTUGlOMkRJRUZYNjZIVk5L?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxOTjJHN2xRN1Y3emR3c2pkRG9uMjJIYjhKZnY2d19ObFJuS1dHRVJ1UFc5aHdRWFpVUS1oYUpjdE5mWUhZRmF4cG5iVzN3R2pzWGxRekJiS0J4WWZCcnF1YXpzX0l1LVdRTjIzcTZQSzExS25kRXA3S2kzN2ZobkxRTkU2ZTlHQjlrcW5FRVZHSFRfYXFIRERVQWJLVkNybXlSQUJXVnFPUQ?oc=5</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2990,52 +2990,52 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K47" s="1" t="n">
-        <v>46076.5</v>
+        <v>46076.45950231481</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Local Town Fidenza Italian</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>("Fidenza" OR "Parma" OR "Piacenza" OR "Cremona") AND (protesta OR "minaccia bomba" OR esplosione OR sparatoria OR accoltellamento OR evacuazione OR "operazione di polizia" OR arresto) AND -calcio AND -Serie AND -mercato</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Leao, polemica dopo Milan - Parma: la protesta social per gol di Troilo - Virgilio</t>
+          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Leao, controversy after Milan - Parma: the social protest over goals from Troilo - Virgilio</t>
+          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 13:23:00 GMT</t>
+          <t>Tue, 24 Feb 2026 05:25:22 GMT</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxOV05fZEVJUUNKa3plVU9UWkVSS3BYRFBlNjZxUVo1OUJjTDdiSkFpOXBFZ0IxWDFYN3dseWt4dFVlVFZVbVp5UVFaVnM4azlpZVF5QXZZMXpmWGV2eUFsNU5pdGtIWHhzcC1UbldUTjZUR0pGaGJDeC1vajZseVBMbmlQLTdWbmp2dDlGMlRKUDlESW1jMm5zSDhUUVN6WDd0YzZtOXNNYjk4RFpYOU1SMC1QWU9ZS2hHcFVjeXZGaXAtYUwycGNrdldkUGRHV2fSAdQBQVVfeXFMT2dYVXJ1TG4yRVIwWmZ3ZnhVNTlDemh6b196NlB1eFVYSFRpa3czVTZ1TVdibW9LVURjZ2FEb1Ftc25hc0g5YkI1ZU4waGJFYU1HbG9tV3pmcEtERG1ZNzBJMkJtcGxza3k4V0g3U3ZkNU9OeTk1RHp3VnU2Ry1TMGtWTEpDeEVuVVdYS2ROZ2x5djlhSndhTDJvb3B5U19wYldQUkQxTm00ZEMtWjJscEgzUU5fTTlRYjBsbHV1N2poNWViVERTWFdIbkwxTTRBREhyNGg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE03RUZJdVVWTG5jTlA1R0dmc2YyQ3Z2S1ExYmhkN0FENFJGamUwenJsSFFPWGpKc3B2aFBaeHRYVDR3aWM1SXg0YWZFVDk0N3d4a0Jz?oc=5</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3045,52 +3045,52 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>it</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>IT:it</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K48" s="1" t="n">
-        <v>46076.55763888889</v>
+        <v>46077.22594907408</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Village Fidenza (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>("Fidenza Village" OR "Fidenza") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Fulgor Fidenza - Nuova Pallacanestro Vigevano: 89 - 94 tabellino campionato di Basket: Serie B Nazionale Girone A - basketmarche.it</t>
+          <t>Demo-Termine heute, 24.02.2026: Hier gibt's am Dienstag Demos gegen AfD, Menschenhass und Rechtsruck - News.de</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Fulgor Fidenza - Nuova Pallacanestro Vigevano: 89 - 94 Basketball championship scoreboard: National Serie B Group A - basketmarche.it</t>
+          <t>Demo dates today, February 24th, 2026: Here on Tuesday there will be demos against AfD, misanthropy and the shift to the right - News.de</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 03:57:00 GMT</t>
+          <t>Tue, 24 Feb 2026 06:04:43 GMT</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxPVklxcUQyVFRfaXl4bmRWYWFubU9hZkNfRzFyYTVaamx1aDRrN1IyOER1cDZrcWV3QVdnVFlaQjQybnZ3SHRLVTBZdXFpeHJudkJsOC1ONWs2ZEZaNXNCd2N6WkQwa0J4SS1RMjdNS3AtZ0t6c3NKU0UyYkZieUtEeUYyd0RJZHpBOVJpV09ybkRpZXJ0dEJERHF0b1FMcVBVYndvQXZSanl3ejQ3ckhJSlZjYUxMNzkyVnJaR3NKeXhqSi1nVzZZdHZTeGJfeHVfUWdIWElMV1Bwdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwJBVV95cUxPTGdUUkg2a1JYTDFRNDFrZTJfejZYeTZZc1dOeC1sYkNIOVQ4eXFXU2t2X1BXaTJsaHlsSmJXcUM1MWlpVmdXZXpBZ3ZiOUpPd2NhOG1OSUNfZWRhR1o0dEVWX2hZT0pCVk1WMmV6T1BmaFI3V0lEYjdrTUlPMUZvM1hMdHd1UWdnak13VFlMa1FydXF0cUZWd2ZTRjJWaTBCNmMyelAtdlI1Z3kyNndzZ0NSRjNkeTYwZWludW9WNVVPWThLbWw2ZXRpU2ZMdUxXcTZZOUllbG42OGp1dDBpbXlWeGE2X0xOakFnYnpxbXoyWE1HVks5bDZoVUs2QTMzbXpTWVh4a9IBjAJBVV95cUxNVlA5c1FOUjBhdmxMUWhDQk8xbDhPTFlENjAtM0hCS2pmX0M1VUZxcC1WblZQTWdhRjlhT2NWbUZWSG5NZWpLby1sYlJMTnA0X2JFeWNNcVFvNHpqQlJBcmY2VHc1QTYtc2xnTEVFRlFGTXRnZDFRNktpTFFVTG1vRmhtSGtvdTRDX0ktZm9QanY3SzBLTFo3enRWc3hSODJIejdMcGFqdGVpU3owaF92NmdKNkd4ek9OMFlfcE5pNldoNExVOGU5VjIxUDB3alBORWFRM0pRWXJVT0JlSkR3TmJOaTZhOWxQUncybTNxZGFpN2NGRWdCU0N5dE81blBrSUxjbld6cHBRc25X?oc=5</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -3100,21 +3100,681 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K49" s="1" t="n">
+        <v>46077.25327546296</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Village Wertheim (fallback)</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Jon Wertheim suggests the reason why Serena Williams may return to the WTA Tour - Tennishead</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Jon Wertheim suggests the reason why Serena Williams may return to the WTA Tour - Tennishead</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Mon, 23 Feb 2026 22:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNdXRXQ1JpcjVLX3Vkd3RzbW5VMWR1SW1qQ1hwc0RfUi0xZG5nQktYRXhYcEstZ3BSb1pMVU8yeklCS3dycGdhMW14WVZKVUdyOUtjN2YwMllOQ3JxOGo0VVhCX1VCM3AyLUFQVHMwZzZDbXNKb0prSkJITVlJbm1ka0ZDY2g5X3hJQ2llel9EM01mdjRaYklTazA5dHA0WGU0LUdmeHVn?oc=5</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
           <t>en-GB</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
+      <c r="I50" t="inlineStr">
         <is>
           <t>GB</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr">
+      <c r="J50" t="inlineStr">
         <is>
           <t>GB:en</t>
         </is>
       </c>
-      <c r="K49" s="1" t="n">
-        <v>46076.16458333333</v>
+      <c r="K50" s="1" t="n">
+        <v>46076.91666666666</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Betrunkener Autofahrer wird in Ingolstadt auf Heimweg von Polizei erwischt - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Drunk driver is caught by police in Ingolstadt on the way home - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Mon, 23 Feb 2026 11:49:59 GMT</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPWjhucDdvek5HMVVQUWR4LVhhbnFzUmNVeGVrbzQ1b2p6TDdST0ZNcENYejA3RGdNZ3h1aGlESzhnRHVuTHRzMmJIMGRVNjdhdlZ4TkdaVjVjWGExUjFOWS03YVdHT2NqSmRkbXM0RUh5dVlpUzNPOVM5LXFDVnBmMG5Gb2lVQmluM0d3V0ZibWtMSmNKX2Q1LUZjYXNVYWlQSUl5QkFNRXROOS00VngwbUNFWVdkdw?oc=5</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K51" s="1" t="n">
+        <v>46076.49304398148</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Polizei stoppt 66-jährige Autofahrerin mit 1,6 Promille - RegionalReporter</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Police stop 66-year-old driver with 1.6 per mille - RegionalReporter</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 03:38:40 GMT</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNZ01KNnczSFRPLTlLZUNzb1pXWTBqbGR0LWxFTXR0ZHZWb1pza0ctYmFSd3VmRUhLcjdsVXZDS1d5NUsteUN3b01FSW9lZ213MndZMWxnUDlFTkVYcnJZQjg2Mkg2WmdOSGpSUmZNeERVd3pHUlhwMjJva0JQWlNfS1lFREcyVmZfbzMzMkprZ3dlRWVWbzRKd3ZQLWhVS0FrMFVDUnRMMXRNdDN6NDhRbFhndzE3Zw?oc=5</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K52" s="1" t="n">
+        <v>46077.15185185185</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Unter Vorwand ins Haus gelassen: Täter stiehlt Geldbörse einer Seniorin - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Let into the house under pretext: perpetrator steals wallet from senior citizen - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 06:42:59 GMT</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxOUzZOZmpZeWJ4MGZ6Z003ZG5oYVIwZDhtN2k1VU9BM2FSLTgxWXlxcDc3eXBBOUxVY2h4SzVXU29tRXpxZzBZZW9mNFhGbXg1TWVRWUIyQzgzaGZac2N5c28wZ0pyV2hUWEhfblk2cUpGMFZmNDV2QTk3a0JZNXZfTFRqTUppSU1rSVRQa2NvSTlTX3ZEdE56U29HWTdSUmM1QXAyS2JGNkZzZ0llNm8xY1hLNWN5MXVsRHhLV1J5bGhmN3pRczRQZ3BLZXBSbVFETkZ3UkUzRURrNk0?oc=5</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K53" s="1" t="n">
+        <v>46077.27984953704</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Alin Coen live in Regensburg: „Du bedeutest mir die Welt“ – Ein Konzert voller Emotionen - RegionalReporter</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Alin Coen live in Regensburg: “You mean the world to me” – A concert full of emotions - RegionalReporter</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 03:47:07 GMT</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxNaGZyR041TjVBbXZOa0NudVppUlh4Zm1Gc1BFNmwzRmFaZjNvMExzaHBoMmh4Y1plTUk5QW1VM0lWTHNSMmN0NmJsZmlkbHpZa0dxdGhzMzNvYnhlOU1BRnlOeHdUclJKLWNjaUhHMWNFWFFxMDBjYlJWcUtidGJKQVNLOFNia1laaWVXbjR1N3JkUlQyS2dLTGZ5Uk56SThmQXFRMzYwaTVYam9wdnUxZndURUxSSEx2cDl3S1RDVGhub1dob2pxeWx0TTltXzN2bWpFVWR3?oc=5</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K54" s="1" t="n">
+        <v>46077.15771990741</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Beifahrerin lebensgefährlich verletzt: Stundenlanger Stau auf A9 nach Unfall mit Lastwagen - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Passenger critically injured: hours-long traffic jam on the A9 after an accident with a truck - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 05:08:22 GMT</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQRXl1MWhlRzRsY0RRYVZPdTBPWG9FLW9TdGl2QmdMenY2b3EyeFNGZGdZMVNoajRVc3FWeTBUeEZqanVrOEpmUTF1SDdtblFVYXRhOG5RYTcteGZqRnBLUVJ4ZTgxU2hIZ2x4dGxfaFRYN3ZIYVplS3A4VjBHVnBrU1AyRGhtNV95VDVkREo1LTJYSThBUHRJTS0weENUekpNaU9ySUlUY1g2YnJVa2E3RnZhRnV6OHQ2VnNJT2VpZ2M2SklKdmZN?oc=5</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K55" s="1" t="n">
+        <v>46077.21414351852</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>SPD Frauen Ingolstadt fordern gerechte Gesundheitsversorgung für Frauen - RegionalReporter</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>SPD women in Ingolstadt demand fair health care for women - RegionalReporter</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 04:53:13 GMT</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxQWTVvZndQRWxzYWswTXQtRHNrV01FQUwwRlRsQXlqS1h4V3NPZVNsRlMyelVnd2FPV3dJSHY0UGk4cExDb0FIYkV0aGhRX184WUxRLTdpRFB5dXR2WUQxYm00RlNiU09lN050cFptMU5MRDRXSXg1cXNqZnNpUGNsOVUyazhqQTJZQmEzckI3Qy1KbWVKSzYwa2tSWVhjM0hLR0pFSktqOS1kazFDSXNXd2lWaF9BaEtBZ0Y5ZUdnVXhXUE0?oc=5</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K56" s="1" t="n">
+        <v>46077.20362268519</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Solidarischer Hochwasserschutz: Regionale Allianz setzt auf dezentrale Maßnahmen und Echtzeit-Frühwarnsystem - RegionalReporter</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Solidarity flood protection: Regional alliance relies on decentralized measures and real-time early warning system - RegionalReporter</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 05:04:48 GMT</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxQbGI4VVlKYUJfeGhaTGpqVXg3ZDZqTzBnUXBqUngwQ1l2dkxFakRZN2QwTm9HTDVORC03bnpaNGVaV2FBWlNXS2VBY0dqNlRmdXpiNGVKdGR6aGxUSkJwelhkMUdTU0lUVktmSTNmcVI0NHBBbGpXZUowZnpRT2hKWHJlSFhKa1VJYVMxTkZ2VjRBVTR0dUFKVnlqNF9rdllKYndwRW5hdUNGUVZfVDhMb3BUNFJqcFQxZVhueXJVT2dZUm1iU1Z6VUNoV3MwUkhsd3BZVi1oZEdpZXlHR1NvYVppckZrLU5IZEp4SEdHWjVvcEFMODg0?oc=5</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K57" s="1" t="n">
+        <v>46077.21166666667</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Village Ingolstadt (fallback)</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Important note: Municipal construction work restricts access to the parking lot - EHC Red Bull München</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Important note: Municipal construction work restricts access to the parking lot - EHC Red Bull München</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Mon, 23 Feb 2026 16:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNdUdtZFdTODlzV1RXU2NEWGRNeGwtWjRtODUtYWI3bkZfRXVNVjhNWTBhWnNYcGVmZUtYdHJsOWYtX0NRV0xteEwxTFlJU3J4VVUxREFmaDB3dTVTaTRjdG5YM2t6VE5yZUFKRV90MnN4WURuRERQeW9CYzZaZlZhS0lOS2lHTUZvZml2RzVIc0dmdFVHemlTVjJLcV9pTjk5RkxUYnF4UFNoNlptU2c?oc=5</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K58" s="1" t="n">
+        <v>46076.66666666666</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Village Ingolstadt (fallback)</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Lamborghini Technology Boss To Head Audi R&amp;D - AutoSpies.com</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Lamborghini Technology Boss To Head Audi R&amp;D - AutoSpies.com</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Mon, 23 Feb 2026 13:01:28 GMT</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1YYnl0N0FVLXZlckdFZVVPUE1VaGZqSmp3VTg0Y1BzWjlqN3pVams4QVYxZV9IQTVYZTEyWUFzSjE3UjRJQ3RIMjBXUEFnQ2JFVllwa0c0WUVXMXI2MUh1NnF3VG96U2xpTFpDbg?oc=5</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K59" s="1" t="n">
+        <v>46076.54268518519</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND ("minaccia bomba" OR "pacco sospetto" OR "pacco esplosivo" OR sparatoria OR accoltellamento OR "attentato" OR "operazione di polizia" OR esplosione OR evacuazione) AND -Olimpiadi AND -pattinaggio AND -sci AND -Cortina AND -calcio AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Sparatoria al campo nomadi di Zola Predosa (Bologna): giovane ferito alle gambe - Il Resto del Carlino</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Shooting at the Zola Predosa gypsy camp (Bologna): young man wounded in the legs - Il Resto del Carlino</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Mon, 23 Feb 2026 22:54:30 GMT</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxQNENFR2txSTcwcFdrc01hbnRrSVZ1N19nNHZ2N3A3WUxsSzNHTkVBNnJUY3loUTN6QjBmc1Z3QjVyN2tqZS15UGpHdi1NbnFtTFh3TFFlTm9ITjNzMnVibXhDX1lKdUlMcFAyMl9jWk5MOXRISFQzVWdYZFhHdXA4QktBcWRfTk84MnpyNGt0WQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K60" s="1" t="n">
+        <v>46076.95451388889</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Local Town Fidenza Italian</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>("Fidenza" OR "Parma" OR "Piacenza" OR "Cremona") AND (protesta OR "minaccia bomba" OR esplosione OR sparatoria OR accoltellamento OR evacuazione OR "operazione di polizia" OR arresto) AND -calcio AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Leao, polemica dopo Milan - Parma: la protesta social per gol di Troilo - Virgilio</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Leao, controversy after Milan - Parma: the social protest over goals from Troilo - Virgilio</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Mon, 23 Feb 2026 13:23:00 GMT</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxOV05fZEVJUUNKa3plVU9UWkVSS3BYRFBlNjZxUVo1OUJjTDdiSkFpOXBFZ0IxWDFYN3dseWt4dFVlVFZVbVp5UVFaVnM4azlpZVF5QXZZMXpmWGV2eUFsNU5pdGtIWHhzcC1UbldUTjZUR0pGaGJDeC1vajZseVBMbmlQLTdWbmp2dDlGMlRKUDlESW1jMm5zSDhUUVN6WDd0YzZtOXNNYjk4RFpYOU1SMC1QWU9ZS2hHcFVjeXZGaXAtYUwycGNrdldkUGRHV2fSAdQBQVVfeXFMT2dYVXJ1TG4yRVIwWmZ3ZnhVNTlDemh6b196NlB1eFVYSFRpa3czVTZ1TVdibW9LVURjZ2FEb1Ftc25hc0g5YkI1ZU4waGJFYU1HbG9tV3pmcEtERG1ZNzBJMkJtcGxza3k4V0g3U3ZkNU9OeTk1RHp3VnU2Ry1TMGtWTEpDeEVuVVdYS2ROZ2x5djlhSndhTDJvb3B5U19wYldQUkQxTm00ZEMtWjJscEgzUU5fTTlRYjBsbHV1N2poNWViVERTWFdIbkwxTTRBREhyNGg?oc=5</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K61" s="1" t="n">
+        <v>46076.55763888889</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-02-24 14:50 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K53"/>
+  <dimension ref="A1:K73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -535,32 +535,32 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Shoplifting UK</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>("shoplifting" OR "retail theft" OR "retail crime" OR "shop theft" OR "pickpocket") AND ("UK" OR "England" OR "Britain") AND ("gang" OR "organised" OR "trend" OR "rise" OR "survey" OR "report")</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Retailers sound alarm as shoplifting reaches 5.5 million incidents across UK - EasternEye</t>
+          <t>REVIEW: 'It's longevity speaks for itself' Shan Shui at Bicester Village continues to prove its mettle - Ox In A Box</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Retailers sound alarm as shoplifting reaches 5.5 million incidents across UK - EasternEye</t>
+          <t>REVIEW: 'It's longevity speaks for itself' Shan Shui at Bicester Village continues to prove its mettle - Ox In A Box</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 10:27:32 GMT</t>
+          <t>Tue, 24 Feb 2026 06:00:00 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxQNHZxbGRlR01sS215TlJRRHpQcXAwRDZzdGRNTUc0SG43OFRLcmlhUHlQTHhKcEtmQm4xZWZ3Y3p4UzNPUUs4dk50cC1tNnlrYUxib0x0N0k2T3VVRW00ejNVWU9OREU0OGNxZXFka2FPaW9QUVVoMmE1Z0pnWk9uc1ZGek5Td0YzMEhJSklma0J1SUhuNFEzNWxYdE5fVGtrTWs4WExabw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxQNHhwYkgyd1ZmTnNNLVZCd3otNHlNa2VLRHhuYlN0VDZlQlk2Y1M2WFVLSUNJUDhVQW0yclppd01lNTU1N0JyUGhGb2ZfZ1hnWFJmUEhkZnZTd2Z3RW1ZbmFZeDBZMXlUTnVOWkFjbmdsdGx2TXEySDF3bF8yZVJTb3pvNVhVczVoTXdDbnBWSU14bTdyNW5GSW9zVEg5RU9FYlloWnltSkZtVURCT0JWNUdnQ0NlaUN3UEkyenZXNA?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -584,38 +584,38 @@
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46077.43578703704</v>
+        <v>46077.25</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>London Marylebone Incident (fallback)</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>("London Marylebone" OR "Marylebone station")</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Railway veteran of 64 years returns to Flying Scotsman footplate - Chiltern Railways News</t>
+          <t>'Disgusting' bins and rubbish at Oxfordshire Sainsbury's condemned - Oxford Mail</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Railway veteran of 64 years returns to Flying Scotsman footplate - Chiltern Railways News</t>
+          <t>'Disgusting' bins and rubbish at Oxfordshire Sainsbury's condemned - Oxford Mail</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 11:06:48 GMT</t>
+          <t>Tue, 24 Feb 2026 05:00:00 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxNcWdvdkd5cGZ3QmRMYjFQaExNdUx0S3dVcmdEelVjcUpwNUhKbENHMlJRRVFCeWxoZjJQMko2UXhOaVV5d0N1aDF1SVdDZXBOUDJoRmFsV1AtLXFZdkpjdUdWNXlxTWNBb1lnZmNnQVMwLUJVak9JVGNJRWo4SmdBT1dQWGcwLWk4NlRLcTd0OVlHbXppYTJTSkx3WGYya2xmb21WbUFHd211Zw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOdXNXbzM5M1gwd1ZmUm5VWHdqYVZ4T0swWVNoaDlxaEk3dFNzWUxmODBnQklwNF9JOERhckV0RGVmNTF3aF9xcVVEQ3M2TzRORDBNVXJtcDdpeHV6ekVaMEVsWTUtVUZ2N2Y3THFrUmJMaVFMT29nNFNic2V5MmUwZ2pYUkc1dkhaakE1WjdkVFpQU2p1NFdpLUd3?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -639,38 +639,38 @@
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46077.46305555556</v>
+        <v>46077.20833333334</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>London Marylebone Incident (fallback)</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("London Marylebone" OR "Marylebone station")</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Railway enthusiasts flock to Banbury to watch as 50-year-old train sets off on farewell journey - Banbury Guardian</t>
+          <t>Rising UK Engagement with Chinese Automakers and Asia-Pacific Industry - IDTechEx</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Railway enthusiasts flock to Banbury to watch as 50-year-old train sets off on farewell journey - Banbury Guardian</t>
+          <t>Rising UK Engagement with Chinese Automakers and Asia-Pacific Industry - IDTechEx</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 10:28:00 GMT</t>
+          <t>Tue, 24 Feb 2026 04:33:36 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxNaDlnYVhpRlVxSXcxQXpzRzhaZVBTZzdhRmxESzFScjBxanNhTHVkN3IyZTFZUXgxazRRU1RMV0pBUUpYZnkxZnFQYmU4VGkwdWJFdnE5ZzRHemtjWHFWMTY3dHpPOWdkaWR1UjZWcXZUWG5sYV9iemNMQXFkVWtkTmpUeGdyWlJTbHBOWXFtT3NDMFd5SE52eUQ2S0pKYXg3dG1OMlZXVEdzaldqcXQzX1p1MXJoLUpIU0J4b0JDQ1FvdXU1U3ljV0Qyc25QeE9PRGlYc1dDY0dlcXp1ZDRxVzg0dVBvLVk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPeDRlc29GOWdqOVQwYm5ZLS1BYUhHbXE4ZWFLOEp3ZEp2NU9kSHF2LVFyZmN5WW5Vb3lnWDdCRTUtZkY5REQ5ZVNNd29MRHZKdmVMRzFUcHZNTFhNN1VvZUVvcGQ3UHFibWRENE1mZG5EcTB1ODZlT2ZNYVA5dDJZeGhJUVgtUGZZeFo5T003V1ItUmR2b294YzVESUhzUVEzeG55TWVVY2JSaDhKeFBUSklzSURvZW5nNUNkcjFR?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -694,38 +694,38 @@
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46077.43611111111</v>
+        <v>46077.19</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Politie Brussel West vindt bijna drie kilogram cannabis en plantagemateriaal - HLN</t>
+          <t>Changes announced for Oxford Tube services to and from London - Oxford Mail</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Police Brussels West finds almost three kilograms of cannabis and plantation material - HLN</t>
+          <t>Changes announced for Oxford Tube services to and from London - Oxford Mail</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 13:58:28 GMT</t>
+          <t>Tue, 24 Feb 2026 07:29:15 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQVDNCRUxNSms1VFBKUXBxVTdkcGVlb2p3MGZiajBHcmFqN0oyR19uaDY5UnIwcXFQc3lQY3JncXR6blFKR0wyUVpSZ2d4UzRMeDh5UU50QllENEdBaEx3Nk1XbmNlZWE4d2Rnd2hMUVVoY3dqSjh2eWFTSnVzel9OTlV6dXBwZjVubXFWVWhhSTY3X2R1enUyM0J4bFRDYmNYTXF5U0k4aVMzRWlzaUl6UUVNNWI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxPaTRYa2NPSkxzZE1UWjRJSjU3eXZ3TkZka3VXdGd0YndMdHpscHJzSmJ6cWRRTGhNM2plYjFDX1hJeS00T1FMMGtnc3BsaEN1SmZ1dVYzSUFqc3pwTmtDSG12LWlRY3dkcXBxVTFUUjlubGs1dFhLMG9weGZYelhKcmZCYTQ5T1NoX292cHBWdGN4Zw?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -735,52 +735,52 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46077.58226851852</v>
+        <v>46077.31197916667</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Trio krijgt drie jaar cel voor schietpartij achter winkelcentrum, maar schutter gaat vrijuit - GVA</t>
+          <t>One of the UK’s biggest villages to become a new town – with cosy pubs and historic canal - The Sun</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Trio gets three years in prison for shooting behind shopping center, but shooter goes free - GVA</t>
+          <t>One of the UK’s biggest villages to become a new town – with cosy pubs and historic canal - The Sun</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 11:39:00 GMT</t>
+          <t>Mon, 23 Feb 2026 15:11:00 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8wFBVV95cUxOUXduU0hBQ2g5c0puak1mdjJQUzBfdEwxNk92RFdaemd6ZzZTTkI2dkdWWmlZV1RTTVV5cC1IdmZubHlNQTVuY0dmdlJDQ1hoRU9GSVBfNTFLQ0o4RmdoZHU0REptS3JBTVU2ek9JMmtTWFItbVpuSS0tM0o1MzVGSW9TNFFiRTFJY2VTalhyQkhsSmR1V0YtNkJCWDN2dFJIYms5cUlKUkZ4Rmh1Tm5zQVdJVVBoNUNpY2ZJOG5zNVI2YnJkRTlGdTAtbVRrekRqeWo3MEFrUkVCX04tZnZzQV80MUJKa2x4V2xxVkVweXN4ZGM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxQTFdPODFXLUpCeFczUnFia3EtVG9wRmExQUV3cUppMmFkWEQ3Z1RzZFBHZVMxRl8yNThsc1JTajdfQjdzWmg2T2VSeDlSd1NWVWFjMmlxLXBaZ2dqVEhiR2FrMFhSTWV1dUNtbDF6SWpSZmtBRC1TWnh5Ykt1MDVESW5mR0U?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -790,52 +790,52 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46077.48541666667</v>
+        <v>46076.63263888889</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Shoplifting UK</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("shoplifting" OR "retail theft" OR "retail crime" OR "shop theft" OR "pickpocket") AND ("UK" OR "England" OR "Britain") AND ("gang" OR "organised" OR "trend" OR "rise" OR "survey" OR "report")</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Voortvluchtige drugsbaas bestelt vanuit Turkije poging tot gijzeling in Berchem en moet 7 jaar naar cel - GVA</t>
+          <t>Organised Retail Crime Surges in UK Costing Billions Annually - streamlinefeed.co.ke</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Fugitive drug boss orders an attempted hostage-taking in Berchem from Turkey and has to go to prison for 7 years - GVA</t>
+          <t>Organised Retail Crime Surges in UK Costing Billions Annually - streamlinefeed.co.ke</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 11:28:25 GMT</t>
+          <t>Tue, 24 Feb 2026 06:52:41 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogJBVV95cUxNZV9xLWN3R3ZhZHYwUEY4LTktS3hKTXNDbFhTMnRLSHByY1NKWDlUNlVtS1pwSDFhdDFidEl6NEJDbHNLZkJZcTJ3bUkxYzNSNnNPbktjUG9HaXpUNGI1TzBKc1J2c3Fld0pqNWtVWnRiSnd5b1NEcFY1b21oLWUyaVQzNXRIZkJza0RQdW1ici1QM0hfam92a1lHWFNIcXgxQnNvcklLMWwyOXpzci1wUWVtdXdMbmdGeTg4YldQMUx6amszckRuZHlCVEpBV0F1dkU3SEpzaXNiQmZtMzYtVzZTZllOTERxTFpqZUR3ZFVoTGNSZlZSVHp6c1NUNk8yMDIxZk9FdXZOYlZ6eE1Bd3N4bm0ySXhYdzM2NjVVd1IxUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxQYXAwZGpoTUZsSlVHOUpRbDl3OUsycnA1RkEwNE9IdHE1S3FiZEhZbXdwcENSa3dSTEE4aDZIVTB6ZXJWZWx4LXN2N25WWUJrNzcySnlkV0dxWlhsQUI4aHUxalJ5LXhGSG1HeVZPMjRwWWE5Ykt1TUN1dFNZQVZDTXB0ZkVmbGFuNU5weEVZckJud0lRVkZZ?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -845,52 +845,52 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46077.47806712963</v>
+        <v>46077.28658564815</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Shoplifting UK</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("shoplifting" OR "retail theft" OR "retail crime" OR "shop theft" OR "pickpocket") AND ("UK" OR "England" OR "Britain") AND ("gang" OR "organised" OR "trend" OR "rise" OR "survey" OR "report")</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Gravin Diana du Monceau de Bergendal opnieuw voor rechter voor verwaarlozing van 270 dieren: “Al zes inbeslagnames in 15 jaar” - HLN</t>
+          <t>Retailers sound alarm as shoplifting reaches 5.5 million incidents across UK - EasternEye</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Countess Diana du Monceau de Bergendal again in court for neglect of 270 animals: “Already six seizures in 15 years” - HLN</t>
+          <t>Retailers sound alarm as shoplifting reaches 5.5 million incidents across UK - EasternEye</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 13:07:30 GMT</t>
+          <t>Tue, 24 Feb 2026 10:27:32 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxOVlFnbkZRT0RIRkNUQjYxNjFxWlkxX3RESk1NMHZremJEbmhYX3lNcEJYLTBnN0pkck5jeFdWQ2NkUVh0VFRCbWt3T2d6QkF5V1pBUFlkRmRrRGNmekJtYVBjMTl5a1hZZXBma0tRM25PWmwwQ3d3UDd0bEwybXNPZHVIeUV5R3pyNkdIc3d3V25VZVB4bE9TUmtxNU1heEVnUTZMYndkSUtnY2Y0cUg4N29FRF9RTEJzMklOVHlwbGRyTXpVOVVwLWh3bFl5UzlnRjIxc2I3bEk3MEJzb3NhNmhHXzRRUU14cWRBNVFHVjZGZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxQNHZxbGRlR01sS215TlJRRHpQcXAwRDZzdGRNTUc0SG43OFRLcmlhUHlQTHhKcEtmQm4xZWZ3Y3p4UzNPUUs4dk50cC1tNnlrYUxib0x0N0k2T3VVRW00ejNVWU9OREU0OGNxZXFka2FPaW9QUVVoMmE1Z0pnWk9uc1ZGek5Td0YzMEhJSklma0J1SUhuNFEzNWxYdE5fVGtrTWs4WExabw?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -900,52 +900,52 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46077.546875</v>
+        <v>46077.43578703704</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>London Marylebone Incident (fallback)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("London Marylebone" OR "Marylebone station")</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Antwerpen dooft verlichting aan 45 gebouwen en monumenten tijdens Earth Hour - HLN</t>
+          <t>Railway enthusiasts flock to Banbury to watch as 50-year-old train sets off on farewell journey - Banbury Guardian</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Antwerp turns off lights on 45 buildings and monuments during Earth Hour - HLN</t>
+          <t>Railway enthusiasts flock to Banbury to watch as 50-year-old train sets off on farewell journey - Banbury Guardian</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 12:00:13 GMT</t>
+          <t>Tue, 24 Feb 2026 10:28:00 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOVzR6UXJtbHMtY1FGS0t6eVZOdjNvcEFlX21xOU1WdGZGb0tPaHpndGtwdXJ4bE5nV2prVG1xM0ZQbUlsTHhkbzVZX0p0cThqWU5XQkRRZk9pbXJrZGI2VjRCelEtaXpYYUhuZnY5WUY0WXhQOGdfWDB3QWF1QWR4NVFNVjM2NVkzUjdkTlJkcVNxQ01XMERzWWU1ajkxWmVBSVFWYTlvSmN2VElyNU1uOF9jbWdUdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxNaDlnYVhpRlVxSXcxQXpzRzhaZVBTZzdhRmxESzFScjBxanNhTHVkN3IyZTFZUXgxazRRU1RMV0pBUUpYZnkxZnFQYmU4VGkwdWJFdnE5ZzRHemtjWHFWMTY3dHpPOWdkaWR1UjZWcXZUWG5sYV9iemNMQXFkVWtkTmpUeGdyWlJTbHBOWXFtT3NDMFd5SE52eUQ2S0pKYXg3dG1OMlZXVEdzaldqcXQzX1p1MXJoLUpIU0J4b0JDQ1FvdXU1U3ljV0Qyc25QeE9PRGlYc1dDY0dlcXp1ZDRxVzg0dVBvLVk?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -955,52 +955,52 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46077.50015046296</v>
+        <v>46077.43611111111</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>London Marylebone Incident (fallback)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("London Marylebone" OR "Marylebone station")</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Antwerpse takelpionier failliet: takeldienst Viaene legt na meer dan 50 jaar de boeken neer - HLN</t>
+          <t>Railway veteran of 64 years returns to Flying Scotsman footplate - Chiltern Railways News</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Antwerp towing pioneer bankrupt: towing service Viaene closes its books after more than 50 years - HLN</t>
+          <t>Railway veteran of 64 years returns to Flying Scotsman footplate - Chiltern Railways News</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 10:34:08 GMT</t>
+          <t>Tue, 24 Feb 2026 11:06:48 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxNanBoV2o1anpZNlhuVEdxS29TaUh6VXdodFVkZTExeW1uUkZsZElSendqbzhoczRLTVdvOWRKcE9Wa2lINkVfQjRtRjBYSVdvck5wM0RPeFpMaFdpcjR5LWYxUndSNDczZGg3Tk5zbzVYQUdyWThVQVg3dEF5UEE3aVdoRFZIWFhINlFlN3NWM2V5YzQxU1FZSXJ1OThxcDMyeldEWk91MlFwbWRGb3ptNE9VbUZTcExhZWcyeU9SY00yYTF5alNaeA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxNcWdvdkd5cGZ3QmRMYjFQaExNdUx0S3dVcmdEelVjcUpwNUhKbENHMlJRRVFCeWxoZjJQMko2UXhOaVV5d0N1aDF1SVdDZXBOUDJoRmFsV1AtLXFZdkpjdUdWNXlxTWNBb1lnZmNnQVMwLUJVak9JVGNJRWo4SmdBT1dQWGcwLWk4NlRLcTd0OVlHbXppYTJTSkx3WGYya2xmb21WbUFHd211Zw?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1010,52 +1010,52 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46077.44037037037</v>
+        <v>46077.46305555556</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>London Marylebone Incident (fallback)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("London Marylebone" OR "Marylebone station")</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Waarom laat je een vriend op straat achter om te sterven? Heerlenaar Johnny E. (43) moet na conflict binnen motorclub Kanun vijf jaar de cel in - De Limburger</t>
+          <t>Farewell tour for mark III trains raises £20,000 for charity - RailAdvent</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Why leave a friend on the street to die? Heerlen resident Johnny E. (43) has to go to prison for five years after a conflict within motorcycle club Kanun - De Limburger</t>
+          <t>Farewell tour for mark III trains raises £20,000 for charity - RailAdvent</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 14:01:37 GMT</t>
+          <t>Mon, 23 Feb 2026 15:56:00 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwJBVV95cUxPZUV2S0NpbC1iRTlwRlpBbXB0QnBqNnZkeE9SWUQxLVdWRHp4MXloQXBvMlhNTVhXaFZJVUZKN2o2NGh1b1VyOFFJYlBsb0I4ZjJieFl5MnBYcDhYQ2Q4ZUZUVUotOExudHBNYkZlT1doSmxDd3lLbjQ0Y2FlRVZoT1JJUmFfNnN6WXBFVnZLLVNSbE9tVUJ5WWRFMmlsSk9teVFsdkNUNDlVR244Q3RnUEpjWk1HbkhHaXNDWks4T0UzYTRxMmpRQlduTGNkTUZzWmZDTmJMNC1BSFlGV0FZVG1idS1aekR2OFFrblVkMTAwQWtZVVktclJXVjNzOVhBQ3EwVUI5ZW42OUZQNS1haGdTSTFFMlNXRHdDcWllRHdWck84dTIwYlBRbU1yY3c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNQlVtd1h0QVIyR2VBYkFsR2RoN1lUd0UzMWZPMDVydUtCdEVvUEpNRGdHWG1IaHBjRzUxdGJvQ19FRVQxXzhQbGRCd2tLMGViaUZ6WVN5UThidXBGVnBUT3FsS3A5dGJJS0R5S2ZFeVR0UGNjSnd4NGpfQVBhSHVES0ZhTlZvaVVITDFQNXpYazd5N3VUWkllNW5OeWJYRk1jZFBuN21n?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1065,21 +1065,21 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46077.58445601852</v>
+        <v>46076.66388888889</v>
       </c>
     </row>
     <row r="13">
@@ -1095,22 +1095,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Explosief gegooid naar woning in Eygelshoven: geen gewonden, wel flinke schrik en beschadigde auto - De Limburger</t>
+          <t>Drugsbaas bestelt vanuit Turkije aanslag op papa die zoontje afzet op school in Berchem: “Voor 50 miljoen euro aan drugs gestolen” - HLN</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Explosive thrown at home in Eygelshoven: no injuries, but quite a fright and damaged car - De Limburger</t>
+          <t>Drug boss orders attack from Turkey on father who drops son off at school in Berchem: “50 million euros worth of drugs stolen” - HLN</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 09:46:26 GMT</t>
+          <t>Tue, 24 Feb 2026 11:28:51 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5gFBVV95cUxOd0xSOHdvOXluc2R6b0hTV3pfMnBqUXVULVo4TFhTYkNOVzBSc1F6bjJFY0hVRjRVSEJ4cEo0UDlONU9yenRORzFOSWR1U2hzYVJVbGNTMXNsLUdSMUlKZjhNOEFQNG54cm0zVVc3YjhlelJGSFI3N1pESHJ2RmFqSVZvb2pNU29nZjNHNm9id3l4Y08wQmNWNDFnekcwbklORVd0V2VFc0xaMzBkcU5YZENvVkNoYmpxMGZzelM2aXhTQzJTZmlEcEpvclNsWWkzbXN5Y3VUQnNkY09aLXlVWFVxSUw3dw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-gFBVV95cUxNX1NManE1aGM0dUxmMXhDYUEyX19pdFRGcmZPWGtCN0U4QTFzSkVLQjRaODI2aWNqWkd1cVA0U3AyeloyRVo0aUgtQkpxaGtEY3JzMzBZUjdHMGhyUmxGT081NG1RSDdKdXJQa2tWSEpub1BSUk1IY0VRSUhrZTBySVJPTm9XSjBFSmlBTTdkbzBBRkpfc0FNdU1UX21jNER5eXJleHBJcFA5Z05JWkdMeXRpOVVGU2FzOWYycEtCak53MzdFeVdIakwyVnVKdXh4MmZiUFlDV3ViemJfc29ncWczOWhiV1lDVm03V1RLSDROYWFrLWFkcXFn?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1134,7 +1134,7 @@
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46077.40724537037</v>
+        <v>46077.47836805556</v>
       </c>
     </row>
     <row r="14">
@@ -1150,22 +1150,22 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Opnieuw incident aan Antwerpse gevangenis: politie grijpt in na mislukte poging om pakketjes over muur te gooien - HLN</t>
+          <t>Vals bomalarm aan Grote Synagoge in Brussel: “Volgens eerste elementen weer zogenaamde grap” - Nieuwsblad</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Another incident at Antwerp prison: police intervene after failed attempt to throw packages over a wall - HLN</t>
+          <t>False bomb alarm at Great Synagogue in Brussels: “According to first elements, another so-called joke” - Nieuwsblad</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 12:38:35 GMT</t>
+          <t>Tue, 24 Feb 2026 03:20:00 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxPbGtHUkJLT01KeFFCU1ZHR3dTRUpOdlhVSVl3b2hKRXViSUNGZmJPRTJiMjZzemx1MjNzRGtRZzFDUElVMllrSDZoUWNnekNJU2hITWtDVlBobTRzSTB1c20wNnZoTklISm1qTEQ2N0YycmFvakZzY0xyT0NIRGxHaW5WWHpVWE5xYXFpYjRDalZPb01rMHFERWszOUx5U1Q4U1J2Uk9VU2NyY2ZvYVlJNjBVR2RyLWx5dURtU0x6clJfNXlFa2ctejRqS0NELTI5cVZfQ2pUN05PblVLRHltUG5WQWM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxPLVNGa1QzTEV5X253bFc0c0pCX0NmNVphY2tGVHJkN3BjS2tyd3BHSmo4cGtsY09FaTR5NjhKNU9Dd01rQjY1c0wwZUFQWVdlTlBSTjFMcDZaenRISzJqTUlTNTJmOFAzbVF0Ti14Vjl5aXZlNkhmSWM5NkNKcjlwNUxTWHJOUnBuQU01Q2tIUmVjdkhTd1V3S1F5dWNwd3NxQ0d2WTFwNlI3aVV5MjR6X3gxQVRRRmVmekllYTdoUUYxeG10cTRqb2hyZkI1eEtOMGRlLTllTmVUY2JPRFlXQUhYdEdIWnc?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1189,7 +1189,7 @@
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46077.52679398148</v>
+        <v>46077.13888888889</v>
       </c>
     </row>
     <row r="15">
@@ -1205,22 +1205,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Beurtelings verkeer op de Kapelsesteenweg door bekabelingswerken - HLN</t>
+          <t>Trio krijgt drie jaar cel voor schietpartij achter winkelcentrum, maar schutter gaat vrijuit - GVA</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Alternating traffic on the Kapelsesteenweg due to cabling works - HLN</t>
+          <t>Trio gets three years in prison for shooting behind shopping center, but shooter goes free - GVA</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 12:05:04 GMT</t>
+          <t>Tue, 24 Feb 2026 11:39:00 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxPVVVoM3lVUzdhOWJUT2lGSi1HbDRHQmExeG1falVTUEt1WEdBRFgwRlJJWUJIV0xmd0M2UmlkdTN5X3RDa2Y4b1FjU2RzSGdFMmdXMHNsSGZhUXBIeHR0Mkh4MDhVdTREbTFsYXV6UUtxRzRIM2ZCM09MQkg0RXo5c1Y0YXcxZ3lSSmhyM3dpemoyMU13UlJNSVR0LTI1ek5sWGN6cWxn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8wFBVV95cUxOUXduU0hBQ2g5c0puak1mdjJQUzBfdEwxNk92RFdaemd6ZzZTTkI2dkdWWmlZV1RTTVV5cC1IdmZubHlNQTVuY0dmdlJDQ1hoRU9GSVBfNTFLQ0o4RmdoZHU0REptS3JBTVU2ek9JMmtTWFItbVpuSS0tM0o1MzVGSW9TNFFiRTFJY2VTalhyQkhsSmR1V0YtNkJCWDN2dFJIYms5cUlKUkZ4Rmh1Tm5zQVdJVVBoNUNpY2ZJOG5zNVI2YnJkRTlGdTAtbVRrekRqeWo3MEFrUkVCX04tZnZzQV80MUJKa2x4V2xxVkVweXN4ZGM?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46077.50351851852</v>
+        <v>46077.48541666667</v>
       </c>
     </row>
     <row r="16">
@@ -1260,22 +1260,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Showing Off brengt visuele poëzie van Ziekenhuisschool Antwerpen naar M HKA: “Ik ben precies een echte kunstenaar!” - HLN</t>
+          <t>Vals bomalarm aan Grote Synagoge - BRUZZ</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Showing Off brings visual poetry from the Antwerp Hospital School to M HKA: “I am just a real artist!” - HLN</t>
+          <t>False bomb alarm at Great Synagogue - BRUZZ</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 14:38:05 GMT</t>
+          <t>Mon, 23 Feb 2026 18:42:22 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxQN0dJaG1VRGdjZWk1b0ljQWdTbmZtaDBxZU9UQU9CbFE0WHJaazJ2Y2k3S2RUVVdoN1NuRnJYejRVMkR2SlZ5UTlkaHdPcFZHRGpzdGtRQ3lLU29mcjhJVTlXWW9Ja2dPSXVmdlRnTTZnUkQwMHRHZUtPRUwtRWFwZkVuVVVCT3Y2VklTM3VHSGw5QnFHYWNPNHE1bnprQktCWlVrQXV5LWNWbUZGMVVVUk90T0oxaWhqSjZJU3hUM2NUUEliZDlKSzZvLWF3SlBGcVdSbFJpQTFVd21lNy1WU2JFc0c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNUmhvam1VWGcxVmZOSEEwLXh4cHp0ZzBPa0dpR3dxRzJpcGFzRnY3Ylc5TlRPZVllcExRbnpBT0NhSVdiRUY5em1MZGFsdk1CcmVvQVphUkVxMG5nS29BT3FCWW1QWGN1QzVuT1lTVC1wZ0tSUmZQSTI4RjdHdmZYMkR0ZzlFb2dU?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46077.60978009259</v>
+        <v>46076.7794212963</v>
       </c>
     </row>
     <row r="17">
@@ -1315,22 +1315,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Maart is Jeugdboekenmaand met meer dan 100 activiteiten - HLN</t>
+          <t>‘Spion van Poetin’ opgepakt in Brussel: zakenman zou militaire technologie aan Rusland leveren - De Morgen</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>March is Youth Book Month with more than 100 activities - HLN</t>
+          <t>'Putin's spy' arrested in Brussels: businessman allegedly supplies military technology to Russia - De Morgen</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 11:16:34 GMT</t>
+          <t>Tue, 24 Feb 2026 02:00:07 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxNYnVLZVc1VjNxVmRLaVpZWTk1XzlLVTBrV1d3bmdOZlNELXpFZDNpS3BhQ25QcmMzX0doVUdMY0NsWU5YMzg5VlF0WThSQVpiTk1EdHdHelFuMXJjbkdadldvV1hQWW9ZTzZFNWRhSzhnbVZTSk4yS3ducjlpWHV4U1NkeEVoQ29fZjZPRlFUbzJlRmRyOUVMNHpB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQODlCWFZTUFlFb01fd2dRN05EWTBuT3YzVEN6YUhDWnRnR1FfN3Y5NjdXcWJaUGtjSzZ3bkJpWGFLVkd5VEpHNzF6ZElHSC1RUGZFZlRGZUkxTHJ2MXBJOWlVMkI1aUJGX2VqeEdHU2ZWUzhqMFJFNkxuSXgzcWFSR1Z0dmxrTUJmdmpacVZnTEplVDItbUp5WHoxbkFlcnRGYmVka1dMbGt1Wk5GeTZkb3Jma0swcDhJSkdiRy15bFNMQlFwV2hJNVBnOVk?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1354,7 +1354,7 @@
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46077.46983796296</v>
+        <v>46077.08341435185</v>
       </c>
     </row>
     <row r="18">
@@ -1370,22 +1370,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>19-jarige krijgt vier jaar cel voor brandstichting bij juwelierszaak in Antwerpen - GVA</t>
+          <t>Politie Brussel West vindt bijna drie kilogram cannabis en plantagemateriaal - HLN</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>19-year-old gets four years in prison for arson at a jewelry store in Antwerp - GVA</t>
+          <t>Police Brussels West finds almost three kilograms of cannabis and plantation material - HLN</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 11:25:42 GMT</t>
+          <t>Tue, 24 Feb 2026 13:58:28 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxQa0lwTTV0TjFWaE9SaWlLNFIzVzgzX2N6S2Uzekt3Z2tLWjhrRGZnRS1aWjRXWjU0dDF6VlZHelNiNkd1UmtjSE43MGN4VmVEeDFmX01GUTR0N0x0dmdvS3NiSFVVNEV6Ym1IVUg4WEFPb0paMWhCai12YU9Gd24tWHZPSm1GUzNXbUd6YUI2VE1xaURaYlA5QllGcGUwRnpuQ3JuWWNLbTc1MkJQX182Y19NN1FZTk9iTzctR3h4eDVnWkZIa1pSWHN1WkM0QkF6eFVBTzUtQ2VaRFk2Zm1VT2pRQl8yMGpqNEhTUWlB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQVDNCRUxNSms1VFBKUXBxVTdkcGVlb2p3MGZiajBHcmFqN0oyR19uaDY5UnIwcXFQc3lQY3JncXR6blFKR0wyUVpSZ2d4UzRMeDh5UU50QllENEdBaEx3Nk1XbmNlZWE4d2Rnd2hMUVVoY3dqSjh2eWFTSnVzel9OTlV6dXBwZjVubXFWVWhhSTY3X2R1enUyM0J4bFRDYmNYTXF5U0k4aVMzRWlzaUl6UUVNNWI?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1409,7 +1409,7 @@
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46077.47618055555</v>
+        <v>46077.58226851852</v>
       </c>
     </row>
     <row r="19">
@@ -1425,22 +1425,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Drie personen proberen pakjes over gevangenismuur te gooien, politie rukt uit en rijdt wagen klem: “Ook minderjarige in auto” - HLN</t>
+          <t>Waarom laat je een vriend op straat achter om te sterven? Heerlenaar Johnny E. (43) moet na conflict binnen motorclub Kanun vijf jaar de cel in - De Limburger</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Three people try to throw packages over the prison wall, police arrive and crash the car: “Also a minor in the car” - HLN</t>
+          <t>Why leave a friend on the street to die? Heerlen resident Johnny E. (43) has to go to jail for five years after a conflict within motorcycle club Kanun - De Limburger</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 11:41:34 GMT</t>
+          <t>Tue, 24 Feb 2026 14:01:37 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxPOVNDVFlPaHBTcG1tMmc4SjlqZkFESUg0LUpFQ0hmbEhISGhva0I1Yl9IcTk0X2s3cVdFTGNkRXB5UDJvWGYtM3dzcDVKdVhmMkhJNlU1UG1YMXc3MkI5c3Z6U3pKeTBMTGUxZjN0LXBoT0lnbXpObFZEYmpGYkxkS29VUno3dTZrb2VNMFVJcFk0emhFUl8xVG90enZvRmdkeDZRWndiOWNZM2hZU0ptMFBrbVZGWThyRnpjb013RnM4MDNtdE5HdWpDM2VXcUFPNDY5M01qdjlPNXREMExQR3I5UlBpTk9EY1pCNkJIYWR0QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirwJBVV95cUxPZUV2S0NpbC1iRTlwRlpBbXB0QnBqNnZkeE9SWUQxLVdWRHp4MXloQXBvMlhNTVhXaFZJVUZKN2o2NGh1b1VyOFFJYlBsb0I4ZjJieFl5MnBYcDhYQ2Q4ZUZUVUotOExudHBNYkZlT1doSmxDd3lLbjQ0Y2FlRVZoT1JJUmFfNnN6WXBFVnZLLVNSbE9tVUJ5WWRFMmlsSk9teVFsdkNUNDlVR244Q3RnUEpjWk1HbkhHaXNDWks4T0UzYTRxMmpRQlduTGNkTUZzWmZDTmJMNC1BSFlGV0FZVG1idS1aekR2OFFrblVkMTAwQWtZVVktclJXVjNzOVhBQ3EwVUI5ZW42OUZQNS1haGdTSTFFMlNXRHdDcWllRHdWck84dTIwYlBRbU1yY3c?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1464,7 +1464,7 @@
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46077.48719907407</v>
+        <v>46077.58445601852</v>
       </c>
     </row>
     <row r="20">
@@ -1480,22 +1480,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Stad Antwerpen genomineerd voor Vlaamse Verkeersveiligheidsprijs: “Minder verkeerslichten binnen zone 30” - HLN</t>
+          <t>Valse bommelding aan Grote Synagoge in Brussel: omgeving en tramverkeer tijdlang afgesloten - HLN</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>City of Antwerp nominated for Flemish Road Safety Award: “Fewer traffic lights within zone 30” - HLN</t>
+          <t>False bomb threat to Great Synagogue in Brussels: area and tram traffic closed for a while - HLN</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 09:48:33 GMT</t>
+          <t>Mon, 23 Feb 2026 19:18:38 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxQMmZMVXphNzNLM0ZZNjFUZXpLUjhwMEF3YjI1d3FrX3ViUG9UV1drOEFFYzZtaGdZX1BwajhRZHhrcUYxRVktNENzSVktUHVMTzZycDFOSG1jZ1NiR0E0Qnk2YXdxQURVOGRFeDVqX1NUb0hiSjdHZUZTRDVLNkhmLWdJekFUNkx5YlY2QzgySVJqYXlGSXBENUNTanptQi1YR0ViU1ljTDJ4SXVERHR6b2FrQ0MwXzJLQ1RPOHBGZ1dHNWhONXpHOGpDRHhyN2Y0MkR0Sm9XOW0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxNWTVCY1dETU45MTMzQ1l4YXhSaVQyWjhjQjRtd1E0OEdMNllTQnZ5SlJiN2Rod3JUaTlMMTU3bGM2U01jSkJuUkpCUlExQXl3MUFFcE1acFdpRVY4MnQtcVdoZW5zSHlGZDBIRWlGQTFtLWd6RzJraG9iWWd2RHdJSktMYkRfaWFBN3prOUFTQTZyS1F6OUdfOWs3RzFqSzlGRF9LbDFsUG5LM1pyOGxSbWJKamItVXRmMTM0UW5EbXlmeWc3eFE?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1519,7 +1519,7 @@
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46077.40871527778</v>
+        <v>46076.80460648148</v>
       </c>
     </row>
     <row r="21">
@@ -1535,22 +1535,22 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AG Vespa zet Wolstraatcomplex in de markt: ateliers van vzw Ercola blijven tot 11 juli - HLN</t>
+          <t>Gravin opnieuw voor rechter voor verwaarlozing van 270 dieren in Brussel: “Zes inbeslagnames in 15 jaar” - HLN</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>AG Vespa puts Wolstraat complex on the market: workshops of non-profit organization Ercola will remain until July 11 - HLN</t>
+          <t>Countess again in court for neglect of 270 animals in Brussels: “Six seizures in 15 years” - HLN</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 12:28:35 GMT</t>
+          <t>Tue, 24 Feb 2026 13:03:38 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPdm9fSkhTTFNrSUNnRnRYOWowZm1zUERzY2Q1M2xYdmZSOVg4RnctSnZveVBlSGlWZ1ZvYnRram52cTVjNW9La0RSSFFjQ2V2UXV1OGlqdTNibG9CUWZQSnA3aWZJNnBFNm9GcEtQQzhDVTVUSHBodG9rQnctaF9vNVdHWW81RW5zbXlKanV0QVJPeHYtNm50RTUxM2k1UHh1cVJIMzlIcmZGdF9lY2h2RkdKZnVTQVY5d2NWdEdUTnc5dw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxNTmVTUGtHaF84MHFKTnpoVFprUC05R0Zvb3ZjdlNFcWFVYmt1TTJZYXRIZDd3bGtDMk1UTmxDSkE4V3ktRll5dkEyeVhqamxRSk40OUg1NVVJOFhCM09uWUsxaDNhMUNGZng3TFU3ZDg5cmtwYndNY2UwRGR5bUJwNVJWek1jbFFhX1JGaERGdmh4RnAxdWJJckMwQ0JTcjdIVzBOalpDemNjYnB0d0RwVHU1YUg3aE5FeEJoVU1WYkNsQXl2NURKX2k2UVhJdElpWE9CTml5eVlUUQ?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1574,7 +1574,7 @@
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46077.51984953704</v>
+        <v>46077.54418981481</v>
       </c>
     </row>
     <row r="22">
@@ -1590,22 +1590,22 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Asbest vrijgekomen bij afbraakwerken in Markgravewijk, werf stilgelegd en pv opgesteld tegen aannemer - HLN</t>
+          <t>Notoire drugsbaron ‘Flash’ gelinkt aan granaataanslag in Knokke-Heist - Nieuwsblad</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Asbestos released during demolition works in Markgravewijk, site shut down and report drawn up against contractor - HLN</t>
+          <t>Notorious drug lord 'Flash' linked to grenade attack in Knokke-Heist - Nieuwsblad</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 11:22:43 GMT</t>
+          <t>Tue, 24 Feb 2026 01:45:00 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxOYklwVUNDTmRCUm5ZbldoWlJjMloyQjd6TENkajRIZGN0NHprRTFZM0dPdFJEYTE0VmJ2UGVlZFdDd3cyMlJFUEVFRUM0UVF0MmphUXpWeE9NaV9zRmZwenliaDFycmNxMUZlQkJjanhoQ3o0MWF4WS0wenFhSXk0R19qSjdWdjdTM1dKYUxrbWZEWksyamNUa2J1SkhvM3ZwTGRycndPUlBNOUExVnBvZEdQbXpYX203UG84TkJnMjJ2YnAzUkwtYUp1cEtyV2tTbkxTRURB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-AFBVV95cUxOREMtU3Z3Q2ZUQmh2dTJKWHB5SDFYVklncFk0ZE1fUGRWUnJyUjN1OUktTGh1a29ma0ZFdFZYWENEQ3NwQUNrNEYwcW1JREdkTF9HaWlRR2pfOU04eHBXQXlHOFZKVUs3dzBvaFEyZll3eGNJUklvOFl1a0E0bnAybHFOT29YaGQyS21nUFYtd2c4VGVkZ19fb2FjQ2RtS29HZXdsLXp5R3F5RHh6VnFoTld6VTNOc3RXWlJ6dmhlTUJiTzRCTEpRVDBQdmxxYU1XbFhSdFJBTUNDLVQ0Y2Q0Qm5UTDdOekNqLWVGV2hlUWc0RVcwM0lnaQ?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1629,7 +1629,7 @@
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46077.4741087963</v>
+        <v>46077.07291666666</v>
       </c>
     </row>
     <row r="23">
@@ -1645,22 +1645,22 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Wat betekenen de plannen van Antwerpen voor de stadskas? Zo evolueert de schuld de komende zes jaar - HLN</t>
+          <t>Antwerpen dooft verlichting aan 45 gebouwen en monumenten tijdens Earth Hour - HLN</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>What do Antwerp's plans mean for the city coffers? This is how the debt will evolve over the next six years - HLN</t>
+          <t>Antwerp turns off lights on 45 buildings and monuments during Earth Hour - HLN</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 08:31:33 GMT</t>
+          <t>Tue, 24 Feb 2026 12:00:13 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxOam9oWTQ1czAwZ2pWSTRYY291YkJ0bU5qUXcxV29jZWwtVTRMY1lBaTd2SWE3NXg4TlB1OTd0RFJ2Y1pXdldkUTVBOUZsWnc0LUtuVm1raVp3TURMUEYzYkNLU1UwRm1yOXhWZlRxaHpnZmhLZlI5cTJZOU1NS2dhTlk1MVM4b3drRkhodmp2Ynd5dXRqYlpZVEtseVhxNG1tUV82OUhIcXJiTVVEWGtNTlB3SUtMM3pvVWNpT1JPNTd3cXZQTE5tb3lsLWxkYXdMem9j?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOVzR6UXJtbHMtY1FGS0t6eVZOdjNvcEFlX21xOU1WdGZGb0tPaHpndGtwdXJ4bE5nV2prVG1xM0ZQbUlsTHhkbzVZX0p0cThqWU5XQkRRZk9pbXJrZGI2VjRCelEtaXpYYUhuZnY5WUY0WXhQOGdfWDB3QWF1QWR4NVFNVjM2NVkzUjdkTlJkcVNxQ01XMERzWWU1ajkxWmVBSVFWYTlvSmN2VElyNU1uOF9jbWdUdw?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1684,38 +1684,38 @@
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46077.35524305556</v>
+        <v>46077.50015046296</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Brussels shines Ukrainian colors on buildings as EU marks four years of Russia's full-scale war - Euromaidan Press</t>
+          <t>Tiener móét van ‘Zero’ naar Antwerpen rijden... Wat later woedt brand bij juwelier en krijgen hotelgasten rook binnen - HLN</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Brussels shines Ukrainian colors on buildings as EU marks four years of Russia's full-scale war - Euromaidan Press</t>
+          <t>Teenager has to drive from 'Zero' to Antwerp... A little later, a fire rages at a jeweler and hotel guests ingest smoke - HLN</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 13:30:36 GMT</t>
+          <t>Tue, 24 Feb 2026 04:36:58 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOTVkweWFzUUNLdXBoYTJPUGNWeFI3c01LV1pqRWU2eExiOUFwOUE2MlZGaFBySWVJUmdUWGotM1BDS1lydWgwcEpZR3FlbHpuZmpDVVkyYWhNQnBSTEpMS1VscG9HOE1pREFTUlM0VHF4UV9UUjRybFNmaHpWMDlvdE5kZUt5d2lRYW9ENmFkQVFoMnZyRzY3VllEYVkzWEU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5gFBVV95cUxQX21rWDN5aHZDUzI2X1hIb1JxaDRVRXlEYlhMaGt2Uld4RjIwWGhDWWl4aVZsTVBlMndIVUZ2UFg1WUhGM0tMVXJTc3N3cFctUWJVNl9QNHRmWXpRWHowTkljR2dtNnhFSHJaY04zS01WYl83Y0gzcG5famVkOUs0TGJWZlpTX201U2hvOEdPVmFCNVNpV1pxb2VkallKbEtfc3Z2NGEwdmRZSmxObEVDQXAyM0ZPeWpORXhWMUJNOGo4UDZDQ0dheDBCY3ktYlVVblNHQ2VGalpTZVNWZzRfQmtkaVEyQQ?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1735,42 +1735,42 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46077.56291666667</v>
+        <v>46077.19233796297</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>West must support Ukraine ‘every day until bloodshed stops’: NATO chief Mark Rutte - The Straits Times</t>
+          <t>Antwerpse takelpionier failliet: takeldienst Viaene legt na meer dan 50 jaar de boeken neer - HLN</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>West must support Ukraine ‘every day until bloodshed stops’: NATO chief Mark Rutte - The Straits Times</t>
+          <t>Antwerp towing pioneer bankrupt: towing service Viaene closes its books after more than 50 years - HLN</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 10:27:00 GMT</t>
+          <t>Tue, 24 Feb 2026 10:34:08 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxQZnNnQURka1FpeVppWjNTcnRjSmpQVHA1d0VQRXN3MkR5aWtqTW02SVduMExEbUJQYWp0X3dPbzVySndQZTBuQzlSOGF5V25pSFFVN2RNemFsU2Z1SzNpTzBfUU5HenlhREJtNGUydFpuNG1US1JtbE83NENfZ1RlY0dhSDY0TnRjeWU1bk0xOXJmNndmNE1VQnBJdUQ4VloyeE03YmdXTXpIUkZ4ZmZ0UEg4d2ZqaGwtdEh4UTFITExSWDhsZXZCclY1NEhZSHF5SmV1TlgyLU9oZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxNanBoV2o1anpZNlhuVEdxS29TaUh6VXdodFVkZTExeW1uUkZsZElSendqbzhoczRLTVdvOWRKcE9Wa2lINkVfQjRtRjBYSVdvck5wM0RPeFpMaFdpcjR5LWYxUndSNDczZGg3Tk5zbzVYQUdyWThVQVg3dEF5UEE3aVdoRFZIWFhINlFlN3NWM2V5YzQxU1FZSXJ1OThxcDMyeldEWk91MlFwbWRGb3ptNE9VbUZTcExhZWcyeU9SY00yYTF5alNaeA?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1780,7 +1780,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1790,42 +1790,42 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46077.43541666667</v>
+        <v>46077.44037037037</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Alerte à la bombe levée à la Grande Synagogue de Bruxelles - 7sur7.be</t>
+          <t>Oplettende voorbijganger helpt politie inbreker te klissen op lijnbus richting Antwerpen - HLN</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Bomb alert lifted at the Great Synagogue of Brussels - 7sur7.be</t>
+          <t>Attentive passerby helps police catch burglar on scheduled bus to Antwerp - HLN</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 12:16:00 GMT</t>
+          <t>Tue, 24 Feb 2026 01:58:36 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOOTRkZE1mSU1wNTNCODJ6TEt2WWtuTF9yMUR4c1BOb3ptMExaU0ZJSUFyek96ZnpGaHRGRFd6aElmLU9WeXN4ZEZZazVsLTRUNDREamdwTGlMLXhsSHZoLTYta2gxNlBzUlhmRkdCaWZub0xBQl94VTdDZmZhU2s5b1R5TWRpd3BZV3JDS1NTRWRsUjZtemdVLTdaTmkzVDJEVzRCNA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPSVVWMEZtMTZNTVN3YnZYTjhHMGl5blBYNVVoZ2pTOWVzYlhKMm1hVkZRUWtmNEVIcWdRalJteGJuR3VSSU9IWEhUNTQ5aG9GWDBfYUNpb0dZdll4c2NJRTlCTXlIUDFNSkFMTWtQZ0I2SUU1b1Z1TGNhUzlUTWZ4dVlvd0lEQ0c0ZFVfbGZJellkNkFfSGdhU2pTSExLcUFod1JxMEZuVlE0UjExQnRQTHdQM1dTTUp4YldiazRYTmxTaVE?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1845,42 +1845,42 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46077.51111111111</v>
+        <v>46077.08236111111</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Vakantiehuis Fabiola in Maasmechelen voor kinderen met een beperking krijgt toch nog 1 jaar subsidies van Vlaanderen - VRT</t>
+          <t>Antwerpse Vervoerregioraad verwerpt besparingsplannen van De Lijn: “Terug naar de tekentafel” - HLN</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Holiday home Fabiola in Maasmechelen for children with disabilities will still receive subsidies from Flanders for 1 year - VRT</t>
+          <t>Antwerp Transport Regional Council rejects De Lijn's savings plans: “Back to the drawing board” - HLN</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 07:52:45 GMT</t>
+          <t>Tue, 24 Feb 2026 13:08:51 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE5OenpKUkhrQ1AxTlBhUlRETGdRSFpRaVJKOW9TelBUUXdpU01tdmEwZ0VFM2dvR05IaFViZkVWM0YxLVlwU2ZETUxJbld6c3NrTm1DU1Z1SWlzZG9PNWFyZEJMSEVyX2hCY1BIa1RGaHdtQi1OQU9pR3ozdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxNZ2hxaTJvZkxLVUJBOUt5d28yc2dPMmpaZ0lueFc3WHVYd01WMWlweDBQVTk5OFRTMVlJQUxFUXpwRFFfSEJEWGtkcnJPTi1zelo5T1pvelFOTTQ1V3J2cnlaY21saUFUMHU0QTlSeC1xMk4tTzRFNndIek84QmxrS0FLbThyek1yU09ueVlhemZiaWF4OGc4VE44SnM3cXE3RDlqSkxwSy1XUzlVVGtuTXhWb29ETm9zNmRYbTJiRlpfdHlyTVl1Qg?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1904,38 +1904,38 @@
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46077.32829861111</v>
+        <v>46077.5478125</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Halen keurt aangepast meerjarenplan goed na budgetfout van 5,4 miljoen euro - VRT</t>
+          <t>Beurtelings verkeer op de Kapelsesteenweg door bekabelingswerken - HLN</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Halen approves adjusted multi-year plan after budget error of 5.4 million euros - VRT</t>
+          <t>Alternating traffic on the Kapelsesteenweg due to cabling works - HLN</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 09:32:52 GMT</t>
+          <t>Tue, 24 Feb 2026 12:05:04 GMT</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPOTItcThiT1hZQjVXaDA5TEI5RUlVdmt5N1UzR2hEelF2aVBXemRfcTdNbk9xUk5sY2NfWkpJdmIycHN5TThoaVNnVVpCWjgzYXExeFpZUk91bVhhdFhiZ0szcDNRT3Nua3RCSTVUa1BTSGRUdU42TXJ3NzVYSXdFMTRZMkwwUVpqaURzNXJMMVIwbk1rNzNSQVdVaUVvdHRVNGNWcURCUzA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxPVVVoM3lVUzdhOWJUT2lGSi1HbDRHQmExeG1falVTUEt1WEdBRFgwRlJJWUJIV0xmd0M2UmlkdTN5X3RDa2Y4b1FjU2RzSGdFMmdXMHNsSGZhUXBIeHR0Mkh4MDhVdTREbTFsYXV6UUtxRzRIM2ZCM09MQkg0RXo5c1Y0YXcxZ3lSSmhyM3dpemoyMU13UlJNSVR0LTI1ek5sWGN6cWxn?oc=5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1959,38 +1959,38 @@
         </is>
       </c>
       <c r="K28" s="1" t="n">
-        <v>46077.39782407408</v>
+        <v>46077.50351851852</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Environ 50 emplois menacés par la faillite de IKKS Belgique - RTBF</t>
+          <t>Maart is Jeugdboekenmaand met meer dan 100 activiteiten - HLN</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Around 50 jobs threatened by the bankruptcy of IKKS Belgium - RTBF</t>
+          <t>March is Youth Book Month with more than 100 activities - HLN</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 09:35:30 GMT</t>
+          <t>Tue, 24 Feb 2026 11:16:34 GMT</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQZE84MHM2aGc2b0JUc0dFQ0NzbXRhQTBKbDNILXRpN3o3Q1VxMmZnXzRIVXQxMlFUWjJ5U1ZWWjZFeFNCTEZ4bmlYN2VJOWpNLTRoRFREMlpITHhSTWFsN01STkN1THFxZmd3cEFPeFlSWVQyNm85Z0pVOW1LM2xnS29zeVJyUklsNGpDMDdJNDIxZENMbldhWXE1SHk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxNYnVLZVc1VjNxVmRLaVpZWTk1XzlLVTBrV1d3bmdOZlNELXpFZDNpS3BhQ25QcmMzX0doVUdMY0NsWU5YMzg5VlF0WThSQVpiTk1EdHdHelFuMXJjbkdadldvV1hQWW9ZTzZFNWRhSzhnbVZTSk4yS3ducjlpWHV4U1NkeEVoQ29fZjZPRlFUbzJlRmRyOUVMNHpB?oc=5</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2000,7 +2000,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2010,42 +2010,42 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K29" s="1" t="n">
-        <v>46077.39965277778</v>
+        <v>46077.46983796296</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Courtois va investir en Belgique : deux clubs mentionnés - FootNews.BE</t>
+          <t>19-jarige krijgt vier jaar cel voor brandstichting bij juwelierszaak in Antwerpen - GVA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Courtois will invest in Belgium: two clubs mentioned - FootNews.BE</t>
+          <t>19-year-old gets four years in prison for arson at a jewelry store in Antwerp - GVA</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 12:39:21 GMT</t>
+          <t>Tue, 24 Feb 2026 11:25:42 GMT</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxNTlJDdTgzUm84dnhidVNwNUtTZGJqbWZZOVJmSHBzU1QyYmk4QV9ZanJ5TG12cXFKVDhVSHplR2dudWVsb3RlWjZUd0FpVmhHZFJfQzFnTlpvMnJwX2Y1Q3RLY1lzTlNWQ0JNSXAyalBMNm9YazVTenlGUXdranlMbjlwWUpSSlppbjF6SXU1aGJJd185?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxQa0lwTTV0TjFWaE9SaWlLNFIzVzgzX2N6S2Uzekt3Z2tLWjhrRGZnRS1aWjRXWjU0dDF6VlZHelNiNkd1UmtjSE43MGN4VmVEeDFmX01GUTR0N0x0dmdvS3NiSFVVNEV6Ym1IVUg4WEFPb0paMWhCai12YU9Gd24tWHZPSm1GUzNXbUd6YUI2VE1xaURaYlA5QllGcGUwRnpuQ3JuWWNLbTc1MkJQX182Y19NN1FZTk9iTzctR3h4eDVnWkZIa1pSWHN1WkM0QkF6eFVBTzUtQ2VaRFk2Zm1VT2pRQl8yMGpqNEhTUWlB?oc=5</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2055,7 +2055,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2065,42 +2065,42 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K30" s="1" t="n">
-        <v>46077.52732638889</v>
+        <v>46077.47618055555</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Official | Ousmane Dembélé and Fabián Ruiz out of PSG’s Champions League return leg - Get French Football News</t>
+          <t>Stad Antwerpen genomineerd voor Vlaamse Verkeersveiligheidsprijs: “Minder verkeerslichten binnen zone 30” - HLN</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Official | Ousmane Dembélé and Fabián Ruiz out of PSG’s Champions League return leg - Get French Football News</t>
+          <t>City of Antwerp nominated for Flemish Road Safety Award: “Fewer traffic lights within zone 30” - HLN</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 13:32:37 GMT</t>
+          <t>Tue, 24 Feb 2026 09:48:33 GMT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxNRHZ4dm0tREV0cjFucHowcUNrWGlJTVljdlFXcjNtdFg0OUh4a2hWb25ucnlzMkNMdThqU25BNm1yaHhBRk8zTDRwcHdHRHZFRUNBSVlHcXZjdDJFQU95SEVCM20wQm1YNmFzczRjdzE5UmZUY2NpWldzMWRfdXpSVmo4ZlpsVHdNOWo1aVFGcVRBc0I5RjVyYkRGeXZmVTBGZkFvNy0xZFVxa2JNZ0RzeGt2dHJCZTZHUTU1RXRZbzNpQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxQMmZMVXphNzNLM0ZZNjFUZXpLUjhwMEF3YjI1d3FrX3ViUG9UV1drOEFFYzZtaGdZX1BwajhRZHhrcUYxRVktNENzSVktUHVMTzZycDFOSG1jZ1NiR0E0Qnk2YXdxQURVOGRFeDVqX1NUb0hiSjdHZUZTRDVLNkhmLWdJekFUNkx5YlY2QzgySVJqYXlGSXBENUNTanptQi1YR0ViU1ljTDJ4SXVERHR6b2FrQ0MwXzJLQ1RPOHBGZ1dHNWhONXpHOGpDRHhyN2Y0MkR0Sm9XOW0?oc=5</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2110,52 +2110,52 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K31" s="1" t="n">
-        <v>46077.56431712963</v>
+        <v>46077.40871527778</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>LolaLiza acquired by three board members following management buyout - fashionunited.uk</t>
+          <t>Halfuur file op E313 richting Antwerpen na ongeval op aansluiting met Antwerpse Ring - HLN</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>LolaLiza acquired by three board members following management buyout - fashionunited.uk</t>
+          <t>Half-hour traffic jam on E313 towards Antwerp after accident on connection with Antwerp Ring - HLN</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 14:08:23 GMT</t>
+          <t>Tue, 24 Feb 2026 07:35:25 GMT</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPNExOajRSMzJtQk9kOENCeXlHM25OUm5vVWQyUkszamgzQjVOMm92anAtdHN2QXhFLUVMLUptNVJ0YzV5dFJWTE5OeVNCMFVobnlyelUzeFBadlNFV3hCRVI0Y3pUTExVYU9TNFdwVUNsaXhyQjc2QW5MZlh3Rk9rejhZUDhEU1h3LUVQWHhBWHNHWG80NUltV2hxd1YwWmhRVVZyOHotOUdQeEp6UlVQYi1iVDZWcHFOanBzWWFB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxPOHNXVzE2SUxteEFZb21NakZYTTBBNmlvRGJDTWwzVjF1Ykh1d1pFNTZpcjQ2VWFqc1dwMEpWMm1mWFZkVk0talpZOUx0dnBWUEhqMlA3WkFDUWo5SkRTVlhoeVZTSXFsT3RfVU5UTkpKWEM2bC1kdGw4eUdVNmRIaXZyR0xKQVgwTnJrTG5pYTV3ZDRwdHBJZ0hlR0hreGlORnNjbjRhMExHRDJaYnVvRE5saUV5amFQWV9kUVpFby0?oc=5</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2165,52 +2165,52 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K32" s="1" t="n">
-        <v>46077.5891550926</v>
+        <v>46077.31626157407</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Village Maasmechelen (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>("Maasmechelen Village" OR "Maasmechelen") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>IKKS declared bankrupt in Belgium: dozens of jobs at risk - fashionunited.uk</t>
+          <t>Wat betekenen de plannen van Antwerpen voor de stadskas? Zo evolueert de schuld de komende zes jaar - HLN</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>IKKS declared bankrupt in Belgium: dozens of jobs at risk - fashionunited.uk</t>
+          <t>What do Antwerp's plans mean for the city coffers? This is how the debt will evolve over the next six years - HLN</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 13:03:27 GMT</t>
+          <t>Tue, 24 Feb 2026 08:31:33 GMT</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOUW54aFlQc196RnJXM0FfVWU5a2JSN2w2MXdiZVg0Z2U2aXdKZENsNThtVWVvQjg3U0FwUUQ2Qk5SZF9rSnVqQWxrc1VzOUNzcVRfbWVXNWFCUW80ckl3MHJlaTZvUElidlBqZWNlSm85a1otTXNBMkpYTlQ1YzJBcDVNNkY1a2o2OUJtNG1HYnItU2RodXRXb1pXMVFOTkF6ejk3cEY4ZTdRbTA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxOam9oWTQ1czAwZ2pWSTRYY291YkJ0bU5qUXcxV29jZWwtVTRMY1lBaTd2SWE3NXg4TlB1OTd0RFJ2Y1pXdldkUTVBOUZsWnc0LUtuVm1raVp3TURMUEYzYkNLU1UwRm1yOXhWZlRxaHpnZmhLZlI5cTJZOU1NS2dhTlk1MVM4b3drRkhodmp2Ynd5dXRqYlpZVEtseVhxNG1tUV82OUhIcXJiTVVEWGtNTlB3SUtMM3pvVWNpT1JPNTd3cXZQTE5tb3lsLWxkYXdMem9j?oc=5</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2220,52 +2220,52 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K33" s="1" t="n">
-        <v>46077.5440625</v>
+        <v>46077.35524305556</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Wertheim Village: Polizei stoppt mutmaßlichen Seriendieb - Fränkische Nachrichten</t>
+          <t>Asbest vrijgekomen bij afbraakwerken in Markgravewijk, werf stilgelegd en pv opgesteld tegen aannemer - HLN</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Wertheim Village: Police stop suspected serial thief - Fränkische Nachrichten</t>
+          <t>Asbestos released during demolition works in Markgravewijk, site shut down and report drawn up against contractor - HLN</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 09:34:00 GMT</t>
+          <t>Tue, 24 Feb 2026 11:22:43 GMT</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxNempGdjdfTkxudlBkZnlNYlNUS3h0MEluS3JYU2tOVW9zamM4QUdCODMyNTAwc0ZDY0NCYXpReG9wOTVtOUY2eW9rWmhxT0RHaUdubGNoWVN3SjBCaE8tSlBpSTlneF9aQnNMdHR0VDI3Wjk4el80OU91akJGYWV4aVVuM01SejN5NC1rQlg0WElRd2VJbXVhZEtjZEVwdDAtYlZnSFFjazhjOExOcGszYmt1X0hEUlZyQjl3aTRWXzZxWHJ1NXlJ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxOYklwVUNDTmRCUm5ZbldoWlJjMloyQjd6TENkajRIZGN0NHprRTFZM0dPdFJEYTE0VmJ2UGVlZFdDd3cyMlJFUEVFRUM0UVF0MmphUXpWeE9NaV9zRmZwenliaDFycmNxMUZlQkJjanhoQ3o0MWF4WS0wenFhSXk0R19qSjdWdjdTM1dKYUxrbWZEWksyamNUa2J1SkhvM3ZwTGRycndPUlBNOUExVnBvZEdQbXpYX203UG84TkJnMjJ2YnAzUkwtYUp1cEtyV2tTbkxTRURB?oc=5</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2275,52 +2275,52 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K34" s="1" t="n">
-        <v>46077.39861111111</v>
+        <v>46077.4741087963</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Unfallfluchten in Aschaffenburg und Kleinostheim | Foto: Dirk Ceelen - main-echo.de</t>
+          <t>Royal Caribbean bets on flexibility with new Discovery Class vessels - Travel Tomorrow</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Accident escapes in Aschaffenburg and Kleinostheim | Photo: Dirk Ceelen - main-echo.de</t>
+          <t>Royal Caribbean bets on flexibility with new Discovery Class vessels - Travel Tomorrow</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 13:03:01 GMT</t>
+          <t>Tue, 24 Feb 2026 13:53:01 GMT</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxQMW02WVZqN19mTERhVXdiT194SUtPU2ZxVTJ3dGNKd2ZLQzVmM2lxb3lTdWpHVjBqOVlFTFVOYXE0d0czbUpZQzFFU19OT294MmdqVlU3d2M1QzFWUndPbm02SVBvakFlc0tVSnl6YXJjOUNaN2FvNUYwX1pOOGJ3aVJoZjlPOU9DWnFRZlBlZG5uNXN4N3ZvWnpYN21VX2M1Skppd2c4Zw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNXzV4T21XbFJaMGdnTnl0X2FFTzhwUk9aZ0Q1TWRVTENZRXpWU1hWRGJnY3VzcGZQNFRHcmg3TFpLTVN5NnBDZ3ZhX19wcmhtT1VncmtlcGFIYTRKRUxYd2R0d0R3dDM4eUN2Vk9GWHdFWVZ1NnBpV0drZkxXRGtUN2FBejJyNng1ak5iMTVWeUx5ampWcnBVanlMU3Q?oc=5</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2330,52 +2330,52 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K35" s="1" t="n">
-        <v>46077.54376157407</v>
+        <v>46077.57848379629</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Marktheidenfeld: Polizei kontrolliert erfolgreich - aschaffenburg.news</t>
+          <t>Brussels shines Ukrainian colors on buildings as EU marks four years of Russia's full-scale war - Euromaidan Press</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Marktheidenfeld: Police check successfully - aschaffenburg.news</t>
+          <t>Brussels shines Ukrainian colors on buildings as EU marks four years of Russia's full-scale war - Euromaidan Press</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 14:09:08 GMT</t>
+          <t>Tue, 24 Feb 2026 13:30:36 GMT</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxNM0F0V01ZMjFGbzFpQ0FldUNxRnI4UkplZ2daMUlzTXNvWGM2WnlUZGprenhxMXBfSkRrLTFkWUU2c2VFODdxRTU1bWF2bVNZeW9zWWVPaEtGU0ZfdUdGbVBKOGt3dEdmaUszMTdlZnFuNUV6b0JWUEFtVjBlTmdFQXh5SXhuZTN2eVVzelU2Z29RUU9wNGw2Z1Vn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOTVkweWFzUUNLdXBoYTJPUGNWeFI3c01LV1pqRWU2eExiOUFwOUE2MlZGaFBySWVJUmdUWGotM1BDS1lydWgwcEpZR3FlbHpuZmpDVVkyYWhNQnBSTEpMS1VscG9HOE1pREFTUlM0VHF4UV9UUjRybFNmaHpWMDlvdE5kZUt5d2lRYW9ENmFkQVFoMnZyRzY3VllEYVkzWEU?oc=5</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2385,52 +2385,52 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K36" s="1" t="n">
-        <v>46077.58967592593</v>
+        <v>46077.56291666667</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+          <t>West must support Ukraine ‘every day until bloodshed stops’: NATO chief Mark Rutte - The Straits Times</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+          <t>West must support Ukraine ‘every day until bloodshed stops’: NATO chief Mark Rutte - The Straits Times</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 12:52:25 GMT</t>
+          <t>Tue, 24 Feb 2026 10:27:00 GMT</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE03RUZJdVVWTG5jTlA1R0dmc2YyQ3Z2S1ExYmhkN0FENFJGamUwenJsSFFPWGpKc3B2aFBaeHRYVDR3aWM1SXg0YWZFVDk0N3d4a0Jz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxQZnNnQURka1FpeVppWjNTcnRjSmpQVHA1d0VQRXN3MkR5aWtqTW02SVduMExEbUJQYWp0X3dPbzVySndQZTBuQzlSOGF5V25pSFFVN2RNemFsU2Z1SzNpTzBfUU5HenlhREJtNGUydFpuNG1US1JtbE83NENfZ1RlY0dhSDY0TnRjeWU1bk0xOXJmNndmNE1VQnBJdUQ4VloyeE03YmdXTXpIUkZ4ZmZ0UEg4d2ZqaGwtdEh4UTFITExSWDhsZXZCclY1NEhZSHF5SmV1TlgyLU9oZw?oc=5</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2440,52 +2440,52 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K37" s="1" t="n">
-        <v>46077.53640046297</v>
+        <v>46077.43541666667</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Streit bei Auto-Kauf in Aschaffenburg: Männer gehen aufeinander los | Foto: Karl-Josef Hildenbrand/dpa - main-echo.de</t>
+          <t>Landmark Scottish museum set to reopen in 2026 after major renovations - Travel Tomorrow</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Dispute when buying a car in Aschaffenburg: Men attack each other | Photo: Karl-Josef Hildenbrand/dpa - main-echo.de</t>
+          <t>Landmark Scottish museum set to reopen in 2026 after major renovations - Travel Tomorrow</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 12:34:53 GMT</t>
+          <t>Tue, 24 Feb 2026 11:37:51 GMT</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxQNXA4Vkl0TlZ2Ui1SOTgxNWVUcF8xdXdtOUJsODFOalIybVlxTkU3SURZVHc5aTFsdHNHMGR1SXNvNWZGdlgyT0dzbHZmbmtQMklfbERteC1yMWw4WFVvUzhGSWQyb1J6X3hPcmRBVkFfVkxMbEtkWDMtbGZWckV4LTZVLXBvUUk5ZEFNMlJ3SE80TXZ0V2JEakttUjJkWmtoX3djX01wY2dUbDhoLXQtRm1qVXpwZzlfM2UxWXRTYng?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxORGJ2bWpnWEhuN0JwZ3pXU1FBQzYwWWxWRGZOTUFleFlQZmt1d3NKd0FwWjdzal83cXZLS3hxV201SmU5NHRyOGQzeURSampqR19yYnFfR2NSSnFSWllIYk9adGdBM25ndGFzTnc5LXk5MlVNdEllY05VUXh3YXJqbjk5eDVMTGxTZ3I4a1NacjF3bFUzTTZCZFVQT3BneEk?oc=5</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2495,52 +2495,52 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K38" s="1" t="n">
-        <v>46077.52422453704</v>
+        <v>46077.48461805555</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Kleiderdieb in Untersuchungshaft - NOKZEIT</t>
+          <t>Hungary Blocks EU’s 20th Russia Sanctions as Oil Row Sparks Explosive Brussels Showdown - The Times of India</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Clothes thief in custody - NOKZEIT</t>
+          <t>Hungary Blocks EU’s 20th Russia Sanctions as Oil Row Sparks Explosive Brussels Showdown - The Times of India</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 08:58:15 GMT</t>
+          <t>Mon, 23 Feb 2026 17:55:34 GMT</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFBKUUNfaWVwNkcxMmtpalVDTWxaMGNYQl8zZEVkWlFUMVk0UjFYa0Y0OEpFMERfaGMtSUI1dlU4cHVxLUJJMWxnV3FMcFdnNnQzc2s4RVVnamxfLXRxRjR3a3VYNkd0Q2pTcGVPb0lpTFE2ZE9KZUE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxOTlJDdnZJcUhhajNFWEtvMldrV0NBVDlQbThJYXI2MVBCbktZNWQ4dEtWVEc1bW9KT0RkRTFGcENzamNHQXd2STBjMVRQc1N5S3pvdHJ1TGFjeTc0STZMZ0t4MFY5RGJuNnowc3ZFcDRaV1VZQkNqNWF1Q21hcEcyc1VqTi05SUl0eF9nQ1lYYlFoQXNuWjdsM3c5TnNUeGliX3dvLUdwSWk0YzY0eENTb3hhNDJFN3VBMHZpRlViQ0lrcVkzLUFXS1BGdzNyZkd2ZDBMdzdEU1JSOUxHV0ZsdGZHRU9LSGl3SHpRQnd4RW5YdS1Udlp5S19jVdIBgAJBVV95cUxQSno4aUl4RDNXXzh6UXNFdWJyMHh3SkJzbEd5NFI4ZE5PRFRHWE10ZllZXzNVam1LdXZWYnBaeU9PYkJvcks2VXRLeEZlRFR0VFp1N21XZVdiMGZXaGszMER3OERaR0hHbDREYndvQ0ROdmFEa0l1dkFxemVRNkJBOGtNVFNWQjJpeW5DWjFneTBBMDlQbjlOVXRBanNybjNMR2ZZQkRyM1lRUDNHV0YtT3pYbVAwbTNuX1BBckZRa3RfeHd1SHhlOVZheldMTzh4eEZuWkZWa2VTWXNfaDV0TWx5a2lqcm4zZmhDaFpEQ09PMXhlYnRVRDJqRXNQdERG?oc=5</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2550,52 +2550,52 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K39" s="1" t="n">
-        <v>46077.37378472222</v>
+        <v>46076.7469212963</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Herrmann begrüßt deutliches Personalplus für die Bayerische Polizei - aschaffenburg.news</t>
+          <t>EU adds eight Russian officials to human rights sanctions list - The Straits Times</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Herrmann welcomes a significant increase in personnel for the Bavarian Police - aschaffenburg.news</t>
+          <t>EU adds eight Russian officials to human rights sanctions list - The Straits Times</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 11:06:28 GMT</t>
+          <t>Mon, 23 Feb 2026 15:16:00 GMT</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxNU0FPOVFwS1pZal9xUnlUNDVjT0wzY2xwRG5TUmdob3JERkNFdld6ZHdVTHJBdnAxOGl6VW5jeTNxMmxtWjZfSVdkczVTaVdTNFBIaEN0VzBTbUkzRHk0QlBJSEU0bEk0aVJIT0lsdnV6VE91WUZDMGRybGhMSmVMWEM1R2hId1pvN3E2Z3BOT2xYZk5vMm03Vjk3dHNfV3ZhS05OM3RqX3J0b25uUTRadzZLaDJXWk5KbzdmLTZ0OA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxQTU1vZDZ1QWVmS3RBUktpb3I4a3pkN1FFaGtkRkl3U0FKOUVQUF9Ec0VmVld3ZHJXQ3B6aGpZS3dxU3hzdms4Y2w5cGZWZGw5UlZmenVlRl9ZdkZidEd2OFUtRll3UlFIbXAzTGpUeVNhZUZlVUlBbUp2azdxYnROMDRFYmRYOFhVLTNMd3pWQXhmaUg2Qk9LNDdxd3BxM3BqelAtSVctWXNPVzRETmZySFZLcjdDcEpDR3BOTnJ4X1l1dw?oc=5</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2605,52 +2605,52 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K40" s="1" t="n">
-        <v>46077.46282407407</v>
+        <v>46076.63611111111</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Unfallflucht an Rastanlage Spessart: Schaden an Kleintransporter | Foto: Stephan Jansen (dpa) - main-echo.de</t>
+          <t>Alerte à la bombe levée à la Grande Synagogue de Bruxelles - 7sur7.be</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Accident escape at Spessart rest area: damage to small van | Photo: Stephan Jansen (dpa) - main-echo.de</t>
+          <t>Bomb alert lifted at the Great Synagogue of Brussels - 7sur7.be</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 13:03:26 GMT</t>
+          <t>Tue, 24 Feb 2026 12:16:00 GMT</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOQkJUQUtFSW5nMU05Unk5Vmx5ZkJXem1XV2JHVEFKSjBISGN6OU5wZElaUjlWZ0pZMGc0MHlJcEJqcDRSNy1od1dCY0dQdUZVX1VWdHJwSk9aMUljaXoxLWxmbWdZSnhMU0EtcE9DXzlRQVEyNVlpd1R5NnVvSElCVVF5TjB2VHZpLVpOUTJvYkdTVHlSTVhudzI4YmI0YnUycUpFLWtFMndDby04OU1aRWVZY2MwQmVKTE44?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOOTRkZE1mSU1wNTNCODJ6TEt2WWtuTF9yMUR4c1BOb3ptMExaU0ZJSUFyek96ZnpGaHRGRFd6aElmLU9WeXN4ZEZZazVsLTRUNDREamdwTGlMLXhsSHZoLTYta2gxNlBzUlhmRkdCaWZub0xBQl94VTdDZmZhU2s5b1R5TWRpd3BZV3JDS1NTRWRsUjZtemdVLTdaTmkzVDJEVzRCNA?oc=5</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2660,52 +2660,52 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K41" s="1" t="n">
-        <v>46077.54405092593</v>
+        <v>46077.51111111111</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Helmstadt: Nach Einbruch in Einfamilienhaus – Zeugen gesucht - Radio Gong Würzburg</t>
+          <t>La Ville de Bruxelles supprime une taxe pour l’installation de panneaux photovoltaïques - 7sur7.be</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Helmstadt: Witnesses wanted after a break-in in a single-family home - Radio Gong Würzburg</t>
+          <t>The City of Brussels removes a tax for the installation of photovoltaic panels - 7sur7.be</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 14:00:00 GMT</t>
+          <t>Tue, 24 Feb 2026 08:48:00 GMT</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOeHEydHhfR29sSVFqWENkVEU5ekVMTnRTcmFoZXhIeFJNVTMzSGN5dzNjZjVtZVk0TnhtSjRNUmRTRC1OdndqNVV1MDJadHZUdlU5UjBtTVV1b2k0TC0wX25XXzdGQnk4VVR5Rno1akhMM19aOGRNZURrcmJ4cEh2Z05UVFpqQURvalNLcU8zcWZ4RG1PdWc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxPRWg0V2dNa1lZdG1wUWp4V181cklFS3JlWnc0VkRIOEN3STFyRUtURmRRSlQ2U04xQlVMWERsbE12eXpqUDE4QjZPTFl1TDBOVzk4N0YtQzRGSXVYcE9QZDJnem0yZ0xGSkRLN0RWQzJfSDJYbDl6VmktQUQzMFZGRXBYcWpIX3J5SnVlWVlIeXlQVW0zbHNCQ0NNWXZyN2VXVWdLTWVYTU9BOGkwMGhWUmZDQ0o0aUg3bVd0ay04TjBWLWxo?oc=5</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2715,52 +2715,52 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K42" s="1" t="n">
-        <v>46077.58333333334</v>
+        <v>46077.36666666667</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Würzburg: Messerattacke auf Zeugen Jehovas - Idea.de</t>
+          <t>Trafic de stupéfiants à Montignies-sur-Sambre: Un individu arrêté - Télésambre</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Würzburg: Knife attack on Jehovah's Witnesses - Idea.de</t>
+          <t>Drug trafficking in Montignies-sur-Sambre: An individual arrested - Télésambre</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 14:00:03 GMT</t>
+          <t>Mon, 23 Feb 2026 15:16:10 GMT</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiekFVX3lxTE55UThGQWVSVnBMUGM3RFpMeDJJbjc2Zi00aVhuV1lVeW9rZmw0WXdNdmZFY0REWGpQZUtUelROVXl5RE9KMkhJNlRoNUNvN09sS3Z3aTVjMWp3N0ZWc05CZmdGeWVPUzR3VXhBMFNkTnVWWWNTOFlwcnJ3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNSXp2bmZ5TlN5YkZZLTBhalF5SmRHRGd4Mk50dWZZdW82WngwNXVXTDNSUXdfdWZET2t1dlNCcjZLTVdOY01DYTBQaVMzY3draDBabE13cHlYZ0xJeGNwYlhGdkNLU0JkMGZvSW5xZGZxX0FWLWtFRmF6N0R0TFlhdFVnZXNPczVNUG9zT0ZYMUl6TlFUQ09SbHFPeUZ2SFk?oc=5</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2770,52 +2770,52 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K43" s="1" t="n">
-        <v>46077.58336805556</v>
+        <v>46076.63622685185</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Erfolgreicher Callcenterbetrug: Falscher Polizist holt Wertgegenstände ab, Kripo ermittelt - Mainfranken News</t>
+          <t>La justice alerte contre le phishing via de fausses applications: “Impossible de distinguer le vrai du faux” - 7sur7.be</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Successful call center fraud: Fake police officer picks up valuables, police investigate - Mainfranken News</t>
+          <t>Justice warns against phishing via fake applications: “Impossible to distinguish real from fake” - 7sur7.be</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 14:06:37 GMT</t>
+          <t>Tue, 24 Feb 2026 06:20:46 GMT</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxNRkZoQVNGWmlQVjB6c210V3RQRjYzeWxmU1RkQmJURFJhajlmQkVvRjI4V3d4U3AyQm1GajFjYUlteHcyYV9LcTQ3Z3ZMdklUbm9DemlqMkdvRnlTeHJJd1AzejlhMjlFOGJGYklWQlZ6cHRYekZYNkttNUFReWlieW5WVGY0aTRuVWRVZUZIRlpSZ1B5clJnMEh5VWtqVXZXbHZ3SnN5T0ZvSEJVa3h5X3hGdmxyV2pfSDVCejJ3Smd0NE9s?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxQOHpEb0RWNVpvS08zNmdON0xCMzUwN3VHZ21lcnFtS2syVEd6ZVAyNVJSdmduUy1vRVhpOUwtaV8xSksxVHA2UkNmRm4zQk5oMkpUVUplQzB4QU92SWRFTFNrQjZ6M0g3di1FeW1ZM1dXbmEweV9ISTRzZUR2ZUg5NVNabHdNajZRdE43bElzZVBodU5NUzl5OTZsMGJvam1fdTBVczE4RHc5UE9sd2NkdDFSNEdmNnF0X0ZLMUtzbllsZzhzbDhXVXB2UkF2S0RkN0FPcm1SaW9pNW93Z2c?oc=5</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2825,52 +2825,52 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K44" s="1" t="n">
-        <v>46077.58792824074</v>
+        <v>46077.2644212963</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Frammersbach: Falsche Spendensammler - aschaffenburg.news</t>
+          <t>Opnieuw laadkabels gestolen, nu in Maasmechelen en Lanaken - VRT</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Frammersbach: Fake fundraisers - aschaffenburg.news</t>
+          <t>Charging cables stolen again, now in Maasmechelen and Lanaken - VRT</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 14:06:56 GMT</t>
+          <t>Mon, 23 Feb 2026 16:16:31 GMT</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNQmphdE5lMlFNZTFQYTdWTzBNU1pHMUc2YWlxZXFPc1BZWlBWZ2lnME9Xa29OcmFCeE5XeTlZS21YRTVSeGU1OEUtOHdCZTNwZE1CWHoyQkl1VlZfcDJQQmphOGh6V1J5YWs3cmhLSmU5Z2tFbGJuWGJBQlZxbEJPYXo4T2stUlVW?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQLXpEcnVvUUFXZTVvb0o3cEl0bG8taUR5R3ZmT1RybVhhNDBXeHFaNHZ3TWlabXpySzljU3JiTTlPc09uaElITUlISDhBTERBcW10ZEdvV3otMG4xZm50R1IzOEpzX05sVzVMb3VwMGNyenk0MWNIYlY3andhSWpNdWQ4d3NNTlowbGZDV0FXYTNLRHc4RjdaczdLaTJiRG8?oc=5</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2880,52 +2880,52 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K45" s="1" t="n">
-        <v>46077.58814814815</v>
+        <v>46076.67813657408</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Obernburg: Unfallflucht schnell geklärt - aschaffenburg.news</t>
+          <t>Vakantiehuis Fabiola in Maasmechelen voor kinderen met een beperking krijgt toch nog 1 jaar subsidies van Vlaanderen - VRT</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Obernburg: Escape accident quickly resolved - aschaffenburg.news</t>
+          <t>Holiday home Fabiola in Maasmechelen for children with disabilities will still receive subsidies from Flanders for 1 year - VRT</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 14:07:44 GMT</t>
+          <t>Tue, 24 Feb 2026 07:52:45 GMT</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxQWDdoMzlzRi04dVVnRzU4ZmFHbElQdTh1SFVrZWFJakZUYUVRQlk4MExVam5lb3U3XzFWVy1keWczZzJ1a3pBai1GR0E4bDRYR3JiMWY0UVVtb0ZDaFdaR3NCa1ItcjRSajg1Ny1kOFJFaFI4VWVnd0pBR1FfMndCNFV5SFFIQVgtVml3ZFUwc3kwX0hvUzRURDNwVDdkVHV3czBQVTlR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE5OenpKUkhrQ1AxTlBhUlRETGdRSFpRaVJKOW9TelBUUXdpU01tdmEwZ0VFM2dvR05IaFViZkVWM0YxLVlwU2ZETUxJbld6c3NrTm1DU1Z1SWlzZG9PNWFyZEJMSEVyX2hCY1BIa1RGaHdtQi1OQU9pR3ozdw?oc=5</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2935,52 +2935,52 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K46" s="1" t="n">
-        <v>46077.5887037037</v>
+        <v>46077.32829861111</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Blitzer in Aschaffenburg aktuell am Dienstag: Hier nimmt die Polizei am 24.02.2026 Raser ins Visier - News.de</t>
+          <t>Halen keurt aangepast meerjarenplan goed na budgetfout van 5,4 miljoen euro - VRT</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Speed ​​cameras in Aschaffenburg currently on Tuesday: Here the police are targeting speeders on February 24th, 2026 - News.de</t>
+          <t>Halen approves adjusted multi-year plan after budget error of 5.4 million euros - VRT</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 09:18:00 GMT</t>
+          <t>Tue, 24 Feb 2026 09:32:52 GMT</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxPTVBpWlNVVWhJQTJIZ0xMUkVmR2dOWmtjZkxfaDJIcDJXUHo1Z2d0T0RGOVJXdmVmRV9PQ0p1ZUg2dlVaYXhqVERySGpCM00zeGlxNnZWMjZfQzRPZzhHTFRrODVTNUlLcFRGTnpQQzJFa3pZaDNjQzRaOGpMWno3Z3ZZaEpma0xtbDVzU3I5TV9EaGVnbmpHdzlWRUxmY3NMeFg3RnhxWDRfZElOeXVDeXVXZnpaaXNwTjNWc1IyaXNTQmZMbVlZa09qVURBYTJsQmlUdDZXUEVEeDFXZHNPZE9TQmtiSmk2M3puY9IB8gFBVV95cUxOeHd5dHFsS0VxRHViWnMwbzlwYjl2VFhheTA4a0xFTjNCcWM0S0VQR1ZkRms1eVFWdzVrcUp0RFhhSkZqRE1fUmFVd3VQVVZWVkNrNHE5Y2g5U20yMlNKb0h0T0MwTVRsRkxoa1pvdU52MzFNUE9ac0FBdjRQTE5Xbko3cjNGaTkwX190N2wxUjljcGRsLTJJZEZfM2h1aHVFcTBkYUJLaExSMm9zUXQwRE5hd00wVVc4YVMyQ0ZfQWlJU3B5Y09obzh0bHFBUGpsWmw4VC1mUFd3dmVxUS14b09IRGhxeEhzLXQwV1MzdnVZZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPOTItcThiT1hZQjVXaDA5TEI5RUlVdmt5N1UzR2hEelF2aVBXemRfcTdNbk9xUk5sY2NfWkpJdmIycHN5TThoaVNnVVpCWjgzYXExeFpZUk91bVhhdFhiZ0szcDNRT3Nua3RCSTVUa1BTSGRUdU42TXJ3NzVYSXdFMTRZMkwwUVpqaURzNXJMMVIwbk1rNzNSQVdVaUVvdHRVNGNWcURCUzA?oc=5</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2990,52 +2990,52 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K47" s="1" t="n">
-        <v>46077.3875</v>
+        <v>46077.39782407408</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Corona-Zahlen im Landkreis Aschaffenburg aktuell: Die Coronavirus-News aus der Region - News.de</t>
+          <t>Booba : un procès requis contre le rappeur pour le cyberharcèlement de Magali Berdah - CNews</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Current Corona numbers in the Aschaffenburg district: The coronavirus news from the region - News.de</t>
+          <t>Booba: a trial required against the rapper for the cyberharassment of Magali Berdah - CNews</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 10:39:00 GMT</t>
+          <t>Mon, 23 Feb 2026 15:03:57 GMT</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_wFBVV95cUxQaUEzVnI1RndRNXNjVEEzZ1phUmhtempTcElXZld6R1lVQTZuYmFKQWdYN25qclF5TE54T0UzTU9iWnZSc0RydTlpMGRjZ3ZyM1hWZDh2SlBHLXJPTTN2T0d1SDJkT1RSU1FpckR2bGQ3MHlTU2MzWU1WdUVtTnRvdzN5LTJSRVJ1Q1dqMFlOS2lia1E2bWNxZ2RUMzhzS3Z3Q1ExcHlyYUxydTFkU0lIZ2hIMlZNRDZXZmlOREFzVUs2YmxrN0lOZ0FDWGxCZzIxY1djYl9RLUJGeExvOG9VZ0gyTF9WODdVdVp5LS1WOTZRNkNlQkwxZWdBZG01VmPSAYQCQVVfeXFMTUphRTNneGpNMmxrczR4aGUtLS1PT0swYXJ4T2RWOWVvZU5XNG4xckFrSm8wT2RSVUNCSG5GQlJCcm9vX1p0THJITHAtN0xldjhacjR2VXFfUWVCdXg5SjFlSEpTN2lQLVE5M1AzcjhVdEVTa3ROV0tFbmNhWlVmcXBjUUw5ZzFfZkE1amdCdFZxRkd2c2x3dk1DbXRYR1FBWW9sY1g5ZjhPNXE5WXF0U204Z3RHWlVGVDlKdG1YeVAtYXB6ZGhoZ3pXMEp0cTNyS0o2dXhGRDFDV2JCYWlWbDFfXzZVVmJ1RjRKV09aZzNqZ3pETERxU2cxUUhYM0dNZ0xlSV8?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPOFUyODdiVzRYWEh6cWZKWlY2M2UxQjZJcy1PSEJ5TDNDQ1dhVDVfSjUyOWcxQlNsaEF4Z3NVZDJTc2J5eEpCZ0hyZjFYYTY1a1RKbWtTUTdFellXWndJOTZZckROSzNsekdYM2k3VzBJc3htS0t6djc3S185RUJSZl9fanMtNVVDWXlQb2RkbjRZQy1tbDJhQ2Jxcm1RbE92UFRONDlOZmlDRTRES014NjB3SVZtSkM1U1FQTXp4R0F2UdIBwgFBVV95cUxPOFUyODdiVzRYWEh6cWZKWlY2M2UxQjZJcy1PSEJ5TDNDQ1dhVDVfSjUyOWcxQlNsaEF4Z3NVZDJTc2J5eEpCZ0hyZjFYYTY1a1RKbWtTUTdFellXWndJOTZZckROSzNsekdYM2k3VzBJc3htS0t6djc3S185RUJSZl9fanMtNVVDWXlQb2RkbjRZQy1tbDJhQ2Jxcm1RbE92UFRONDlOZmlDRTRES014NjB3SVZtSkM1U1FQTXp4R0F2UQ?oc=5</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3045,52 +3045,52 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K48" s="1" t="n">
-        <v>46077.44375</v>
+        <v>46076.62774305556</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Village Wertheim (fallback)</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Jon Wertheim suggests the reason why Serena Williams might be planning a WTA Tour return - Yahoo Sports</t>
+          <t>Courtois va investir en Belgique : deux clubs mentionnés - FootNews.BE</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Jon Wertheim suggests the reason why Serena Williams might be planning a WTA Tour return - Yahoo Sports</t>
+          <t>Courtois will invest in Belgium: two clubs mentioned - FootNews.BE</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 13:17:11 GMT</t>
+          <t>Tue, 24 Feb 2026 12:39:21 GMT</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxOYl8yTkRYaUVVaUU4eE4wZk1aSTVxbkNEVzg5MHF5aTI1bGZnZkxweHgzM3MwUU9BekdUVVNlV3pPV0J4NkJuM0ptYzlsa1JxNUNCZjNqdmdldHkzRnNMSnpidGhTb2h3LUYwR3VXU3BnX1Z4ZDY0dkJRd3JiMUpYT0FZbjVyNzJf?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxNTlJDdTgzUm84dnhidVNwNUtTZGJqbWZZOVJmSHBzU1QyYmk4QV9ZanJ5TG12cXFKVDhVSHplR2dudWVsb3RlWjZUd0FpVmhHZFJfQzFnTlpvMnJwX2Y1Q3RLY1lzTlNWQ0JNSXAyalBMNm9YazVTenlGUXdranlMbjlwWUpSSlppbjF6SXU1aGJJd185?oc=5</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -3100,52 +3100,52 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K49" s="1" t="n">
-        <v>46077.55359953704</v>
+        <v>46077.52732638889</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Sexueller Übergriff am Bahnhof: Kripo Ingolstadt sucht Zeugen - Augsburger Allgemeine</t>
+          <t>Official | Ousmane Dembélé and Fabián Ruiz out of PSG’s Champions League return leg - Get French Football News</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Sexual assault at the train station: Ingolstadt police are looking for witnesses - Augsburger Allgemeine</t>
+          <t>Official | Ousmane Dembélé and Fabián Ruiz out of PSG’s Champions League return leg - Get French Football News</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 14:34:12 GMT</t>
+          <t>Tue, 24 Feb 2026 13:32:37 GMT</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxOYVpQc2ZubWFubEFJeVhURXhHUWlPa24td1QzXzVWS0dmdEJCN0VVRGNfNjEyZjNuTEZyN3IwWWo0cFQ0SjRYQUs2VXBJWGUwMXY2ZG9wc2V3UmM2WW5ZaUZkVTNWXy1mcVpNcXd2NE5SRklKSDh3aklIcUMwWDJnSGxyNms4N2ZETzg5QTQxZzd6Q1dJQ1B3akVZMkR6UElYenU3clBPOXRLaTNmTGVxYjdLU0NsQmY1ZXJEcVBSWmVlZGpmZS1BeFBqeUFZQXdJaWZKRHBKbw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxNRHZ4dm0tREV0cjFucHowcUNrWGlJTVljdlFXcjNtdFg0OUh4a2hWb25ucnlzMkNMdThqU25BNm1yaHhBRk8zTDRwcHdHRHZFRUNBSVlHcXZjdDJFQU95SEVCM20wQm1YNmFzczRjdzE5UmZUY2NpWldzMWRfdXpSVmo4ZlpsVHdNOWo1aVFGcVRBc0I5RjVyYkRGeXZmVTBGZkFvNy0xZFVxa2JNZ0RzeGt2dHJCZTZHUTU1RXRZbzNpQQ?oc=5</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3155,52 +3155,52 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K50" s="1" t="n">
-        <v>46077.60708333334</v>
+        <v>46077.56431712963</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Schwerer Auffahrunfall am Brückenkopf Ingolstadt: Beifahrer eingeklemmt und schwer verletzt - RegionalReporter</t>
+          <t>LolaLiza acquired by three board members following management buyout - fashionunited.uk</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Serious rear-end collision at the Ingolstadt bridgehead: passenger trapped and seriously injured - RegionalReporter</t>
+          <t>LolaLiza acquired by three board members following management buyout - fashionunited.uk</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 07:57:13 GMT</t>
+          <t>Tue, 24 Feb 2026 14:08:23 GMT</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxNb2w4ekV5aHlhNHcwSEJKaUlBN2hpd0ZVUW56eHFPTXlFMGVLYjkyMVRPT0hUTjllLUdONnY1bExmUUJnSk9SR1lmQTBjZV9oV1JHNWQwV0RnTXB2Q3ZPdFR1di1IZjBETzFJd2FTY05aYmE5LWpsdC1nSGI4X05ENkMyelJvazdFeVFJSkN2SUZWSUZLWm9fSk1NRXFjOFhhV3I5cXRLZmJJNkFyRDVSS3Z5Q1ByMVFpV0V4VHVKVXUzalJIQ2pHSkl4WU1YZU5xbjdYbldYYlJHV3R2Z2JtSDYyazE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPNExOajRSMzJtQk9kOENCeXlHM25OUm5vVWQyUkszamgzQjVOMm92anAtdHN2QXhFLUVMLUptNVJ0YzV5dFJWTE5OeVNCMFVobnlyelUzeFBadlNFV3hCRVI0Y3pUTExVYU9TNFdwVUNsaXhyQjc2QW5MZlh3Rk9rejhZUDhEU1h3LUVQWHhBWHNHWG80NUltV2hxd1YwWmhRVVZyOHotOUdQeEp6UlVQYi1iVDZWcHFOanBzWWFB?oc=5</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3210,52 +3210,52 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K51" s="1" t="n">
-        <v>46077.33140046296</v>
+        <v>46077.5891550926</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Village Las Rozas La Roca</t>
+          <t>Village Maasmechelen (fallback)</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>("Las Rozas outlet" OR "La Roca outlet" OR "Las Rozas Village" OR "La Roca Village")</t>
+          <t>("Maasmechelen Village" OR "Maasmechelen") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Movie-style robbery in Catalonia: in just a few minutes, 120 e-bikes worth over 300,000 euros are stolen - Brujulabike.com</t>
+          <t>IKKS declared bankrupt in Belgium: dozens of jobs at risk - fashionunited.uk</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Movie-style robbery in Catalonia: in just a few minutes, 120 e-bikes worth over 300,000 euros are stolen - Brujulabike.com</t>
+          <t>IKKS declared bankrupt in Belgium: dozens of jobs at risk - fashionunited.uk</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 09:21:06 GMT</t>
+          <t>Tue, 24 Feb 2026 13:03:27 GMT</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPd0dBclgxSVlFV1dtaEgzNklSZENrcDBPVF9kbEZOWUZhMGtfS3BsS01WWlpwMERQMHVtUUcxaG1EaFlyV3NONy05ZlQ1TzRPTG9lVDUtZE5xVVZEbUdBTFdkNlB5TEhTb0FmSWJlOFpqTXVVLWhvd1JaYzkzNGNMaVBmaGpSaWZ0dHJ1cnBXQndERXZMN2ZhSWJSNlFPNHQ5MFMwbUF1WHRIXzBXOUxpQmtYdWgyNlpDaVhEdjcwYXBGLUtQNzQwdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOUW54aFlQc196RnJXM0FfVWU5a2JSN2w2MXdiZVg0Z2U2aXdKZENsNThtVWVvQjg3U0FwUUQ2Qk5SZF9rSnVqQWxrc1VzOUNzcVRfbWVXNWFCUW80ckl3MHJlaTZvUElidlBqZWNlSm85a1otTXNBMkpYTlQ1YzJBcDVNNkY1a2o2OUJtNG1HYnItU2RodXRXb1pXMVFOTkF6ejk3cEY4ZTdRbTA?oc=5</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -3279,61 +3279,1161 @@
         </is>
       </c>
       <c r="K52" s="1" t="n">
-        <v>46077.38965277778</v>
+        <v>46077.5440625</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Wertheim Village: Polizei stoppt mutmaßlichen Seriendieb - Fränkische Nachrichten</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Wertheim Village: Police stop suspected serial thief - Fränkische Nachrichten</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 09:34:00 GMT</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxNempGdjdfTkxudlBkZnlNYlNUS3h0MEluS3JYU2tOVW9zamM4QUdCODMyNTAwc0ZDY0NCYXpReG9wOTVtOUY2eW9rWmhxT0RHaUdubGNoWVN3SjBCaE8tSlBpSTlneF9aQnNMdHR0VDI3Wjk4el80OU91akJGYWV4aVVuM01SejN5NC1rQlg0WElRd2VJbXVhZEtjZEVwdDAtYlZnSFFjazhjOExOcGszYmt1X0hEUlZyQjl3aTRWXzZxWHJ1NXlJ?oc=5</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K53" s="1" t="n">
+        <v>46077.39861111111</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Reichenberg: Frontalzusammenstoß auf der B19 bei Würzburg: Zwei Autofahrerinnen schwer verletzt - Main-Post</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Reichenberg: Head-on collision on the B19 near Würzburg: Two drivers seriously injured - Main-Post</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Mon, 23 Feb 2026 20:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxON0VPNERZb21RaF8xWTQtUzVObjNuUUw5LXpNbEVyOGtLQ3I2eWc2STlOUEd2OTU3UUVMNlVhNlRvTGFSQmxvb181ZkxJNzFtQXI5NGoxZHJPZ0gtbUVBd0l6Wm96UjREZ3JnV3dfNjYyQklGWVlSUTVLRjZrRE5mU3E5dVFaNU5WdE0yblAxWHIzR1hJdU1JVFEyZnEyMFVneGhHTl9UVF8zYnZPTVM2bTQtT3l1RUg4WFc2WHhVekMxVTZCRmo4eXA5THhKRzRibTE1UkpFaGJqYW1qaXhZZ3VJcFpVYUVrNGh6Qkc2NDQyS19FMFItR2E4V3k?oc=5</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K54" s="1" t="n">
+        <v>46076.83333333334</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Streit bei Auto-Kauf in Aschaffenburg: Männer gehen aufeinander los | Foto: Karl-Josef Hildenbrand/dpa - main-echo.de</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Dispute when buying a car in Aschaffenburg: Men attack each other | Photo: Karl-Josef Hildenbrand/dpa - main-echo.de</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 12:34:53 GMT</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxQNXA4Vkl0TlZ2Ui1SOTgxNWVUcF8xdXdtOUJsODFOalIybVlxTkU3SURZVHc5aTFsdHNHMGR1SXNvNWZGdlgyT0dzbHZmbmtQMklfbERteC1yMWw4WFVvUzhGSWQyb1J6X3hPcmRBVkFfVkxMbEtkWDMtbGZWckV4LTZVLXBvUUk5ZEFNMlJ3SE80TXZ0V2JEakttUjJkWmtoX3djX01wY2dUbDhoLXQtRm1qVXpwZzlfM2UxWXRTYng?oc=5</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K55" s="1" t="n">
+        <v>46077.52422453704</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Herrmann begrüßt deutliches Personalplus für die Bayerische Polizei - aschaffenburg.news</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Herrmann welcomes a significant increase in personnel for the Bavarian Police - aschaffenburg.news</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 11:06:28 GMT</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxNU0FPOVFwS1pZal9xUnlUNDVjT0wzY2xwRG5TUmdob3JERkNFdld6ZHdVTHJBdnAxOGl6VW5jeTNxMmxtWjZfSVdkczVTaVdTNFBIaEN0VzBTbUkzRHk0QlBJSEU0bEk0aVJIT0lsdnV6VE91WUZDMGRybGhMSmVMWEM1R2hId1pvN3E2Z3BOT2xYZk5vMm03Vjk3dHNfV3ZhS05OM3RqX3J0b25uUTRadzZLaDJXWk5KbzdmLTZ0OA?oc=5</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K56" s="1" t="n">
+        <v>46077.46282407407</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 05:25:22 GMT</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE03RUZJdVVWTG5jTlA1R0dmc2YyQ3Z2S1ExYmhkN0FENFJGamUwenJsSFFPWGpKc3B2aFBaeHRYVDR3aWM1SXg0YWZFVDk0N3d4a0Jz?oc=5</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K57" s="1" t="n">
+        <v>46077.22594907408</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Unfallfluchten in Aschaffenburg und Kleinostheim | Foto: Dirk Ceelen - main-echo.de</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Accident escapes in Aschaffenburg and Kleinostheim | Photo: Dirk Ceelen - main-echo.de</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 13:03:01 GMT</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxQMW02WVZqN19mTERhVXdiT194SUtPU2ZxVTJ3dGNKd2ZLQzVmM2lxb3lTdWpHVjBqOVlFTFVOYXE0d0czbUpZQzFFU19OT294MmdqVlU3d2M1QzFWUndPbm02SVBvakFlc0tVSnl6YXJjOUNaN2FvNUYwX1pOOGJ3aVJoZjlPOU9DWnFRZlBlZG5uNXN4N3ZvWnpYN21VX2M1Skppd2c4Zw?oc=5</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K58" s="1" t="n">
+        <v>46077.54376157407</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Marktheidenfeld: Polizei kontrolliert erfolgreich - aschaffenburg.news</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Marktheidenfeld: Police check successfully - aschaffenburg.news</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 14:09:08 GMT</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxNM0F0V01ZMjFGbzFpQ0FldUNxRnI4UkplZ2daMUlzTXNvWGM2WnlUZGprenhxMXBfSkRrLTFkWUU2c2VFODdxRTU1bWF2bVNZeW9zWWVPaEtGU0ZfdUdGbVBKOGt3dEdmaUszMTdlZnFuNUV6b0JWUEFtVjBlTmdFQXh5SXhuZTN2eVVzelU2Z29RUU9wNGw2Z1Vn?oc=5</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K59" s="1" t="n">
+        <v>46077.58967592593</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Blitzer in Aschaffenburg aktuell am Dienstag: Hier nimmt die Polizei am 24.02.2026 Raser ins Visier - News.de</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Speed ​​cameras in Aschaffenburg currently on Tuesday: Here the police are targeting speeders on February 24th, 2026 - News.de</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 09:18:00 GMT</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxPTVBpWlNVVWhJQTJIZ0xMUkVmR2dOWmtjZkxfaDJIcDJXUHo1Z2d0T0RGOVJXdmVmRV9PQ0p1ZUg2dlVaYXhqVERySGpCM00zeGlxNnZWMjZfQzRPZzhHTFRrODVTNUlLcFRGTnpQQzJFa3pZaDNjQzRaOGpMWno3Z3ZZaEpma0xtbDVzU3I5TV9EaGVnbmpHdzlWRUxmY3NMeFg3RnhxWDRfZElOeXVDeXVXZnpaaXNwTjNWc1IyaXNTQmZMbVlZa09qVURBYTJsQmlUdDZXUEVEeDFXZHNPZE9TQmtiSmk2M3puY9IB8gFBVV95cUxOeHd5dHFsS0VxRHViWnMwbzlwYjl2VFhheTA4a0xFTjNCcWM0S0VQR1ZkRms1eVFWdzVrcUp0RFhhSkZqRE1fUmFVd3VQVVZWVkNrNHE5Y2g5U20yMlNKb0h0T0MwTVRsRkxoa1pvdU52MzFNUE9ac0FBdjRQTE5Xbko3cjNGaTkwX190N2wxUjljcGRsLTJJZEZfM2h1aHVFcTBkYUJLaExSMm9zUXQwRE5hd00wVVc4YVMyQ0ZfQWlJU3B5Y09obzh0bHFBUGpsWmw4VC1mUFd3dmVxUS14b09IRGhxeEhzLXQwV1MzdnVZZw?oc=5</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K60" s="1" t="n">
+        <v>46077.3875</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Demo-Termine heute, 24.02.2026: Hier gibt's am Dienstag Demos gegen AfD, Menschenhass und Rechtsruck - News.de</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Demo dates today, February 24th, 2026: Here on Tuesday there will be demos against AfD, misanthropy and the shift to the right - News.de</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 06:04:00 GMT</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihwJBVV95cUxPTGdUUkg2a1JYTDFRNDFrZTJfejZYeTZZc1dOeC1sYkNIOVQ4eXFXU2t2X1BXaTJsaHlsSmJXcUM1MWlpVmdXZXpBZ3ZiOUpPd2NhOG1OSUNfZWRhR1o0dEVWX2hZT0pCVk1WMmV6T1BmaFI3V0lEYjdrTUlPMUZvM1hMdHd1UWdnak13VFlMa1FydXF0cUZWd2ZTRjJWaTBCNmMyelAtdlI1Z3kyNndzZ0NSRjNkeTYwZWludW9WNVVPWThLbWw2ZXRpU2ZMdUxXcTZZOUllbG42OGp1dDBpbXlWeGE2X0xOakFnYnpxbXoyWE1HVks5bDZoVUs2QTMzbXpTWVh4a9IBjAJBVV95cUxNVlA5c1FOUjBhdmxMUWhDQk8xbDhPTFlENjAtM0hCS2pmX0M1VUZxcC1WblZQTWdhRjlhT2NWbUZWSG5NZWpLby1sYlJMTnA0X2JFeWNNcVFvNHpqQlJBcmY2VHc1QTYtc2xnTEVFRlFGTXRnZDFRNktpTFFVTG1vRmhtSGtvdTRDX0ktZm9QanY3SzBLTFo3enRWc3hSODJIejdMcGFqdGVpU3owaF92NmdKNkd4ek9OMFlfcE5pNldoNExVOGU5VjIxUDB3alBORWFRM0pRWXJVT0JlSkR3TmJOaTZhOWxQUncybTNxZGFpN2NGRWdCU0N5dE81blBrSUxjbld6cHBRc25X?oc=5</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K61" s="1" t="n">
+        <v>46077.25277777778</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Village Wertheim (fallback)</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Jon Wertheim suggests the reason why Serena Williams may return to the WTA Tour - Tennishead</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Jon Wertheim suggests the reason why Serena Williams may return to the WTA Tour - Tennishead</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Mon, 23 Feb 2026 22:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNdXRXQ1JpcjVLX3Vkd3RzbW5VMWR1SW1qQ1hwc0RfUi0xZG5nQktYRXhYcEstZ3BSb1pMVU8yeklCS3dycGdhMW14WVZKVUdyOUtjN2YwMllOQ3JxOGo0VVhCX1VCM3AyLUFQVHMwZzZDbXNKb0prSkJITVlJbm1ka0ZDY2g5X3hJQ2llel9EM01mdjRaYklTazA5dHA0WGU0LUdmeHVn?oc=5</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K62" s="1" t="n">
+        <v>46076.91666666666</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Unter Vorwand ins Haus gelassen: Täter stiehlt Geldbörse einer Seniorin - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Let into the house under pretext: perpetrator steals wallet from senior citizen - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 06:42:59 GMT</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxOUzZOZmpZeWJ4MGZ6Z003ZG5oYVIwZDhtN2k1VU9BM2FSLTgxWXlxcDc3eXBBOUxVY2h4SzVXU29tRXpxZzBZZW9mNFhGbXg1TWVRWUIyQzgzaGZac2N5c28wZ0pyV2hUWEhfblk2cUpGMFZmNDV2QTk3a0JZNXZfTFRqTUppSU1rSVRQa2NvSTlTX3ZEdE56U29HWTdSUmM1QXAyS2JGNkZzZ0llNm8xY1hLNWN5MXVsRHhLV1J5bGhmN3pRczRQZ3BLZXBSbVFETkZ3UkUzRURrNk0?oc=5</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K63" s="1" t="n">
+        <v>46077.27984953704</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Polizei stoppt 66-jährige Autofahrerin mit 1,6 Promille - RegionalReporter</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Police stop 66-year-old driver with 1.6 per mille - RegionalReporter</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 03:38:40 GMT</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNZ01KNnczSFRPLTlLZUNzb1pXWTBqbGR0LWxFTXR0ZHZWb1pza0ctYmFSd3VmRUhLcjdsVXZDS1d5NUsteUN3b01FSW9lZ213MndZMWxnUDlFTkVYcnJZQjg2Mkg2WmdOSGpSUmZNeERVd3pHUlhwMjJva0JQWlNfS1lFREcyVmZfbzMzMkprZ3dlRWVWbzRKd3ZQLWhVS0FrMFVDUnRMMXRNdDN6NDhRbFhndzE3Zw?oc=5</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K64" s="1" t="n">
+        <v>46077.15185185185</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Schwerer Auffahrunfall am Brückenkopf Ingolstadt: Beifahrer eingeklemmt und schwer verletzt - RegionalReporter</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Serious rear-end collision at the Ingolstadt bridgehead: passenger trapped and seriously injured - RegionalReporter</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 07:57:13 GMT</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxNb2w4ekV5aHlhNHcwSEJKaUlBN2hpd0ZVUW56eHFPTXlFMGVLYjkyMVRPT0hUTjllLUdONnY1bExmUUJnSk9SR1lmQTBjZV9oV1JHNWQwV0RnTXB2Q3ZPdFR1di1IZjBETzFJd2FTY05aYmE5LWpsdC1nSGI4X05ENkMyelJvazdFeVFJSkN2SUZWSUZLWm9fSk1NRXFjOFhhV3I5cXRLZmJJNkFyRDVSS3Z5Q1ByMVFpV0V4VHVKVXUzalJIQ2pHSkl4WU1YZU5xbjdYbldYYlJHV3R2Z2JtSDYyazE?oc=5</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K65" s="1" t="n">
+        <v>46077.33140046296</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Sexueller Übergriff am Bahnhof: Kripo Ingolstadt sucht Zeugen - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Sexual assault at the train station: Ingolstadt police are looking for witnesses - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 14:34:12 GMT</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxOYVpQc2ZubWFubEFJeVhURXhHUWlPa24td1QzXzVWS0dmdEJCN0VVRGNfNjEyZjNuTEZyN3IwWWo0cFQ0SjRYQUs2VXBJWGUwMXY2ZG9wc2V3UmM2WW5ZaUZkVTNWXy1mcVpNcXd2NE5SRklKSDh3aklIcUMwWDJnSGxyNms4N2ZETzg5QTQxZzd6Q1dJQ1B3akVZMkR6UElYenU3clBPOXRLaTNmTGVxYjdLU0NsQmY1ZXJEcVBSWmVlZGpmZS1BeFBqeUFZQXdJaWZKRHBKbw?oc=5</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K66" s="1" t="n">
+        <v>46077.60708333334</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Alin Coen live in Regensburg: „Du bedeutest mir die Welt“ – Ein Konzert voller Emotionen - RegionalReporter</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Alin Coen live in Regensburg: “You mean the world to me” – A concert full of emotions - RegionalReporter</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 03:47:07 GMT</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxNaGZyR041TjVBbXZOa0NudVppUlh4Zm1Gc1BFNmwzRmFaZjNvMExzaHBoMmh4Y1plTUk5QW1VM0lWTHNSMmN0NmJsZmlkbHpZa0dxdGhzMzNvYnhlOU1BRnlOeHdUclJKLWNjaUhHMWNFWFFxMDBjYlJWcUtidGJKQVNLOFNia1laaWVXbjR1N3JkUlQyS2dLTGZ5Uk56SThmQXFRMzYwaTVYam9wdnUxZndURUxSSEx2cDl3S1RDVGhub1dob2pxeWx0TTltXzN2bWpFVWR3?oc=5</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K67" s="1" t="n">
+        <v>46077.15771990741</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Beifahrerin lebensgefährlich verletzt: Stundenlanger Stau auf A9 nach Unfall mit Lastwagen - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Passenger critically injured: hours-long traffic jam on the A9 after an accident with a truck - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 05:08:22 GMT</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQRXl1MWhlRzRsY0RRYVZPdTBPWG9FLW9TdGl2QmdMenY2b3EyeFNGZGdZMVNoajRVc3FWeTBUeEZqanVrOEpmUTF1SDdtblFVYXRhOG5RYTcteGZqRnBLUVJ4ZTgxU2hIZ2x4dGxfaFRYN3ZIYVplS3A4VjBHVnBrU1AyRGhtNV95VDVkREo1LTJYSThBUHRJTS0weENUekpNaU9ySUlUY1g2YnJVa2E3RnZhRnV6OHQ2VnNJT2VpZ2M2SklKdmZN?oc=5</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K68" s="1" t="n">
+        <v>46077.21414351852</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>SPD Frauen Ingolstadt fordern gerechte Gesundheitsversorgung für Frauen - RegionalReporter</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>SPD women in Ingolstadt demand fair health care for women - RegionalReporter</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 04:53:13 GMT</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxQWTVvZndQRWxzYWswTXQtRHNrV01FQUwwRlRsQXlqS1h4V3NPZVNsRlMyelVnd2FPV3dJSHY0UGk4cExDb0FIYkV0aGhRX184WUxRLTdpRFB5dXR2WUQxYm00RlNiU09lN050cFptMU5MRDRXSXg1cXNqZnNpUGNsOVUyazhqQTJZQmEzckI3Qy1KbWVKSzYwa2tSWVhjM0hLR0pFSktqOS1kazFDSXNXd2lWaF9BaEtBZ0Y5ZUdnVXhXUE0?oc=5</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K69" s="1" t="n">
+        <v>46077.20362268519</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Solidarischer Hochwasserschutz: Regionale Allianz setzt auf dezentrale Maßnahmen und Echtzeit-Frühwarnsystem - RegionalReporter</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Solidarity flood protection: Regional alliance relies on decentralized measures and real-time early warning system - RegionalReporter</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 05:04:48 GMT</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxQbGI4VVlKYUJfeGhaTGpqVXg3ZDZqTzBnUXBqUngwQ1l2dkxFakRZN2QwTm9HTDVORC03bnpaNGVaV2FBWlNXS2VBY0dqNlRmdXpiNGVKdGR6aGxUSkJwelhkMUdTU0lUVktmSTNmcVI0NHBBbGpXZUowZnpRT2hKWHJlSFhKa1VJYVMxTkZ2VjRBVTR0dUFKVnlqNF9rdllKYndwRW5hdUNGUVZfVDhMb3BUNFJqcFQxZVhueXJVT2dZUm1iU1Z6VUNoV3MwUkhsd3BZVi1oZEdpZXlHR1NvYVppckZrLU5IZEp4SEdHWjVvcEFMODg0?oc=5</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K70" s="1" t="n">
+        <v>46077.21166666667</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Village Ingolstadt (fallback)</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Important note: Municipal construction work restricts access to the parking lot - EHC Red Bull München</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Important note: Municipal construction work restricts access to the parking lot - EHC Red Bull München</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Mon, 23 Feb 2026 16:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNdUdtZFdTODlzV1RXU2NEWGRNeGwtWjRtODUtYWI3bkZfRXVNVjhNWTBhWnNYcGVmZUtYdHJsOWYtX0NRV0xteEwxTFlJU3J4VVUxREFmaDB3dTVTaTRjdG5YM2t6VE5yZUFKRV90MnN4WURuRERQeW9CYzZaZlZhS0lOS2lHTUZvZml2RzVIc0dmdFVHemlTVjJLcV9pTjk5RkxUYnF4UFNoNlptU2c?oc=5</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K71" s="1" t="n">
+        <v>46076.66666666666</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Village Las Rozas La Roca</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>("Las Rozas outlet" OR "La Roca outlet" OR "Las Rozas Village" OR "La Roca Village")</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Movie-style robbery in Catalonia: in just a few minutes, 120 e-bikes worth over 300,000 euros are stolen - Brujulabike.com</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Movie-style robbery in Catalonia: in just a few minutes, 120 e-bikes worth over 300,000 euros are stolen - Brujulabike.com</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 09:21:06 GMT</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPd0dBclgxSVlFV1dtaEgzNklSZENrcDBPVF9kbEZOWUZhMGtfS3BsS01WWlpwMERQMHVtUUcxaG1EaFlyV3NONy05ZlQ1TzRPTG9lVDUtZE5xVVZEbUdBTFdkNlB5TEhTb0FmSWJlOFpqTXVVLWhvd1JaYzkzNGNMaVBmaGpSaWZ0dHJ1cnBXQndERXZMN2ZhSWJSNlFPNHQ5MFMwbUF1WHRIXzBXOUxpQmtYdWgyNlpDaVhEdjcwYXBGLUtQNzQwdw?oc=5</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K72" s="1" t="n">
+        <v>46077.38965277778</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
           <t>High Level City Italy Italian</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B73" t="inlineStr">
         <is>
           <t>("Milano" OR "Bologna") AND ("minaccia bomba" OR "pacco sospetto" OR "pacco esplosivo" OR sparatoria OR accoltellamento OR "attentato" OR "operazione di polizia" OR esplosione OR evacuazione) AND -Olimpiadi AND -pattinaggio AND -sci AND -Cortina AND -calcio AND -Serie AND -mercato</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C73" t="inlineStr">
         <is>
           <t>Zola Predosa (Bologna), sparatoria al campo nomadi: «Un pregiudicato colpito alle gambe» - Corriere di Bologna</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D73" t="inlineStr">
         <is>
           <t>Zola Predosa (Bologna), shooting at the nomad camp: «A criminal hit in the legs» - Corriere di Bologna</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="E73" t="inlineStr">
         <is>
           <t>Tue, 24 Feb 2026 08:41:43 GMT</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="F73" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxPTXZ3cFF6NURKMDl5cGZSWFJWQ2ZRWk95Z2ItemVwYmlVd1BhMm9LX2Z5YmJiOFp5b2lNVE00TVdpWUlnb2VLd3B2VnJnckU1R096NU5nTFM0dmFlU2o1WUlWakN2dkttY2Z3YlZ6akF5TnhZb3g5QkV2ZXRXSnRvR0IxZ1dRMjMxWmVaNUNTcXJIaUVYVXp5eXdwdUN6ek54Z2o2dVdybmwzUC1MS1pBMjQ1d1g5UWZFSXQtMi1MeXhleU9LWlBMeV9HaUhDczQ1bmRIMVVxaHZKR3hsWWZ0c05rUTZ5ZXFpWFdV0gHwAUFVX3lxTFBIZXFtcm93OHQ3bmZIcTdUcXV1VmN1Tm56S0dld3pCVDEtS2ZYdVB1bHYwNzBqUjhyc3ZhSUM0S3p6b09JQmtiOWI3ZmlfOUs5OWxMci0tX2NFckV2V0VKQ3Uxam1rWWtEa1dpdWdZcHA1T0JVLTVneS16d05NVmxJVjBOMDdDcHJaUW5lYS1JamdtcGFlMHhneTJkTE4zeWZtbXhNZWRtWUZQbHpIR09sNWxGZ3ktLVVVSVZlWG55eXYzX3BQV0M0MkppUVlNWU1PU3czUnRMTUNRVkVzWUlyYWhPZGs2MUFULTU2RnNFcw?oc=5</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
         <is>
           <t>it</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr">
+      <c r="I73" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr">
+      <c r="J73" t="inlineStr">
         <is>
           <t>IT:it</t>
         </is>
       </c>
-      <c r="K53" s="1" t="n">
+      <c r="K73" s="1" t="n">
         <v>46077.36230324074</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-02-26 14:47 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K56"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,32 +480,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Value Retail Brand</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>B&amp;M European Value Retail S A : Prospectus - Migration - marketscreener.com</t>
+          <t>Uitbaatster van bekend Antwerps café Kiebooms klaagt drugsoverlast aan: "Dealen en gebruiken gebeurt open en bloot" - VRT</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>B&amp;M European Value Retail S A : Prospectus - Migration - marketscreener.com</t>
+          <t>Owner of the well-known Antwerp café Kiebooms complains about drug nuisance: "Dealing and using happens openly" - VRT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 11:51:05 GMT</t>
+          <t>Thu, 26 Feb 2026 14:08:20 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxORnRLQnN2cTNWWW1pT0RGT01Hc3ZCRXNxZmdWZzZaaVZVMDdpYzRpQnB0ZDNNbWVsdEFxSnhYSGk1RC1YNkNwWVRSc1Y1cUZUcUpuNVhMQ3lpQUdwTUlRT1o5d1pfZVdQSE5aRlZNMHZER0hrOWRQS25MYkQ2T1JyQUVOYnZ3OFZqM1BiTGJYaklNTXFRNGtGMG1nalJkOWxTU0lLdndn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNbjR1dnVXUzQxV292QzN3LTZNTWZpM1E1LWhoX3VmNmlZQk1OSTlIaUhwNFM5MEJzcnA3U0xPd1NwSGVHSXVGb3Y0RFJZVU5jd1V6ZjhvTUttTjJKY2hBRzkyR3l2UFJWeDhGNHR2enFvMVNfMzhXdFJNMDktRXA1b1hSU1dDdzViTEthMmtMeThENE1HZjIxbzN5RQ?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -515,52 +515,52 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46078.49380787037</v>
+        <v>46079.58912037037</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Value Retail Brand</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>B&amp;M European Value Retail (LON:BME) Share Price Crosses Above 50-Day Moving Average - Should You Sell? - MarketBeat</t>
+          <t>Schoten gelost in Brusselse Matongewijk: één gewonde - HLN</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>B&amp;M European Value Retail (LON:BME) Share Price Crosses Above 50-Day Moving Average - Should You Sell? - MarketBeat</t>
+          <t>Shots fired in Brussels' Matonge district: one injured - HLN</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 11:18:55 GMT</t>
+          <t>Thu, 26 Feb 2026 12:45:26 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxQcHFXTEZaaGNtSW1ibVVBT0NDaGpEZUxpOTU3d09xRElNX29wbEJBaU1Jc05NUUZobWg0REtXY3d6MU9Xci1sU0JNRVRzQUg2dnYxVFpiSy1DNGxUV2FBRmh1T3JhdWN5bnJxc2dySEppY2lmUnpZZHV2TVBTWjRMcUVrMUxWUzBaaDZmMjhPaWxSa0l1UFJHczFOaHJ2dk9rdzMzVGJacFpURkVfSjEtNzNwekhJOUJ2LWd5d2pHSll4RDU5c2N0UGcxdm5WWkZlWkc1LTB0bzFjdWVxbmYwb1dqWQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOTzdTWXEyQUpvR2otOTlmaHgxMDNPRGNuMWpPZlNrVU5iZ1dRM0JCbmZmM09EYXhVTk5jRzl1T1RtN3lPbEthUzh5djFEYS1PRFZuekJKQ0pWZWRtLTlTd0UtSUoxcDgwTmJFMUZFVl9HNV9ic3Foelh5Xy1XWmdSV3phMHczblQ0eEd4ZWhSRVJtdw?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -570,52 +570,52 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46078.47146990741</v>
+        <v>46079.53155092592</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Value Retail Brand</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>B&amp;M Publishes Prospectus Ahead of Jersey Migration and London Listing Move - TipRanks</t>
+          <t>Persoon gewond na schietpartij in Matongewijk - BRUZZ</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>B&amp;M Publishes Prospectus Ahead of Jersey Migration and London Listing Move - TipRanks</t>
+          <t>Person injured after shooting in Matongewijk - BRUZZ</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 11:37:09 GMT</t>
+          <t>Thu, 26 Feb 2026 09:21:26 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPNElkenJwY0R3U1AyNnpVeU1VclhkejRWUFhEOVlPUXY1VTJ3azBhRVI5eVc1T3ZQRG5vN1hMMy05MUJPQUkzRGdreUNVWmd4VnBPYVRScTFoSkFvUGVjMWExZjg2bDZXWms0a1Q2anpjWTNSZC1nTXU3WDJwbDJVMW5BVmhvRk9kYXo4WXoyVHVmTHJiSE8zM0ZZT2t3QVAtY09KOUpxUEpReFR5NVU1SGZiQ2p6SkJ4a1pzMUtqVFVPcTg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxQdTk5YW5kRE9iSXBpLVJrWnpfMGFNRkQtTGxIem1Dek93VlcwN25fUkhXaHIwRmJyaXVwTE10Ml9KdC1iN0FodE5XLTdjbHpNYmxYZHF0bkNVZzB6TWRKck50bWV2U2V6RzMwSF9TY1Rrb0FjTnU2TTJpYWNlSTRIV2dGaGVRQlN5bzdmMXN1NTh3WXoxRXZsQ2R3bmtJX3R6d1J5d3R2WQ?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -625,52 +625,52 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46078.48413194445</v>
+        <v>46079.38988425926</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Cotswolds described as the Hamptons of London: top hotels, restaurants and shops - artthreat.net</t>
+          <t>Gewonde bij schietpartij in winkelgalerij in Matongewijk - Nieuwsblad</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Cotswolds described as the Hamptons of London: top hotels, restaurants and shops - artthreat.net</t>
+          <t>Injured in shooting in shopping arcade in Matongewijk - Nieuwsblad</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 23:29:44 GMT</t>
+          <t>Thu, 26 Feb 2026 10:14:13 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxQVzJVSmc0ZVMxQ0NnU1lBREZSRjIydFo0VzVjdDNqTGFOWmhIZ0pPakEyX081b3dVcUF4bHBHZ3lkQnk3Y1dZcnNQNEh1NXZ1V3ZmaWYtd0Jua0V4aGhuYTU3MGtjY1FpVGlRYW1GMnY3YXZzMmtYdFZjMlZPQklrOURZWDMzWmlxQmFrT1hIRTVzMVZiaGpqTjhJTWczYUVYaUlZVmxpSDJVdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPLTNMd2RpdjJKWC02d2dwZDZsM21qb2VDTjBPeUszdElIQlFBOWU2LS1xYzhxeWkyV3ZFMG5sakpDSGxhVk51WVhfRWt3bzVJeUlRNnAzV0pEUXdWeEVYYmJSRF9iUWxuSGtnTnNRdlNQS0ZPNWRvZ1liaDYtWnFRZ3BrYUlRVXB2cXd5UVpJYWN3eUpSS2F4STMtdk5QaHdqWEtSa0FXT2lJRWVta2x5Tzd5QnRaS2NWXzVj?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -680,52 +680,52 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46078.97898148148</v>
+        <v>46079.42653935185</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Latest update on closure from city centre sandwich bar - Oxford Mail</t>
+          <t>Minderjarige verdachte steekpartij Mol vrij onder voorwaarden: nog een jongere in gesloten instelling - GVA</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Latest update on closure from city centre sandwich bar - Oxford Mail</t>
+          <t>Minor suspected of stabbing Mole released under conditions: another young person in a closed institution - GVA</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 16:00:00 GMT</t>
+          <t>Thu, 26 Feb 2026 09:41:46 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxQRlp2RTlpNXNRZkl4eEdMMzF2cVZVbDBJRC1nQjAyQnhobUN0SkcxMEE2OFItdnlBalptekFQeTJRWTNJcUl4RlhTbFBsSUVTekhYbmQxNlhRLVhxZmpFbk9SWE5EQ3pnajdyV3JWdFkzMV9Oa2oyVGl5SnY1RE8wZ3lIZmR6QUo1R0QzMTZFVU01R1U?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8wFBVV95cUxQUzdtUjdYaEhfaWtqS01WbGMwXzZIdFZZX29rNGRNTHFYYm5lbDJaM3F3aE0zM2ctaGM4VlJTU2RDYVVnVERjejBXZnF4eXM1OHAxN2FYaGw2cmxsWFNYOW1mRHdrMHhDRzNRR3lRX1RkemhyNkswYXE3NllLS1VwdVhZN2Y5eEtEZnlCMVRUUVNZNGc3MjM4a09SU0dsbWdfQ3NoUlVOd3RxZ1NWSGhmN1VQdjZRelBaeXdreHFzQ1ZPUmtfY1pPNXlLdG16Mm0wODI3N1BOTWx4VDk0aEVzcURKSDRIUlhQQW5qWjBodXVMR3c?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -735,52 +735,52 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46078.66666666666</v>
+        <v>46079.40400462963</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>From Bargain Bins to “Mini-Vacations”: China’s Outlet Boom Deepens as Sales Rise 9% - 一财全球Yicai Global</t>
+          <t>Medewerkers Arnhems autobedrijf gewond na schietpartij, burgemeester spreekt van ‘afschuwelijke daad’ - Automotive Online</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>From Bargain Bins to “Mini-Vacations”: China’s Outlet Boom Deepens as Sales Rise 9% - 一财全球Yicai Global</t>
+          <t>Employees of Arnhem car company injured after shooting, mayor speaks of 'horrible act' - Automotive Online</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 09:13:54 GMT</t>
+          <t>Thu, 26 Feb 2026 12:19:43 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQQVhnQ0Y1UWRwRmdlb3JBNlR3NG9RYzhSZ0thTkhtWHRKWW1rbjdRYmJKeXJzeE8wMUpiVTZ5aV8tWTVZQnA1LU5NejhlREM2SmluVjI4T0dKMk5kdjBtQkQ1WXhmWkJHVFV6YlgzcXBfaTdKME45SVFZV1Aya3pfRTZPVFBBSTFrd0JBZHNlbmd3R0lNa1VTZ2NFcS1QTmhvVy00S2p4Mmt6SkVwTXU2QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxOWXF3QnBVS3NHa2xIQllYQmpCc3VBNDQtVVpfbjVlR2EtVTlfSjh3b2RMemRLNlJfeWxlT2ZwRzhaaUdvUU9EQTF4OGw4N044TzhpUnFTY2tabWZsNkpadlZfYzdGQU5Gd0VmQkFGaWxWVkpINUJNaWE5SWhyUWIwbzctOUh5SklRWTVzYjZMaGVMX0wzTU9fVHhtTjJ2LWYzVkJiOEVhOG9Fc0JlSDllbTJJVllNQlNYOWJndTV2ZmlaZWNIQlU2djh4RWViZmp4RGtRZmY0c2FaSDR6ak0zZE1tcUdtNHRxdmc?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -790,52 +790,52 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46078.38465277778</v>
+        <v>46079.51369212963</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Shoplifting UK</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>("shoplifting" OR "retail theft" OR "retail crime" OR "shop theft" OR "pickpocket") AND ("UK" OR "England" OR "Britain") AND ("gang" OR "organised" OR "trend" OR "rise" OR "survey" OR "report")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Shoplifting on the rise in Scotland - Scottish Grocer &amp; Convenience Retailer</t>
+          <t>Tot 28 maanden cel gevraagd voor schietpartij aan Truiense supermarkt - Nieuwsblad</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Shoplifting on the rise in Scotland - Scottish Grocer &amp; Convenience Retailer</t>
+          <t>Up to 28 months in prison asked for shooting at Truiense supermarket - Nieuwsblad</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 08:32:50 GMT</t>
+          <t>Thu, 26 Feb 2026 11:31:27 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxOY1NoSnNJUHdDZVlIYkRJazd4c01fay1YMjNDQU83U0pPczJYdmRwbUFKQzV3S21sTFBnQXNoWmhhNjVoWG03N1ZZUnJRSnpzdC0wamFZY3lRWWpBMmFzTmh1LVlzT3RlYlZabDYzWG81emRxRnFxUWVZVGNuU0xDSTJn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxPN2JSbkd1NEhpSnNwcjZzdUVLWi1IYktjdF9DV1E4STZSVEIzRnBDV0d3cVFiTDRPNHQ1NE5IWWZ1bzQ5TEdfd1lIVTJWYmppNEI4OEEyWEdsd2M5UjY2TjFmdnVSdFY0bDF2Z213czdNNU1FSGlCT0NSejg3REFyZnhwWmVlemJfRmhhNEVmMjVfSXVqdkJUYlotQzFUX0Rkek5Zb3FMQTFta0JGanJxc0s1cHMxcHlYY2lidHNlWDBOcUY2UlYtUnV2Qjd2cXo2cFNR?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -845,21 +845,21 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46078.35613425926</v>
+        <v>46079.48017361111</v>
       </c>
     </row>
     <row r="9">
@@ -875,22 +875,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Explosie aan openbare camera’s baart privacywaakhond zorgen - De Standaard</t>
+          <t>Na beroep blijft hoofdverdachte taximoord Geel in de cel - Nieuwsblad</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Explosion of public cameras worries privacy watchdog - De Standaard</t>
+          <t>After appeal, main suspect in Geel taxi murder remains in jail - Nieuwsblad</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 05:30:00 GMT</t>
+          <t>Thu, 26 Feb 2026 09:02:03 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPTUJmTFZIODZ3UWpNWlJXNVQ2NTZlcDF3M2xtam9BTUlHWDZPYUFFU0pGRGlYOXJKVXNDT1BKMTVrMUxwQUlNNHB4anZkeFc2aE1TOHg5emlQSDBQQ1N3LVRsWS02QmJwWWtZZHNWYVB1SDJKOURaWDNvckdjMHVKLU9ZMm5uYnhtTjc1eEVpa3p0R3YwZDZ2MmZvbmFNY2ZxbTdxaHFPbEZlR0k?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPb0M1NGtlOE13MFpPNE43ZHRzQXhoLW1TWmRmMXpNYVNvN2lGSUdYT0dZRHVGUEpGdF9vdER6bTlTcTlIaE1MZ3N4V2ozcXcwS3BrMTlqQ1JiQzR1cWNxZExmOTFBRzFQV3NjV0ZNckV6NUZpZVZGVUw4YkFPaDRrZFpIWURXYzYyaEtBTFY0RjNETXMwdHpVTGVVUk1YWUllTTgxOC11M1BoWFFFOW0xU3NhVk5GYWRFV09DRGtzUjl5SjA?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -914,7 +914,7 @@
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46079.22916666666</v>
+        <v>46079.37642361111</v>
       </c>
     </row>
     <row r="10">
@@ -930,22 +930,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Jens Grieten (Kompass Klub): "Goed dat technocommunity duidelijk zegt wat niet kan" - VRT</t>
+          <t>212 explosies door lachgas in verbrandingsoven Isvag: “Afval wordt nu voorgesorteerd om incidenten te beperken” - Nieuwsblad</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Jens Grieten (Kompass Klub): "It's good that the techno community clearly says what is not possible" - VRT</t>
+          <t>212 explosions due to nitrous oxide in Isvag incinerator: “Waste is now pre-sorted to limit incidents” - Nieuwsblad</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 23:00:29 GMT</t>
+          <t>Thu, 26 Feb 2026 10:08:21 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxNaEpjUlo2Q04wMV9Vam9XdlRBdTdRQlUybmhrTlJjei0tTHRhbENIRHB5UmhsaUxuZjltM2NzaEFReWRwNWFsbEszRFFrYzhYNktvVnhoaTgyUkdXREgtLVRCVFBVX0dkd3FNNkVXUGQyVVBHTzV1MmVvVkh1cm1mQXVJeXVfZ0kzWHVUNDJYaENnVkw1YkgxNVppYjJDREpLaGY0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimwJBVV95cUxNV0g1Z2lGMmFVU3Ntc1praGtDVmJpb2FoT01QOE1kWHRvbDVGNjNKdXRNVUw1dVZHZXBpNVB0ck5Fa2luZ1lYOC1OTjdrNDJWRkhndjBkV2JjVXFfWC11R1N2Z2RjYy1rX1lFWjJKY0tMREZqV3laV3c5cThwMzEya3RuMjNQV0hTUmVpcDhhWERiaGh0eHVIN3VRR3hKcGNMTndkeUUydUlKV0d6VnJNTW4zRUcyM2U2NjdvY1JYeHRkOHNzcUJxRE4tLVZIMU5SX0RUeUlIMDZEWUptZHZNT0NPejhwcm1oazRNUTlEVloyeEd4aU15OTVicGF5Wk9jRjdoWjYtaXpNMnJkR3NDV1VsbUN6eWpRNzY4?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -969,38 +969,38 @@
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46078.95866898148</v>
+        <v>46079.42246527778</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Staatssecretaris Erkens snel naar Brussel voor beschikbaarheid CO2 in de kas - Nieuwe Oogst</t>
+          <t>Ukraine war latest: Russia makes Moscow 'terrorist attack' claim as talks continue in Geneva - Sky News</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>State Secretary Erkens quickly goes to Brussels for the availability of CO2 in the greenhouse - New Harvest</t>
+          <t>Ukraine war latest: Russia makes Moscow 'terrorist attack' claim as talks continue in Geneva - Sky News</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 10:00:00 GMT</t>
+          <t>Thu, 26 Feb 2026 07:58:52 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNQWZDWTliTDZRMU1Ub3BtNHhTSDFXTWRmUzBZNlpVZV9LRDhZeU9DOWY4b0Q5STc0U1ZNb2NON2tDY1NoR29GdXdxRTNIUGZXcUI1NEJJUzlIV2dubl9kUGdvYjNiN1NYZDRpY05PUmZVWTFpR2d6Yk5kZXZHejZVVXN5a1U0Zkxpa3lwZU5SbGN4eUZ1OS1MRm1fbjlzMENkc2NyNHVGT3FxdkQ4bDMweV9ITVpBeWluSXFpenln?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxOenB6YjJ4YVM4bU1jR2hreUI3UmNwa2tfUTU4VVNUVm9tM2hycVFnLWtYN0FBZkpDNEtrRWlDWk5KVW96QmVPdVRoVEptZ0JOWllFRDc1cWY1S1hiLUxsSnFTRms5MjZlNWZPdXBHV0RCeENQejlZc2N6RUlJekYwQnBPU28tN3lxc2UyZWlVZUZGR2ZFeGVVb19EcVpWMHBPUFUxV1RBc3NzQW5SNEtJNEJKOVZYTi1PcmRYcTdHenBUbDQwSXBfeUpkLVVtbVJQVWdJYk5Pc20wZw?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1020,42 +1020,42 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46078.41666666666</v>
+        <v>46079.3325462963</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Verdachte van taximoord in Geel probeert tevergeefs vrij te komen: ook in beroep blijft A.B. (20) aangehouden - HLN</t>
+          <t>Bomb Threats Spark Chaos in West Bengal's Postal Services - Devdiscourse</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Suspect of taxi murder in Geel tries in vain to be released: A.B. also remains on appeal. (20) arrested - HLN</t>
+          <t>Bomb Threats Spark Chaos in West Bengal's Postal Services - Devdiscourse</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 09:43:43 GMT</t>
+          <t>Thu, 26 Feb 2026 08:19:46 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxNS2pxcUxaMEF6Nm96R3p0Z2VzSVhGblZfTktvV0VGVlJXb0tMU2FVLVJ4YU5kYTFEakdZRVJ4aU1ZcmdWMkYwd1FNVThPUDQ1SG1tXzd2YndKRTVxSnZ0aEN6ajlXSHdqdUI3RWV1aHVMcTJoZlBpVmhLaUsxUWpYXzR1aVNWNGpVbWZNNmhaZEFZYWRUdF9Eay1FWXdHWmozYzVhRVBSV09zdmtJU25fUmN1bTFEMzBoUmZKVHNfWURnWTc0YXd0M2FfM1JYZ0ZLNXNZeU5R?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOVnE4aW04dHlhVGIxQl9HdVctMks4SnJhQmgxWXpqd1h5WmFiU0VtRUtROTdDcmM5cmp2b2R5Q0cxcm1SYVYwdlJTbFhLS3hlQ0piSGJyZWc3UkJsTl9SdDNZSWUwU2FmZFpEQmtVcGU3Z1prNVc1SHdBX0Z5QTlzcnFOZHE4ZFoyQlQ1WmIzeDRWM1VzaUwwUjRDYWlQRkh1OW5YS0JRUU9jSFBPeUJBaU9ORzRTQdIBtgFBVV95cUxOVnE4aW04dHlhVGIxQl9HdVctMks4SnJhQmgxWXpqd1h5WmFiU0VtRUtROTdDcmM5cmp2b2R5Q0cxcm1SYVYwdlJTbFhLS3hlQ0piSGJyZWc3UkJsTl9SdDNZSWUwU2FmZFpEQmtVcGU3Z1prNVc1SHdBX0Z5QTlzcnFOZHE4ZFoyQlQ1WmIzeDRWM1VzaUwwUjRDYWlQRkh1OW5YS0JRUU9jSFBPeUJBaU9ORzRTQQ?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1075,42 +1075,42 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46078.4053587963</v>
+        <v>46079.34706018519</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Bom barst in dancewereld: top-dj’s beschuldigd van seksueel wangedrag, optredens in sneltempo geschrapt - HLN</t>
+          <t>South Korea and UAE Forge $35 Billion Defence Alliance - Devdiscourse</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Bombshell explodes in the dance world: top DJs accused of sexual misconduct, performances quickly canceled - HLN</t>
+          <t>South Korea and UAE Forge $35 Billion Defence Alliance - Devdiscourse</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 07:57:50 GMT</t>
+          <t>Thu, 26 Feb 2026 08:34:35 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxQaTJaVF9JOXJmVjVHcndLMzM4TThwWjBSV3hkbG10VTlUTFBJU1NfdGVvZC1XdHVxOWZJOW9jU0FLRTJ0a0RIbnVueFBoNEZtQlgwdlo4b0ZJdEk1NkcyNS1jbU1QQjNHMHlSaE94azd6QTgzc2xkMzlSSjIyN09CeXZDel9xNmRWVTJfQm5FQV9zb3JrUzdwNkZjNTVCdjZrRmxKZTlKdkFmQzVkWVdSOFFQQkJHMjBUaTdydUpUbF9MLW1GcjNxRV9zMWlxdEtNeFZn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPRVFodHBSSXVzeXE4ZG5mOFdiRFRISG1KOHBqcVRnOS1nZFhEZ2RrQUJhX3piNkRQOG5lN1R6dUNZV1RTRC1BTHJxTHlDbE5BSDZnQTZHaThSaWxiajZRX1lzbTVVSEExYjdXM1YxRVdTWmhBdER4eXZTZG5ySTBLRFFyeVd1MW9fUmNDVFYyalNKcy13NERDNk52SWVJaFlYTWY3emVLd2xRUFBuYVVQRtIBsAFBVV95cUxPRVFodHBSSXVzeXE4ZG5mOFdiRFRISG1KOHBqcVRnOS1nZFhEZ2RrQUJhX3piNkRQOG5lN1R6dUNZV1RTRC1BTHJxTHlDbE5BSDZnQTZHaThSaWxiajZRX1lzbTVVSEExYjdXM1YxRVdTWmhBdER4eXZTZG5ySTBLRFFyeVd1MW9fUmNDVFYyalNKcy13NERDNk52SWVJaFlYTWY3emVLd2xRUFBuYVVQRg?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1130,42 +1130,42 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46078.3318287037</v>
+        <v>46079.35734953704</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Man op elektrische step slaat op de vlucht na routinecontrole in Brussel-West: politie vindt meer dan 1 kilo marihuana - HLN</t>
+          <t>The Cost of Defending NATO's Eastern Flank - Devdiscourse</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Man on electric scooter flees after routine check in Brussels West: police find more than 1 kilo of marijuana - HLN</t>
+          <t>The Cost of Defending NATO's Eastern Flank - Devdiscourse</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 15:18:41 GMT</t>
+          <t>Thu, 26 Feb 2026 08:24:37 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxNMnlETE5uMDVNNFA4R3FWT2EtNUFXSlJkdERxZHhHZ1prSHhiUVlUVWJDdWE2bnV1NzgyYl9oYVRHd09QcmV3NjkwcHVpbGd0dEdEdG9rRHBhUmlaWkZRcW51dVpnb081MkpFRlgtQTJXYzZRVlhXenFkZ0dEM3BwbGROTTBaS0RTZUxvMDhERGo1eGJtczktZU42aEFtRjl1UGVkZ2d0Q0NjVWE3TkVsSXJlUXhkWUx0OGxLSHg5ZGxUY2VXN1NNRF9Nd1Ytb3pVVmktZjQ0Um4zS3BRaXZfeGU5ZEVwWmhoM1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxPMVJZbjdoMTM0VXZfSmJTOWdvUFVpODRYcUNybzA0WDZNWlg2NDlCek1fVFRib0J5dF9UR2N0SHJqV0xIUzl6MlpoQW1Da2RhaTF5UEozcnVaRVdYV20wTjEzNUc0cUJfWmVfUnBDQlJYdGhaOFhRMm12clhiTjBCX09OVjJFQUY3VzJCMlJXVHJRTG1YeEN2X1FpVjIyWGtxS0HSAaIBQVVfeXFMTzFSWW43aDEzNFV2X0piUzlnb1BVaTg0WHFDcm8wNFg2TVpYNjQ5QnpNX1RUYm9CeXRfVEdjdEhyaldMSFM5ejJaaEFtQ2tkYWkxeVBKM3J1WkVXWFdtME4xMzVHNHFCX1plX1JwQ0JSWHRoWjhYUTJtdnJYYk4wQl9PTlYyRUFGN1cyQjJSV1RyUUxtWHhDdl9RaVYyMlhrcUtB?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1185,11 +1185,11 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46078.63797453704</v>
+        <v>46079.35042824074</v>
       </c>
     </row>
     <row r="15">
@@ -1205,22 +1205,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>False bomb threat at Brussels Airport prompts security response, no evacuation required - Aviation24.be</t>
+          <t>British Nationals Jailed in Bali for Drug Offenses - Devdiscourse</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>False bomb threat at Brussels Airport prompts security response, no evacuation required - Aviation24.be</t>
+          <t>British Nationals Jailed in Bali for Drug Offenses - Devdiscourse</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 10:40:50 GMT</t>
+          <t>Thu, 26 Feb 2026 08:58:11 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxNSFFvV1Itc3d0a2YtTS1zQzBpLTRta2RQWnBZU2c4akI4Um1tSXNabVhWb2doeWI5T1BCM0taSVdFY3kwUDV2UkZJRFFYejJ1STBtcWRDRjRDUmlvX2kzZWVNN3NyOENzQkdBR0JLUXJpZlc5ckM5Z3Y3T0RSaXhwNjAyTXF1M1ljemVaczdOZHo4SXpaVUlLYnUzN3E2NEh0T05xM0lSSTRJVmJ2cS1vT25SbzI4Mkd5UDZCQ2RtYlZrSTlabFg1TW5MdGtBTHo5ekhfY1JwdF9Sdlk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNSWNGM3VmaHJSdmtpZWFjSGxDU293eFZpWjVlMjhNRTFCUXd2S0lFUGVZYXpYOHR1VUNNRG9YS3ZZTF9NSjlqZkZtZ0x5ZUdDZVJyWjZ1ZmlQb3NVb2JPc1cydmRia193cmN5dnNLQkZUMGl2Z0kwZTNTeGhoN3FRU01YenJPVHUxa05ITkJ4ck9FNHYyLTZ5aThQdnltV2RjSUdiTHBVZGVJakxvdEHSAa4BQVVfeXFMTUljRjN1ZmhyUnZraWVhY0hsQ1Nvd3hWaVo1ZTI4TUUxQlF3dktJRVBlWWF6WDh0dVVDTURvWEt2WUxfTUo5amZGbWdMeWVHQ2VSclo2dWZpUG9zVW9iT3NXMnZkYmtfd3JjeXZzS0JGVDBpdmdJMGUzU3hoaDdxUVNNWHpyT1R1MWtOSE5CeHJPRTR2Mi02eWk4UHZ5bVdkY0lHYkxwVWRlSWpMb3RB?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1244,38 +1244,38 @@
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46078.44502314815</v>
+        <v>46079.37373842593</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Ireland eyes closer cooperation with NATO neighbours to handle maritime threats - The Straits Times</t>
+          <t>Alerte à la bombe levée à la Grande Synagogue de Bruxelles - 7sur7.be</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Ireland eyes closer cooperation with NATO neighbours to handle maritime threats - The Straits Times</t>
+          <t>Bomb alert lifted at the Great Synagogue of Brussels - 7sur7.be</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 15:22:16 GMT</t>
+          <t>Thu, 26 Feb 2026 11:10:56 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxQM2ppZS1xNFdnNTZlbFBVazZoUWRVblpDbnVVVGlvWmJuMlJqamJEdzY3UnY1eFQwMC1sV0o2dl9nZE9WODNnVXpybDA2Ym5YRjJmN29YczBwR2VheEdZUFpnWXFVTXdlVTd5cU91Zm5zb3I1R1VLakJrQVVDX0ltQ1lGZHh3eGZMZUNyZmxYWE1wRkkxb0xXVWRJNTAzQVBFMzBsbUFzN2RsRWF2QUFmNHFkYjVYcHdKczBDVDBoWUpFOU5oM1BZRHAyUjI0UUNBNC10aFZWc0IyUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNNUcyd1ZldmRua3FWVTVNa1RyYmdmNG9JVW01VUs0Z1FETXRkSTFFMEpfSmxjRzVjaHVSQ0tnLV8wQmNYQVZTdWpNRDNRYjZuaWFCdUFpYmxGMUhBbjBGOTJyV05adDBFdjhIcG5lbGIzLVIyUGpnakF0RlVGN3lrR0lralBudHF0WGF2SGdwSHU4di1UT24yTko0X0VUY0NmaThPQmt3?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1295,42 +1295,42 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46078.64046296296</v>
+        <v>46079.46592592593</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Spirit Airlines to exit second bankruptcy as smaller, restructured carrier - Aviation24.be</t>
+          <t>Fusillade signalée à Matonge : une personne blessée transportée à l’hôpital - BruxellesToday</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Spirit Airlines to exit second bankruptcy as smaller, restructured carrier - Aviation24.be</t>
+          <t>Shooting reported in Matonge: injured person taken to hospital - BruxellesToday</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 15:34:21 GMT</t>
+          <t>Thu, 26 Feb 2026 09:21:00 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPU18ydTBZVGxoYWJ2cjRvQk45UHNGZE1GNVRfczhTenoydTA1ZlgxaUVrdXgtQXp6ZWs0Mmd4bWhGVHY5cy1QMXdxMkJSb0tDTlg4anJzTnFpT2FUMnZ4ejV3V2ZPV3RCOGlkTWRpUTRjMHZSbWpxUXo4M28xemVzeDhTSVNqV3NnT0R2VWtYZzk3OGZGbU5zMGtBQnVDTUY1OGViOExRMTNYbk1uRF92VHdJalVKRmxzZE1lUHVRdy1sNDM0UHF4dg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxNcEt2MEJuaERUd1FtRzh6S3YyUXBvYi05VjRKUjZpOHhvSW9UUnR1Rk54ZnRCb0FONnJJV1VxQTVEcHV2eFlMNXl5WU02cnN3QUdnb054Sk5aLTVYelBtYjVQUlJhUnp3NEFYbXJxSzk4Q0tSbWJSbE5SVmxwWWp3UlFGTQ?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1350,42 +1350,42 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46078.64885416667</v>
+        <v>46079.38958333333</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>U.S. Airforwarders Association criticises 10% import surcharge, warns of supply chain disruption - Aviation24.be</t>
+          <t>En appel, l’étudiant en médecine reconnu coupable de viol et d’agression bénéficie à nouveau d’une suspension du prononcé - VRT</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>U.S. Airforwarders Association criticises 10% import surcharge, warns of supply chain disruption - Aviation24.be</t>
+          <t>On appeal, the medical student convicted of rape and assault once again benefits from a suspension of the sentence - VRT</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 16:06:30 GMT</t>
+          <t>Thu, 26 Feb 2026 10:41:11 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxORERBYk5UUzVzUC13Q1R3SktnQ2gxN0F4SjFxR0dfZmt1cGtCNDRTMnUzYU9oeUlUYmpFZkRWT25FU3ppa1d4X2E5ZlFEUHllMEU3aW9WTlZKQUZPdVJvQVJyNkE0U2RwdDFsbDJtQUlEMUlNaER0M2hseDFCTmFhb0tiNmJNM1l4MmVsd0JGQzF2YXZzVzJZRFEtN21HczdtNmxmdVBmQ3pmR19WNVNJVTFCMU9WMnBXMTVKVXlsWHM5b0MzUTg2X01zbzZpMGhreHY3Y1VCODZKcDFhYldCYmw2cXpCQzVHSEtCY015UFNpU3hUdHRB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNeHpLMEw4Rl9jRUxXVnNib0xGTjZhRzJ4NnQ2WDdnM2szenhkS3M1Wmh2ZktQWVR2bkN1M1ptdkNGTU9NVWY0VlVnWGtxbzM0NWZObDhWOGRaYmxzbUNCM0pmdlgwMnFLdXhhMnBLU1BUZmNPWWtCdS14SVYtOHJEV1dVS0JkTHp3QlNvazNlN1lZcGdON0htNGhHQUc1cEZ4WUlIdTBn?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1395,7 +1395,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1405,42 +1405,42 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46078.67118055555</v>
+        <v>46079.4452662037</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Etihad deploys A380 to Bangkok from October 2026, bringing The Residence to Thailand - Aviation24.be</t>
+          <t>Coups de feu dans le quartier Matonge à Ixelles, une personne à l’hôpital - 7sur7.be</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Etihad deploys A380 to Bangkok from October 2026, bringing The Residence to Thailand - Aviation24.be</t>
+          <t>Gunshots in the Matonge district of Ixelles, one person in hospital - 7sur7.be</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 14:42:33 GMT</t>
+          <t>Thu, 26 Feb 2026 10:46:00 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxNRkhFdmhYaC1PTG9YcERvYVNtVEVHWG1nbWVoQW80Y1J6ZldzckNkRVVHYjhvdUpTVUxHcVF2bDVZQ1QyaWQweDBQdUw3eTRxaGJIV0lFZHg3Tk5CVEM5N18tbkNtRTcwNnJRbENya29IZDY0Njk3bXVIcWJqTEhMN285SWtMMzZ0ZWFMRkIzekVvczdWbW5uV29QY2ItQml6UGVJc2wxWjVpS3VrWUxzUDhxVE9KYVUtTzBjcU9VZmNXNXJUNkN5RlRZZEZ0ajZFLVJBRA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOd1pVT2NvcTc1QlZLR2M0eGR5ZmJ3QlB3Vk9iU09OS2g2X0dtMVJWUHF6MU1tRVdHUTB4Y3F4RmlwTmlVOHFLWUJ1TlFBZlhpT0lvb21MRzZzOFg0ZEQ5ZkIteTJVY0FGSmNFcmozQzNyVUVwX0Q2X0Y5TFhST283aGh5T0dvd3dLWDNsVzhuOW1abEJNa3J2QlBXRHJPVGMtU1VuNnB5bmE0YmdORXVVRmJWM0pEZw?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1450,7 +1450,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,42 +1460,42 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46078.61288194444</v>
+        <v>46079.44861111111</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>IAG Cargo launches 24/7 global AOG service as demand for rapid aircraft recovery grows - Aviation24.be</t>
+          <t>Métros 2 et 6 interrompus entre Delacroix et Bockstael - BruxellesToday</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>IAG Cargo launches 24/7 global AOG service as demand for rapid aircraft recovery grows - Aviation24.be</t>
+          <t>Metros 2 and 6 interrupted between Delacroix and Bockstael - BruxellesToday</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 15:56:28 GMT</t>
+          <t>Thu, 26 Feb 2026 10:09:00 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxQQVF1ZEFLLWJqNWdoTFVkQVhZX1JiNlNyTlBndDRNekZwYzhKdlQ4VDhMWFZYXy1XZFRpeTU5Ylg3UTVoLXhZNlRJN011RGZvR041SVNmTkdnQnNyZVRkTjFQYl84TGVLekRMSjQ4V0xWTjBwOEhibTlydVlBZkxEU2Nodi1kdlEtZUxYRll5Zk1kVXN4a0JXVVplbGFTQ0Nva0dsVTB1V042Y3NpaTM0MjFNSWt0M1loNW5XQm1WMzczd29KWTNUZ0xlM3VBcEpzc1JfTldDOVJzbzhuZUVUYXFYUzhVQkNCcldyX3VXUERxUEpwMFczOHdEamwyUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxNNkphLVFkWm1RLWlrUm1ESFVtU3I3M202Mzdmd3pqYnFqYXRTc2NINkxHcHJfMXZ6QW9GZ2FTZ21UNlM5RVEtVnJLV05RWGxMOHg5SFBiMzZVQXc3SHJoZzkwS1pZeTJZUVl6ZlVnYnd0QWtIRVFuOHFHVm5hY3hBX1BCSE5XZVBFTGowVnhZVmc?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1515,42 +1515,42 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46078.66421296296</v>
+        <v>46079.42291666667</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Federal Ombudsman: 6,000+ regulatory breaches recorded around Brussels Airport in 2025 - Aviation24.be</t>
+          <t>Un inspecteur de police pris en flagrant délit en train de sniffer de la cocaïne dans un commissariat - 7sur7.be</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Federal Ombudsman: 6,000+ regulatory breaches recorded around Brussels Airport in 2025 - Aviation24.be</t>
+          <t>Police inspector caught red-handed snorting cocaine in police station - 7sur7.be</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 15:26:22 GMT</t>
+          <t>Thu, 26 Feb 2026 12:04:00 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxQQ1RrV1ZyX0pjRUVNV1pJX3dLT0NDX1AwWnJwZkJJSzZjNFdwdWVBRmtXQm11UzhSVXRUUG9tS2FWX0I1bFdKQWpfbzdGc2lNOXpGSHUtNU9pYVZNSHdBQll6Zmg1dlg4Mzd0eDdXdElvZnZ2UGpDQTMxX0NvbHlGeXA3U2ctaFkxeUNqcm0tZDdrek9aUTVPM2VtZ2pPZk9GY1Y4NTN3TV9xVUtqX2k0c0dRM1BkaXlMSUN6cXBYZWhmVDZGOTQxY09MdGNGWjhZZlZoWVVsaVpZbkFo?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxQclk4YnA0RkhMTzEycWdDd3JlQnctZ2swbDFZYXUxaXZFZDZNTDBZbUg2TVR2cjBsdTVCdkw0ZVhsWlVtelR6OEJrUGQzNnRnS2xkSWFncm5mUkRaS3R1X1FBRU1lbnNETHUtMVJXUEFnSFlmUDlxVkV0bHktVElBRHJXcGY3UTlPSENFTktoTVJSeWlLOVBzYzl4MjNtTXVRT294M1NITDN4MzAwX0EzX09JUUtFT0FodF9ISGxjTHk4enlPTGZmLU1WOEFiQ1o1RjUyUXN5WjVHRG9zTXc?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1560,7 +1560,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1570,42 +1570,42 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46078.64331018519</v>
+        <v>46079.50277777778</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>TUI fly Amsterdam–Montego Bay flight diverts to Bermuda, and afterwards to Cancun - Aviation24.be</t>
+          <t>Assassin’s Creed maker Ubisoft cuts jobs, sparks strike - AOL.com</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>TUI fly Amsterdam–Montego Bay flight diverts to Bermuda, and afterwards to Cancun - Aviation24.be</t>
+          <t>Assassin’s Creed maker Ubisoft cuts jobs, sparks strike - AOL.com</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 17:09:14 GMT</t>
+          <t>Thu, 26 Feb 2026 08:31:09 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxQdlhkNkwwOG1xN3BkdWY0S2Y0WkFqZU10SzFfTVc5aXNmdG12WHppZmZUdGJDdnhmSTluQjRObWNvQXYzMFhqNW1SUnIwbE5qRlg4RFZhSm1JMDA5c05XdldMSEpGNzlQNVo4cmxiQXhjUGpzOG1LR1JOeVQtNktqck0tVlZxUXlOaFBxTTBsbzQ1Q3FZem9MaE5saDM4VGFIN3VuRkhDalhfcG13QXVjX1ZWNC13SWx6bG1GbGo5WV9EUkZ1dlFQNHhVTDR0b0dYYjFQS2k2S0ZFWWJrb05hcjFzVQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxNT1h3QWd4eHNRQlFGRDh4UExSNTZiUHp4d1R4c0lxcG5LWEhsQU5sZklnUWlBYzlOV2hNREZ1Uk9haW1WdlQ0MUF5c3E5Y3pPTFc4czRwd3dBOGpCS0M1RkdvaHNXSUZNRi1fT19xZHVJYThNRk9fNmZwQXIxc1l5Umxn?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1620,47 +1620,47 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46078.71474537037</v>
+        <v>46079.35496527778</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Plus d’une vingtaine d’agressions au CPAS de la Ville de Bruxelles : des sanctions sur le RIS envisagées - BruxellesToday</t>
+          <t>Falscher Uni-Arzt ruft an: Tausende Euro Beute in Würzburg-Heidingsfeld | Foto: Wolf von Dewitz (dpa-Zentralbild) - main-echo.de</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>More than twenty attacks at the CPAS of the City of Brussels: sanctions on the RIS envisaged - BruxellesToday</t>
+          <t>Wrong university doctor calls: Thousands of euros in loot in Würzburg-Heidingsfeld | Photo: Wolf von Dewitz (dpa central image) - main-echo.de</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 11:32:00 GMT</t>
+          <t>Thu, 26 Feb 2026 10:22:47 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNblV2Mk45V3MtT0hiU0J4cEVLSkk0QVFOOXFRS05TTUVwZVk2NVFmWG9COV9Od001MDcxdzBnTWpydVlnWVFEOUk4MlNOLUMySGJkZFFpM3hPNVZJMExmSXVkVS1mQW0zQ3E0d1pLTjFwMjZ5a0tqQ1RJLVRjc1NrdE55eGVJMDFSMkYyWQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxQSllxUHA4ZGpoSlFmY1gzYllYcEVaeVZmU3laTnRaWU5sYURJZ3IzTTdkdnltWkRlM040aUtoZ1lxZk1yUm9WMGFSbzhKdHlKQmZVVlhSUlJaYVZUOGRmQjlfa185eG5vd3VKOUt0amFLT0ZUZU9LdWI1NDg5TXIyN25GemdEZ29jNEVHOUhFdnhkVU9GMnAxMjNxcUJrRlpUbmhHaWliOENhdG9LM0FSMWFEZEtVaDV4QmFZMUVrSE02MzYxd2c?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1670,52 +1670,52 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46078.48055555556</v>
+        <v>46079.43248842593</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Le CPAS de la Ville de Bruxelles a recensé 26 incidents violents en 2025 - BX1</t>
+          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>The CPAS of the City of Brussels recorded 26 violent incidents in 2025 - BX1</t>
+          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 15:36:56 GMT</t>
+          <t>Thu, 26 Feb 2026 09:29:48 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxOanBUYWg1T3JISGlCRU9qdlhJNXJjaXpxeVM0RG95eWNGS1NHUHRITDN1dFQyWVJreG9WdEw2OTBndEJQXy1QWXF4Nm0zS0JZRUFRUWprYy13MFRTdlJDdEF4czJ3Y1BfYnpBME14UGU0Rmpyc3I3VER2eU40aDJweDBXODB6VE5wc2JNUFNsekNNNDUzZXl1Q05QWG9HNXpPc24tUnhXUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE03RUZJdVVWTG5jTlA1R0dmc2YyQ3Z2S1ExYmhkN0FENFJGamUwenJsSFFPWGpKc3B2aFBaeHRYVDR3aWM1SXg0YWZFVDk0N3d4a0Jz?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1725,52 +1725,52 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46078.65064814815</v>
+        <v>46079.39569444444</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Les trams 4 et 10 interrompus brièvement - BruxellesToday</t>
+          <t>Unterfranken: Trickbetrug mit falscher Arzt Masche häuft sich - Charivari Würzburg</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Trams 4 and 10 briefly interrupted - BruxellesToday</t>
+          <t>Lower Franconia: Fraud with false doctor scams is increasing - Charivari Würzburg</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 16:44:02 GMT</t>
+          <t>Thu, 26 Feb 2026 11:13:00 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxQZFh5dEZoX2dFSEhWcXNiTThkek9ISEx6SXRJbDJHOWs0VHh0RmVMQmRoblc1NjhzMXBVbE1KR2FFUEFlc3V2UXpJMmlQZDJKN0p1cGF6TlRkcVFHLWU4YVZlWWx5UEt3cGUzNGdDQ3h4eDVGQWtYSkZqc1FCLVJrUkhGTQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNSTRTbUYzUmlxdFVlemx5ZEhUX09PLXJlc1Z2cGdLbDlKU2Z0MEE1Wm1DeUJ4UWRiT0lkeHd3ZUx6TVBfdlluNkVWalA1Mi1sT0xMSnRyNE12YzhieTg0emdpbkNzelRhOW52NmZaaFlycUxhX3Z2YWdOX2dyckl4QlhxU09oSzhOSU1KZnZvNjJsdTlUNXBMMmVUdUNIN00?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1780,52 +1780,52 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46078.69724537037</v>
+        <v>46079.46736111111</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>18,9°C à Bruxelles: record de chaleur battu pour un 25 février - 7sur7.be</t>
+          <t>Mobile Blitzer in Prosselsheim aktuell am Donnerstag: Hier nimmt die Polizei am 26.02.2026 Raser ins Visier - News.de</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>18.9°C in Brussels: heat record broken for February 25 - 7sur7.be</t>
+          <t>Mobile speed cameras in Prosselsheim currently on Thursday: Here the police are targeting speeders on February 26th, 2026 - News.de</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 13:24:03 GMT</t>
+          <t>Thu, 26 Feb 2026 09:18:59 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNVUxQbFR1U2NjQXJ0bWFIbEx6REd1YlhFZFJ2eVpmQkRveFFZNU5jdWVoUFM4U3FhTl95eXVRMTlYb1lKcEhTNDRGYXoybUZOQ0dhNFZkMHdHdGRYTkNJd0UxbjlxN09KSE80a2FmQ095d0pWczY4TzMwZXBZTjVySEQ2cnYzY3pKMnJYWUwtTEhXQ0ZLUlR4VF8wRFh3cFlTOUE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNbjNUOG5zWkZlNDJfWUM4ZTIzV2pCa2hyZVdHajYtcFF5QkM2OTRvSkFjUVpFT19adzhuT0EtYzBEUXA2SjdxR1hjMjVXQWtxYThmaWxpazR4X3ZpeDJfRWNsNFJlRzI0VHN6ZnItRTNWelA3WXJ4NlZ3VTFaSHVpUnBhNlFJa2lVdjZRV2dFR09mRHJoZGdxZVhLN3lfaGRuX2NfeE9ONzJuOE5iZk9xNExEaWItQTE2dmw3R0tuaVNtaFJ5dlRXRzBObmFlT3N3a2stSjBUdVNDam9ZNnc4cHltTExjZGNLTlBPZFUxZVBlaDZsMENrMUVwRVB4ZjA2N2J4d3RIMXlCNjVVME4tRtIBlgJBVV95cUxPNktVejlZZVRSWFZ6Y2Q5S01TQ25adENrV0ZITEo0NXRiMmFLdFV2cUhCY0lLNm0xM3NRYVFQNkJyck5zMmJ5MGV6TDNLaG5ZQl8ydHpjUnN2WDNoMmd1RnVuYU9OZ2ZOdzNRbzUtZGFuSmhHLVRlOXdJS1NZQmF3Y044VWtGR2pQNVpGLVZXd0FELUhlRWdnZ2tRVXNBc1pvdUlMOHZWSUhCc1lMRFBqUkpZT2lLNk5pekpKU29zaW42WDN3VFRBbVBxLTJjM0RNdEtVNGpEemZzOVhmTzRSNjhTVGw0ZDV5NjExVHpyUGdQNFZnajAzZmh4WjlXd0QzblJWSUN0SmFNdEpUenQ5aTh1QlQ1QQ?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1835,52 +1835,52 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46078.55836805556</v>
+        <v>46079.38818287037</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>"Un scooter faisait des roues arrière" : un couple s'est fait passer à tabac devant le centre commercial Basilix à Berchem-Sainte-Agathe - BruxellesToday</t>
+          <t>Polizei stoppt 19-Jährigen mit ungewöhnlich schnellem E-Bike - Augsburger Allgemeine</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>“A scooter was spinning backwards”: a couple was beaten up in front of the Basilix shopping center in Berchem-Sainte-Agathe - BrusselsToday</t>
+          <t>Police stop 19-year-old with unusually fast e-bike - Augsburger Allgemeine</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 08:06:02 GMT</t>
+          <t>Thu, 26 Feb 2026 10:30:03 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQbUtkQ2xUMFo0NUdZR1NDNGdBU2V3bzhURWt4Q2tBSXZib1AzX01ZQmI0V21CbExjZ3M3bTdoekQ4eTJicmpLVVFaanUtN3lDTDRicFpqQ3pPTG1wWi00S1dud09hM3RDSGg4QnJmc1cwTkJIRDVtc3dUbjJZZmFMN1g3Umk0YWt0UnJ3am5RcllkdWJJ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxPaDB3RnJLa3M2cFRlWGxnVjhIZGtrTG5zZFlncmxTaFEydGVXT3ktUkEycXJWV1BkT0tvdVQ3d19rYmxqeHVLeFIyM0dTZmRaVW1RbFpLT0Nuald4X0Vvc0xnaF9vWU5DdTVVN1MwMEExTUhaR3V0dk9xMTJvcXJ3RGVtQWJWaURuMXVVZ0hZckJaZFBOREZYSDB2eGpjem50Z1hhdGYzVkNVVTRrMVJyakNQQQ?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1890,52 +1890,52 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46078.33752314815</v>
+        <v>46079.43753472222</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>La CGSP Cheminots dépose un préavis de grève de trois jours sur le rail en mars - 7sur7.be</t>
+          <t>Polizeibekannter 19-Jähriger handelt sich erneut Strafanzeigen in Ingolstadt ein - Pfaffenhofen Today</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>The CGSP Cheminots files a three-day strike notice on the rail in March - 7sur7.be</t>
+          <t>19-year-old known to police files new criminal charges in Ingolstadt - Pfaffenhofen Today</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 14:26:00 GMT</t>
+          <t>Thu, 26 Feb 2026 14:34:33 GMT</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxNeTJ0Y1BCeXZpRjlQZmNJWFE3NTRGTWFHUE11U0lpaHVvSElGN0dCd25NX1hONXVPQ2Z0MHI3V1AtemVoRXd1ek0zeXdmTUlWcU9yLVVHV0c0NmYyTlQ0X1JibkJwNzFKTFpGRFU4eWRWXzlrZ3RMSWJuNS1pRHlOVkZ2NnBOR1FRNk9YSlpPUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMia0FVX3lxTE0zaUNPRFlYQ09mV0FhZzlaemNFSV9ybi0wMEE2T3NtV2hEZ0xodnd4ck9KV0pXMVN1WVRoMmxmZTVkVFpIbmJybFM5ZjdmMUd2T0tZUkN2QThnQnNHVE4zYzhFQ2s1SnZ1V3lN?oc=5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1945,52 +1945,52 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K28" s="1" t="n">
-        <v>46078.60138888889</v>
+        <v>46079.60732638889</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Politiezone Limburg Regio Hoofdstad ijvert voor eigen TikTokaccount: "Jongeren bereiken in hun eigen leefwereld" - VRT</t>
+          <t>Zwei Verletzte bei Frontal-Zusammenstoß zwischen Transportern in Ingolstadt - Pfaffenhofen Today</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Police zone Limburg Capital Region is working towards its own TikTok account: "Reaching young people in their own living environment" - VRT</t>
+          <t>Two injured in head-on collision between vans in Ingolstadt - Pfaffenhofen Today</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 07:37:41 GMT</t>
+          <t>Thu, 26 Feb 2026 12:47:11 GMT</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxNai1yalVwN0dOTG1mbU1heHFLTEVLYzhPaDBNVndkd1A3S29YRk5XeGVoTk1wdzNZRTNNX05xa2d3TmtqRVhMbzVoYXFUR3dsaThPNm1Fdll0OFFfNEZqS1VzM0I1dUZBQUR1R0NpbFMxUXNKVmMwRXBFLXBuZWZxNg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE5pTXVwUVlaRHpJY1ZWUTR5NkMyVS1nSERtOEtseUFkbDZPRXRBc3BHbTVReXNOM3dETG00YUxESFVSZGJXaTRsbU1vbS1XNmpUbGNIUVhVb0gzSnpGcWl3RmYzc2h3VmM2VUdON05xMDdMQQ?oc=5</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2000,52 +2000,52 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K29" s="1" t="n">
-        <v>46079.31783564815</v>
+        <v>46079.5327662037</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Minister van Binnenlandse Zaken Quintin (MR) pleit bij bezoek aan politiezone LRH in Hasselt opnieuw voor fusies van zones - VRT</t>
+          <t>Kleintransporter krachen frontal ineinander – zwei Menschen verletzt - Augsburger Allgemeine</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Minister of the Interior Quintin (MR) again calls for mergers of zones during a visit to the LRH police zone in Hasselt - VRT</t>
+          <t>Small vans crash into each other head-on – two people injured - Augsburger Allgemeine</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 17:04:05 GMT</t>
+          <t>Thu, 26 Feb 2026 09:14:45 GMT</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxNbWgyV2ZETTdWd1lWZjA0eEkxU0lud29pV0Q5dWFqdmpTTFVhaWJBTTBJdTJmZmxUc2ZxUUhlcXc3VVR5Vm96b3ZoelVYNGY4OGZ4SUk1ZW05Y0VUeUJEUjNtN1FHb0ozZ2Q4TWxtLS1rUHVTcEF5MG80VVByNW9fN0p0dlU3TlExRTVKREZVRldWR3pTZ1ZpTElZbzNnT1d5Vl9hS0NmcTI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxOWEhJbnVGd3NuTWplRjFWbHNVVC1ldWl2b1lDVXgzMmItTlRZZHlFRW5Pd1ZwQUZoeVJRbC0yWTQxZzBUOURGTHp3bTY4Vlk3SUJ3MUNOVG1sNTdVUHV2cWpSRjd0NUJQVktnanZsOGp4enVnSjRMNUxFZUg5WVVNNTBUOWNaSDItdVltNXViZFVVeHVlb0tzM3hYTW5wUWxVdUp2NFQ5d1J1Z1R1Ymk5TTJuemFHd053WWtjbEFPT1laa1JnOXQ3eHRoSkNyb2dS?oc=5</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2055,52 +2055,52 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K30" s="1" t="n">
-        <v>46078.71116898148</v>
+        <v>46079.38524305556</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Twee auto's branden uit op privéterrein achter huis in Stevoort, oorzaak nog onduidelijk - VRT</t>
+          <t>Nach Vergewaltigung am Bahnhof in Pfaffenhofen: Mutmaßlicher Täter gefasst - Pfaffenhofen Today</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Two cars burn out on private property behind a house in Stevoort, cause still unclear - VRT</t>
+          <t>After rape at the train station in Pfaffenhofen: Suspected perpetrator caught - Pfaffenhofen Today</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 08:01:15 GMT</t>
+          <t>Thu, 26 Feb 2026 13:59:11 GMT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPS1ZUaU5WUzRCU0tiM3BRRTYtNXpFSlFSeUs3UjYzMHg1TDhheGJwQk1HMDNBSVNhRXh2aEFOaFZqNnpZdTlJSHRfQm1aVzNlamZ2R0tIM0NycGZVOHoyVmF5TUotM0M0RHd1dTRzTkdDNXlVZTN5UERuZHBFdlNhYUVZSnJGN3NtZHp0YkRUc1drVXViSkRKM3ZCOFc5ak4tNmxPZDh3bw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxNRDdYaE16bEI1eFZrV3NXU2t6SGZobUxDMVlOYi1vV3JfSGxPdC1Ed2JPb3k2b0dvZnJ4TzVtWmMxc3Z2UUstNnRWV1JaODFKY0VSc3RfYm44NmMycHRManVrd2EzT0h0b1FOOGdmWnJENVJqN3hiMUNzUWFSQUFmLUVfWlVkVkNvdVRLalhfOGw?oc=5</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2110,52 +2110,52 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K31" s="1" t="n">
-        <v>46078.33420138889</v>
+        <v>46079.5827662037</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Après la France, Thibaut Courtois s'attaque à la Belgique : le Diable Rouge va devenir actionnaire d'un club - Walfoot.be</t>
+          <t>Tablet und Kopfhörer aus Elektromarkt geklaut: Täter scheitern beim Fluchtversuch - Augsburger Allgemeine</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>After France, Thibaut Courtois attacks Belgium: the Red Devil will become a shareholder of a club - Walfoot.be</t>
+          <t>Tablet and headphones stolen from electronics store: Perpetrators fail in their attempt to escape - Augsburger Allgemeine</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 19:00:00 GMT</t>
+          <t>Thu, 26 Feb 2026 10:18:52 GMT</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxOd2R4T3hFY1laTzNheVhhYmptRGFyNzdLdG1HNFZNSTRRY016dG03UTJ2MGhoRFZoUmZpdThjem5nNURLaEs4YnVIRV80OEVMd0tEem1vdWVjdVJub1VPMnFIUXRub2dSUVMwYThDcHhJZk1COGtvOUtxb0E5blpIR0JSQ1JLRVNtNERJOC1sNFRua3JGRXZ5WDBqR3ZNWk93aDUteXN1dElNQWZQMC1mUXYxRUlYQ2JsSnpyWEpSVElFN1E4Ry1ldWRZZjZxLTI4OXpBRy1JYVRvMVnSAeABQVVfeXFMTXhOMUR2WkRnOW4xcGVBVl9KZ3U4Y3JLU2lqV096aV94MDgxWUxGcjk1WGdIbDFVdEdZMUVfY1Rka0tUbGR4ZVc1ZDFUQ2xCTFhPUjVCczRrTVdYNHd4VEVXamxDWGNGRnBIay1VM0htT2hWWUc0SWJvLVBNY2ZKdjhIWnQ4UWk4NUhPdEFNbkI4U3ZmZXEyamdpVXQ3NVZQZWt2a0RIUzJEMUhvRG5ETS1NOER2VXUyVnE1M1hIbVFmWHh3T3A1RnpQMWJjb0NSRjNITXdFMzBHY25CcWxWQ3M?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxQZzhvanhqeTBURENLb1pYYVZQY0FSdUNsMlpTaGVDS2tUQ0Q5VnIzaGh2UjFkc1AtcnZsU25XSnhWMFNXa0xSeGhZR0FocmRvRUNXVWFBVkxPUExsSUJGVUplQVRnNmh2ODdCOFR4eE1pWDlfWWZTbG5qbGJNcV9EVURQMFl5d3hBUGVUZmNKMjIyeV9lY3ByYkNUdkY0ZTRyNi1udzdwWEhlMi04MEVIX2xBbzJYRjhnTDFhcGpab2c?oc=5</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2165,52 +2165,52 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K32" s="1" t="n">
-        <v>46078.79166666666</v>
+        <v>46079.42976851852</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French</t>
+          <t>Village Ingolstadt (fallback)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Vrai ou faux. Le député LFI Raphaël Arnault a-t-il été condamné pour avoir protégé une manifestation LGBT ciblée par l'ultradroite ? - Radio France</t>
+          <t>Red Bull München signs Latvian national team defender Alberts Smits - EHC Red Bull München</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>True or false. Was LFI MP Raphaël Arnault convicted for protecting an LGBT demonstration targeted by the ultra-right? - Radio France</t>
+          <t>Red Bull München signs Latvian national team defender Alberts Smits - EHC Red Bull München</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 11:23:03 GMT</t>
+          <t>Thu, 26 Feb 2026 11:00:00 GMT</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxPd0hMVEw5NlBKdXdBMlVrWk4xREZZZnU5RmxDUVpwUHJqTndLeWZ5ODV3dUozZndOTDFpLUpBWHJkMjA3Z1p5TVM0TVNzOHBYbURfSnl6NzJSeWdJazJKYko0NW1MVXdKTmo3cVNjYWxYaGZLX2RNZXctVVlGaDhlYWNNc25VQUJWZ2pXZVA3NjdnSkRqMGtLczZOdjRKNzM0aThJeUVzai1fX2E2d1BpdVY4ZHQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxQdU0tU0RQRUFaNGpSNUE3R0lyZ1M3VEozSXhqcUN0VUh1WU1YLU9KbGpEVWxVWUZfNTBsd1ZuSk9GWnNTd0N1elJuSDJta1hZcEkxSDNMTWtjMzl0MVZCYmJnbnlzcXJPd2ZZbi14UXRtdTM5S05TcWk2TnRIOC1NODZoMkRQQkRFRkxpWjk3T2xGQXRKbkZ3aEIyZzk2cER6ZW4zNExkT3F6c0pu?oc=5</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2220,52 +2220,52 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K33" s="1" t="n">
-        <v>46078.47434027777</v>
+        <v>46079.45833333334</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French</t>
+          <t>Local Town Fidenza Italian</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
+          <t>("Fidenza" OR "Parma" OR "Piacenza" OR "Cremona") AND (protesta OR "minaccia bomba" OR esplosione OR sparatoria OR accoltellamento OR evacuazione OR "operazione di polizia" OR arresto) AND -calcio AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Le fisc belge réclame 1,5 milliard d’euros à Nike: le procès s’ouvre jeudi - 7sur7.be</t>
+          <t>Parma, un arresto per le tre suore uccise in Burundi nel 2014: chi è Harushimana Guillaume - Adnkronos</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Belgian tax authorities demand 1.5 billion euros from Nike: trial opens Thursday - 7sur7.be</t>
+          <t>Parma, an arrest for the three nuns killed in Burundi in 2014: who is Harushimana Guillaume - Adnkronos</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 05:49:00 GMT</t>
+          <t>Thu, 26 Feb 2026 12:46:00 GMT</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxNYWFMblVnV2JUSndYZVA1TjJtcU1FbTJSVlFKMmFRR29KSmd5V1ZVRkI1YVZ3NWdNRlB6Rzl4ZDRPaFJmZ294bW9wLUp3V01DdVVkZmtXTnBzSlMzMGpCWGE0SUM5TmhsNzJkVmduTlJTeFZhTnVId1N2T1paZUc5OG5SRDJyMVdkd0NPbi1iMG5pTnZNS3JJaTMyQTBpTmhNQ2ltV0FlOEtUYTVWTTdycA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxNOGYwQVJHbF9ReFVKWWNWaC0wM2RJb2hZMk5EdG1JdXNQOEF2clhmR3ZTVThzbFhfc3hteVdBT25xUlJnTlFXc1V5QjB1U2Z2VElLX09GcUx6LVFkeXFBZGlTWUM0RHdMZm40TGlTMUZTakxhT1VZMkRsYk51VGNrWjVfZUUxemhXc1l3a1lQWVVUN08xOExmOTRzYmdMMGVDZUctbHFzU1Fwa1hUNTZHeDlSTlBlSnBOdVVyNGRPSTE2OHVTUTh3?oc=5</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2275,1231 +2275,21 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K34" s="1" t="n">
-        <v>46079.24236111111</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Local Town Wertheim German</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Main-Spessart: Polizei nimmt falsche Spendensammler fest - Radio Gong Würzburg</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Main-Spessart: Police arrest fake fundraisers - Radio Gong Würzburg</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Wed, 25 Feb 2026 15:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxQTlBoR3NYVDh4bkpwUHhmLXdlcHZpZ0VpLVE4eW1WYTBiajFMMHdhMmF0a2xCcllSb0VrT0d4eUUxVFo3aXh5ck1uQkkzUkl5VzdQQWVxNVNIUXM3U3dqQUl4X3hVQ3dYWFJqYkJjRm1YWFJ1V24wYXVJWTVtQm1ydDNEVEU2bXZBZjVQejBfcktqcE0?oc=5</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K35" s="1" t="n">
-        <v>46078.625</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Local Town Wertheim German</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Herrmann: Wechsel an der Spitze des Polizeipräsidiums Unterfranken - aschaffenburg.news</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Herrmann: Change at the top of the Lower Franconia police headquarters - aschaffenburg.news</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Wed, 25 Feb 2026 12:29:43 GMT</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPblZ5bjRhZmwxUjdVbElESmtfSkxtSmZyZmpKWDc3ekVUTXYwWmRjMVk2aDVGc0FRa0YtcmNudzJVdUNSc3EzSk8zeWhvSGdJTkRTQzA1SDdCbDBGRUZ4RjU5WkpGYXhHb3ZpUUFrVEtrZWJLNkpfM1g5QzhSQTZaeWE2Tmk4cmJNTWxscS1KYkFXMTRrR0hFa3YwcDB1RmtSTl9OM2RsNXZrcnFZdFBZ?oc=5</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K36" s="1" t="n">
-        <v>46078.52063657407</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Local Town Wertheim German</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Unterfranken: Mehr Verletzte auf den Straßen 2025 - Charivari Würzburg</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Lower Franconia: More injured people on the roads 2025 - Charivari Würzburg</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Thu, 26 Feb 2026 04:29:00 GMT</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOdVBiVzJ1Unh3MlJlYlpITGhBSTgtN3FmcUZFVHVCT3pCRm9kRUp1a0hGYXRlOFpHRmZzRkhlLXotOHJydDRSOENkQUdLa2tRMEMtSUZ1aDVqYlhuY251b2VPWEhHRGp5Qmw2dmVPRklWR2x6bV9xNHpyT1FFRDZ0VkdlVmVXTUUzYWRPVHJjVQ?oc=5</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K37" s="1" t="n">
-        <v>46079.18680555555</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Local Town Wertheim German</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Würzburg/Kitzingen: Zahlreiche Anrufe von Betrügern in Mainfranken: Falscher Arzt oder Polizist ruft an - Main-Post</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Würzburg/Kitzingen: Numerous calls from fraudsters in Mainfranken: Fake doctor or police officer calls - Main-Post</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Wed, 25 Feb 2026 13:06:09 GMT</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi-gFBVV95cUxQczVZTXVxaElDRlgtcGl3emlESGNYdFh5LW1fSlFMcmNSZXZNZlBGeEYwOFA3N0pVR1ZLeEpsZ3NpejdXa29VYThvblBRa2xUWWg1T0JWdXE1RkVydERCQ3hqTHlhelpBWU5hREp5U1BGMG5jZlJHYlc3MVJ5R0oyekliUF96Ml8ySFdPYzBjeGl6dUZLZUt3b21FbEdDN1cyQklCc1hHbHFVc1BXWHBnV2ZEaURidlhnV0pMSzBHelRWbHRSOFdna3puWVpuV3QyZ1ppaHpxMTNjVEtZbmZIaGZ5LW9OZi1tS2lYa1JIeE9QVGR3RUtoQXJB?oc=5</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K38" s="1" t="n">
-        <v>46078.5459375</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Local Town Wertheim German</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Würzburg und Kitzingen: Zahlreiche Fälle von Telefonbetrug - inFranken.de</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Würzburg and Kitzingen: Numerous cases of telephone fraud - inFranken.de</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Wed, 25 Feb 2026 12:14:00 GMT</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxNUnhNMDF3d3l3S0tqeWlNdEJraVlaaXVXSTFBdFFrcUIzNHRXcEYtcFNoLVlVS3BMZzFNY1hjWlQ5b183eGFYdHVrUDhvbG9CWC1HTGhibTlRRXhrMnlLMUlBWFMxY3l6MUpuc3VJdUtkSGh2R2ExOEp1d2hEdUpJX2M0RklFeHVGOVRZUkF6V0lES1Z4Y0s1LTVHb1dXdGp5bVBESVNDcnFaalV5MTJyN01OUW5odldvaGRB0gG7AUFVX3lxTE1SeE0wMXd3eXdLS2p5aU10QmtpWVppdVdJMUF0UWtxQjM0dFdwRi1wU2gtWVVLcExnMU1jWGNaVDlvXzd4YVh0dWtQOG9sb0JYLUdMaGJtOVFFeGsyeUsxSUFYUzFjeXoxSm5zdUl1S2RIaHZHYTE4SnV3aER1SklfYzRGSUV4dUY5VFlSQXpXSURLVnhjSzUtNUdvV1d0anltUERJU0NycVpqVXkxMnI3TU5Rbmh2V29oZEE?oc=5</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K39" s="1" t="n">
-        <v>46078.50972222222</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Local Town Wertheim German</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Mainfranken: Trotz Warnung – Callcenterbetrüger wieder erfolgreich - Charivari Würzburg</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Mainfranken: Despite warnings – call center fraudsters successful again - Charivari Würzburg</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Wed, 25 Feb 2026 14:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxNZllFZWRoOW5GS1hkdmxITUFlenF6Nm1mYlVob01rN2Q3TEx3emlzRU1GaE0xVWE1UWJ2ZUVzLUlJS21pa3NyMkhVdmhXWWVJUzVLTUlMWEhlaFJjWEthZUJaYy1tYVVsRGhWOEZiWTJodGx3QWVwTGR1WlNkVEZKdkFQYkpOMVdUYTg2bHhCS0tGNmRKX1lKT1RvM1U2QkZfQXMw?oc=5</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K40" s="1" t="n">
-        <v>46078.58333333334</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Local Town Wertheim German</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Aschaffenburg: Schleierfahndung deckt mutmaßlichen Einbruchsdiebstahl auf - aschaffenburg.news</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Aschaffenburg: Veil manhunt uncovers suspected burglary - aschaffenburg.news</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Wed, 25 Feb 2026 16:14:47 GMT</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxNMVZ1dmtOc0hzMVJjWkIwV3ZvQ3dudHBncUZ1a2tSNjd4RGpjWEVXX0FVWWhHUDM4N21ub0s5NXZRcDBlMkZYdV9mNDNGT0hlbnd1bXoxeUo1UGx4UThmRUp1Vy14ZEpxeFBYNk5ocXM1NS1STXk2ZDRUSGFTUGFSNENtMUJJMFFQUW5QTDdGWlViWjMxR0hrVDV2UlVaWHRTYWRZN0lXeUlGRVRETEF4alBBRzEyTVk3TVM4?oc=5</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K41" s="1" t="n">
-        <v>46078.67693287037</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Local Town Wertheim German</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Nach Streitigkeit unter Unbekannten - Schaden an Glastür - aschaffenburg.news</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>After a dispute between strangers - damage to the glass door - aschaffenburg.news</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Wed, 25 Feb 2026 12:23:36 GMT</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOZnI4UW9KcU5SM0ltNnFWakhJeXpvdGgxdHQxMXRyR2RMak9objhiZkY2VUJUSEpvZkZXNHBzNm1zSzE2d2pvN0hFT0ZsbEhXZzN1N1hGMUo1MXhXY3BneVhWbjVMUEdjdnNyZU9WMGlMY2RmVFFzUlNQSW11VVdTcVJXdWduaUw5Q1ktWDY5b0xTcGZFSTh3ZEZxVmVDck1CZnVsRkV2LVYxMEFZUklBTEZwVGt1NEFtb1d0Um93eHI0eVJGVlBjTjFDOHF0QQ?oc=5</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K42" s="1" t="n">
-        <v>46078.51638888889</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Village Wertheim (fallback)</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>'What excellence looks like': FSU trustees extend president's contract - Tallahassee Democrat</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>'What excellence looks like': FSU trustees extend president's contract - Tallahassee Democrat</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Wed, 25 Feb 2026 20:54:00 GMT</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxQRlhsRjR3dXRfZ3ZhazdmX1FpVjZLbEJMdEdrZmNBVW05REpfNjBvR1JRb3dLUkVMNDlfekdzbkFEOWp4QVZIQ3A3eVV6cFNVb1Z4NTlMRWRDTUcycjQ2SDc3bU1KVDJMbkhSSHV3WmFvZUJ5ZVp6SnlNN2JIa210MHFkZW4weUVLM3J4aGViNXJiczVqNVlHWEw4aGkydXlBTlFnQ1BwMWNyU1YwM0hWUmFFejhjcjM3UlUwRGhXSk1VckduWlNtRFg2SmIxSXRodGZWMw?oc=5</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K43" s="1" t="n">
-        <v>46078.87083333333</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Village Wertheim (fallback)</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Jon Wertheim says Serena’s unfinished business at Wimbledon fuels speculation - Tennis Tonic</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Jon Wertheim says Serena’s unfinished business at Wimbledon fuels speculation - Tennis Tonic</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Wed, 25 Feb 2026 19:15:51 GMT</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOMjVOSGZuWVNUbzFTN0JLUWJaZVp0b2lzYnQwVkIzNFVHV1psZ2l2VXFRTEdlWXZ1ek1BYVpUMnA0dDlKMGVTTDZGRXNUVUhGekFTRExEelpJVHBIZ3d1TVN0Y2V5M1JwenBqUHVuc0NqY2dMaUFURmZrQmNxQUJnVGVTZ1BRSTk5cGZWY2FVU1hGcUx3bDVrZXc5OFdhcGdjaG91OHRvNzJGRzhKbks2bGZ2VUhSWjdRTlY1Qw?oc=5</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K44" s="1" t="n">
-        <v>46078.80267361111</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Local Town Ingolstadt German</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Bekifft auf der Autobahn: Polizei stoppt Autofahrer bei Holledau - Augsburger Allgemeine</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Stoned on the highway: Police stop drivers near Holledau - Augsburger Allgemeine</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Wed, 25 Feb 2026 09:11:53 GMT</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOTFVxM1lJN0FVcHFqLTRvNmdZME9mT1lwTVJpWFgzU0dVa0lWMWxrSlNMVzhUSjZCaFd2VlF2MG9CTHlsVUY2QTVGaENQdUFWSm95aWFzQmltUUZWaWs0S2hTS09COGdXOWdpdHBoYUhzQnZKdzJrUFprNWtCNi1IQUtvZnNCY1JuVUxOWUhJa0pKdmFscWFlcWtQWGZfVkNlMXZWNlJIRVdXa1Q3UHpONlhBYzFHVkZyVjFOeQ?oc=5</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K45" s="1" t="n">
-        <v>46078.38325231482</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Local Town Ingolstadt German</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Mit 2,4 Promille durch Lindach: 33-Jähriger verursacht Unfall und fährt davon - Augsburger Allgemeine</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>With 2.4 per mille through Lindach: 33-year-old causes accident and drives away - Augsburger Allgemeine</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Wed, 25 Feb 2026 08:56:42 GMT</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxPWVFzbGJzMDlkWXkzaFVmZzMwbzB2aVFpcFd4WFdMdFpfLUJ6OF9wWlg0NmJzOXdQVnd3RmQ4QXFrQ3hpUHl4QlExaWJyQWxkQ3JEZHlRQ0tQUW9vZ2R3ZVJadzJvUjdJZEk1X2ZNLU5DSmViTnd5aGhKbXVWaWRKcm5xQzJuOE1BVFFCUnFvZ1AzeGozWEtZczEyQmtDWUJNbjAyM21Vb2hWNUhMMjB0UFZkek5aWWFwT0VoVHJDTXNZUi12VW1DSFVsYmNMZw?oc=5</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K46" s="1" t="n">
-        <v>46078.37270833334</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Local Town Ingolstadt German</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Augsburg/Kempten/Lindau/Ingolstadt/Schwaben/Oberbayern - Am Donnerstag, Freitag und Samstag der verg - AD HOC NEWS</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Augsburg/Kempten/Lindau/Ingolstadt/Swabia/Upper Bavaria - On Thursday, Friday and Saturday the forg - AD HOC NEWS</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Wed, 25 Feb 2026 13:57:49 GMT</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQYjR2V0ExRkdOVEd3Y3lzZHY0YmhtWTFYUDM5NjNOZC1wODl0Zkx1bUlqSXRBTllWRGVyX2NIV0V4dnUtdHB1Z1RvT3dKSWg4MmtJeTJwSENObVNJbWJWNnpCUjhKdl9HbVZDeWQ0ZGlDYXZvUXd5YU8zSmN0VENnNGtDZmVOak5MamlDZzNDWTRlblpSMElxYWN5cV9XYkdfS2MwalFFdDI2RFIyOTVNUjB2U2lCenZjUHB3SjVB?oc=5</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K47" s="1" t="n">
-        <v>46078.58181712963</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Local Town Ingolstadt German</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Mann klaut Mountainbike – nun sitzt er im Gefängnis - Augsburger Allgemeine</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>Man steals mountain bike - now he's in prison - Augsburger Allgemeine</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Thu, 26 Feb 2026 07:11:33 GMT</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQdG9hTURrQkdSQzRveWFBV25xTlFHSEQtenktcG5YbFpqcFc3Mm5MUnA5WHNNTS1nNU91TGNxWkhoZzV6S09wSHlXUmU1Vk53RmlhSkNFR2tBY3ZTYVZjM3JVUTREX0REb0QwT2RGMjdFUF9GNXByNnJ6VkdDZDZ0d09NNlBtd3NlcWtEelNYWG0wMlYwa0VWTnpYS3ZMVEY5SXAyR1dxNEdLQ3EzSnhycUwwNA?oc=5</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K48" s="1" t="n">
-        <v>46079.2996875</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Local Town Ingolstadt German</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Illegales Fischen am Kapellbuck: Polizei Eichstätt sucht Zeugen - Augsburger Allgemeine</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Illegal fishing on the Kapellbuck: Eichstätt police are looking for witnesses - Augsburger Allgemeine</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Wed, 25 Feb 2026 13:13:05 GMT</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPYWZORTQxZWRJZTJtS0tIRGVmanhNMkcwWmhJMDNTWTFjeVViWXBTRmsyY25HRGx3dHQtSGxET3hFN0hBVElXU3VJdk5wOFoxaWtlSXBzbkV5eG9jYUh3T0NIaEF2SE5VdkdLT3pvdVJrVFVHYVcxN3I1UjJrR05hLXJWNUpNNndCRXF4Njlma3duNVQya0UtTV9GTGQxWGVnT2c4Vjd3R2p4VExvZjRNUlQ5YkxBWUhvZGc?oc=5</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K49" s="1" t="n">
-        <v>46078.55075231481</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Village Ingolstadt (fallback)</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Granit Stein set for WBA Continental super-middleweight title fight in May - British Boxing News</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Granit Stein set for WBA Continental super-middleweight title fight in May - British Boxing News</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>Wed, 25 Feb 2026 18:36:29 GMT</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE9lZ2ctMEFpRDZMTmthLVZSajRYal91QW5sM0xTVXhKU3otd2lyZDQ4U3V5SXJwbXpZd3d3Sk1wSnAyRDlaVkJXMjNzSkIxQXZkcV9fMDNKOG8xYmNOR0E4Qkd0Z2VsdkdjNFNoRGMtTTFfNGZXbk5vcVduSE0?oc=5</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K50" s="1" t="n">
-        <v>46078.77533564815</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>Village Ingolstadt (fallback)</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>German regulator spots competitive broadband markets in Munich, Cologne, Ingolstadt and Wolfsburg - Telecompaper</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>German regulator spots competitive broadband markets in Munich, Cologne, Ingolstadt and Wolfsburg - Telecompaper</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Wed, 25 Feb 2026 14:32:36 GMT</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxQdXl6S25JZHZnbmNhYTdUZGp1ZWdDejB4bnQ3T19lUHBNNHhNeWl6Z09BNVRlMGlha0NfZ1IzSGhXN0h5dGRYM1VUbEdWQXdBdVUteFdZdVRGTFRPTjUzSzRqdUN0RkNxRGg1cVlTeTBEclBIZ3JVU0I5Yk8zRGJMR3BVTUJZZnJtMlBwRjBlemkzLS1BMklNVDJaSlFEVnVTSzE5X0FhcWN0cWlDdWNjNEV5Y1NUaF9wRThkX1YyOHNPZUNvelBmOVpVSTZfaFFXVk9vTg?oc=5</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K51" s="1" t="n">
-        <v>46078.60597222222</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>Village Bicester Kildare</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester outlet" OR "Kildare outlet")</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Naas Book Club welcomes renowned Irish author to celebrate International Women’s Day - Ireland Live</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>Naas Book Club welcomes renowned Irish author to celebrate International Women’s Day - Ireland Live</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>Wed, 25 Feb 2026 18:35:15 GMT</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOTzZhUFpjUjNqTWRfNnhqcmR6MjJ2RGprVHVoX05QZE9SaHUxUmJib3R2cElHcUJpZmpDcEUzbXowYW9fUGRuTmpHV3ZHSWY2dDM3dU1ycEY3QXlmM3NpdXpXNHc3RG0wVmtWUmJOM2VKYzR6dGZFS2xjZlVEc21zbTBDYkZ0RHpYZVRxdms2N2tkRk1EbXg1LUJrcTNDQjFqWE9oYVM3UzBsRGYtUzFFQTZSMXJrTnhjSHdYeFVlYU53M2FHeGthbzFxUVJ2LTEwMUY4dFpTc1c?oc=5</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K52" s="1" t="n">
-        <v>46078.77447916667</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Village Bicester Kildare</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester outlet" OR "Kildare outlet")</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>3,200 people per GP in Kildare 'unsustainable' - TD - Ireland Live</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>3,200 people per GP in Kildare 'unsustainable' - TD - Ireland Live</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Wed, 25 Feb 2026 21:40:38 GMT</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPd09GbXg4WGJMWXRLTnRudjgxVVlMcEhtcGt3a0h3WHhoMktNQnRPNDc0ckVwdjFYOGdHWnB4UVk0eUMyYmM2Q3ZpWXpIeUxVWDItWVZKbjZyMFl0SUhHUG1feWY3TWtscHk4NERHQnBhMWNPRG9OcVhlcjh0VGJvT0VndDVZTUR1WmZTVTZQZ252NVBBRVFxcDZsTTRWUnMtazdWMTBDQlY?oc=5</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K53" s="1" t="n">
-        <v>46078.90321759259</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Village Bicester Kildare</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester outlet" OR "Kildare outlet")</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Steal Her Style: Karen Koster's chic Sandro sundress as she reunites with Alan Hughes - MSN</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>Steal Her Style: Karen Koster's chic Sandro sundress as she reunites with Alan Hughes - MSN</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>Wed, 25 Feb 2026 09:35:11 GMT</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi7wJBVV95cUxORGlaU2xKMmxhdmZVS2EyNk9odjNmQ2NNUmQtY3ZhWW1RODN1N1AyS0xZZzVGWVlud1kzOUJ1RzQzZnVTcmRDMlY5Q0hUNEp2aldieUV4U1dQMHIwUGtnVndLV1lDY3VkUWtjNFZvVEFKbURFdHNRMjNTVWtSRHFvUmlaSXdYeWZWdmlGVDFMdDhZcjRqUXRzdEtqNTF6ZWxiYXRpclhnYzRwVUQ2Sm5xUFcxYlhNUktLU2JrZDZkNE5MVWJudjVyVVQtN09WTHMzNFBFSC1LRXZ0NzFmV2tibWctazVVX1c2RS1HemJNb3pteDFEa2Q4RWtDUks3TTBWUkJmN1A5dnJ4MWRhcGxObWtLSzZHTEw3d1UzV0M5NWp5cTNPY1JKdTdnQVJGRlB4T2xzVktIN0UtVU9uaDBnUGRldm12YjQ0elh5UzM3cXpZYjJqY0M4clVlM3VEdXdKQXhJdkNKblluQ0hHZEgw?oc=5</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K54" s="1" t="n">
-        <v>46078.39943287037</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>High Level City UK Ireland</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>("London" OR "Dublin") AND ("terror" OR "bomb threat" OR "suspicious package" OR "police operation" OR "counter terrorism" OR "stabbing attack" OR "shooting incident") AND -"bomb squad" AND -film AND -movie AND -filming AND -"New London" AND -Connecticut</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>What are school officials instructed to do (and not do) amid a bomb threat? - London Free Press</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>What are school officials instructed to do (and not do) amid a bomb threat? - London Free Press</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Wed, 25 Feb 2026 19:49:14 GMT</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNbXc2MTViTVZjQUpDd1FxVy16MXdnZ2NjV1ZEYkQ5VDd4YTVLMWFob09SeS1fT3Z6a3lDb3pQajI5NWJ0c2I3VGVTbGZnTUZfREMzNnpfY3I3RGhndktPaG54YW5tNXotclI3VTZER3VjTVlod3ZUMElveUpLNlVMOERmZXVuRGF5YkFDMWxwdHhOU3B3MHg0eHloYlpQSGxi?oc=5</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K55" s="1" t="n">
-        <v>46078.82585648148</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>Local Town Fidenza English</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>("Fidenza outlet" OR "Designer Outlet Fidenza" OR "Fidenza Village" OR "Parma" OR "Piacenza" OR "Cremona") AND (protest OR bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR evacuation OR "police operation") AND -football AND -transfer</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Man shot, killed by Parma police identified - FOX 8 News</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>Man shot, killed by Parma police identified - FOX 8 News</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Wed, 25 Feb 2026 14:49:58 GMT</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTFBES0ZWdG1QWXpjTVVqVVRoNGdzN1lDWXhRQ1pPX2lMdW1WdFhnSklSZUlGQmV1ck9KUXA1Y05NYUdjSmFDd2sxYl84aG9DZmw1elowS3BQNklmV0VQY2g0dHNtVEtDS0ZJVlhkSDU1UXpYVzDSAXhBVV95cUxPUGZsdmZUNUNlS3hJQ3JsdzVHc2VZQXRULXY4TlUyV0dqYmVMLTZFT0NpQ1pWX2NHc09tOGpyVDVIb0JaelI5N1ljb2gxZG5KOHpybTVyUGpvVVRWdlItQ0dBX0NNZnBfUGpYS1Q0anRWQUs5WEgwWTM?oc=5</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K56" s="1" t="n">
-        <v>46078.61803240741</v>
+        <v>46079.53194444445</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-02-27 07:53 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:K47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,32 +480,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Brand Protest</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Gucci" OR "Ralph Lauren" OR "Dior" OR "Armani" OR "Louis Vuitton" OR "Burberry" OR "Prada" OR "Nike" OR "Canada Goose" OR "Hugo Boss" OR "Moncler" OR "Saint Laurent" OR "Loro Piana" OR "Lacoste" OR "Versace" OR "Jimmy Choo" OR "Michael Kors" OR "Missoni" OR "Kiton" OR "Aquazzura" OR "Tumi") AND ("protest" OR "animal rights" OR "fur free" OR "PETA" OR "activist") AND -BAFTA AND -"red carpet" AND -"awards" AND -"wears" AND -"dressed in"</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Uitbaatster van bekend Antwerps café Kiebooms klaagt drugsoverlast aan: "Dealen en gebruiken gebeurt open en bloot" - VRT</t>
+          <t>Dior's "Coquettecore" Bow Bag Is The It Accessory Of Spring 2026 - Bustle</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Owner of the well-known Antwerp café Kiebooms complains about drug nuisance: "Dealing and using happens openly" - VRT</t>
+          <t>Dior's "Coquettecore" Bow Bag Is The It Accessory Of Spring 2026 - Bustle</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 14:08:20 GMT</t>
+          <t>Thu, 26 Feb 2026 13:01:25 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNbjR1dnVXUzQxV292QzN3LTZNTWZpM1E1LWhoX3VmNmlZQk1OSTlIaUhwNFM5MEJzcnA3U0xPd1NwSGVHSXVGb3Y0RFJZVU5jd1V6ZjhvTUttTjJKY2hBRzkyR3l2UFJWeDhGNHR2enFvMVNfMzhXdFJNMDktRXA1b1hSU1dDdzViTEthMmtMeThENE1HZjIxbzN5RQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiY0FVX3lxTE1fZUMzM1FrR2c3cWphemRwVzExb2h2dUprMXVmcFRXTmxBTGVHVWlva0lLUk5ZdGM3ZUpFTV94TzkwOExYdnc3T3Y0VXFGTkpJaVh5UUhnYWlQell0REJRNzJkTQ?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -515,52 +515,52 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46079.58912037037</v>
+        <v>46079.54265046296</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Schoten gelost in Brusselse Matongewijk: één gewonde - HLN</t>
+          <t>Retail, AI, IT Sectors Ignite Opportunities Amidst Valuation Puzzles - Whalesbook</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Shots fired in Brussels' Matonge district: one injured - HLN</t>
+          <t>Retail, AI, IT Sectors Ignite Opportunities Amidst Valuation Puzzles - Whalesbook</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 12:45:26 GMT</t>
+          <t>Fri, 27 Feb 2026 07:09:21 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOTzdTWXEyQUpvR2otOTlmaHgxMDNPRGNuMWpPZlNrVU5iZ1dRM0JCbmZmM09EYXhVTk5jRzl1T1RtN3lPbEthUzh5djFEYS1PRFZuekJKQ0pWZWRtLTlTd0UtSUoxcDgwTmJFMUZFVl9HNV9ic3Foelh5Xy1XWmdSV3phMHczblQ0eEd4ZWhSRVJtdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxPRnNrM19RZVV2VG9IT01sa215ZE9jbUNSUFFrYVhBbkVQMllGQ1o2ZjE1ejU1b05BT1lrNEloaHpIV0hvZjNCeFVCazhIcEI5WEgzalU3Q05wSmVrbEQzUU1NUUsycnpSY2R0aUxpVWplNkFtaVlDeks1RFlMSk1tUHZ3WEZWT3c0MDVXSFFpdTR0cVUzZGNJNDNpbmlXVTVLa2k5VllKTl91bGJ2cVU3Q1FTNVQwX3FxeDN3ck5JaWxVejdtRFotSjFzN3hnT0ZKY3c?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -570,52 +570,52 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46079.53155092592</v>
+        <v>46080.29815972222</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>PETA Broad Search</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>"PETA" AND ("Italy" OR "UK" OR "Germany" OR "Belgium" OR "Spain" OR "France") AND ("fashion" OR "designer" OR "outlet" OR "luxury retail" OR "shopping village") AND (protest OR rally OR demonstration OR campaign OR action)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Persoon gewond na schietpartij in Matongewijk - BRUZZ</t>
+          <t>Italy Fashion Protest - the-messenger.com</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Person injured after shooting in Matongewijk - BRUZZ</t>
+          <t>Italy Fashion Protest - the-messenger.com</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 09:21:26 GMT</t>
+          <t>Thu, 26 Feb 2026 20:16:44 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxQdTk5YW5kRE9iSXBpLVJrWnpfMGFNRkQtTGxIem1Dek93VlcwN25fUkhXaHIwRmJyaXVwTE10Ml9KdC1iN0FodE5XLTdjbHpNYmxYZHF0bkNVZzB6TWRKck50bWV2U2V6RzMwSF9TY1Rrb0FjTnU2TTJpYWNlSTRIV2dGaGVRQlN5bzdmMXN1NTh3WXoxRXZsQ2R3bmtJX3R6d1J5d3R2WQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxPQkxKREQ3LWFXRTV0dlpHTWJsVHJwZnBuMmdNUTFTbFctbzhjRE12cUNzUUlUQlVJTzdVSjhZZDZKNkR3MEJWczBUUUR6VFNlalJKRWwyUERadTE4Vm84Z2g3bkYzRTEwVmtwUHRCNWJHa3N4TWRjWFp0N2s5T01LMkVmNmNlaVprR3d6RzBLV1NCdw?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -625,52 +625,52 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46079.38988425926</v>
+        <v>46079.8449537037</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>London Marylebone Incident (fallback)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("London Marylebone" OR "Marylebone station")</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Gewonde bij schietpartij in winkelgalerij in Matongewijk - Nieuwsblad</t>
+          <t>Londoners walk from Marylebone to Baker Street to see if it's quicker than Bakerloo line - My London</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Injured in shooting in shopping arcade in Matongewijk - Nieuwsblad</t>
+          <t>Londoners walk from Marylebone to Baker Street to see if it's quicker than Bakerloo line - My London</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 10:14:13 GMT</t>
+          <t>Fri, 27 Feb 2026 07:08:21 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPLTNMd2RpdjJKWC02d2dwZDZsM21qb2VDTjBPeUszdElIQlFBOWU2LS1xYzhxeWkyV3ZFMG5sakpDSGxhVk51WVhfRWt3bzVJeUlRNnAzV0pEUXdWeEVYYmJSRF9iUWxuSGtnTnNRdlNQS0ZPNWRvZ1liaDYtWnFRZ3BrYUlRVXB2cXd5UVpJYWN3eUpSS2F4STMtdk5QaHdqWEtSa0FXT2lJRWVta2x5Tzd5QnRaS2NWXzVj?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxOUlRKbW5JSzA4b0FuVTVsTVNRbUJwWUVSV3hndDRUM1JPUzZIVlBXbllqNFJydDI0Y056b1E0MnhPVVU5d2RFSUw3aXpWMHBnUGJoeEF6dkJNa2NLV3RMUmFJendCX2Z6MFNZaXBRa1YwT0NjUFNuNWIwRW1fY21nTFV6TERycERIQzduWW1VR096dDhXZHZ4NERna9IBoAFBVV95cUxOd1hLM3NZQUV5TDB6eFkwd19KbEZQUGhyVVBCcTFiLXRmSTF6QzlsTzlpNFZGbWpDbC12RkJtd254TUxJQW1qY3p3RmNCbl9UVFFMQkpCOW50WXNOV3ZXLUlLVkxsX1JyS1pWTzRuUzczY0Rsbml6UlA0VWRfNk1fMlkzbndJSTFpYktDVXFrTHZrNktKY295QXVnSUNBZGdt?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -680,21 +680,21 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46079.42653935185</v>
+        <v>46080.29746527778</v>
       </c>
     </row>
     <row r="6">
@@ -710,22 +710,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Minderjarige verdachte steekpartij Mol vrij onder voorwaarden: nog een jongere in gesloten instelling - GVA</t>
+          <t>Uitbaatster van bekend Antwerps café Kiebooms klaagt drugsoverlast aan: "Dealen en gebruiken gebeurt open en bloot" - VRT</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Minor suspected of stabbing Mole released under conditions: another young person in a closed institution - GVA</t>
+          <t>Owner of the well-known Antwerp café Kiebooms complains about drug nuisance: "Dealing and using happens openly" - VRT</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 09:41:46 GMT</t>
+          <t>Thu, 26 Feb 2026 14:08:20 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8wFBVV95cUxQUzdtUjdYaEhfaWtqS01WbGMwXzZIdFZZX29rNGRNTHFYYm5lbDJaM3F3aE0zM2ctaGM4VlJTU2RDYVVnVERjejBXZnF4eXM1OHAxN2FYaGw2cmxsWFNYOW1mRHdrMHhDRzNRR3lRX1RkemhyNkswYXE3NllLS1VwdVhZN2Y5eEtEZnlCMVRUUVNZNGc3MjM4a09SU0dsbWdfQ3NoUlVOd3RxZ1NWSGhmN1VQdjZRelBaeXdreHFzQ1ZPUmtfY1pPNXlLdG16Mm0wODI3N1BOTWx4VDk0aEVzcURKSDRIUlhQQW5qWjBodXVMR3c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNbjR1dnVXUzQxV292QzN3LTZNTWZpM1E1LWhoX3VmNmlZQk1OSTlIaUhwNFM5MEJzcnA3U0xPd1NwSGVHSXVGb3Y0RFJZVU5jd1V6ZjhvTUttTjJKY2hBRzkyR3l2UFJWeDhGNHR2enFvMVNfMzhXdFJNMDktRXA1b1hSU1dDdzViTEthMmtMeThENE1HZjIxbzN5RQ?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46079.40400462963</v>
+        <v>46079.58912037037</v>
       </c>
     </row>
     <row r="7">
@@ -765,22 +765,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Medewerkers Arnhems autobedrijf gewond na schietpartij, burgemeester spreekt van ‘afschuwelijke daad’ - Automotive Online</t>
+          <t>Eén keer schieten kost 1 miljoen, het systeem zelf 1,1 miljard: 10 vragen over de luchtafweer voor de Antwerpse haven - GVA</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Employees of Arnhem car company injured after shooting, mayor speaks of 'horrible act' - Automotive Online</t>
+          <t>One shot costs 1 million, the system itself 1.1 billion: 10 questions about the anti-aircraft defense for the port of Antwerp - GVA</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 12:19:43 GMT</t>
+          <t>Fri, 27 Feb 2026 00:56:00 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxOWXF3QnBVS3NHa2xIQllYQmpCc3VBNDQtVVpfbjVlR2EtVTlfSjh3b2RMemRLNlJfeWxlT2ZwRzhaaUdvUU9EQTF4OGw4N044TzhpUnFTY2tabWZsNkpadlZfYzdGQU5Gd0VmQkFGaWxWVkpINUJNaWE5SWhyUWIwbzctOUh5SklRWTVzYjZMaGVMX0wzTU9fVHhtTjJ2LWYzVkJiOEVhOG9Fc0JlSDllbTJJVllNQlNYOWJndTV2ZmlaZWNIQlU2djh4RWViZmp4RGtRZmY0c2FaSDR6ak0zZE1tcUdtNHRxdmc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxPWnRubWNTTk9tRUhYRk56Ml9telpneWhLa21TX3JZLVZtQkNLOUpZeGRkdm1iWjhlTDE4MFFwZDNQWnB4Mno4bmhyTzhFM0puZ1l6Q1BXYXBlNTZTTDUtQkNZRDZJbHY1cGpSbXBmUHRmZEM5WGJaODdVRjJSajBTWWZ3VGkxdFFOcFc2dVFkWkE5djJQYzFnU0NuQllmN1UwcW9DSjI4a2hSTXVnOWZUbmNJWmkxVUJtYUhadS1vRUZkNEtJNnQwM21WTkc5b0hCME1fcU1kMTBYUG4wZUJUSWJKd0ZmeEdVZ3RCSkd5UFM?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46079.51369212963</v>
+        <v>46080.03888888889</v>
       </c>
     </row>
     <row r="8">
@@ -820,22 +820,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Tot 28 maanden cel gevraagd voor schietpartij aan Truiense supermarkt - Nieuwsblad</t>
+          <t>Persoon gewond na schietpartij in Matongewijk - BRUZZ</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Up to 28 months in prison asked for shooting at Truiense supermarket - Nieuwsblad</t>
+          <t>Person injured after shooting in Matongewijk - BRUZZ</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 11:31:27 GMT</t>
+          <t>Thu, 26 Feb 2026 09:21:26 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxPN2JSbkd1NEhpSnNwcjZzdUVLWi1IYktjdF9DV1E4STZSVEIzRnBDV0d3cVFiTDRPNHQ1NE5IWWZ1bzQ5TEdfd1lIVTJWYmppNEI4OEEyWEdsd2M5UjY2TjFmdnVSdFY0bDF2Z213czdNNU1FSGlCT0NSejg3REFyZnhwWmVlemJfRmhhNEVmMjVfSXVqdkJUYlotQzFUX0Rkek5Zb3FMQTFta0JGanJxc0s1cHMxcHlYY2lidHNlWDBOcUY2UlYtUnV2Qjd2cXo2cFNR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxQdTk5YW5kRE9iSXBpLVJrWnpfMGFNRkQtTGxIem1Dek93VlcwN25fUkhXaHIwRmJyaXVwTE10Ml9KdC1iN0FodE5XLTdjbHpNYmxYZHF0bkNVZzB6TWRKck50bWV2U2V6RzMwSF9TY1Rrb0FjTnU2TTJpYWNlSTRIV2dGaGVRQlN5bzdmMXN1NTh3WXoxRXZsQ2R3bmtJX3R6d1J5d3R2WQ?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46079.48017361111</v>
+        <v>46079.38988425926</v>
       </c>
     </row>
     <row r="9">
@@ -875,22 +875,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Na beroep blijft hoofdverdachte taximoord Geel in de cel - Nieuwsblad</t>
+          <t>Schoten gelost in Matongewijk in Brussel: één gewonde - HLN</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>After appeal, main suspect in Geel taxi murder remains in jail - Nieuwsblad</t>
+          <t>Shots fired in Matonge district in Brussels: one injured - HLN</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 09:02:03 GMT</t>
+          <t>Thu, 26 Feb 2026 16:35:25 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPb0M1NGtlOE13MFpPNE43ZHRzQXhoLW1TWmRmMXpNYVNvN2lGSUdYT0dZRHVGUEpGdF9vdER6bTlTcTlIaE1MZ3N4V2ozcXcwS3BrMTlqQ1JiQzR1cWNxZExmOTFBRzFQV3NjV0ZNckV6NUZpZVZGVUw4YkFPaDRrZFpIWURXYzYyaEtBTFY0RjNETXMwdHpVTGVVUk1YWUllTTgxOC11M1BoWFFFOW0xU3NhVk5GYWRFV09DRGtzUjl5SjA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxQMjc5LWZNdlE2Y2N3Z1ptdERVOEJoRVowLWZrcUFPdFMwZ0JDRGM3VldhV3pGLWZrQ3BGXzgxSVZnVlBtaWZEbUo2eE1KWUN5T2JBVi1jZ3h6WEs0cF9wYmJ0ekJNRmU1TmlhdWpjWVdnck8xN1dTcXc3N19KUW1zdE1iTkU1Tmp2NWdOMmxUc2JUcmc?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -914,7 +914,7 @@
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46079.37642361111</v>
+        <v>46079.69126157407</v>
       </c>
     </row>
     <row r="10">
@@ -930,22 +930,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>212 explosies door lachgas in verbrandingsoven Isvag: “Afval wordt nu voorgesorteerd om incidenten te beperken” - Nieuwsblad</t>
+          <t>Gewonde bij schietpartij in winkelgalerij in Matongewijk - Nieuwsblad</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>212 explosions due to nitrous oxide in Isvag incinerator: “Waste is now pre-sorted to limit incidents” - Nieuwsblad</t>
+          <t>Injured in shooting in shopping arcade in Matongewijk - Nieuwsblad</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 10:08:21 GMT</t>
+          <t>Thu, 26 Feb 2026 10:14:13 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimwJBVV95cUxNV0g1Z2lGMmFVU3Ntc1praGtDVmJpb2FoT01QOE1kWHRvbDVGNjNKdXRNVUw1dVZHZXBpNVB0ck5Fa2luZ1lYOC1OTjdrNDJWRkhndjBkV2JjVXFfWC11R1N2Z2RjYy1rX1lFWjJKY0tMREZqV3laV3c5cThwMzEya3RuMjNQV0hTUmVpcDhhWERiaGh0eHVIN3VRR3hKcGNMTndkeUUydUlKV0d6VnJNTW4zRUcyM2U2NjdvY1JYeHRkOHNzcUJxRE4tLVZIMU5SX0RUeUlIMDZEWUptZHZNT0NPejhwcm1oazRNUTlEVloyeEd4aU15OTVicGF5Wk9jRjdoWjYtaXpNMnJkR3NDV1VsbUN6eWpRNzY4?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPLTNMd2RpdjJKWC02d2dwZDZsM21qb2VDTjBPeUszdElIQlFBOWU2LS1xYzhxeWkyV3ZFMG5sakpDSGxhVk51WVhfRWt3bzVJeUlRNnAzV0pEUXdWeEVYYmJSRF9iUWxuSGtnTnNRdlNQS0ZPNWRvZ1liaDYtWnFRZ3BrYUlRVXB2cXd5UVpJYWN3eUpSS2F4STMtdk5QaHdqWEtSa0FXT2lJRWVta2x5Tzd5QnRaS2NWXzVj?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -969,38 +969,38 @@
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46079.42246527778</v>
+        <v>46079.42653935185</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Ukraine war latest: Russia makes Moscow 'terrorist attack' claim as talks continue in Geneva - Sky News</t>
+          <t>Politie onderzoekt mogelijke schietpartij in Haelen, arrestaties bij tankstation Born - De Limburger</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Ukraine war latest: Russia makes Moscow 'terrorist attack' claim as talks continue in Geneva - Sky News</t>
+          <t>Police investigate possible shooting in Haelen, arrests at Born - De Limburger gas station</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 07:58:52 GMT</t>
+          <t>Fri, 27 Feb 2026 05:33:38 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxOenB6YjJ4YVM4bU1jR2hreUI3UmNwa2tfUTU4VVNUVm9tM2hycVFnLWtYN0FBZkpDNEtrRWlDWk5KVW96QmVPdVRoVEptZ0JOWllFRDc1cWY1S1hiLUxsSnFTRms5MjZlNWZPdXBHV0RCeENQejlZc2N6RUlJekYwQnBPU28tN3lxc2UyZWlVZUZGR2ZFeGVVb19EcVpWMHBPUFUxV1RBc3NzQW5SNEtJNEJKOVZYTi1PcmRYcTdHenBUbDQwSXBfeUpkLVVtbVJQVWdJYk5Pc20wZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxQZjNhYTAzWG9FSDhiU1huaVVyQTMtcU54SjZJNDNBM19ORk9rekRveVI3T0ZhWU1DbTFpdzhWaTduNEtaZnQ2SFM3TTk5TXNFZU5ZTm44UTZXdnN0a184bTdXbHhSakgwODVtQnZKQlNNTXJNSFFmZ2dUMDRfTXRiZzBTVG1MSWFLNnduREZKeXZWMWUwb0RPQzRBVHpibUxKWmExeERVcV9qYnhXdWF1UjhRRHRrTktFTFdrT0VSejJMSFVoNWRfNUFWNzI1dTB3M21lb2ZoVnplMXc3?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1020,42 +1020,42 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46079.3325462963</v>
+        <v>46080.23168981481</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Bomb Threats Spark Chaos in West Bengal's Postal Services - Devdiscourse</t>
+          <t>Duitse zakenkrant: BMW en Brussel in gesprek over lagere importtarieven op Mini’s uit China - Automotive Online</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Bomb Threats Spark Chaos in West Bengal's Postal Services - Devdiscourse</t>
+          <t>German business newspaper: BMW and Brussels in discussions about lower import tariffs on Minis from China - Automotive Online</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 08:19:46 GMT</t>
+          <t>Thu, 26 Feb 2026 11:09:53 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOVnE4aW04dHlhVGIxQl9HdVctMks4SnJhQmgxWXpqd1h5WmFiU0VtRUtROTdDcmM5cmp2b2R5Q0cxcm1SYVYwdlJTbFhLS3hlQ0piSGJyZWc3UkJsTl9SdDNZSWUwU2FmZFpEQmtVcGU3Z1prNVc1SHdBX0Z5QTlzcnFOZHE4ZFoyQlQ1WmIzeDRWM1VzaUwwUjRDYWlQRkh1OW5YS0JRUU9jSFBPeUJBaU9ORzRTQdIBtgFBVV95cUxOVnE4aW04dHlhVGIxQl9HdVctMks4SnJhQmgxWXpqd1h5WmFiU0VtRUtROTdDcmM5cmp2b2R5Q0cxcm1SYVYwdlJTbFhLS3hlQ0piSGJyZWc3UkJsTl9SdDNZSWUwU2FmZFpEQmtVcGU3Z1prNVc1SHdBX0Z5QTlzcnFOZHE4ZFoyQlQ1WmIzeDRWM1VzaUwwUjRDYWlQRkh1OW5YS0JRUU9jSFBPeUJBaU9ORzRTQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxPMUJBb1ZsZXVwMDRreWdUUGxRWmxKUl9OY3ZhdVZDNDZVWmxDSjBLWncxM0pjdGRYN2hCV1hPLWpUWlY0SXU1MkgzdTJVMVo2Zk1kbTVyVktFRVZUcWRlTGVKbGpabHEzYlVkVGZvRzRtWFlyWlA1Ynh2T3AxQkVqa1hidDFYaGRBTUZjam5JVkdoSTJXUWxuOXo0LU9NUmR4UEl4UnExbVFqQThZZlQyX3hSbzdIZEJkYV9NM3BEa3pnMmcxMi1BUkd3Y3FiU0hBdjA3UzVXUU9lbFN6a0E?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1075,42 +1075,42 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46079.34706018519</v>
+        <v>46079.46519675926</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>South Korea and UAE Forge $35 Billion Defence Alliance - Devdiscourse</t>
+          <t>Bedrijvenpark in Temse al hele dag afgesloten na schietpartij: “Poort geramd en geschoten met kalasjnikovs” - HLN</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>South Korea and UAE Forge $35 Billion Defence Alliance - Devdiscourse</t>
+          <t>Business park in Temse closed all day after shooting: “Gate rammed and shot with Kalashnikovs” - HLN</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 08:34:35 GMT</t>
+          <t>Thu, 26 Feb 2026 15:10:19 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPRVFodHBSSXVzeXE4ZG5mOFdiRFRISG1KOHBqcVRnOS1nZFhEZ2RrQUJhX3piNkRQOG5lN1R6dUNZV1RTRC1BTHJxTHlDbE5BSDZnQTZHaThSaWxiajZRX1lzbTVVSEExYjdXM1YxRVdTWmhBdER4eXZTZG5ySTBLRFFyeVd1MW9fUmNDVFYyalNKcy13NERDNk52SWVJaFlYTWY3emVLd2xRUFBuYVVQRtIBsAFBVV95cUxPRVFodHBSSXVzeXE4ZG5mOFdiRFRISG1KOHBqcVRnOS1nZFhEZ2RrQUJhX3piNkRQOG5lN1R6dUNZV1RTRC1BTHJxTHlDbE5BSDZnQTZHaThSaWxiajZRX1lzbTVVSEExYjdXM1YxRVdTWmhBdER4eXZTZG5ySTBLRFFyeVd1MW9fUmNDVFYyalNKcy13NERDNk52SWVJaFlYTWY3emVLd2xRUFBuYVVQRg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxPVHpDdGFjbzN6SG5EeUpzaVF0LXFhNjZRVXNwYWxwRWRBZGJjZ1RfenRqaEN3azBXM1RRWFVkVXVHR2FDajI2ZmtvNEFaSHdmSUQzMkdDYVc5WU1qdV9xMHhQd25Jdjk3V1J2RTJJRUtUTTJMNXJhNzlJUVhzYzFkVXVTd2I0d2NyUkN1TU01MVlkMndOSWNLLWdmZFBoWDRQMzRYQzNVaWE5LXhfVHZ2Ujl4VVFYSm1faXhyRUo1Tzc1X1hQWV8zakF6dVh5QXZmT0dNaHd3?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1130,42 +1130,42 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46079.35734953704</v>
+        <v>46079.63216435185</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>The Cost of Defending NATO's Eastern Flank - Devdiscourse</t>
+          <t>Minderjarige verdachte steekpartij Mol vrij onder voorwaarden: nog een jongere in gesloten instelling - GVA</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>The Cost of Defending NATO's Eastern Flank - Devdiscourse</t>
+          <t>Minor suspected of stabbing Mole released under conditions: another young person in a closed institution - GVA</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 08:24:37 GMT</t>
+          <t>Thu, 26 Feb 2026 09:41:46 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxPMVJZbjdoMTM0VXZfSmJTOWdvUFVpODRYcUNybzA0WDZNWlg2NDlCek1fVFRib0J5dF9UR2N0SHJqV0xIUzl6MlpoQW1Da2RhaTF5UEozcnVaRVdYV20wTjEzNUc0cUJfWmVfUnBDQlJYdGhaOFhRMm12clhiTjBCX09OVjJFQUY3VzJCMlJXVHJRTG1YeEN2X1FpVjIyWGtxS0HSAaIBQVVfeXFMTzFSWW43aDEzNFV2X0piUzlnb1BVaTg0WHFDcm8wNFg2TVpYNjQ5QnpNX1RUYm9CeXRfVEdjdEhyaldMSFM5ejJaaEFtQ2tkYWkxeVBKM3J1WkVXWFdtME4xMzVHNHFCX1plX1JwQ0JSWHRoWjhYUTJtdnJYYk4wQl9PTlYyRUFGN1cyQjJSV1RyUUxtWHhDdl9RaVYyMlhrcUtB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8wFBVV95cUxQUzdtUjdYaEhfaWtqS01WbGMwXzZIdFZZX29rNGRNTHFYYm5lbDJaM3F3aE0zM2ctaGM4VlJTU2RDYVVnVERjejBXZnF4eXM1OHAxN2FYaGw2cmxsWFNYOW1mRHdrMHhDRzNRR3lRX1RkemhyNkswYXE3NllLS1VwdVhZN2Y5eEtEZnlCMVRUUVNZNGc3MjM4a09SU0dsbWdfQ3NoUlVOd3RxZ1NWSGhmN1VQdjZRelBaeXdreHFzQ1ZPUmtfY1pPNXlLdG16Mm0wODI3N1BOTWx4VDk0aEVzcURKSDRIUlhQQW5qWjBodXVMR3c?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1185,42 +1185,42 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46079.35042824074</v>
+        <v>46079.40400462963</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>British Nationals Jailed in Bali for Drug Offenses - Devdiscourse</t>
+          <t>Medewerkers Arnhems autobedrijf gewond na schietpartij, burgemeester spreekt van ‘afschuwelijke daad’ - Automotive Online</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>British Nationals Jailed in Bali for Drug Offenses - Devdiscourse</t>
+          <t>Employees of Arnhem car company injured after shooting, mayor speaks of 'horrible act' - Automotive Online</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 08:58:11 GMT</t>
+          <t>Thu, 26 Feb 2026 12:19:43 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNSWNGM3VmaHJSdmtpZWFjSGxDU293eFZpWjVlMjhNRTFCUXd2S0lFUGVZYXpYOHR1VUNNRG9YS3ZZTF9NSjlqZkZtZ0x5ZUdDZVJyWjZ1ZmlQb3NVb2JPc1cydmRia193cmN5dnNLQkZUMGl2Z0kwZTNTeGhoN3FRU01YenJPVHUxa05ITkJ4ck9FNHYyLTZ5aThQdnltV2RjSUdiTHBVZGVJakxvdEHSAa4BQVVfeXFMTUljRjN1ZmhyUnZraWVhY0hsQ1Nvd3hWaVo1ZTI4TUUxQlF3dktJRVBlWWF6WDh0dVVDTURvWEt2WUxfTUo5amZGbWdMeWVHQ2VSclo2dWZpUG9zVW9iT3NXMnZkYmtfd3JjeXZzS0JGVDBpdmdJMGUzU3hoaDdxUVNNWHpyT1R1MWtOSE5CeHJPRTR2Mi02eWk4UHZ5bVdkY0lHYkxwVWRlSWpMb3RB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxOWXF3QnBVS3NHa2xIQllYQmpCc3VBNDQtVVpfbjVlR2EtVTlfSjh3b2RMemRLNlJfeWxlT2ZwRzhaaUdvUU9EQTF4OGw4N044TzhpUnFTY2tabWZsNkpadlZfYzdGQU5Gd0VmQkFGaWxWVkpINUJNaWE5SWhyUWIwbzctOUh5SklRWTVzYjZMaGVMX0wzTU9fVHhtTjJ2LWYzVkJiOEVhOG9Fc0JlSDllbTJJVllNQlNYOWJndTV2ZmlaZWNIQlU2djh4RWViZmp4RGtRZmY0c2FaSDR6ak0zZE1tcUdtNHRxdmc?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1240,42 +1240,42 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46079.37373842593</v>
+        <v>46079.51369212963</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Alerte à la bombe levée à la Grande Synagogue de Bruxelles - 7sur7.be</t>
+          <t>Tot 28 maanden cel gevraagd voor schietpartij aan Truiense supermarkt - Nieuwsblad</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Bomb alert lifted at the Great Synagogue of Brussels - 7sur7.be</t>
+          <t>Up to 28 months in prison asked for shooting at Truiense supermarket - Nieuwsblad</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 11:10:56 GMT</t>
+          <t>Thu, 26 Feb 2026 11:31:27 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNNUcyd1ZldmRua3FWVTVNa1RyYmdmNG9JVW01VUs0Z1FETXRkSTFFMEpfSmxjRzVjaHVSQ0tnLV8wQmNYQVZTdWpNRDNRYjZuaWFCdUFpYmxGMUhBbjBGOTJyV05adDBFdjhIcG5lbGIzLVIyUGpnakF0RlVGN3lrR0lralBudHF0WGF2SGdwSHU4di1UT24yTko0X0VUY0NmaThPQmt3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxPN2JSbkd1NEhpSnNwcjZzdUVLWi1IYktjdF9DV1E4STZSVEIzRnBDV0d3cVFiTDRPNHQ1NE5IWWZ1bzQ5TEdfd1lIVTJWYmppNEI4OEEyWEdsd2M5UjY2TjFmdnVSdFY0bDF2Z213czdNNU1FSGlCT0NSejg3REFyZnhwWmVlemJfRmhhNEVmMjVfSXVqdkJUYlotQzFUX0Rkek5Zb3FMQTFta0JGanJxc0s1cHMxcHlYY2lidHNlWDBOcUY2UlYtUnV2Qjd2cXo2cFNR?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1295,42 +1295,42 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46079.46592592593</v>
+        <v>46079.48017361111</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Fusillade signalée à Matonge : une personne blessée transportée à l’hôpital - BruxellesToday</t>
+          <t>Na beroep blijft hoofdverdachte taximoord Geel in de cel - Nieuwsblad</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Shooting reported in Matonge: injured person taken to hospital - BruxellesToday</t>
+          <t>After appeal, main suspect in Geel taxi murder remains in jail - Nieuwsblad</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 09:21:00 GMT</t>
+          <t>Thu, 26 Feb 2026 09:02:03 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxNcEt2MEJuaERUd1FtRzh6S3YyUXBvYi05VjRKUjZpOHhvSW9UUnR1Rk54ZnRCb0FONnJJV1VxQTVEcHV2eFlMNXl5WU02cnN3QUdnb054Sk5aLTVYelBtYjVQUlJhUnp3NEFYbXJxSzk4Q0tSbWJSbE5SVmxwWWp3UlFGTQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPb0M1NGtlOE13MFpPNE43ZHRzQXhoLW1TWmRmMXpNYVNvN2lGSUdYT0dZRHVGUEpGdF9vdER6bTlTcTlIaE1MZ3N4V2ozcXcwS3BrMTlqQ1JiQzR1cWNxZExmOTFBRzFQV3NjV0ZNckV6NUZpZVZGVUw4YkFPaDRrZFpIWURXYzYyaEtBTFY0RjNETXMwdHpVTGVVUk1YWUllTTgxOC11M1BoWFFFOW0xU3NhVk5GYWRFV09DRGtzUjl5SjA?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1350,42 +1350,42 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46079.38958333333</v>
+        <v>46079.37642361111</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>En appel, l’étudiant en médecine reconnu coupable de viol et d’agression bénéficie à nouveau d’une suspension du prononcé - VRT</t>
+          <t>212 explosies door lachgas in verbrandingsoven Isvag: “Afval wordt nu voorgesorteerd om incidenten te beperken” - Nieuwsblad</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>On appeal, the medical student convicted of rape and assault once again benefits from a suspension of the sentence - VRT</t>
+          <t>212 explosions due to nitrous oxide in Isvag incinerator: “Waste is now pre-sorted to limit incidents” - Nieuwsblad</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 10:41:11 GMT</t>
+          <t>Thu, 26 Feb 2026 10:08:21 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNeHpLMEw4Rl9jRUxXVnNib0xGTjZhRzJ4NnQ2WDdnM2szenhkS3M1Wmh2ZktQWVR2bkN1M1ptdkNGTU9NVWY0VlVnWGtxbzM0NWZObDhWOGRaYmxzbUNCM0pmdlgwMnFLdXhhMnBLU1BUZmNPWWtCdS14SVYtOHJEV1dVS0JkTHp3QlNvazNlN1lZcGdON0htNGhHQUc1cEZ4WUlIdTBn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimwJBVV95cUxNV0g1Z2lGMmFVU3Ntc1praGtDVmJpb2FoT01QOE1kWHRvbDVGNjNKdXRNVUw1dVZHZXBpNVB0ck5Fa2luZ1lYOC1OTjdrNDJWRkhndjBkV2JjVXFfWC11R1N2Z2RjYy1rX1lFWjJKY0tMREZqV3laV3c5cThwMzEya3RuMjNQV0hTUmVpcDhhWERiaGh0eHVIN3VRR3hKcGNMTndkeUUydUlKV0d6VnJNTW4zRUcyM2U2NjdvY1JYeHRkOHNzcUJxRE4tLVZIMU5SX0RUeUlIMDZEWUptZHZNT0NPejhwcm1oazRNUTlEVloyeEd4aU15OTVicGF5Wk9jRjdoWjYtaXpNMnJkR3NDV1VsbUN6eWpRNzY4?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1395,7 +1395,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1405,42 +1405,42 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46079.4452662037</v>
+        <v>46079.42246527778</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Coups de feu dans le quartier Matonge à Ixelles, une personne à l’hôpital - 7sur7.be</t>
+          <t>Russia says it will retaliate after EU shrinks its diplomatic mission in Brussels - Al Arabiya English</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Gunshots in the Matonge district of Ixelles, one person in hospital - 7sur7.be</t>
+          <t>Russia says it will retaliate after EU shrinks its diplomatic mission in Brussels - Al Arabiya English</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 10:46:00 GMT</t>
+          <t>Thu, 26 Feb 2026 14:05:00 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOd1pVT2NvcTc1QlZLR2M0eGR5ZmJ3QlB3Vk9iU09OS2g2X0dtMVJWUHF6MU1tRVdHUTB4Y3F4RmlwTmlVOHFLWUJ1TlFBZlhpT0lvb21MRzZzOFg0ZEQ5ZkIteTJVY0FGSmNFcmozQzNyVUVwX0Q2X0Y5TFhST283aGh5T0dvd3dLWDNsVzhuOW1abEJNa3J2QlBXRHJPVGMtU1VuNnB5bmE0YmdORXVVRmJWM0pEZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxOUUx3MlR6QWVkbEVZTno3bGdUVm10NlFnTG1QTjFMN19wUHBidXQzMUxuempCSDRWU2YwNWZWclhjQTZmRTNVYmFxeS1sYXJvN2pCNmQwa0d6R1pMOVkyQ0pqc3VsUHU0bDM5dVM0elRObUJ0Znphekc0LWFLRHFLbmxVNms4Mk5GNldQOEU1N1pUYnptYV92MzY4SzZKb01uNVlGTVlOaVhKU1pZck1zeDhyem5haVktOEFFZ2RONTM0dmZTX1Z5LVRHaVhJNVBlR0l30gHTAUFVX3lxTE5RTHcyVHpBZWRsRVlOejdsZ1RWbXQ2UWdMbVBOMUw3X3BQcGJ1dDMxTG56akJINFZTZjA1ZlZyWGNBNmZFM1ViYXF5LWxhcm83akI2ZDBrR3pHWkw5WTJDSmpzdWxQdTRsMzl1UzR6VE5tQnRmemF6RzQtYUtEcUtubFU2azgyTkY2V1A4RTU3WlRiem1hX3YzNjhLNkpvTW41WUZNWU5pWEpTWllyTXN4OHJ6bmFpWS04QUVnZE41MzR2ZlNfVnktVEdpWEk1UGVHSXc?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1450,7 +1450,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,42 +1460,42 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46079.44861111111</v>
+        <v>46079.58680555555</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Métros 2 et 6 interrompus entre Delacroix et Bockstael - BruxellesToday</t>
+          <t>Bomb Threats Spark Chaos in West Bengal's Postal Services - Devdiscourse</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Metros 2 and 6 interrupted between Delacroix and Bockstael - BruxellesToday</t>
+          <t>Bomb Threats Spark Chaos in West Bengal's Postal Services - Devdiscourse</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 10:09:00 GMT</t>
+          <t>Thu, 26 Feb 2026 08:19:46 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxNNkphLVFkWm1RLWlrUm1ESFVtU3I3M202Mzdmd3pqYnFqYXRTc2NINkxHcHJfMXZ6QW9GZ2FTZ21UNlM5RVEtVnJLV05RWGxMOHg5SFBiMzZVQXc3SHJoZzkwS1pZeTJZUVl6ZlVnYnd0QWtIRVFuOHFHVm5hY3hBX1BCSE5XZVBFTGowVnhZVmc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOVnE4aW04dHlhVGIxQl9HdVctMks4SnJhQmgxWXpqd1h5WmFiU0VtRUtROTdDcmM5cmp2b2R5Q0cxcm1SYVYwdlJTbFhLS3hlQ0piSGJyZWc3UkJsTl9SdDNZSWUwU2FmZFpEQmtVcGU3Z1prNVc1SHdBX0Z5QTlzcnFOZHE4ZFoyQlQ1WmIzeDRWM1VzaUwwUjRDYWlQRkh1OW5YS0JRUU9jSFBPeUJBaU9ORzRTQdIBtgFBVV95cUxOVnE4aW04dHlhVGIxQl9HdVctMks4SnJhQmgxWXpqd1h5WmFiU0VtRUtROTdDcmM5cmp2b2R5Q0cxcm1SYVYwdlJTbFhLS3hlQ0piSGJyZWc3UkJsTl9SdDNZSWUwU2FmZFpEQmtVcGU3Z1prNVc1SHdBX0Z5QTlzcnFOZHE4ZFoyQlQ1WmIzeDRWM1VzaUwwUjRDYWlQRkh1OW5YS0JRUU9jSFBPeUJBaU9ORzRTQQ?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1515,42 +1515,42 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46079.42291666667</v>
+        <v>46079.34706018519</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Un inspecteur de police pris en flagrant délit en train de sniffer de la cocaïne dans un commissariat - 7sur7.be</t>
+          <t>Brussels Airport emerges as a major drug trafficking hub amid rising corruption cases - Aviation24.be</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Police inspector caught red-handed snorting cocaine in police station - 7sur7.be</t>
+          <t>Brussels Airport emerges as a major drug trafficking hub amid rising corruption cases - Aviation24.be</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 12:04:00 GMT</t>
+          <t>Thu, 26 Feb 2026 22:11:36 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxQclk4YnA0RkhMTzEycWdDd3JlQnctZ2swbDFZYXUxaXZFZDZNTDBZbUg2TVR2cjBsdTVCdkw0ZVhsWlVtelR6OEJrUGQzNnRnS2xkSWFncm5mUkRaS3R1X1FBRU1lbnNETHUtMVJXUEFnSFlmUDlxVkV0bHktVElBRHJXcGY3UTlPSENFTktoTVJSeWlLOVBzYzl4MjNtTXVRT294M1NITDN4MzAwX0EzX09JUUtFT0FodF9ISGxjTHk4enlPTGZmLU1WOEFiQ1o1RjUyUXN5WjVHRG9zTXc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxNZmsxNzdRd3hUYUpCZFVQVTdOVFlVRk95Snl6eDk5LWg3RnFTblNFMnc2YzFYa0UwQ09zeGRlYU0yN3VZUHJqZkM4eEQtbnlxcFVfeXl1ZVA5RjBXX2hDS1FmWHJIOGhJYTRpUjNDbVFkTXU0eG1kMnJhbzlfM0xMUUcwQkRSV3BWM2dseDB6ME5oTDN4OHFzRFZ0cE1jU3J1QlJZMjhsY2kwNXNtcVMxUFh1U1pSdjVvYVVhQ3JQUjk0Z25pTENzcS1xZWtCZ3Q0dXgyN3o1REVOeVZT?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1560,7 +1560,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1570,42 +1570,42 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46079.50277777778</v>
+        <v>46079.92472222223</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Assassin’s Creed maker Ubisoft cuts jobs, sparks strike - AOL.com</t>
+          <t>South Korea and UAE Forge $35 Billion Defence Alliance - Devdiscourse</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Assassin’s Creed maker Ubisoft cuts jobs, sparks strike - AOL.com</t>
+          <t>South Korea and UAE Forge $35 Billion Defence Alliance - Devdiscourse</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 08:31:09 GMT</t>
+          <t>Thu, 26 Feb 2026 08:34:35 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxNT1h3QWd4eHNRQlFGRDh4UExSNTZiUHp4d1R4c0lxcG5LWEhsQU5sZklnUWlBYzlOV2hNREZ1Uk9haW1WdlQ0MUF5c3E5Y3pPTFc4czRwd3dBOGpCS0M1RkdvaHNXSUZNRi1fT19xZHVJYThNRk9fNmZwQXIxc1l5Umxn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPRVFodHBSSXVzeXE4ZG5mOFdiRFRISG1KOHBqcVRnOS1nZFhEZ2RrQUJhX3piNkRQOG5lN1R6dUNZV1RTRC1BTHJxTHlDbE5BSDZnQTZHaThSaWxiajZRX1lzbTVVSEExYjdXM1YxRVdTWmhBdER4eXZTZG5ySTBLRFFyeVd1MW9fUmNDVFYyalNKcy13NERDNk52SWVJaFlYTWY3emVLd2xRUFBuYVVQRtIBsAFBVV95cUxPRVFodHBSSXVzeXE4ZG5mOFdiRFRISG1KOHBqcVRnOS1nZFhEZ2RrQUJhX3piNkRQOG5lN1R6dUNZV1RTRC1BTHJxTHlDbE5BSDZnQTZHaThSaWxiajZRX1lzbTVVSEExYjdXM1YxRVdTWmhBdER4eXZTZG5ySTBLRFFyeVd1MW9fUmNDVFYyalNKcy13NERDNk52SWVJaFlYTWY3emVLd2xRUFBuYVVQRg?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1620,47 +1620,47 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46079.35496527778</v>
+        <v>46079.35734953704</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Falscher Uni-Arzt ruft an: Tausende Euro Beute in Würzburg-Heidingsfeld | Foto: Wolf von Dewitz (dpa-Zentralbild) - main-echo.de</t>
+          <t>The Cost of Defending NATO's Eastern Flank - Devdiscourse</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Wrong university doctor calls: Thousands of euros in loot in Würzburg-Heidingsfeld | Photo: Wolf von Dewitz (dpa central image) - main-echo.de</t>
+          <t>The Cost of Defending NATO's Eastern Flank - Devdiscourse</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 10:22:47 GMT</t>
+          <t>Thu, 26 Feb 2026 08:24:37 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxQSllxUHA4ZGpoSlFmY1gzYllYcEVaeVZmU3laTnRaWU5sYURJZ3IzTTdkdnltWkRlM040aUtoZ1lxZk1yUm9WMGFSbzhKdHlKQmZVVlhSUlJaYVZUOGRmQjlfa185eG5vd3VKOUt0amFLT0ZUZU9LdWI1NDg5TXIyN25GemdEZ29jNEVHOUhFdnhkVU9GMnAxMjNxcUJrRlpUbmhHaWliOENhdG9LM0FSMWFEZEtVaDV4QmFZMUVrSE02MzYxd2c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxPMVJZbjdoMTM0VXZfSmJTOWdvUFVpODRYcUNybzA0WDZNWlg2NDlCek1fVFRib0J5dF9UR2N0SHJqV0xIUzl6MlpoQW1Da2RhaTF5UEozcnVaRVdYV20wTjEzNUc0cUJfWmVfUnBDQlJYdGhaOFhRMm12clhiTjBCX09OVjJFQUY3VzJCMlJXVHJRTG1YeEN2X1FpVjIyWGtxS0HSAaIBQVVfeXFMTzFSWW43aDEzNFV2X0piUzlnb1BVaTg0WHFDcm8wNFg2TVpYNjQ5QnpNX1RUYm9CeXRfVEdjdEhyaldMSFM5ejJaaEFtQ2tkYWkxeVBKM3J1WkVXWFdtME4xMzVHNHFCX1plX1JwQ0JSWHRoWjhYUTJtdnJYYk4wQl9PTlYyRUFGN1cyQjJSV1RyUUxtWHhDdl9RaVYyMlhrcUtB?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1670,52 +1670,52 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46079.43248842593</v>
+        <v>46079.35042824074</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+          <t>British Nationals Jailed in Bali for Drug Offenses - Devdiscourse</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+          <t>British Nationals Jailed in Bali for Drug Offenses - Devdiscourse</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 09:29:48 GMT</t>
+          <t>Thu, 26 Feb 2026 08:58:11 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE03RUZJdVVWTG5jTlA1R0dmc2YyQ3Z2S1ExYmhkN0FENFJGamUwenJsSFFPWGpKc3B2aFBaeHRYVDR3aWM1SXg0YWZFVDk0N3d4a0Jz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNSWNGM3VmaHJSdmtpZWFjSGxDU293eFZpWjVlMjhNRTFCUXd2S0lFUGVZYXpYOHR1VUNNRG9YS3ZZTF9NSjlqZkZtZ0x5ZUdDZVJyWjZ1ZmlQb3NVb2JPc1cydmRia193cmN5dnNLQkZUMGl2Z0kwZTNTeGhoN3FRU01YenJPVHUxa05ITkJ4ck9FNHYyLTZ5aThQdnltV2RjSUdiTHBVZGVJakxvdEHSAa4BQVVfeXFMTUljRjN1ZmhyUnZraWVhY0hsQ1Nvd3hWaVo1ZTI4TUUxQlF3dktJRVBlWWF6WDh0dVVDTURvWEt2WUxfTUo5amZGbWdMeWVHQ2VSclo2dWZpUG9zVW9iT3NXMnZkYmtfd3JjeXZzS0JGVDBpdmdJMGUzU3hoaDdxUVNNWHpyT1R1MWtOSE5CeHJPRTR2Mi02eWk4UHZ5bVdkY0lHYkxwVWRlSWpMb3RB?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1725,52 +1725,52 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46079.39569444444</v>
+        <v>46079.37373842593</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Unterfranken: Trickbetrug mit falscher Arzt Masche häuft sich - Charivari Würzburg</t>
+          <t>Alerte à la bombe levée à la Grande Synagogue de Bruxelles - 7sur7.be</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Lower Franconia: Fraud with false doctor scams is increasing - Charivari Würzburg</t>
+          <t>Bomb alert lifted at the Great Synagogue of Brussels - 7sur7.be</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 11:13:00 GMT</t>
+          <t>Thu, 26 Feb 2026 11:10:56 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNSTRTbUYzUmlxdFVlemx5ZEhUX09PLXJlc1Z2cGdLbDlKU2Z0MEE1Wm1DeUJ4UWRiT0lkeHd3ZUx6TVBfdlluNkVWalA1Mi1sT0xMSnRyNE12YzhieTg0emdpbkNzelRhOW52NmZaaFlycUxhX3Z2YWdOX2dyckl4QlhxU09oSzhOSU1KZnZvNjJsdTlUNXBMMmVUdUNIN00?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNNUcyd1ZldmRua3FWVTVNa1RyYmdmNG9JVW01VUs0Z1FETXRkSTFFMEpfSmxjRzVjaHVSQ0tnLV8wQmNYQVZTdWpNRDNRYjZuaWFCdUFpYmxGMUhBbjBGOTJyV05adDBFdjhIcG5lbGIzLVIyUGpnakF0RlVGN3lrR0lralBudHF0WGF2SGdwSHU4di1UT24yTko0X0VUY0NmaThPQmt3?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1780,52 +1780,52 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46079.46736111111</v>
+        <v>46079.46592592593</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Mobile Blitzer in Prosselsheim aktuell am Donnerstag: Hier nimmt die Polizei am 26.02.2026 Raser ins Visier - News.de</t>
+          <t>Fusillade signalée à Matonge : une personne blessée transportée à l’hôpital - BruxellesToday</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Mobile speed cameras in Prosselsheim currently on Thursday: Here the police are targeting speeders on February 26th, 2026 - News.de</t>
+          <t>Shooting reported in Matonge: injured person taken to hospital - BruxellesToday</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 09:18:59 GMT</t>
+          <t>Thu, 26 Feb 2026 09:21:00 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNbjNUOG5zWkZlNDJfWUM4ZTIzV2pCa2hyZVdHajYtcFF5QkM2OTRvSkFjUVpFT19adzhuT0EtYzBEUXA2SjdxR1hjMjVXQWtxYThmaWxpazR4X3ZpeDJfRWNsNFJlRzI0VHN6ZnItRTNWelA3WXJ4NlZ3VTFaSHVpUnBhNlFJa2lVdjZRV2dFR09mRHJoZGdxZVhLN3lfaGRuX2NfeE9ONzJuOE5iZk9xNExEaWItQTE2dmw3R0tuaVNtaFJ5dlRXRzBObmFlT3N3a2stSjBUdVNDam9ZNnc4cHltTExjZGNLTlBPZFUxZVBlaDZsMENrMUVwRVB4ZjA2N2J4d3RIMXlCNjVVME4tRtIBlgJBVV95cUxPNktVejlZZVRSWFZ6Y2Q5S01TQ25adENrV0ZITEo0NXRiMmFLdFV2cUhCY0lLNm0xM3NRYVFQNkJyck5zMmJ5MGV6TDNLaG5ZQl8ydHpjUnN2WDNoMmd1RnVuYU9OZ2ZOdzNRbzUtZGFuSmhHLVRlOXdJS1NZQmF3Y044VWtGR2pQNVpGLVZXd0FELUhlRWdnZ2tRVXNBc1pvdUlMOHZWSUhCc1lMRFBqUkpZT2lLNk5pekpKU29zaW42WDN3VFRBbVBxLTJjM0RNdEtVNGpEemZzOVhmTzRSNjhTVGw0ZDV5NjExVHpyUGdQNFZnajAzZmh4WjlXd0QzblJWSUN0SmFNdEpUenQ5aTh1QlQ1QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxNcEt2MEJuaERUd1FtRzh6S3YyUXBvYi05VjRKUjZpOHhvSW9UUnR1Rk54ZnRCb0FONnJJV1VxQTVEcHV2eFlMNXl5WU02cnN3QUdnb054Sk5aLTVYelBtYjVQUlJhUnp3NEFYbXJxSzk4Q0tSbWJSbE5SVmxwWWp3UlFGTQ?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1835,52 +1835,52 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46079.38818287037</v>
+        <v>46079.38958333333</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Polizei stoppt 19-Jährigen mit ungewöhnlich schnellem E-Bike - Augsburger Allgemeine</t>
+          <t>La 72e Opération Arc-en-Ciel aura lieu les 14 et 15 mars et cherche des bénévoles - Télésambre</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Police stop 19-year-old with unusually fast e-bike - Augsburger Allgemeine</t>
+          <t>The 72nd Operation Arc-en-Ciel will take place on March 14 and 15 and is looking for volunteers - Télésambre</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 10:30:03 GMT</t>
+          <t>Thu, 26 Feb 2026 16:07:00 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxPaDB3RnJLa3M2cFRlWGxnVjhIZGtrTG5zZFlncmxTaFEydGVXT3ktUkEycXJWV1BkT0tvdVQ3d19rYmxqeHVLeFIyM0dTZmRaVW1RbFpLT0Nuald4X0Vvc0xnaF9vWU5DdTVVN1MwMEExTUhaR3V0dk9xMTJvcXJ3RGVtQWJWaURuMXVVZ0hZckJaZFBOREZYSDB2eGpjem50Z1hhdGYzVkNVVTRrMVJyakNQQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOT3lMZVlfSUo4QW5VaXRjZUdlZ2xpYW5BY2ZkX0wwTzhuYjVObDNtZDJNblhXb3Q3UXgyMWdzdGNLdVJaVEJkTzV4VHJ6Z3AyYnkwQVFfZTF5MW1DQzBpaVRZOFYxZlN3VmJhS1Z1WVdOYXl3OGRybmtsQmtpWWJ2djdjb2FtU0ZTVllRelhTU1dyTlM0R1VicGE4dm5xcVNsUkRKelhGOFhLVmpGbjdCMXdMX21KcXh6R1Zmb3k0ZXRyMnZq?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1890,52 +1890,52 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46079.43753472222</v>
+        <v>46079.67152777778</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Polizeibekannter 19-Jähriger handelt sich erneut Strafanzeigen in Ingolstadt ein - Pfaffenhofen Today</t>
+          <t>Invasion de renards sur les voies: métros 2 et 6 interrompus entre Delacroix et Bockstael - BruxellesToday</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>19-year-old known to police files new criminal charges in Ingolstadt - Pfaffenhofen Today</t>
+          <t>Invasion of foxes on the tracks: metros 2 and 6 interrupted between Delacroix and Bockstael - BrusselsToday</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 14:34:33 GMT</t>
+          <t>Thu, 26 Feb 2026 10:09:00 GMT</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMia0FVX3lxTE0zaUNPRFlYQ09mV0FhZzlaemNFSV9ybi0wMEE2T3NtV2hEZ0xodnd4ck9KV0pXMVN1WVRoMmxmZTVkVFpIbmJybFM5ZjdmMUd2T0tZUkN2QThnQnNHVE4zYzhFQ2s1SnZ1V3lN?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNX0N5c0tWaTctU3BIX20yRXNHNGVLUWNVeEtTUG1laDFKcjhyMHo4YTI4dkFxSGM0LUtRNlRsMGM5N0lDYkkxSHpsclgtWGNPa2dWaXBmYk0wd1ZjRnlEdFlrMUVDa1JjX0RpakxwS01Lc0pvUUl1Z1ZBM0h3dDhKZnB3dlJzRklrcFByTldORGE4Z3pNbVU5b2FhQQ?oc=5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1945,52 +1945,52 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K28" s="1" t="n">
-        <v>46079.60732638889</v>
+        <v>46079.42291666667</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Zwei Verletzte bei Frontal-Zusammenstoß zwischen Transportern in Ingolstadt - Pfaffenhofen Today</t>
+          <t>Coups de feu dans le quartier Matonge à Ixelles, une personne à l’hôpital - 7sur7.be</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Two injured in head-on collision between vans in Ingolstadt - Pfaffenhofen Today</t>
+          <t>Gunshots in the Matonge district of Ixelles, one person in hospital - 7sur7.be</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 12:47:11 GMT</t>
+          <t>Thu, 26 Feb 2026 10:46:00 GMT</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE5pTXVwUVlaRHpJY1ZWUTR5NkMyVS1nSERtOEtseUFkbDZPRXRBc3BHbTVReXNOM3dETG00YUxESFVSZGJXaTRsbU1vbS1XNmpUbGNIUVhVb0gzSnpGcWl3RmYzc2h3VmM2VUdON05xMDdMQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOd1pVT2NvcTc1QlZLR2M0eGR5ZmJ3QlB3Vk9iU09OS2g2X0dtMVJWUHF6MU1tRVdHUTB4Y3F4RmlwTmlVOHFLWUJ1TlFBZlhpT0lvb21MRzZzOFg0ZEQ5ZkIteTJVY0FGSmNFcmozQzNyVUVwX0Q2X0Y5TFhST283aGh5T0dvd3dLWDNsVzhuOW1abEJNa3J2QlBXRHJPVGMtU1VuNnB5bmE0YmdORXVVRmJWM0pEZw?oc=5</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2000,52 +2000,52 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K29" s="1" t="n">
-        <v>46079.5327662037</v>
+        <v>46079.44861111111</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Kleintransporter krachen frontal ineinander – zwei Menschen verletzt - Augsburger Allgemeine</t>
+          <t>Elmed | La Tunisie et ses partenaires européens intensifient les préparatifs à Bruxelles - Kapitalis</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Small vans crash into each other head-on – two people injured - Augsburger Allgemeine</t>
+          <t>Elmed | Tunisia and its European partners intensify preparations in Brussels - Kapitalis</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 09:14:45 GMT</t>
+          <t>Thu, 26 Feb 2026 20:14:14 GMT</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxOWEhJbnVGd3NuTWplRjFWbHNVVC1ldWl2b1lDVXgzMmItTlRZZHlFRW5Pd1ZwQUZoeVJRbC0yWTQxZzBUOURGTHp3bTY4Vlk3SUJ3MUNOVG1sNTdVUHV2cWpSRjd0NUJQVktnanZsOGp4enVnSjRMNUxFZUg5WVVNNTBUOWNaSDItdVltNXViZFVVeHVlb0tzM3hYTW5wUWxVdUp2NFQ5d1J1Z1R1Ymk5TTJuemFHd053WWtjbEFPT1laa1JnOXQ3eHRoSkNyb2dS?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQTHY0dnFmbzZQZ1FQNzIySFFjWk1QUWxQTUNrSDU5bGkyRF8wSURTc2FyWGQwM3ZwNWUwR3gzR2t3R0lubU0yZ2Z0RmlacS1lWmJsTHBBb1pVVmRTa1h2RnVEMGJBTU1ENXMtMTRqSkFTSWhScVZqOWMwX3FlanhFTVl5NEFfMzVwMjVnQUhpU1JXb3Mtb0ZIUzRZYzIzZTE2bFJnOU00MHZsZnhKemJRNExmNmJ5M3ZIOTVKUlNZRndranJHbjRv?oc=5</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2055,52 +2055,52 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K30" s="1" t="n">
-        <v>46079.38524305556</v>
+        <v>46079.84321759259</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Nach Vergewaltigung am Bahnhof in Pfaffenhofen: Mutmaßlicher Täter gefasst - Pfaffenhofen Today</t>
+          <t>Gabès | Verdict dans l’affaire des unités polluantes - Kapitalis</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>After rape at the train station in Pfaffenhofen: Suspected perpetrator caught - Pfaffenhofen Today</t>
+          <t>Gabes | Verdict in the polluting units case - Kapitalis</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 13:59:11 GMT</t>
+          <t>Thu, 26 Feb 2026 19:49:09 GMT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxNRDdYaE16bEI1eFZrV3NXU2t6SGZobUxDMVlOYi1vV3JfSGxPdC1Ed2JPb3k2b0dvZnJ4TzVtWmMxc3Z2UUstNnRWV1JaODFKY0VSc3RfYm44NmMycHRManVrd2EzT0h0b1FOOGdmWnJENVJqN3hiMUNzUWFSQUFmLUVfWlVkVkNvdVRLalhfOGw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOVWhfWEZYMENQSkFEUV8weUNRNTVjN1cwWDhMWklybWZMSTJib1RXZExGS1I3T2RteUt4bkptWkZYVk1LeHhRdEhlcE1RQkRFVUNuQjBuRVRNSDJlM3M4SUJaekNHX1JJTEJ3cVhOZk53SGNtc2VQLTl4VVAzVkRibzJJc0V0NGREUG9pRXhPWVUwYjlySVE?oc=5</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2110,52 +2110,52 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K31" s="1" t="n">
-        <v>46079.5827662037</v>
+        <v>46079.82579861111</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>Local Town Maasmechelen French</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Tablet und Kopfhörer aus Elektromarkt geklaut: Täter scheitern beim Fluchtversuch - Augsburger Allgemeine</t>
+          <t>INFO EUROPE 1 : avec une hausse 57% en un an, les saisies de cocaïne en région parisienne ont dépassé celles de cannabis en 2025 - Europe 1</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Tablet and headphones stolen from electronics store: Perpetrators fail in their attempt to escape - Augsburger Allgemeine</t>
+          <t>INFO EUROPE 1: with a 57% increase in one year, seizures of cocaine in the Paris region have exceeded those of cannabis in 2025 - Europe 1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 10:18:52 GMT</t>
+          <t>Fri, 27 Feb 2026 05:20:00 GMT</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxQZzhvanhqeTBURENLb1pYYVZQY0FSdUNsMlpTaGVDS2tUQ0Q5VnIzaGh2UjFkc1AtcnZsU25XSnhWMFNXa0xSeGhZR0FocmRvRUNXVWFBVkxPUExsSUJGVUplQVRnNmh2ODdCOFR4eE1pWDlfWWZTbG5qbGJNcV9EVURQMFl5d3hBUGVUZmNKMjIyeV9lY3ByYkNUdkY0ZTRyNi1udzdwWEhlMi04MEVIX2xBbzJYRjhnTDFhcGpab2c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxNM1NMQnpHRVo1YXZBLWJ3eFRwc1cwOExxSnV3YmEzVUc2UDNRand3Z1lXdXp1cE9BVW5LNmVyUVpZdGxpb0tRN1FWZFRIU19BdDh6bFFmVnVQVmptMjNveFNLUWVPWW5JOE91a1l0aWppU2ZNMXJyR1prNFFqOTJTSVFycWloMGJRUXNKUFU0QmJOeGhpUnlPbWFCZHVjQUU4UVhoNmhQVl9ZZFd0QV9NOEVEU0dhWEhLbG05ZmQwTG81TzBBaHUxSGZEZ0EyUzE1WUl6QUp1SWxLVzJKdUYzQ2NGZzUwd2FwVXgxZEhPZmozbTN6X3VHMmFHMzJ0QdIBgwJBVV95cUxNTEtuTjVOMno0OHgxQ0QzbXlMSnI2T29ZY1ZzY3puc2dRS0NxdEdBcXI1bFN1QmhKYjhtemdPWTg0WUdSU3g0SUt6TE5xODFSVTZhWVphVE81cEFaRkg3aWJaaC1UVmFuMGNiYnBGcDNYRDcyOV9DZHdwVUZMaU5IdWgxRENFNmxYdWJCWDltaFBwRE05WHlDRGJCUDhsN0k0OUFFSWNrX2lHbXdjUDE0anU5Rk5MeW5mZVZoZWZ1el9WSlhLRHZqTmV0NkNodVRnX3hPSG9FTDlMTk5WTHdvQWpzNjF1NkJhTmJlNEFlcXNxbkh6WWM0dlJqSlZFY3dGSUlZ?oc=5</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2165,52 +2165,52 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K32" s="1" t="n">
-        <v>46079.42976851852</v>
+        <v>46080.22222222222</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Village Ingolstadt (fallback)</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Red Bull München signs Latvian national team defender Alberts Smits - EHC Red Bull München</t>
+          <t>Assassin’s Creed maker Ubisoft cuts jobs, sparks strike - AOL.com</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Red Bull München signs Latvian national team defender Alberts Smits - EHC Red Bull München</t>
+          <t>Assassin’s Creed maker Ubisoft cuts jobs, sparks strike - AOL.com</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Thu, 26 Feb 2026 11:00:00 GMT</t>
+          <t>Thu, 26 Feb 2026 08:31:09 GMT</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxQdU0tU0RQRUFaNGpSNUE3R0lyZ1M3VEozSXhqcUN0VUh1WU1YLU9KbGpEVWxVWUZfNTBsd1ZuSk9GWnNTd0N1elJuSDJta1hZcEkxSDNMTWtjMzl0MVZCYmJnbnlzcXJPd2ZZbi14UXRtdTM5S05TcWk2TnRIOC1NODZoMkRQQkRFRkxpWjk3T2xGQXRKbkZ3aEIyZzk2cER6ZW4zNExkT3F6c0pu?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxNT1h3QWd4eHNRQlFGRDh4UExSNTZiUHp4d1R4c0lxcG5LWEhsQU5sZklnUWlBYzlOV2hNREZ1Uk9haW1WdlQ0MUF5c3E5Y3pPTFc4czRwd3dBOGpCS0M1RkdvaHNXSUZNRi1fT19xZHVJYThNRk9fNmZwQXIxc1l5Umxn?oc=5</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2234,61 +2234,776 @@
         </is>
       </c>
       <c r="K33" s="1" t="n">
-        <v>46079.45833333334</v>
+        <v>46079.35496527778</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>Local Town Maasmechelen English (fallback)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Laatste kleinere cinema van Hasselt sluit zich aan bij grotere broer Cineville maar behoud goedkoop tarief en lokaal karakter - Truiensnieuws.be</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Hasselt's last smaller cinema joins bigger brother Cineville but retains cheap rates and local character - Truiensnieuws.be</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Thu, 26 Feb 2026 13:37:56 GMT</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxNMjJNdUEzRU54WXdQSW9EOXF2b0o2b0hLQTBRR0lTUUo1TU5CRVZFbnJKeTlnaHl1a1lxYnFlNHhxUzhTZ2Y2cm11M1VhSG1WRkVNa3BJV0pKdThyQW9fQkF5TkJLZjFET0VaUnpYSEg0U3hwRF9haGpBbGZacUVLdHJPTlJLU3B2anpjd1VkdkFOendjdHI5R0wzNmxIMDNBcXU0d3ltOFY2bGdVRFBiVEF6aWh4TlZlcEpudlMtZjRNYXBYY3BEc1kyNnRGcGI1UDdzMy1NV3I0elF4S0RQOVlqU25QSUcxaHdaSi1IX0tTUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K34" s="1" t="n">
+        <v>46079.56800925926</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Würzburg: Straba-Demo zieht durch die Stadt - Radio Gong Würzburg</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Würzburg: Straba demo moves through the city - Radio Gong Würzburg</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Fri, 27 Feb 2026 04:30:00 GMT</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxPZGRPUVBsQ015MnEwME1DUVpHNUJVa29LRmJoQXhyTEUxWmtWTGN5dHZzVGhyU0Zya2lyREJ1ZGd6d3F6b2hfT3A4S2p4Rl9MVzRtMk42OGFBcGdDS0lNT2VnaC1mRGpIYk9BRjRaTzZwczhNczlUOHhrMi0yQW1TNFFFSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K35" s="1" t="n">
+        <v>46080.1875</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Polizei Würzburg warnt vor dreisten Telefonbetrügern - Fränkische Nachrichten</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Würzburg police warn of brazen telephone scammers - Fränkische Nachrichten</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Thu, 26 Feb 2026 14:40:00 GMT</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxQSFFZVG9yZjVWa1Z0VmtWYUNKc3JaMEtWY0ZpVDBlcU0zSEFmc0t5LW9tRmxVRHFPWFdlYUM4aV9vWVJ4c0l2UUg4Q2pFMl9WQjdSM1oxWGk4X1ZKMThRaHpGYkxsTy1vR2k1QThwclNlQWJUOFlUZUtJTXpvZkNrMFl6NTFIQXd2X0c3Umk3aERhazF0OHoxTFh5X3J5UE5PZld4SERlY21CS01lblNpNTVlMGxyd2prdkw1QVV6bXFGZk1VVDM3cW9TQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K36" s="1" t="n">
+        <v>46079.61111111111</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Falscher Uni-Arzt ruft an: Tausende Euro Beute in Würzburg-Heidingsfeld | Foto: Wolf von Dewitz (dpa-Zentralbild) - main-echo.de</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Wrong university doctor calls: Thousands of euros in loot in Würzburg-Heidingsfeld | Photo: Wolf von Dewitz (dpa central image) - main-echo.de</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Thu, 26 Feb 2026 10:22:47 GMT</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxQSllxUHA4ZGpoSlFmY1gzYllYcEVaeVZmU3laTnRaWU5sYURJZ3IzTTdkdnltWkRlM040aUtoZ1lxZk1yUm9WMGFSbzhKdHlKQmZVVlhSUlJaYVZUOGRmQjlfa185eG5vd3VKOUt0amFLT0ZUZU9LdWI1NDg5TXIyN25GemdEZ29jNEVHOUhFdnhkVU9GMnAxMjNxcUJrRlpUbmhHaWliOENhdG9LM0FSMWFEZEtVaDV4QmFZMUVrSE02MzYxd2c?oc=5</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K37" s="1" t="n">
+        <v>46079.43248842593</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Mobile Blitzer in Prosselsheim aktuell am Donnerstag: Hier nimmt die Polizei am 26.02.2026 Raser ins Visier - News.de</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Mobile speed cameras in Prosselsheim currently on Thursday: Here the police are targeting speeders on February 26th, 2026 - News.de</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Thu, 26 Feb 2026 09:18:59 GMT</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNbjNUOG5zWkZlNDJfWUM4ZTIzV2pCa2hyZVdHajYtcFF5QkM2OTRvSkFjUVpFT19adzhuT0EtYzBEUXA2SjdxR1hjMjVXQWtxYThmaWxpazR4X3ZpeDJfRWNsNFJlRzI0VHN6ZnItRTNWelA3WXJ4NlZ3VTFaSHVpUnBhNlFJa2lVdjZRV2dFR09mRHJoZGdxZVhLN3lfaGRuX2NfeE9ONzJuOE5iZk9xNExEaWItQTE2dmw3R0tuaVNtaFJ5dlRXRzBObmFlT3N3a2stSjBUdVNDam9ZNnc4cHltTExjZGNLTlBPZFUxZVBlaDZsMENrMUVwRVB4ZjA2N2J4d3RIMXlCNjVVME4tRtIBlgJBVV95cUxPNktVejlZZVRSWFZ6Y2Q5S01TQ25adENrV0ZITEo0NXRiMmFLdFV2cUhCY0lLNm0xM3NRYVFQNkJyck5zMmJ5MGV6TDNLaG5ZQl8ydHpjUnN2WDNoMmd1RnVuYU9OZ2ZOdzNRbzUtZGFuSmhHLVRlOXdJS1NZQmF3Y044VWtGR2pQNVpGLVZXd0FELUhlRWdnZ2tRVXNBc1pvdUlMOHZWSUhCc1lMRFBqUkpZT2lLNk5pekpKU29zaW42WDN3VFRBbVBxLTJjM0RNdEtVNGpEemZzOVhmTzRSNjhTVGw0ZDV5NjExVHpyUGdQNFZnajAzZmh4WjlXd0QzblJWSUN0SmFNdEpUenQ5aTh1QlQ1QQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K38" s="1" t="n">
+        <v>46079.38818287037</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Polizei nimmt nach Vergewaltigung am Bahnhof mutmaßlichen Täter fest - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Police arrest suspected perpetrator after rape at train station - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Thu, 26 Feb 2026 14:46:18 GMT</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPYVRuOElyUVowQUlwajVxa2RVM2Z4X01qbDFTMmdXc1A2anJ0LTdYRFlwTWtaMVBhcU1hSzk5RUF1cjdkTXBqV3hzajlPQWRjd09JUjRUSUd3V21GdlBNTENiclU0WDUtQmhSYVIteXRfUEF4NDZHTFFuajlleXEyQ2pQMjI3Q2xxU18yM3dmdE9SYkFqclhEVERfM1dpXzF5ek0zVzE1YlktQUF5ZEdxTzZXQjFsZFdzSEc4?oc=5</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K39" s="1" t="n">
+        <v>46079.61548611111</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Polizei stoppt 19-Jährigen mit ungewöhnlich schnellem E-Bike - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Police stop 19-year-old with unusually fast e-bike - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Thu, 26 Feb 2026 10:30:03 GMT</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxPaDB3RnJLa3M2cFRlWGxnVjhIZGtrTG5zZFlncmxTaFEydGVXT3ktUkEycXJWV1BkT0tvdVQ3d19rYmxqeHVLeFIyM0dTZmRaVW1RbFpLT0Nuald4X0Vvc0xnaF9vWU5DdTVVN1MwMEExTUhaR3V0dk9xMTJvcXJ3RGVtQWJWaURuMXVVZ0hZckJaZFBOREZYSDB2eGpjem50Z1hhdGYzVkNVVTRrMVJyakNQQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K40" s="1" t="n">
+        <v>46079.43753472222</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Polizeibekannter 19-Jähriger handelt sich erneut Strafanzeigen in Ingolstadt ein - Pfaffenhofen Today</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>19-year-old known to police files new criminal charges in Ingolstadt - Pfaffenhofen Today</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Thu, 26 Feb 2026 14:34:33 GMT</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMia0FVX3lxTE0zaUNPRFlYQ09mV0FhZzlaemNFSV9ybi0wMEE2T3NtV2hEZ0xodnd4ck9KV0pXMVN1WVRoMmxmZTVkVFpIbmJybFM5ZjdmMUd2T0tZUkN2QThnQnNHVE4zYzhFQ2s1SnZ1V3lN?oc=5</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K41" s="1" t="n">
+        <v>46079.60732638889</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Zwei Verletzte bei Frontal-Zusammenstoß zwischen Transportern in Ingolstadt - Pfaffenhofen Today</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Two injured in head-on collision between vans in Ingolstadt - Pfaffenhofen Today</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Thu, 26 Feb 2026 12:47:11 GMT</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE9Xams1SmpXLXFKeGhVOVptX1FBRlp3UDRISVRtQXFRSV9Zb2t1ZnllM19CUHQ5ZE1fTEx6QjNLdmtxelJQRUwwc3BIX1N6QmNwcE5mdUNKZmFJZ2RiOGExbUc3LWNQajhWR3ZYQ292Q0IxNExDV0Nz?oc=5</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K42" s="1" t="n">
+        <v>46079.5327662037</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Kleintransporter krachen frontal ineinander – zwei Menschen verletzt - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Small vans crash into each other head-on – two people injured - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Thu, 26 Feb 2026 09:14:45 GMT</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxOWEhJbnVGd3NuTWplRjFWbHNVVC1ldWl2b1lDVXgzMmItTlRZZHlFRW5Pd1ZwQUZoeVJRbC0yWTQxZzBUOURGTHp3bTY4Vlk3SUJ3MUNOVG1sNTdVUHV2cWpSRjd0NUJQVktnanZsOGp4enVnSjRMNUxFZUg5WVVNNTBUOWNaSDItdVltNXViZFVVeHVlb0tzM3hYTW5wUWxVdUp2NFQ5d1J1Z1R1Ymk5TTJuemFHd053WWtjbEFPT1laa1JnOXQ3eHRoSkNyb2dS?oc=5</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K43" s="1" t="n">
+        <v>46079.38524305556</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Village Ingolstadt (fallback)</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>DEL preview, match day 46: EHC Red Bull München visits Augsburg - EHC Red Bull München</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>DEL preview, match day 46: EHC Red Bull München visits Augsburg - EHC Red Bull München</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Thu, 26 Feb 2026 16:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPeDNpYl94LXY4YnpEYWhjSXpJS2ZCWWk3eUtPQnZkS19WYXctRGprcHRfT2xCMXYxR2FYRzFQTzZ0dXhHbFc1cHBsUmhLYXQ4b2FrdEtTcVQwc1hYc3hlNnN2UEkwOWtBWThxNFNnM3pwTDZUY2k5b29XV2t6WTRYT2xYREFHd3ExaEFIUE5KM0xYYkZuZzNZY3FxTEFuOWtrNWpPTHlWTEI?oc=5</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K44" s="1" t="n">
+        <v>46079.66666666666</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Village Ingolstadt (fallback)</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Red Bull München signs Latvian national team defender Alberts Smits - EHC Red Bull München</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Red Bull München signs Latvian national team defender Alberts Smits - EHC Red Bull München</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Thu, 26 Feb 2026 11:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxQdU0tU0RQRUFaNGpSNUE3R0lyZ1M3VEozSXhqcUN0VUh1WU1YLU9KbGpEVWxVWUZfNTBsd1ZuSk9GWnNTd0N1elJuSDJta1hZcEkxSDNMTWtjMzl0MVZCYmJnbnlzcXJPd2ZZbi14UXRtdTM5S05TcWk2TnRIOC1NODZoMkRQQkRFRkxpWjk3T2xGQXRKbkZ3aEIyZzk2cER6ZW4zNExkT3F6c0pu?oc=5</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K45" s="1" t="n">
+        <v>46079.45833333334</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND ("minaccia bomba" OR "pacco sospetto" OR "pacco esplosivo" OR sparatoria OR accoltellamento OR "attentato" OR "operazione di polizia" OR esplosione OR evacuazione) AND -Olimpiadi AND -pattinaggio AND -sci AND -Cortina AND -calcio AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Milano, doppia aggressione nella notte: 19enne arrestato per rapina ed indagato per tentato omicidio - Affaritaliani</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Milan, double attack in the night: 19 year old arrested for robbery and investigated for attempted murder - Affaritaliani</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Thu, 26 Feb 2026 09:15:10 GMT</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxPX2YteU5YbTM0MGdyZ0pWXzhFcmZIX05Mc1Bidkd1MXJKQy0tdmhwNFpCMkpXSlZKeno3djQ2M0VKOUhVMHFoUFNyLXVHWmpIQlg0aENDNDFkT1NKazNUR0RraTBZQUVYbGtZQk9nMHo0ajYzbkdUTVpNblVWM2tvV1EzOXFVOG1wMzdzVUV2cVA5LTQ2RldQd3JlR0s?oc=5</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K46" s="1" t="n">
+        <v>46079.38553240741</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
           <t>Local Town Fidenza Italian</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>("Fidenza" OR "Parma" OR "Piacenza" OR "Cremona") AND (protesta OR "minaccia bomba" OR esplosione OR sparatoria OR accoltellamento OR evacuazione OR "operazione di polizia" OR arresto) AND -calcio AND -Serie AND -mercato</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>Parma, un arresto per le tre suore uccise in Burundi nel 2014: chi è Harushimana Guillaume - Adnkronos</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>Parma, an arrest for the three nuns killed in Burundi in 2014: who is Harushimana Guillaume - Adnkronos</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E47" t="inlineStr">
         <is>
           <t>Thu, 26 Feb 2026 12:46:00 GMT</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F47" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxNOGYwQVJHbF9ReFVKWWNWaC0wM2RJb2hZMk5EdG1JdXNQOEF2clhmR3ZTVThzbFhfc3hteVdBT25xUlJnTlFXc1V5QjB1U2Z2VElLX09GcUx6LVFkeXFBZGlTWUM0RHdMZm40TGlTMUZTakxhT1VZMkRsYk51VGNrWjVfZUUxemhXc1l3a1lQWVVUN08xOExmOTRzYmdMMGVDZUctbHFzU1Fwa1hUNTZHeDlSTlBlSnBOdVVyNGRPSTE2OHVTUTh3?oc=5</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
         <is>
           <t>it</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="I47" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="J47" t="inlineStr">
         <is>
           <t>IT:it</t>
         </is>
       </c>
-      <c r="K34" s="1" t="n">
+      <c r="K47" s="1" t="n">
         <v>46079.53194444445</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-03-01 07:40 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,32 +480,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Value Retail Brand</t>
+          <t>Brand Protest</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
+          <t>("Gucci" OR "Ralph Lauren" OR "Dior" OR "Armani" OR "Louis Vuitton" OR "Burberry" OR "Prada" OR "Nike" OR "Canada Goose" OR "Hugo Boss" OR "Moncler" OR "Saint Laurent" OR "Loro Piana" OR "Lacoste" OR "Versace" OR "Jimmy Choo" OR "Michael Kors" OR "Missoni" OR "Kiton" OR "Aquazzura" OR "Tumi") AND ("protest" OR "animal rights" OR "fur free" OR "PETA" OR "activist") AND -BAFTA AND -"red carpet" AND -"awards" AND -"wears" AND -"dressed in"</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>B&amp;M European Value Retail S A : Creates 30 Jobs for Locals with Brand New Diss, Norfolk Store - marketscreener.com</t>
+          <t>Dior’s Exclusive Dior Or Ramadan Collection Epitomises Elegance and Grace - A&amp;E Magazine</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>B&amp;M European Value Retail S A : Creates 30 Jobs for Locals with Brand New Diss, Norfolk Store - marketscreener.com</t>
+          <t>Dior’s Exclusive Dior Or Ramadan Collection Epitomises Elegance and Grace - A&amp;E Magazine</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 08:53:04 GMT</t>
+          <t>Sat, 28 Feb 2026 08:25:17 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxObHRuQUhqcllSTUotUXlXVElTTFgwbERBZjBpUkFBaWtDZUhHSkgxZ1dDcjFHalllaXI5bWh6cHUzdWM4MXgwS2lpbURUWHNkMEppajMtd1dwSnJMNWRqWERNU1I0NllrQnFMd3A2clcxWjFrQlZ6RER4WVVtVGxwd3lETzlqMXQ4OFBXNGZMWlB6ODFjejNvZGh1UmpFUU1INmMxVjI4bWRIVTZ2RGtydl9SdHo3dV9Da295M3g0ZjRrcTYwUXVndV8zdDY2UGpCVGgwb3BkOUJISWM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxQcTNRLU9FMGxMXzhQMlk5SlRwNF9TZWZNWVlnSEhfeV9CMEUwYjdLVU1uMU1aaU9jS3lkV2hETExfTFRZNU1SRTZiUGZUR1dvNTBjalVqSnhiZVhPeHpXZzBSU2NFZWFGM3ZUOEliRDFQcTNrU2RZUUtxVGtfQndQaHhLUWNsalpKbjh6aUtlR094ZE1YZmVOaEpiTmNOTkdXTGdN?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -529,38 +529,38 @@
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46081.37018518519</v>
+        <v>46081.35089120371</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BV Logistics Disruption</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>("DHL" OR "UPS" OR "DPD" OR "FedEx" OR "Royal Mail" OR "Parcelforce" OR "EVRI" OR "Dropit") AND (disruption OR strike OR failure OR delay) AND ("UK" OR "United Kingdom" OR "Britain") AND -dental AND -"pay dispute" AND -"postal vote"</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Royal Mail warns 20 UK areas won't receive post on time this weekend – full list - Express.co.uk</t>
+          <t>B&amp;M European Value Retail S A : Creates 30 Jobs for Locals with Brand New Diss, Norfolk Store - marketscreener.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Royal Mail warns 20 UK areas won't receive post on time this weekend – full list - Express.co.uk</t>
+          <t>B&amp;M European Value Retail S A : Creates 30 Jobs for Locals with Brand New Diss, Norfolk Store - marketscreener.com</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 10:47:00 GMT</t>
+          <t>Sat, 28 Feb 2026 08:53:04 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxNdWFkbzRSX2hQT1J5cjFJazJoQno1LV9tOEtaTExvYnJZVkF2ck5MOXRLQUg1TjdnTG9GQlZuQ3dIN2llaXRNU1I5MzNVS3ZyNEY3cFVCa3JISTQwWmdvdTBqZFl5REhkSHl2T2x2ZE40cjZLc0xNRnVWV2k0aVd2SzVYRXJwd1HSAYwBQVVfeXFMTWVRUmVlRHZxajY2Q0czS01XMDQ2M01TN3p1bnEyTGZXS0NwMFNad1VmbndpME1uTU9OR0tVMVA5OTQ1b2JiZFNSN3RONk9JVzZ6OUhyVmllTVZJdVBlQ0VRaWtDWnBTblZNMTJjS3pTWURYZDZiZDBqbTliM0RNaTJVdXFBOGVoU05hWlM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxObHRuQUhqcllSTUotUXlXVElTTFgwbERBZjBpUkFBaWtDZUhHSkgxZ1dDcjFHalllaXI5bWh6cHUzdWM4MXgwS2lpbURUWHNkMEppajMtd1dwSnJMNWRqWERNU1I0NllrQnFMd3A2clcxWjFrQlZ6RER4WVVtVGxwd3lETzlqMXQ4OFBXNGZMWlB6ODFjejNvZGh1UmpFUU1INmMxVjI4bWRIVTZ2RGtydl9SdHo3dV9Da295M3g0ZjRrcTYwUXVndV8zdDY2UGpCVGgwb3BkOUJISWM?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -584,38 +584,38 @@
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46081.44930555556</v>
+        <v>46081.37018518519</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Explosie in Anderlecht: appartementsgebouw en voormalig tankstation onbewoonbaar - HLN</t>
+          <t>Dollar Tree, Inc. (DLTR): A Bull Case Theory - Insider Monkey</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Explosion in Anderlecht: apartment building and former gas station uninhabitable - HLN</t>
+          <t>Dollar Tree, Inc. (DLTR): A Bull Case Theory - Insider Monkey</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 10:40:17 GMT</t>
+          <t>Sat, 28 Feb 2026 20:00:45 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxOdmFTNmVmeVFpRC13MENWemxqWE8tSlR5RE1PaF9ZY0FkcFk1OGd0U1Vnb0NvUDBlRXhPR1huWHh1cWh1NGZkVTJZZmdTT2R4a1NEVDVwRGtzX2dvUmExeTRKdVMwclphOXNaUVdBTHBXcjlneHNiZ3dJWjJmMlpIZEFtSk16R0c1RkRvOUdFT210RGJtd2lWT1ByZ2duTnhtc3dMTTVtSkhEbHJJcm85YUxVNy0tcG5m?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxQMkFPVkxVZ2pNc1Y0V25USnltLXF1UDdoMmxPOU1Lb1NqMDlESHVSSVRUY09yM0kxU1BxQ1NDa251OHBZa0xQM3ZWeVNUZHliNUVnT0FIam5UV3JUSzZKWmZxakR6d3BXcXdidWxGcU9TVVNrM0U3Yk50Vk8tODYzSl9Vem1rZ3hGbXVTOUFR0gGWAUFVX3lxTE40dHFZalFmUjNXa0dXQ1dEZTZDaXRFNjRad21janYweWdFeHR0NndSbloydkZpcGQ3d0RuZGxFQnVMMi1JSE0ybGpKWEZNZ25iRi1RYkp2S2dkbEgwUktRaHJPY3VwcnhjRnRZLTktZWQ3MDFaLUt5MUsxM3NBbTZ5WndER3VOdzRXTGxWcjJUcDFMc29fUQ?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -625,52 +625,52 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46081.44464120371</v>
+        <v>46081.83385416667</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Logistics Disruption</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("DHL" OR "UPS" OR "DPD" OR "FedEx" OR "Royal Mail" OR "Parcelforce" OR "EVRI" OR "Dropit") AND (disruption OR strike OR failure OR delay) AND ("UK" OR "United Kingdom" OR "Britain") AND -dental AND -"pay dispute" AND -"postal vote"</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Raad van State legt bom onder voorstel voor lagere LEZ-boetes - BRUZZ</t>
+          <t>Royal Mail warns 20 UK areas won't receive post on time this weekend – full list - Express.co.uk</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Council of State puts bomb under proposal for lower LEZ fines - BRUZZ</t>
+          <t>Royal Mail warns 20 UK areas won't receive post on time this weekend – full list - Express.co.uk</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 11:16:08 GMT</t>
+          <t>Sat, 28 Feb 2026 10:47:00 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxPWDl4MjB2WS00b1VZZk92cjNFNWhIdEZCY2tPQXhET0N3cFY3NlhSTmRQdl9GcFlLQW9oWnpzUUZtQ0ZYcnJXQ0YwdUdPbW5FMldxNXR5R1hNQzV5MW8yY0xfcW5RMTNsdWRCanZnUVAzNHhXWkY0OFkzYUVmZFZHZGtidFdjTkx4dDYtMkFPM1VRNkxpUDI1RnpqWllLYzFuZFdqcjF3bTE0dw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxNdWFkbzRSX2hQT1J5cjFJazJoQno1LV9tOEtaTExvYnJZVkF2ck5MOXRLQUg1TjdnTG9GQlZuQ3dIN2llaXRNU1I5MzNVS3ZyNEY3cFVCa3JISTQwWmdvdTBqZFl5REhkSHl2T2x2ZE40cjZLc0xNRnVWV2k0aVd2SzVYRXJwd1HSAYwBQVVfeXFMTWVRUmVlRHZxajY2Q0czS01XMDQ2M01TN3p1bnEyTGZXS0NwMFNad1VmbndpME1uTU9OR0tVMVA5OTQ1b2JiZFNSN3RONk9JVzZ6OUhyVmllTVZJdVBlQ0VRaWtDWnBTblZNMTJjS3pTWURYZDZiZDBqbTliM0RNaTJVdXFBOGVoU05hWlM?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -680,52 +680,52 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46081.46953703704</v>
+        <v>46081.44930555556</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Former petrol station explodes in Anderlecht - The Brussels Times</t>
+          <t>"Af en toe opgeschrikt door explosie": Vlamingen gestrand op grote luchthavens in Golfregio - VRT</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Former petrol station explodes in Anderlecht - The Brussels Times</t>
+          <t>"Occasionally startled by explosion": Flemish people stranded at major airports in the Gulf region - VRT</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 11:15:00 GMT</t>
+          <t>Sat, 28 Feb 2026 15:14:04 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxOeWFacnRqcHFrSERIbnNXbFV3QmJqSFI3RGpWcjdvQXNvWHN4YUdoTVFOdG1jYUcxbl9lLTNyNFNqMUNaekZoWkJ3Z01tZS1RMTQyeWh6TnhDV01mZ3RoTWkwdkRUZHZBMXVPcm1HdzdtaGJ5YlNLRE9hbnVoTWJNb1p0eHgzQXZmQURNQVBQaGJDX2FE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOVTVfLWU3SXJqRDY5dHlaV3g3XzdzVXdNbEo1TnN5WHlGTEtVbEhyR3Yxd2pENDJZeGxHUmw2VDA0UmxnSEhMVlZuVUZUbF9CZXpqNWV4T3FYejNZOEpsQ3R3UHJXZENxeUs0cVZSckVaZGx6ZTV0cEtDcWpVSnNCU3Y2WFpoOTZmMmVsQk9XcXRCa3RmcFA5LTRUTGlrLW5oVmt1X1AwUEE?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -745,42 +745,42 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46081.46875</v>
+        <v>46081.63476851852</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>EU withdraws Middle East personnel after US-Israel strike Iran - The Straits Times</t>
+          <t>Explosie in Anderlecht: appartementsgebouw en voormalig tankstation onbewoonbaar - HLN</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>EU withdraws Middle East personnel after US-Israel strike Iran - The Straits Times</t>
+          <t>Explosion in Anderlecht: apartment building and former gas station uninhabitable - HLN</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 10:57:48 GMT</t>
+          <t>Sat, 28 Feb 2026 10:40:17 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxPWGpNTTQ1UHdHTlBFcEN0UjFybUlMUEVMbjRLVlJ4bkFHME0xQUcyd1FoY2V0NUNuOFlkd0xBNFptMkRQR244Sm52czhXeEJCZXNGR0s2ODJacmhyRk9ZVXZSMVZpWW9jM2tFMWxrVy1IdlZNYUJFdG5HTnV5by0zUXo2T0dFb0FIcTY2RkdZM0F3aENZVDNmdXhMWFhCQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxOdmFTNmVmeVFpRC13MENWemxqWE8tSlR5RE1PaF9ZY0FkcFk1OGd0U1Vnb0NvUDBlRXhPR1huWHh1cWh1NGZkVTJZZmdTT2R4a1NEVDVwRGtzX2dvUmExeTRKdVMwclphOXNaUVdBTHBXcjlneHNiZ3dJWjJmMlpIZEFtSk16R0c1RkRvOUdFT210RGJtd2lWT1ByZ2duTnhtc3dMTTVtSkhEbHJJcm85YUxVNy0tcG5m?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -800,42 +800,42 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46081.45680555556</v>
+        <v>46081.44464120371</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>World leaders fear broader escalation after attack on Iran - Manila Bulletin</t>
+          <t>Raad van State legt bom onder voorstel voor lagere LEZ-boetes - BRUZZ</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>World leaders fear broader escalation after attack on Iran - Manila Bulletin</t>
+          <t>Council of State puts bomb under proposal for lower LEZ fines - BRUZZ</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 13:52:47 GMT</t>
+          <t>Sat, 28 Feb 2026 11:16:08 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxOellfbDBWTVl2QTE1R3FWZzdEcEk1UG5TRHBjaVZHWlBYbmJXSUxxYmRkOEhRblluTk9FNEhwTjR0b0s3SzNKdG5DMkRPYlFud0R6N01nNjNXbHN4OGdyWDdzeDZDSDdTV2dvTGNvTXhiSXo2Z1YzcEVHcmRHT05reWJSVVJYUnE3SWdYTTlaRGU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxPWDl4MjB2WS00b1VZZk92cjNFNWhIdEZCY2tPQXhET0N3cFY3NlhSTmRQdl9GcFlLQW9oWnpzUUZtQ0ZYcnJXQ0YwdUdPbW5FMldxNXR5R1hNQzV5MW8yY0xfcW5RMTNsdWRCanZnUVAzNHhXWkY0OFkzYUVmZFZHZGtidFdjTkx4dDYtMkFPM1VRNkxpUDI1RnpqWllLYzFuZFdqcjF3bTE0dw?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -855,42 +855,42 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46081.57832175926</v>
+        <v>46081.46953703704</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>EU Leaders Urge Restraint on Iran Situation - Devdiscourse</t>
+          <t>Loenhout verslaat Minderhout na hattrick R. Driessens - Nieuwsblad</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>EU Leaders Urge Restraint on Iran Situation - Devdiscourse</t>
+          <t>Loenhout beats Minderhout after hat trick R. Driessens - Nieuwsblad</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 10:41:48 GMT</t>
+          <t>Sat, 28 Feb 2026 22:05:00 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPVmxfVHFUUUJvbm1wcGdwYWdFQmo3alprRC1JWHUwVnJfaDdYeUMza2hDQWkzQnI2WmpHQUhfMGlvNmNhUGZ2UGptRjBJMV9pNEV0WWF3d2g5ZjJBN3lfWmhDTngtUWZlX2VvOHBwUU8yOW5RUTlTVGlZN2dkb2gxZWtXX2xnSFozRnltOXhjTEIyQ1I1WTBreFowMXZISzJob0F1T9IBpAFBVV95cUxPVmxfVHFUUUJvbm1wcGdwYWdFQmo3alprRC1JWHUwVnJfaDdYeUMza2hDQWkzQnI2WmpHQUhfMGlvNmNhUGZ2UGptRjBJMV9pNEV0WWF3d2g5ZjJBN3lfWmhDTngtUWZlX2VvOHBwUU8yOW5RUTlTVGlZN2dkb2gxZWtXX2xnSFozRnltOXhjTEIyQ1I1WTBreFowMXZISzJob0F1Tw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxPamM0VlY1M1JPQUNseWYzWFp5TE1sZmFiTGs0M1YzNGJ4RW83S3VRT1luSC03LVlPVTRSa0RyRW11Z200eS0tZ1BmZHRGYW93TkJXVXlxenNTTXBWbmJXd01wTE1EcGgzaW9haWNsUmVsX3NyR2tsYVB5ekRISDB2WFU4SS1PVVhaOGtZZTNyS254NUxHSXA5ekhCMGVTRDNiNEhGZk1LbkxqeWxlX3BLYXVWMXAzNGIwQ2RJUGktUGtJQ1E3UUpobEFJaUNDLXkzbHdz?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -910,42 +910,42 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46081.44569444445</v>
+        <v>46081.92013888889</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Explosion à Anderlecht : un immeuble à appartements temporairement inhabitable, aucun blessé - BX1</t>
+          <t>LIVE Midden-Oosten | Explosie op bekende ‘palmeiland’ in Dubai: beelden tonen grote rookpluim bij hotel - De Gelderlander</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Explosion in Anderlecht: apartment building temporarily uninhabitable, no injuries - BX1</t>
+          <t>LIVE Middle East | Explosion on the famous 'palm island' in Dubai: images show a large plume of smoke at hotel - De Gelderlander</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 10:28:00 GMT</t>
+          <t>Sat, 28 Feb 2026 16:05:00 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQalp1ODR5WVRrQVhPTmJpOFVaUnFnZDNQaC02bEhQTDkwRnJNcG04Z3VnVWYxOHFsQ2p0RnNScmtCN1NVV01OWXd1RDQ3S1lhNWxFUjE5OTR5d2FqSnBFZkgyellMUVRvR1gwUVMzV0Jfa1l5RFd1UDUzOUxPeW01TXJqbU5VZ3dfcjBOMXpMWWZMSTlUU2JQV2V5dTIxYmZ6WE5hQ3Uzc2pxN3pNem4zRzJ5V0NLeUFpc0d1WDBB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxPem5yNEJIVGhITFF5Q0JpemRya0kyNUc4eEtrOEtPLS1tdDh4VTRuMG5YXzNJN0lOR0x0emwwMENuN242M3V0Q0VwX1VNOFFFdVlLS0xudFU4bHgzN0lLRWtobFdHLWQ1Z3ptOEJnaDVBY1lHUnVuU3lWMVZYZDUwSnVDUGljMlItYWZHLVJPOVhkelNHdzlsTEkwcHJhb2FTRnlxeF9RdndDT3c5TElGQVVQakxwdmtWNGFVRk1PZFF4NUp1VWx3aVI1UnRRb3pGWTczb3RQZ1BOXzJFMFdvaXo1Rkc0ZG8?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -955,7 +955,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -965,42 +965,42 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46081.43611111111</v>
+        <v>46081.67013888889</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>L’OTAN examine le renforcement de ses capacités nucléaires - سانا</t>
+          <t>World leaders react cautiously to U.S. and Israeli strikes on Iran - PBS</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>NATO examines strengthening its nuclear capabilities - سانا</t>
+          <t>World leaders react cautiously to U.S. and Israeli strikes on Iran - PBS</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 11:04:15 GMT</t>
+          <t>Sat, 28 Feb 2026 17:20:20 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE5Wa0oyYTdqZXhoNFRESmxsaXFaVlZtVlV0cnc4bHdRRUhwSGQ1ajFBTHZ2b05RYWFyMFQ0aFYtektuX3h4a21vZ1NwVE9UaVlsYW1J?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxQLUJXZDl4eVN5LUUwa3VzbTcxdk9sWWJNSDR6SG9acXZ2b0dUa1Y2T3RjUVhWVHRMam5oOThFdnlSbUY5QUUxLVRuNTZObU1GTko4dmZLUlhrWTZsRGZ4RWVqV1IwNklTSTloZk9xRmVDeUdRT0pOcVdTbm5pajZCODJpblVlX3ZFejAxUjN5eWpqdWlSdWtQRmZSWm8yVnI3bHfSAacBQVVfeXFMTnFhODl4OW9ZckRRSDFjeGRfU0Fjb21rMjNhOThyaHJUS09QSmVPMVYxT1NnTHZnNTh5Q254TTlqOXFKZzJtUXNxa0N6bFRPMHkwc3ZjVmQ2Z21Ka2pGUW44OFFaU2I4OEdrR19LX1UxaHJ1clJZeEpSMlUzLTF1WFgzZXhqVU1kdXhkTkhuamI3T0FiUHcwNzJSLW5YRHRlWS1WbFRkYm8?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1020,42 +1020,42 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46081.46128472222</v>
+        <v>46081.7224537037</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Accord UE-Mercosur : Emmanuel Macron critique l’application provisoire décidée par Bruxelles - Capital.fr</t>
+          <t>World leaders fear broader escalation after major US and Israeli attack on Iran - SILive.com</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>EU-Mercosur agreement: Emmanuel Macron criticizes the provisional application decided by Brussels - Capital.fr</t>
+          <t>World leaders fear broader escalation after major US and Israeli attack on Iran - SILive.com</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 08:49:40 GMT</t>
+          <t>Sat, 28 Feb 2026 13:49:00 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxPVmJieGlWamItX1hMSGVCczVyRmRYR0hZcGRONldodE5leXozQlJjY0pySTQzcEtGNU5VUF9PMTMydWVjcDR5QUo0bUo4cDIyZXVUOVhzVEdJVHFZS0FHVjNrNjNNcHZYNWJESzFqNDQyWWZIaWlzV1hhVnV2Nzl1bGYwb3IwT2pzbVpwRDY3WUduSnNwX094Yk84U1lsdVVJQk1DSDhQWTdfN3YzZ0pYal9kNllab01BcFZHb2FfZmJhTEFodXF2UE40QzA4VzFJMVRPQ2tWNA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxQb2lZeXRCcThuSjdkcGViU2hJTEpSbUtOTjJNemNUQWxweXYyMDlfT3F4ZE1MWWNjb2xPYzhhQ2RZTDkxRGdBbGQ1bFlLblVXVjcxZzQ5bDh1RGVpYkxER1ZjREhZRjd2LUpkbjVqZU00ak9vQ1dmTlo4cHJXNFRrMGZ4TEN6WkUxUjNZcHktM0lBU3Z3b2RtampQa2FfT09TNnJvTnRQSExpX0ZSVnV1aXM5aU16Slc4QmN4ODgxSdIB0wFBVV95cUxQeThVM3lXRmYtNzlUZkFWVE5oeUJMdWtpcmcySzJSc1MxQmdKWV9TV01rYURDVzBTR1dJcF8yY3VTdXpNWkRkQWVkMHRiZDBOQ0t1dl9INEJUd3NHNER3SnJVMkoxeXZXSFgwWktNc29zQllROXA0RDlFeFFMTUxYV2IyM1h6cWJ2anNmc0M5MjRvOVZiODl2enYteFVQWG5aZllIV05DMTgzNmFNcF96RXpyTjVBdEhlZW5HbDd0OERMVGJDS1lKMmU2bm1CNHJaNkNV?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1075,42 +1075,42 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46081.36782407408</v>
+        <v>46081.57569444444</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Meurtre de David Polfliet : crime homophobe ou "chasse au pédophile" - BruxellesToday</t>
+          <t>EU caught in the crosswinds after US–Israel strikes on Iran: energy, shipping and security risks surge - EU Reporter</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Murder of David Polfliet: homophobic crime or “pedophile hunt” - BruxellesToday</t>
+          <t>EU caught in the crosswinds after US–Israel strikes on Iran: energy, shipping and security risks surge - EU Reporter</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 12:04:37 GMT</t>
+          <t>Sat, 28 Feb 2026 17:10:36 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxQQlNSV3ZjX2FYSm1xTUI5TWJfSnVJVzRxdEZzRnU3azNQUkNPMUJwQnVFR21OLXdWQ2g1YmRQTHBaTndNWDBBRndvREVjRUxRdExNOXptbjIyT2o3Y1JXWmRCWFFQTWxRLTFBQlFCTlFSdlg0OV9ucUc3NEJ4eVRIYTU5RDdTM1RGWEhKS2pOeHpRcVMzcU1nQWd3WQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxNZ0d4aG5WZWdHdHBWZ19aNmdvRWVwUm1mTkhaa18xcERUTXZnMDF1RG9TLUZMNHgwMlRaMXJ5N29TRzl0cl9MMjJlQ0xOUEpXV2lUWTZlUHBLeEVXWVY4dEJ0N3JvVHVYR2ctNV9aaDFrWG0ycGZiUm1NcnNqbnBtRWlrbF81RndGUnl4NXptVkVTbl9PRTk2cFpjakVIOWZmc1dtM2ZhQ0k5cFZISFI1clJNRXZSQ1RaNjF6T0hWVnUxcUJUQmM1UHBiVGVhMTlFTU9NaHJDTEFaTXJ5?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1130,42 +1130,42 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46081.50320601852</v>
+        <v>46081.71569444444</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Warme maaltijd moet rust en verbondenheid brengen in wijk Ter Hilst in Hasselt - VRT</t>
+          <t>Former petrol station explodes in Anderlecht - The Brussels Times</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Hot meal should bring peace and solidarity to the Ter Hilst district in Hasselt - VRT</t>
+          <t>Former petrol station explodes in Anderlecht - The Brussels Times</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 10:26:04 GMT</t>
+          <t>Sat, 28 Feb 2026 11:15:25 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPZlNReUNVMGNsV3ZNRlE5YXMwcDRuYnppMWlQUmxVT3VDNzNfYW9tVGFyTlBaUHFocFhKQ3BjMlotMHJOR2h3Mmw4WWhnaldSZnVNY3FwZHo0VFB1NEpLVVQwU0ctbk1iZVZyYXRaOTJ3OGJYeEJiMmhMVmxhWUN5c0hVT3pPU010SlMyOUE5NzdORDJYTGZZWFlhbEhLQ2VwcXVvSzdUdEo?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxOeWFacnRqcHFrSERIbnNXbFV3QmJqSFI3RGpWcjdvQXNvWHN4YUdoTVFOdG1jYUcxbl9lLTNyNFNqMUNaekZoWkJ3Z01tZS1RMTQyeWh6TnhDV01mZ3RoTWkwdkRUZHZBMXVPcm1HdzdtaGJ5YlNLRE9hbnVoTWJNb1p0eHgzQXZmQURNQVBQaGJDX2FE?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1185,42 +1185,42 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46081.43476851852</v>
+        <v>46081.46903935185</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Handball (SHL) | Visé, la révolte avec du sang neuf, à Hasselt : « On va disposer d’un groupe plus étoffé pour les prochains matchs » - Sudinfo</t>
+          <t>Dubai authorities say drone debris causes fire at Burj Al Arab Hotel - HESPRESS English - Morocco News</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Handball (SHL) | Visé, the revolt with new blood, in Hasselt: “We will have a larger group for the next matches” - Sudinfo</t>
+          <t>Dubai authorities say drone debris causes fire at Burj Al Arab Hotel - HESPRESS English - Morocco News</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 11:00:00 GMT</t>
+          <t>Sat, 28 Feb 2026 23:24:47 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPV3RvZjJUUnJ3dW1oSHhBUlliNDBFS0ZHUkZmWEZsT1lIWlVXZVZMRlU5QmdRS3ZZSjV3SXR3bzJUa19SaDdPd3VRNFdhS25YM25nTGVJRFFFeFIzZk5FdGliNmhfb1B2MThMNGJjSk14cnJVVlNFckVLSDN3NWJQcFd2ODJKTUx1VXh0M1ZsS3B3Q2Vjd3lQb3BNN0xHbEJHanU2b2ZBMktqMm82Nnozb2d0OF80ZURGdURmMHU4YVh0MTlKclhlUg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxOMUVwS3B0VkNDWG5ZZC0wcW5idzhqNTB4UUJFWGVzS1BrWF9sUTJNNkhuTU9odEhSX1hSUUx0UzZFbWt5VWNrWXlua1loYW1FM1lKNE5JRmJ2SlBaVElwM1FlcnJvY096eTZIVTRGbURlZUFURlh1UUd5aW0xYWNHWTdBU1dJdUthMmJ4U2hlYzRxZVIyVXBnRFhQRENLczZaUV9VQ0Nyaw?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1240,42 +1240,42 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46081.45833333334</v>
+        <v>46081.97554398148</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Highlights: RSCA Futsal 21-1 Sensei Sushi Anderlecht (Futsal League) - Anderlecht</t>
+          <t>EU withdraws Middle East personnel after US-Israel strike Iran - The Straits Times</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Highlights: RSCA Futsal 21-1 Sensei Sushi Anderlecht (Futsal League) - Anderlecht</t>
+          <t>EU withdraws Middle East personnel after US-Israel strike Iran - The Straits Times</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 14:10:27 GMT</t>
+          <t>Sat, 28 Feb 2026 10:57:48 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxOZW9SV3hPdlpHN0hfaVFlR3h0aVlVMlA3ZzYtLTFObWY3a2FpdnRYOUVNZktHMUtleGRaMF9va1ZsZ3NpR3BTd2hkMS1fMUl1elhrQ3IwTmNqN2xQWWhLYzlGTldiLVd2RTZCTnlieFdQUWVGM3c2SkE0d3NfVDVXMmZHOEhJQ2xfc04wNnB2d05MYnEtUzdEQg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPZUNpQUQ0b25Dck1nc0ZqTlZiMml4TW9YUG1Ccm5uT3ZDVVR1dUpGbi1ISHQxaHpNSWJLeS14OXprS2pfeTR1UFJhYjNMQnhqZExteV82MUkxR3g5Q0UyZVB1Rkt4Ql9KTGppZ3NqbVNseE1tcTZuVTVReFhPSGx6S3dyeWZHY0tBWl9QcFNhTVdSQVdkYzg5LVFhTFJ5UW52Q3hpQl9URkNpLUct?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1290,47 +1290,47 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46081.59059027778</v>
+        <v>46081.45680555556</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Waldaschaff: Polizei sucht Zeugen nach Angriff nach Faschingsparty - aschaffenburg.news</t>
+          <t>EU Leaders Urge Restraint on Iran Situation - Devdiscourse</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Waldaschaff: Police are looking for witnesses after an attack after a carnival party - aschaffenburg.news</t>
+          <t>EU Leaders Urge Restraint on Iran Situation - Devdiscourse</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 10:06:38 GMT</t>
+          <t>Sat, 28 Feb 2026 10:41:48 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPT2JycGhsRDBGX19melROOXNVUXNVWE9VTGszVC1JOG5lU2x4UHZBT19hU0w5a3RQenFwendXc2pPem9DMTdRc21RZDZUS1JFWnpMaElhcUlxUV8yVXhTcmNtOGZIcTFHQWhmNlhZc0JJWlBTS3M4WThRY1JqbTlfbVVwRGp2VE9OeUkxVlF6ZGQxLW5RejJIM2FhNjFpSURBQXV2SmJXWUFmbjl5QmlXN1diS1FoWVNpYnNOSTZsaEVSQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPVmxfVHFUUUJvbm1wcGdwYWdFQmo3alprRC1JWHUwVnJfaDdYeUMza2hDQWkzQnI2WmpHQUhfMGlvNmNhUGZ2UGptRjBJMV9pNEV0WWF3d2g5ZjJBN3lfWmhDTngtUWZlX2VvOHBwUU8yOW5RUTlTVGlZN2dkb2gxZWtXX2xnSFozRnltOXhjTEIyQ1I1WTBreFowMXZISzJob0F1T9IBpAFBVV95cUxPVmxfVHFUUUJvbm1wcGdwYWdFQmo3alprRC1JWHUwVnJfaDdYeUMza2hDQWkzQnI2WmpHQUhfMGlvNmNhUGZ2UGptRjBJMV9pNEV0WWF3d2g5ZjJBN3lfWmhDTngtUWZlX2VvOHBwUU8yOW5RUTlTVGlZN2dkb2gxZWtXX2xnSFozRnltOXhjTEIyQ1I1WTBreFowMXZISzJob0F1Tw?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1340,52 +1340,52 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46081.42127314815</v>
+        <v>46081.44569444445</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Streit am Morgen: Nach Messerangriff in Würzburg keine Hinweise auf Psychose - Bayern - Neue Presse Coburg</t>
+          <t>Explosion à Anderlecht : un immeuble à appartements temporairement inhabitable, aucun blessé - BX1</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Argument in the morning: No evidence of psychosis after knife attack in Würzburg - Bavaria - Neue Presse Coburg</t>
+          <t>Explosion in Anderlecht: apartment building temporarily uninhabitable, no injuries - BX1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 09:15:48 GMT</t>
+          <t>Sat, 28 Feb 2026 10:28:00 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxPZXhycWdQbTY3cC1kWTVIMXk5ektJb1FwMkZHRkt5NE5JcDkyNWxxZU1qbHB6R25VdWpUWFU1YWdGVnVKQzZ0RjRyM3RQX2xQcm1lZklFQ29KLWE5MUpuenpiLTVpS1RCQldOX2xPcjNyajl4Y2pPNnJ5SjRabm5zNU5YMHhiMlRqUTV5R2dnY3VVbU9rS0JtX1FUeXZVYV9IQWNvWnIzVzMwelRvZTdEZmpvNkcxY0ZvR3V0NEJzcXFnWi1pM2JscmRQRXVhb1dPaTgwLXg5cnJfLVAwcV9lOGNsM2g?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQalp1ODR5WVRrQVhPTmJpOFVaUnFnZDNQaC02bEhQTDkwRnJNcG04Z3VnVWYxOHFsQ2p0RnNScmtCN1NVV01OWXd1RDQ3S1lhNWxFUjE5OTR5d2FqSnBFZkgyellMUVRvR1gwUVMzV0Jfa1l5RFd1UDUzOUxPeW01TXJqbU5VZ3dfcjBOMXpMWWZMSTlUU2JQV2V5dTIxYmZ6WE5hQ3Uzc2pxN3pNem4zRzJ5V0NLeUFpc0d1WDBB?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1395,52 +1395,52 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46081.38597222222</v>
+        <v>46081.43611111111</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Weibersbrunn: Ausweichmanöver wegen ausschwenkendem Lkw - aschaffenburg.news</t>
+          <t>L’OTAN examine le renforcement de ses capacités nucléaires - وكالة الأنباء السورية – سانا</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Weibersbrunn: Evasive maneuvers due to truck swerving - aschaffenburg.news</t>
+          <t>L’OTAN examines the regeneration of nuclei capacity - Syrian News Agency - SANA</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 10:09:22 GMT</t>
+          <t>Sat, 28 Feb 2026 11:04:15 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxOSVRRVGwzbGUxTU1zaE05RWRzYWdvMTFONWYzOThvNHg0TjdPbXM0ci0ya1BCNllwdnhTT1lhcXluLWM0eEVNWTVsRXZOYnlBeE1hOWZiMVU2Q28tblg1S3pRNkxPWmc0ZjJWUWdZVFJ3UFI3Mkxaakc1TEJBenNQekRnU1lsaDhNMzB2amx0T0dvM0lPRmRLakc2VVVWNHY1dXBHaWVVQ240Q1p5V2h5Yk5JLTViMkVqV1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE5Wa0oyYTdqZXhoNFRESmxsaXFaVlZtVlV0cnc4bHdRRUhwSGQ1ajFBTHZ2b05RYWFyMFQ0aFYtektuX3h4a21vZ1NwVE9UaVlsYW1J?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1450,52 +1450,52 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46081.42317129629</v>
+        <v>46081.46128472222</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German (fallback)</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>("Ingolstadt")</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Livecenter - Adler Mannheim</t>
+          <t>"Ils m'ont enfermé dans un égout": Zakaria, 15 ans, grièvement brûlé à Anderlecht revient sur ce qui lui est arrivé - BruxellesToday</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Livecenter - Adler Mannheim</t>
+          <t>“They locked me in a sewer”: Zakaria, 15, seriously burned in Anderlecht, talks about what happened to him - BruxellesToday</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 11:42:36 GMT</t>
+          <t>Sat, 28 Feb 2026 16:45:00 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiTEFVX3lxTE9YM3hUZnd3U2M4OXZHTFNnY3BpdV9Cb0c5UnFWOUd4U2cydVQ4QldYZVpITTUwV3JYaXBKcUFKdDhFUHFEZDExWmhkZ3U?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNaVlPc085QkU3dDB1Uk9zT25JSFl6RDNOUHlKcFY1dzVmazYxcW9PckFvWW96TDlXaGFDRVhkVEpSa25NSGtWZXNIUXIyTlhRSjdYTnB2aWlMcnptZVUxQ2d5UUwzbnBBRGZIdHJ6ZDA2SHoxTjNfdVo2bHcxTXpmbV96eHdSSThpeWVzdVJIS3hrWDBHbFF0eFk2bmV0bUNqTUJmVVBn?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1505,52 +1505,52 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46081.48791666667</v>
+        <v>46081.69791666666</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German (fallback)</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>("Ingolstadt")</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Liveticker | SV Wehen Wiesbaden - FC Ingolstadt 04 : | 26. Spieltag | 3. Liga 2025/26 - kicker.ch</t>
+          <t>Accord UE-Mercosur : Emmanuel Macron critique l’application provisoire décidée par Bruxelles - Capital.fr</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Live ticker | SV Wehen Wiesbaden - FC Ingolstadt 04: | 26th matchday | 3rd League 2025/26 - kicker.ch</t>
+          <t>EU-Mercosur agreement: Emmanuel Macron criticizes the provisional application decided by Brussels - Capital.fr</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 12:31:44 GMT</t>
+          <t>Sat, 28 Feb 2026 08:49:40 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE96UlJjV091cnBqbDNKWXVDaTNQdnhrVnZpOFNFTnQwdm0yME9WRkx4ZXh6SXlROWtvNDJ3MEdIWDVkelhHNGtqV0gyUEs3YjhJVVh6QTFsNmFYNFZUcEVYbGJLMzJvWDNqVlNEX3ZKb0NDcEYydVNBQTgtVDAxQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxPVmJieGlWamItX1hMSGVCczVyRmRYR0hZcGRONldodE5leXozQlJjY0pySTQzcEtGNU5VUF9PMTMydWVjcDR5QUo0bUo4cDIyZXVUOVhzVEdJVHFZS0FHVjNrNjNNcHZYNWJESzFqNDQyWWZIaWlzV1hhVnV2Nzl1bGYwb3IwT2pzbVpwRDY3WUduSnNwX094Yk84U1lsdVVJQk1DSDhQWTdfN3YzZ0pYal9kNllab01BcFZHb2FfZmJhTEFodXF2UE40QzA4VzFJMVRPQ2tWNA?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1560,52 +1560,52 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46081.52203703704</v>
+        <v>46081.36782407408</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German (fallback)</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>("Ingolstadt")</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Neues Projekt im Tierheim Ingolstadt: Kinder lesen Hunden vor - Donaukurier</t>
+          <t>Meurtre de David Polfliet : crime homophobe ou "chasse au pédophile" - BruxellesToday</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>New project at the Ingolstadt animal shelter: Children read to dogs - Donaukurier</t>
+          <t>Murder of David Polfliet: homophobic crime or “pedophile hunt” - BruxellesToday</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 12:05:20 GMT</t>
+          <t>Sat, 28 Feb 2026 12:04:37 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQb01ZY3MtWUtzYnpZNmMzUGlhV21HRmMzNVhLcnFnRlcyZm9wRnZQZUl3cU5pcXlrTW5xSUJBWHA1djh4TjVoUkV3UDh6QU9nVDFJdDc2OThSVEtadWNnbGtuWVVISGlsSmlhRENIcDZaUTBfZEpWcmxibkxGTXdITVJwYlpERTZ3OWc4aU1wbWpkTndCRXdKbkpQbDVzUF9XdUgwNHYtcGtUbUNuSEdXRjhGVnpRUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxQQlNSV3ZjX2FYSm1xTUI5TWJfSnVJVzRxdEZzRnU3azNQUkNPMUJwQnVFR21OLXdWQ2g1YmRQTHBaTndNWDBBRndvREVjRUxRdExNOXptbjIyT2o3Y1JXWmRCWFFQTWxRLTFBQlFCTlFSdlg0OV9ucUc3NEJ4eVRIYTU5RDdTM1RGWEhKS2pOeHpRcVMzcU1nQWd3WQ?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1615,52 +1615,52 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46081.5037037037</v>
+        <v>46081.50320601852</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German (fallback)</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>("Ingolstadt")</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ÖPNV-Streik: Auch Passau, Landshut, Regensburg und Ingolstadt am Samstag betroffen - Wochenblatt.de</t>
+          <t>Fietser (59) vlucht weg van politiecontrole in Hasselt en belandt in Demer - VRT</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Public transport strike: Passau, Landshut, Regensburg and Ingolstadt also affected on Saturday - Wochenblatt.de</t>
+          <t>Cyclist (59) flees from police control in Hasselt and ends up in Demer - VRT</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 08:25:21 GMT</t>
+          <t>Sat, 28 Feb 2026 15:23:45 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxOTzNQVm1lMVVuZWdyaXRJbzhSMTJ1RTMzcmxBWHNXZTdsMzZ1bXYzRlpUYVhwRHlEMTVjT1VYMFJDeVFMcmpPS0Q5eWRlZjhoaFNsN2NYaGlzaGVhZ1VCMDE0b0d0XzNGSU92Sy0yUkRRN3ZzMVRkaFpIYzhydmtTUk9PMmowWWVPeFE0ZmpFUEdKd0lEV1kzWjRsQ3kxNkhsNEJWU1lUU3JVd25SZ3ROWTY4RzZCQ2NXVFhjc3pMOTZLbUtHT0hLLVBMajgxOFR4T3M3eXZqU3BHSmc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE5jZVQzeHVNeGJaa3BEOGxCTkNyWnlZZjFodmFQdW9yTWRDdjlWYjN6UGJ0U1hEVjE4bGFLLWpVZWszT0ZWcGVWNmQzSzJUcHN1WGExYkJjek9TQTczQnp1NjZiY0lSRGh2TmwyLTdDUV9tcDRfN0FRbk1uazc1V1E?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1670,52 +1670,52 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46081.3509375</v>
+        <v>46081.64149305555</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German (fallback)</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>("Ingolstadt")</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Kölner Haie - ERC Ingolstadt (Highlights) - SPORT1</t>
+          <t>Warme maaltijd moet rust en verbondenheid brengen in wijk Ter Hilst in Hasselt - VRT</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Kölner Haie - ERC Ingolstadt (highlights) - SPORT1</t>
+          <t>Hot meal should bring peace and solidarity to the Ter Hilst district in Hasselt - VRT</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 10:00:40 GMT</t>
+          <t>Sat, 28 Feb 2026 10:26:04 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxQOVhMT0tOZUdKeW8yQ0IxZVFYSmoyTE1Ec1g2cnV5Nnd0bThZSnZJTldyZkRMVHlFWDllOHhEaXR6YngzSWxSbDhGVjZkT0wxUTJRVWtnajh4cnRjazc0OXVsN3NWSzJyWk5JTHlVNGMyWWdNYnh3c2FDNklNb3JvdUJNR3N2b2ZlaXVYZzV4MlplSnJtNXlLNkdfRmdZY1VvYWtJbnZhT1dITUwtZGhaYmd3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPZlNReUNVMGNsV3ZNRlE5YXMwcDRuYnppMWlQUmxVT3VDNzNfYW9tVGFyTlBaUHFocFhKQ3BjMlotMHJOR2h3Mmw4WWhnaldSZnVNY3FwZHo0VFB1NEpLVVQwU0ctbk1iZVZyYXRaOTJ3OGJYeEJiMmhMVmxhWUN5c0hVT3pPU010SlMyOUE5NzdORDJYTGZZWFlhbEhLQ2VwcXVvSzdUdEo?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1725,52 +1725,52 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46081.41712962963</v>
+        <v>46081.43476851852</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German (fallback)</t>
+          <t>Local Town Maasmechelen French</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>("Ingolstadt")</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>SV Wehen Wiesbaden - FC Ingolstadt 04 im Live-Stream und TV: Wohin gehen heute die Punkte bei SV Wehen gegen Ingolstadt? - News.de</t>
+          <t>Handball (SHL) | Visé, la révolte avec du sang neuf, à Hasselt : « On va disposer d’un groupe plus étoffé pour les prochains matchs » - Sudinfo</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>SV Wehen Wiesbaden - FC Ingolstadt 04 in the live stream and TV: Where do the points go at SV Wehen against Ingolstadt today? - News.de</t>
+          <t>Handball (SHL) | Visé, the revolt with new blood, in Hasselt: “We will have a larger group for the next matches” - Sudinfo</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 08:56:34 GMT</t>
+          <t>Sat, 28 Feb 2026 11:00:00 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxQQ083NUlVRlV6TmROOF9FeUtwRm9YRFUxM1F0R3VwY3JIbkxtcGRLY3Z2XzZwWThnSkF6QngydUcxSXZqU1RVTUp1UnkxMjFwVG9VUVA5eTdmWDd6SnN2M0hhenJrdEhmZ3ZqV2lWeXd3cXZWNkNuQ1liZFU4NzhZbXVxODNRM24xeUtUbFZqbXFxNXB1TnJUeU42MVI4VGpISFhKRUpfQnhUOE5Vd1lrUjRYZlRrc041ZnROUDVZcHYyN3NGcWNFS1pNRC1wMEdDOUxZTjRLOTVKalNJd2VoM3BFSXZ3OFUzRTMwSjhoMmpUZm1jM3JYZnZlMlrSAYICQVVfeXFMTm9hY2p6RzlrVG1VcnQxSmJPNklqREFXRWpKa2RWbjI0anFlSzFoY28zajc3ZGNEcEd0OE05VWxIQkJqTFQ4NFFfd1F3VUlWVXRDWGU0MEtwanVkLWRyWEFna2REZnFLWHNuM2thb3VqZXhDYVVPbXp4WVFuclFVdXY4VW1MNFA1VWNiV3JSVmlYUThXajhZRkRwNWR6RGlKa1owdUtoMTUwZWlnQnRwTFM5T3EzTlRWZTdZQ1UwLU8xTGtvN0k5OUQ5blpJQmNHTGI5dE54azJQcVFFRnA5aXB6WXFpaWF6VHI3UXE4VWh2TXFSUk5QV2ptSDAtRzJNRlpB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPV3RvZjJUUnJ3dW1oSHhBUlliNDBFS0ZHUkZmWEZsT1lIWlVXZVZMRlU5QmdRS3ZZSjV3SXR3bzJUa19SaDdPd3VRNFdhS25YM25nTGVJRFFFeFIzZk5FdGliNmhfb1B2MThMNGJjSk14cnJVVlNFckVLSDN3NWJQcFd2ODJKTUx1VXh0M1ZsS3B3Q2Vjd3lQb3BNN0xHbEJHanU2b2ZBMktqMm82Nnozb2d0OF80ZURGdURmMHU4YVh0MTlKclhlUg?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1780,52 +1780,52 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46081.37261574074</v>
+        <v>46081.45833333334</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German (fallback)</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>("Ingolstadt")</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Verein Schanzer Wildparkfreunde in Ingolstadt gegründet - Donaukurier</t>
+          <t>Highlights: RSCA Futsal 21-1 Sensei Sushi Anderlecht (Futsal League) - Anderlecht</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Schanzer Wildlife Park Friends Association founded in Ingolstadt - Donaukurier</t>
+          <t>Highlights: RSCA Futsal 21-1 Sensei Sushi Anderlecht (Futsal League) - Anderlecht</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 12:38:02 GMT</t>
+          <t>Sat, 28 Feb 2026 14:10:27 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxNVmtlZTRTTnVZTUJsQ3FVMU1uY0xnMzBXcXFweHBJSmhVMm5pLUZ3MXhOejk1eXA3dUh2YTN6dDRabXJTbFQ5WHpsUThDdmNxSTNKZkwwdmZVYVA3dGdhSlh4U1hoaWx4VGt3aDhmV0x1OHFoTEZ4YlVsU0NZQXozbEpMSi1MazEyN2JuSmtIb2FfOXduZXUybXN0dGZWWUxBWjFhMm5VbXhZWUJKNzVTNQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxOZW9SV3hPdlpHN0hfaVFlR3h0aVlVMlA3ZzYtLTFObWY3a2FpdnRYOUVNZktHMUtleGRaMF9va1ZsZ3NpR3BTd2hkMS1fMUl1elhrQ3IwTmNqN2xQWWhLYzlGTldiLVd2RTZCTnlieFdQUWVGM3c2SkE0d3NfVDVXMmZHOEhJQ2xfc04wNnB2d05MYnEtUzdEQg?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1835,52 +1835,52 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46081.52641203703</v>
+        <v>46081.59059027778</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German (fallback)</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>("Ingolstadt")</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>„Die Milchstraße“: Kammerphilharmonie Ingolstadt spielt Piccolokonzerte in der Fronte - Donaukurier</t>
+          <t>AI Prediction: Roeselare Daisel vs Sporting Hasselt - First Amateur Division 01/03 - inbet.io</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>“The Milky Way”: Kammerphilharmonie Ingolstadt plays piccolo concerts in the Fronte - Donaukurier</t>
+          <t>AI Prediction: Roeselare Daisel vs Sporting Hasselt - First Amateur Division 01/03 - inbet.io</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 13:07:52 GMT</t>
+          <t>Sun, 01 Mar 2026 04:14:03 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiS0FVX3lxTFB3amdWVGdjblNUdGNEWDFBc1JqRGpRazVvUTE2WEpDQ29IV281alc1MUt1bGdZZ21fYzFFUTlrM0lmdzNET0xaZ21iZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxOZndFU05ET1doZnlZaEpwenNkUE94MjVCaG5mdmd1SVBCUy03ckhUQjRYMXpjNGh5bXQ5aTExR0treU1DenV2UFJFbTFHRWs3elZsOXgwUWUtdHBsWkJfRjVuTkNwZUhNekplREtVN0trMWROVWZqTVlmYThKTFpudVlqX0NJekU?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1890,52 +1890,52 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46081.54712962963</v>
+        <v>46082.17642361111</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>("Ingolstadt")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Eishockey | Spiele - Tabellen - News - Live-Ticker - Kicker</t>
+          <t>Waldaschaff: Polizei sucht Zeugen nach Angriff nach Faschingsparty - aschaffenburg.news</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Ice hockey | Games - Tables - News - Live Ticker - Kicker</t>
+          <t>Waldaschaff: Police looking for witnesses after attack after carnival party - aschaffenburg.news</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 07:48:37 GMT</t>
+          <t>Sat, 28 Feb 2026 10:06:38 GMT</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiVEFVX3lxTE1NN2pCNzRrN3VGS1NHOFFoZXJqeFQtMDJ4QUh6MmJ4ZGZUeXpvM1pub1JZTGJPcktsbXUzbGR2X09uWTMzNGh6ODlONmotb0Q5SDlySA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPT2JycGhsRDBGX19melROOXNVUXNVWE9VTGszVC1JOG5lU2x4UHZBT19hU0w5a3RQenFwendXc2pPem9DMTdRc21RZDZUS1JFWnpMaElhcUlxUV8yVXhTcmNtOGZIcTFHQWhmNlhZc0JJWlBTS3M4WThRY1JqbTlfbVVwRGp2VE9OeUkxVlF6ZGQxLW5RejJIM2FhNjFpSURBQXV2SmJXWUFmbjl5QmlXN1diS1FoWVNpYnNOSTZsaEVSQQ?oc=5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1959,38 +1959,38 @@
         </is>
       </c>
       <c r="K28" s="1" t="n">
-        <v>46081.32542824074</v>
+        <v>46081.42127314815</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>("Ingolstadt")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Gitarrist Michael Schenker gibt ein Konzert in der Eventhalle am Westpark in Ingolstadt - Donaukurier</t>
+          <t>Streit am Morgen: Nach Messerangriff in Würzburg keine Hinweise auf Psychose - Bayern - Neue Presse Coburg</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Guitarist Michael Schenker gives a concert in the event hall at Westpark in Ingolstadt - Donaukurier</t>
+          <t>Argument in the morning: No evidence of psychosis after knife attack in Würzburg - Bavaria - Neue Presse Coburg</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 07:37:58 GMT</t>
+          <t>Sat, 28 Feb 2026 09:15:48 GMT</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiS0FVX3lxTE5mcW5KRUJxa1FfYmZGMU16SkIyVXdKYkh5Q1Q3dm5sVWxHY1UxVW8tZ3RRSmpLeGFQOEVmU3VvUFEzQU9kNV9yWkNTNA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxPZXhycWdQbTY3cC1kWTVIMXk5ektJb1FwMkZHRkt5NE5JcDkyNWxxZU1qbHB6R25VdWpUWFU1YWdGVnVKQzZ0RjRyM3RQX2xQcm1lZklFQ29KLWE5MUpuenpiLTVpS1RCQldOX2xPcjNyajl4Y2pPNnJ5SjRabm5zNU5YMHhiMlRqUTV5R2dnY3VVbU9rS0JtX1FUeXZVYV9IQWNvWnIzVzMwelRvZTdEZmpvNkcxY0ZvR3V0NEJzcXFnWi1pM2JscmRQRXVhb1dPaTgwLXg5cnJfLVAwcV9lOGNsM2g?oc=5</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2014,7 +2014,282 @@
         </is>
       </c>
       <c r="K29" s="1" t="n">
-        <v>46081.31803240741</v>
+        <v>46081.38597222222</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Weibersbrunn: Ausweichmanöver wegen ausschwenkendem Lkw - aschaffenburg.news</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Weibersbrunn: Evasive maneuvers due to truck swerving - aschaffenburg.news</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Sat, 28 Feb 2026 10:09:22 GMT</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxOSVRRVGwzbGUxTU1zaE05RWRzYWdvMTFONWYzOThvNHg0TjdPbXM0ci0ya1BCNllwdnhTT1lhcXluLWM0eEVNWTVsRXZOYnlBeE1hOWZiMVU2Q28tblg1S3pRNkxPWmc0ZjJWUWdZVFJ3UFI3Mkxaakc1TEJBenNQekRnU1lsaDhNMzB2amx0T0dvM0lPRmRLakc2VVVWNHY1dXBHaWVVQ240Q1p5V2h5Yk5JLTViMkVqV1E?oc=5</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K30" s="1" t="n">
+        <v>46081.42317129629</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Ukrainerin verweigert Verlassen der Asylbewerberunterkunft - RegionalReporter</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Ukrainian woman refuses to leave asylum seekers' accommodation - RegionalReporter</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Sun, 01 Mar 2026 07:03:04 GMT</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxOemRhYjhRS2NxZU1PSFZWTmpaOENTb2NqZDdOa1pTS2lrai1CQ2JTLVp3ckVnOWpqRlBEMlpRLS1PLUxhbV9QYmVsS25oLVJjeU9XVEc1VEFZNXJBYlZJbnhxTnlrRU5RNEwtRzZuSzJrV0dDd3c4eDc5MTUtYmNkLVBETkFmS21YX3BlRXZQU1Q1VWF5aVAzWGRxSG9UNE5heEVGN2xTVlR4Mk5OMEFaOU1aUHJ5OFNU?oc=5</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K31" s="1" t="n">
+        <v>46082.2937962963</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>KEC hatte zu Beginn Schwierigkeiten.: Die Kölner Haie haben mit 6:3 gegen den ERC Ingolstadt gewonnen. - Rheinische Anzeigenblätter</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>KEC had difficulties at the beginning: The Kölner Haie won 6:3 against ERC Ingolstadt. - Rhenish advertising papers</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Sat, 28 Feb 2026 17:42:06 GMT</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQM0p3cC00Z2k1aXk0R25VWk84bEk3dXR0RkRDLUluUG9LWWoxTmNoMzJVa19QVDRHOHc5QU50Y2JRZTVqOXdKRVJDV1VNRHcwMEZlaE03dzZjZlRsTVV5dmI2ajI1S3FDQTE4ckZIZ1FWaWF5d2tMZnpLOXdVQ09aenYteUk2MUpUSUhXUU9XakhNNW9mU2psN0FWZ0NPaUZDa3E4aE1HTy16aWw2OGxiRnh5dkNnbFY2S3NBVXFDVlpVUjRmSlpF?oc=5</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K32" s="1" t="n">
+        <v>46081.73756944444</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Bundesliga: Bayern gewinnen beim BVB - Fans haben Ärger mit der Polizei - RevierSport online</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Bundesliga: Bayern win at BVB - fans have trouble with the police - RevierSport online</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Sat, 28 Feb 2026 19:40:35 GMT</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxOVWdubmNlZXF1TkVaS19NUFQ4U2ZJbTRfbzdDT3ZIR1hiaXc4UnNfTzVfcl83RHhRZkk2ODJnRmFTcGFCUmxvcWlLZU9ZbjRzMkduaWJzcUZlUTlRY0NMS0VTOE5PMzg4bThBb0pEUXdzM1NlclNzODNuSXV6bkpFWlJPX1hZaExzcnZPQkV6cDhPODQzaVl2Z3Q3MkRZSEY4enE3TzIyWGJJek56Q0ZESTNiREEzZzBfSFo4cXpGdlc0QQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K33" s="1" t="n">
+        <v>46081.81984953704</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Village Ingolstadt (fallback)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>FC Ingolstadt 04 vs. Mannheim: live game updates, stats, play-by-play - Yahoo Sports UK</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>FC Ingolstadt 04 vs. Mannheim: live game updates, stats, play-by-play - Yahoo Sports UK</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Sat, 28 Feb 2026 19:19:54 GMT</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOREVtNFlJR0lRTEZ4RjFmZXF2aU1WMkxNWldKQURQRWppZjFWUEhyekJuaDV4enNCQ1g3MHRuZzJXS1JrV0JkLU1DSnJXOGx2bXNkT0ZvUUhxQXJnVTRxckNCOGpTUDVPZjB1bzVxQkJqeXBkejFxWlg4aG9lTkNfTTBqdnVpcXNkZzN4RExn?oc=5</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K34" s="1" t="n">
+        <v>46081.80548611111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-03-01 14:25 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,32 +480,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Brand Protest</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>("Gucci" OR "Ralph Lauren" OR "Dior" OR "Armani" OR "Louis Vuitton" OR "Burberry" OR "Prada" OR "Nike" OR "Canada Goose" OR "Hugo Boss" OR "Moncler" OR "Saint Laurent" OR "Loro Piana" OR "Lacoste" OR "Versace" OR "Jimmy Choo" OR "Michael Kors" OR "Missoni" OR "Kiton" OR "Aquazzura" OR "Tumi") AND ("protest" OR "animal rights" OR "fur free" OR "PETA" OR "activist") AND -BAFTA AND -"red carpet" AND -"awards" AND -"wears" AND -"dressed in"</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Dior’s Exclusive Dior Or Ramadan Collection Epitomises Elegance and Grace - A&amp;E Magazine</t>
+          <t>B&amp;M European Value Retail: The UK Discount Beast US Traders Are Watching - AD HOC NEWS</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Dior’s Exclusive Dior Or Ramadan Collection Epitomises Elegance and Grace - A&amp;E Magazine</t>
+          <t>B&amp;M European Value Retail: The UK Discount Beast US Traders Are Watching - AD HOC NEWS</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 08:25:17 GMT</t>
+          <t>Sun, 01 Mar 2026 13:19:09 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxQcTNRLU9FMGxMXzhQMlk5SlRwNF9TZWZNWVlnSEhfeV9CMEUwYjdLVU1uMU1aaU9jS3lkV2hETExfTFRZNU1SRTZiUGZUR1dvNTBjalVqSnhiZVhPeHpXZzBSU2NFZWFGM3ZUOEliRDFQcTNrU2RZUUtxVGtfQndQaHhLUWNsalpKbjh6aUtlR094ZE1YZmVOaEpiTmNOTkdXTGdN?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxOV2NhNXFZcmFfUnVVYXUwMGRKbVFNZ3BhU0RqTmVKOWt4Q0FSNXRvcW1KQUkzREYyUzNxUXpBVUZGeV9Ldktwc1o1TllYcXRLcjdTNUx0MWZkZWlQZ3JNdno1eEhHcjJxSXJGTm52cjFKb0FkZ3hFVTVOTFdYVnRLY1FqODVIT09mYmxBRTNXX2xCMWZCQWFHMnRvV0VPRXl0aWw5NzVQZmYxUWJMQm01UzlnSDNzbVdxZTFreG8zMC0xVVU?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -529,38 +529,38 @@
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46081.35089120371</v>
+        <v>46082.55496527778</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Value Retail Brand</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>B&amp;M European Value Retail S A : Creates 30 Jobs for Locals with Brand New Diss, Norfolk Store - marketscreener.com</t>
+          <t>Explosie bij woning in Venlo, politie doet onderzoek - De Limburger</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>B&amp;M European Value Retail S A : Creates 30 Jobs for Locals with Brand New Diss, Norfolk Store - marketscreener.com</t>
+          <t>Explosion at home in Venlo, police are investigating - De Limburger</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 08:53:04 GMT</t>
+          <t>Sun, 01 Mar 2026 13:55:21 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxObHRuQUhqcllSTUotUXlXVElTTFgwbERBZjBpUkFBaWtDZUhHSkgxZ1dDcjFHalllaXI5bWh6cHUzdWM4MXgwS2lpbURUWHNkMEppajMtd1dwSnJMNWRqWERNU1I0NllrQnFMd3A2clcxWjFrQlZ6RER4WVVtVGxwd3lETzlqMXQ4OFBXNGZMWlB6ODFjejNvZGh1UmpFUU1INmMxVjI4bWRIVTZ2RGtydl9SdHo3dV9Da295M3g0ZjRrcTYwUXVndV8zdDY2UGpCVGgwb3BkOUJISWM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxPN0dXMDBnX0lwakEzbHQySHhLd1BUOElucDZWc1ZiczlVOXYzMWdOVXJDZktkN2c4QjR5aHZjMHpCS1FQQldPSzZqdUY3c2VDSkpjeXVIRTJ3QUtFbzdyODkyTTRyU3FzY1gwWmJ1a1FYYzAwNnd3czBOZzBUU3B1TFI4cmxLc3Azd2ZseHlKNU95bWdwMExQa0gxZlpPYjRLTXV1TTB5N29pdE1DYUE?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -570,52 +570,52 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46081.37018518519</v>
+        <v>46082.58010416666</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Value Retail Brand</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Dollar Tree, Inc. (DLTR): A Bull Case Theory - Insider Monkey</t>
+          <t>Leslie &amp; Agnes treden op in 50+ Ontmoetingspunt - De Gelderlander</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Dollar Tree, Inc. (DLTR): A Bull Case Theory - Insider Monkey</t>
+          <t>Leslie &amp; Agnes perform in 50+ Meeting Point - De Gelderlander</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 20:00:45 GMT</t>
+          <t>Sun, 01 Mar 2026 11:51:00 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxQMkFPVkxVZ2pNc1Y0V25USnltLXF1UDdoMmxPOU1Lb1NqMDlESHVSSVRUY09yM0kxU1BxQ1NDa251OHBZa0xQM3ZWeVNUZHliNUVnT0FIam5UV3JUSzZKWmZxakR6d3BXcXdidWxGcU9TVVNrM0U3Yk50Vk8tODYzSl9Vem1rZ3hGbXVTOUFR0gGWAUFVX3lxTE40dHFZalFmUjNXa0dXQ1dEZTZDaXRFNjRad21janYweWdFeHR0NndSbloydkZpcGQ3d0RuZGxFQnVMMi1JSE0ybGpKWEZNZ25iRi1RYkp2S2dkbEgwUktRaHJPY3VwcnhjRnRZLTktZWQ3MDFaLUt5MUsxM3NBbTZ5WndER3VOdzRXTGxWcjJUcDFMc29fUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxONW5pM29Fd0N3YURZcDVodU4yQXhhMnZwWDVYZl9yOEtPVmFGVHVTUGZmTDJWQVNsSllNSzhBQTdHNUV5eHZIQVY3OVIweFBwQUZhQWxEX29HWWJCanh1U2JzdnVqbkZ3eVpaci1sc1h4UHUzbktNU3NaU1JYTkNYVC1kMlp4UmFOMlRsMFZwWXk4cEp0YWNCM1daMlg?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -625,52 +625,52 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46081.83385416667</v>
+        <v>46082.49375</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BV Logistics Disruption</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("DHL" OR "UPS" OR "DPD" OR "FedEx" OR "Royal Mail" OR "Parcelforce" OR "EVRI" OR "Dropit") AND (disruption OR strike OR failure OR delay) AND ("UK" OR "United Kingdom" OR "Britain") AND -dental AND -"pay dispute" AND -"postal vote"</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Royal Mail warns 20 UK areas won't receive post on time this weekend – full list - Express.co.uk</t>
+          <t>‘Domme fout’ leidde liquidatie Khamenei in: zo kwam geheime operatie opeens in stroomversnelling - De Limburger</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Royal Mail warns 20 UK areas won't receive post on time this weekend – full list - Express.co.uk</t>
+          <t>'Stupid mistake' led to Khamenei's liquidation: this is how the secret operation suddenly gained momentum - De Limburger</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 10:47:00 GMT</t>
+          <t>Sun, 01 Mar 2026 10:49:29 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxNdWFkbzRSX2hQT1J5cjFJazJoQno1LV9tOEtaTExvYnJZVkF2ck5MOXRLQUg1TjdnTG9GQlZuQ3dIN2llaXRNU1I5MzNVS3ZyNEY3cFVCa3JISTQwWmdvdTBqZFl5REhkSHl2T2x2ZE40cjZLc0xNRnVWV2k0aVd2SzVYRXJwd1HSAYwBQVVfeXFMTWVRUmVlRHZxajY2Q0czS01XMDQ2M01TN3p1bnEyTGZXS0NwMFNad1VmbndpME1uTU9OR0tVMVA5OTQ1b2JiZFNSN3RONk9JVzZ6OUhyVmllTVZJdVBlQ0VRaWtDWnBTblZNMTJjS3pTWURYZDZiZDBqbTliM0RNaTJVdXFBOGVoU05hWlM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxNd0w3QVZQdXpoR2xGSmwwaGUyU0R4M0pmRFo0dTZyS0g5UHNCa2xDeEVrcC1YMzROakliOGRsYTlTZl9ZNU5UOTlrNXlJM2pfS2lJakMwWWU5d0s0VFlkR3VMcHFuVm1odTBEX1ZwWmVGcXNidHNNeGZfck1RVjFCcE0yRGNua0dvbEFNNEZfTkluREVTSUYwVjNQVmJnWml5SnJwWWhteUtyMldiaXo2SGhIZ25Gc1VHbEw5Q21CVF9mRzVQV1lVSno3c0RySWt2ZmVTcjFPelFvMV9v?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -680,21 +680,21 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46081.44930555556</v>
+        <v>46082.45103009259</v>
       </c>
     </row>
     <row r="6">
@@ -710,22 +710,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>"Af en toe opgeschrikt door explosie": Vlamingen gestrand op grote luchthavens in Golfregio - VRT</t>
+          <t>Poging tot brandstichting van auto in Venlo - De Limburger</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>"Occasionally startled by explosion": Flemish people stranded at major airports in the Gulf region - VRT</t>
+          <t>Attempted arson of car in Venlo - De Limburger</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 15:14:04 GMT</t>
+          <t>Sun, 01 Mar 2026 07:26:49 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOVTVfLWU3SXJqRDY5dHlaV3g3XzdzVXdNbEo1TnN5WHlGTEtVbEhyR3Yxd2pENDJZeGxHUmw2VDA0UmxnSEhMVlZuVUZUbF9CZXpqNWV4T3FYejNZOEpsQ3R3UHJXZENxeUs0cVZSckVaZGx6ZTV0cEtDcWpVSnNCU3Y2WFpoOTZmMmVsQk9XcXRCa3RmcFA5LTRUTGlrLW5oVmt1X1AwUEE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxPTDd2Sk0tSG5TaEEyZmJSdEh5UjJsUGE1bGdZZ0tOQVM4Q050eGp2T09leUI1Z0hrV2NXTjVZazhtbXZZc0hyYUhtWmw3ZHZxc202SzZod043RUJiYXZCX2NnclJMVllEM2NTekhqNFdSc08yM0pXdi11TDdjT1cyc0RfTVNVaGNFWGhfWXowa2k0ZzRVVkpLd09mdw?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -749,38 +749,38 @@
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46081.63476851852</v>
+        <v>46082.31028935185</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Explosie in Anderlecht: appartementsgebouw en voormalig tankstation onbewoonbaar - HLN</t>
+          <t>World leaders urge return to talks after U.S. and Israeli strikes kill Iran leader Ali Khamenei - WRDW</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Explosion in Anderlecht: apartment building and former gas station uninhabitable - HLN</t>
+          <t>World leaders urge return to talks after U.S. and Israeli strikes kill Iran leader Ali Khamenei - WRDW</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 10:40:17 GMT</t>
+          <t>Sun, 01 Mar 2026 11:38:00 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxOdmFTNmVmeVFpRC13MENWemxqWE8tSlR5RE1PaF9ZY0FkcFk1OGd0U1Vnb0NvUDBlRXhPR1huWHh1cWh1NGZkVTJZZmdTT2R4a1NEVDVwRGtzX2dvUmExeTRKdVMwclphOXNaUVdBTHBXcjlneHNiZ3dJWjJmMlpIZEFtSk16R0c1RkRvOUdFT210RGJtd2lWT1ByZ2duTnhtc3dMTTVtSkhEbHJJcm85YUxVNy0tcG5m?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxQcmZXbmpXeWQ4cC1kTXNGVFk5eVZtREpLdUNzb0d3WjFqd001eVVra3lDRVVuREdMWGxFa1NaUDhXS1FyNGZMaDh5VG5vU2gwS0JYN00tQU9rSUhRVVZHbjBUWG1td3piOERTblNzRHFiVjNBampXd2l5M2NtU21PNENfTjVfNVRlb3F5c2Mzc0tFUG9VWUdWVmVhM3p5dUhFbWtYYjY2N3poRHNHVmoxanJ6dmktbXdOMkloOTFjZzRiXzlyX29YVVZXelRTWknSAc8BQVVfeXFMUHJmV25qV3lkOHAtZE1zRlRZOXlWbURKS3VDc29Hd1oxandNNXlVa2t5Q0VVbkRHTFhsRWtTWlA4V0tRcjRmTGg4eVRub1NoMEtCWDdNLUFPa0lIUVVWR24wVFhtbXd6YjhEU25Tc0RxYlYzQWpqV3dpeTNjbVNtTzRDX041XzVUZW9xeXNjM3NLRVBvVVlHVlZlYTN6eXVIRW1rWGI2Njd6aERzR1ZqMWpyenZpLW13TjJJaDkxY2c0Yl85cl9vWFVWV3pUU1pJ?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -800,42 +800,42 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46081.44464120371</v>
+        <v>46082.48472222222</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Raad van State legt bom onder voorstel voor lagere LEZ-boetes - BRUZZ</t>
+          <t>Latest developments after US, Israeli strikes kill Iran’s Khamenei - Brussels Signal</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Council of State puts bomb under proposal for lower LEZ fines - BRUZZ</t>
+          <t>Latest developments after US, Israeli strikes kill Iran’s Khamenei - Brussels Signal</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 11:16:08 GMT</t>
+          <t>Sun, 01 Mar 2026 10:03:46 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxPWDl4MjB2WS00b1VZZk92cjNFNWhIdEZCY2tPQXhET0N3cFY3NlhSTmRQdl9GcFlLQW9oWnpzUUZtQ0ZYcnJXQ0YwdUdPbW5FMldxNXR5R1hNQzV5MW8yY0xfcW5RMTNsdWRCanZnUVAzNHhXWkY0OFkzYUVmZFZHZGtidFdjTkx4dDYtMkFPM1VRNkxpUDI1RnpqWllLYzFuZFdqcjF3bTE0dw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNM2cyc0hkVVN6OWl4b015NEg5OE9WRDFCTURIczFfenZ3ZzFWQzlpdk84dW1fYkhSTDhvcXliQW92cWJLODlEbUplV1JZS0VPWDdBMWNfTFdOTFU3dUpLZm9TdkdnQXRtdzhkYk5ReTJyLU1rb3VaMGFKSkhSR2F1eWt3cTV1NFRtMXFfbGllMmZlT084dkZlNjBTNzcxUjFY?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -855,42 +855,42 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46081.46953703704</v>
+        <v>46082.41928240741</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Loenhout verslaat Minderhout na hattrick R. Driessens - Nieuwsblad</t>
+          <t>"C'était pour l'aider à se préparer à un copain" : 30 mois requis contre l'oncle qui a initié sa nièce de 11 ans aux sextoys - BruxellesToday</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Loenhout beats Minderhout after hat trick R. Driessens - Nieuwsblad</t>
+          <t>“It was to help her prepare for a boyfriend”: 30 months required against the uncle who introduced his 11-year-old niece to sex toys - BruxellesToday</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 22:05:00 GMT</t>
+          <t>Sun, 01 Mar 2026 14:01:00 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxPamM0VlY1M1JPQUNseWYzWFp5TE1sZmFiTGs0M1YzNGJ4RW83S3VRT1luSC03LVlPVTRSa0RyRW11Z200eS0tZ1BmZHRGYW93TkJXVXlxenNTTXBWbmJXd01wTE1EcGgzaW9haWNsUmVsX3NyR2tsYVB5ekRISDB2WFU4SS1PVVhaOGtZZTNyS254NUxHSXA5ekhCMGVTRDNiNEhGZk1LbkxqeWxlX3BLYXVWMXAzNGIwQ2RJUGktUGtJQ1E3UUpobEFJaUNDLXkzbHdz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE1UZzVxX2V1UGpTOHBkZy16amxENkFQMzRTQzRzOXRYTnpyYkl5S2lQMHFNM1pzNkdIOEhSbWE3azNaUGRLUERWbW9KMm5pSlN1RUo1ZHA0X2RtVTVINHhXdTNlWmV1cVdXc2hxZ05RTjhxaXNodG5OT1BHVEFKYTQ?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -910,42 +910,42 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46081.92013888889</v>
+        <v>46082.58402777778</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>LIVE Midden-Oosten | Explosie op bekende ‘palmeiland’ in Dubai: beelden tonen grote rookpluim bij hotel - De Gelderlander</t>
+          <t>Une collision “grave” avec un tram à Etterbeek: un homme coincé dans sa voiture - 7sur7.be</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>LIVE Middle East | Explosion on the famous 'palm island' in Dubai: images show a large plume of smoke at hotel - De Gelderlander</t>
+          <t>A “serious” collision with a tram in Etterbeek: a man stuck in his car - 7sur7.be</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 16:05:00 GMT</t>
+          <t>Sun, 01 Mar 2026 10:40:00 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxPem5yNEJIVGhITFF5Q0JpemRya0kyNUc4eEtrOEtPLS1tdDh4VTRuMG5YXzNJN0lOR0x0emwwMENuN242M3V0Q0VwX1VNOFFFdVlLS0xudFU4bHgzN0lLRWtobFdHLWQ1Z3ptOEJnaDVBY1lHUnVuU3lWMVZYZDUwSnVDUGljMlItYWZHLVJPOVhkelNHdzlsTEkwcHJhb2FTRnlxeF9RdndDT3c5TElGQVVQakxwdmtWNGFVRk1PZFF4NUp1VWx3aVI1UnRRb3pGWTczb3RQZ1BOXzJFMFdvaXo1Rkc0ZG8?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOTlg0a1R2dENOYnlpTzFUT0JqT1U2b0wteHBuZklBLUc4cFdqQjVmeGdQenBNVTh4eXpjMTBHNDdSOUczZlZuWjg0d2VqSGROQ1ZySGZUNTJKSWhxVXR3ZHdwV2xBekx4a3lwLXN6bUw5dk5wUzFSNHJ5RlduR05qZkhLQU93RVFudVhvRnE0MUlZb1o1em1EWVMwZkp5ZXRWZWhQVTdhNVZPYnhGUHo4ekdYMEdEN210R3hZbA?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -955,7 +955,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -965,42 +965,42 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46081.67013888889</v>
+        <v>46082.44444444445</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>World leaders react cautiously to U.S. and Israeli strikes on Iran - PBS</t>
+          <t>Depuis Bruxelles, des Congolais de la diaspora montent contre la déstabilisation de la RDC - Radio Okapi |</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>World leaders react cautiously to U.S. and Israeli strikes on Iran - PBS</t>
+          <t>From Brussels, Congolese from the diaspora are rising against the destabilization of the DRC - Radio Okapi |</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 17:20:20 GMT</t>
+          <t>Sun, 01 Mar 2026 08:22:30 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxQLUJXZDl4eVN5LUUwa3VzbTcxdk9sWWJNSDR6SG9acXZ2b0dUa1Y2T3RjUVhWVHRMam5oOThFdnlSbUY5QUUxLVRuNTZObU1GTko4dmZLUlhrWTZsRGZ4RWVqV1IwNklTSTloZk9xRmVDeUdRT0pOcVdTbm5pajZCODJpblVlX3ZFejAxUjN5eWpqdWlSdWtQRmZSWm8yVnI3bHfSAacBQVVfeXFMTnFhODl4OW9ZckRRSDFjeGRfU0Fjb21rMjNhOThyaHJUS09QSmVPMVYxT1NnTHZnNTh5Q254TTlqOXFKZzJtUXNxa0N6bFRPMHkwc3ZjVmQ2Z21Ka2pGUW44OFFaU2I4OEdrR19LX1UxaHJ1clJZeEpSMlUzLTF1WFgzZXhqVU1kdXhkTkhuamI3T0FiUHcwNzJSLW5YRHRlWS1WbFRkYm8?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOM2JsbUlfVE5LZ1ktX2swbExvX1JmTDdmRWxkS0d1WXg2WGhKRnNzWXpkV3gzTkhwNHBzeWl3WU5SQTlhVXdxQkt6V240OU9hXzZXd05ZNWFIREJ1U2xhMHF4bFlFa2xkSnZYWk9ZSS1wUU1VR0RoYW1Pb29XbUR5bHdfRE1YMjZHbmFQTmdrVHgxVTkyS2l0Sm1CNnJkWVR1Yk1vR1N6Y3RvU05GNkU3UXJOclF2UDRkRVl3?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1020,42 +1020,42 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46081.7224537037</v>
+        <v>46082.34895833334</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>World leaders fear broader escalation after major US and Israeli attack on Iran - SILive.com</t>
+          <t>Euerbach: Autofahrer flüchtet vor Polizeikontrolle - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>World leaders fear broader escalation after major US and Israeli attack on Iran - SILive.com</t>
+          <t>Euerbach: Driver flees from police checkpoint - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 13:49:00 GMT</t>
+          <t>Sun, 01 Mar 2026 13:09:00 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxQb2lZeXRCcThuSjdkcGViU2hJTEpSbUtOTjJNemNUQWxweXYyMDlfT3F4ZE1MWWNjb2xPYzhhQ2RZTDkxRGdBbGQ1bFlLblVXVjcxZzQ5bDh1RGVpYkxER1ZjREhZRjd2LUpkbjVqZU00ak9vQ1dmTlo4cHJXNFRrMGZ4TEN6WkUxUjNZcHktM0lBU3Z3b2RtampQa2FfT09TNnJvTnRQSExpX0ZSVnV1aXM5aU16Slc4QmN4ODgxSdIB0wFBVV95cUxQeThVM3lXRmYtNzlUZkFWVE5oeUJMdWtpcmcySzJSc1MxQmdKWV9TV01rYURDVzBTR1dJcF8yY3VTdXpNWkRkQWVkMHRiZDBOQ0t1dl9INEJUd3NHNER3SnJVMkoxeXZXSFgwWktNc29zQllROXA0RDlFeFFMTUxYV2IyM1h6cWJ2anNmc0M5MjRvOVZiODl2enYteFVQWG5aZllIV05DMTgzNmFNcF96RXpyTjVBdEhlZW5HbDd0OERMVGJDS1lKMmU2bm1CNHJaNkNV?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxQeVZJNy1mVGIzZ2V2emN6c3VYYWs3dFM5S1BPQ05yLV9UOGVnQk1NWUM3a3VZVlhNWnJYeGptS0tNSHN1cEtxX0o5VHFBc2t5X3ZWTGt4SkstOG9WZEowZzhVNkVTVGJDOEhZU242Z0d5VEJGZXVGS093bGVza0VYcXBvUFpjenRSWlI1UQ?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1065,52 +1065,52 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46081.57569444444</v>
+        <v>46082.54791666667</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>EU caught in the crosswinds after US–Israel strikes on Iran: energy, shipping and security risks surge - EU Reporter</t>
+          <t>Unfallfluchten, Autokratzer und Eierwerfer | Foto: Jens Buettner (dpa) - main-echo.de</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>EU caught in the crosswinds after US–Israel strikes on Iran: energy, shipping and security risks surge - EU Reporter</t>
+          <t>Hit and run, car crashes and egg throwers | Photo: Jens Buettner (dpa) - main-echo.de</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 17:10:36 GMT</t>
+          <t>Sun, 01 Mar 2026 11:36:26 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxNZ0d4aG5WZWdHdHBWZ19aNmdvRWVwUm1mTkhaa18xcERUTXZnMDF1RG9TLUZMNHgwMlRaMXJ5N29TRzl0cl9MMjJlQ0xOUEpXV2lUWTZlUHBLeEVXWVY4dEJ0N3JvVHVYR2ctNV9aaDFrWG0ycGZiUm1NcnNqbnBtRWlrbF81RndGUnl4NXptVkVTbl9PRTk2cFpjakVIOWZmc1dtM2ZhQ0k5cFZISFI1clJNRXZSQ1RaNjF6T0hWVnUxcUJUQmM1UHBiVGVhMTlFTU9NaHJDTEFaTXJ5?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxPS1hnZDFGQkVqeE9hRTlRY1pNbVBtbmRKbEkwSzZIQzRSVENyMFczOXllOGg3SUxYaG8ybngtOTVEeU0zWWZfZnFPRUdBYVA0NmVmSmVuZUs0OGJvdFFhX1VNWUZzaV9DdnRGcWRDX2kxZklMemw2SkdFaDFoZ0NtVHdXZEJnZnlRU2NhZDlLc05Kb2dLTnk3bmJ5YnN6QQ?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1120,52 +1120,52 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46081.71569444444</v>
+        <v>46082.48363425926</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Former petrol station explodes in Anderlecht - The Brussels Times</t>
+          <t>15-Jähriger liefert sich Verfolgungsjagd durch Aschaffenburger Innenstadt | Foto: Carsten Rehder (dpa) - main-echo.de</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Former petrol station explodes in Anderlecht - The Brussels Times</t>
+          <t>15-year-old chases through Aschaffenburg city center | Photo: Carsten Rehder (dpa) - main-echo.de</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 11:15:25 GMT</t>
+          <t>Sun, 01 Mar 2026 10:01:41 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxOeWFacnRqcHFrSERIbnNXbFV3QmJqSFI3RGpWcjdvQXNvWHN4YUdoTVFOdG1jYUcxbl9lLTNyNFNqMUNaekZoWkJ3Z01tZS1RMTQyeWh6TnhDV01mZ3RoTWkwdkRUZHZBMXVPcm1HdzdtaGJ5YlNLRE9hbnVoTWJNb1p0eHgzQXZmQURNQVBQaGJDX2FE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxOd2twSWJDYWhXVjhyclZ1RF81NGxFbTUxamlzWm0xU1VKRk5OT3pGS0xUbWkzMWlpOEZCT1Q3UHFnNUlNb2xTTmdnczZmcThvVVp1RkJWQXRJd3hBT2NLN1o3TnNlZ3NXX1p4UDZhSVV2aWhoTGY3Ujc4RkFwczVtSThFODBRaDdra1V5ZjhSV1BWcll1MWV5RktjTDRaYzRMMVgwNEJpdTRwQnVLNWt6S3YxaWU3ZzJtUDdnVHFadlJrbmFhdlJtZlFB?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1175,52 +1175,52 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46081.46903935185</v>
+        <v>46082.41783564815</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Dubai authorities say drone debris causes fire at Burj Al Arab Hotel - HESPRESS English - Morocco News</t>
+          <t>Nach Messerangriff in Würzburg: Keine Hinweise auf Psychose | Foto: Michaela Johannsen (dpa) - main-echo.de</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Dubai authorities say drone debris causes fire at Burj Al Arab Hotel - HESPRESS English - Morocco News</t>
+          <t>After knife attack in Würzburg: No evidence of psychosis | Photo: Michaela Johannsen (dpa) - main-echo.de</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 23:24:47 GMT</t>
+          <t>Sun, 01 Mar 2026 10:37:20 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxOMUVwS3B0VkNDWG5ZZC0wcW5idzhqNTB4UUJFWGVzS1BrWF9sUTJNNkhuTU9odEhSX1hSUUx0UzZFbWt5VWNrWXlua1loYW1FM1lKNE5JRmJ2SlBaVElwM1FlcnJvY096eTZIVTRGbURlZUFURlh1UUd5aW0xYWNHWTdBU1dJdUthMmJ4U2hlYzRxZVIyVXBnRFhQRENLczZaUV9VQ0Nyaw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxONkM3U0l6TFZWaUF1dV9CX1hqcWV1TjM5c1kzTWxlcjNreWN0aVFhXzZsUDRIOHZVcjdKcnRaSElTZGgtejljajdXYWhBbTltVkQ0RnYxaklMUW5VMGgxN3hGbVJrVktrSHN0dFF0MzZXSTF5QlVKeVRZVFluV2JNSWxvZzdMeW9IYndWN2t2MUlQMmR4a0ZLNGkxMFUwNTJjTVdNb1F2VnFHMS1PR3JVZ0YyaS14UQ?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1230,52 +1230,52 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46081.97554398148</v>
+        <v>46082.44259259259</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>EU withdraws Middle East personnel after US-Israel strike Iran - The Straits Times</t>
+          <t>Darum ermittelt die Staatsanwaltschaft gegen Beamten der Polizei Marktheidenfeld | Foto: Marijan Murat/dpa - main-echo.de</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>EU withdraws Middle East personnel after US-Israel strike Iran - The Straits Times</t>
+          <t>That's why the public prosecutor's office is investigating officers from the Marktheidenfeld police Photo: Marijan Murat/dpa - main-echo.de</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 10:57:48 GMT</t>
+          <t>Sun, 01 Mar 2026 11:08:20 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPZUNpQUQ0b25Dck1nc0ZqTlZiMml4TW9YUG1Ccm5uT3ZDVVR1dUpGbi1ISHQxaHpNSWJLeS14OXprS2pfeTR1UFJhYjNMQnhqZExteV82MUkxR3g5Q0UyZVB1Rkt4Ql9KTGppZ3NqbVNseE1tcTZuVTVReFhPSGx6S3dyeWZHY0tBWl9QcFNhTVdSQVdkYzg5LVFhTFJ5UW52Q3hpQl9URkNpLUct?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxOQkU2ci1Ieng4YXBFbzM0eTFFZWl3ZzVkcFE3SkZRNFpSWERhdld2dWJRR1l0UWZxQTNMbmNVV09yOGUwbnpfakYxSnBTX25Ca1A0OGhrcngtV0c4ZzJSb0V6Y2FNczFVa3NXd1B6eV9KcHoyOUNkLU9wbVFsdGxzNzVxNXFyV3ZucGlTc2NWbVJpNUxpRnV3Sm9oYnNBRklDal9nblZWMTExNmRHNlpON0dMNUlha285WkVOczVyU0ZBaElXWS1RR0FQdjNlT0RfbEtRT1hzd01YSzQ?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1285,52 +1285,52 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46081.45680555556</v>
+        <v>46082.46412037037</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>EU Leaders Urge Restraint on Iran Situation - Devdiscourse</t>
+          <t>Blitzer in Würzburg aktuell am Sonntag: Hier nimmt die Polizei am 01.03.2026 Raser ins Visier - News.de</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>EU Leaders Urge Restraint on Iran Situation - Devdiscourse</t>
+          <t>Speed ​​cameras in Würzburg currently on Sunday: Here the police are targeting speeders on March 1st, 2026 - News.de</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 10:41:48 GMT</t>
+          <t>Sun, 01 Mar 2026 13:15:55 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPVmxfVHFUUUJvbm1wcGdwYWdFQmo3alprRC1JWHUwVnJfaDdYeUMza2hDQWkzQnI2WmpHQUhfMGlvNmNhUGZ2UGptRjBJMV9pNEV0WWF3d2g5ZjJBN3lfWmhDTngtUWZlX2VvOHBwUU8yOW5RUTlTVGlZN2dkb2gxZWtXX2xnSFozRnltOXhjTEIyQ1I1WTBreFowMXZISzJob0F1T9IBpAFBVV95cUxPVmxfVHFUUUJvbm1wcGdwYWdFQmo3alprRC1JWHUwVnJfaDdYeUMza2hDQWkzQnI2WmpHQUhfMGlvNmNhUGZ2UGptRjBJMV9pNEV0WWF3d2g5ZjJBN3lfWmhDTngtUWZlX2VvOHBwUU8yOW5RUTlTVGlZN2dkb2gxZWtXX2xnSFozRnltOXhjTEIyQ1I1WTBreFowMXZISzJob0F1Tw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxOWEs0WUU4QzFMVWt2eS1pSnctVGxnLXBLQWZBZllOSkltR0JzTDRKdk1NUVlhdXNWLURtTUUyZXY0ZnVZZFhrQmxTNy1SdW5OYWNLc1RSNmtKM1lkQ2V2dWNLQXNSUm1JQWFDcG52YmFMVktwVW1KdGZRWVBUNURRODUtT2txZ3RvOEtTRlQtNVRqbV80VDF0eWRIYlB1R0lqek55bjNFWE5WWVQ2ZVo5LXFjVUgtSFJkUGV5WklaRGhENk9ZcTBTb0FYNUdEa0ZxS29McXpnZWJieUVmSE5ka0k0ZFpocXfSAewBQVVfeXFMTk5mTXF1M1NvOEZVVFhlTXk1eWg1YVg5T053TEtMRWNfN3NlWm5ENmZiSEVpTFpJVTc5M1hJaW5TakpNa1dLZTJ5LThOTFJsQndBVnY5MEFTTXQwSmZZcjZOckVISmloS2ZyVjlYU1NUVGRhc3RVRldEck4yZlJDa3pObHFxWFRJdTNUMHlIeXJ1YmpWUXRnLXJoeHZGMTl4M0ZyNVVkZDdkN1VJLWtrMkh3UU12cmxtcUlpc0FqSDVybmdFcTBxR1l4X050cW03S3daSDBhbHZmTXBpUzd4TmhqSHhwNDdzcmZ5UWM?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1340,52 +1340,52 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46081.44569444445</v>
+        <v>46082.55271990741</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Explosion à Anderlecht : un immeuble à appartements temporairement inhabitable, aucun blessé - BX1</t>
+          <t>Polizei-News Nürnberg, 01.03.26: Halskette entrissen - Zeugen gesucht - News.de</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Explosion in Anderlecht: apartment building temporarily uninhabitable, no injuries - BX1</t>
+          <t>Police News Nuremberg, March 1, 2026: Necklace snatched - witnesses wanted - News.de</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 10:28:00 GMT</t>
+          <t>Sun, 01 Mar 2026 10:47:02 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQalp1ODR5WVRrQVhPTmJpOFVaUnFnZDNQaC02bEhQTDkwRnJNcG04Z3VnVWYxOHFsQ2p0RnNScmtCN1NVV01OWXd1RDQ3S1lhNWxFUjE5OTR5d2FqSnBFZkgyellMUVRvR1gwUVMzV0Jfa1l5RFd1UDUzOUxPeW01TXJqbU5VZ3dfcjBOMXpMWWZMSTlUU2JQV2V5dTIxYmZ6WE5hQ3Uzc2pxN3pNem4zRzJ5V0NLeUFpc0d1WDBB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQeG9XaEpTdFVBeGRuMjdSYXR1SlhLSS04X1hlaVFSY3Rnd0YtRzJNdFppVVRPTERnQkZrZWw2NUFndmhyRm1Wa09XT2hUak1lOEdWREI2TVdqTENZZldXZGVRQVJDZGhESHJnYy1na2Q1d2t4bndpbEI5dFdWUndpVXItb2oxYjA1S0p0N3o3REhIdUFlUUx0atIBngFBVV95cUxOWGtnVDZuUmZtbzQxRzFJUmhiUkh6ajNrb1pRS2lZXzV1S2JrYmQyUkJDdzFfUTF2bDVka2hmRlNTYU5zM1E5cDVfOWpJYVY2dDRYNEJuUkYzUUZYTVlBZmd1SnE4OXZRcXFjZlh4aGtEb09uQkdyMWhpVEE1WXM5eDZRWlpSX3lUSjFSakl4enctenUxblp3ZUJmNjdKQQ?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1395,52 +1395,52 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46081.43611111111</v>
+        <v>46082.4493287037</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>L’OTAN examine le renforcement de ses capacités nucléaires - وكالة الأنباء السورية – سانا</t>
+          <t>Polizeifahndung Nürnberg, 01.03.26: Bei Verkehrskontrolle Betäubungsmittel und mehrere Fahndungsnotierungen festgestellt - News.de</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>L’OTAN examines the regeneration of nuclei capacity - Syrian News Agency - SANA</t>
+          <t>Police search Nuremberg, March 1, 2026: Narcotics and several wanted notices were found during a traffic stop - News.de</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 11:04:15 GMT</t>
+          <t>Sun, 01 Mar 2026 10:47:01 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE5Wa0oyYTdqZXhoNFRESmxsaXFaVlZtVlV0cnc4bHdRRUhwSGQ1ajFBTHZ2b05RYWFyMFQ0aFYtektuX3h4a21vZ1NwVE9UaVlsYW1J?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxNOEpNcTJyeUE4VGRHSm5aQk5fcGh3MTlmcmppeDFDaVpuN0lGMVFRQWRxM294ekUyNjFYUVozdHZqWVZsVVhpV0R1T0tZV0lnelJZSG9ucWY1elBlUG1NdHVGemE3UV85YlpSd2VOQlBoR24yd1QxVHgyWlNXdkkyOUt0STFJRWhKaXZjcldQMVg1MWt6MG1nWWZTTVRBNzg5d3VXOFFibzVLWDloUVFHZHlaV0R2bUlFZ3JmQWxJMNIBxAFBVV95cUxOVlN3Y1lGMXd3VU9xTVhFbmpwN2YzTHdTZ3Rla0ZldnRRc3l3bjFWT1Zpbk8ySlp2TDNvX1J6M1NfdHFSOXlMVGVMVUNRV2ZyenMyNzhiLWhIQlotNXpHVHAtODlxWlJuTzdJX2hNb1NfYjJudS1yeVZJbHA5eVhIdVZjWm10Q09IZHBmcnhzQ0N2WkExZm1WQkNmNW8zQWo5MUFGR1BqcFBRRlV4LWdkVUw4Y1lCTVFnNkFhQXdkWmZTQzNI?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1450,52 +1450,52 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46081.46128472222</v>
+        <v>46082.44931712963</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>"Ils m'ont enfermé dans un égout": Zakaria, 15 ans, grièvement brûlé à Anderlecht revient sur ce qui lui est arrivé - BruxellesToday</t>
+          <t>Polizei-News Nürnberg, 01.03.26: Gestohlenes Lieferfahrzeug tauchte bei Ladendiebstahl wieder auf - News.de</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>“They locked me in a sewer”: Zakaria, 15, seriously burned in Anderlecht, talks about what happened to him - BruxellesToday</t>
+          <t>Police News Nuremberg, March 1, 2026: Stolen delivery vehicle reappeared in case of shoplifting - News.de</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 16:45:00 GMT</t>
+          <t>Sun, 01 Mar 2026 10:47:02 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNaVlPc085QkU3dDB1Uk9zT25JSFl6RDNOUHlKcFY1dzVmazYxcW9PckFvWW96TDlXaGFDRVhkVEpSa25NSGtWZXNIUXIyTlhRSjdYTnB2aWlMcnptZVUxQ2d5UUwzbnBBRGZIdHJ6ZDA2SHoxTjNfdVo2bHcxTXpmbV96eHdSSThpeWVzdVJIS3hrWDBHbFF0eFk2bmV0bUNqTUJmVVBn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxNb0lKZ3pJVmVhOEQ1LTViWTI2czQyM1RFaE5IY0hlMncyaVhLRDE2cGFuQk82YldJZHo4bWpVanh3OGN6MzQyOERyQ3Rqd29BNmd1X1FVdFFqU0ZwNEZYVndubFBaZ19NWVlJZGw5dnhnVVJiVGRJekgzX3lGUEtpZVFKbVUtS0VVNGdCc3V4R0t4dkk2enU4b1FR0gGaAUFVX3lxTE1vSUpneklWZWE4RDUtNWJZMjZzNDIzVEVoTkhjSGUydzJpWEtEMTZwYW5CTzZiV0lkejhtalVqeHc4Y3ozNDI4RHJDdGp3b0E2Z3VfUVV0UWpTRnA0RlhWd25sUFpnX01ZWUlkbDl2eGdVUmJUZEl6SDNfeUZQS2llUUptVS1LRVU0Z0JzdXhHS3h2STZ6dThvUVE?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1505,52 +1505,52 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46081.69791666666</v>
+        <v>46082.4493287037</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Accord UE-Mercosur : Emmanuel Macron critique l’application provisoire décidée par Bruxelles - Capital.fr</t>
+          <t>Amtsbekannter 29-Jähriger tickt in Ingolstadt aus: Drei Polizisten verletzt - Pfaffenhofen Today</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>EU-Mercosur agreement: Emmanuel Macron criticizes the provisional application decided by Brussels - Capital.fr</t>
+          <t>Well-known 29-year-old ticks off in Ingolstadt: Three police officers injured - Pfaffenhofen Today</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 08:49:40 GMT</t>
+          <t>Sun, 01 Mar 2026 12:57:08 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxPVmJieGlWamItX1hMSGVCczVyRmRYR0hZcGRONldodE5leXozQlJjY0pySTQzcEtGNU5VUF9PMTMydWVjcDR5QUo0bUo4cDIyZXVUOVhzVEdJVHFZS0FHVjNrNjNNcHZYNWJESzFqNDQyWWZIaWlzV1hhVnV2Nzl1bGYwb3IwT2pzbVpwRDY3WUduSnNwX094Yk84U1lsdVVJQk1DSDhQWTdfN3YzZ0pYal9kNllab01BcFZHb2FfZmJhTEFodXF2UE40QzA4VzFJMVRPQ2tWNA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFBvamRMTVlQOWd3bWlUcUFZUGxnVUR1V2ZHLVBFTUJMMTVvVWs5b3RSWVVUdGxOWnAzZHpTRnVUY0dxMG5vRnNzSGRqWXlEM2RGTHRIXy1MZzNOdw?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1560,52 +1560,52 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46081.36782407408</v>
+        <v>46082.53967592592</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Meurtre de David Polfliet : crime homophobe ou "chasse au pédophile" - BruxellesToday</t>
+          <t>Kontrolle auf der A9 bei Manching: Etliche Anzeigen für Fahrer und Firmen-Chef - Pfaffenhofen Today</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Murder of David Polfliet: homophobic crime or “pedophile hunt” - BruxellesToday</t>
+          <t>Control on the A9 near Manching: Several advertisements for drivers and company bosses - Pfaffenhofen Today</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 12:04:37 GMT</t>
+          <t>Sun, 01 Mar 2026 13:49:11 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxQQlNSV3ZjX2FYSm1xTUI5TWJfSnVJVzRxdEZzRnU3azNQUkNPMUJwQnVFR21OLXdWQ2g1YmRQTHBaTndNWDBBRndvREVjRUxRdExNOXptbjIyT2o3Y1JXWmRCWFFQTWxRLTFBQlFCTlFSdlg0OV9ucUc3NEJ4eVRIYTU5RDdTM1RGWEhKS2pOeHpRcVMzcU1nQWd3WQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTFBmZ08ybkRQM00xOGNTdThLX3BqWFBrM0FyZHFfcUY5RTJheWcyVFFYTmdmaGdxbEVWZ1AwYW9rTHlkZmw1ZUF3Ym4ybEFfWjE3enRjM0RuczFPaWNGNGxjNzhR?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1615,52 +1615,52 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46081.50320601852</v>
+        <v>46082.57582175926</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>Village Ingolstadt (fallback)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Fietser (59) vlucht weg van politiecontrole in Hasselt en belandt in Demer - VRT</t>
+          <t>FC Ingolstadt 04 - MSV Duisburg ai prediction 04.03.2026 3. Liga - Livetipsportal.com</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Cyclist (59) flees from police control in Hasselt and ends up in Demer - VRT</t>
+          <t>FC Ingolstadt 04 - MSV Duisburg ai prediction 03/04/2026 3. Liga - Livetipsportal.com</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 15:23:45 GMT</t>
+          <t>Sun, 01 Mar 2026 08:01:06 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE5jZVQzeHVNeGJaa3BEOGxCTkNyWnlZZjFodmFQdW9yTWRDdjlWYjN6UGJ0U1hEVjE4bGFLLWpVZWszT0ZWcGVWNmQzSzJUcHN1WGExYkJjek9TQTczQnp1NjZiY0lSRGh2TmwyLTdDUV9tcDRfN0FRbk1uazc1V1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPbUtOZV96NU56ZDlBa3d6VGZWMVczSTY1aG9RdmxpWEZHTDhzMllMMDVrSmZWTWlWN1ZLcDhYc0xtTGg0TWkxaFdlSU1RWHFwMlV0UkpaS2piLTZkcEN4MzJxQmtxSG1NUk1JSXR3QUFlaUp4V1QyMkJyc1JJb0NIQVFjSHFFeGNWdDJUMUFCSVRMQ3Y5cDN1NlVoS2F0VEs3NXhVdA?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1670,52 +1670,52 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46081.64149305555</v>
+        <v>46082.33409722222</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Warme maaltijd moet rust en verbondenheid brengen in wijk Ter Hilst in Hasselt - VRT</t>
+          <t>Six Roald Dahl films returning to Bicester cinema - Yahoo News UK</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Hot meal should bring peace and solidarity to the Ter Hilst district in Hasselt - VRT</t>
+          <t>Six Roald Dahl films returning to Bicester cinema - Yahoo News UK</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 10:26:04 GMT</t>
+          <t>Sun, 01 Mar 2026 13:00:00 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPZlNReUNVMGNsV3ZNRlE5YXMwcDRuYnppMWlQUmxVT3VDNzNfYW9tVGFyTlBaUHFocFhKQ3BjMlotMHJOR2h3Mmw4WWhnaldSZnVNY3FwZHo0VFB1NEpLVVQwU0ctbk1iZVZyYXRaOTJ3OGJYeEJiMmhMVmxhWUN5c0hVT3pPU010SlMyOUE5NzdORDJYTGZZWFlhbEhLQ2VwcXVvSzdUdEo?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE5mTFh3b0RaTmlseVlPMXZzQnBfZXB0enJuSVJGdlNvWHU2TTZpSTUxMkZqWHo5Nk9oT2lFWEU0aW9pUFZOajR0ZHBjZFh6c210X0ZRRmpWaVNDRUJUaDhKNUJXekx1RG56NFFTVDhPTDlKQmdrN2RGYnQ2UQ?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1725,52 +1725,52 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46081.43476851852</v>
+        <v>46082.54166666666</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Handball (SHL) | Visé, la révolte avec du sang neuf, à Hasselt : « On va disposer d’un groupe plus étoffé pour les prochains matchs » - Sudinfo</t>
+          <t>Pupils debate internet access at Kildare semi-finals - kildare-nationalist.ie</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Handball (SHL) | Visé, the revolt with new blood, in Hasselt: “We will have a larger group for the next matches” - Sudinfo</t>
+          <t>Pupils debate internet access at Kildare semi-finals - kildare-nationalist.ie</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 11:00:00 GMT</t>
+          <t>Sun, 01 Mar 2026 14:00:40 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPV3RvZjJUUnJ3dW1oSHhBUlliNDBFS0ZHUkZmWEZsT1lIWlVXZVZMRlU5QmdRS3ZZSjV3SXR3bzJUa19SaDdPd3VRNFdhS25YM25nTGVJRFFFeFIzZk5FdGliNmhfb1B2MThMNGJjSk14cnJVVlNFckVLSDN3NWJQcFd2ODJKTUx1VXh0M1ZsS3B3Q2Vjd3lQb3BNN0xHbEJHanU2b2ZBMktqMm82Nnozb2d0OF80ZURGdURmMHU4YVh0MTlKclhlUg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPTWJxUFhsRzQzVmxqRXpJZG03bVcyemlKcUNGU2RxSXBYeVp5Zk5tSE5sV1pEYnJubno5ZFpuQXFuSGZfVTRPUldROEZLUFotRGkxNVFNQXBBOFp4cnU1LV9vZWtTU2RoYmdDLVdzQ2J1bVRUTGJYRUJQNW5YZWZWYXhyeWhZWWdaRHVOSVVFZVlPWW8tOG5qWXdyVEw2T2hQak0tYnFpdWVLa0Ew?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1780,52 +1780,52 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46081.45833333334</v>
+        <v>46082.5837962963</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Highlights: RSCA Futsal 21-1 Sensei Sushi Anderlecht (Futsal League) - Anderlecht</t>
+          <t>Kildare primary school 'not fit for purpose' according to report - Kildare Now</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Highlights: RSCA Futsal 21-1 Sensei Sushi Anderlecht (Futsal League) - Anderlecht</t>
+          <t>Kildare primary school 'not fit for purpose' according to report - Kildare Now</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 14:10:27 GMT</t>
+          <t>Sun, 01 Mar 2026 12:00:00 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxOZW9SV3hPdlpHN0hfaVFlR3h0aVlVMlA3ZzYtLTFObWY3a2FpdnRYOUVNZktHMUtleGRaMF9va1ZsZ3NpR3BTd2hkMS1fMUl1elhrQ3IwTmNqN2xQWWhLYzlGTldiLVd2RTZCTnlieFdQUWVGM3c2SkE0d3NfVDVXMmZHOEhJQ2xfc04wNnB2d05MYnEtUzdEQg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxNbzRkZllMTmxqd01mM1QyV3FDM2tyWDIwTFF6R1luYWxDWVU2MXFOMU90amFRd0tEWXRxbURFU3hZODlTREYzTXB6ZUJNVG1fTFRCS2ZsMnZ6ZThUUEZCTlI4bDFyZnZaUXp6dGloZmFCNGF0T3NxNF9Vcmh6VVQyWDlXZFZ5ZnJzcXR6bGVqMy1uZWNPZzFsTlJhWUxaVVpPT2RVLXp0VFN1Mkp1WUFQd2lyby1Vb2VGaGc?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1849,38 +1849,38 @@
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46081.59059027778</v>
+        <v>46082.5</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>AI Prediction: Roeselare Daisel vs Sporting Hasselt - First Amateur Division 01/03 - inbet.io</t>
+          <t>The two things you should never do when washing your wool clothing - Bicester Advertiser</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>AI Prediction: Roeselare Daisel vs Sporting Hasselt - First Amateur Division 01/03 - inbet.io</t>
+          <t>The two things you should never do when washing your wool clothing - Bicester Advertiser</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Sun, 01 Mar 2026 04:14:03 GMT</t>
+          <t>Sun, 01 Mar 2026 09:35:50 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxOZndFU05ET1doZnlZaEpwenNkUE94MjVCaG5mdmd1SVBCUy03ckhUQjRYMXpjNGh5bXQ5aTExR0treU1DenV2UFJFbTFHRWs3elZsOXgwUWUtdHBsWkJfRjVuTkNwZUhNekplREtVN0trMWROVWZqTVlmYThKTFpudVlqX0NJekU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxQc3RlblhnN3BZTFNvT0RpRnBDNFMzdG5hOXhGS2FMUXhxdGh6THN5eDg1eTQzbG9vZjFxN2xwLXZmVXpDdzZUOU9aQjZqaE8zS0M5TEVEbFZnd1BHRUpuRl95cjFERmpUcVQ4S1dnZFk1d1MteVVlbEZlNHdtMm9LTmw2eUFSMTN2OGE0NHRyRlBqSGZHNjhPZElYbnJFRnVyZDZQODQ3UjRtaWhxWmc?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1904,38 +1904,38 @@
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46082.17642361111</v>
+        <v>46082.39988425926</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Waldaschaff: Polizei sucht Zeugen nach Angriff nach Faschingsparty - aschaffenburg.news</t>
+          <t>The one brushing method you should always avoid to help save your teeth - Bicester Advertiser</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Waldaschaff: Police looking for witnesses after attack after carnival party - aschaffenburg.news</t>
+          <t>The one brushing method you should always avoid to help save your teeth - Bicester Advertiser</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 10:06:38 GMT</t>
+          <t>Sun, 01 Mar 2026 14:06:21 GMT</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPT2JycGhsRDBGX19melROOXNVUXNVWE9VTGszVC1JOG5lU2x4UHZBT19hU0w5a3RQenFwendXc2pPem9DMTdRc21RZDZUS1JFWnpMaElhcUlxUV8yVXhTcmNtOGZIcTFHQWhmNlhZc0JJWlBTS3M4WThRY1JqbTlfbVVwRGp2VE9OeUkxVlF6ZGQxLW5RejJIM2FhNjFpSURBQXV2SmJXWUFmbjl5QmlXN1diS1FoWVNpYnNOSTZsaEVSQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQQlhIM2o4LVBqUDFMam82c3lCMHJSUlllTnA0cXVHUzlRb05QNEZkLUlWTjd3b0ZLRlNRTTNSWlgxMzBFV3I5cF9pbDlLR2dnaGJ5SzM5WG0yQkE1TGtXTmx3ZU9vZDdjTUJUcGZsVlVjX2pvdm16YmJ6bF83V3FKQkVMMlpXdm1NOXl0S3VUTTRXM2N3cnZMTzJNZ0Y2MmZ4aXJPaUdHUnJfaTA?oc=5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1945,52 +1945,52 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K28" s="1" t="n">
-        <v>46081.42127314815</v>
+        <v>46082.58774305556</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Streit am Morgen: Nach Messerangriff in Würzburg keine Hinweise auf Psychose - Bayern - Neue Presse Coburg</t>
+          <t>Olivia Dean crowned as UK queen of pop among BRIT Awards 2026 winners - Bicester Advertiser</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Argument in the morning: No evidence of psychosis after knife attack in Würzburg - Bavaria - Neue Presse Coburg</t>
+          <t>Olivia Dean crowned as UK queen of pop among BRIT Awards 2026 winners - Bicester Advertiser</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Sat, 28 Feb 2026 09:15:48 GMT</t>
+          <t>Sun, 01 Mar 2026 07:25:50 GMT</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxPZXhycWdQbTY3cC1kWTVIMXk5ektJb1FwMkZHRkt5NE5JcDkyNWxxZU1qbHB6R25VdWpUWFU1YWdGVnVKQzZ0RjRyM3RQX2xQcm1lZklFQ29KLWE5MUpuenpiLTVpS1RCQldOX2xPcjNyajl4Y2pPNnJ5SjRabm5zNU5YMHhiMlRqUTV5R2dnY3VVbU9rS0JtX1FUeXZVYV9IQWNvWnIzVzMwelRvZTdEZmpvNkcxY0ZvR3V0NEJzcXFnWi1pM2JscmRQRXVhb1dPaTgwLXg5cnJfLVAwcV9lOGNsM2g?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxPUXFMbjZnaFZBWFlqR0xoSU1pTWpQVGY4SnFXa3NlOGhTSHdHYkkxdEpWSDVHZDgtY3V5VXZlU3AtbnBWUHFsWkl6cnJfeVJYOW5hcEJpa01HMXNhVDZZY3N5VTBpdGpDYnVoRld1VGhiN1pIQlAyWWlwLVlkRW82c3MzVTRKOGl4bjZac3VRdDdNWFB6RjRrZkF2V0piVEJ5V1AxUC1OVEoydG5LMDNCR3RsS3RhdHI2TThrN21xNA?oc=5</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2000,296 +2000,21 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K29" s="1" t="n">
-        <v>46081.38597222222</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Local Town Wertheim German</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Weibersbrunn: Ausweichmanöver wegen ausschwenkendem Lkw - aschaffenburg.news</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Weibersbrunn: Evasive maneuvers due to truck swerving - aschaffenburg.news</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Sat, 28 Feb 2026 10:09:22 GMT</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxOSVRRVGwzbGUxTU1zaE05RWRzYWdvMTFONWYzOThvNHg0TjdPbXM0ci0ya1BCNllwdnhTT1lhcXluLWM0eEVNWTVsRXZOYnlBeE1hOWZiMVU2Q28tblg1S3pRNkxPWmc0ZjJWUWdZVFJ3UFI3Mkxaakc1TEJBenNQekRnU1lsaDhNMzB2amx0T0dvM0lPRmRLakc2VVVWNHY1dXBHaWVVQ240Q1p5V2h5Yk5JLTViMkVqV1E?oc=5</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K30" s="1" t="n">
-        <v>46081.42317129629</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Local Town Ingolstadt German</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Ukrainerin verweigert Verlassen der Asylbewerberunterkunft - RegionalReporter</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Ukrainian woman refuses to leave asylum seekers' accommodation - RegionalReporter</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Sun, 01 Mar 2026 07:03:04 GMT</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxOemRhYjhRS2NxZU1PSFZWTmpaOENTb2NqZDdOa1pTS2lrai1CQ2JTLVp3ckVnOWpqRlBEMlpRLS1PLUxhbV9QYmVsS25oLVJjeU9XVEc1VEFZNXJBYlZJbnhxTnlrRU5RNEwtRzZuSzJrV0dDd3c4eDc5MTUtYmNkLVBETkFmS21YX3BlRXZQU1Q1VWF5aVAzWGRxSG9UNE5heEVGN2xTVlR4Mk5OMEFaOU1aUHJ5OFNU?oc=5</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K31" s="1" t="n">
-        <v>46082.2937962963</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Local Town Ingolstadt German</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>KEC hatte zu Beginn Schwierigkeiten.: Die Kölner Haie haben mit 6:3 gegen den ERC Ingolstadt gewonnen. - Rheinische Anzeigenblätter</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>KEC had difficulties at the beginning: The Kölner Haie won 6:3 against ERC Ingolstadt. - Rhenish advertising papers</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Sat, 28 Feb 2026 17:42:06 GMT</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQM0p3cC00Z2k1aXk0R25VWk84bEk3dXR0RkRDLUluUG9LWWoxTmNoMzJVa19QVDRHOHc5QU50Y2JRZTVqOXdKRVJDV1VNRHcwMEZlaE03dzZjZlRsTVV5dmI2ajI1S3FDQTE4ckZIZ1FWaWF5d2tMZnpLOXdVQ09aenYteUk2MUpUSUhXUU9XakhNNW9mU2psN0FWZ0NPaUZDa3E4aE1HTy16aWw2OGxiRnh5dkNnbFY2S3NBVXFDVlpVUjRmSlpF?oc=5</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K32" s="1" t="n">
-        <v>46081.73756944444</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Local Town Ingolstadt German</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Bundesliga: Bayern gewinnen beim BVB - Fans haben Ärger mit der Polizei - RevierSport online</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Bundesliga: Bayern win at BVB - fans have trouble with the police - RevierSport online</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Sat, 28 Feb 2026 19:40:35 GMT</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxOVWdubmNlZXF1TkVaS19NUFQ4U2ZJbTRfbzdDT3ZIR1hiaXc4UnNfTzVfcl83RHhRZkk2ODJnRmFTcGFCUmxvcWlLZU9ZbjRzMkduaWJzcUZlUTlRY0NMS0VTOE5PMzg4bThBb0pEUXdzM1NlclNzODNuSXV6bkpFWlJPX1hZaExzcnZPQkV6cDhPODQzaVl2Z3Q3MkRZSEY4enE3TzIyWGJJek56Q0ZESTNiREEzZzBfSFo4cXpGdlc0QQ?oc=5</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K33" s="1" t="n">
-        <v>46081.81984953704</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Village Ingolstadt (fallback)</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>FC Ingolstadt 04 vs. Mannheim: live game updates, stats, play-by-play - Yahoo Sports UK</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>FC Ingolstadt 04 vs. Mannheim: live game updates, stats, play-by-play - Yahoo Sports UK</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Sat, 28 Feb 2026 19:19:54 GMT</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOREVtNFlJR0lRTEZ4RjFmZXF2aU1WMkxNWldKQURQRWppZjFWUEhyekJuaDV4enNCQ1g3MHRuZzJXS1JrV0JkLU1DSnJXOGx2bXNkT0ZvUUhxQXJnVTRxckNCOGpTUDVPZjB1bzVxQkJqeXBkejFxWlg4aG9lTkNfTTBqdnVpcXNkZzN4RExn?oc=5</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K34" s="1" t="n">
-        <v>46081.80548611111</v>
+        <v>46082.30960648148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-03-03 07:50 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K61"/>
+  <dimension ref="A1:K64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -535,32 +535,32 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>London Marylebone Incident (fallback)</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>("London Marylebone" OR "Marylebone station")</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Kiyori opens in former Marylebone bank vault - The Spirits Business</t>
+          <t>B&amp;M tries to win back Britain’s discount shoppers - Financial Times</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Kiyori opens in former Marylebone bank vault - The Spirits Business</t>
+          <t>B&amp;M tries to win back Britain’s discount shoppers - Financial Times</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 11:37:32 GMT</t>
+          <t>Tue, 03 Mar 2026 05:00:15 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxNckx0R2xuZF80T2FGcXR0U0duRndZWVNMVl9ZNlNTS3hkNE9haUh6WlBMYk52ZGxZb2ZUQjdYeDF2Y0lvZ3RoNWYzWUtRcU8wcEwwNVA2eF8tRDRtVnRfSEZvcFBUZlJPTngxRkNmYnhsc3FTYk5VazVhakUtMklaY2VDQ0dHZTJIZ1VGYW9XLUl2UQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE81MENCdWdEaHB0ZjVMWFRNVjVDU21NTGNGMkRkTEdRMGR6QS16ZDVMX0EtelZ0QnBobEdLOWhDZnFFTlZ0UmN4WndxTDhiR2NrXzM3SXhZWXhQX2dDTGpGWTlsVUdoSVRDLVA4eUdNRmg?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -584,38 +584,38 @@
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46083.48439814815</v>
+        <v>46084.20850694444</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Nick Bril verschijnt opnieuw voor de rechter in Antwerpen - HLN</t>
+          <t>Sainbury's in town centre gets warning from council on 'appalling' bins - Oxford Mail</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Nick Bril appears again in court in Antwerp - HLN</t>
+          <t>Sainbury's in town centre gets warning from council on 'appalling' bins - Oxford Mail</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 10:11:51 GMT</t>
+          <t>Mon, 02 Mar 2026 16:00:00 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxQQmY0bExkenY3SWFsRGxWZzRWdHhZZlFodzFpZUZDNlpKbUlJUy1ydkNmczNSRFVwbXVZdHAtaEFZRGJKVm9kcmFDa1N5dXJHYk9SQWFrdm01SUNkalltcmJPVktHSmR0MXFJOExlSEVWenlSXzk0SUtaVi1BbzZZeXBZXzNtU1RldFlqSG5maDdoNVFPbkFNZmNnUDU1dC11UmFmag?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxOTzljY0tiMFp2cGl2VGJRSGw5YzVsWGpoM0twNWJDMEFmb2p3ZTNVQ3lEVXdQUkZFcElUaHRtYnVIU1FmNmw0bGl1XzV0V1hpMDljbVhoMm45VUtmYmJsTU1nQVE0QXRLM1h4MjZkc214S1lONHZKeWVjZEVwbGlRQk5Zdkx3QVA3NjRPbUdnVVBqT1hScWFiRQ?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -625,52 +625,52 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46083.42489583333</v>
+        <v>46083.66666666666</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Between Cyprus and Brussels: The Collapse of Europe’s Containment Policy in the Face of Iranian Terror - Jerusalem Center for Security and Foreign Affairs</t>
+          <t>'I've given up on hospitality. The £15,000 pay isn't worth the stress' - BBC</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Between Cyprus and Brussels: The Collapse of Europe’s Containment Policy in the Face of Iranian Terror - Jerusalem Center for Security and Foreign Affairs</t>
+          <t>'I've given up on hospitality. The £15,000 pay isn't worth the stress' - BBC</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 08:41:26 GMT</t>
+          <t>Tue, 03 Mar 2026 00:10:14 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPcDRJR2N6eXRFam4yVDk2b0VwczhaOFExbTUzRkQzcTgzZERLcnBQYkZIeTVJMEZKLUo4SXYyWE1fM0FISGVRZDk2ekVocVFyT3RCZTNwb3hwM2M4bTF6b1lza1NLUUU0NlNQdFNaSU42YnNJbndnS1dmdC1PZm9neGY3NGQxWDR4UU03OElmTkZVeFdWcVozN3c5WjlSbEtvWDZSclFmMkdwcUtYTlhSUHUtTTlnRm1UQ1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE5OcGdYb3UtdHZwRFRyTUg4UTBFc2FhTEhHa1dSTVVjN1B4eG13dWx6OThKV0J6aGVxV21ybENrbjJQWU1CQ2tidE1nVkZtNjJUX3BKWFBpRDJNdw?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -685,47 +685,47 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46083.36210648148</v>
+        <v>46084.00710648148</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>London Marylebone Incident</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("London Marylebone" OR "Marylebone station") AND (incident OR disruption OR closure OR police OR bomb OR explosion OR stabbing OR shooting OR "suspicious package")</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Polish President ‘knew about US attack’, while PM Tusk wants de-escalation - Brussels Signal</t>
+          <t>Marylebone services hit by sudden disruption – what we know - London Now</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Polish President ‘knew about US attack’, while PM Tusk wants de-escalation - Brussels Signal</t>
+          <t>Marylebone services hit by sudden disruption – what we know - London Now</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 10:12:52 GMT</t>
+          <t>Mon, 02 Mar 2026 16:21:37 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxPRTJfcThDd0hNUzhUbHBydGlYYUVhZV9CcHE5U2VGeU9aYUdjZEtDd0lSSDRXTThTM2RNVWFQa3J6MUJqaldhdzlxQThRTTFBa1hnWTkyMEpqelF5T0pjSUNGNHZHR1dGM3VNNkU4WjA4ZHE4X1VvNkJkUHVGajYtSlBYc2xRdEtqMnhqdjlSa1MyNTFIamNQN0pjMXJWM29JN3cxdWRfTTlUdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxONWVCNjN1aHpNMEhTLTVwbmtKSnVvbi1mMEdvenI1S0sxdjBsUU9pSy1kQkxSZ1VmT3FaZ0ozWGNQdmdSUmJHV3ZrczJjVlVZcGgzRWhjOFpKdWNmb0hncWltZFMxX1NnT3RiZTNRYW1PUzNRY1JDYy0tX3N6dzFiWEE3OWVPa2xMY3VaT05hY1BVZk0?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -740,47 +740,47 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46083.42560185185</v>
+        <v>46083.68167824074</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Middle East airspace closures trigger widespread flight suspensions - Travel Tomorrow</t>
+          <t>Na arrestatie op Antwerpse Eilandje: wordt voortvluchtige diamantair uitgeleverd aan India? - Nieuwsblad</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Middle East airspace closures trigger widespread flight suspensions - Travel Tomorrow</t>
+          <t>After arrest on Antwerp Eilandje: will fugitive diamond dealer be extradited to India? - Nieuwsblad</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 08:43:37 GMT</t>
+          <t>Tue, 03 Mar 2026 05:03:43 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxQVWpGQlpoRFB2dTU4THMzM2I5Q3d0eFpyaG5XTTB3dUI1V2p5ajhNeXVvRHUtY1pHR2FqQ045V3BJM3ZIZk9Ec2pELVo3MVVjbk5mY0p1eFpvczAzSks2QlRKSFkybW16V1R3RGZuZUJCeTJHa3RxN21DZjcwdzRKWkZPOXpOQktta0FuTHR1OW03RDg2aV9mcWpOZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxOVkxRZGo5aUFfTmhBdE1wdTZKMm5vWXJOMWlQRkJiMHlIN0NIbUNLaUNmRUF1LUt1bnZMaEM4dFNPM2Itd2oxSDEyRXVWai1kNkpfSnJ1cHdSS3FEZmhzODh6dHhUejhiME01M3BaTTMyRXJuSnNMdTV0TEkwWFU2SmFITXJzRC1rVjN5OEkzb1VYdk1zc241RTZjNHlJbnc1bkJRZ3BfQUpjR0trVnFKUXdEVjk5V2ZOb0pHdm1ROFRweTlvbTQ1ZjljeHhQOFh5WnJRaWVveXFzZFQ1cS13MjFheDdCaVllTEg5Y3RYejg2dFhnWno4bEpiZlRWUWswd1E?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -800,42 +800,42 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46083.36362268519</v>
+        <v>46084.21091435185</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Le taux d’alcool du chef Nick Bril était d’au moins 1,52 mg/l au moment de l’accident - 7sur7.be</t>
+          <t>Spoorverkeer tussen Geraardsbergen en Aat onderbroken na vondst verdacht pakket - GVA</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Chef Nick Bril's alcohol level was at least 1.52 mg/l at the time of the accident - 7sur7.be</t>
+          <t>Rail traffic between Geraardsbergen and Aat interrupted after suspicious package was found - GVA</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 13:35:41 GMT</t>
+          <t>Tue, 03 Mar 2026 03:23:31 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOM0pUX3JQRS1yZ0gxbUlrMDBEZHRldFpoWnE3WHIxc01LREhUNmxsbzFqUkxyVEg0cDdJRU5WeVN2aHVNVS1Gd3E3TWJ2OUhXaGxwbUFVV203bXdRNFd5NVdfanFsMTh1V00tZ3VhOVFJd19CTWhKeE5MT3RyYkpCcE9QNGRFQUg3eTZHRVNnQ1A5YW5QZ0ZVYUZrdUlhRl9XMWtTMUpIMGw0anlzY3R3UlJGd2FkV1RXdzJrTUp0bEdHUkRG?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxOTXFSZE5lWUo4R0Z4cWlVLVNJZ1JEVmZ3bGVzUWh6YmlYbHV3TTdPTXpqQUNoLUY1bk5KZmozeThBaWZhcXV6T1lzOXFobk1uTkVTcW1zQ2xRSGNVaEs3ZjNSTGFKejJ0eXRnTTZnTVBGTGVxR0lWZ0phZlR4WnU1UndnS0FQSnlRLXozRmdsV0FFVjQ0WnF1eVpPejZaZGJfWVdvZWx1ejBGMTFGUXMtZTNjT0NHWVZjaWo5ZmF1ZkVmZw?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -855,42 +855,42 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46083.56644675926</v>
+        <v>46084.14133101852</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Une caméra sur la tente d’un sans-abri à Forest : "Je veux juste savoir qui me harcèlent" - BruxellesToday</t>
+          <t>'Nieuwe' Rembrandt ontdekt: Het visioen van Zacharias in de tempel - VRT</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>A camera on the tent of a homeless person in Forest: “I just want to know who is harassing me” - BruxellesToday</t>
+          <t>'New' Rembrandt discovered: The vision of Zacharias in the temple - VRT</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 11:32:00 GMT</t>
+          <t>Mon, 02 Mar 2026 15:41:16 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxOR1F6cklWcndKX0wtQUd1SGROWnNjaEhlU3hrMjZlUFBVaEVsc3BXWFhabGJpYndNVTF5cGlEc0dBalNrekhaRVlvaGNUNlJYUVpWaHB0dmhmbWJlNVFacGk2RFcxMkJzTXJwdVlVZzlyWWV5UEVpcHBrVzV1cDVwa0N5Z2VsQjA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQWjZReUJhd3g4dnRrWUNZSHRoOGVMVDByV0trb3RpOFBLSmJBYVdGWkhDRjVna044WmRRT09iOU9sS1NSN3FlTzFLUlZuYkNBZE8tczFkYkNjdEx3elU3bDYxczlvQVZGMDk4bmE0VUxCQmRfY3QxT21aNWRMRnJxSlg2dHhOS3BlaHF6bmtQWEJpb2kwdExHaWYzbGczZUxxOGFsdHdwaU9MNEk?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -910,42 +910,42 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46083.48055555556</v>
+        <v>46083.65365740741</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Hasselt geeft negatief advies over het besparingsplan van De Lijn: “Niet opnieuw de zwakste regio treffen” - HLN</t>
+          <t>Politie treft 187 zakjes 'erectiesiroop' aan in winkel in Koekelberg - BRUZZ</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Hasselt gives negative advice about De Lijn's savings plan: “Don't hit the weakest region again” - HLN</t>
+          <t>Police find 187 bags of 'erection syrup' in the store in Koekelberg - BRUZZ</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 11:43:12 GMT</t>
+          <t>Mon, 02 Mar 2026 18:11:07 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxNWk5kWGVxeTctdXN0N09mNjhfbkQ0cDNtLWJUTnppeXlFR1R3RC13RHh3TWtjQWRKZVYtdmljNFB2VmpOdllwblY0T2R4ZWFlVnRlbUxBc2pFN2lmeVdVbExTUmJBX1J1QUVkbVRIM1lidGg0b2c1MHV5MnpubmZDZjJhWGpTOG9ONmpYX1hOeFNHQ0lRYUZiUzBtc1dlczI0M2llSlg2QVNoNEcyWjlwWVNqYjFuUnk0cHhTeEpJcjl2VC1ncjlPTDYxUDFQR3d3ekd2WmZzOA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOMkcyQThacndzYkxmQ2Zod3U0T290VkpwSjRudmt6Yy1lSGVuVUJKdFZNQ3BPY0FYcHc4V3lOcjRGSkpLSzZCVFVSWEFpZlFhT2FyWEdGTGc4YzczYVJVSk1LeEt0SG9QV3A0NWFPTHlfNHVNMy1CaUY0cERZZVl0TWhrcGNIWWVxUnNiWUlzYURxNFlEeTlzVmdaSXV4bUh1VnRIUjBmelRjOFU?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -969,38 +969,38 @@
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46083.48833333333</v>
+        <v>46083.75771990741</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Kapittel start met toekomstverkenning van het religieus erfgoed in Hasselt - Otheo</t>
+          <t>Moeder ontdekte dat nieuwe vriend 2,5 jaar lang haar minderjarige dochters misbruikte: “Hij is een bijzonder laffe man” - pzc.nl</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Kapittel starts with a future exploration of the religious heritage in Hasselt - Otheo</t>
+          <t>Mother discovered that new boyfriend abused her underage daughters for 2.5 years: “He is a very cowardly man” - pzc.nl</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 11:19:58 GMT</t>
+          <t>Mon, 02 Mar 2026 18:16:00 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNM2lqUkJHMEtBMExydzVrcXdWelFPd2E4TXlWeGVUU3hKSEFXX3FrY0hvMm1raDZuWHFjOWRjSUtXNDRkaWhGMEgxdkptVjlCS2MzS0tzWnZCMEh2TFRDMTRVb1RDeGlaTU9UbTRTWFpqbnV5RkZHbHVRa2dER2o5Q1BfcHB3WE1HTVljU25xNGVvSWV6QTQyblZoVmVEdlpsZU9saVNB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxOZkplWUQ4Wk9oZEdOWXFZNmZjc2xsaFpZM2htWkJkYVZOUWR2X3REQkJ3OWU5aERBSnVZcmFQTFg1dDh2VzNzZExlOWQ1TDJTZ2gtWU9tSFJtVlEyWTd4Zk1oNWJ3YzA4S0k1a0ktbVFzenZsUGlrQ1BhZlRMZkFhVDNvN0liRXRXZVljVXVnR3ZlSXlzTThwc1pVVmNadnRZbWxiVS03bUtpR2RDTEVUVmlsS204QjdKc3ZMZDlMMEY2dVJJaDJnYTJaVDluRDUyZHVBVU9nNUluam1GeEh5STdPNFZzTnh4RXRz?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1024,38 +1024,38 @@
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46083.47219907407</v>
+        <v>46083.76111111111</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Hasselt zoekt ontwerper voor uitbreiding Stedelijke Basisschool Rapertingen - HBVL</t>
+          <t>Elf jaar procederen en nóg komen Fibonacci en Saxo Bank er niet uit - Het Financieele Dagblad</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Hasselt is looking for a designer for the expansion of Rapertingen Urban Primary School - HBVL</t>
+          <t>Eleven years of litigation and still Fibonacci and Saxo Bank cannot reach an agreement - Het Financieele Dagblad</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 11:46:48 GMT</t>
+          <t>Mon, 02 Mar 2026 16:22:19 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQVFYxbXJsZlhlWGZnWGJYRjRLTUFBdHZNWkF0bnpIQ0Z6aXg2T09VZ0p6WHJXanRKSzdxV1o0bnpBbVZpaHR3bzBKTVJUUC1KVjI1a2FUb2poVDB6NkRLS3FSOW9uQzJMSnJZek1aM3lzWWNSSGZGVzhZcHU1XzI0MFA0N09BY2FNdDU1VFJnSUN2SDZxQUNzUUFsdWs4WW80N1QydWlhdFNrSkVULWxrczNucnVmVjlMczNyeGw4c0k4UzBSNDd3MDBDRHg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxNbmhLZHFDaFF2ck44NzdSMk9SSUlHVFdXeVAySXozazQ2bWtqclRBSUlOQ3VkZGQwMDhyQUdHd3ZhNVpXUjFwZDRLTlZ5RlV1R3Vldk8wQURZT3lOTnpDUk1jQUczcTRHSFNHWXZFMkpFclM3aksxX3dXdS1kdTFXcU45Rm1BS1RMWVlEWUg1SGhRNnVXMFg0TVBfdVJucDNGWlhn?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1079,38 +1079,38 @@
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46083.49083333334</v>
+        <v>46083.68216435185</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Kermisvereniging reikt oorkonde uit aan stad Hasselt voor waarborgen van kermiscultuur - Nieuwsblad</t>
+          <t>Parket onderzoekt verdacht overlijden van vrouw (81) in Brasschaat - HLN</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Fair association presents a certificate to the city of Hasselt for guaranteeing fair culture - Nieuwsblad</t>
+          <t>Public prosecutor's office investigates suspicious death of woman (81) in Brasschaat - HLN</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 13:08:00 GMT</t>
+          <t>Mon, 02 Mar 2026 18:48:42 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxPdG9NdGxFcm85d3BUbURaUlFQYjVvOTAtbXVaXzNsbXlOdm5xeXZVenI3c0k5QTg1ZkdFNDk1eDZxVzBkdktJSHRDbmhSQktYajVEdHhCbkUtMlRXWnVnd3pGNnFzbkd0a1lkb0ZtQUNNTlhveXJYSFlJZ3dJR3JMaDQ0cFEyOXZZRlRLbFY2QnRYX1B4dTNBYTlDX002T21XRFdWejlra2NweFVvVFhoV3h1OWJSLWJqa016VHNKc2FRQmtZX0x5UHh6MHo2RDNaS3pvd2JMRExaQ3VLX0IxWVlWMA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxQUUxSNkxkX3B4MDJaa3h4UjkwYUdvVkpyRHBuVWs1UFZTRXRIc2hKUkhRWFFuVzVCOTNSMUs3ZVNoY1ZmbHRmNWdyR2xjcndUZW9aM2tpR1NGaWw3a3RsWmI0elJwbFppNDVrazc0TEpXZUdlMmJQZEFLS3pxcnZFVkVkX2JNTWhtXy1Naklhc1lRUU1BTTN6WlQycFNqanpMelFqMS1UMA?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1134,38 +1134,38 @@
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46083.54722222222</v>
+        <v>46083.78381944444</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Politie houdt verkeerscontroles in Hasselt: twee e-stepbestuurders onder invloed, motorrijder betrapt aan meer dan 200 km per uur - HLN</t>
+          <t>Nick Bril verschijnt opnieuw voor de rechter in Antwerpen - HLN</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Police conduct traffic checks in Hasselt: two e-scooter drivers under the influence, motorcyclist caught driving more than 200 km per hour - HLN</t>
+          <t>Nick Bril appears again in court in Antwerp - HLN</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 14:38:12 GMT</t>
+          <t>Mon, 02 Mar 2026 10:11:51 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxOaVhNWXB1dEpSREsyb28wOFU2T2FwUkhEN1BnSC1tdDh5T1l5Y1NuZEVEa1NQU0RkSEtBNWJwYlc4akFUaDZ1WHBIVmhCS2VxUU1fZEQ4T1pweEVXZGxWc3R5dmIydDhUSGZuSkVBWTJuem1ZRjhTTElNQzBaNHJsaFJPM01lSkFhUWJrYThwcUl0S2dSS18zamcyZ09FbnpHZTFxTmZYR2Z3TUFLNWc3b0ZMMDNtS3R0eDdwb2JtZDBQUVl5NHhBdDcydU5oZjNQWGtvbHo0Ym5CLXpSMEVTbldVbVVRVGx4cDJBM21JeEZ4UzRUYjNr?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxQQmY0bExkenY3SWFsRGxWZzRWdHhZZlFodzFpZUZDNlpKbUlJUy1ydkNmczNSRFVwbXVZdHAtaEFZRGJKVm9kcmFDa1N5dXJHYk9SQWFrdm01SUNkalltcmJPVktHSmR0MXFJOExlSEVWenlSXzk0SUtaVi1BbzZZeXBZXzNtU1RldFlqSG5maDdoNVFPbkFNZmNnUDU1dC11UmFmag?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1189,38 +1189,38 @@
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46083.60986111111</v>
+        <v>46083.42489583333</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Pas getrouwd: Christophe Kidjemet en Audrey Lambrix in Hasselt - Nieuwsblad</t>
+          <t>Between Cyprus and Brussels: The Collapse of Europe’s Containment Policy in the Face of Iranian Terror - Jerusalem Center for Security and Foreign Affairs</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Newly married: Christophe Kidjemet and Audrey Lambrix in Hasselt - Nieuwsblad</t>
+          <t>Between Cyprus and Brussels: The Collapse of Europe’s Containment Policy in the Face of Iranian Terror - Jerusalem Center for Security and Foreign Affairs</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 09:05:01 GMT</t>
+          <t>Mon, 02 Mar 2026 08:44:23 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxNZWYwNy1QYlFjclVLOW5xOGVJRlF6TGZ3QmgwMFNvZlFkdmtIaXVfRUlwdkFXR0dyWU9hM2tQYzJiQ2d5Y3h3RUliLTRPSW1HRmRNaVJLZlFDdEVUTlk1M1BocUtNckFXTWFwbktOeDZsQkdvMlFEUmFoWVByOHZ1eUpKeHZWc0VQM1pXYURCVVRTVU1WX01Uc1RTVDJPc081YVJfX3FacmJxNTg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPcDRJR2N6eXRFam4yVDk2b0VwczhaOFExbTUzRkQzcTgzZERLcnBQYkZIeTVJMEZKLUo4SXYyWE1fM0FISGVRZDk2ekVocVFyT3RCZTNwb3hwM2M4bTF6b1lza1NLUUU0NlNQdFNaSU42YnNJbndnS1dmdC1PZm9neGY3NGQxWDR4UU03OElmTkZVeFdWcVozN3c5WjlSbEtvWDZSclFmMkdwcUtYTlhSUHUtTTlnRm1UQ1E?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1240,42 +1240,42 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46083.3784837963</v>
+        <v>46083.36415509259</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>“Alles onder de 800 euro is meteen weg”: huren in Hasselt blijft strijd tegen schaarste - HLN</t>
+          <t>Unprepared EU tries to stay out of Middle East war — but can that last? - politico.eu</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>“Everything under 800 euros is immediately gone”: renting in Hasselt remains a battle against scarcity - HLN</t>
+          <t>Unprepared EU tries to stay out of Middle East war — but can that last? - politico.eu</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 10:38:12 GMT</t>
+          <t>Tue, 03 Mar 2026 03:01:00 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxOOHBLUDJMeWtqR242cVpNS01iRXc5S3g0clMtM0pSa0hqQ0xlZTZ5TEozdDBrUnZybzdFOHJIS25pZ3Y0cFJOMFNnZGw4S2MtRVg0SXVKNWpYN0FTZDR6VldOTnRwOFd4Zm90eHRqM3Q1VEtiSUF5Q1Q2N2VtSmNDMXphczM2ZEF2WklwRVJUSzhjNFFOSW83czR1R3BRanlvdTF1cC00Z1JyTlpPZFdFbGJ0bm9mRG1abmltTE1R?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxPQ25BWVFkcVpwUlk4eHU0MU1FaXZCV0N4NGwxNlp1Z09jT0lOcGNRS1FWQkZ5T2gxa2dPTGlodUZQSEkxdlBfQVFQQWpYWHhNQUlFOGJtb0JQR1B0UmZLT3pvOW5ydnRUS0tYUkc3ZVRsbXF3X0RlUVZhLTc2SHZVTk9WMHpfRTQ?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1295,42 +1295,42 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46083.44319444444</v>
+        <v>46084.12569444445</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Pas getrouwd: Kaat en Sander in Hasselt - HBVL</t>
+          <t>War touches Europe as Iran strikes military bases, threatens oil supply - Courthouse News</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Newly married: Kaat and Sander in Hasselt - HBVL</t>
+          <t>War touches Europe as Iran strikes military bases, threatens oil supply - Courthouse News</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 10:02:36 GMT</t>
+          <t>Mon, 02 Mar 2026 15:58:42 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxPSTJnM1YzT0pZNEF0VWNOUFpSRmpUd0NUVS1OTm9SOVI4X2o4elhyMGg4cGU0b3Y5a19vWjlWY1RaRXNZUTNld2RfQTAtdFlET05qLUJPWFJBWE5oa3Q5R2hHbE1pUWVwbEI2UnJmY0Y0b0ZmZGlHTlUxLXJLMmhyOU5LWE0xVk5jekNkSmV1dTNHY2dNaFJyZVNoaw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPZi01ZF9VcEtHVll0ZUlUdXpzZjNYMVIyRE1GaUNNOWVBM2xLUEl3bzBRM192cmZvZGdXZC00dktJWWpaRUlCT3NKWE1FQkhwNnhIMnV4dmRJT3pwT3htX1hGanNUdnpBLUlyMEFrYU1CUkpNWm9IQTNVUF9rTGVweUc4ODhiQTlndEYzMktrZG5zbVVvdWdZRVV3Yk9PblpBUTFXag?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1350,42 +1350,42 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46083.41847222222</v>
+        <v>46083.66576388889</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Gemeente gaat Centraal Kerkbestuur bij de les houden - HLN</t>
+          <t>Iran war: Will Europe's split on US strikes backfire? - DW.com</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Municipality will keep the Central Church Board on its toes - HLN</t>
+          <t>Iran war: Will Europe's split on US strikes backfire? - DW.com</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 14:07:59 GMT</t>
+          <t>Mon, 02 Mar 2026 18:59:01 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxPYTcyV29lbzU5NzFQeWt5bE83aHUzNXFRazVOelVybU1MdkcwUG85dXlTQjRTRzZjdHNSX1lkcXNHQWx2bGNvMklERkxjUDluNlBPaU5yR1J6QVhwSnZEaWFQakhNbWNvbUxTOUdBQVliTUNidVV2bG1zdGRKbmZoU0dfXzlqZUJ4WjYzZHZqWlN0dFk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNNVRHakYtY0RxbWRUQkhLYlIzNS1fZ1JaR2N1aXc4QkZ0YUllaEpic0dNVEZVSmlVR0NUZGZBUGVhT080VlJTVFZWWkhVcEVYTjdBblpqSVh0cDYwYTl0RUdPeUpJYjY5ZWUyV1VqM0gtQlM5dzJ2ZmdMRjNmb1hYbzdiczc2N2d1dHJGdDdlUnI0dTFnZlHSAZYBQVVfeXFMT2F3Tnc0bURaUzFxMXZVN3pJUVZYRlpyMlZuVWd5NmV4d1JsUHp3Q25VRDZhU0RYR0h3b3I2Q3NrSHZ3c2pYZGNJMXUwQ3VCUkIzRENPWTJKOEZUQ0o2WGlEai1HbGFXMlFtZDlpeTVjc0p0bW9sa2FLdmNkNzhXX2Y2UGJUOWJvWnI4emg3QVVMeThlRkpB?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1395,7 +1395,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1405,42 +1405,42 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46083.58887731482</v>
+        <v>46083.79098379629</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Pas getrouwd: Kaat Kelgtermans en Sander Moesen in Hasselt - Nieuwsblad</t>
+          <t>NATO's Rutte praises US, Israeli military action against Iran but says alliance won't be involved - AL-Monitor</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Newly married: Kaat Kelgtermans and Sander Moesen in Hasselt - Nieuwsblad</t>
+          <t>NATO's Rutte praises US, Israeli military action against Iran but says alliance won't be involved - AL-Monitor</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 09:05:01 GMT</t>
+          <t>Mon, 02 Mar 2026 17:22:37 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxQUEk0enZHYVRWYmctOHRMTzQtc0YwS0xPOTBQSGJ0ZUhEYmtzZE5fMDk3LWJ3TWk4VjhVVDlkSEFoTklJNTlXZUdCdjVZYzhWclVMTElVc2U2dEs5SWlSODVjNWZrTklhclZGQ2NYcVR0N21xdXBILVNjYkxRNFVCbW43c0ZiTjdEd01MUEpqQzJpcUVEU01oQW1ocHp2WHMtNldr?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxQazJuM3R0U1dWNWhQcEc4Z191MkxVY1gxdWdwOEROZlBCUVZyTmUyaFg2cFhzbGpPWHJZU19wdFJGTURWXzJPano3UGU4MWZZMmVWeU04aFBNTVJMb0c0SDNSbXBzdnVETzZMNFJqMDhUTE1lUml4ZzRmRlo4cWFHR0VRTUZqUWt1LWdoWEJMdUY3ZG1fZnJudVpDaGk5aWFRbjZIcEhtdEZRYWtiVWZrbUhsX3VNVnJxREJodXQwdGpSTmg1?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1450,7 +1450,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,42 +1460,42 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46083.3784837963</v>
+        <v>46083.72403935185</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Acht rijbewijzen ingetrokken voor gsm’en aan het stuur - HBVL</t>
+          <t>Thousands protest Trump in Belgium ahead of NATO summit - AOL.com</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Eight driver's licenses revoked for mobile phones at the wheel - HBVL</t>
+          <t>Thousands protest Trump in Belgium ahead of NATO summit - AOL.com</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 14:40:03 GMT</t>
+          <t>Mon, 02 Mar 2026 16:29:44 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPNlp4M2NnR0tUdE1PUG9RcWdlT19IWmhCUGU2ZXd2MHNnVU16U2VMeU1FdXpCS01aazM0LTdSQ2tnQldzR1kxc3Z4bDhWdTNOZkNtSXpNZE1MUHNtTUxLT2owb1RnUTRWYU8wNkloVzl0UE0zeG9mS0drTjZwSWNuZnJPNXhtT1VjSFFrbmZOcFhGR1hENlM3SnQ2R3RBX01XMnRpS2dGMDVBaUxFR0tv?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiZEFVX3lxTE14dHJMa1ZhTXE1bTJDd3NjN1p5R2NjVGMtaHlyYUg5R0R2Z0tQWDJDTTgyVGsxeTBvUGtYNU1jTndlZDJPS3J3c1hMcnhTVWFlSXNHSlhqc241UEF4QmRYUVZ6ZE0?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1515,42 +1515,42 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46083.61114583333</v>
+        <v>46083.68731481482</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Bijna 1.500 studiekiezers op infodag Hogeschool PXL: “Een studiekeuze maken is steeds meer een gezinsbeslissing” - HLN</t>
+          <t>The ‘Great Pyjama’ debate takes off at Tampa Airport - Travel Tomorrow</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Nearly 1,500 prospective students at PXL University of Applied Sciences information day: “Making a study choice is increasingly a family decision” - HLN</t>
+          <t>The ‘Great Pyjama’ debate takes off at Tampa Airport - Travel Tomorrow</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 11:23:12 GMT</t>
+          <t>Mon, 02 Mar 2026 15:19:42 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi3wFBVV95cUxPOWcyai1Cd0ZBVnpQS2ZHN052OWtqUEMwaThFUmxKZnBrTVJXMnl6MGZ1MFBQRmhUNDFCNC10d2c2RnZKQ0c0c0twZENLTGVjY3NwaEo5VmI1MDZxNkV0VmdkVDVnaWxXUGJyVzFEMXFDOUZzcm82anpnU1NVSV9hdlVuNExFeE5JeVdDQWdxSEhBRzcwNlJCSW9RNG9GMEhpQ3A0Q0drVldzajR0RlJXLWd5eFkyMXVSQzRGemV1UjRsUzh6T1VhWUVKSWc3dEtsVWJKSXBSZ0NoR1FwcjJB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxPbURwRjRNeXBnY1d5V3BaSk1TUW9wd1AyR05lSnd0WHZ5d3lKNTJOTy1Lc0FTckhMZmtzRW5OcGF5UW83blp2bHk5NEtKVzRudXFxUER4V2ktNFI4ZXdrY0VfTXdLWUhXdTBUdWRvZUVtbjFoWk8wQ0dWLVE4S0ZrdkRzLUU?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1560,7 +1560,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1570,42 +1570,42 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46083.47444444444</v>
+        <v>46083.63868055555</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Limburger (56) riskeert vijf jaar cel voor fraude van 6,8 miljoen euro - HLN</t>
+          <t>European Markets Fall As Middle East Tensions Escalate - bernama</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Limburger (56) risks five years in prison for fraud of 6.8 million euros - HLN</t>
+          <t>European Markets Fall As Middle East Tensions Escalate - bernama</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 13:57:30 GMT</t>
+          <t>Tue, 03 Mar 2026 05:15:00 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxObndXS2NyUHJSMGFwcnhoQU5MN19Icy0wQVMtSmU2NnhpZzczd2U2RDc2V25QMEEzdTJKSlBGZDhfRWJuczJJS011Rk9OLVQ5eGFGRlJCUzRCbmRLZ1FfZHU4dGxxTWkxb0kyZ2lxMzRtRngxV0FnTVRUaDMyRjZVTTJPeDNGbTJlV1BYLVVOdUdYYVhBSXMwSFV5a09jVU1jWF9Ybk5KUW4?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTFBmRldFWmR4SnlkWnpvbndwRkNzZ3FBUXYxaWZRUW1fVG05WFQxVUVCTERmOFlLclBZMTI1UEtLZmRDdzY4cTlsdENjUDA4ZHBvWnJFeE95eHdYYTZ3ZDQ1T2xn?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1615,7 +1615,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1625,42 +1625,42 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46083.58159722222</v>
+        <v>46084.21875</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Vervoerregioraad Limburg geeft negatief advies over besparingsplan De Lijn: “Gemiste kans om te kiezen voor het minst slechte scenario” - HLN</t>
+          <t>Polish President ‘knew about US attack’, while PM Tusk wants de-escalation - Brussels Signal</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Limburg Regional Transport Council gives negative advice about De Lijn's savings plan: “Missed opportunity to choose the least bad scenario” - HLN</t>
+          <t>Polish President ‘knew about US attack’, while PM Tusk wants de-escalation - Brussels Signal</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 11:43:12 GMT</t>
+          <t>Mon, 02 Mar 2026 10:12:52 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxQUlpKMF9Rc3hNWHlpOGlaYmE3bGFsNy1HbUVEUzVmV2VGaEpQTnpKSEtwOEZiZVhpMzVnd2xaRkRpZWlxVzNsblgxc3JwOXpZdWI3MXhDOWlVb05XQzA2WDFiVWNMT3NRak8xOV9TNWE1ckVWTHdXSTBjYm91R2RuWk5iXzRDc2pxVW9WaGJQX1l6WmhoQk5zZU9YM2ZJdHRubV9PTjU2RDdFM2R5RVItSDM1NGlhWTRjSlBBNVpwVVdTRXlYVDFteVhfVWJsazBqNXl1YkVzNTJfSjZRTnFxYU9qcEZhZGdhRHRocFZwbENzZVN4MDFIQjBLVXU4dw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxPRTJfcThDd0hNUzhUbHBydGlYYUVhZV9CcHE5U2VGeU9aYUdjZEtDd0lSSDRXTThTM2RNVWFQa3J6MUJqaldhdzlxQThRTTFBa1hnWTkyMEpqelF5T0pjSUNGNHZHR1dGM3VNNkU4WjA4ZHE4X1VvNkJkUHVGajYtSlBYc2xRdEtqMnhqdjlSa1MyNTFIamNQN0pjMXJWM29JN3cxdWRfTTlUdw?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1680,42 +1680,42 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46083.48833333333</v>
+        <v>46083.42560185185</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Brons en zilver voor ADE dansschool in Brussel - HLN</t>
+          <t>Middle East airspace closures trigger widespread flight suspensions - Travel Tomorrow</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Bronze and silver for ADE dance school in Brussels - HLN</t>
+          <t>Middle East airspace closures trigger widespread flight suspensions - Travel Tomorrow</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 10:37:57 GMT</t>
+          <t>Mon, 02 Mar 2026 13:24:26 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxOWV9pZWw4N25SRWs4UVlnMTEtVjhvQktSWmpJekRiVTN0OE1KTkdOenBGUzlWYlpYZUZaVHVKRm05TnNXQmpzYzVDT215cW1TYk9iblZsZnFQRDMtVEJ0V2VBN201VEJKNk9QMFdqeTVnSENKTE5Qd0RuaHk5OXZ1d0M0UG1jY2FWSXc4?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxQVWpGQlpoRFB2dTU4THMzM2I5Q3d0eFpyaG5XTTB3dUI1V2p5ajhNeXVvRHUtY1pHR2FqQ045V3BJM3ZIZk9Ec2pELVo3MVVjbk5mY0p1eFpvczAzSks2QlRKSFkybW16V1R3RGZuZUJCeTJHa3RxN21DZjcwdzRKWkZPOXpOQktta0FuTHR1OW03RDg2aV9mcWpOZw?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1735,42 +1735,42 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46083.44302083334</v>
+        <v>46083.55863425926</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Volgend schooljaar is er keuze uit zes trajecten in de derde bachelor Journalistiek aan PXL Hogeschool: “Het vak is veel breder dan mensen denken” - HLN</t>
+          <t>Dix ans après les attentats de Bruxelles : un peu plus de 88 millions d'euros versés par les assurances aux victimes - VRT</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Next school year there will be a choice of six tracks in the third bachelor's degree in Journalism at PXL University of Applied Sciences: “The profession is much broader than people think” - HLN</t>
+          <t>Ten years after the Brussels attacks: just over 88 million euros paid by insurance to victims - VRT</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 12:41:49 GMT</t>
+          <t>Mon, 02 Mar 2026 16:18:57 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijAJBVV95cUxOS2ZDLV95ZC0teHJ5eUU0czdUXzNzM2pzbXk0SzRqcmhKQlhTRUZsRnZJbE9NNW5uVFFKOG13SkJmZjVINGFQd1F1dGo0NDI2X0d0dFF2VThSLVFPUmEtZTlUeGVZRXZfQzF2Vm9PUW9ZVUo4cEVSNE9IVmNuRHY5LXRTbFZvNXFSaG5nVFFuT2RSa3lERmNMSDM1MFhIMDBXMzU0eGhqRFdaVnlFc1Z4eUxjOEJwQ0hNRjJLQzlkXzVGQzFad0RhNGlMMkpLaExpcG9TMTRvY2NwR2VCSmxNdUMtQVZUa0lodVJBN0RXQk1hN0JoRlhEUkpudWJIVDFlUnRuelNMbEdLc0I4?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxPcTVJN1ppV080NHV4MUlMb0tBeVlWQWk3ckEybXN5LVNidklBMGZUdFhwa3B6T1RrdXNJbmtFSG4tVnB4Ymx5ZmlMQmVDTFZuRXJmMFEySkctV0V6eXJiZXdneDlIS21sV2s4T0d2alNWYWgxZlpxenpOZWtpSGhzVjNtRS1MOFRBcF9PLWptLW1COEZSM0ZGc1ZUajF1d2xzTFVIbXFB?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1780,7 +1780,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1790,42 +1790,42 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46083.52903935185</v>
+        <v>46083.67982638889</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Dit zijn de voetbaluitslagen uit Hasselt van het weekend van 28 februari en 1 maart | Foto - HLN</t>
+          <t>Une caméra sur la tente d’un sans-abri à Forest : "Je veux juste savoir qui me harcèle" - BruxellesToday</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>These are the football results from Hasselt for the weekend of February 28 and March 1 | Photo - HLN</t>
+          <t>A camera on the tent of a homeless person in Forest: “I just want to know who is harassing me” - BruxellesToday</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 11:57:27 GMT</t>
+          <t>Mon, 02 Mar 2026 11:32:00 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxNeEN3azNjYXBfTnRoU2tfWEFGZ3dUeWdWc3BNSk5Gd0JrLXZCdllPOVFZY0djUE83SHgwRVBra1lZYWpYUmVVUS1kT04ydjhGeHVrNEZ6cE1ncXlzSUp1NUt6aVdTZEI4aG1nNGV1cjR4aU0wbkpxbldpMjdqVEMxUHBJdmhqaktidVlvNV8tQlBNaC13UXV6dWNCdm1NSWxnaGZtZ1hNZFpXb1BiMGZYSDNXaG5MR1RrVXF0dFBnMWw3d0pEcFBKWUFB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxOR1F6cklWcndKX0wtQUd1SGROWnNjaEhlU3hrMjZlUFBVaEVsc3BXWFhabGJpYndNVTF5cGlEc0dBalNrekhaRVlvaGNUNlJYUVpWaHB0dmhmbWJlNVFacGk2RFcxMkJzTXJwdVlVZzlyWWV5UEVpcHBrVzV1cDVwa0N5Z2VsQjA?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1845,42 +1845,42 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46083.49822916667</v>
+        <v>46083.48055555556</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Hemelspark krijgt onderhoudsbeurt: “We zorgen dat het hier fijn blijft om te wandelen” - HLN</t>
+          <t>“Un scandale”: le centre Jean Gol exclu de la Foire du Livre - 7sur7.be</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Hemelspark receives maintenance: “We ensure that it remains pleasant to walk here” - HLN</t>
+          <t>“A scandal”: the Jean Gol center excluded from the Book Fair - 7sur7.be</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 12:33:12 GMT</t>
+          <t>Mon, 02 Mar 2026 14:52:00 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQaDRrejNwV1FwcWJuQ0RuMjVPNWFHeVVjVkp3S2paYWJVZGYzQzJBVl8tWkJWRjdMU0twSk13MXUyNkI0SVRZeFhvOWgtdVV5OGZNWlp5bFBTX2VESmlhbkVSc0FQYUxlZUFnbHhqellMdzRmdlhjSl9TOFNFbjh6c1Z0b0pVU0hfLVV5b2RJV2xhSVhrZGF2cDZNaVM4LTV5LVpmVU9WWktvemNvN0dJZ1NQTWRZY2E1a0stbndB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxPdlkweVpwUWdzV2x5djJQLUxpcnR4RTd2cWdKRF9JMV83MGVkTTJ3Y2RlMFpCV2VZN1VUWDNSVVJ6X2RQc0ttaTlzaC1aWWZLUWtUVWZXTjNaaEpEdDlPZXpaNXJNdjJ6ajRFTzZHWVB5cUdsYURrbUJmUXJkaFQ0Z1Z5RlZwZFNXVXdQT2dfMEJXdi1oZHc2X0VZM3NpQQ?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1900,42 +1900,42 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46083.52305555555</v>
+        <v>46083.61944444444</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Man (32) veroordeeld wegens afpersing van student (21): “Hij werd agressiever en agressiever” - HLN</t>
+          <t>Slimme verkeerslichten maken kruispunten veiliger - Nieuws365</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Man (32) convicted of extortion from student (21): “He became more aggressive and aggressive” - HLN</t>
+          <t>Smart traffic lights make intersections safer - News365</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 12:13:12 GMT</t>
+          <t>Mon, 02 Mar 2026 15:01:25 GMT</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxOU3FaOTVfa0ZGZWZVUVo2YXZuc3k1N2JfMFNBY3pIa3BkWmY0YmYySXRzLUZCNkxPekdDUWxvMG1yVmxyOTRVZmF2YzBHZllnVlc5NUNCTU1udnRfV20tcXJtbUM0QVloeFg0bWx6OGtQemFoTHVBZFdDLWpkcGFSVGs3RUIyZmgxQ3JnRGZjVmQwTVhhcWx5QVFiUmw0ck02VVEwQ0ZaRUN0NTY5QzAzUHA5WF9GN0x0RHBGV3A3Nlk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxOMDJocjd6c2xfZkVTSnNGdnFva1dxOEg0QURLaGxGNGNVaGpoNnZQYktMeWJ5UUlZUW5fNHoxa0FYS0JFY1k1UVlLcFVORlJzZ000N3o0dmF1a0ZTRkg4ZjNIQkM5X0RRaVo4UnVUeFVNNFhWSmRYMUdxVjA0bHZzRmc3cXhDMGt4anc?oc=5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1959,13 +1959,13 @@
         </is>
       </c>
       <c r="K28" s="1" t="n">
-        <v>46083.50916666666</v>
+        <v>46083.62598379629</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1975,22 +1975,22 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>UHasselt start bouw van nieuw onderzoeksgebouw BIOMED-VISION op Health Campus Limburg - HLN</t>
+          <t>Dernier ex-aequo, le Club NXT giflé par les U23 d'Anderlecht : "C'est la première fois qu'on mérite de perdre" - Walfoot.be</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>UHasselt starts construction of new research building BIOMED-VISION on Health Campus Limburg - HLN</t>
+          <t>Last tie, Club NXT slapped by the Anderlecht U23s: "It's the first time we deserve to lose" - Walfoot.be</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 11:13:12 GMT</t>
+          <t>Mon, 02 Mar 2026 14:00:00 GMT</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxNR2tHeWozSnFic1dMaTdfbjFRdnp4SjYzbERjeWJjRnN5VXJKaUFldVdUUFZjemx5TXZLVDRBNWFyNW5fV0JnTmE2Sm9FS3BET2hUWl9JM0dFQWRKcVhDaDhVYV9iZEZuaUVqWnRWd1doU3l2Mnd2NC1fUWpJeXV6SlR5anNWOVNxY184ZHlPNlI0bldsbmlycWdZWW9kUzRfVEZIN09ZTVhXODNBVWwtWXFtd2lodU1MaXV4a2NQcmg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3wFBVV95cUxOQWVSc25aRDEwLVpxV2VaNFdoS3pmVEVsVGxsdFVuM3dGMEVNby0xcmxPeHZqazFwbThpdlZuX1lnd0s3cHk1TUZHQ1R1SzlpTlRIQUJaZzM3Nkcwdl9pUTkwRG9lcjZUY2J6TV9yajZYQjdwMjdhazN1dGpHam43aTZiMVVZamlfa3JKNDZONmRVNmMydzVZMU1LZWpaR1JQTmZNSkcwdk1Nb09MS3lDMHd6V0dkblpuY19ubWp2anRZbVNXTU1yTXlGOE9QNWg1LTAtb1NaVHkwWGtHd1A40gHfAUFVX3lxTE5BZVJzblpEMTAtWnFXZVo0V2hLemZURWxUbGx0VW4zd0YwRU1vLTFybE94dmprMXBtOGl2Vm5fWWd3SzdweTVNRkdDVHVLOWlOVEhBQlpnMzc2RzB2X2lROTBEb2VyNlRjYnpNX3JqNlhCN3AyN2FrM3V0akdqbjdpNmIxVVlqaV9rcko0Nk42ZFU2YzJ3NVkxTUtlalpHUlBOZk1KRzB2TU1vT0xLeUMwd3pXR2RuWm5jX25tanZqdFltU1dNTXJNeUY4T1A1aDUtMC1vU1pUeTBYa0d3UDg?oc=5</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2000,7 +2000,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2010,17 +2010,17 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K29" s="1" t="n">
-        <v>46083.4675</v>
+        <v>46083.58333333334</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2030,22 +2030,22 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>42e editie Hasselt Fine Art Fair - De Nieuwe Ster Maastricht</t>
+          <t>Sécurité des musées : Laurence des Cars auditionnée ce mardi par la commission d'enquête parlementaire - CNews</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>42nd edition Hasselt Fine Art Fair - De Nieuwe Ster Maastricht</t>
+          <t>Museum security: Laurence des Cars heard this Tuesday by the parliamentary commission of inquiry - CNews</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 08:05:47 GMT</t>
+          <t>Tue, 03 Mar 2026 05:50:00 GMT</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTFBMbFRQNjBRU0xzczl5MnFuOVV2aVVNNUNjVDNMaHZVNkp2S1c5VDMxdkt4WjdveDV3OXBnZ2JDTncxN3daN0RUY25lR0liYVE4Yjd1aGRsTFpJU1lEYXZwVXhfOTEtUVdqZUhVTWk0dngwMWdZX3RiUV9zaw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxNbU9EQVp4Rk5YT0k3UDRpdmtVWHgzd1llaHViYng5aGRhVTB4TUtCUEdfd1VZRG9ua21KeGlQcjRlSDZZOTRWLUVSUEgyeDQxSjAtN1p6THMzUm9ZOHU2bkR4bG83TTV3cjlBd2hOc3BRaFhHa1JDLTEtZ24tMFdqOXVUb0s2TmdtRTdhMmc1LWctTWxjZlQtOWJBMnFZT09oZWFTXzZRRjZyWlEtU2U0aHBrU0plVUxYREFV0gG7AUFVX3lxTE1tT0RBWnhGTlhPSTdQNGl2a1VYeDN3WWVodWJieDloZGFVMHhNS0JQR193VVlEb25rbUp4aVByNGVINlk5NFYtRVJQSDJ4NDFKMC03WnpMczNSb1k4dTZuRHhsbzdNNXdyOUF3aE5zcFFoWEdrUkMtMS1nbi0wV2o5dVRvSzZOZ21FN2EyZzUtZy1NbGNmVC05YkEycVlPT2hlYVNfNlFGNnJaUS1TZTRocGtTSmVVTFhEQVU?oc=5</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2055,7 +2055,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2065,17 +2065,17 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K30" s="1" t="n">
-        <v>46083.33734953704</v>
+        <v>46084.24305555555</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2085,22 +2085,22 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Fina rijdt op haar 90ste nog elke week naar de yogales - HBVL</t>
+          <t>Samy Debah : le conseiller municipal de Garges-lès-Gonnesse jugé pour participation à la reconstitution d'un mouvement dissous, dès ce mardi - CNews</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>At the age of 90, Fina still drives to yoga class every week - HBVL</t>
+          <t>Samy Debah: the municipal councilor of Garges-lès-Gonnesse tried for participation in the reconstitution of a dissolved movement, from this Tuesday - CNews</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 09:00:00 GMT</t>
+          <t>Tue, 03 Mar 2026 06:10:00 GMT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxNMjN1cnVuaWJ5TVZGVUllbm85cmhyMW9uaTZ2VmJiWHdTT3htSXRZdGRfV2lCSVhBdWR0Tm54ek9ZTjlXVFdTV2tkcXAtXzllc25ISEY5WWFWaFlZZ0hPRmFLQzdRdFFKTjdlWXN1a1hiMzRQRjNyaDNvYjdTVUJyeVN4QVhsQXRYc0pBc2RnT1NVd2dwaEsyWkFhSEZmc3RGNnRhMGl5Ti1tTmEyY0xqZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPUGtWN1RWMDVxcjlfZ0pabXgyZ3JXRkFfcWc1RktyQmN0UWc3aWVYN1V2RXZlQWY5bWdFQWtnUlFQcndJa3FXdEJmeFpsMjdOaEJKM1lDZjRETzRyVHdrcWxUeVJoVXJUaEgtRmdWTEpwcW9qbGtTY0cyMkVBampsODJRamNQbTZ5bUQ3RlRJaERjeUtxR2M3SkdBcjRNd3lPTzdRMmh3XzVuWnROQm5jeXdtT2FLYTBNTWh5TXA4clBIUdIBwgFBVV95cUxPUGtWN1RWMDVxcjlfZ0pabXgyZ3JXRkFfcWc1RktyQmN0UWc3aWVYN1V2RXZlQWY5bWdFQWtnUlFQcndJa3FXdEJmeFpsMjdOaEJKM1lDZjRETzRyVHdrcWxUeVJoVXJUaEgtRmdWTEpwcW9qbGtTY0cyMkVBampsODJRamNQbTZ5bUQ3RlRJaERjeUtxR2M3SkdBcjRNd3lPTzdRMmh3XzVuWnROQm5jeXdtT2FLYTBNTWh5TXA4clBIUQ?oc=5</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2110,7 +2110,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2120,17 +2120,17 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K31" s="1" t="n">
-        <v>46083.375</v>
+        <v>46084.25694444445</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2140,22 +2140,22 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>LEVENSVERHAAL. Luitenant-kolonel Patrick (57) leefde voor carnaval en zijn familie: “Dat we niet weten wat er op die snelweg gebeurde, knaagt” - HLN</t>
+          <t>Hasselt University starts construction new biomedical research complex - belganewsagency.eu</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>LIFE STORY. Lieutenant Colonel Patrick (57) lived for Carnival and his family: “The fact that we don't know what happened on that highway is gnawing” - HLN</t>
+          <t>Hasselt University starts construction new biomedical research complex - belganewsagency.eu</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 08:49:56 GMT</t>
+          <t>Mon, 02 Mar 2026 14:13:00 GMT</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAJBVV95cUxQUmhTanp0cVhCQl9SNlkyUElKUUF5RlYtRFhyRFpjc0Y5Ql9oV3NsVHpQRnJVbHJRRWZDWjc3Vy1KVXJMWWhZd0pXdEZqWS1ObExKOXVqenltQks3N0NxdnI4SEFaN0Fwa25HeXY2RkRTbDE5Q3FUYThza2duN1pKN2lmYW5FWHUtS1lUVUtxYloxSzRISVBhSGR5eE5ncThDSVF1MkluTE1hUFlyc2Zyb0pnbkItTFlpbS1ZNF9BRmZiUVNROUhzN0hhT2gxNWJ1czIxS18wZEMxdG44NldhZWdIQnFMMXpCN2V5RkpyYjh1Q1pIYTVWTUJvYlNPU3N1WEJmNmdMNEU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxORGFjc2FQVS1sTXM4VFNMYm5EVlNMZV9zZ3luOXNzVl95ZG8zMmhvTmloanRoUGJHRkxjNk12RmQ4RmFqVXlRU1JoaWYyZHZ4Qzg3SjJWYWtacjF0QWJOZnhRMEU4ajhKQ3ZOX3ZmQWpIZjZEQjdWTzB0V1FLM21sUDk2WE5Jd0ZWYW9YLW1GZ0t4MnVVSlRZY3FHZ1paSzE3RWxn?oc=5</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2165,27 +2165,27 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K32" s="1" t="n">
-        <v>46083.36800925926</v>
+        <v>46083.59236111111</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2195,22 +2195,22 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Dertiger veroordeeld voor afpersing op Dusartplein na dreigen met fles - Nieuwsblad</t>
+          <t>Just an hour from Brussels, this spectacular 2.5-hectare garden instantly transports you to Japan, with its cherry blossoms and stunning traditional pavilions. - Bruxelles Secrète</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Thirty-something convicted of extortion on Dusartplein after threatening him with a bottle - Nieuwsblad</t>
+          <t>Just an hour from Brussels, this spectacular 2.5-hectare garden instantly transports you to Japan, with its cherry blossoms and stunning traditional pavilions. - Bruxelles Secrète</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 12:47:29 GMT</t>
+          <t>Tue, 03 Mar 2026 06:00:16 GMT</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxQRFZGbEdmX28wOTN5WTZ4X3JhUTBQNVF0dnJlNG5OdGJOR3JVTEo5Mkd3RkJiQU5rTWlYVDVEUmQwNGd5ZlNPOHNMWU5vRWhLSWpveWgyYlAzemtCQW54ZGZqdDhmZnE3Y2dGSHhnUnhFdjRZV05aYmpUQkdiN1ZWdVYwMHlhQnB2Wm0zY0pfNzRsemgxXzktcW5HQzE2dTA0NU5XOE03YmdZaGxDRXEwTnR4VGMyZ2kwS214X0xkZklHVzU0dWM0MjRHS1RWZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE5PUGhjelJlZTN6dkNiUE9sWkFSNk5sRi1JMlozNFFvLW1EVWJuM3c0c0UyRjlNUk5Ob2FmV0JPMGhfUFpCZURINTRxLXZWU3U4ZW1VQm5nUE9KZVdzaE43SDM0MUlYbThWdkpBRTN2REpBM2s?oc=5</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2220,27 +2220,27 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K33" s="1" t="n">
-        <v>46083.53297453704</v>
+        <v>46084.25018518518</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2250,22 +2250,22 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Wanneer de schulden je boven het hoofd groeien: zoveel mensen in Lanaken worden bijgestaan door een schuldbemiddelaar | Foto - HLN</t>
+          <t>UHasselt start bouw van nieuw complex "om onderzoek naar chronische aandoeningen zoals kanker, multiple sclerose, dementie en reuma verder te laten groeien - Truiensnieuws.be</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>When the debts grow over your head: so many people in Lanaken are assisted by a debt mediator | Photo - HLN</t>
+          <t>UHasselt starts construction of a new complex "to further grow research into chronic conditions such as cancer, multiple sclerosis, dementia and rheumatism - Truiensnieuws.be</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 09:45:59 GMT</t>
+          <t>Mon, 02 Mar 2026 13:54:06 GMT</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9gFBVV95cUxNWFlCUGJReDNpc1U3R0M0M1BhVVdyNHNFOHBnUF8yU3FMWUFNN2tOb1dkbml1cXE0N09mWlBObTRDTmw2c0lKc2c1dFdYWlJqaHMzMlBGV183bE13dS10bE9hc1EtYWw1RXd4MFpHQXF1SGZOdzV5YTFkXzdmenlLVnFLbGJSUVJ3R09wZW84dFZBRUNkZldFNDBTRUZRTjJveVFkSDJiWENDdTVjQ09jSmFfYkQ0MWNXei1fZGFlTGlQbGVWYVVSQ1BqZ2FEUXNtXzR5V1BlTnM4SDV4a2VlSHgyRjU0UVVpX0N5X1FCYmc4WWQyOEE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgJBVV95cUxQWklVMTVTWVhpdS01NndmR3YydE5ZMkJWNFV6Wmlac1FMYnlLZ3c2bzBjdVZxZ2tyYW5kZHZIRWotNW82OHU1UVFEa3lxdXFuNFYwbVR6QXlkMEg4a0dTZHpDRzJZY1JCVFRRN2NVRm1rU3JLZGtPRFVEMVc5Q182eDhWbkpsUjRJUkQ5MVhsR2M0ODFLX2QwSFljRGFfM0RNYWtmcGNCMDNXcFNlYjJUNDJCT0UwSVBOeDIyQ09ELU5LMGUtdU9CeWpZUm5tMks0Rm44NUUwZHlQdEx2MDhLbmhKTmpESGV5cmR2N2VVRDlHajcyNTZGalpuZmdfWVBWT3J0WFYwYnlGVUFqNFQ2MTB5RTlzR1hqZnc?oc=5</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2275,52 +2275,52 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K34" s="1" t="n">
-        <v>46083.40693287037</v>
+        <v>46083.57923611111</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Aux USA débute le procès contre le monopole de Live Nation, une société de divertissement qui détient aussi un quasi-monopole en Belgique - VRT</t>
+          <t>25-Jährige sowie 4-Jähriger Sohn vermisst – Wer kann Hinweise geben? - Die Bayerische Polizei</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>In the USA the trial begins against the monopoly of Live Nation, an entertainment company which also holds a quasi-monopoly in Belgium - VRT</t>
+          <t>25-year-old and 4-year-old son missing - who can provide information? - The Bavarian Police</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 12:31:00 GMT</t>
+          <t>Mon, 02 Mar 2026 11:22:34 GMT</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxQdm9pcDF0Tnd2bkdnUkY2YWdqc2laUXRibmtBbkQ3XzNHVjUyWl9PbTJfYnVxVnZEclFfcWM4ZHdWblNvVW8ybnQxNmR5VF9YYXZUYzhuV1cxU2FXSHFWQkdxRUtJOU84ZXdmaEh4ZkktZkVUX1NiTXlxd3VmbG5ZTXFQTEV6TlNQbTBwalFuaEV0WW5kVXozaFdyN2w3MjE0RXdkWXpB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxNSFJOVkZTRTN0bl9jMWZsVnR0Mk9aa0p1Njh5Y2JJeVRMc0JhQm56d2FSRVhjU3lib01jakdhVVV6OUMzc0VqNDdyNUtoaXlIOGpBNEVVVWRJZThOdVhzUk1fMXY4S1NuLWhGZzZmTVVqOFlJSFU5NmdqMnFqWDczOGdR?oc=5</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2330,52 +2330,52 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K35" s="1" t="n">
-        <v>46083.52152777778</v>
+        <v>46083.47400462963</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Hasselt University starts construction new biomedical research complex - belganewsagency.eu</t>
+          <t>Unterfranken: Polizei behält Sicherheitslage nach Nahost-Eskalation im Blick - Charivari Würzburg</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Hasselt University starts construction new biomedical research complex - belganewsagency.eu</t>
+          <t>Lower Franconia: Police keep an eye on the security situation after the Middle East escalation - Charivari Würzburg</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 14:13:00 GMT</t>
+          <t>Tue, 03 Mar 2026 04:14:00 GMT</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxORGFjc2FQVS1sTXM4VFNMYm5EVlNMZV9zZ3luOXNzVl95ZG8zMmhvTmloanRoUGJHRkxjNk12RmQ4RmFqVXlRU1JoaWYyZHZ4Qzg3SjJWYWtacjF0QWJOZnhRMEU4ajhKQ3ZOX3ZmQWpIZjZEQjdWTzB0V1FLM21sUDk2WE5Jd0ZWYW9YLW1GZ0t4MnVVSlRZY3FHZ1paSzE3RWxn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOaEZYbWwxSTVVRzhaMXlMOTg2SjQ4a2UxSTNkSmtqdW5LeWZhd08yVkRUeWUxUHowWVJlNGRHSnAtUjJyVHRxdm90QVVnN2ZCRVdmM1B2RVVfSjVTejNROFFLMjR2VTBKVVBWLXNMdFI1cjFEZ05kVFF0cXRDQmRtQXRQX2tsOUtSLVFzMEpJaWFLaEJCM2I2RDdYd2RzSTlxSThNbW1SY01TYml1QnY3ZF9Sdw?oc=5</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2385,21 +2385,21 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K36" s="1" t="n">
-        <v>46083.59236111111</v>
+        <v>46084.17638888889</v>
       </c>
     </row>
     <row r="37">
@@ -2415,22 +2415,22 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Würzburg: 25-Jährige und ihr Sohn werden vermisst - Radio Gong Würzburg</t>
+          <t>Messerattacke in Würzburg: Beschuldigter stirbt in der Polizeizelle - Berliner Zeitung</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Würzburg: 25-year-old and her son are missing - Radio Gong Würzburg</t>
+          <t>Knife attack in Würzburg: Accused dies in police cell - Berliner Zeitung</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 13:00:00 GMT</t>
+          <t>Mon, 02 Mar 2026 10:41:19 GMT</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxPcDhwNjN3OVdOSmpjWkhwbmg3Wk1oUUI3NVF0S1prQVhDWXJIR2poaG9xS3J6LTNuTy16RC11TGZlT0E3b1JqYXpWMEpxbk1CaTMtM0EtMkRjM0h6M1Vpakpqc085b1R0SVdkTExyeF9WTTIycDBsX1ZQX3pFRFNlT0xrTXJBd0pMLWZXTw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxPNklzVVAxNmFtVExYMmdGS0Z5Zm5Ydm55c3pNVV9JZ2JHcGk4YTA0dVI5VmVxMUdja3FpX0wwQjVLR3BQS2dycW1RdWJqVUVXc3VlclVpbWY4cm44ZjBMM3RheEhwSFBVQTlDZWNLeldLeU9mdzNHY2piMHpESnJQMXE2ME45X3FfVm9SV2FnU2c2SFY1eTkwZGVPZGVFd000ZGs1M3JuWDd4QVpoS0ZhU0RlejV6amM?oc=5</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2454,7 +2454,7 @@
         </is>
       </c>
       <c r="K37" s="1" t="n">
-        <v>46083.54166666666</v>
+        <v>46083.4453587963</v>
       </c>
     </row>
     <row r="38">
@@ -2470,22 +2470,22 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Messerattacke in Würzburg: Beschuldigter stirbt in der Polizeizelle - Berliner Zeitung</t>
+          <t>Würzburg: Mutter (25) und Sohn (4) vermisst - Junge leidet an Autismus - inFranken.de</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Knife attack in Würzburg: Accused dies in police cell - Berliner Zeitung</t>
+          <t>Würzburg: Mother (25) and son (4) missing - boy suffers from autism - inFranken.de</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 10:41:19 GMT</t>
+          <t>Mon, 02 Mar 2026 11:40:00 GMT</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxPNklzVVAxNmFtVExYMmdGS0Z5Zm5Ydm55c3pNVV9JZ2JHcGk4YTA0dVI5VmVxMUdja3FpX0wwQjVLR3BQS2dycW1RdWJqVUVXc3VlclVpbWY4cm44ZjBMM3RheEhwSFBVQTlDZWNLeldLeU9mdzNHY2piMHpESnJQMXE2ME45X3FfVm9SV2FnU2c2SFY1eTkwZGVPZGVFd000ZGs1M3JuWDd4QVpoS0ZhU0RlejV6amM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxNM2JHTUpheFF2SENvbERVTzFwWEROR2t5WC13RGd5RGJNRFJ2RzNkMnRmTncxN3JQX09QOFUxSmxzUlJ2dkhnRnNnSTk4eFBKU2w4U2ZLS2hEaHpOLXVZeGVKZ184R01iUGtab0ZYTS1lbUozV0NzUTRBY3NxZjZ4ZHJHS0tyU0gtV2RZSVdfMEdDek1IWVhiZWZOYVdBMXlMejNuRnVVUmJMR3RIbzhvM25VOUtyNUNGM3hJQ1BJUlA0QdIBwgFBVV95cUxNM2JHTUpheFF2SENvbERVTzFwWEROR2t5WC13RGd5RGJNRFJ2RzNkMnRmTncxN3JQX09QOFUxSmxzUlJ2dkhnRnNnSTk4eFBKU2w4U2ZLS2hEaHpOLXVZeGVKZ184R01iUGtab0ZYTS1lbUozV0NzUTRBY3NxZjZ4ZHJHS0tyU0gtV2RZSVdfMEdDek1IWVhiZWZOYVdBMXlMejNuRnVVUmJMR3RIbzhvM25VOUtyNUNGM3hJQ1BJUlA0QQ?oc=5</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2509,7 +2509,7 @@
         </is>
       </c>
       <c r="K38" s="1" t="n">
-        <v>46083.4453587963</v>
+        <v>46083.48611111111</v>
       </c>
     </row>
     <row r="39">
@@ -2525,22 +2525,22 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Würzburg: Mutter (25) und Sohn (4) vermisst - Junge leidet an Autismus - inFranken.de</t>
+          <t>Messerangreifer vom Würzburger Hauptbahnhof tot in Zelle gefunden - Spiegel</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Würzburg: Mother (25) and son (4) missing - boy suffers from autism - inFranken.de</t>
+          <t>Knife attacker from Würzburg Central Station found dead in cell - Spiegel</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 11:40:00 GMT</t>
+          <t>Mon, 02 Mar 2026 19:46:00 GMT</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxNM2JHTUpheFF2SENvbERVTzFwWEROR2t5WC13RGd5RGJNRFJ2RzNkMnRmTncxN3JQX09QOFUxSmxzUlJ2dkhnRnNnSTk4eFBKU2w4U2ZLS2hEaHpOLXVZeGVKZ184R01iUGtab0ZYTS1lbUozV0NzUTRBY3NxZjZ4ZHJHS0tyU0gtV2RZSVdfMEdDek1IWVhiZWZOYVdBMXlMejNuRnVVUmJMR3RIbzhvM25VOUtyNUNGM3hJQ1BJUlA0QdIBwgFBVV95cUxNM2JHTUpheFF2SENvbERVTzFwWEROR2t5WC13RGd5RGJNRFJ2RzNkMnRmTncxN3JQX09QOFUxSmxzUlJ2dkhnRnNnSTk4eFBKU2w4U2ZLS2hEaHpOLXVZeGVKZ184R01iUGtab0ZYTS1lbUozV0NzUTRBY3NxZjZ4ZHJHS0tyU0gtV2RZSVdfMEdDek1IWVhiZWZOYVdBMXlMejNuRnVVUmJMR3RIbzhvM25VOUtyNUNGM3hJQ1BJUlA0QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxQQ3k1djRja2VzT00yMklrdzliTW5xOUl0Qm9zY3NlNi1kanMzODZ2NEozMFpQanU3Wm5Pd2ZjVUJ6Z00zNEFRcS1kTTg5N0F3bzRaV0kwQ3p2WkRmSlE3VnZPZUEwUlNXV2N6R1dNdkZfcFFCeWVPWlNhcU9wVUF5T1VQT2RUQWtYbU5ZUFFOc2xkNG5pRWlzSWNsclJwdkdkSGl4Y3FFeWtpaEtaalZZQi0tdGllMk9ZRFk5aTk5UmpOWFg5NTB1WHN4NGR5Snpub0J3?oc=5</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2564,7 +2564,7 @@
         </is>
       </c>
       <c r="K39" s="1" t="n">
-        <v>46083.48611111111</v>
+        <v>46083.82361111111</v>
       </c>
     </row>
     <row r="40">
@@ -2580,22 +2580,22 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>25-Jährige sowie 4-Jähriger Sohn vermisst – Wer kann Hinweise geben? - Polizei Bayern</t>
+          <t>Mit dem Zug von Pforzheim nach Würzburg: Darum wartete am Gleis die Bundespolizei auf zwei Frauen - PZ-news</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>25-year-old and 4-year-old son missing - who can provide information? - Bavaria Police</t>
+          <t>By train from Pforzheim to Würzburg: That's why the federal police were waiting for two women at the platform - PZ-news</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 11:22:34 GMT</t>
+          <t>Tue, 03 Mar 2026 05:45:00 GMT</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxNSFJOVkZTRTN0bl9jMWZsVnR0Mk9aa0p1Njh5Y2JJeVRMc0JhQm56d2FSRVhjU3lib01jakdhVVV6OUMzc0VqNDdyNUtoaXlIOGpBNEVVVWRJZThOdVhzUk1fMXY4S1NuLWhGZzZmTVVqOFlJSFU5NmdqMnFqWDczOGdR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxQYUd5TURCcnhYY1FERWkyUTk3NUVYZDEwUDI2U2hOVU5vYThKV1FjUXJfUDQ5ZVlfcEh6ODNzNmdodVZKNFVwYXFtRzc5c0trRVhVMVVYNjF5UE0wM2w2d1hsdkFWYkMycXFfX0NFclp4MnJvUGIwZlZLeWo2ZjRQSTlwU1B0NDdmWk9WYzBiN1lDSmticHpWalhvSTVjRm12M2NjV19CNHZHdjlEX2dRSEF3ZHMyekZKSk84MndzLVBZVnZmRkxLeUh5bTdEbzdvWEZ3SlIyZ2Mta0tyTWR6RVRnTjk4dTdVWV80?oc=5</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2619,7 +2619,7 @@
         </is>
       </c>
       <c r="K40" s="1" t="n">
-        <v>46083.47400462963</v>
+        <v>46084.23958333334</v>
       </c>
     </row>
     <row r="41">
@@ -2635,22 +2635,22 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Mutter und Kind in Würzburg vermisst – intensive Suche - Fränkische Nachrichten</t>
+          <t>Würzburg: 25-Jährige und ihr Sohn werden vermisst - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Mother and child missing in Würzburg – intensive search - Fränkische Nachrichten</t>
+          <t>Würzburg: 25-year-old and her son are missing - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 12:54:00 GMT</t>
+          <t>Mon, 02 Mar 2026 13:00:00 GMT</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxPUHp2a0VyZC15WF9YWkp6ME1oU3dZQm5DLW9SY24zS2RTSDdReGVZLThJUnZOaFFQZUdxRXUyOVpFOG5JRGFKV1l0cFRNUFhhWmJIcVhZUENPeS1qQTlQS1FEUDlWcEdKNEwwckxnUTZwa1EyTTJDSktwbHIwdEsxS09tQ3B5blJEdDYzZXRGMGtMSEFaZmdDWl9CUU1WUzlCd2ViM1JoVHFndm5IbG1xa0NwbURCWjJ5MjFERkQycGQtTEt6M01XOWtR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxPcDhwNjN3OVdOSmpjWkhwbmg3Wk1oUUI3NVF0S1prQVhDWXJIR2poaG9xS3J6LTNuTy16RC11TGZlT0E3b1JqYXpWMEpxbk1CaTMtM0EtMkRjM0h6M1Vpakpqc085b1R0SVdkTExyeF9WTTIycDBsX1ZQX3pFRFNlT0xrTXJBd0pMLWZXTw?oc=5</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2674,7 +2674,7 @@
         </is>
       </c>
       <c r="K41" s="1" t="n">
-        <v>46083.5375</v>
+        <v>46083.54166666666</v>
       </c>
     </row>
     <row r="42">
@@ -2690,22 +2690,22 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Wertheim: Geschwindigkeitskontrollen - main-echo.de</t>
+          <t>25-Jährige und vierjähriger Sohn in Würzburg vermisst | Foto: ME-Grafik: Lena Schickling - main-echo.de</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Wertheim: Speed ​​controls - main-echo.de</t>
+          <t>25-year-old and four-year-old son missing in Würzburg | Photo: ME graphics: Lena Schickling - main-echo.de</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 10:59:33 GMT</t>
+          <t>Mon, 02 Mar 2026 11:29:51 GMT</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOUDRUWS1uZlZlLWJsQXF6X0hMY005MzZ3ZHBJandFWDBadzlkU3hjQ1VXN0NPQlVEQ21nYlRoLU1SOXAwdnhwRm41MkxMa29UbzdsM0FzbGxTcDAtYzZsWnp1QkswU01EQVVCeFVoZmVDYlRoc1ZYbTlkNmpjTlJOcjhxak93cFdJM2thd0d5eFI5WEp3SFE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNcHVqZXpxazlvU2RNeFdvVFZsQlBqbkVIZE8xQlpFY1VJWklOaFRqWGR0VmdhakRCQTlQRmxzRngtRDVDcGxDb0FVYkVhU2ZWQWJOcXdJLTZ2SXpIWVA0U0JDMWNRa0VFbjdqak1jRTVvUzk0bXJva2Y1MjFJVFZ1b2FObXZvSXlaTHNEaGFJUDN4N3BDTzRHSlpZaERhQTdWUWUtbkFna2tqUW5qRFQxeDl3?oc=5</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2729,7 +2729,7 @@
         </is>
       </c>
       <c r="K42" s="1" t="n">
-        <v>46083.45802083334</v>
+        <v>46083.4790625</v>
       </c>
     </row>
     <row r="43">
@@ -2745,22 +2745,22 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Polizei-News Aschaffenburg / Würzburg / Essen, 02.03.26: Sechs Jahre Haft für Embargoverstoß mit Luxusautos in Würzburg und Essen - News.de</t>
+          <t>Mutter und Kind in Würzburg vermisst – intensive Suche - Fränkische Nachrichten</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Police News Aschaffenburg / Würzburg / Essen, March 2, 2026: Six years in prison for violating the embargo with luxury cars in Würzburg and Essen - News.de</t>
+          <t>Mother and child missing in Würzburg – intensive search - Fränkische Nachrichten</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 12:08:02 GMT</t>
+          <t>Mon, 02 Mar 2026 12:54:00 GMT</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQRlBaRWJ4eE05QlRYZUZBb1dWd01WQXVldG1icEFvM2hYVGwwbHc4YnlpNVR2REdJTUhXRVFMcVVndjRlTy1vWWRyVkwyQVEzZHQ4bWkwN3RUS2N3Q2JWeC1BWEd6RS1ucTJOZTJSUE5FdnZCTHhVMWFCOFBfNlNFeDBWYUZyb2J1MDVHWjNCSXhPd19GUnFvOHpOVXd1VWpfTWZlN0JrOHRFNTVaTElrTNIBtgFBVV95cUxOZWl1eVFfZ2kxaDZ5bUdkMWU1NWhQaE5QX1NBVVJEOXN0bDB3MTJQZDJCMTl5emlrTko4aXhSUmN4X3lhUlBtaTdjZjZQbWdWY2pVT3VHU1loNFBsQkE0QWZGcnM3ejZjbTdaU3pVVDF3OV9rd2Z1MXFJdk9TVUE3Qk03Sy1qdjBaRHFHdFdObG5mT1Vfbi1TekFBdnZOVEE5a29nYk83cEdlSERzb3ZxcUk4TTMxdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxPUHp2a0VyZC15WF9YWkp6ME1oU3dZQm5DLW9SY24zS2RTSDdReGVZLThJUnZOaFFQZUdxRXUyOVpFOG5JRGFKV1l0cFRNUFhhWmJIcVhZUENPeS1qQTlQS1FEUDlWcEdKNEwwckxnUTZwa1EyTTJDSktwbHIwdEsxS09tQ3B5blJEdDYzZXRGMGtMSEFaZmdDWl9CUU1WUzlCd2ViM1JoVHFndm5IbG1xa0NwbURCWjJ5MjFERkQycGQtTEt6M01XOWtR?oc=5</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2784,7 +2784,7 @@
         </is>
       </c>
       <c r="K43" s="1" t="n">
-        <v>46083.50557870371</v>
+        <v>46083.5375</v>
       </c>
     </row>
     <row r="44">
@@ -2800,22 +2800,22 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Blitzer in Würzburg aktuell am Montag: Hier nimmt die Polizei am 02.03.2026 Raser ins Visier - News.de</t>
+          <t>Polizei-News Aschaffenburg / Würzburg / Essen, 02.03.26: Sechs Jahre Haft für Embargoverstoß mit Luxusautos in Würzburg und Essen - News.de</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Speed ​​cameras in Würzburg currently on Monday: Here the police are targeting speeders on March 2nd, 2026 - News.de</t>
+          <t>Police News Aschaffenburg / Würzburg / Essen, March 2, 2026: Six years in prison for violating the embargo with luxury cars in Würzburg and Essen - News.de</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 13:17:49 GMT</t>
+          <t>Mon, 02 Mar 2026 12:08:02 GMT</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxPRHVqeEF6MXpUYjhxZVJtWUxnQjdXMnZuRmN5MkVjUzR2am8wX0xxa192aFVrSnRBVE5rZVJ4eXVhWU8wTzA1SmZDQndnRVJsU3MyWGxSWUpGY2h5ZFhEa21YSGU4dHdEZ0NQWmNPc0hXVEtzbF8zUkVVRkVxTEpjbjNsTkFmLUFRa1puZDQ1SldXQTRoV1c3alhETU9PdVZFeDZPY01HbUV0UWdSbDFWMWdLbGNJQlRUakxKOEFCeFl1SHhZQ05LSUdhTFpHUVh5bjE3WVdhdmt4U21CckRCYm1DcUzSAeoBQVVfeXFMTjFXcHpBak5pWkZuTEUzeFp5di1wNVFSR2p6TGc0YUp0cmFoeWRQSFJFSU1nSnRBd3JHN0ZfWng3ekpfbi15WjFZQTFlcW9BUGg4VTRMWElfZUZVM19uTHdzTFpFX3ZlQVNrWmJfalpxZ3ppS01HLWk4RDkwb1RHX2x6SHBYLVlLX2JvbS1ST3h0N2ZaT2pTaHVnLUZneW9BRE9RZVladzJ4WlNwTVJxTkZRekdrakNQc3JPNmhVdHkxOF9JaTJrYkkxaFVnLWhWbTRNMnlzdmhjVk84WEVWUTQyWEo0MXBqOTV3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQRlBaRWJ4eE05QlRYZUZBb1dWd01WQXVldG1icEFvM2hYVGwwbHc4YnlpNVR2REdJTUhXRVFMcVVndjRlTy1vWWRyVkwyQVEzZHQ4bWkwN3RUS2N3Q2JWeC1BWEd6RS1ucTJOZTJSUE5FdnZCTHhVMWFCOFBfNlNFeDBWYUZyb2J1MDVHWjNCSXhPd19GUnFvOHpOVXd1VWpfTWZlN0JrOHRFNTVaTElrTNIBtgFBVV95cUxOZWl1eVFfZ2kxaDZ5bUdkMWU1NWhQaE5QX1NBVVJEOXN0bDB3MTJQZDJCMTl5emlrTko4aXhSUmN4X3lhUlBtaTdjZjZQbWdWY2pVT3VHU1loNFBsQkE0QWZGcnM3ejZjbTdaU3pVVDF3OV9rd2Z1MXFJdk9TVUE3Qk03Sy1qdjBaRHFHdFdObG5mT1Vfbi1TekFBdnZOVEE5a29nYk83cEdlSERzb3ZxcUk4TTMxdw?oc=5</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2839,38 +2839,38 @@
         </is>
       </c>
       <c r="K44" s="1" t="n">
-        <v>46083.55403935185</v>
+        <v>46083.50557870371</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>5000 Euro Schaden: Unbekannter bricht in Geschäftsgebäude in Schrobenhausen ein - Augsburger Allgemeine</t>
+          <t>Blitzer in Würzburg aktuell am Montag: Hier nimmt die Polizei am 02.03.2026 Raser ins Visier - News.de</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>5000 euros in damage: Unknown person breaks into commercial building in Schrobenhausen - Augsburger Allgemeine</t>
+          <t>Speed ​​cameras in Würzburg currently on Monday: Here the police are targeting speeders on March 2nd, 2026 - News.de</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 13:35:16 GMT</t>
+          <t>Mon, 02 Mar 2026 13:17:00 GMT</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxOLVUyU0lSMldhUGdzVDFWbkc5WjBwTmx1c3pJZXpuZUEtUjdkQ0lleEg5b3MzTm50WGdaRElIQk1qcXdudlJOYUN1aVkwZ0U1U0VCSzJ4NERoZl9BekVPb21wVzJ0RmF0ZThpdTVQbFZURE1pZ1NBUVFjTk5maWo1NmdwckJrSVZFcU9Pd3Y2RmtCZlNXaHBJWkNJZHR0V1d0dHQ5aDE3SFY0S2RPTXBBa0dZb2JZT09RZ0dqOW5ZbFhXMmpCbUVEVHpoQlcyaGUy?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxPRHVqeEF6MXpUYjhxZVJtWUxnQjdXMnZuRmN5MkVjUzR2am8wX0xxa192aFVrSnRBVE5rZVJ4eXVhWU8wTzA1SmZDQndnRVJsU3MyWGxSWUpGY2h5ZFhEa21YSGU4dHdEZ0NQWmNPc0hXVEtzbF8zUkVVRkVxTEpjbjNsTkFmLUFRa1puZDQ1SldXQTRoV1c3alhETU9PdVZFeDZPY01HbUV0UWdSbDFWMWdLbGNJQlRUakxKOEFCeFl1SHhZQ05LSUdhTFpHUVh5bjE3WVdhdmt4U21CckRCYm1DcUzSAeoBQVVfeXFMTjFXcHpBak5pWkZuTEUzeFp5di1wNVFSR2p6TGc0YUp0cmFoeWRQSFJFSU1nSnRBd3JHN0ZfWng3ekpfbi15WjFZQTFlcW9BUGg4VTRMWElfZUZVM19uTHdzTFpFX3ZlQVNrWmJfalpxZ3ppS01HLWk4RDkwb1RHX2x6SHBYLVlLX2JvbS1ST3h0N2ZaT2pTaHVnLUZneW9BRE9RZVladzJ4WlNwTVJxTkZRekdrakNQc3JPNmhVdHkxOF9JaTJrYkkxaFVnLWhWbTRNMnlzdmhjVk84WEVWUTQyWEo0MXBqOTV3?oc=5</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2894,38 +2894,38 @@
         </is>
       </c>
       <c r="K45" s="1" t="n">
-        <v>46083.5661574074</v>
+        <v>46083.55347222222</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Kildare community rally at dementia inclusive event - Kildare Now</t>
+          <t>Polizei-News Essen, 03.03.26: Unbekannter versucht Geld aus Supermarktkasse zu rauben - Fotofahndung - News.de</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Kildare community rally at dementia inclusive event - Kildare Now</t>
+          <t>Police News Essen, March 3, 2026: Unknown man tries to rob money from supermarket checkout - photo search - News.de</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 12:00:00 GMT</t>
+          <t>Tue, 03 Mar 2026 07:08:02 GMT</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOWGszQ1BoWHNCT0d0bWo2UVBXb3Q3bkJKUTVUSkZ1VTBMTWhDQWhoNUt5NVFQZm5CSTNmUVEtOElSZ3hMMU8wclY2bkEzQ296a3lGZEhjc1hjVFpQZFFwUXh6eGxLZmdNczF2VzN3OTBGNHBYYzBQM2NBRDBLMHVxNVNoTzhGRWs2bERSOTRTZDF4WEJXQU1lNXQwcEJkaUhzd0pkVnE5R2k4dw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQa3FjTkhEOEM5ekJGclVqRGV2QWNlc2FRNGxFN1dwMks0WEtGbjdrdl9QOGlvTlRObnFSS19XVnFwOVhuQkw4VzVYQlFIYjJwVWRWRXZ1LTFQOUNVVG9QR1QxVC1WYmR0cjU1ZjIzYl85TF9FV0RTNVpOX2dDOURVbXM4bzBCeHFCWTdKNHMzazJYdXZ50gGaAUFVX3lxTE5kQTBRXy1JdW5qeXp3VEFKQnFmdmpQOXZkMEVvTEZZczVzYkkxbkZLZlVKTmRzNEVNNzh5VDdMcDJXcTNKdzlKeV9vcXV2b1VVMlh3c3N3ZHp6QmlCeGUxU0YzZ0xVNHNiXzRaZEZvSVNYNjdodFJMSDdRRzVYUU1LQmZHcjd0emxwZVBLTGZlNFgyMDZtcUx6ekE?oc=5</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2935,52 +2935,52 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K46" s="1" t="n">
-        <v>46083.5</v>
+        <v>46084.29724537037</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Number of gardaí stationed in Kildare remains near record levels despite slight decrease - Kildare Live Leinster Leader</t>
+          <t>5000 Euro Schaden: Unbekannter bricht in Geschäftsgebäude in Schrobenhausen ein - Augsburger Allgemeine</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Number of gardaí stationed in Kildare remains near record levels despite slight decrease - Kildare Live Leinster Leader</t>
+          <t>5000 euros in damage: Unknown person breaks into commercial building in Schrobenhausen - Augsburger Allgemeine</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 11:01:08 GMT</t>
+          <t>Mon, 02 Mar 2026 13:35:16 GMT</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxQZy12ZHpwakdiQ0hkYldPcUphcm1pTFc3WXJ0dWhPMFM4OFloS2M5M192YWdlc3JveUJhbTJmT05wQ2l1Q0RNdGJQUGJDeUlYTndXVDVfXzZ3RjVGRF9OT1JXN2dOaGpQYnIzOUY0ZUxBX1NLYVZ6ZXVhSWJnWksxZ3pQcjZtd1JRNXRURUFmTEVncXg1c0dveHh3ekp0SGw3ZHRNVWtVR0lnSTk0d0c4aGl2ZzI3Sjg5am1PNmRQNGY3WUJvVUJiNHQ3WGdxdDczNG9GQURFWnZrVnBMazluZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxOLVUyU0lSMldhUGdzVDFWbkc5WjBwTmx1c3pJZXpuZUEtUjdkQ0lleEg5b3MzTm50WGdaRElIQk1qcXdudlJOYUN1aVkwZ0U1U0VCSzJ4NERoZl9BekVPb21wVzJ0RmF0ZThpdTVQbFZURE1pZ1NBUVFjTk5maWo1NmdwckJrSVZFcU9Pd3Y2RmtCZlNXaHBJWkNJZHR0V1d0dHQ5aDE3SFY0S2RPTXBBa0dZb2JZT09RZ0dqOW5ZbFhXMmpCbUVEVHpoQlcyaGUy?oc=5</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2990,52 +2990,52 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K47" s="1" t="n">
-        <v>46083.45912037037</v>
+        <v>46083.5661574074</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Las Rozas English</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Las Rozas" OR "La Roca del Vallès" OR "Mataró" OR "Badalona") AND (protest OR bomb OR explosion OR shooting OR stabbing OR evacuation OR "police operation" OR arrest) AND -football AND -transfer</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Two Kildare homes in the running for RTÉ Home of the Year - Kildare Now</t>
+          <t>A fire at a school in Badalona forced the evacuation of 500 people for an hour - Diari ARA</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Two Kildare homes in the running for RTÉ Home of the Year - Kildare Now</t>
+          <t>A fire at a school in Badalona forced the evacuation of 500 people for an hour - Diari ARA</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 12:30:00 GMT</t>
+          <t>Mon, 02 Mar 2026 15:57:50 GMT</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNNW9faXVtZ2pJNTloeV9sSjdfSXoyRHMwOEItWjlrLXg2WE9zVHVGdHNOeHUzeURzc0YzMV9vMnhVTkJ1RHhsbGE0UUhRaFpuQmZSY3JZSENYMU1IRG5ueDQ1X0dmZmR2aHdGMmJaNC1oX3RGeTF4aW5rRjU5Qloyd1ptcWVHd0w4WkdoNFl0QjJaNEdjNEFKYWRXQXdpZmF3TmZwbnNOYTlndWt1cUp4ZTZYZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxPeFplNjZZNkFzc3ZCY2t3TGFOSlB0TzFvT0wxU0ZDbXFXZy1vY2pRVGhZWUxBLUV0c2NHaWJkX0p5a1JBOVhKYTBKalJCZThQWFZoMHl6UTVRNDFHdzFVOHJtbHdBRlF6U1BEUEVmcHRSMnRxVFloN1VubGNkZGgzY1VNVTU5dVdkazVla1NxRm9hOVRGajFoaG9ZUDNTSC1qQWFFOHJLQ0FvY2Q2UWZVcUp3WFhORDIt0gG-AUFVX3lxTE5BeXMwcTlTeGZHT0liQlpPZ0d4RGNhaXNNOTFaT3NGZXJadEF5TlF3RlNiQkhMSDk4V0dhb0MxbWV4MVBCMlBxcnZaRGRhVXhSRS1YbUNaTE45b1FTSXNFWDNWSUxoaXpJN0p5ME8yQk10SGtfeXdFa1E2dVdwUFdSUERnVlptTUN2STZiUEdVNjk0X1RHNG45dDJVd2NvVTJ4bnVrcWZUZ0xhTFlCODRrakJKcEtaREZxektDMkE?oc=5</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3059,38 +3059,38 @@
         </is>
       </c>
       <c r="K48" s="1" t="n">
-        <v>46083.52083333334</v>
+        <v>46083.66516203704</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Village Bicester Kildare</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester outlet" OR "Kildare outlet")</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Jessie Buckley: Hamnet role changed who I am - kildare-nationalist.ie</t>
+          <t>Number of gardaí stationed in Kildare remains near record levels despite slight decrease - Ireland Live</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Jessie Buckley: Hamnet role changed who I am - kildare-nationalist.ie</t>
+          <t>Number of gardaí stationed in Kildare remains near record levels despite slight decrease - Ireland Live</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 07:51:58 GMT</t>
+          <t>Mon, 02 Mar 2026 17:28:10 GMT</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxPSE5UbG05ZXhhYmJRYmFCUVk2YjlwdDRHUlpfVGI0TmhhbnFfV3FjWXRjaWU4UnRNTTA2ejRhSXQ3SDJjVWNSajh1ZGJqRzZPWDh4MjRUQk5GVGxraERHWDRKcVhYU1dKUW1ScDlraC1KMWRjRFdUWkdQYW9IajRweDdJMWxRQmV4WFA0MkJoM0ZZOU93T0swc3RGNHhhX2xk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3wFBVV95cUxPcm94X0w2R2N4UERvejlrVFk2V3l4WWlXOFJfZXlSZ1ZVUHd2TTQweE92bXF5QzEwTDVfTEsxcHQ4cmtXWVNHUWlSaVpBbzIzaDNfcWhoUHFMRHRkTERiZHBFbEJBdEExVE4tRGRpOXg1al9vMW9sb2VudlF4NXZiOS0wQ3p1SWh4ZTBPS3M5RlRqXzF4dTdUVHFvUHBvUEtJQzZMVHBoX1B2T0J3SEVsTVlFdU5lUVI4VFpwajIxZWxwb3BnNk1JWFI2VGd2YTJXVlNEMXFuYnRWbV83NE9r?oc=5</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -3114,38 +3114,38 @@
         </is>
       </c>
       <c r="K49" s="1" t="n">
-        <v>46083.32775462963</v>
+        <v>46083.72789351852</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>High Level City Italy English</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Milan" OR "Milano" OR "Bologna") AND ("Italy" OR "Italian") AND (protest OR demonstration OR rally OR "civil unrest" OR strike OR blockade OR march) AND -football AND -transfer AND -Serie AND -"fashion week" AND -catwalk AND -runway</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Kildare Death Notices for today: Monday, March 2 2026 - Kildare Live Leinster Leader</t>
+          <t>Demonstration Alert – March 2, 2026 - U.S. Embassy and Consulates in Italy (.gov)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Kildare Death Notices for today: Monday, March 2 2026 - Kildare Live Leinster Leader</t>
+          <t>Demonstration Alert – March 2, 2026 - U.S. Embassy and Consulates in Italy (.gov)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 11:33:45 GMT</t>
+          <t>Mon, 02 Mar 2026 16:29:30 GMT</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxPdHV4a3puYkplRTY4ODItNDVmRlBHU2kxc2xJZF9Mek5tMGRSbkZLXzcwR251SlpoM2U5bzRwaWRGcWVxbmVjZXYyWENIX2RjU2xsV2dFUjBIWGROR21DWENkZDZJQ1RiaHNhcWJxVmF0U0NSU0RfSWUtTHptM1Z3Y2VuSTdrcGhVd2Rmb0U0WmFBdG1lbVNLQ2lPQlhjQlZvNUljd0sxOVhNdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTE9DdmczQjNFbnNBVUVSUGZxa0t3cXp5ZThxUTZoUGp4OFhNNGN4bEljbFU4V3VrS0xBUEdudUhkVDUwTFUtakhIeUtmQTZyakRueUNDb3N2MFV3UGhaNEUyTWRaSnl1am1VMkE?oc=5</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3160,47 +3160,47 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:en</t>
         </is>
       </c>
       <c r="K50" s="1" t="n">
-        <v>46083.48177083334</v>
+        <v>46083.68715277778</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>High Level City Italy English</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Milan" OR "Milano" OR "Bologna") AND ("Italy" OR "Italian") AND (protest OR demonstration OR rally OR "civil unrest" OR strike OR blockade OR march) AND -football AND -transfer AND -Serie AND -"fashion week" AND -catwalk AND -runway</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Kildare artists and creatives feature in first ever guide for wetlands communities - Kildare Now</t>
+          <t>A multi-sector 24-hour strike will commence in Milan, Italy on March 9. - SafeAbroad</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Kildare artists and creatives feature in first ever guide for wetlands communities - Kildare Now</t>
+          <t>A multi-sector 24-hour strike will commence in Milan, Italy on March 9. - SafeAbroad</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 14:30:00 GMT</t>
+          <t>Mon, 02 Mar 2026 19:20:50 GMT</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxPOFh1ekVybGhFMkRkd01JbTV4WjVqckVRMlVjMTlPSGZqa2VxaTNHZlpBSTM2ejA1ektBZzlYUzNKV3YzOURSbXQwdVVXdWxuRkIyaGlRYlVEVlI0Szd3R0hkWmIyYmNlTGFjVmdWR2tXZnhvR0R1ejF1WF9YZ0Y0S1pManB5RkQ1OEFGNkEzc3NXdXhOZllld2ZyMF9PR2xvSUoxN25uUVhWSkVFdW9RdERWNjlsWlNnSnE3Ty15OF94bWlKc3dDQXlfSGJQM3F0T1M5LQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxOWUNRWDlEcUprbEFXS3pNZHpnZHJJRFdOTk5HUGZCbjVxbHlNMHdxczNRenpLOXZaclFnWElRQlVISDF1R2phZE50QmhTdHY5TzltckhBOUdxOXNRc1lKQnpYY1Jha1JHdTdoWDY5cGxPN3htUzNRY0Z1cGlhT05mMjdVZmlmX0xoTkxYdHhkWXluUWM4bDdaT2hwUGZPWDZRTmNkQVBXYw?oc=5</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3215,47 +3215,47 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:en</t>
         </is>
       </c>
       <c r="K51" s="1" t="n">
-        <v>46083.60416666666</v>
+        <v>46083.80613425926</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>High Level City Italy English</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Milan" OR "Milano" OR "Bologna") AND ("Italy" OR "Italian") AND (protest OR demonstration OR rally OR "civil unrest" OR strike OR blockade OR march) AND -football AND -transfer AND -Serie AND -"fashion week" AND -catwalk AND -runway</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Young people in Kildare to be hit hardest by government rent hike measures - Kildare Now</t>
+          <t>Fresh starts at Gucci, Fendi and Marni set the tone at Milan Fashion Week: 5 trends and buzzwords - KSAT</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Young people in Kildare to be hit hardest by government rent hike measures - Kildare Now</t>
+          <t>Fresh starts at Gucci, Fendi and Marni set the tone at Milan Fashion Week: 5 trends and buzzwords - KSAT</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 13:30:00 GMT</t>
+          <t>Mon, 02 Mar 2026 11:22:58 GMT</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxNemdYcENxQlRvSlJxSEdWVWRwUDFRWGVkQnNQSFVsWG1ZZ2VHV3VCYldiZnVlM3prZlVfSk5Da1dYTDlOYUZCNWtwOGlhOEY2Zm5yTlpXa0V1azRZbU9ZakM3ZGFhWjFDQmZnQTZDSEJYRE1YV01GTkx2aTNYYzFVWXRGNTlxNWItQlFOTE5XVHc2cW1qOXJyUUw5OFFNNk5KTFhzejdhcmg5VEFKUTAydEE2ZTVnYkFYb2dEVjFmbWRzaHVZTld3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxPa3d1cXBwRjQ0Q3FwanNuTHM3Ykg5b2Q0OWNOalR0NHpqa0d0V1JZWkgxZUZ5VTlyTDNKbG5Rcm1xTGMzNHlWX2xwYkhTTlF3UFp6dGJLMTJzRkVoX1QtaWE2bWhyWnNkZnZjeHJVNEVpVnU1VWg3VkxBRjRmSzdyZGFpUk96NEhnbThOWkh6NkM0UUdoQ0NjRy1GbTVoQ2ZOekdWREdId0NBMV93QzJCbERUODlhZFB5VWx1TnJsVGVzc0dVUE41SmdSNWdhem4xM3pvZF9yRXYwdw?oc=5</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -3270,47 +3270,47 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:en</t>
         </is>
       </c>
       <c r="K52" s="1" t="n">
-        <v>46083.5625</v>
+        <v>46083.47428240741</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Inside Christian Horner and Geri Halliwell's £9.2m countryside mansion - Bicester Advertiser</t>
+          <t>Sciopero trasporti marzo 2026: quando si fermano treni, aerei e mezzi pubblici locali - Italia Oggi</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Inside Christian Horner and Geri Halliwell's £9.2m countryside mansion - Bicester Advertiser</t>
+          <t>Transport strike March 2026: when trains, planes and local public transport stop - Italia Oggi</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 13:02:42 GMT</t>
+          <t>Tue, 03 Mar 2026 06:39:03 GMT</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxNWWhsU0RpVzI5cnpnQWkxOFFPdnpqbG5EVVlYZnExWFFoTDBTXzFqRTJ0Uy1XdDhqQ0RfUXhiR2l6SHc5WlQ0RlRvVERGcHdER2tGVzVPTWlfajFpOUo3eEcySW1xRVYtVl9RSU9OWTItOW5CdkRUWkg4dGJ4d2YyS0VHQnRVWUF3MHpESFhiWm9ERjBJNm5JalhobHlrQkxCUmFhMw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOQzJqcF85TU9pOVRPcWoyYzFJYzJYRGx2X3I0QnI0cVJNRG05UUZCNl93YlEtUEpKZFZ1WnhXSlUyTm1ZbTMxQ0xKdURUaVNvd1RiaVFVUWdSWXpGNm10MzB3Vmp5WlcwSTY1czhaQUZoQXg1OHVHUDFmallBNEhmdWdLc0hpbmNzR1QwbGNxSUhjU29VS2huUnVKcjQ3dnNmby1MMENEOFV5MjVBRkJYLUgyeUxoZlE4ai0tY2ZQdzZ4cUtPTWlhc3hJNFVBUmZQYUdNbk5xV1ktRG5QdjZJSnJ3?oc=5</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3320,52 +3320,52 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K53" s="1" t="n">
-        <v>46083.54354166667</v>
+        <v>46084.27711805556</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Cat Deeley returns to This Morning after short absence and admits blunder - Bicester Advertiser</t>
+          <t>Iran: Milano scende in piazza contro la guerra - Collettiva</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Cat Deeley returns to This Morning after short absence and admits blunder - Bicester Advertiser</t>
+          <t>Iran: Milan takes to the streets against the war - Collective</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 10:26:30 GMT</t>
+          <t>Mon, 02 Mar 2026 15:37:57 GMT</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxNb2Y0T29XaUE4OXhuRldpZnBNRUl5WFdvT0xXNDRPOG5pY3FhMWxTcnZCWVYzVmVvMzRZdExhUlduNlRRZzdnVTVmVmNqeXJpdjYwVGZ6RllDQ0ZKdFBwR2VsSVp3Y2cwSG4wNl96dERrUXpuR1BEWmdjWFpGU0dvOEVJYjRDU2JRV2VCN0RMdnRzZ2R1Mlo3aHB5UWN5Y1ZWSFlTTmFqWG5MZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxPYmN6VEN1aWlsM1BEM2dOODlva0FFNGZ1M21CeHVHck8tSlFnVVRiMGxYemtkN0E4RllCNWh4YmxjVHlaZDRGVi1ISmNHdFRoRXBvSkdzOVFwMzBVVWNDS2ZVUGJhenhxdW81Nkd3a0U1Z0xrdHdUZWxnNWI1bkVuQmNWaUhfQm9FQmZuUDhmTEhoWXZlQ1RGdQ?oc=5</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -3375,52 +3375,52 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K54" s="1" t="n">
-        <v>46083.43506944444</v>
+        <v>46083.65135416666</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Kildare people urged to apply for ESB apprenticeships - Kildare Now</t>
+          <t>Bologna, manganelli sul presidio a difesa del Pilastro - il manifesto</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Kildare people urged to apply for ESB apprenticeships - Kildare Now</t>
+          <t>Bologna, batons on the garrison to defend the Pillar - il manifesto</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 10:09:00 GMT</t>
+          <t>Mon, 02 Mar 2026 23:13:18 GMT</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNVXo0VjVZZzJMZmY4Nk9oU3pXTlctdUpTZk5HVzFuOTJpeG1hT2NLSVZCbDV1X2NwX0xEdWdYa2drOXhTNDFlQjBidldwUk5fLVE3TThGZ256bEJ5MFlWNC1VMUlhaUJ2czZWbzV5ZmJXdXhYSmNUVVBWRFRlXzNodWRrdnVNMjlfTGQ0aUVGaUYyd09OV0NDRF93SUhqSzhqN2c5em9BU2pIdDhCbWc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxPd01RMHB6ZnFWMXBiZEhzdFlKWlZibW9wNFJIeUpSVlR3aDZuMjNaYUFVZVZrWVhBLXVXU1g5d0hVdlphVXN0MkdqLVJnMTJHQ0k2emk4UHM0eUlDNV9oak5kZjlMa1JYaUNjd0JlTFJGLU9xd0pqWGhNZVlaRTBWdTNR?oc=5</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -3430,52 +3430,52 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K55" s="1" t="n">
-        <v>46083.42291666667</v>
+        <v>46083.96756944444</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>March Premium Bonds winners revealed - see if you won £1 million - Bicester Advertiser</t>
+          <t>Sciopero 9 marzo 2026: coinvolto anche il personale dell’Ausl di Bologna - Il Resto del Carlino</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>March Premium Bonds winners revealed - see if you won £1 million - Bicester Advertiser</t>
+          <t>Strike 9 March 2026: Bologna Local Health Authority staff also involved - Il Resto del Carlino</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 09:21:40 GMT</t>
+          <t>Mon, 02 Mar 2026 15:08:53 GMT</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPOTA0aXhmSkhKX28xRThFVUUtODctemhNZDh6QjlaYXdTUE85aVB5SWpGNlBFcm43Q1U0WVJZWVQya3kyd0xZZE02UDB4TDNYYnM4RFpoYjM1MlJvSmt3bnRuVUFteXlfVmN5S3dTMUY5ampjV2Y1QzRxMnpfNGhfSHBxWGxoMUFMaHE5Sk9xM0s4aGxVY05ZUXdWcGk1VmxYOEZTWU5EZTRINDQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxPak82cnZHQ29ld3p1QkdfelA4WjlOZnBuSXNha2FhQmJXbFBtRm1UR2NGcTRwRXJIZmpadGdhWE9BWmFPMV91ZDdrQmYwTndLZmJBQ2FBRXRPNDQ0ZHpaVFRMU181bms5ZXJnTHU0dEprSW9ackIzWkZNdzlYWWdtUDFOOUZieU5SbXZWOA?oc=5</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -3485,52 +3485,52 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K56" s="1" t="n">
-        <v>46083.3900462963</v>
+        <v>46083.63116898148</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Inflation falls slightly in Feburary to 2.4% - kildare-nationalist.ie</t>
+          <t>Iran, presidio sotto il consolato Usa a Milano: “La sinistra ci ha ignorati” - La Stampa</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Inflation falls slightly in Feburary to 2.4% - kildare-nationalist.ie</t>
+          <t>Iran, garrison under the US consulate in Milan: "The left has ignored us" - La Stampa</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 14:15:42 GMT</t>
+          <t>Mon, 02 Mar 2026 18:50:00 GMT</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNelFKM2xTQ0hTZDhIa0RkUHgwbi1jYmNjdV9FaWl3eFphRko0aHBlZnN4QXZDQ1drN3BKSTAyZDBYcFp4a2pfUVVaT0ItTjZZVWlpN2o3d2VJYU1MNy1USE91UWtqU0ZGUWNTQlNoS3RHMXNybTBUNXBZeWhJSjk3TEpjSFFsWVZOc3RYNkVZMlBQX3ExckVYTU5iSmM5a1Jf?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxNakhza1dvVGx3VUZvRzhIeF81LWxNcW94b2lFcHpxR2tIcEtLN200TVVwQXA0RUZ0RFBiU3pna2l0N0ZtbHFiU0xiQlFCLWhwSjFFMk5PWG9UTldEOTZHOVQwWFVHU25qQi02TjBWa19GZlVCbHdibUpaNkxqbnU2WU1fVmdoLWNKSFY3cnBtRmFKOWgwVXlCM0lMZkJNelFXQTQ3OEtlSdIBnAFBVV95cUxNQlNRd1REaHZBdmxGcW40TEE1RFdaTVY1R3UtR1dYcG5UWm9IX3l1MVhIazg3UURxYVBfWGNZWjBFd0x3amVwLTl6S2NVTndhVFNJVWMtTkd0ZEdsWkVoM05oV2JpV19faFBPMVN0elZ1QTVKSXQ3UE9DMVM3XzRGa3ZZanlHSHNBcXFQd2l3Nmg0QW5RcmFmTkVtVUY?oc=5</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -3540,52 +3540,52 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K57" s="1" t="n">
-        <v>46083.59423611111</v>
+        <v>46083.78472222222</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Irish peacekeepers in Lebanon ‘safe’, minister says - kildare-nationalist.ie</t>
+          <t>Gli iraniani fanno festa davanti al consolato di Milano e alla fine ripuliscono la strada: il video - milanotoday.it</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Irish peacekeepers in Lebanon ‘safe’, minister says - kildare-nationalist.ie</t>
+          <t>The Iranians celebrate in front of the consulate in Milan and in the end clean up the street: the video - milanotoday.it</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 10:50:19 GMT</t>
+          <t>Mon, 02 Mar 2026 09:23:11 GMT</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxQTkFiWHhUWVMwaXpINm8zLXNnSjROYTA2a3dPdzFpbjJ3Ml94bjF1OHl2LVdZdzJ3TnZtZXdmQ2R3UGNHSzZGME1MZEZkMWdrSlpxUXdPenFCRUFaUHlxZXhBVGZvbHB2QngxZlVCcEdTLV82SU1GUTFCcDdfUTN6Y3V3Q2dkbWVwdHkzLUtpMjJkZXhsNzlqNTlRMWdqbzJiTlFza3k5NA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQcGo1Yzg4OTFGVmFUa2haUDlJYXdNMVlSbGg5eXlMYVRwUTdiN09IY2liVmhReWV5djh0aXAzaGtwZjlfUklkdzlxX3hCS2ZHMFpKbGZma3FkWGJBVXpXV2pYSUlrbjN0N3Q4MjNUNWcxMlZzbm43aGZOUXVzNklGMENyNzNLdzlTWnYycC1yTVNaTFg0VjV0Y2x5b0k?oc=5</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -3595,52 +3595,52 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K58" s="1" t="n">
-        <v>46083.4516087963</v>
+        <v>46083.39109953704</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Two teenagers killed in collision in Co Mayo named locally - kildare-nationalist.ie</t>
+          <t>Sgombero del presidio ambientalista, tre arresti a Bologna - ANSA</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Two teenagers killed in collision in Co Mayo named locally - kildare-nationalist.ie</t>
+          <t>Clearance of the environmentalist garrison, three arrests in Bologna - ANSA</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 14:00:41 GMT</t>
+          <t>Mon, 02 Mar 2026 14:40:20 GMT</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOSW5lbnF0RzlNUGFWbUp3OWk0ZXptanluUnYzVjZyQlVuUVJxd1A3bXlrRVN0ZkV6OW9FMXBDZUd4M1gybWVtcm9fbnN2ZzNsQXdORzlMY04yVGJxNnlkbUxnUm45eVQ2TzBieG93a2UzRjliWUZwYlZQLXA3NnpQX3JnanVzS2RXeWxnSVZwYW53cV9PTGZ3SnppYzRkSU5taS1sUzlDQ2Z1NTM0X0p6ZURNcDA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxPc1lndWswUnpSZjhsZXBlb08xUmQwMUxHVm53WGFqaUpBNlNNYWlsZm5VOXQxQk1ITmM3MFZHZi1YaVJGSjlpR2kwdUtyY0dfQUR3Q0lyTFZwUTJjelBtUzItRXZDZ2ZJeWhtUTZHbUYxN21na1REaVp1aDRGQTEtR2pWSFRVTlNmeHh2cEw2VnpfTHAwWko4NXVtTGtWUHBwcllQZDJuZmJSNS16eEMxTUFId2lkRGs4bHJOQm01VTJlaEhHV1UyRExFRFpqOHE0MzNUeXdjRGR4NldfU2oxV1QtSG91TnIzMnllYdIB7AFBVV95cUxPc1lndWswUnpSZjhsZXBlb08xUmQwMUxHVm53WGFqaUpBNlNNYWlsZm5VOXQxQk1ITmM3MFZHZi1YaVJGSjlpR2kwdUtyY0dfQUR3Q0lyTFZwUTJjelBtUzItRXZDZ2ZJeWhtUTZHbUYxN21na1REaVp1aDRGQTEtR2pWSFRVTlNmeHh2cEw2VnpfTHAwWko4NXVtTGtWUHBwcllQZDJuZmJSNS16eEMxTUFId2lkRGs4bHJOQm01VTJlaEhHV1UyRExFRFpqOHE0MzNUeXdjRGR4NldfU2oxV1QtSG91TnIzMnllYQ?oc=5</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -3650,52 +3650,52 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K59" s="1" t="n">
-        <v>46083.58380787037</v>
+        <v>46083.61134259259</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Three teenagers arrested after garda pursuit on the M1 - kildare-nationalist.ie</t>
+          <t>Manifestazione davanti a Consolato Milano - Moked - il portale dell’ebraismo italiano</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Three teenagers arrested after garda pursuit on the M1 - kildare-nationalist.ie</t>
+          <t>Demonstration in front of the Milan Consulate - Moked - the portal of Italian Jewry</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 09:45:14 GMT</t>
+          <t>Mon, 02 Mar 2026 11:30:54 GMT</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPbFhwbFhtNi1aM3ZSSnpya1BaWkd4S0xzREpMUGNxaGJLY3BNdDJSeDhaM19DblVHUWs4MVhXQzllRzEta2ppUGlSbFVtcnR6NHBVWE1IV1B3SW4wSVFUYVlnRjhNNFFfdkc2Smp2M3g1SHd6NHJoQTVZRUszS2pkZVhmYWpSMjZZSXA0LVVSMEFwSHBjaGFxMDZ1MjM0SkhRSFBRRkdBQjAtOXF5NWlj?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxPMmRiTWFJbnVmVWFEc1A2THJBWi1DaEw0dk9fMHJXblRhaEVEN2p5REhpcF9ETkN0OGhVeExRN242clJRdGVFZmNiX3cwb2RvZWRtU3V2bzViZVVVT2g2QmJoZjk4aGo0cWYzdEJoOTNHeG82cEFIcVZDWGpsM0FvaXU4NXV4LTNQUWtYcXpweEU0T01NMmx3WE5mU1BFSnVIbkg5YmNxMUk0SE5wZUlLVWxxejBCaE0zOF9YMEJ4TmFjNjE2eUVLTFVFVjlsTzQ0TG82QWJJbDd2M3ZJdnljZlp0S3FqZTQ0LW1uV281MVNGXzk1dlQzQkZMOVUzVi1nZjNETnZXLTd6bDlFazhzbw?oc=5</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -3705,52 +3705,52 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K60" s="1" t="n">
-        <v>46083.40641203704</v>
+        <v>46083.47979166666</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>What the papers say: Monday's front pages - kildare-nationalist.ie</t>
+          <t>Iran, presidio sotto consolato Usa Milano: contestata manifestante pro Pal - Giornale Radio</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>What the papers say: Monday's front pages - kildare-nationalist.ie</t>
+          <t>Iran, garrison under US consulate Milan: pro-PAL protester challenged - Giornale Radio</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Mon, 02 Mar 2026 08:19:27 GMT</t>
+          <t>Mon, 02 Mar 2026 17:47:14 GMT</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxQYjJOckJJQk5WbHdvTG95UjFBX19JbDNnQkczN2dQZDFxbjVSekhnWmZsRS0wYlRUMGZkWUljWURoTkEzb0xxdFFlS25tVFRMQzMzQmZZM3MwM0tPMklKek83LWFUYjhnYncxZnFtbzhIN1lvWF9pY3ZHakdkTkxaaVU0VEZhUjYzZ2NDSUJyQTFneEgyV2xFU00zdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOMDJaQXp0UnJSb3RNcWVWWGNMQlptcXFsOTZyYU54OGI4alBDbDcxcDNTYlVFM3k1UC1ESVJTbWVldzJoM0lyeEpTODRmQ0lDSzlsZjJsUDEzZXBxYWxocUpGLUt4RnpqelBOazk1dGdRSXpJRy11VUY0OVpFdU9ndW1VRGUyRGZwZjh2bTljWlVnaWpfVklJM3JhRVNqRm0xdnB1NHVWaGp1UQ?oc=5</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3760,21 +3760,186 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K61" s="1" t="n">
-        <v>46083.34684027778</v>
+        <v>46083.74113425926</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Assalto al cantiere dopo lo sgombero. Bologna teatro di un’altra guerriglia - Il Resto del Carlino</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Attack on the construction site after the eviction. Bologna theater of another guerrilla war - Il Resto del Carlino</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Tue, 03 Mar 2026 04:03:34 GMT</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxQempFSTBVVU53akxMVGVUN05zM21kVmpmZkxzU1FhbVVVUUtOTnlIRl9mOXJHVk9NODVMU1JVMk5XcjJ4aHZIbHRJaWtCeHlJYVpnSk51RmdDSmhkdnVhd053S3p6RzlkaUIxal90VFZOYlIxd00zenBLcVJXLXFTMUYzNEhZY2M5T19YUjNB?oc=5</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K62" s="1" t="n">
+        <v>46084.16914351852</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Violenza contro le donne a Milano. Ogni giorno più di 7 chiedono aiuto. Dal 2019 i numeri sono raddoppiati - Il Giorno</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Violence against women in Milan. Every day more than 7 ask for help. Since 2019 the numbers have doubled - Il Giorno</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Tue, 03 Mar 2026 03:56:15 GMT</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE1yaWNuaWFhUnNLU3RaM185UEtGcWg1YlF2MDl1SnVvbWFrc0NzeS1GTWFVRk1jNTBVbW14bGJ4cGNFZUlmX3VvVU9maTRnc2FtSXpiX1pUc21HZ1VLX1FhcmppUGR2RjJEenp6SEJJNzJwUk92Y1ZnNWxjeWZJX0U?oc=5</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K63" s="1" t="n">
+        <v>46084.1640625</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Firenze, attivista iraniana contro il corteo di pacifisti. Il video - La Nazione</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Florence, Iranian activist against the pacifist march. The video - The Nation</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Mon, 02 Mar 2026 11:13:16 GMT</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxNWTJaNE1TSUVhYUU3bVhtOG52eXVaR0NZbEVIMTIxRkM3LVFreDVkY0dlNTBLc0JqRzNyMXpWNXpYSHg1ZFhLYjA5ZGJwRmR2XzIwbDBTVmNYbkFjZFVwVHhOZHpKQ0ZfVWE2WDBhYktTcVRwd0JDUzQwSWxQMTAzQ1I1QzlZUkhNV01pRC1DQTBXV2lJZk5aTnJFYjJTeFJVekFSVXg0Nzk?oc=5</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K64" s="1" t="n">
+        <v>46083.4675462963</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-03-05 07:51 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K44"/>
+  <dimension ref="A1:K61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,32 +480,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Scotch Corner Outlet Village targets £25.5m via stock market funding - Place Yorkshire</t>
+          <t>B&amp;M European Value Retail PLC Dividends – TRADEGATE:7Z5 - TradingView</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Scotch Corner Outlet Village targets £25.5m via stock market funding - Place Yorkshire</t>
+          <t>B&amp;M European Value Retail PLC Dividends – TRADEGATE:7Z5 - TradingView</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 11:05:00 GMT</t>
+          <t>Wed, 04 Mar 2026 21:03:18 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxQR2N3S2wwWnplWVd0aXVKcVl1bXFJODNTODZacEFHc1EwVGdNck4yanVhSUw4b3B0eHNMSExFZ190R1c1QkZIdlFZU25ZUm93bjI3UjNIaGd1TEtkZnprRmtPbTFQcEdWVjFrTWZkaU5QNEUwdUJPWDU1d240UThpMjFpX3pTU0xMZ0FXN3ctNkRTU1VVS3A0WlpxQjFzbk5iaE5V?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE1VQjM3bS1FRjZDT2VreDhXdVFNUXZxRmxuUWNvLUNqQXVLSjNQQXZ4TUlCUlNsbl8wcEI3VGpzLS15U1dXVUgxU2lVYVpYbkVraS1mSzNnWkg3TWp2Y0hyTUYwTVpFNTFZcW1fc0dYOVlfS2p5YXlBSllFUQ?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -529,38 +529,38 @@
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46085.46180555555</v>
+        <v>46085.87729166666</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Major update on new Yorkshire designer village packed with big names earmarked for 2027 opening - Yorkshire Live</t>
+          <t>Target’s 2026 Turnaround: Analysts Bullish as Growth Returns - TradingView</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Major update on new Yorkshire designer village packed with big names earmarked for 2027 opening - Yorkshire Live</t>
+          <t>Target’s 2026 Turnaround: Analysts Bullish as Growth Returns - TradingView</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 11:22:47 GMT</t>
+          <t>Wed, 04 Mar 2026 18:07:00 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQcXM3clpMbVJwQlg3VUxyNlc2RnVjRV91cElXVHpRS1IxREhsX1FldnI2dExXdXhkZ3NwRVVmanAtRzBxYmF4X1lFM2w3a0k1bmR2MHBsMm9Bd0tWTWlSaGlhX21iR19FZXBXREhmWUxGNl9YNFExQl9rUWFWdmxhX2FFVlNmclVQVnNNY2hZSHdLQ3ZBTFRZeGY4Y2x0b3PSAaQBQVVfeXFMTUJKVjQxdVNCakYzclJYMUt4aWFIYWVON2NidElPX1U0dHJoTHl4NzJFVld6WXAyY3JsY19vTzhaSXBSZmNPVVI0dVNnanRxVlFaaElDS2hoSTF6QnNUdHRWcHdHOUE2eWRfZk9vVktXZmZUR1dPMkE2a05fRW55OFV1eW5uUS15UzZLRGwzeW9jTFZxNS01YnFzWHNfa1gyN09idHg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQbUFBQml4UkZ5V0xEOGpVdFRlM2xXQmdTQUYxWjJubzVuTUptYzY4X2JKUExIT1Z1UEFablVjeHRKTzJqRE9TZUdqM244LW1SRy1JM0RFTG1RdG9nMGxVZ0l4VWZpMVpadFNkeF84dFlpZ1pNQnBxNGh0Vlo2eE9GOUVKWTFyWjhFZEUtMURjQjZkdkxodm1NdDUxWlkwakNzY2dKZnNBTVZfYTd3UEdLcUpRSXRqc09IVUZLRw?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46085.47415509259</v>
+        <v>46085.75486111111</v>
       </c>
     </row>
     <row r="4">
@@ -600,22 +600,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>“Our vision is to make perfectly imperfect hotels” Oberland co-founders - Boutique Hotelier</t>
+          <t>Global tech and beauty company opens store at Bicester Village - Oxford Mail</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>“Our vision is to make perfectly imperfect hotels” Oberland co-founders - Boutique Hotelier</t>
+          <t>Global tech and beauty company opens store at Bicester Village - Oxford Mail</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 09:40:46 GMT</t>
+          <t>Wed, 04 Mar 2026 15:28:20 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTFBjWFppNUg2TTJaQWVrRWwyWkU3MnBjN29EN1ZnaU5EUTF6bkpZZ3BHT3I3NV9aTEo1RVROWjFWT3AzaGgyZDA4X1lROVc0dHI3dnA1R05qdFRTUEEtOGRVV1V2eWktQUlMVWw1XzR6Z0p6RHY4dE0wSEFjUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNbUQxRXJaQW5HcGtKTklWc1ZDUU5hQjNDM1RfTVJ1V0ZWM09mV3dBcXVvd0xQdFlZQWJMNEkzcjJ1Wk9tNlBHTHVvMm41ODdpQVBNamgweldIbnVUbTVkVHczUnpLZ0NNOVEzZjZuRVJUTVFYbmkyb0pDUl8wNVV0Y2FIYUxmdnV3YVlQRUk2WHdOd0NrckE?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46085.40331018518</v>
+        <v>46085.64467592593</v>
       </c>
     </row>
     <row r="5">
@@ -655,22 +655,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>East West Rail scheme: A route to prosperity - Property Week</t>
+          <t>Dyson Opens Immersive Boutique At Bicester Village - 365retail.co.uk</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>East West Rail scheme: A route to prosperity - Property Week</t>
+          <t>Dyson Opens Immersive Boutique At Bicester Village - 365retail.co.uk</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 11:48:37 GMT</t>
+          <t>Wed, 04 Mar 2026 16:45:51 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxQbml3OVFpWmRDX2RqZGowaV9UYjlMLXpTbV9MMFZwMC0yempxd3JyUlZFODhOanNqZEpac3pZMGVtNTBGSDdoY1ljWTZWMHZmVXhVY1dxNTdhR1JQUjBSWm1OdzlXbXZUN3h0WG9sbDRXZExZMGVTU0ZRbUhlZHpkczIzR1phazg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQWmF6amVxcmxrSFRuQlpqVlB6eUZIc3EwWnJzeFV5LS0zcWxiNnRlSmwyY1RLSnV2VGVla0FPc3FILV82dTBsaDN1c0pMQXhIT1hWak92SjY4WmRWeV9KbkdHWjlGWEs3MlhxSG5BY2k5WUpHQjJKVDZfODhPMFg2Ng?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46085.49209490741</v>
+        <v>46085.69850694444</v>
       </c>
     </row>
     <row r="6">
@@ -710,22 +710,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>'I make between £800 and £2,000 a month on zero-hours contracts. There's no consistency' - AOL.com</t>
+          <t>Scotch Corner Outlet Village targets £25.5m via stock market funding - Place Yorkshire</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>'I make between £800 and £2,000 a month on zero-hours contracts. There's no consistency' - AOL.com</t>
+          <t>Scotch Corner Outlet Village targets £25.5m via stock market funding - Place Yorkshire</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 10:55:19 GMT</t>
+          <t>Wed, 04 Mar 2026 11:05:00 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE84UkdzeExGN2xLSUh5VnBiUlNFTkI1ZWl1bVo2RFVEeVUwdnZaSjNuS2hrOVhlam9pamJzUTRGRWZsOER6Y0hXRFpxTGs4bXZzdTZ4YXNxVlVaNXpCUTVuT3pHeXVlOHA5V3FLZHVUa3ZtYVV4aXNVUDZEek4?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxQR2N3S2wwWnplWVd0aXVKcVl1bXFJODNTODZacEFHc1EwVGdNck4yanVhSUw4b3B0eHNMSExFZ190R1c1QkZIdlFZU25ZUm93bjI3UjNIaGd1TEtkZnprRmtPbTFQcEdWVjFrTWZkaU5QNEUwdUJPWDU1d240UThpMjFpX3pTU0xMZ0FXN3ctNkRTU1VVS3A0WlpxQjFzbk5iaE5V?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -749,38 +749,38 @@
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46085.45508101852</v>
+        <v>46085.46180555555</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Schietpartij in restaurant in Zele - HLN</t>
+          <t>Major update on new Yorkshire designer village packed with big names earmarked for 2027 opening - Yorkshire Live</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Shooting in restaurant in Zele - HLN</t>
+          <t>Major update on new Yorkshire designer village packed with big names earmarked for 2027 opening - Yorkshire Live</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 10:50:34 GMT</t>
+          <t>Wed, 04 Mar 2026 11:24:00 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxQNFZaVVFnMVRvSjVGNXZZRVEtTE1OWmJObEI5dlZQdkdOa2tLUkJTVWVrdmd5ZHZFblRWdlBrRi1FbE0zTkFyWWNIbERSdmZ6MmREZUYzUmEyblVUa2gzQTBrS2M1cFRiMGpmSmxyV3Vqb3gtdFI0OVdqWno2UnE3Z01najNmdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQcXM3clpMbVJwQlg3VUxyNlc2RnVjRV91cElXVHpRS1IxREhsX1FldnI2dExXdXhkZ3NwRVVmanAtRzBxYmF4X1lFM2w3a0k1bmR2MHBsMm9Bd0tWTWlSaGlhX21iR19FZXBXREhmWUxGNl9YNFExQl9rUWFWdmxhX2FFVlNmclVQVnNNY2hZSHdLQ3ZBTFRZeGY4Y2x0b3PSAaQBQVVfeXFMTUJKVjQxdVNCakYzclJYMUt4aWFIYWVON2NidElPX1U0dHJoTHl4NzJFVld6WXAyY3JsY19vTzhaSXBSZmNPVVI0dVNnanRxVlFaaElDS2hoSTF6QnNUdHRWcHdHOUE2eWRfZk9vVktXZmZUR1dPMkE2a05fRW55OFV1eW5uUS15UzZLRGwzeW9jTFZxNS01YnFzWHNfa1gyN09idHg?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -790,52 +790,52 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46085.45178240741</v>
+        <v>46085.475</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Man probeert iPhone aan te kopen via valse bankapp en vlucht weg: “Bij zijn arrestatie 1 kg hasj gevonden” - Nieuwsblad</t>
+          <t>Death of university student to be investigated at inquest tomorrow - This Is Oxfordshire</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Man tries to purchase iPhone via fake banking app and flees: “1 kg of hashish found during his arrest” - Nieuwsblad</t>
+          <t>Death of university student to be investigated at inquest tomorrow - This Is Oxfordshire</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 14:14:07 GMT</t>
+          <t>Wed, 04 Mar 2026 16:30:00 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimwJBVV95cUxNVkUycDI4NVZMR1BEbDRxbTRxSkFKSmtPTTFmNEwySjdWLUhfOUJDMXBXLVFqdVBrVm9KNFl3MDRrOVh0akdWLUZtZjFWV1paRVB5Y043QlpQOGJuaHJzLVhiMDY3YzNxZW9YRER3ZEhWcXZlYnBQUE9jSWM3djIzT3V3Y0ltSXVsTWsxVVdtRUxpbG9FWVhUM0JRVkhCeXUzWUh4a0hJT05rV1AwcjhvTGoyQURRSjF3ZVBWRFdsQnp2dGE4cy1PSFdyZFo4bmRoVENveWNhU0ZwazQySXpieW1SeXJWNUIyWVN6RGdqUUVnclU5WVJQS0Framt2WnkydXU3dWJBd3BwSGEya21QZVBVc0VUNkwtWGdz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxNNkZZMGhfMG1xcEdCYjFRemJDSFhiUHYyOWk3UXB2eFZQZFF4TmtoWUhXRF9QZ1U3d01ELWJUd2VMRUhoWlhtX0hIUElLQUprNjFTSVJnYlNLTGZiVGhwS1VCcGwzM0I3WFhnRkpqSGlCVTRLRW1GUmZfS1Z1cF9IVDM1QlYwcndQVUpiby1rRXFWWU0tQVpsXw?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -845,52 +845,52 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46085.59313657408</v>
+        <v>46085.6875</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Ex-partner van slachtoffer Grote Markt opgepakt op verdenking van moord - GVA</t>
+          <t>Trains to London Marylebone to be cancelled for weekend - Oxford Mail</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Ex-partner of Grote Markt victim arrested on suspicion of murder - GVA</t>
+          <t>Trains to London Marylebone to be cancelled for weekend - Oxford Mail</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 13:09:50 GMT</t>
+          <t>Wed, 04 Mar 2026 16:59:31 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPblgyQ3R2S3VTZkY3X05lVTBvQlRSNWttdkNtSHNHSUdjT0N6MXlsRXFQRXRwRjFjNEk1TlhNa3dvc2xnWTlnZVBYdXB3ZzlWYV9acG5tTTdlWUNDclRVdFQ0N0sybHRDN01QN3dHQnFWSG5FelZnT2hlcDQ5R1laUTJZQ1ItN01mV180Rlg0Yk1fQWEtLXFLQm5wUDVCUTRDbFV5MC0zVjZfMjNjSldobw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxObGl0YWltVEdDdWVwTC1TQmRaWUhva0ZxdXNzc3FYc3NOcGZoNDZOWFM5MW94U3YzemVDVkxMUzJNa0o4OE42Z2ViLUJuYmN0WHlWd1pyQ3NLNGRXUWFYZFRNRDZ1aG5EUHBVTjJKVUNLUkNoOFJZLV83TVE5elhteThDdUtfRGVicjVZVENvSQ?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -900,21 +900,21 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46085.54849537037</v>
+        <v>46085.70799768518</v>
       </c>
     </row>
     <row r="10">
@@ -930,22 +930,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>“Dit nieuws schrikt ondernemers af”: bezorgde Unizo-voorzitter nadat criminelen schoten lossen op bedrijventerrein - Nieuwsblad</t>
+          <t>“Precies een aflevering van de Kardashians”: ruzie tussen drie vrouwen mondt uit in explosie in Deurne - Nieuwsblad</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>“This news scares entrepreneurs”: concerned Unizo chairman after criminals fire shots on business park - Nieuwsblad</t>
+          <t>“Exactly an episode of the Kardashians”: argument between three women results in explosion in Deurne - Nieuwsblad</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 10:37:23 GMT</t>
+          <t>Thu, 05 Mar 2026 00:15:49 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxPZGNOQTRyWVRtbmF6T05zTmYtS3ZIU0FSaVI5Q1drcFBXVFhqVkJ5UjFGcnVldUlBQ1ZzZkJXVTZWUEpiWXFTZ3B5S3FESklhcW95Q1o3ekZBemhERFMwVi10a3NoZG9jWFNQUVFIRGw3Mms3TGZKdndvaU1ZZDJpUzdVTW00YlFSc01RLUFWTkVWVXMzc05mTUJfU1JQQTRiMm8xd0NzMWZTZWVZbnlMTWtObFpzR0ZqWktDOWNYMHFDY21NeV9OTGJuNG94VkhNNXVjelhRTmRUblY4UXoyWUZGM3hLMlJ6UHJpYklXVl9KODRnRmxCaFNJc3prWjZTTE4taA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijwJBVV95cUxPWmFQQ0JGMmNKR2E2cVhYY0VFcFdydGZJVkV5cWR4cDZQZFFhb3FVQXdqWUJuaHVGYWs5ZGN2WWxISmpoNzNUZW1ZdUU1T2hZbm5xdXh1MXZ0TjJZUzRxVzFpRG16TVNIUEdNR2lMUVN2U1VLU2lFbWUzaDZDMG9rLUNfZzFGZGhzT0xzbTJyVmU1UHVKOTVCTUpjVFNpeEpXclVsbEhaemk1aDl0Umhsb1g2R01zMWtoNmpmWExCWm9naElSYjFyQ0pMdGlheVFvYW9VWXc1S25RZnlNV1hNOVFqVHFDMlY4OFFYaHlQM1NfZENOQUtBRHd0eHJhVEsxM0pvNWVGbVA0dy1fOWRJ?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -969,38 +969,38 @@
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46085.44262731481</v>
+        <v>46086.0109837963</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>As Israelis and Palestinians, We Shall Go Together to Brussels – Le Taurillon - treffpunkteuropa.de</t>
+          <t>“Financieel kan dit erger worden dan corona”: reisbureaus vrezen zware verliezen door oorlog Midden-Oosten - GVA</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>As Israelis and Palestinians, We Shall Go Together to Brussels – Le Taurillon - treffpunkteuropa.de</t>
+          <t>“Financially this could be worse than corona”: travel agencies fear heavy losses due to war in the Middle East - GVA</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 13:04:46 GMT</t>
+          <t>Thu, 05 Mar 2026 03:00:00 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQamJub2NMM2dvT1JKYkl5bUNOa2stb0tBb0FCZ1AxN3BLV3NFcHdaQW1takY2cld6V2RVeUNyNVFvNDNFZ3VkVGRWblBDNktqdU5UY2E4YnVyYmpsN0x6dE1QZGxWOXpWc3NFc21nejlsRnNKWWFoQTI5RnhkMU1GRTRPbmt4RzdUU2w4QVM5YWNkNWh6Tlo4cA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgJBVV95cUxQcDBqdzRrRkU0N245czVaVFZBV2RxVzJhX2FXRGRKN0c2Q1I1bDhHUHJSaHluMEYtWnJXa1NvUURTRGVDMlNQdHNST1dfeHJlZGNBbHJ2R2c0RW5WVFdwaUJaTktCRm1UY0RuLWdzcHZvU2hFU2ZFNmlrYzlHbWkzNjF5cGI5UWZoVllOZDVxc1ozUE0xbHdXbUxjTVZHcWxrUk8tbFlEZEpnaDlNeTN6VUI4Y0p6VmhCcllCSUZnSTZNTjlfemZJZHV4MnEycUdJeTdTQkEtTHlBT29TeWlvZVlNdDZFZUM1UjhJeTZXaTFhYkRsQkdzSnhDZ1NCSEswb2p5ZWhka2ZnaUhfN09YNm5zbTctd0hQcVE?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1020,42 +1020,42 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46085.54497685185</v>
+        <v>46086.125</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>The Iran war will be long, bloody, and ruinous - Brussels Signal</t>
+          <t>Schietpartij in restaurant in Zele - HLN</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>The Iran war will be long, bloody, and ruinous - Brussels Signal</t>
+          <t>Shooting in restaurant in Zele - HLN</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 08:20:35 GMT</t>
+          <t>Wed, 04 Mar 2026 10:50:34 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxPYnI4Z0dJSXREZkUwZGdCT00yZFpjM1VOQ2xLVTNQR1lmUTZ5ajNUZldiUUZfUnF5STMySzVSOXp1bTdpLTl5djFfOHNiNk5NWVB1TUpiSHBrakR2UW9yeWZtc1JlWlhjejR4NDUtc1EySnlhVHBNVk1rdmZYZ1lIamZybkw5QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxQNFZaVVFnMVRvSjVGNXZZRVEtTE1OWmJObEI5dlZQdkdOa2tLUkJTVWVrdmd5ZHZFblRWdlBrRi1FbE0zTkFyWWNIbERSdmZ6MmREZUYzUmEyblVUa2gzQTBrS2M1cFRiMGpmSmxyV3Vqb3gtdFI0OVdqWno2UnE3Z01najNmdw?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1075,42 +1075,42 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46085.34762731481</v>
+        <v>46085.45178240741</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>UK catamaran company to offer wind-powered crossings to France in 2026 - Travel Tomorrow</t>
+          <t>“Je zult branden”: vrouw zou brandbom gegooid hebben naar voordeur van vriendin nadat vriendschap verzuurt - pzc.nl</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>UK catamaran company to offer wind-powered crossings to France in 2026 - Travel Tomorrow</t>
+          <t>“You will burn”: woman allegedly threw a firebomb at girlfriend's front door after friendship turns sour - pzc.nl</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 10:08:42 GMT</t>
+          <t>Wed, 04 Mar 2026 18:19:00 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPRndSQjBkbER5Y2Q3MXRDT3U4TXF5cFpocmk4bFYyQ2VESnl6bWhmMFJzOWtSUFk5T0pJb1NkNXhSUGtTS1hqM0lNQkFaNF90QlB3LWdCNzdyV2RtTDdjNGZTbVZHSmFSaVFlYjNCT21FWmV1NFJyeTVSdDJXMVc2V3Z6VC0wMVB0QlBGdThtVWZDRlNRNHdDTEM1R1plX00?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8wFBVV95cUxPWjFVV0pOTGZJTHprbXc5WDBrSVpoR1RDUHhrSG9ZQm94emo1ckh4XzRIemVyVjBSaXVPU3BrOHFLcEpTRmViV3NKd2RQOGtReHFGOUNUbV9HNE03VWVnRWtzZXV4Nlo5ZUNuMVVLVTVtVWY0TmhtN25CSENMa2dNYXVpRGlrU0FkdEZmSFBqWHQwTnlZS0NoR3JTOW1HTnBlZkxiSWdIdkVnelJCRjk1WEx3YnJsVUgxZDNvazM0ZWxKa0ZaeGJGMFBQbk1JSTF0OTZaUmF1VmZ2MWRTYzlobHJreHVWYkFUemJiOFdtbEZWek0?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1130,42 +1130,42 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46085.42270833333</v>
+        <v>46085.76319444444</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Pakistan confirms airspace fully open amid fake news reports - Travel Tomorrow</t>
+          <t>Is gedwongen hulpverlening hét redmiddel voor De Coninckplein? “Dit mag geen openbare-ordemaatregel worden” - Nieuwsblad</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Pakistan confirms airspace fully open amid fake news reports - Travel Tomorrow</t>
+          <t>Is forced assistance the solution for De Coninckplein? “This should not become a public order measure” - Nieuwsblad</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 09:43:42 GMT</t>
+          <t>Thu, 05 Mar 2026 01:08:26 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxNcDV5Nng5NkR0d2dBLThJRi1pYXZvTDRRNG45SW9sSkwyUGtOYUJCd0tNRGlBZmE5WFVNcDhyT0ZSbzBBWGR2cHFORHJZbUx1R0daSUNUc0hKTFJ6bVFITmFIbkNVWHdvdXJzel9BV3ZaUVVkMExwaEl2dTJTdHA1c1ZyQWtCaThKVF9sdGRzS2FnZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgJBVV95cUxOSDNiUjMyZzU5Z1hpaXVpSnF2TVBzeWd3ejdvVnRYeC12UzVhR3dVSlZabTNXRzNKUTA1Q3pHM0p3bU1wLVJ5VnE0Z01halYwMHMyaWZLTXhJVlluVFdfYlA1LWVrc1VPaDhiMElnTllQNTg1WUhKdDlnZ0FWUWZZbG5kV2J3R1F4emI4eUpnV2RKdUIzdkhlMzVpZUpZckFWUXRmclR6UC1RQnZFR2dzazFDRnJYTXFpSV9EaHhteHdvMUZWcUs3NmtMUGhOeFZGcHlmbVQzWTBSVDRpLTQ4QUtqWkpkNUZqNlFLLXM4UzZteGNsQ2JtejMzWWtCemtsZGxTNUV6b1pmNUZ5cVFYOVJIS3N1UQ?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1185,42 +1185,42 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46085.40534722222</v>
+        <v>46086.04752314815</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2 twintigers krijgen werkstraffen voor tientallen graffititags in Hasselt - VRT</t>
+          <t>Stoomaccumulator geplaatst bij Sappi Maastricht - De Limburger</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2 people in their twenties receive community service for dozens of graffiti tags in Hasselt - VRT</t>
+          <t>Steam accumulator installed at Sappi Maastricht - De Limburger</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 13:31:44 GMT</t>
+          <t>Wed, 04 Mar 2026 16:16:46 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxQNXc5M1hIZG1lamVwVzlxLXhzTl9LMFRfXzlCdzgzV293ZXVWRnRaTHk2VGdqQ25fT2YyazdjY3prUDRYcFAzYkZFQ0VxYmhEejlVTmg4eDJfQ0hrWmpUV29Wc3JqdmFCWEZNUk1PblBVaWJ4cEQ4N1hjbVF4SHBLdGJDR1ZQdmVpaHdRWEtGOXp6VmJxRlRTV29VaUpLSlZhT2ptakxIVjY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxQaTJidDdUdmx2eDdUbGhBZEZxNEx0X3NIeGp5S3Z6OXhmUUlFbm42ZkZRTE1zY0h0YXJ2ZXNua1hLUmZvcFhMNmVDY2l3LTNfUTFRbi1oR0hkTTNrVVRTcmo5aWtNcl9Pck45TTRzTkxZOFBKY0VyZE4tbEFDWnFzRWVYb19hMEtmLW40UUNuQU5EdWtEamFEcFpfcFUxbnJR?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1244,38 +1244,38 @@
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46085.5637037037</v>
+        <v>46085.67831018518</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Une grande première: la Coupe du monde de cyclocross va faire escale en Écosse - 7sur7.be</t>
+          <t>Man probeert iPhone aan te kopen via valse bankapp en vlucht weg: “Bij zijn arrestatie 1 kg hasj gevonden” - GVA</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>A great first: the Cyclocross World Cup will stop in Scotland - 7sur7.be</t>
+          <t>Man tries to purchase iPhone via fake banking app and flees: “1 kg of hashish found during his arrest” - GVA</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 10:15:00 GMT</t>
+          <t>Wed, 04 Mar 2026 14:13:58 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQV2I0NHFLMHZJTmdoR0ZjSkxId213ZlVqTzBLSWJTRDJTV2FtWl9pdm1IWjJSZ0ppODhESlVfRlhTdXEtY0IyWVU0NTlRUDU0WTRJSjZRb1VxY2tXa2RDNDJNempQa1NwTW02Q2kzNHBOb2tIcE5yd2ptMXRUUXNLUUlOWEtCTHlwLW0wT2p4OE1yTDdlWUFVbjNHdEZHaUlRM3BaSEVJZWUwMmZQdEkzYTJCQVpSRjlm?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgJBVV95cUxPeF8xcy0wTDFyQU5FTFJMdGRzQ2JMMFdrUEdJMDhQczg2SzNJeTBGVlpjeVFyWEd4UFQ4S2g0SmZNeDhacXBZOVJ4Y0I4bmJtQ0MwSEM2U1dyejIxY3c4cHh4QTRwZ3FpdFp4cDQ1NG1keGhTb0JlQWd5VmswdGJYVHlrejFGdmpRNzFHVVZWMkUtRm9fSXhMalRhZlN4N19FZUZkTnd6dUxsWVZkZlFzVUJoYURpekNyd1k1U05tbTVRMGtPMTFmYmVncVdEenlnMmFPSXoxMEkwaldXTkNVQ2xDNzNGWkU4V2c2TGh0TnBRcjJNZTFlRDJiRnpodmFKY2JFT0RPaTktcHZIUC0zNzlR?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1295,42 +1295,42 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46085.42708333334</v>
+        <v>46085.59303240741</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>The best of both worlds at KPMG Accountancy Hasselt - KPMG</t>
+          <t>Ex-partner van slachtoffer Grote Markt opgepakt op verdenking van moord - Nieuwsblad</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>The best of both worlds at KPMG Accountancy Hasselt - KPMG</t>
+          <t>Ex-partner of Grote Markt victim arrested on suspicion of murder - Nieuwsblad</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 09:33:41 GMT</t>
+          <t>Wed, 04 Mar 2026 13:05:15 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPSHFXOC1teDYxSmhWNzFrdE9tbVU4SzBqcFliY0NaRURpRjNoUE5Fb19HcDQ1WGt2YVVfS2k1bHM2VU9ta2d6VzVOemtuSmdiRGI3Z3l6OS1lTV9CemNrRTVqRXNULXUzS1NScm1paVp5N3RvbFVaUEJ0UG93XzJDY1ViWmxZdDNxVDlFNUxiTjRLcTF4a1ZmU2VPcHNxSEpPdHcyM3VGRlA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxOaEN2ek9pbmVQdzRUcm9jN3dob1dvV2JGa3VXbnhXdFU4WHJrcEZYU0l2c29nLTRpZ01TMUdQODJ0aDExblJKMnhUUDlZVEdEdGZRaWVfVnY5TUZCM241cllRUDViU3hsUXFkV0VXU2s5c1VkRnZZOE5XWEZscDVxeFpyVHpUbEpfUE5XemRjbTJUcDExV2FIS0ZjWU5kMFdkUXdqbGxRQmFzMjdKRlkxWUQtSUhybEFZZ0xXbnhYR01SLUwyLVR3T1l6NS1wYzZnbi1MY1Q2YlpUOXBJamlUVzlENkNPdVNoR1E?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1340,52 +1340,52 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46085.3983912037</v>
+        <v>46085.5453125</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Brendlorenzen: 17-Jähriger liefert sich Verfolgungsjagd mit der Polizei - Charivari Würzburg</t>
+          <t>Twee minderjarigen plegen gewapende overval in nachtwinkel Ekeren - Nieuwsblad</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Brendlorenzen: 17-year-old chases police - Charivari Würzburg</t>
+          <t>Two minors commit armed robbery in Ekeren night shop - Nieuwsblad</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 14:00:00 GMT</t>
+          <t>Wed, 04 Mar 2026 15:00:58 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxOMlByX0xhT2xSOEZLTWpXczBQVnlCVWZ1T0ZacGJ6Wm15Z3AxS250RVZBVHczVDkxNTBtQmJDZ1V5MTVNc1N3MDlZWmpUSFRGQmZyckM1SEZ4TkRQbXBybHhqUG5fcDI1QVFnZ1dmckRPNWpiU3A3OXQyV1UtLWxBaFZLQ1dyWjRjMHdHbE5RSlFSU3dQcjF3RnJZeHF3RkUxc1FnOEQxbzV3RjJ4?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxQNDNJOVhkVUVVWHJZYjdDcmtzeDBtWXRSMTR0N3RMOHdXbV90bGd1dnN1dENhYzBZX0hTS3VjN1ZkU2xFcjBZa0ttUDFPMUNLOWY5V1BTc3ZEMXhwaVA1R0JwMzFDa3N4VTVYdHFuWUxNWWRNcWRManNLbmItTUJtUDcyR3ZjMnNkQXlJRkxfMjdmMU5WQU4yVUtyRHgtdVQyeElSTGNFVlVhTkIzRXhEdFRfMDNVbWxKd1BkVTYyYndPU0V6Rmx2di1HT0RfN2JueERwcTg4NF9UemJzSnlxNGF3?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1395,52 +1395,52 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46085.58333333334</v>
+        <v>46085.62567129629</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Kitzingen: Herrenlose nasse Tüte und drei Unbekannte beschäftigen Polizei - Radio Gong Würzburg</t>
+          <t>“Dit nieuws schrikt ondernemers af”: bezorgde Unizo-voorzitter nadat criminelen schoten lossen op bedrijventerrein - Nieuwsblad</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Kitzingen: Abandoned wet bag and three unknown people employ the police - Radio Gong Würzburg</t>
+          <t>“This news scares entrepreneurs”: concerned Unizo chairman after criminals fire shots on business park - Nieuwsblad</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 13:15:00 GMT</t>
+          <t>Wed, 04 Mar 2026 10:37:23 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPay1CSjA4VWZzbnZsRjhMZXVram52bGlHeWY3ZUJ0NjhGc19HMWlYNFFWVnNTcEc5X0NvbWtNVGQ5dTBBQWN4WnVZb09lbHY1QzhrSTNmWWtrUzFIZDBNY01fM0ZCR1VtWVRlQVFLWGNBWExlQTJITkQxNzg0T3ZkQXFSZXNhaGt0TXVZYlg5Ymp1X2FpeWoxNnRjNlFJRXJQVWQwdDF2dDJPMDFk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxPZGNOQTRyWVRtbmF6T05zTmYtS3ZIU0FSaVI5Q1drcFBXVFhqVkJ5UjFGcnVldUlBQ1ZzZkJXVTZWUEpiWXFTZ3B5S3FESklhcW95Q1o3ekZBemhERFMwVi10a3NoZG9jWFNQUVFIRGw3Mms3TGZKdndvaU1ZZDJpUzdVTW00YlFSc01RLUFWTkVWVXMzc05mTUJfU1JQQTRiMm8xd0NzMWZTZWVZbnlMTWtObFpzR0ZqWktDOWNYMHFDY21NeV9OTGJuNG94VkhNNXVjelhRTmRUblY4UXoyWUZGM3hLMlJ6UHJpYklXVl9KODRnRmxCaFNJc3prWjZTTE4taA?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1450,52 +1450,52 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46085.55208333334</v>
+        <v>46085.44262731481</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Würzburg: 20-Jährige springt in Würzburg ihrer Tasche hinterher in den Main – dann wird die Strömung zu stark - Main-Post</t>
+          <t>Mysterieuze doeken en luifel schermen vliegveld Beek af: wat is er aan de hand? - De Limburger</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Würzburg: 20-year-old jumps into the Main in Würzburg after her bag - then the current becomes too strong - Main-Post</t>
+          <t>Mysterious cloths and awning shield Beek Airport: what's going on? - The Limburger</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 08:40:27 GMT</t>
+          <t>Wed, 04 Mar 2026 17:30:00 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwJBVV95cUxPcm5yQ1ZsbXpfaGUxU1lKcnp1bjJLRG1QTk05eU5PbEZEV216dFBQaFU3Vk5nVlZjLUpLRjVmSGFZQVlkeVlTaUJic0N6elZ0dWJ6SDR3RE5CbjZiYngwcUZKVU1NTW8yQjcyaWtUMXRYT3ktSF9kbjNnQ3RtRzFhMnBQdWMyS002WjhWaXNXVTMtRktSUzdsODRBYVFKSDNXWUh4Zk9oOUdDdHJFekpfN19hZ3RJMUR3dGhubU93TW5PeUNWdFRFUTBLS2I4aHpiOHFrTkZuUkhQYXdDMmhSMkYzRFd4T25iN3cxWXFDNEpXR0RBVzBYbG9FY1JuWEhFREdOUEJXZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxNbGEzQ1lTZENLQVJsb3dWbjhhdWZfUnZ6OWp1ZHY1MlhiVkM2TXMxM05TSzNjbDdfSkNONXNCMk5vakhjU21tLXVRWGoyd0tzcUotZDlTejBBWVZtdWpzWlNkaGdpQ096eXNVcjVaRzI5U1IyNE9BLVVpcDZEYXlwNlpHUUY5RDhBZ3E4V0pyLUlaN1BuUjRIZHFYb0NNQmt4Z2ZWSFJBVXdnaWxjV2MwUHdReFpkQnJaSGpLbWR3cEtKWFVHVUVR?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1505,52 +1505,52 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46085.36142361111</v>
+        <v>46085.72916666666</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Polizeibericht: Krommenthal | 13-Jährige vermisst - Wer kann Hinweise geben? - meine-news.de</t>
+          <t>“Dit waait niet over”: Sarah Ferguson vreest definitief einde van koninklijk leven na arrestatie Andrew - HLN</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Police report: Krommenthal | 13-year-old missing - who can provide information? - my-news.de</t>
+          <t>“This will not blow over”: Sarah Ferguson fears definitive end to royal life after Andrew arrest - HLN</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 13:44:53 GMT</t>
+          <t>Wed, 04 Mar 2026 19:03:10 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxPSGt1eXRTbXRLNE1SZnJnYUJHNHFpa2NSV25oWE4tQ1EyYmh4N0lCX1NicDFVSTcxdDBNVEZPQVRYUm9LQUZZcjdoODlqQjd1VkI0LWRNSkgzOVhRaDBHUXYwUTBMYnZtTm12dWw5SWVCSmlBNVdJbV9BRnAzVXY5d1Mwa3FDQW5SdjJUSXBUSGZLeUp5Mlpaa1FjQlJWdUZlN1pXVGZjekhGQzRNSFY2RVJoTjY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxQLWhMNGltQ2szaHRuTjJINDBseGM3TEdxNkxoUUhKV05vc0RPWXlQeDJXQm85a1dZX1Zxd0tvQ0NuVVdfRmxmN09kSDNKd0tFMTBFaG1lMGo2SHZVXzhZaVl2aTh0b0V2ZU1UblE0Y0lQaVk4ZXExNTYtQ05qTFY3SkNjT0pCUWFzN01EOFpoM3RFLWxpemM2QVdmODRmMUd0SEx6dVN1SGpKdEJYbjM4QllqaVFJVlhNSXhQVklIQTc5MVJVNHNqX1JULXhiRTFROXlF?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1560,52 +1560,52 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46085.57283564815</v>
+        <v>46085.79386574074</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Hundebiss und mehrere Sachbeschädigungen in Würzburg - SW1.News</t>
+          <t>Geen vluchten vanaf Brussels Airport op 12 maart door nationale staking - De Limburger</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Dog bite and multiple property damage in Würzburg - SW1.News</t>
+          <t>No flights from Brussels Airport on March 12 due to national strike - De Limburger</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 12:35:01 GMT</t>
+          <t>Wed, 04 Mar 2026 16:23:46 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxObndrOEIwTm5pWjU4b25EaHRKRThqRGU1WUFTdldNa0UzQ043ZGEySnFnX0JYVkppSDlSbEc2Zkp4RWhuQmg5SDk1Y2NQOW91YnM2NjJRTXpFNDd2LVM3RU9kVGhYVUEtSjA5Ml85UGYzTXZHblh5V0UwRmJNRFBPN2lsNWtmT0QzQmt3SzRNVFBFa0w3SXRB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxNMklHakQ2VFVmM2JCVDhJRlVfWFRkeTNKN0VNSVkxN0Q5TGh5azVOUXVleHZ2dHNOM3R6VUFUUlhTRVBUSUI2bVJiTHdLNjI1cmJ5MnYzWHdtMG1HaXc3ajRQM0NEQThwTmVfWWVsNWVpdWswN1pLNnNHZEhfN0ZwQVJHVG5JLXN2VWphODBJbjE1VVg2NHJfLVJzbm01a2JHa0dyVDBCSms3R1l5bEZUVmJWdzRmcG5qM1FiNw?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1615,52 +1615,52 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46085.52431712963</v>
+        <v>46085.6831712963</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Wiesthal: 13-Jährige vermisst - Radio Gong Würzburg</t>
+          <t>As Israelis and Palestinians, We Shall Go Together to Brussels – Le Taurillon - treffpunkteuropa.de</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Wiesthal: 13-year-old missing - Radio Gong Würzburg</t>
+          <t>As Israelis and Palestinians, We Shall Go Together to Brussels – Le Taurillon - treffpunkteuropa.de</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 14:10:00 GMT</t>
+          <t>Wed, 04 Mar 2026 13:04:46 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE9QWEtqdUh5RG9WRjQ1OFFtR0FtTC1lUlhSaXl1Uk5fdUVtWW1RN0VOY2c5ckxIZTdoNWYxNmVxRGZJTEQxd2lLdzRkZ1AtMmVSSHpia3NqSWNtNTktLVFQVFZ0U0NVWWZpcHJuQXRua3E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQamJub2NMM2dvT1JKYkl5bUNOa2stb0tBb0FCZ1AxN3BLV3NFcHdaQW1takY2cld6V2RVeUNyNVFvNDNFZ3VkVGRWblBDNktqdU5UY2E4YnVyYmpsN0x6dE1QZGxWOXpWc3NFc21nejlsRnNKWWFoQTI5RnhkMU1GRTRPbmt4RzdUU2w4QVM5YWNkNWh6Tlo4cA?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1670,52 +1670,52 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46085.59027777778</v>
+        <v>46085.54497685185</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Polizeibericht: Heimbuchenthal | Navigationsgerät sowie eine Dashcam entwendet - meine-news.de</t>
+          <t>The Iran war will be long, bloody, and ruinous - Brussels Signal</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Police report: Heimbuchenthal | Navigation device and a dashcam stolen - meine-news.de</t>
+          <t>The Iran war will be long, bloody, and ruinous - Brussels Signal</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 10:48:36 GMT</t>
+          <t>Wed, 04 Mar 2026 08:20:35 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxOeC12WEU5ZjFwOWhJT18xck40MWZvNnU3bElqYlhJbkJ4X21pMDV6bk9udkgwUFdiT3dmdE9qNnlkM0ZNQm1iQVF3NlcxRm0tRXJsM015SUJiRE1yTzFMdFRuVUpLSVZKM3RMZFlZOC1uMWNWUUU0Q2FNUjNNSGoyeG1SUTQyNkhvUldFU1ZxTjE2Vm5VdlY3U3k0dXBsX2VqLXZiaGxRaWpINm9DUjdOUDd5QUlMOVZ0NVBtakpKaw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxPYnI4Z0dJSXREZkUwZGdCT00yZFpjM1VOQ2xLVTNQR1lmUTZ5ajNUZldiUUZfUnF5STMySzVSOXp1bTdpLTl5djFfOHNiNk5NWVB1TUpiSHBrakR2UW9yeWZtc1JlWlhjejR4NDUtc1EySnlhVHBNVk1rdmZYZ1lIamZybkw5QQ?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1725,52 +1725,52 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46085.45041666667</v>
+        <v>46085.34762731481</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Diebstahl vom Firmenhof einer Kitzinger Werkstatt: Wer hat von einem Mercedes alle vier Reifen abmontiert und entwendet? - Mainfranken News</t>
+          <t>UK counter-terror police ‘arrest partner of Labour MP on suspicion of spying for China’, reports say - Brussels Signal</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Theft from the yard of a Kitzingen workshop: Who removed and stole all four tires from a Mercedes? - Mainfranken News</t>
+          <t>UK counter-terror police ‘arrest partner of Labour MP on suspicion of spying for China’, reports say - Brussels Signal</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 11:01:00 GMT</t>
+          <t>Wed, 04 Mar 2026 14:41:25 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxNUUlvdXEzcmJoV3pwdXM5NXJGdWd4S1Vod05IUXdmcmlvVDBMUmpPaDQwRHQ1akpXWXNfdHNnRlB0UU9DT01mYUtXTjdROFdVWXBvQzJxUzQ1X2g1UnlxdjNtR3g3ME83Q01mZGdXT1lJUTJCcmtFVXVuSVZXOElVaU1ZRWNaZ3JFbjhwU0NDeHlPUjJDNHR0d1IwaXFLU1c0a0tNZHp0Uk9tOXJSUFpLQ3VlaE5nQWxkclIzYl90dzd4NkdUdGowMHBvV3lxaktlcklNU3dZem1yUXYteEFXaEtVam1hS1d6SEJj?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQQWVld3B5OENWME1yUTlCQ21OS0lUY2JOY0tkWmdOMmg1T2QzcjIxcGpWdzdYeHgtT2thUGV6VHJMdGNQaHRwNlBjRDRISlB3bkc0RGk3N3VlMzVob1FtQkFpblRsTVd1ZG9tNE1YcWlzRVAxRjVxSWVFS180SWNVT29VWUFVSHpqdV9VblpOVV9ndGwySDB0VjhMdUl5ZURvS2tlOGhFeU9PMnFIRzB0OWdVOHZscTVmdHk4YVgyYUdzQVhHeFFIZGhZRVI?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1780,52 +1780,52 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46085.45902777778</v>
+        <v>46085.61209490741</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Mainfranken: Mehrere Fahrten unter Alkohol- und Drogeneinfluss - Charivari Würzburg</t>
+          <t>Pakistan confirms airspace fully open amid fake news reports - Travel Tomorrow</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Mainfranken: Several trips under the influence of alcohol and drugs - Charivari Würzburg</t>
+          <t>Pakistan confirms airspace fully open amid fake news reports - Travel Tomorrow</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 13:30:00 GMT</t>
+          <t>Wed, 04 Mar 2026 09:43:42 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxNQ0JlWndGZThFV05fbmpFMFl0emdISk4tb2NxLU8teVFFN2RCQl8xRGxKbzJ3Wm9JUnhUSlNQMmFjbEt0RVZkWGNZWEJVcGVYaTdaLW9iZjZaaEphS1U1dl9YVnVkOVFtN1o1dnlwanRDWk1BUHpkOWpZMmxMOWlic094OS1lWXd2ellTNDhLN1FCaHhUdUR4OUVfM2NKQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxNcDV5Nng5NkR0d2dBLThJRi1pYXZvTDRRNG45SW9sSkwyUGtOYUJCd0tNRGlBZmE5WFVNcDhyT0ZSbzBBWGR2cHFORHJZbUx1R0daSUNUc0hKTFJ6bVFITmFIbkNVWHdvdXJzel9BV3ZaUVVkMExwaEl2dTJTdHA1c1ZyQWtCaThKVF9sdGRzS2FnZw?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1835,52 +1835,52 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46085.5625</v>
+        <v>46085.40534722222</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Polizei stoppt Fahrer in Mainfranken: Verdacht auf Drogenkonsum - Fränkische Nachrichten</t>
+          <t>2 twintigers krijgen werkstraffen voor tientallen graffititags in Hasselt - VRT</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Police stop driver in Mainfranken: suspected drug use - Fränkische Nachrichten</t>
+          <t>2 people in their twenties receive community service for dozens of graffiti tags in Hasselt - VRT</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 10:14:00 GMT</t>
+          <t>Wed, 04 Mar 2026 13:31:44 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxQamMxVW9weWRHZUlYMXhucTBuT3JTR2NxN3otOGZ3di1CUHNpUkxIQmF1UmdSSG94TXhYUVl5dnFwX0xzX0R0Mmx6V3J3dUNyTjRhVXZTamI4WHpWeWRmY1NLbF9fM1pzRk1hbU9CQ0VPZk5hamRQb1NSeGEyQWRTdDk1dXZXMXVLUS00d3FFdFNiY3BXMThFbnRfNURubVlEMkdUeVBkTW5YSDFtRjB2UzB4S2praEpPUGE3Q2tsWTRSU2RuRzV4S0tFZEIxWEVRWWRUMTFB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxQNXc5M1hIZG1lamVwVzlxLXhzTl9LMFRfXzlCdzgzV293ZXVWRnRaTHk2VGdqQ25fT2YyazdjY3prUDRYcFAzYkZFQ0VxYmhEejlVTmg4eDJfQ0hrWmpUV29Wc3JqdmFCWEZNUk1PblBVaWJ4cEQ4N1hjbVF4SHBLdGJDR1ZQdmVpaHdRWEtGOXp6VmJxRlRTV29VaUpLSlZhT2ptakxIVjY?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1890,52 +1890,52 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46085.42638888889</v>
+        <v>46085.5637037037</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Mobile Blitzer in Reichenberg aktuell am Mittwoch: Mobile Blitzer am 04.03.2026 - News.de</t>
+          <t>Statistiques Royal Knokke FC - Tienen - RueDesJoueurs</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Mobile speed cameras in Reichenberg currently on Wednesday: Mobile speed cameras on March 4th, 2026 - News.de</t>
+          <t>Statistiques Royal Knokke FC - Tienen - RueDesJoueurs</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 09:19:50 GMT</t>
+          <t>Wed, 04 Mar 2026 08:57:21 GMT</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxOOHZFZUVtMGU4WDBJZURfZUJNbl80eGNVODV3WVRfSUE4X3dDcUhTZnhtX255M20tTU4zdzB1V3NjQzU2UUc5SHNIcGx5Q0txNWVYVHJlWVJjYVZUY2x3dXdKc3dfc3UtN1B1VEtCWEFrYTd2VzFLT3FnNHF6V3JLTnJVWnVXeXBBSGNRVzR4NzBKMk94Uk5wanVITHRHMWJWdlR6YTZ4TGpxemJ2UEI5cG5GQ2tfUi1JOVRURzhCR2hJSUF1MUY0NDRySV9IS3hfYVRQU3BCWnl0cVZwSDY3aTBzTW1HRjDSAewBQVVfeXFMTTE0d2NMeXFlSEhHb0VCb0JIOXJRQ19rbXRQY1p4Z0QwX0V1ZlhVZ0lBQlludlAtZEZiWGVIX1hTNGhyc3EyM3RXNFByZjNKMFlPN3Bib05MV3pzZERpWFBxSndfdXl1ZUs1VGlqeGZoT0EzalBOWXRhY2hXSTNlUURITFFIOTNoRmpEbElzMW5rQ1dUSXFweFZJUUpRM3hIRlBRbEI4ak0yV3JfSml0UERzYmJIUDdQMkdzMFlhVWZHOXFnV05IdTRrZkpwWVMtd1RwT1R1LW5obXc5RFVybkpnMTczYU5xS2lnczk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxQY1Ywb0ZIeXVITXdROG5ROExUZ3ZhZ0dIWWhpX1BCdXJnaXgxem53MkpBQXNqb0tFOFNZbUx6LVhsTVMtamlidXRPZVg0YWpvSDJrVXREVkVaMFFiN2YxMGV4Y0JGZjFlZEpEN19NbndHQlZpOERoZmFUdVJETFZ5T3RBRXFBTkk5bHRIVzZaTW4?oc=5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1945,52 +1945,52 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K28" s="1" t="n">
-        <v>46085.38877314814</v>
+        <v>46085.37315972222</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Schulstreik in Ingolstadt: Schulleiter der FOS/BOS droht Schüler:innen mit Anzeige wegen angeblichen Hausfriedensbruch - Klasse Gegen Klasse</t>
+          <t>"Vague brune" en vue aux municipales ? Ces chiffres qui montrent que tous les voyants (ou presque) sont au vert pour le RN - La République du Centre</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>School strike in Ingolstadt: FOS/BOS headmaster threatens to report students for alleged trespassing - class against class</t>
+          <t>“Brown wave” in sight in the municipal elections? These figures which show that all the lights (or almost) are green for the RN - La République du Center</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 13:30:45 GMT</t>
+          <t>Thu, 05 Mar 2026 03:31:00 GMT</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxNR09RdFFZMHhDSnlzdk5MQ3BwUGJxRWN1NVpKZVFEZklEX01yTGNUUVJmZzdhUTkwM3ltbEVSeG1RQk1EWFJfSWpHVXdRRHM3bnpVRUZtR0NPazVKelM4UzJIdk95Sy12Wkg5TG5veWRrMzZYbTV1Q3VuZElUUkRhUHVkdWR1ZEpMMGxGdlphYnk1UnE2U0pPa19fOUM2MXJpN2R5Rm5Qd1Y0SnY5UjdpZWpCT1o0T3JLMUhaaUo5WWNJMk41d1UzV0Rha2VfRGM3Vzl5Z2FhTnVXMWUwSXZ3Mk91Y2VFTlk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi_wFBVV95cUxPcTRJcFlaR2ctSFdTLUg4X29weEdjMmd4M25ieVdKNXZHQklkd29lWmdOZE8xX3FyTTNZSVh1SVdlUFR0d0FVWnNhRnhXRzdaRDIzS2QybXJRWEZGeTFoaDZPeVpRbXZrQUpsTVFSbUVuWUVoNURpTUh0YjNETGVxa2piOTJFZmZFR24yRUYyMzVZRjV1aEc3c3dmM2xfTFA5anNYRlVUSjdRRzhBSW54RzhNcE4zcGdlNndCdmhWVFBKTVp1LUw5VFlYVmhqRlJqQV9UaURZT21feXRobTQ2YjJrdzJOU1hLWFgzSjFqN3JubGFnMVpzLTBua1BlSjg?oc=5</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2000,52 +2000,52 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K29" s="1" t="n">
-        <v>46085.56302083333</v>
+        <v>46086.14652777778</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Lebensgefährliche Verletzungen: Motorrad-Fahrer (21) verunglückt bei Ingolstadt - Pfaffenhofen Today</t>
+          <t>Prison : Avant le « masterplan », le gouvernement a proposé de détenir des personnes sur un bateau et envoyer les détenus sans « titre de séjour » en Estonie - Bruxelles Dévie</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Life-threatening injuries: Motorcycle driver (21) has an accident near Ingolstadt - Pfaffenhofen Today</t>
+          <t>Prison: Before the “masterplan”, the government proposed to detain people on a boat and send detainees without “residence permit” to Estonia - Bruxelles Dévie</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 13:35:11 GMT</t>
+          <t>Wed, 04 Mar 2026 20:00:29 GMT</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiZEFVX3lxTE1mc3FhTmxyanVMeFB6YU1hNjFXWjdZOTJEaFBSS0ZOX1poR3NhanQ0Z3gwMHEwN0p0MHVsTnRYQWJDbTl6LUVQRW9xenlpZy1RMXpOSllRb3hUUGtWQVhLN0gzUEY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikwJBVV95cUxNTUNCbUg0RTFMOUQ2bmRvYVh0ckdyQlNZMHFWVWdfZjdLckVKOGZnRnM1Rl9DSmNzWnVPYlBSMGJSZFhJdVpNa1lETG1mNkNkazJKVEVRRUFDWWVkTjZJdmY2MndMVXBWYlFIYmNqOXN1a1FVcy1oellTZFBjRl81UEpzaFZoV3UzalJTZDFNYkRzRnkzS1lYdXdBSXVPTkxiWjk4Wkk1eVdGeWNJYnl2ZnR0QTUxeUVSampKand4OFBZcVY1OE5OU0F6aFlRekNUMlIxZE1WUTNtQ3E2b1JxVjMtWUFmYXFXSjR3Qm5Fb3ROVGs3bG8zY0NrRWpIM0p6bGFjd19Td2N5alljN0NIV3FNOA?oc=5</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2055,52 +2055,52 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K30" s="1" t="n">
-        <v>46085.56609953703</v>
+        <v>46085.83366898148</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Village Ingolstadt (fallback)</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Audi Suggests Gas-Fueled Supercar Could Return One Day - inkl</t>
+          <t>Qualifications Euro 2026 de handball féminin - La Belgique décroche une victoire historique face à la Macédoine du Nord - DHnet</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Audi Suggests Gas-Fueled Supercar Could Return One Day - inkl</t>
+          <t>Euro 2026 women's handball qualifications - Belgium achieves historic victory against North Macedonia - DHnet</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 10:54:24 GMT</t>
+          <t>Wed, 04 Mar 2026 22:06:00 GMT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxNcDFiaGtUYkRPWFR3TExMelFqR01CZ1dEVzVmTGhIMk5fOV8zUHlyZU5iRVhQNXQxcEtObjNscG1sNm1POXlXOGtkZHdvXzJBMmhkWUY3ajJDZzlWa1pLR2t1VUczVjhCOUkwVDJLS1Z4LW9QTDJEa3l1R0pLalE1UVBmR1p0OUU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogJBVV95cUxNMlZCMFgyNEVIMExLSHk2S3BRN0c2cHdtMGFkbTdKNEtBRUhyWW4tMzNxNEdnV3hsUExldHVWdGdQODQ2eVlPSEtwNnlxSndtcVhyX0hGa0J4eHZPSjFpQ2s5R0VHR3E1aDBudjJmTWNkWmVyU0VVcEVvalVxVFhpZDNZc1kzUlFwdGNkM0ZDeUc5LWVCVWN3TGg3TXdvamphR21odzZkNktUNjZmWjYwOF82cjFyeEpicWRJdnh0amtCSnBtRXBEMjNvWmhPUjJZM3kydGNzZ05HV1hEM2phVHhTUmx1OU5DTmZ4TjJOcEVIWG1oemxrVUdVRVg1QWhqcXNPUTFIQ3JTamRWSVh5WFVGcGRLcUN1bUNUU1RLdWp0dw?oc=5</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2110,52 +2110,52 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K31" s="1" t="n">
-        <v>46085.45444444445</v>
+        <v>46085.92083333333</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Village Ingolstadt (fallback)</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Audi Becomes The Latest To Want A Luxury 4x4 Off Roader - Auto Spies</t>
+          <t>Une grande première: la Coupe du monde de cyclocross va faire escale en Écosse - 7sur7.be</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Audi Becomes The Latest To Want A Luxury 4x4 Off Roader - Auto Spies</t>
+          <t>A great first: the Cyclocross World Cup will stop in Scotland - 7sur7.be</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 13:03:11 GMT</t>
+          <t>Wed, 04 Mar 2026 10:15:00 GMT</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTE9McURiYnVhNWEyYWg3MUlaV2pHMldzem4tT21ldUt0dTBINGQ1Und5UXhpWWhHU3pCWkFTOTFlWEJPMHR2WHBKYTFJN1ozTndUeUdsYlZqaTBfWFdCZjE5VU5LNEJsTDdpc0NZcWdB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQV2I0NHFLMHZJTmdoR0ZjSkxId213ZlVqTzBLSWJTRDJTV2FtWl9pdm1IWjJSZ0ppODhESlVfRlhTdXEtY0IyWVU0NTlRUDU0WTRJSjZRb1VxY2tXa2RDNDJNempQa1NwTW02Q2kzNHBOb2tIcE5yd2ptMXRUUXNLUUlOWEtCTHlwLW0wT2p4OE1yTDdlWUFVbjNHdEZHaUlRM3BaSEVJZWUwMmZQdEkzYTJCQVpSRjlm?oc=5</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2165,52 +2165,52 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K32" s="1" t="n">
-        <v>46085.54387731481</v>
+        <v>46085.42708333334</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Village Las Rozas La Roca (fallback)</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>("Las Rozas Village" OR "La Roca Village" OR "Las Rozas" OR "La Roca") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Captain Fresh completes acquisition of Frime to expand tuna presence in Europe - WEAREAQUACULTURE</t>
+          <t>Météo Belgique - Toute la météo en Belgique, en régions et communes par communes - RTBF Actus - RTBF</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Captain Fresh completes acquisition of Frime to expand tuna presence in Europe - WEAREAQUACULTURE</t>
+          <t>Weather Belgium - All the weather in Belgium, in regions and municipalities by municipality - RTBF News - RTBF</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 10:06:37 GMT</t>
+          <t>Wed, 04 Mar 2026 19:16:55 GMT</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOTndjdnR6NEdJQlVUV0xKNm1lUFVlbUxIOHdOaHhRYXIzSmdKUjM3eTNLTWU2VmNDVHg3NVNVRXFHTEdPM2RLVFYwSnAzRDlMT0NFei1mbkNJVHJfdVBNTEpxWGUyODhXNDZSczlzT3VvU2k3UTcyTFRfQWx3QXJUZHFCRW8zRHdmd3lYWWpjUzVrcjFqNDkxUlNoYzZ2OUJnbjIxNHFKOGNZRUZqQVFPbzJ3RWF1MFNyenlqWNIBygFBVV95cUxPTzdBRVQ0VWlkcUowZzBaVF9Fa05DWDM4U0hsN0N1eHFsWHo4clBwODNmcEJzdkhZczJjR001SGtzSFhTaXljYkNtbDM2ZHhaNVN1dDdQWGtfTi1VbFVhbWZwRXhiS2d3a1Y3NUZibFdReUZ0enhaZ3NoN0p1S0ZDMk1aMkVSNXBETjQ2VWcxUVlWYi10WlNzMjJqa19hdE51YUVBRlk5SWh6cWVsQjh2S0pyQ1lFOGNyRzNVUmZiNm5LVVBjUW1SVWVB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiSEFVX3lxTE14UV9iaVNZdjV1X05LRU5DcHNONmRZaXA4YkllNURTWm1CVGoxazBIT2g2V0t1TUZKbTljdjFsS1NrMDh1aUJqaw?oc=5</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2220,52 +2220,52 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K33" s="1" t="n">
-        <v>46085.42126157408</v>
+        <v>46085.80341435185</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>LATEST: Work to start immediately on €17m Army building in Kildare - Kildare Now</t>
+          <t>La Chambre votera la semaine prochaine sur une nomination à la Cour constitutionnelle - DHnet</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>LATEST: Work to start immediately on €17m Army building in Kildare - Kildare Now</t>
+          <t>House to vote next week on Constitutional Court nomination - DHnet</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 11:31:00 GMT</t>
+          <t>Wed, 04 Mar 2026 16:25:00 GMT</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxONy1yNllPOVZRNjN0V1JZaHprY09YR2MxNE5Oa3ZScUQweEFySHMtZ0VxdXFveExvM083eVlLSnpjdzN1T1NtWHdsUTczYjEyVkdidmtvOUR4eElsaGQtaFc4bk1zcmpza0ctcFN4ZkxZTUZIRlR0bWRqaXdDYTNrY2NTVGhsdDc3WWMyLUZDZ0k0MGZRSjNRVVlWZmZMZi1kQl81c2dFRFQ2R3FWdE1TZzRtMm9xMDlkRkpJXw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxQaERlNFF6b2NZLXVuTmdCSUZDd042ZlVxMXdTUVFhSzRxUG9hMC1jYnlPUHota0c5VEd4c09LV1dhN0duRVVtMFBldTNZZ3ROR2pjMzhienlxWkxCUFZZNWFaQWVRcUVEcWJsd0stdWM4VVZqLVFhX24tNDNXRVk3d2FVUzlmb0NZNElScTRjRDhURVJzT0tkb0RVdFljNksyZmZHc1VXdXkyVU9OM2VQYkNfakNuTGNpTGpoMndDV1pSNDNaT25ZQks3NE5aYUlGSE5UeHZKdFpSb2s5SG5jX0ZabGxySFlVLXZvQnBPeEFZSlNYNlNN?oc=5</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2275,52 +2275,52 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K34" s="1" t="n">
-        <v>46085.47986111111</v>
+        <v>46085.68402777778</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Kildare Ranks Third in Ireland for Maternity and Paternity Benefit Claims in Latest Figures - kfmradio.com</t>
+          <t>Rugby : le dénouement du six nations entre les mains des N°10 ? - francebleu.fr</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Kildare Ranks Third in Ireland for Maternity and Paternity Benefit Claims in Latest Figures - kfmradio.com</t>
+          <t>Rugby: the outcome of the six nations in the hands of the No. 10? - francebleu.fr</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 12:36:26 GMT</t>
+          <t>Wed, 04 Mar 2026 17:00:00 GMT</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxPdmRhanNRS2dUV3F4RUphRWpNR1FONmlicVlOa3FHckpGMm9YdWk4R1lHQ1cyR1VJdFRvUGczTklrSGpZUTJZdkFlSWZPa0JTYUJuRWxDWndDNzlyNVNVbEswTl9Hak5VMTZrRGw4RUxlSGhCNlpXWW9wWWtEQVA0blZhcThfdlpWYUpjMzNUNVl5em9rVVl6Q0h6dEp5VHEyakxnNVpOaFZUSFBTSC1vTkgzWWlVN1NhT1pmOGlCbWNVbThGV3hwajVaTmw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxPNnU0YmpnZ1pRbTJVSFFJNHlTaWt3X2xTR083dnRjVWQwM051eXFyUUlhMlBQZFFLZGgyQXM3MHpTaTNJNERoRm9SNkxXVEdVLWRsMlJhZ2QxdXdZMGJQNTdBTkt1RjFEZGxKa0VETUdsM05pRzVoUnV1OXRBT2puTVZGWFZqQXMxd1VrS2U0YW5IdHgyRXpVSTAzX2d3WlhJWVVxd1FKRC1mN1Q4dWRJOTdCTUZmdm0zZkY4UE9yOA?oc=5</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2330,52 +2330,52 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K35" s="1" t="n">
-        <v>46085.52530092592</v>
+        <v>46085.70833333334</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Maasmechelen English</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bomb OR explosion OR shooting OR stabbing OR evacuation OR police OR arrest OR threat) AND -sport AND -football</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Kildare still battling on all fronts after mixed weekend - kildare-nationalist.ie</t>
+          <t>Fuming French farmers camp out in Paris despite government pledges - The Guam Daily Post</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Kildare still battling on all fronts after mixed weekend - kildare-nationalist.ie</t>
+          <t>Fuming French farmers camp out in Paris despite government pledges - The Guam Daily Post</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 11:00:39 GMT</t>
+          <t>Wed, 04 Mar 2026 19:28:12 GMT</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPRWJQc1RFR2JLakctbmhlZTlXbjVRRDJhUFI3YkY1TVdFMXR6SWVqRmlsZzczNnllUnZlMVZrVTlPQjRJRDlvWmtpWTYzV24xYkVobndycGREZVdkT3UwaDM4b3ItUUlNME9KZUg1WldUZG9YNE9iUXM4UnJxc1JhSTY2STJVamJPeDg5R3lvdUNIU0xnSkQxWG9ObmRHYWN5S1hUNG1mOFdyNnlraWJiVHVB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxOZWVoVHEyYlhGNEJFUndjRmN6b0NDSU9Xd1ZjYTdyMF9hbDkxbG93Tm52SEZZZ1BWdzFNdHJmUXB5cHhyUFdlZ2pfd3ZxRUFaZEpWNnV6Wl9SN0JHQl84QkZ2dzZ0Qlppak81d1FIVmpJNFhLbWxDRk9xNmh2blJ2NFFTU2MtWjhkUXRPdTNJOERHd0lOYXVsYlhuSjNYZmtVM0laM0RrNWF6WTd5bTJhM0dZakw4Y19sMTAycFVObzdNNWFrUUlveE1CWmRmM1NlczFOTkRETW1CU2k3TVUtZGZ4WmRoa2FSQ3pv?oc=5</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2399,38 +2399,38 @@
         </is>
       </c>
       <c r="K36" s="1" t="n">
-        <v>46085.45878472222</v>
+        <v>46085.81125</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Kildare Death Notices for today: Wednesday, March 4 2026 - Kildare Live Leinster Leader</t>
+          <t>Brendlorenzen: 17-Jähriger liefert sich Verfolgungsjagd mit der Polizei - Charivari Würzburg</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Kildare Death Notices for today: Wednesday, March 4 2026 - Kildare Live Leinster Leader</t>
+          <t>Brendlorenzen: 17-year-old chases police - Charivari Würzburg</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 10:03:11 GMT</t>
+          <t>Wed, 04 Mar 2026 14:00:00 GMT</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNQjBiT1JIREpwc18ydmlwbGd6a2NZdlpnMEhjTUhtak5MUUI0Uk1ORjBUVnJVWjRxNGVlcElyWl94OHZyV1hOTEgwcHcxUlBCX1pueTR4UHZqTmNzSktrNzFSSVZVSERDejBNRnVpVE9QSng4MmpuVDc2LUEtS0VfeldRSC1QSXdwYmtaQWZrTmplS2E1amhMTTZmT1BDRklDWlM0ZEl0TEpOU0dvMFE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxOMlByX0xhT2xSOEZLTWpXczBQVnlCVWZ1T0ZacGJ6Wm15Z3AxS250RVZBVHczVDkxNTBtQmJDZ1V5MTVNc1N3MDlZWmpUSFRGQmZyckM1SEZ4TkRQbXBybHhqUG5fcDI1QVFnZ1dmckRPNWpiU3A3OXQyV1UtLWxBaFZLQ1dyWjRjMHdHbE5RSlFSU3dQcjF3RnJZeHF3RkUxc1FnOEQxbzV3RjJ4?oc=5</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2440,52 +2440,52 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K37" s="1" t="n">
-        <v>46085.41887731481</v>
+        <v>46085.58333333334</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Shotguns, bolt-action rifles and cash stolen from Kildare residence - Kildare Now</t>
+          <t>Polizeibericht: Krommenthal | 13-Jährige vermisst - Wer kann Hinweise geben? - meine-news.de</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Shotguns, bolt-action rifles and cash stolen from Kildare residence - Kildare Now</t>
+          <t>Police report: Krommenthal | 13-year-old missing - who can provide information? - my-news.de</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 13:05:00 GMT</t>
+          <t>Wed, 04 Mar 2026 13:44:53 GMT</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxQWGVUVkVXSktfakdoUmNrbHhvTHN1aEdHbmp3RE9JcnJCdGJyVTFRQ2ZDTFRIaDZFanYxaVJwdlFhenlnTHltejA4STROZ0pJZG9KOUY3SFA3bkxQVlVEdjZJWXlHMXJpODlFbHFhX3k3azZTeGM4WkFJd1V0b1V1Vy1XR3U5S3lIY2lhYmFRRjhGTWdTTFVxY21SSmJEZ1U4UnVMS2ZoSzk1RThmUVFaeHFMcVc0UXFoWU1rdEhsdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxPSGt1eXRTbXRLNE1SZnJnYUJHNHFpa2NSV25oWE4tQ1EyYmh4N0lCX1NicDFVSTcxdDBNVEZPQVRYUm9LQUZZcjdoODlqQjd1VkI0LWRNSkgzOVhRaDBHUXYwUTBMYnZtTm12dWw5SWVCSmlBNVdJbV9BRnAzVXY5d1Mwa3FDQW5SdjJUSXBUSGZLeUp5Mlpaa1FjQlJWdUZlN1pXVGZjekhGQzRNSFY2RVJoTjY?oc=5</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2495,52 +2495,52 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K38" s="1" t="n">
-        <v>46085.54513888889</v>
+        <v>46085.57283564815</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>COMMENT: Is Kildare's season Slip Sliding Away? - Kildare Now</t>
+          <t>Stefan Weis wird neuer Polizeipräsident in Unterfranken - Osthessen|News</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>COMMENT: Is Kildare's season Slip Sliding Away? - Kildare Now</t>
+          <t>Stefan Weis becomes the new police chief in Lower Franconia - East Hesse|News</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 12:00:00 GMT</t>
+          <t>Wed, 04 Mar 2026 23:00:38 GMT</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxQbkhRUmJDUVhJVElCZ0s3UHMwbThhcXkxQWY3UGJhbG5LRlZQVXlNSkJlVEpzS29TcGZRcC1PUlJTQ19lTVM5Um5UdVhXNXplVUVKdUZWSFM0VWZXR1VydnlWT0VjbHFiVUhCVElHTXJsTGZhc3VybVEtVWRXYVNNblljWDVTZ1ZNUE9ndE1VZHoyV2hjSWk4Nm93?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxPVG82OURkbVFCcklEd2o1aE52bXhueVFuMXJPRUlXb0k3aTFEMzlaNnhBVFdQUFdBX2xWMm9xS0NvTTBfSmpFdU1SRE1vWnlGVUNNZ1ZHRFBhWm9uQlp3UkdEcjVSaXUweWs3TnJvMUhfQ1dMUjl3WTVLMGVWWS1jeTBmcWxPellOYzMzaFlaZWtaWTV6UVV1bk5VMFA?oc=5</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2550,52 +2550,52 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K39" s="1" t="n">
-        <v>46085.5</v>
+        <v>46085.95877314815</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Recent floods crisis in Kildare raised in Seanad - Kildare Now</t>
+          <t>Kitzingen: Herrenlose nasse Tüte und drei Unbekannte beschäftigen Polizei - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Recent floods crisis in Kildare raised in Seanad - Kildare Now</t>
+          <t>Kitzingen: Abandoned wet bag and three unknown people employ the police - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 12:30:00 GMT</t>
+          <t>Wed, 04 Mar 2026 13:15:00 GMT</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxNMEV5cHl6dUl5SGlLclVRQkhDY1BVQmREcU1CbmJ6ME8zQ2dzakJlUlFNb1FQRDBPUWZtNUZGd1BBQlNtZ3VCcXBVREFDUWpuYjNNNGc5NTgyUlBXSmR6dlRpQTZydFBwblc0aFF5REpfdTNxSlBsczFib011X2dTM3dGdUdMLUJCV0JKbS1qcktZOTZPOXp6cGFBb09NUC0yaXdzQ0hlNA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPay1CSjA4VWZzbnZsRjhMZXVram52bGlHeWY3ZUJ0NjhGc19HMWlYNFFWVnNTcEc5X0NvbWtNVGQ5dTBBQWN4WnVZb09lbHY1QzhrSTNmWWtrUzFIZDBNY01fM0ZCR1VtWVRlQVFLWGNBWExlQTJITkQxNzg0T3ZkQXFSZXNhaGt0TXVZYlg5Ymp1X2FpeWoxNnRjNlFJRXJQVWQwdDF2dDJPMDFk?oc=5</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2605,52 +2605,52 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K40" s="1" t="n">
-        <v>46085.52083333334</v>
+        <v>46085.55208333334</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Tesco shoppers complain ‘screaming’ self-checkouts leave them avoiding UK stores - Bicester Advertiser</t>
+          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Tesco shoppers complain ‘screaming’ self-checkouts leave them avoiding UK stores - Bicester Advertiser</t>
+          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 10:41:33 GMT</t>
+          <t>Thu, 05 Mar 2026 03:02:51 GMT</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxQZk1reU9iRkFScFZXUmhPdEFqR0gyMXUwTUtGSEtPTVdUVVRwSlVZei00dWxZMTU5RG03bHd0V2JWei1BWnBHNVUyek01eWdTZllrQTM4V2dDa2JqUUIwTDQxdldoQ0tLaU1vOWlVMGFLVk9kYnN1OWJpLWNGTnhfaC0wam5SOFozcXNIQjBRMDRqbzMzeEo5aGpiMTBEWEhLVHc0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE03RUZJdVVWTG5jTlA1R0dmc2YyQ3Z2S1ExYmhkN0FENFJGamUwenJsSFFPWGpKc3B2aFBaeHRYVDR3aWM1SXg0YWZFVDk0N3d4a0Jz?oc=5</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2660,52 +2660,52 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K41" s="1" t="n">
-        <v>46085.44552083333</v>
+        <v>46086.12697916666</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Owner of almost 30 Oxfordshire pubs considering significant job cuts - Bicester Advertiser</t>
+          <t>Hundebiss und mehrere Sachbeschädigungen in Würzburg - SW1.News</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Owner of almost 30 Oxfordshire pubs considering significant job cuts - Bicester Advertiser</t>
+          <t>Dog bite and multiple property damage in Würzburg - SW1.News</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 09:22:10 GMT</t>
+          <t>Wed, 04 Mar 2026 12:35:01 GMT</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPTWRaeDFMSGZFd3hsWGY3RE1BSWJGTVBMbmcxSGpfQkVoeXh3MnJvN0x2b1BwdmUzTDZFeTVIR3l5N2pEbzlXSzdXY2VvU0V3RWpRT29venR6a2Jja2c0Z1Rkb0lHSi1Rc3o2RW9qcUtCVU85b3VhOEhwb3BmX1h6T3dUeDBhcExhSmJ1U09US0VaR2xqaDN0aEtIVXF5WWhxRjhyNVVKVTZVRjg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxObndrOEIwTm5pWjU4b25EaHRKRThqRGU1WUFTdldNa0UzQ043ZGEySnFnX0JYVkppSDlSbEc2Zkp4RWhuQmg5SDk1Y2NQOW91YnM2NjJRTXpFNDd2LVM3RU9kVGhYVUEtSjA5Ml85UGYzTXZHblh5V0UwRmJNRFBPN2lsNWtmT0QzQmt3SzRNVFBFa0w3SXRB?oc=5</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2715,52 +2715,52 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K42" s="1" t="n">
-        <v>46085.39039351852</v>
+        <v>46085.52431712963</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Enoch Burke’s mother and sister jailed for contempt of court - kildare-nationalist.ie</t>
+          <t>Wiesthal: 13-Jährige vermisst - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Enoch Burke’s mother and sister jailed for contempt of court - kildare-nationalist.ie</t>
+          <t>Wiesthal: 13-year-old missing - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 12:00:49 GMT</t>
+          <t>Wed, 04 Mar 2026 14:10:00 GMT</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOLUNkaG5xcGVXRkk5c2NlWEV6Q0c3d05Sek9tTHI4RHVyYmFoRkV3YVdsZXU1M1lOR3Fkcm5YNlU5NnJyMzBXUUdpMFBKeEtsZTREMXdYMzc2WGNUTUNfMHVBWTYxOFFNZTh3aVVkNXl2Tm5IVWFWOXBsemplbjZVUGd5bzhzRWxtZEZJMVRrNUNwOEtqaEJHT0t6TVhKeWhGMHdyWXhHZVBfS1VCb3N5N2Q5Q0pNdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE9QWEtqdUh5RG9WRjQ1OFFtR0FtTC1lUlhSaXl1Uk5fdUVtWW1RN0VOY2c5ckxIZTdoNWYxNmVxRGZJTEQxd2lLdzRkZ1AtMmVSSHpia3NqSWNtNTktLVFQVFZ0U0NVWWZpcHJuQXRua3E?oc=5</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2770,52 +2770,52 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K43" s="1" t="n">
-        <v>46085.50056712963</v>
+        <v>46085.59027777778</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>What the papers say: Wednesday's front pages - kildare-nationalist.ie</t>
+          <t>Polizeibericht: Heimbuchenthal | Navigationsgerät sowie eine Dashcam entwendet - meine-news.de</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>What the papers say: Wednesday's front pages - kildare-nationalist.ie</t>
+          <t>Police report: Heimbuchenthal | Navigation device and a dashcam stolen - meine-news.de</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 08:39:38 GMT</t>
+          <t>Wed, 04 Mar 2026 10:48:36 GMT</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQRkM4dnFoUlNCZTdtdkx4VFN6WFRUN0ZmRVI5d0ZjVF9PWndxUFdRMEw5V2xHY1FiczBReGVzVTQ5aHRUT1JwWDhJT1Y5cWI1TGpuVGxNcWdHVjRFOUsycnFqRnRpaTBKQmJkSHpCYmFYc0hPMXg2emhzeW5OdENxSl9teXlyV2tlY0ZoMGJ2OFlvaHhnTkdoRVhoWTJtQkE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxOeC12WEU5ZjFwOWhJT18xck40MWZvNnU3bElqYlhJbkJ4X21pMDV6bk9udkgwUFdiT3dmdE9qNnlkM0ZNQm1iQVF3NlcxRm0tRXJsM015SUJiRE1yTzFMdFRuVUpLSVZKM3RMZFlZOC1uMWNWUUU0Q2FNUjNNSGoyeG1SUTQyNkhvUldFU1ZxTjE2Vm5VdlY3U3k0dXBsX2VqLXZiaGxRaWpINm9DUjdOUDd5QUlMOVZ0NVBtakpKaw?oc=5</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2825,21 +2825,956 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K44" s="1" t="n">
+        <v>46085.45041666667</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Village Wertheim (fallback)</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Tennis Channel streaming service joins Amazon Prime Video Channels - Awful Announcing</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Tennis Channel streaming service joins Amazon Prime Video Channels - Awful Announcing</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Thu, 05 Mar 2026 00:36:38 GMT</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxOT1pDcFJQYmRXUy1YTEQxbTBlUF9Nc0FlUlZZUXlJeVlmTFZwTG5fRzZkemZzVld5RlpicnlHd2hUWjBDaFpybUNRYnZCMGh0WDdQd3hGbjhydTVYRGt1Sk9fcDN5QjVUaUR4bk5nRU4xYVJxSFNGaXo2UEhPLTN6TmMyRk5UTmlUN3VUbTk1T29qQ1Ff0gGaAUFVX3lxTE4wck1ja1E1aXNybXhseUxOSkM4SjJ0OUp3VjI5ZWpJdTdLY0ItWTJncDl5ZTRoYmk4dnZJcDlMR05sQ1dubmJSNkk1Nm85RnpRcG1mTGVISXliVmxlekwtVGRtWlloNjM3ZWptbEF4SHo2d0s0di0yYkhhQjhZRGwxSllhMGRsOWhSY19zMHB3WVhaTGF0TXhtWEE?oc=5</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
           <t>en-GB</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
+      <c r="I45" t="inlineStr">
         <is>
           <t>GB</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
+      <c r="J45" t="inlineStr">
         <is>
           <t>GB:en</t>
         </is>
       </c>
-      <c r="K44" s="1" t="n">
-        <v>46085.36085648148</v>
+      <c r="K45" s="1" t="n">
+        <v>46086.02543981482</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Village Wertheim (fallback)</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Election night photos from Tuesday's primary in Abilene - Abilene Reporter-News</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Election night photos from Tuesday's primary in Abilene - Abilene Reporter-News</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Wed, 04 Mar 2026 15:49:00 GMT</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi9gFBVV95cUxNb1VDSzBHTEE1SkVOSUJhTk8wMGYyaGNXX0kwVkYyQzNDX2YydFhhb2RJdFIwYUo3Ym9YMG85WnRtcVlNekY0aURSelRCZ18wTHNXSGtsLWFsNHhyVzNtUTNTdHRjUVdZWGlnQy1keUFxalM5S2lCMEVMR1BrQXNBb1JYSWVwNVU4MldnaUFvWjU2VkRFWUdyRTRuMFlRQlJCbmZMcG1waUZWZUlGZjRvbTR0N0p0U1lINFVrU29mNVBLUlJmU0JfNTBtV2VXY2hTd1RRTnZ3M0lmenFOMVYwcU04VjF4dEdZZmtHYnl4MmNYYWdzWFE?oc=5</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K46" s="1" t="n">
+        <v>46085.65902777778</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Lebensgefährliche Verletzungen: Motorrad-Fahrer (21) verunglückt bei Ingolstadt - Pfaffenhofen Today</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Life-threatening injuries: Motorcycle driver (21) has an accident near Ingolstadt - Pfaffenhofen Today</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Wed, 04 Mar 2026 13:35:11 GMT</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiZEFVX3lxTE1mc3FhTmxyanVMeFB6YU1hNjFXWjdZOTJEaFBSS0ZOX1poR3NhanQ0Z3gwMHEwN0p0MHVsTnRYQWJDbTl6LUVQRW9xenlpZy1RMXpOSllRb3hUUGtWQVhLN0gzUEY?oc=5</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K47" s="1" t="n">
+        <v>46085.56609953703</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Village Ingolstadt (fallback)</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Audi: New Supercar Could Happen 'Someday' - inkl</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Audi: New Supercar Could Happen 'Someday' - inkl</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Wed, 04 Mar 2026 10:54:24 GMT</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxNcDFiaGtUYkRPWFR3TExMelFqR01CZ1dEVzVmTGhIMk5fOV8zUHlyZU5iRVhQNXQxcEtObjNscG1sNm1POXlXOGtkZHdvXzJBMmhkWUY3ajJDZzlWa1pLR2t1VUczVjhCOUkwVDJLS1Z4LW9QTDJEa3l1R0pLalE1UVBmR1p0OUU?oc=5</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K48" s="1" t="n">
+        <v>46085.45444444445</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Village Ingolstadt (fallback)</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Audi Becomes The Latest To Want A Luxury 4x4 Off Roader - Auto Spies</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Audi Becomes The Latest To Want A Luxury 4x4 Off Roader - Auto Spies</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Wed, 04 Mar 2026 13:44:58 GMT</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxObkhCRHRUSVdoZDZYcFZydkZnXzNFQ0J3UklhamtodXRuM1VGaEZPR2N6VHl2c0NhblJZbmdfZGlvcXNtVFRJTDRhUC1NcXBZWUVRRVFoSVNoT3M5bWt4a1ViSElHVkZ6c2dXeUZaMGNwSnhrMnFMdUxEbVR2TXItQkppSzFiNU1weW9QdnFHU1d4ZDdfNVN0OHVR?oc=5</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K49" s="1" t="n">
+        <v>46085.57289351852</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Village Las Rozas La Roca (fallback)</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>("Las Rozas Village" OR "La Roca Village" OR "Las Rozas" OR "La Roca") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Captain Fresh completes acquisition of Frime to expand tuna presence in Europe - WEAREAQUACULTURE</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Captain Fresh completes acquisition of Frime to expand tuna presence in Europe - WEAREAQUACULTURE</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Wed, 04 Mar 2026 10:06:37 GMT</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOTndjdnR6NEdJQlVUV0xKNm1lUFVlbUxIOHdOaHhRYXIzSmdKUjM3eTNLTWU2VmNDVHg3NVNVRXFHTEdPM2RLVFYwSnAzRDlMT0NFei1mbkNJVHJfdVBNTEpxWGUyODhXNDZSczlzT3VvU2k3UTcyTFRfQWx3QXJUZHFCRW8zRHdmd3lYWWpjUzVrcjFqNDkxUlNoYzZ2OUJnbjIxNHFKOGNZRUZqQVFPbzJ3RWF1MFNyenlqWNIBygFBVV95cUxPTzdBRVQ0VWlkcUowZzBaVF9Fa05DWDM4U0hsN0N1eHFsWHo4clBwODNmcEJzdkhZczJjR001SGtzSFhTaXljYkNtbDM2ZHhaNVN1dDdQWGtfTi1VbFVhbWZwRXhiS2d3a1Y3NUZibFdReUZ0enhaZ3NoN0p1S0ZDMk1aMkVSNXBETjQ2VWcxUVlWYi10WlNzMjJqa19hdE51YUVBRlk5SWh6cWVsQjh2S0pyQ1lFOGNyRzNVUmZiNm5LVVBjUW1SVWVB?oc=5</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K50" s="1" t="n">
+        <v>46085.42126157408</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester outlet" OR "Kildare outlet")</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Public complaints lead to six motorists being caught speeding in Kildare village - The Irish Independent</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Public complaints lead to six motorists being caught speeding in Kildare village - The Irish Independent</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Wed, 04 Mar 2026 16:40:00 GMT</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxQX1ExLVJIVGNBWU5xOFJyVUt4bDNWVGtMRWVvaVdUYk1GM3NkSnktWk1Va3NxUjg5bVNRUHM4OGhmeTB4aWtlQlhMUW10a2h6OFdlNmI1NzU3SEk5ZkNJWVRIb05JblFPUUtVbkZJMU42YWlKdG1ZV3BHc1ZTdEdRUW5DbGRhZDJ6dlM4S1p2MnVjdnh1Q1dYTHVNd0w5TTBCNGUyMDhKQ0R6djUtM2VOeVpGbGVoWkJxam1tMzg4bDhucGp5VW5pQTFzbkZGdUdVQXQ4R1BEckZMWjR4YzFsUg?oc=5</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K51" s="1" t="n">
+        <v>46085.69444444445</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>High Level City France English</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>("Paris" OR "Île-de-France") AND "France" AND ("bomb threat" OR "suspicious package" OR "shooting" OR "stabbing" OR "terror attack" OR "police operation" OR evacuation) AND -Texas AND -"Paris, Texas" AND -film AND -movie AND -football AND -transfer</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>France/Middle East • Paris deploys evacuation plans in face of Iran crisis - Intelligence Online</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>France/Middle East • Paris deploys evacuation plans in face of Iran crisis - Intelligence Online</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Wed, 04 Mar 2026 13:41:12 GMT</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxPWm5obXRPM0Z0MFdvbmJvdW1zbndDcEFvLTBKa0EzQ05lUm41THFUREFMWUNfUnhHai1ic1k2RVFYM1EzX096NVFRdlZKQ0JQUVdhNWg3SngwMUVIN1N5dDdmOC1wODF3eUJpbGZlOWVZV0hySjBlam9zeHdmbzNDcUZiakF4MXh4RjU1V3dYV2xVbjJuTHAxbThBVG94ck5BRHF3emZId3k4MFpycm4wbGtWRVY3dF9WcG9aTHZQalYxYVNTMUdyZy1rMFREeUlUY3c?oc=5</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>FR:en</t>
+        </is>
+      </c>
+      <c r="K52" s="1" t="n">
+        <v>46085.57027777778</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Sciopero trasporti marzo 2026: quando si fermano treni, aerei e mezzi pubblici locali - ItaliaOggi</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Transport strike March 2026: when trains, planes and local public transport stop - ItaliaOggi</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Thu, 05 Mar 2026 04:46:52 GMT</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOQzJqcF85TU9pOVRPcWoyYzFJYzJYRGx2X3I0QnI0cVJNRG05UUZCNl93YlEtUEpKZFZ1WnhXSlUyTm1ZbTMxQ0xKdURUaVNvd1RiaVFVUWdSWXpGNm10MzB3Vmp5WlcwSTY1czhaQUZoQXg1OHVHUDFmallBNEhmdWdLc0hpbmNzR1QwbGNxSUhjU29VS2huUnVKcjQ3dnNmby1MMENEOFV5MjVBRkJYLUgyeUxoZlE4ai0tY2ZQdzZ4cUtPTWlhc3hJNFVBUmZQYUdNbk5xV1ktRG5QdjZJSnJ3?oc=5</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K53" s="1" t="n">
+        <v>46086.19921296297</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Protesta contro il Muba. Tornano liberi i tre fermati. Nessuna misura cautelare - Il Resto del Carlino</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Protest against Muba. The three arrested are freed. No precautionary measures - Il Resto del Carlino</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Thu, 05 Mar 2026 05:13:20 GMT</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxOY3EwLXVoaHVxRDdHeFg4RmNwWWV3QXVuM3NSdHNWZ2RJSlJfOTBKYUJKYzNLOE5jM3pCSmtjMFkyYjZIN2t3RUJMME50N1hrZmJKVk4xeFpySS1qZkpTQV9XM3hxS3Y0T0dvU1N2X1dIU3FiUWp3cGl5VmR5eFZjYVVuWkdpVHBKVDB6bUpzeURDc0U?oc=5</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K54" s="1" t="n">
+        <v>46086.21759259259</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Manifestazioni, mostre e visite gratuite: il programma completo delle iniziative per la Giornata della Donna 2026 a Milano - Secret Milano</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Events, exhibitions and free visits: the complete program of initiatives for Women's Day 2026 in Milan - Secret Milano</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Wed, 04 Mar 2026 15:27:35 GMT</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE0zNG9wSnU3bzNFOFdoSXB3dU02ZGxVQVdkSm55d3lveGNYUnZBcHZhSTZfanBzbkRuN196ZnNHMHFNNU4zMEdvd3hrY2ItVklrZkNqSFBOWGZfN19vemx5WUN0UDgyeWdwaE5IcFlScGI?oc=5</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K55" s="1" t="n">
+        <v>46085.6441550926</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>BOLOGNA: Sgombero presidio ambientalista, Procura chiede 3 divieti di dimora - Teleromagna</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>BOLOGNA: Clearance of environmentalist garrison, Prosecutor's office asks for 3 residence bans - Teleromagna</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Wed, 04 Mar 2026 10:10:37 GMT</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNWGVEX2lmQWdMX1doZ3Npci1MR2lOYmdpdnhXR1RlT2UyVC1lNGZ0Z0xlZ1dnbGNSd201QWpKU1lnNlJIS0puVGpYXzRPVEY5WVRBSXJmM2FzZHVCeVFUb3N6TXlGYjBxYy1nM3pidGltcVJ0cE5ZSDZTalhoNndHSEJVNGY5TW1BaFU1QnBRNnFZQU1QcXl5SXlCOUc4VDVKdjYwR3JmbXpoZnlOVjNVTFZKY1dGZHhsSExJYUtn?oc=5</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K56" s="1" t="n">
+        <v>46085.42403935185</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Scontri nel cantiere del MuBa, scarcerati i tre attivisti. E la protesta smonta | FOTO - BolognaToday</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Clashes at the MuBa construction site, the three activists released from prison. And the protest disintegrates | PHOTO - BolognaToday</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Wed, 04 Mar 2026 12:53:15 GMT</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNZ1JDbDhhczRJQUxYaGNzdVNfcHdfblFzWUttcG12bTd3cjlGeFVOZGczRy1Gb1BIVXdGdnlmTy1vWFpXRGtfN2wtN2lSQUZNeDZvQXh3T2dTTk5sc2JzU0dDaTlkbWJqb21PbWNTWldUZXlsMUM4ZDlpcENMLVowaTRTYkgtSEdLRzRGc3JZTzRIazFRblE?oc=5</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K57" s="1" t="n">
+        <v>46085.53697916667</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Scatta il decreto sicurezza a Bologna, multe fino a 10mila euro agli attivisti del Pilastro dopo i tafferugli - Il Resto del Carlino</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>The security decree comes into force in Bologna, fines of up to 10 thousand euros for Pilastro activists after the riots - Il Resto del Carlino</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Thu, 05 Mar 2026 02:03:41 GMT</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxOYTdJZHk2eFNnOUdGQk45Yl9tTThzd0phTDV4VzVsb2FNcjFxTDhzbmRBWGJza1RjUzRuZ2NkNlFLZV9nZXIzZlVGU19ocHk1M1NQa3JpMldGbjY5Um02cm5DVkMta3hmNDc2bFpkOWpqbjlUUDJZcXNZaE0tVVhkSEU5a2ZXQmJ4M1J3Wm0ySnd6ekJuVm9XTkl0M2JZZ0syeDI2LVhMbk14ZUQxNExvVTVyYVk0ckhaMlVVN2JOTi1DUVNtMGln?oc=5</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K58" s="1" t="n">
+        <v>46086.0858912037</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Per un no sociale al Referendum: dibattito a Milano lunedì 9 marzo, verso la manifestazione nazionale di Sabato 14 - Usb Pubblico Impiego</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>For a social no to the Referendum: debate in Milan on Monday 9 March, towards the national demonstration on Saturday 14 - Usb Pubblico Impiego</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Wed, 04 Mar 2026 10:26:00 GMT</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxNOWJEOTNhaENHN3J1M2JDVUtmMVdicTEwd1BYWEx6NTJtQTAzOTBJTUQtRzF5TTE1Vi16UDhzSDNGZGJNbjc2WlBudk5qc3RrYzJwVXVwSmpnMnNadWhxcVJoTjNDdk92S01sTzFaMEhGUEhiRHdVQU9zdF9wU2xPTnBsMzVLUnhRcVRNWWhrOEF1Y0x3QWdLaTFDYVhzbGRENTRnSy1QUGk4RE4zWUpaWGtOVkZOR2xWenN5c093M1kyV3Frb3JpMnMxemFNbGdzSE5uSzd0YW5kcU5ZZWhiYVlZcC1WU1p6UENzY1YtOXltamFhMWFWSWFuYw?oc=5</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K59" s="1" t="n">
+        <v>46085.43472222222</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>BOLOGNA: QUESTA MATTINA UDIENZA DI CONVALIDA PER LE TRE PERSONE ARRESTATE. MIGLIAIA DI EURO DI MULTA AI RESIDENTI DEL PILASTRO - Radio Onda d`Urto</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>BOLOGNA: VALIDATION HEARING THIS MORNING FOR THE THREE ARRESTED PEOPLE. THOUSANDS OF EUROS IN FINE FOR PILLAR RESIDENTS - Radio Onda d`Urto</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Wed, 04 Mar 2026 12:50:00 GMT</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi-gFBVV95cUxPYUJXS3J1dlFKdTdaLXNGZUZYWFVhMWhnb3lPVUdveTNpdjl4TDR2Z1hRRkM0SGpoSGd2N0xueEthZ2tudHNGRExTanltMEZ3TlAwaTVoVnFjRGZqNDZWUnp3YmpvMkhtS1A0MU14TkcyNGN6aDVfcDg3RFp2aGdtTFZobGxsb1lxRUx2Y2pKaWtZNEI3bUNDelhkM2t2ZmpDNDNzWGdQbHU2d3J0Wk1wd1ZKZWJaVU54OU5pX2FXbmYwUHZMejBpazhCaVJwWV90TGNhSk1uM25PeDdRRmdEQkt6bm9OSzNHSGZjVXNhd3hKeEowNFZrT3hB?oc=5</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K60" s="1" t="n">
+        <v>46085.53472222222</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Guerriglia al Pilastro, smantellato il presidio degli attivisti contro il Museo dei Bambini - Il Resto del Carlino</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Guerrilla at the Pilastro, the garrison of activists against the Children's Museum dismantled - Il Resto del Carlino</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Wed, 04 Mar 2026 12:03:30 GMT</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQR3loRFFSTDJhSHRHUGRoazVaR2FWdnlMRUlha0pST0FQRFZFdEFLemJoOGVuNnpTaEZVZ2laUmsyV0V5a2ZkZHZpcVYyWHh0OG50S0VPWFZYWURlTF83bnZ5WHZDTzBOVWwzUDJDWXhVTjdCLWZfQjdISm1HSWdBcnRR?oc=5</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K61" s="1" t="n">
+        <v>46085.50243055556</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-03-05 14:47 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K61"/>
+  <dimension ref="A1:K66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -490,22 +490,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>B&amp;M European Value Retail PLC Dividends – TRADEGATE:7Z5 - TradingView</t>
+          <t>B&amp;M European Value Retail (LON:BME) Share Price Passes Below 200 Day Moving Average - Here's What Happened - MarketBeat</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>B&amp;M European Value Retail PLC Dividends – TRADEGATE:7Z5 - TradingView</t>
+          <t>B&amp;M European Value Retail (LON:BME) Share Price Passes Below 200 Day Moving Average - Here's What Happened - MarketBeat</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 21:03:18 GMT</t>
+          <t>Thu, 05 Mar 2026 08:20:14 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE1VQjM3bS1FRjZDT2VreDhXdVFNUXZxRmxuUWNvLUNqQXVLSjNQQXZ4TUlCUlNsbl8wcEI3VGpzLS15U1dXVUgxU2lVYVpYbkVraS1mSzNnWkg3TWp2Y0hyTUYwTVpFNTFZcW1fc0dYOVlfS2p5YXlBSllFUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxON0pnSWY4cWJFRDgxLXRXUy14RnJYVnFGWUlpZnAyQXI2b2hFLXV5MDN5U2NuRHFpalE1RURiU2dsTWZPeFRFeXViT29QOTNfaHM2YTZzUG4ycldHQXdRLWNEWUpHZUp1R01fZy1KUzJ5dTVyVVFxZU03d0VUd2lESTZUc1FwTm52VXk1TllnaUVtZGZKMEVBWTRMOFZCZWpuWXZKWDVlUFVUdXp5b2lxMHJtS3UtbHZnc2Rscld3Y3UyNGUyZVJxXy1mOVQxRkUyelpHT0hmanJIQkI5cHFGUEE5UEtUVV8t?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -529,38 +529,38 @@
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46085.87729166666</v>
+        <v>46086.34738425926</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Value Retail Brand</t>
+          <t>London Marylebone Incident</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
+          <t>("London Marylebone" OR "Marylebone station") AND (incident OR disruption OR closure OR police OR bomb OR explosion OR stabbing OR shooting OR "suspicious package")</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Target’s 2026 Turnaround: Analysts Bullish as Growth Returns - TradingView</t>
+          <t>All lines blocked at London Marylebone – here’s what you need to know - London Now</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Target’s 2026 Turnaround: Analysts Bullish as Growth Returns - TradingView</t>
+          <t>All lines blocked at London Marylebone – here’s what you need to know - London Now</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 18:07:00 GMT</t>
+          <t>Thu, 05 Mar 2026 08:40:35 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQbUFBQml4UkZ5V0xEOGpVdFRlM2xXQmdTQUYxWjJubzVuTUptYzY4X2JKUExIT1Z1UEFablVjeHRKTzJqRE9TZUdqM244LW1SRy1JM0RFTG1RdG9nMGxVZ0l4VWZpMVpadFNkeF84dFlpZ1pNQnBxNGh0Vlo2eE9GOUVKWTFyWjhFZEUtMURjQjZkdkxodm1NdDUxWlkwakNzY2dKZnNBTVZfYTd3UEdLcUpRSXRqc09IVUZLRw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxQXzZyNjEtU1lDd2ZvOFY2VDB5c2k2RktPMXpTNERSdXVwYUZUTVBDSkVkMzhSTVgyU2hISUFuNVc4QXlXTVE1LXk2UnJHQTZNWEl1b2Z0ZkEzMFBaR3NBZlNLSmN3cTdfOWU5anowVkFoS2QxSnRYZXVQT1lOLURJanNkZmVfazlhS1ZNR1JGdmdCZndzdWNsU1lvUWxNZ0hLUFJvSA?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -584,38 +584,38 @@
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46085.75486111111</v>
+        <v>46086.3615162037</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>London Marylebone Incident</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>("London Marylebone" OR "Marylebone station") AND (incident OR disruption OR closure OR police OR bomb OR explosion OR stabbing OR shooting OR "suspicious package")</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Global tech and beauty company opens store at Bicester Village - Oxford Mail</t>
+          <t>‘Casey 2’ inquiry launched into Met’s overhaul since Sarah Everard murder - London Evening Standard</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Global tech and beauty company opens store at Bicester Village - Oxford Mail</t>
+          <t>‘Casey 2’ inquiry launched into Met’s overhaul since Sarah Everard murder - London Evening Standard</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 15:28:20 GMT</t>
+          <t>Thu, 05 Mar 2026 12:04:28 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNbUQxRXJaQW5HcGtKTklWc1ZDUU5hQjNDM1RfTVJ1V0ZWM09mV3dBcXVvd0xQdFlZQWJMNEkzcjJ1Wk9tNlBHTHVvMm41ODdpQVBNamgweldIbnVUbTVkVHczUnpLZ0NNOVEzZjZuRVJUTVFYbmkyb0pDUl8wNVV0Y2FIYUxmdnV3YVlQRUk2WHdOd0NrckE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQRGRYNEt2RkxuTUpFLWlULUNkTzU0LV9zTUgzRkZ6dEt6aUNZWk9uMGJYOTlYeHNHd2JjZm9mUk15aUxNWVh2VFNMWDUtMExNdFp4X0x6N2RCak5iNHp3V2hvVW13LXlqRmNNalFDcXM2S2NOM29xNzFHdjBPZ3d1MzlWaGdPVVNuVTdwYm5oOGc0SHozWU5NdURJRGk4SEJzbmtRME1SSXNFTmh6WlJKdlI5V1B2Y2xhbWNvQk5tWElGNm5Pek9Cb1hqTzY?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -639,38 +639,38 @@
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46085.64467592593</v>
+        <v>46086.50310185185</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>London Marylebone Incident</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>("London Marylebone" OR "Marylebone station") AND (incident OR disruption OR closure OR police OR bomb OR explosion OR stabbing OR shooting OR "suspicious package")</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Dyson Opens Immersive Boutique At Bicester Village - 365retail.co.uk</t>
+          <t>Major disruption continues at Marylebone as delays extended - London Now</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Dyson Opens Immersive Boutique At Bicester Village - 365retail.co.uk</t>
+          <t>Major disruption continues at Marylebone as delays extended - London Now</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 16:45:51 GMT</t>
+          <t>Thu, 05 Mar 2026 09:26:57 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQWmF6amVxcmxrSFRuQlpqVlB6eUZIc3EwWnJzeFV5LS0zcWxiNnRlSmwyY1RLSnV2VGVla0FPc3FILV82dTBsaDN1c0pMQXhIT1hWak92SjY4WmRWeV9KbkdHWjlGWEs3MlhxSG5BY2k5WUpHQjJKVDZfODhPMFg2Ng?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxNNEZOak9CQmlPMkdrRFNILVpCa0c0QTdGenJiMmhZUVdWWWFfbDZQRkVmMDNmT2ZsUTE3VGdtUDRORVpIYWYyU2dSRTNpcUhNYWZZXzFYczF5c1B1SnJ5T0phUGwtT05QVjhDdXdTbEpwUWo2bjBfVS13X3NhWHdsNzJxcXUyVFJvQjd1WklaRXp6QllOdy12T2t2TUpfR2RrMFFr?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -694,38 +694,38 @@
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46085.69850694444</v>
+        <v>46086.39371527778</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>London Marylebone Incident</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>("London Marylebone" OR "Marylebone station") AND (incident OR disruption OR closure OR police OR bomb OR explosion OR stabbing OR shooting OR "suspicious package")</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Scotch Corner Outlet Village targets £25.5m via stock market funding - Place Yorkshire</t>
+          <t>Husband of Labour MP questioned after arrest on suspicion of spying for China - London Evening Standard</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Scotch Corner Outlet Village targets £25.5m via stock market funding - Place Yorkshire</t>
+          <t>Husband of Labour MP questioned after arrest on suspicion of spying for China - London Evening Standard</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 11:05:00 GMT</t>
+          <t>Thu, 05 Mar 2026 10:13:35 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxQR2N3S2wwWnplWVd0aXVKcVl1bXFJODNTODZacEFHc1EwVGdNck4yanVhSUw4b3B0eHNMSExFZ190R1c1QkZIdlFZU25ZUm93bjI3UjNIaGd1TEtkZnprRmtPbTFQcEdWVjFrTWZkaU5QNEUwdUJPWDU1d240UThpMjFpX3pTU0xMZ0FXN3ctNkRTU1VVS3A0WlpxQjFzbk5iaE5V?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxORUVZbnJyTFJnaHFvMEs3M1ZPdVhfMFE3RGIwMXlhQ1pZOGd2WXI2elB5Wl9tZThnZFlaLWN5Zms5ZENfa1JKcmM1a2Y0SXZUS0w1bng5UmxCSkE1d2NIRWdEc1Q2emlMSV9sQjRMRnRZdG5nMkVyMUhmRTVndG0zWnRqcWp3dmdQN2tIY0llc25aZnlZdnE4VjFOZFdkZw?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -749,38 +749,38 @@
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46085.46180555555</v>
+        <v>46086.42609953704</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>London Marylebone Incident</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>("London Marylebone" OR "Marylebone station") AND (incident OR disruption OR closure OR police OR bomb OR explosion OR stabbing OR shooting OR "suspicious package")</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Major update on new Yorkshire designer village packed with big names earmarked for 2027 opening - Yorkshire Live</t>
+          <t>Raver nicknamed Nasty guilty of killing deaf woman with single punch - London Evening Standard</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Major update on new Yorkshire designer village packed with big names earmarked for 2027 opening - Yorkshire Live</t>
+          <t>Raver nicknamed Nasty guilty of killing deaf woman with single punch - London Evening Standard</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 11:24:00 GMT</t>
+          <t>Thu, 05 Mar 2026 13:22:34 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQcXM3clpMbVJwQlg3VUxyNlc2RnVjRV91cElXVHpRS1IxREhsX1FldnI2dExXdXhkZ3NwRVVmanAtRzBxYmF4X1lFM2w3a0k1bmR2MHBsMm9Bd0tWTWlSaGlhX21iR19FZXBXREhmWUxGNl9YNFExQl9rUWFWdmxhX2FFVlNmclVQVnNNY2hZSHdLQ3ZBTFRZeGY4Y2x0b3PSAaQBQVVfeXFMTUJKVjQxdVNCakYzclJYMUt4aWFIYWVON2NidElPX1U0dHJoTHl4NzJFVld6WXAyY3JsY19vTzhaSXBSZmNPVVI0dVNnanRxVlFaaElDS2hoSTF6QnNUdHRWcHdHOUE2eWRfZk9vVktXZmZUR1dPMkE2a05fRW55OFV1eW5uUS15UzZLRGwzeW9jTFZxNS01YnFzWHNfa1gyN09idHg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNYkpSTEpxbHo2QjFzS0l5RUtCeXpaS0huMzhYQ01oS2NoYTdweHR5cnJtM3M4eXVZZmhWLVdFWlF2eWUwbXZvTHNVVF95TFN3ckh5SURGV1U3WmRVQVhSWDdUZFY5MXdpZnBNMHlCdFZyLTZVTlJVd3owNUtyNG1VcTlPNWdqbS1Ea1RaR3pRVFl2bk90dEZJaDNBM25UcUU?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -804,38 +804,38 @@
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46085.475</v>
+        <v>46086.55733796296</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>London Marylebone Incident</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>("London Marylebone" OR "Marylebone station") AND (incident OR disruption OR closure OR police OR bomb OR explosion OR stabbing OR shooting OR "suspicious package")</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Death of university student to be investigated at inquest tomorrow - This Is Oxfordshire</t>
+          <t>Risks from Chinese spying ‘not receding’, Speaker warns parliamentary staff - London Evening Standard</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Death of university student to be investigated at inquest tomorrow - This Is Oxfordshire</t>
+          <t>Risks from Chinese spying ‘not receding’, Speaker warns parliamentary staff - London Evening Standard</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 16:30:00 GMT</t>
+          <t>Thu, 05 Mar 2026 11:55:38 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxNNkZZMGhfMG1xcEdCYjFRemJDSFhiUHYyOWk3UXB2eFZQZFF4TmtoWUhXRF9QZ1U3d01ELWJUd2VMRUhoWlhtX0hIUElLQUprNjFTSVJnYlNLTGZiVGhwS1VCcGwzM0I3WFhnRkpqSGlCVTRLRW1GUmZfS1Z1cF9IVDM1QlYwcndQVUpiby1rRXFWWU0tQVpsXw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxNLTlsTzJZS3lUWUl5Z2lfRjEwZDFkaHVXTWdFUzhtRFZINmVYUnpYQ21XdklOM3MzMlhLYmsxRW5URWk1UFViUENZaElPUkNiUXZlc2pndFdtWjdtVGtrTzVYRnFmNmNuY2tLelhiRm5Uemh3NnRSdGxSN0REVFVMRmdpbmVSZnJSY1ZvRkZJTG5qbFJZUnpGTFZvZlBnOFg4cy1ici11eDVfNXJfWi1BVw?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -859,38 +859,38 @@
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46085.6875</v>
+        <v>46086.49696759259</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Trains to London Marylebone to be cancelled for weekend - Oxford Mail</t>
+          <t>Is gedwongen hulpverlening het redmiddel voor drugsoverlast De Coninckplein? “Een zéér drastische maatregel” - GVA</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Trains to London Marylebone to be cancelled for weekend - Oxford Mail</t>
+          <t>Is forced assistance the remedy for drug nuisance at De Coninckplein? “A very drastic measure” - GVA</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 16:59:31 GMT</t>
+          <t>Thu, 05 Mar 2026 10:00:00 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxObGl0YWltVEdDdWVwTC1TQmRaWUhva0ZxdXNzc3FYc3NOcGZoNDZOWFM5MW94U3YzemVDVkxMUzJNa0o4OE42Z2ViLUJuYmN0WHlWd1pyQ3NLNGRXUWFYZFRNRDZ1aG5EUHBVTjJKVUNLUkNoOFJZLV83TVE5elhteThDdUtfRGVicjVZVENvSQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijgJBVV95cUxPbFFlNC13N1ZqSXpHRW8xRkw5VzMwNFQ3ZkVCenhDSHpwTk56eE9OVjA1eGRyNkpHVEs3RTcwVTR6eEpiRWx2bURwSHIzZ0N4MWpFRWFkaHZ6ZFltdFRkd2l5SWlXd2RYc2g1QnZxZWVISDd1UmJHckZIM2dwcy1IN2dBVDlxZDFGYS1oWjgtWHVoUHdtdlJCN1EtNnpMRENXWlB0WnpKakt4RUs4NWIwNW9YMlN2c1FpbXJjNktnbHBWcTJKM3JvTVpoUTVrTHYxeEh5QUs2RDZmdWw4YlRpN0xXWVpRc0IxU0daVmNYVEh0eG9DcXNEeDRQNEs0cDhISnB3eTVfaE5uaC16bUE?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -900,21 +900,21 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46085.70799768518</v>
+        <v>46086.41666666666</v>
       </c>
     </row>
     <row r="10">
@@ -930,22 +930,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>“Precies een aflevering van de Kardashians”: ruzie tussen drie vrouwen mondt uit in explosie in Deurne - Nieuwsblad</t>
+          <t>Appie vzw gaat ijsberen en Lowieke herdenken voor goede doel in De Mosten: “IJsbaden heeft therapeutisch effect” - GVA</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>“Exactly an episode of the Kardashians”: argument between three women results in explosion in Deurne - Nieuwsblad</t>
+          <t>Appie vzw will commemorate polar bears and Lowieke for a good cause in De Mosten: “Ice baths have a therapeutic effect” - GVA</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 00:15:49 GMT</t>
+          <t>Thu, 05 Mar 2026 11:17:52 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijwJBVV95cUxPWmFQQ0JGMmNKR2E2cVhYY0VFcFdydGZJVkV5cWR4cDZQZFFhb3FVQXdqWUJuaHVGYWs5ZGN2WWxISmpoNzNUZW1ZdUU1T2hZbm5xdXh1MXZ0TjJZUzRxVzFpRG16TVNIUEdNR2lMUVN2U1VLU2lFbWUzaDZDMG9rLUNfZzFGZGhzT0xzbTJyVmU1UHVKOTVCTUpjVFNpeEpXclVsbEhaemk1aDl0Umhsb1g2R01zMWtoNmpmWExCWm9naElSYjFyQ0pMdGlheVFvYW9VWXc1S25RZnlNV1hNOVFqVHFDMlY4OFFYaHlQM1NfZENOQUtBRHd0eHJhVEsxM0pvNWVGbVA0dy1fOWRJ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxPVFdZdWhfOVkxMXBvdjRWYjdWakRGd2JWU2hBZFVMenBrVEV1LTJZZE13NzA5NTdaMXlMMGcyZWxQcGNHem44dHdhOExuZWRfSFhPS2laTXhqMkF5OXZqeDQ3TE5HN2hlRGc1amc1MXZXMldicHFjeW5xS05Ld0FVVWRob1B4TE03OHdhZGZESk5YWVB6MG1xUUlRT3FZTFVBRzRST1F3YzBrRHVOWWhzTXkyNVlKN1gwcGZDUUNIbWxOQzVFR21VR2hBdzFGTC1VYzA2TVdpbVY1aDc5VnR0SkhBVWRJbjRRdWVSS3RYSUdkSmNiLU9RNnlMay11VjlKaG5RSUl6aTJucklHdFlBcA?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46086.0109837963</v>
+        <v>46086.47074074074</v>
       </c>
     </row>
     <row r="11">
@@ -985,22 +985,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>“Financieel kan dit erger worden dan corona”: reisbureaus vrezen zware verliezen door oorlog Midden-Oosten - GVA</t>
+          <t>Peiskos Quartet verzorgt springplankconcert in Protestantse Kerk - De Limburger</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>“Financially this could be worse than corona”: travel agencies fear heavy losses due to war in the Middle East - GVA</t>
+          <t>Peiskos Quartet provides springboard concert in Protestant Church - De Limburger</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 03:00:00 GMT</t>
+          <t>Thu, 05 Mar 2026 11:48:20 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgJBVV95cUxQcDBqdzRrRkU0N245czVaVFZBV2RxVzJhX2FXRGRKN0c2Q1I1bDhHUHJSaHluMEYtWnJXa1NvUURTRGVDMlNQdHNST1dfeHJlZGNBbHJ2R2c0RW5WVFdwaUJaTktCRm1UY0RuLWdzcHZvU2hFU2ZFNmlrYzlHbWkzNjF5cGI5UWZoVllOZDVxc1ozUE0xbHdXbUxjTVZHcWxrUk8tbFlEZEpnaDlNeTN6VUI4Y0p6VmhCcllCSUZnSTZNTjlfemZJZHV4MnEycUdJeTdTQkEtTHlBT29TeWlvZVlNdDZFZUM1UjhJeTZXaTFhYkRsQkdzSnhDZ1NCSEswb2p5ZWhka2ZnaUhfN09YNm5zbTctd0hQcVE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxQTHpzcmN5ZGQtX2hmRzgzSEtEZGxMREdQbWVmQ0lKLTlLMHllV2FNbDI2b254V05UQXpmV2ZHaXJPME80amxBbkp6U2pHV1JORFd2TWlOXzg4NDJEWi1UY1BqNTFHLXJyRTMxTDdidjcxalhxOEg1UXd3RlNNaEhpVFltRmRrQ3VZNmJ5aUdPQzZNTGR0dXJMdXZ6dkhiMUJHMVM2UFlwdnlVcm1vTExJSkxJcG1SN1J4M2c?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1024,38 +1024,38 @@
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46086.125</v>
+        <v>46086.49189814815</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Schietpartij in restaurant in Zele - HLN</t>
+          <t>Exclusive-NATO's Rutte Does Not See Need to Invoke Art. 5 After Missile Incident - U.S. News &amp; World Report</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Shooting in restaurant in Zele - HLN</t>
+          <t>Exclusive-NATO's Rutte Does Not See Need to Invoke Art. 5 After Missile Incident - U.S. News &amp; World Report</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 10:50:34 GMT</t>
+          <t>Thu, 05 Mar 2026 12:09:41 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxQNFZaVVFnMVRvSjVGNXZZRVEtTE1OWmJObEI5dlZQdkdOa2tLUkJTVWVrdmd5ZHZFblRWdlBrRi1FbE0zTkFyWWNIbERSdmZ6MmREZUYzUmEyblVUa2gzQTBrS2M1cFRiMGpmSmxyV3Vqb3gtdFI0OVdqWno2UnE3Z01najNmdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxPMWV6eThHVk0zYkVfRkE0ZmUtdUFHT3dqUUFzVGhDYnVkV09vclBBQ1NKc2kyUE40eGtFckFWTDVvXzhUc3Bxb3Bhdk91bjZfV0Uza1dGNHVLd2NwZkhuNHhRQlgzZmxxNVNPaTZTM2N1Wm5FR3FZYmJaVmczblVvandnNTc0eWxkSkdPc0F2MjdaUjlyekFCRUlXQmp0SHh2TDBub3NyVFpKYjAxa3BYRDVsc2NaMEdObVpydEg3NWVadjZsWHJlQVl3U3lkWHlOWGYzclFJZw?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1075,42 +1075,42 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46085.45178240741</v>
+        <v>46086.50672453704</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>“Je zult branden”: vrouw zou brandbom gegooid hebben naar voordeur van vriendin nadat vriendschap verzuurt - pzc.nl</t>
+          <t>Iranian regime “conservative”? Never, the mullahs are like 19th century Bolsheviks - Brussels Signal</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>“You will burn”: woman allegedly threw a firebomb at girlfriend's front door after friendship turns sour - pzc.nl</t>
+          <t>Iranian regime “conservative”? Never, the mullahs are like 19th century Bolsheviks - Brussels Signal</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 18:19:00 GMT</t>
+          <t>Thu, 05 Mar 2026 11:03:11 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8wFBVV95cUxPWjFVV0pOTGZJTHprbXc5WDBrSVpoR1RDUHhrSG9ZQm94emo1ckh4XzRIemVyVjBSaXVPU3BrOHFLcEpTRmViV3NKd2RQOGtReHFGOUNUbV9HNE03VWVnRWtzZXV4Nlo5ZUNuMVVLVTVtVWY0TmhtN25CSENMa2dNYXVpRGlrU0FkdEZmSFBqWHQwTnlZS0NoR3JTOW1HTnBlZkxiSWdIdkVnelJCRjk1WEx3YnJsVUgxZDNvazM0ZWxKa0ZaeGJGMFBQbk1JSTF0OTZaUmF1VmZ2MWRTYzlobHJreHVWYkFUemJiOFdtbEZWek0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOWWFncXVOemxxYm1qOXpycnVRQmRza0Y1NlByR0ZRY0ZQVmVBTlJoTEpoV1dxMENHekJVeE4ySWJSZXBvdTVZeFN1SVZVbERnLVBuZFV1R0syNHNEMThfamlVcUlZNnIzYXZsV185NXdINjhMU1VaWVg2YklRU2U4dXhERHRlMm9hWldXbWpZRVotNTZwUmpaQVFGWi1wM1I3bjlpNTJLQUY2NEpoaDNZU0RQNA?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1130,42 +1130,42 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46085.76319444444</v>
+        <v>46086.46054398148</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Is gedwongen hulpverlening hét redmiddel voor De Coninckplein? “Dit mag geen openbare-ordemaatregel worden” - Nieuwsblad</t>
+          <t>French appeals court lowers charges against police officer facing trial for killing of teenager - The Straits Times</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Is forced assistance the solution for De Coninckplein? “This should not become a public order measure” - Nieuwsblad</t>
+          <t>French appeals court lowers charges against police officer facing trial for killing of teenager - The Straits Times</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 01:08:26 GMT</t>
+          <t>Thu, 05 Mar 2026 12:39:02 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgJBVV95cUxOSDNiUjMyZzU5Z1hpaXVpSnF2TVBzeWd3ejdvVnRYeC12UzVhR3dVSlZabTNXRzNKUTA1Q3pHM0p3bU1wLVJ5VnE0Z01halYwMHMyaWZLTXhJVlluVFdfYlA1LWVrc1VPaDhiMElnTllQNTg1WUhKdDlnZ0FWUWZZbG5kV2J3R1F4emI4eUpnV2RKdUIzdkhlMzVpZUpZckFWUXRmclR6UC1RQnZFR2dzazFDRnJYTXFpSV9EaHhteHdvMUZWcUs3NmtMUGhOeFZGcHlmbVQzWTBSVDRpLTQ4QUtqWkpkNUZqNlFLLXM4UzZteGNsQ2JtejMzWWtCemtsZGxTNUV6b1pmNUZ5cVFYOVJIS3N1UQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxQYlRrLUhUUWEyZkdaV3d1clQ3ZnhNY3BUdzFXd3I3bE01VWt4NlhFYVFkMnVIOHQzWkhaVEhXUDI1T2tkc3dpNUYtcXlYenVCbFV1NGx5NG9VRFFFMU8yMWxqeEJCVXpyMkdoQjBPYzc1blBGR3FKcjdQZW9NNklVTHZ0bWdBUnZqcnhJS0MzMGNTYzZWZ0JOSllDSzd6OWxITWg1VTNpSXBvSVV6ei1QU3BQamVnUHZXcGpzRldMOGVwQVcxR0FTWTBtSXU2UWdvUHo0?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1185,42 +1185,42 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46086.04752314815</v>
+        <v>46086.52710648148</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Stoomaccumulator geplaatst bij Sappi Maastricht - De Limburger</t>
+          <t>Syrian man handed 13-year sentence for Berlin Holocaust memorial stabbing - The Straits Times</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Steam accumulator installed at Sappi Maastricht - De Limburger</t>
+          <t>Syrian man handed 13-year sentence for Berlin Holocaust memorial stabbing - The Straits Times</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 16:16:46 GMT</t>
+          <t>Thu, 05 Mar 2026 10:43:54 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxQaTJidDdUdmx2eDdUbGhBZEZxNEx0X3NIeGp5S3Z6OXhmUUlFbm42ZkZRTE1zY0h0YXJ2ZXNua1hLUmZvcFhMNmVDY2l3LTNfUTFRbi1oR0hkTTNrVVRTcmo5aWtNcl9Pck45TTRzTkxZOFBKY0VyZE4tbEFDWnFzRWVYb19hMEtmLW40UUNuQU5EdWtEamFEcFpfcFUxbnJR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQekhHR1Y3eXo2SU41d1h0aTlmS0NkWG9UUWtHbDRVQVJrUlJjMW9VTjdZV0FIcks5QnV4d09XeHBZUzlwQzJqczBlakF1QklVV1B3OTBDbU13bFNqbUhHNmp2WkZyUmdjUTJIcEU1Y21XcEFiR1piRml2ZFZxZHNiX2Rpckg2NngzUUNSd19LRVoycXBuZEhqQmdaV21mNkctd3JrbFNlZFBXc3FRYzNTRC1OVXlEQQ?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1240,42 +1240,42 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46085.67831018518</v>
+        <v>46086.44715277778</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Man probeert iPhone aan te kopen via valse bankapp en vlucht weg: “Bij zijn arrestatie 1 kg hasj gevonden” - GVA</t>
+          <t>NATO's Rutte backs Macron's nuclear revamp but says US umbrella is ultimate guarantee - The Straits Times</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Man tries to purchase iPhone via fake banking app and flees: “1 kg of hashish found during his arrest” - GVA</t>
+          <t>NATO's Rutte backs Macron's nuclear revamp but says US umbrella is ultimate guarantee - The Straits Times</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 14:13:58 GMT</t>
+          <t>Thu, 05 Mar 2026 12:59:02 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgJBVV95cUxPeF8xcy0wTDFyQU5FTFJMdGRzQ2JMMFdrUEdJMDhQczg2SzNJeTBGVlpjeVFyWEd4UFQ4S2g0SmZNeDhacXBZOVJ4Y0I4bmJtQ0MwSEM2U1dyejIxY3c4cHh4QTRwZ3FpdFp4cDQ1NG1keGhTb0JlQWd5VmswdGJYVHlrejFGdmpRNzFHVVZWMkUtRm9fSXhMalRhZlN4N19FZUZkTnd6dUxsWVZkZlFzVUJoYURpekNyd1k1U05tbTVRMGtPMTFmYmVncVdEenlnMmFPSXoxMEkwaldXTkNVQ2xDNzNGWkU4V2c2TGh0TnBRcjJNZTFlRDJiRnpodmFKY2JFT0RPaTktcHZIUC0zNzlR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxNRFdDN25TY1M3X3J2LUNyOXdPV2dHWU80VHhxUHBtRFJDWVd0Ql94d3dpOGNNRnZMTDBIbHNPcDQ2UHJucWNqVGlJbkNqV1Fxb1hHV29adnlWeVNHSHVUM0VPX2xpSEJEMDFqMFBGTlBUYmk0NWJIclRRa1JpS1VBRXJHYjBQTExJN3ptWERsWTZ2a1ZlRVNLNGJZU3pQb2VxWENoLXdsTl83VWpVazdMTVd5TkZXR2NSNkZGdzRPdHdkU1E3cHAyM0YzZERqM052MHVLSQ?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1295,42 +1295,42 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46085.59303240741</v>
+        <v>46086.54099537037</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Ex-partner van slachtoffer Grote Markt opgepakt op verdenking van moord - Nieuwsblad</t>
+          <t>Highlights of NATO chief's interview with Reuters - The Straits Times</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Ex-partner of Grote Markt victim arrested on suspicion of murder - Nieuwsblad</t>
+          <t>Highlights of NATO chief's interview with Reuters - The Straits Times</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 13:05:15 GMT</t>
+          <t>Thu, 05 Mar 2026 13:34:14 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxOaEN2ek9pbmVQdzRUcm9jN3dob1dvV2JGa3VXbnhXdFU4WHJrcEZYU0l2c29nLTRpZ01TMUdQODJ0aDExblJKMnhUUDlZVEdEdGZRaWVfVnY5TUZCM241cllRUDViU3hsUXFkV0VXU2s5c1VkRnZZOE5XWEZscDVxeFpyVHpUbEpfUE5XemRjbTJUcDExV2FIS0ZjWU5kMFdkUXdqbGxRQmFzMjdKRlkxWUQtSUhybEFZZ0xXbnhYR01SLUwyLVR3T1l6NS1wYzZnbi1MY1Q2YlpUOXBJamlUVzlENkNPdVNoR1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQMHVuSWM5TXZWbG16VmZIT2EtVmY4OUZWZWltU2RyZGg0U3JCTkpNVnNscGhhUHZ3RFhxeEpVUmJXRUdFTnUyZ0IzSHo1d2g1NElSS1B0bFZvV0s3eGJiOS0xNTU2TDVTYkFFV2JvMEZMQWt2VVVXZmEwREVQVGQtQnJ1MFhFQUlTMHhZYUZyOEFfM1pf?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1350,42 +1350,42 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46085.5453125</v>
+        <v>46086.56543981482</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium French (fallback)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Twee minderjarigen plegen gewapende overval in nachtwinkel Ekeren - Nieuwsblad</t>
+          <t>Le Conseil Régional de Sécurité "afin d’évaluer les impacts potentiels pour Bruxelles" aura lieu ce mercredi - BX1</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Two minors commit armed robbery in Ekeren night shop - Nieuwsblad</t>
+          <t>The Regional Security Council "in order to assess the potential impacts for Brussels" will take place this Wednesday - BX1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 15:00:58 GMT</t>
+          <t>Thu, 05 Mar 2026 09:27:13 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxQNDNJOVhkVUVVWHJZYjdDcmtzeDBtWXRSMTR0N3RMOHdXbV90bGd1dnN1dENhYzBZX0hTS3VjN1ZkU2xFcjBZa0ttUDFPMUNLOWY5V1BTc3ZEMXhwaVA1R0JwMzFDa3N4VTVYdHFuWUxNWWRNcWRManNLbmItTUJtUDcyR3ZjMnNkQXlJRkxfMjdmMU5WQU4yVUtyRHgtdVQyeElSTGNFVlVhTkIzRXhEdFRfMDNVbWxKd1BkVTYyYndPU0V6Rmx2di1HT0RfN2JueERwcTg4NF9UemJzSnlxNGF3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxOWjdWYjBpeFFCU3pQU3lsNVhTM2tKUEFFS2stQXhsVWtMbkhRdjRUdU1ucDF1MkkzWGJfczVMcWFGaVZrc3VrQXBVWGpTVmREeDI3M2xlZ21Vd0NFX18waHVmNElJVEQxZzI5d2w1SVlYRzg4eXcwbHNDaGNxUDlkMHpKc1ZaZXY2WF83SmdUZkthd2hiaUdFcGo5czM5TWZoaTJELUxqc29ORHJCOWtZeUV3ZG43YXl3UE5kaHZpUzN2WWhCbHQ4ajBFeGU5cU1VYVBZTkExYktIR054c1R2OE9lNElJMXNNQ2c?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1395,7 +1395,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1405,42 +1405,42 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46085.62567129629</v>
+        <v>46086.39390046296</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium French (fallback)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>“Dit nieuws schrikt ondernemers af”: bezorgde Unizo-voorzitter nadat criminelen schoten lossen op bedrijventerrein - Nieuwsblad</t>
+          <t>Les attentats de Bruxelles : un avocat raconte de l’intérieur "le procès du siècle" - RTBF</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>“This news scares entrepreneurs”: concerned Unizo chairman after criminals fire shots on business park - Nieuwsblad</t>
+          <t>The Brussels attacks: a lawyer tells the story of “the trial of the century” from the inside - RTBF</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 10:37:23 GMT</t>
+          <t>Thu, 05 Mar 2026 13:44:58 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxPZGNOQTRyWVRtbmF6T05zTmYtS3ZIU0FSaVI5Q1drcFBXVFhqVkJ5UjFGcnVldUlBQ1ZzZkJXVTZWUEpiWXFTZ3B5S3FESklhcW95Q1o3ekZBemhERFMwVi10a3NoZG9jWFNQUVFIRGw3Mms3TGZKdndvaU1ZZDJpUzdVTW00YlFSc01RLUFWTkVWVXMzc05mTUJfU1JQQTRiMm8xd0NzMWZTZWVZbnlMTWtObFpzR0ZqWktDOWNYMHFDY21NeV9OTGJuNG94VkhNNXVjelhRTmRUblY4UXoyWUZGM3hLMlJ6UHJpYklXVl9KODRnRmxCaFNJc3prWjZTTE4taA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQRm5qeU1rVEVIelU3UWlRTjRfd05tN0FkS0dMMWxWdUpmVTE2cHRyRUJYMlVMd2Z4VXQ1elE5d1dXZzE1b2VkTlFUMmVnMVF1ZW93UGNSWFVTeEZCdnZyUktXR2hWcXI1cWFNRk1qdEpYRG1VdTFmSEhRTkdueUNrdWlsUGduNXJLSTFEY05CWXRuNDdnNTJIZWdxYVhPVlBzMnZtb3JtS2tEOTVKQWpvcVdtQ0dmblE?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1450,7 +1450,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,42 +1460,42 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46085.44262731481</v>
+        <v>46086.57289351852</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium French (fallback)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Mysterieuze doeken en luifel schermen vliegveld Beek af: wat is er aan de hand? - De Limburger</t>
+          <t>Violence policière : Un homme décède dans un commissariat à Anvers - Bruxelles Dévie</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Mysterious cloths and awning shield Beek Airport: what's going on? - The Limburger</t>
+          <t>Police violence: A man dies in a police station in Antwerp - Brussels Dévie</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 17:30:00 GMT</t>
+          <t>Thu, 05 Mar 2026 11:35:29 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxNbGEzQ1lTZENLQVJsb3dWbjhhdWZfUnZ6OWp1ZHY1MlhiVkM2TXMxM05TSzNjbDdfSkNONXNCMk5vakhjU21tLXVRWGoyd0tzcUotZDlTejBBWVZtdWpzWlNkaGdpQ096eXNVcjVaRzI5U1IyNE9BLVVpcDZEYXlwNlpHUUY5RDhBZ3E4V0pyLUlaN1BuUjRIZHFYb0NNQmt4Z2ZWSFJBVXdnaWxjV2MwUHdReFpkQnJaSGpLbWR3cEtKWFVHVUVR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxPdTBXMGxpUkx1QmpoRlNSMFdDMXRYSnBndUVKWjl4V2lmU19ydW5aTGhLQW9OMU9hOFNOc0llZUd0OFU1RGhjV2haQjV4dHlmRmpRUm1MSWtRTE9oeDMwNkIzZTBHbnZ6UlZFTVJGWDVadmI2SFZ2UWM5SXAtbldPN1FzZExDRnYzblk3Z3NmdkFRTXVNcjdxbG5jRGxsbVRWdEhiMDZB?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1515,42 +1515,42 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46085.72916666666</v>
+        <v>46086.48297453704</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium French (fallback)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>“Dit waait niet over”: Sarah Ferguson vreest definitief einde van koninklijk leven na arrestatie Andrew - HLN</t>
+          <t>Le Facilitateur Marchés publics durables reprend du service - Bruxelles Environnement</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>“This will not blow over”: Sarah Ferguson fears definitive end to royal life after Andrew arrest - HLN</t>
+          <t>The Sustainable Public Procurement Facilitator is back in action - Brussels Environment</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 19:03:10 GMT</t>
+          <t>Thu, 05 Mar 2026 11:12:19 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxQLWhMNGltQ2szaHRuTjJINDBseGM3TEdxNkxoUUhKV05vc0RPWXlQeDJXQm85a1dZX1Zxd0tvQ0NuVVdfRmxmN09kSDNKd0tFMTBFaG1lMGo2SHZVXzhZaVl2aTh0b0V2ZU1UblE0Y0lQaVk4ZXExNTYtQ05qTFY3SkNjT0pCUWFzN01EOFpoM3RFLWxpemM2QVdmODRmMUd0SEx6dVN1SGpKdEJYbjM4QllqaVFJVlhNSXhQVklIQTc5MVJVNHNqX1JULXhiRTFROXlF?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxNSGdLRmRMY0pueC1PRUZnS1NGVF82Si1CeW8wVnpZeEY4T3A5VzJ6V2xncWRSMTZRemh3QjZkWXhBSnNkNm5EeXNOOVdRaUNQSG9UbG14WVZJTUhsUTJqOFNVeGIyZjhYdllQRXUtOEhKeks1UC1IUVFyZUhKNGp3alhkOWZSMmk4VnQ0eHRXOXBUR2tpXzE0LS1CbmM4OVlMNkd0aEZyYw?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1560,7 +1560,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1570,42 +1570,42 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46085.79386574074</v>
+        <v>46086.46688657408</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium French (fallback)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Geen vluchten vanaf Brussels Airport op 12 maart door nationale staking - De Limburger</t>
+          <t>“Bruxelles, vous êtes prêts?”: Helena en concert privé, la Stib vous offre des places - 7sur7.be</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>No flights from Brussels Airport on March 12 due to national strike - De Limburger</t>
+          <t>“Brussels, are you ready?”: Helena in a private concert, the Stib offers you tickets - 7sur7.be</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 16:23:46 GMT</t>
+          <t>Thu, 05 Mar 2026 13:49:00 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxNMklHakQ2VFVmM2JCVDhJRlVfWFRkeTNKN0VNSVkxN0Q5TGh5azVOUXVleHZ2dHNOM3R6VUFUUlhTRVBUSUI2bVJiTHdLNjI1cmJ5MnYzWHdtMG1HaXc3ajRQM0NEQThwTmVfWWVsNWVpdWswN1pLNnNHZEhfN0ZwQVJHVG5JLXN2VWphODBJbjE1VVg2NHJfLVJzbm01a2JHa0dyVDBCSms3R1l5bEZUVmJWdzRmcG5qM1FiNw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPajcxNDVjOTV5bUtNUnN3OGJjaVBlQmZIdnIybVVXdE9aSkh5N3NmWmhpQ0lFMmlLQzh6OHRJM1NDbHh2WTNyeUF6Y1Q2Y0VyWUhGWjIxZl9Fd3J4ejJNVC1iQ3M3U1pxR0h1QkZqdFV4bXpWZlFlb1AxNlh1Vm51SGpCbmQtUlJiU2haM0c4cjBHSmpzSHJOWUNTa2lOX3JPcHdkZlpBbjlmQ1J2Yi1PLU1ZdjN3OFZvNlE?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1615,7 +1615,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1625,42 +1625,42 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46085.6831712963</v>
+        <v>46086.57569444444</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium French (fallback)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>As Israelis and Palestinians, We Shall Go Together to Brussels – Le Taurillon - treffpunkteuropa.de</t>
+          <t>"A Bruxelles, la menace est stable, mais haute, et extrêmement élevée à certains endroits" - La Libre.be</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>As Israelis and Palestinians, We Shall Go Together to Brussels – Le Taurillon - treffpunkteuropa.de</t>
+          <t>“In Brussels, the threat is stable, but high, and extremely high in certain places” - La Libre.be</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 13:04:46 GMT</t>
+          <t>Thu, 05 Mar 2026 10:02:00 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQamJub2NMM2dvT1JKYkl5bUNOa2stb0tBb0FCZ1AxN3BLV3NFcHdaQW1takY2cld6V2RVeUNyNVFvNDNFZ3VkVGRWblBDNktqdU5UY2E4YnVyYmpsN0x6dE1QZGxWOXpWc3NFc21nejlsRnNKWWFoQTI5RnhkMU1GRTRPbmt4RzdUU2w4QVM5YWNkNWh6Tlo4cA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxOOGUxcWdPU2ZiSC1TMmJ3NVh4YklCa3JwdTE3XzJCWWVibzNiNS1ETGtxYUMxQ2dSN1VmbWJuajBnOU9nYkw3Tll0WVlvLTNibW9XMWw5dEhxcjFwSGMtVy1sazJKaE91SG43am5PYVhkRkprbWFEUFB4N3A5T3pGalEtWWdkeU1hbVllS3dYSHZUQmNDYmtMNldObXRlZU9jZGEzR2toV2hkNkh0UEdIN2tZS3dDeC0yX0VjcFRYdjF0dHVMUkpVdFprVGFtdzZYV0lELS1ITloyMXYtc3hvUkRDTUZodmwtMklGTmM1cUgxTEVjNjhF?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1680,42 +1680,42 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46085.54497685185</v>
+        <v>46086.41805555556</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium French (fallback)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>The Iran war will be long, bloody, and ruinous - Brussels Signal</t>
+          <t>Manifestation nationale du 12 mars: les aéroports de Bruxelles et Charleroi fortement perturbés - L'Echo</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>The Iran war will be long, bloody, and ruinous - Brussels Signal</t>
+          <t>National demonstration on March 12: Brussels and Charleroi airports severely disrupted - L'Echo</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 08:20:35 GMT</t>
+          <t>Thu, 05 Mar 2026 11:29:51 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxPYnI4Z0dJSXREZkUwZGdCT00yZFpjM1VOQ2xLVTNQR1lmUTZ5ajNUZldiUUZfUnF5STMySzVSOXp1bTdpLTl5djFfOHNiNk5NWVB1TUpiSHBrakR2UW9yeWZtc1JlWlhjejR4NDUtc1EySnlhVHBNVk1rdmZYZ1lIamZybkw5QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-AFBVV95cUxQTWViYjY5SC1VVWxBV01DMVFaazU5Q2lEVnZRQXZ5Y29ITTl4M0U1N29Hb2s0UXcyaHBCbUpIMjhMaFB0bnlDZV9jUVVTdU1NZl9lOTZjT3l5ZUEyc1Q4WTdnNEh2bmMxbFoxaGw4TUJDSjcyTXNDaWtGdi0zXzNMTmJuYjY3UVQwdFVsQmJ2djdPSnpLeThad09VWEN1Y2UyRVJibmd0ZVVsamhYR2tybEVrZkYzRVEzMWduVkpDN2wzcmhXb2pIOU42Z1NCTVlqRGV5dmw5dU5TUEpzZTFjYUd2YnFJLXdaSnVGS0I0ZDAtY2xkXzVmLQ?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1735,42 +1735,42 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46085.34762731481</v>
+        <v>46086.4790625</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium French (fallback)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>UK counter-terror police ‘arrest partner of Labour MP on suspicion of spying for China’, reports say - Brussels Signal</t>
+          <t>Bruxelles : 100 nouveaux kots pour les étudiants aux revenus modestes - Le Soir</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>UK counter-terror police ‘arrest partner of Labour MP on suspicion of spying for China’, reports say - Brussels Signal</t>
+          <t>Brussels: 100 new kots for students with modest incomes - Le Soir</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 14:41:25 GMT</t>
+          <t>Thu, 05 Mar 2026 09:33:56 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQQWVld3B5OENWME1yUTlCQ21OS0lUY2JOY0tkWmdOMmg1T2QzcjIxcGpWdzdYeHgtT2thUGV6VHJMdGNQaHRwNlBjRDRISlB3bkc0RGk3N3VlMzVob1FtQkFpblRsTVd1ZG9tNE1YcWlzRVAxRjVxSWVFS180SWNVT29VWUFVSHpqdV9VblpOVV9ndGwySDB0VjhMdUl5ZURvS2tlOGhFeU9PMnFIRzB0OWdVOHZscTVmdHk4YVgyYUdzQVhHeFFIZGhZRVI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNWkduYlNTYllkYWtoNW5EQkdmM0hVdi1jTzlYV1VSQUpoNVM0VDZSTDdxdEpiajdfUUFTQzRYSXhrWW90Q0x4Y1AwQ1hORjgwT2REMF9scXpTLTQtc09menc0LVJRblVKd3VRVWFScy05OFJ0QzUwamRQSVhucUY5U3Q3UXJrcGxBZmFoY3hncXhaeGUzX0RsaXZ5SVpfZUlfMG5Pb1A0eVFHeElYQmdCd3hFMm9DZw?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1780,7 +1780,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1790,42 +1790,42 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46085.61209490741</v>
+        <v>46086.39856481482</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium French (fallback)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Pakistan confirms airspace fully open amid fake news reports - Travel Tomorrow</t>
+          <t>Inédit à Bruxelles: Auderghem s'associe à dix commerces, la STIB et la police contre le harcèlement de rue, "l'idée n'est pas de remplacer le 112" - L'Avenir</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Pakistan confirms airspace fully open amid fake news reports - Travel Tomorrow</t>
+          <t>Unprecedented in Brussels: Auderghem joins forces with ten businesses, the STIB and the police against street harassment, "the idea is not to replace 112" - L'Avenir</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 09:43:42 GMT</t>
+          <t>Thu, 05 Mar 2026 12:52:00 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxNcDV5Nng5NkR0d2dBLThJRi1pYXZvTDRRNG45SW9sSkwyUGtOYUJCd0tNRGlBZmE5WFVNcDhyT0ZSbzBBWGR2cHFORHJZbUx1R0daSUNUc0hKTFJ6bVFITmFIbkNVWHdvdXJzel9BV3ZaUVVkMExwaEl2dTJTdHA1c1ZyQWtCaThKVF9sdGRzS2FnZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizgJBVV95cUxOb19pczBBYncyZU1kOGZweTRjaEtjVUVFX0FTZFAzcjZVRnA0S2dEdWFnZHJFdU9Wci04UzdvZG01VENzRVlybllBb1VDeWt3UVF6VG5meVNMQ3c5bVVfZHJsQjZJZGFkdnFpT3dOeHB6ZDZMeTlTNm1PVXpYMURjVUtZNE1FQkctS3FIREFmYjVkalpXRi1YblZvcHJOX1BqTktIS3BHdzlQMFRNQUc5OTFmdVZkWXNzNE5CQU01dVZab0pOYldhTmVqd2FSWWpOa3hQZUszUldwUnNMWS1acTRwakZubDNCaUZCWnpDTEhlMUdweFFlbW82ZU5hcFlTWTUwNHMwVVYxYmx2bzlqaFpxbE1ZUWd2c0F2QnJ2ZG1SaWhDb2Mzb0l2SVBKQ1JuVnFjcTZnSFdvZTVnN1NWb1NLeHprVFZ4WW5fM3h3?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1845,42 +1845,42 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46085.40534722222</v>
+        <v>46086.53611111111</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>High Level City Belgium French (fallback)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2 twintigers krijgen werkstraffen voor tientallen graffititags in Hasselt - VRT</t>
+          <t>Rénovation durable du siège ING Marnix à Bruxelles avec Rockfon Mono Acoustic - Architectura</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2 people in their twenties receive community service for dozens of graffiti tags in Hasselt - VRT</t>
+          <t>Sustainable renovation of the ING Marnix headquarters in Brussels with Rockfon Mono Acoustic - Architectura</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 13:31:44 GMT</t>
+          <t>Thu, 05 Mar 2026 12:52:29 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxQNXc5M1hIZG1lamVwVzlxLXhzTl9LMFRfXzlCdzgzV293ZXVWRnRaTHk2VGdqQ25fT2YyazdjY3prUDRYcFAzYkZFQ0VxYmhEejlVTmg4eDJfQ0hrWmpUV29Wc3JqdmFCWEZNUk1PblBVaWJ4cEQ4N1hjbVF4SHBLdGJDR1ZQdmVpaHdRWEtGOXp6VmJxRlRTV29VaUpLSlZhT2ptakxIVjY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxNenFFZjRYbFJiV0tsM1FGbDUwVkZqR3dGMGFZcEcybzJkVkE5SmdLNVhPTDJHei10TThRVFBfRnJOYWdRY09ydDRWSzN6a0FKSXRSZ1hvSjF2RVRfbzhzaVU2aTlGLUZaSVptNlJtVkg0cjF3aHNnUDNTcnM0a1NWMHBYUndjVlZBbVhMeGJqQ0V3SXJ6bG5HQVBRQmwxWWdzYjh0cUhlMlRmS05IZWdGZlJTLXlqR0V1M2c?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1900,42 +1900,42 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46085.5637037037</v>
+        <v>46086.53644675926</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City Belgium French (fallback)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Statistiques Royal Knokke FC - Tienen - RueDesJoueurs</t>
+          <t>Entre clubbing et jeu culte, ce show immersif de 3 heures à Bruxelles est l’expérience la plus électrique du moment à partager entre amis - Bruxelles Secrète</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Statistiques Royal Knokke FC - Tienen - RueDesJoueurs</t>
+          <t>Between clubbing and cult game, this 3-hour immersive show in Brussels is the most electric experience of the moment to share with friends - Bruxelles Secrète</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 08:57:21 GMT</t>
+          <t>Thu, 05 Mar 2026 10:01:08 GMT</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxQY1Ywb0ZIeXVITXdROG5ROExUZ3ZhZ0dIWWhpX1BCdXJnaXgxem53MkpBQXNqb0tFOFNZbUx6LVhsTVMtamlidXRPZVg0YWpvSDJrVXREVkVaMFFiN2YxMGV4Y0JGZjFlZEpEN19NbndHQlZpOERoZmFUdVJETFZ5T3RBRXFBTkk5bHRIVzZaTW4?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE04Y2dfVmtRMmZkMUV4VThJMjJTbWwwMEd5Tm5mc1gtT25VUEd4QjBzUVBZUjhVeWFsai02Q0R5eGFtNzN6YXp5cE4tNEp1akI3MnZRaktyUHZ2c0kzZXY1dE9LYWktX3pvcWtWNEFXZEc5ZkotVDV4QUFxTQ?oc=5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1959,38 +1959,38 @@
         </is>
       </c>
       <c r="K28" s="1" t="n">
-        <v>46085.37315972222</v>
+        <v>46086.4174537037</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City Belgium French (fallback)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>"Vague brune" en vue aux municipales ? Ces chiffres qui montrent que tous les voyants (ou presque) sont au vert pour le RN - La République du Centre</t>
+          <t>Avec le printemps reviennent les Recyparks à Bruxelles - RTBF</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>“Brown wave” in sight in the municipal elections? These figures which show that all the lights (or almost) are green for the RN - La République du Center</t>
+          <t>With spring, the Recyparks return to Brussels - RTBF</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 03:31:00 GMT</t>
+          <t>Thu, 05 Mar 2026 13:44:32 GMT</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_wFBVV95cUxPcTRJcFlaR2ctSFdTLUg4X29weEdjMmd4M25ieVdKNXZHQklkd29lWmdOZE8xX3FyTTNZSVh1SVdlUFR0d0FVWnNhRnhXRzdaRDIzS2QybXJRWEZGeTFoaDZPeVpRbXZrQUpsTVFSbUVuWUVoNURpTUh0YjNETGVxa2piOTJFZmZFR24yRUYyMzVZRjV1aEc3c3dmM2xfTFA5anNYRlVUSjdRRzhBSW54RzhNcE4zcGdlNndCdmhWVFBKTVp1LUw5VFlYVmhqRlJqQV9UaURZT21feXRobTQ2YjJrdzJOU1hLWFgzSjFqN3JubGFnMVpzLTBua1BlSjg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNb3AxdENtVjFmVjJ2MG4wa0JITHdCT0JBSUVOcnFWeVJGTU5pOFlndmJqWFhSekpyWXMydHdwZ1hOeTBselRYem0zZld1UVd4YmdpRDNpMzNVYVFHRnlUTVhwYzkxSUhUOGdwUUhBMGJReWRBSmlOUDVRUTZuWWdtRlBURUxkT2VZSFlVNGh2TGZqM083VGc?oc=5</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2014,38 +2014,38 @@
         </is>
       </c>
       <c r="K29" s="1" t="n">
-        <v>46086.14652777778</v>
+        <v>46086.57259259259</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City Belgium French (fallback)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Prison : Avant le « masterplan », le gouvernement a proposé de détenir des personnes sur un bateau et envoyer les détenus sans « titre de séjour » en Estonie - Bruxelles Dévie</t>
+          <t>L'enfant de 7 ans renversé par un bus TEC à Bruxelles est toujours en danger de mort - La Libre.be</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Prison: Before the “masterplan”, the government proposed to detain people on a boat and send detainees without “residence permit” to Estonia - Bruxelles Dévie</t>
+          <t>The 7-year-old child hit by a TEC bus in Brussels is still in danger of death - La Libre.be</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 20:00:29 GMT</t>
+          <t>Thu, 05 Mar 2026 11:19:00 GMT</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikwJBVV95cUxNTUNCbUg0RTFMOUQ2bmRvYVh0ckdyQlNZMHFWVWdfZjdLckVKOGZnRnM1Rl9DSmNzWnVPYlBSMGJSZFhJdVpNa1lETG1mNkNkazJKVEVRRUFDWWVkTjZJdmY2MndMVXBWYlFIYmNqOXN1a1FVcy1oellTZFBjRl81UEpzaFZoV3UzalJTZDFNYkRzRnkzS1lYdXdBSXVPTkxiWjk4Wkk1eVdGeWNJYnl2ZnR0QTUxeUVSampKand4OFBZcVY1OE5OU0F6aFlRekNUMlIxZE1WUTNtQ3E2b1JxVjMtWUFmYXFXSjR3Qm5Fb3ROVGs3bG8zY0NrRWpIM0p6bGFjd19Td2N5alljN0NIV3FNOA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi9gFBVV95cUxPekRWV2p3WERVU3hpUzR2c1BiRjc1amFMX2pwVmVMOTZ0MktFUVI5enpiQVZIdnBzVGE5RFNzR01LNVhwRXVyV2VLZWlRVzVtdUZfZi1hWE9CSVJ5WGlNNTFzUzRLU0JtckNkaDR0bUxtcUFZZVg3bERZS21JSTRnMDdqUlpnc0l2TUJVM2JGX3duak42NVc4WWtWY1pIVTJXTFBkWFc3RUozdFRtX1VjNmlxY1Zra1ZvcmpfbUQxQXUwN1hqc2FIWlB1cnN2cmRUSV80NDlwaDV5dkFFVHBnYnp3SjVwcUNxV3hfeHV0VUFsWXU1Nmc?oc=5</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2069,38 +2069,38 @@
         </is>
       </c>
       <c r="K30" s="1" t="n">
-        <v>46085.83366898148</v>
+        <v>46086.47152777778</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City Belgium French (fallback)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Qualifications Euro 2026 de handball féminin - La Belgique décroche une victoire historique face à la Macédoine du Nord - DHnet</t>
+          <t>Le Centre Jean Gol conteste son exclusion de la Foire du livre de Bruxelles devant les tribunaux - Le Soir</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Euro 2026 women's handball qualifications - Belgium achieves historic victory against North Macedonia - DHnet</t>
+          <t>The Jean Gol Center challenges its exclusion from the Brussels Book Fair in court - Le Soir</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 22:06:00 GMT</t>
+          <t>Thu, 05 Mar 2026 13:24:30 GMT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogJBVV95cUxNMlZCMFgyNEVIMExLSHk2S3BRN0c2cHdtMGFkbTdKNEtBRUhyWW4tMzNxNEdnV3hsUExldHVWdGdQODQ2eVlPSEtwNnlxSndtcVhyX0hGa0J4eHZPSjFpQ2s5R0VHR3E1aDBudjJmTWNkWmVyU0VVcEVvalVxVFhpZDNZc1kzUlFwdGNkM0ZDeUc5LWVCVWN3TGg3TXdvamphR21odzZkNktUNjZmWjYwOF82cjFyeEpicWRJdnh0amtCSnBtRXBEMjNvWmhPUjJZM3kydGNzZ05HV1hEM2phVHhTUmx1OU5DTmZ4TjJOcEVIWG1oemxrVUdVRVg1QWhqcXNPUTFIQ3JTamRWSVh5WFVGcGRLcUN1bUNUU1RLdWp0dw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxQdjQ1cUE0b2RpNlFweEJVWmlQaFV0clhDSU01ZExLQWZnbTc5NnFVUTdaMERUYjVDRUJuN282NzFCbmpJeW5IdEQ0cjgwRTFQZHZDdXdwLWtDdXRjcUY5ZVBBZDJHOS1WbnYzYkFaOUd5TTc3MnBKcVZBUjFYSWswdWQ0cGlfRVhlTzJzUTZ4ZHZJS0lMX2VUMWhUS2otQzJmRzJKdjRSc2luWmJRdHJKU1ZEdXFnZ1RVeUUwbVNNTjY?oc=5</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2124,38 +2124,38 @@
         </is>
       </c>
       <c r="K31" s="1" t="n">
-        <v>46085.92083333333</v>
+        <v>46086.55868055556</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City Belgium French (fallback)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Une grande première: la Coupe du monde de cyclocross va faire escale en Écosse - 7sur7.be</t>
+          <t>Attaque contre l'Iran : La Défense rapatriera des Belges coincés aux Émirats arabes unis jusqu'à Bruxelles - BX1</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>A great first: the Cyclocross World Cup will stop in Scotland - 7sur7.be</t>
+          <t>Attack on Iran: Defense will repatriate Belgians stuck in the United Arab Emirates to Brussels - BX1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 10:15:00 GMT</t>
+          <t>Thu, 05 Mar 2026 11:55:00 GMT</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQV2I0NHFLMHZJTmdoR0ZjSkxId213ZlVqTzBLSWJTRDJTV2FtWl9pdm1IWjJSZ0ppODhESlVfRlhTdXEtY0IyWVU0NTlRUDU0WTRJSjZRb1VxY2tXa2RDNDJNempQa1NwTW02Q2kzNHBOb2tIcE5yd2ptMXRUUXNLUUlOWEtCTHlwLW0wT2p4OE1yTDdlWUFVbjNHdEZHaUlRM3BaSEVJZWUwMmZQdEkzYTJCQVpSRjlm?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxNWFlvLVl2eE9uZm10WV9XV1E3UjV0c2xpYmVOLTgtSzZhVHJNcWpKaG5uWXZFT09OeWNIZnRfVFZtVWRaekN4VDRraTFhN0Y4dnBJSUxlUFlEYkhIUkZMNUFhckJ6NU1RT3lramk1SXBkR1ZfdHp0WWEtWEROWmYwdVE1bkpMTk9FbGlsMWZQQW54X0IxLUVNcC00VDZJNHVlV1R3aXNsNXJEMnlZM3VQSk8xSmFXRGpQSF9hb0NFR1ZqV1pfOFFtV1FfemtvQ0k?oc=5</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2179,38 +2179,38 @@
         </is>
       </c>
       <c r="K32" s="1" t="n">
-        <v>46085.42708333334</v>
+        <v>46086.49652777778</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City Belgium French (fallback)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Météo Belgique - Toute la météo en Belgique, en régions et communes par communes - RTBF Actus - RTBF</t>
+          <t>Médiathèque Nouvelle fera des adieux festifs au public lors d’un festival à Bruxelles - RTBF</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Weather Belgium - All the weather in Belgium, in regions and municipalities by municipality - RTBF News - RTBF</t>
+          <t>Médiathèque Nouvelle will bid a festive farewell to the public during a festival in Brussels - RTBF</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 19:16:55 GMT</t>
+          <t>Thu, 05 Mar 2026 10:04:31 GMT</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiSEFVX3lxTE14UV9iaVNZdjV1X05LRU5DcHNONmRZaXA4YkllNURTWm1CVGoxazBIT2g2V0t1TUZKbTljdjFsS1NrMDh1aUJqaw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxNRGJhTnJGS0FxTWdVM3M1YmFNc2ZWU0lMUmVGZ0UtOWxyMGFzX1JMV1prMHMwZUZUajRidUlyMWpZWjE5R1VJZEhyYVlFVVVSUGVDbHdwWTlWZjQzTU8zSTVpNURQWE1QczJxUm1YT2dCT0cyTGtTZU9YVU45dmltZ3loRUttVGIybG5IRFV6TXdMTVhya2UyR2dvd0s0VzcxeGE0Z0JoOHQ0Z2IyUXZCU0UxUlBVMVZyNUZaY2xnZw?oc=5</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2234,38 +2234,38 @@
         </is>
       </c>
       <c r="K33" s="1" t="n">
-        <v>46085.80341435185</v>
+        <v>46086.41980324074</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City Belgium French (fallback)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>La Chambre votera la semaine prochaine sur une nomination à la Cour constitutionnelle - DHnet</t>
+          <t>Les Best Brands Awards 2026 seront remis le 12 mars à Bruxelles - pub.be</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>House to vote next week on Constitutional Court nomination - DHnet</t>
+          <t>The Best Brands Awards 2026 will be presented on March 12 in Brussels - pub.be</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 16:25:00 GMT</t>
+          <t>Thu, 05 Mar 2026 11:56:29 GMT</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxQaERlNFF6b2NZLXVuTmdCSUZDd042ZlVxMXdTUVFhSzRxUG9hMC1jYnlPUHota0c5VEd4c09LV1dhN0duRVVtMFBldTNZZ3ROR2pjMzhienlxWkxCUFZZNWFaQWVRcUVEcWJsd0stdWM4VVZqLVFhX24tNDNXRVk3d2FVUzlmb0NZNElScTRjRDhURVJzT0tkb0RVdFljNksyZmZHc1VXdXkyVU9OM2VQYkNfakNuTGNpTGpoMndDV1pSNDNaT25ZQks3NE5aYUlGSE5UeHZKdFpSb2s5SG5jX0ZabGxySFlVLXZvQnBPeEFZSlNYNlNN?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxPakg2RDFaQjJYc1NhUWJYNEdVWlhxZUthUXlGUGpGbzQ1eTd3amFIWHJMS0t4eTJIUTFmVngtT1pPTVZiT0tmckFoZzN0ZHFLYTByNXVfanFwbjUtVjhoSktXSDZhd0hqTVZKaU1XcjRQNmZqTzZZVk1MVGx6NkR6MU1aVU5hbUR2b2c?oc=5</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2289,38 +2289,38 @@
         </is>
       </c>
       <c r="K34" s="1" t="n">
-        <v>46085.68402777778</v>
+        <v>46086.49755787037</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City Belgium French (fallback)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Rugby : le dénouement du six nations entre les mains des N°10 ? - francebleu.fr</t>
+          <t>Le Centre Jean Gol accepte la main tendue par la Foire du livre - 7sur7.be</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Rugby: the outcome of the six nations in the hands of the No. 10? - francebleu.fr</t>
+          <t>The Jean Gol Center accepts the hand extended by the Book Fair - 7sur7.be</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 17:00:00 GMT</t>
+          <t>Thu, 05 Mar 2026 14:15:00 GMT</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxPNnU0YmpnZ1pRbTJVSFFJNHlTaWt3X2xTR083dnRjVWQwM051eXFyUUlhMlBQZFFLZGgyQXM3MHpTaTNJNERoRm9SNkxXVEdVLWRsMlJhZ2QxdXdZMGJQNTdBTkt1RjFEZGxKa0VETUdsM05pRzVoUnV1OXRBT2puTVZGWFZqQXMxd1VrS2U0YW5IdHgyRXpVSTAzX2d3WlhJWVVxd1FKRC1mN1Q4dWRJOTdCTUZmdm0zZkY4UE9yOA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxOYmhrWDJuQzdKVDJ5LTRpYWdfUDNETmZyVF9ZcjlkdHpsdmotTU1sV0RqNDJmS2sxTmZpRlkzR3d3VG5HSl95blRoNV85dk5lb3Z5RUNEaHQwWHlRTC0yYmhBT1prekU0TEhodG1jcHhpZ0k4UkVGSzQyVVZjbkMtcnVjbXZUcFhiQXlMWmxtd2o5ZHhjTXQ3al8yWkk4R01WYnhEQ1ZB?oc=5</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2344,38 +2344,38 @@
         </is>
       </c>
       <c r="K35" s="1" t="n">
-        <v>46085.70833333334</v>
+        <v>46086.59375</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English</t>
+          <t>High Level City Belgium French (fallback)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bomb OR explosion OR shooting OR stabbing OR evacuation OR police OR arrest OR threat) AND -sport AND -football</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Fuming French farmers camp out in Paris despite government pledges - The Guam Daily Post</t>
+          <t>Le Parc Ouest de Molenbeek demeurera accessible au public de manière permanente - RTBF</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Fuming French farmers camp out in Paris despite government pledges - The Guam Daily Post</t>
+          <t>Molenbeek West Park will remain permanently accessible to the public - RTBF</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 19:28:12 GMT</t>
+          <t>Thu, 05 Mar 2026 11:48:32 GMT</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxOZWVoVHEyYlhGNEJFUndjRmN6b0NDSU9Xd1ZjYTdyMF9hbDkxbG93Tm52SEZZZ1BWdzFNdHJmUXB5cHhyUFdlZ2pfd3ZxRUFaZEpWNnV6Wl9SN0JHQl84QkZ2dzZ0Qlppak81d1FIVmpJNFhLbWxDRk9xNmh2blJ2NFFTU2MtWjhkUXRPdTNJOERHd0lOYXVsYlhuSjNYZmtVM0laM0RrNWF6WTd5bTJhM0dZakw4Y19sMTAycFVObzdNNWFrUUlveE1CWmRmM1NlczFOTkRETW1CU2k3TVUtZGZ4WmRoa2FSQ3pv?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNUUNVOG55OEtBNXFkSTdWTHluaWpQeTUwUUpIWGlKYW12N0NNSUpxQVJQYTcxSGFMSmhZTDgxSlVYaV95MVpjeWs0cjlpaENuMDhBU3k4M2k0X0tMOFNzYkU5S2ZwenJfNG01bmRXUzQtc0dDRzludGhmWFdXMVZwNmkwMHZmdGxudTV4amdHQTdRampMU0hlWW0tcGpPMGRMd0p6Z25pc1FnTGNuNW8zUEFyMEVzZ00?oc=5</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2385,52 +2385,52 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K36" s="1" t="n">
-        <v>46085.81125</v>
+        <v>46086.49203703704</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Brendlorenzen: 17-Jähriger liefert sich Verfolgungsjagd mit der Polizei - Charivari Würzburg</t>
+          <t>Maasmechelaren worden online bevraagd over parkeren - HBVL</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Brendlorenzen: 17-year-old chases police - Charivari Würzburg</t>
+          <t>Maasmechelen residents are asked online about parking - HBVL</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 14:00:00 GMT</t>
+          <t>Thu, 05 Mar 2026 13:07:01 GMT</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxOMlByX0xhT2xSOEZLTWpXczBQVnlCVWZ1T0ZacGJ6Wm15Z3AxS250RVZBVHczVDkxNTBtQmJDZ1V5MTVNc1N3MDlZWmpUSFRGQmZyckM1SEZ4TkRQbXBybHhqUG5fcDI1QVFnZ1dmckRPNWpiU3A3OXQyV1UtLWxBaFZLQ1dyWjRjMHdHbE5RSlFSU3dQcjF3RnJZeHF3RkUxc1FnOEQxbzV3RjJ4?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQUjY4UVB0MnZjN0hnUmhCTGF1RHNyMzlrVGk4Q2JvV0NGb2h6djZFRHd3NktaaW9nYmNOY2Q2V3UzY3FJM3RISXItenBrMEZ4ZVZhQURoVkZtRGpiVEo2WTl1VjZoUU8wT3ppV2ZGcjNuVlRoZW5WbXl6Nzl1ZWZJNHVfREpldW5oSXp3am1tMVd6OUE4Z3A2eFRsNVVITlh3NUxaS0FFOEFISkptSVBnd1h2aw?oc=5</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2440,52 +2440,52 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K37" s="1" t="n">
-        <v>46085.58333333334</v>
+        <v>46086.54653935185</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Polizeibericht: Krommenthal | 13-Jährige vermisst - Wer kann Hinweise geben? - meine-news.de</t>
+          <t>Theater over onze angst voor de dood komt naar CC Hasselt: “Voorstelling gaat uiteindelijk over de tijd die we nog hebben” - HLN</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Police report: Krommenthal | 13-year-old missing - who can provide information? - my-news.de</t>
+          <t>Theater about our fear of death comes to CC Hasselt: “The performance is ultimately about the time we still have” - HLN</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 13:44:53 GMT</t>
+          <t>Thu, 05 Mar 2026 14:42:44 GMT</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxPSGt1eXRTbXRLNE1SZnJnYUJHNHFpa2NSV25oWE4tQ1EyYmh4N0lCX1NicDFVSTcxdDBNVEZPQVRYUm9LQUZZcjdoODlqQjd1VkI0LWRNSkgzOVhRaDBHUXYwUTBMYnZtTm12dWw5SWVCSmlBNVdJbV9BRnAzVXY5d1Mwa3FDQW5SdjJUSXBUSGZLeUp5Mlpaa1FjQlJWdUZlN1pXVGZjekhGQzRNSFY2RVJoTjY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxNR0VjTmo2b2hjTGVEZDJDamwxTlo0ckVBNGVuSEltVEFQUTlibzhrNTJkSUhnR2poVGhCRjZOQXJ3WDZFaVIzcGhsdHc2SHZrQWhlNFpNV29yZWI2RDZhb0VNOVF6dV9YMDBKWDFlQmZ3Q1BfMFRYbU40a2xfVXpKUVdCZ3lmaU0xZVlxeGh5eXdDUzJOckxEYk9GeHBhSW5aekRWdXFGQTNpbnltZFFIWVRWT0RyWkNxSERFRzBPR1o0WVNVblJFemFtbTNYYU9PbkZxQjJSbDZ2djE1SmhaSGx3SDJKV0t4aEZULQ?oc=5</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2495,52 +2495,52 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K38" s="1" t="n">
-        <v>46085.57283564815</v>
+        <v>46086.61300925926</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Stefan Weis wird neuer Polizeipräsident in Unterfranken - Osthessen|News</t>
+          <t>Filmopnames met Charlotte Timmers voor nieuwe “spannende fictiereeks” in Hasselt - Nieuwsblad</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Stefan Weis becomes the new police chief in Lower Franconia - East Hesse|News</t>
+          <t>Filming with Charlotte Timmers for new “exciting fiction series” in Hasselt - Nieuwsblad</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 23:00:38 GMT</t>
+          <t>Thu, 05 Mar 2026 13:52:50 GMT</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxPVG82OURkbVFCcklEd2o1aE52bXhueVFuMXJPRUlXb0k3aTFEMzlaNnhBVFdQUFdBX2xWMm9xS0NvTTBfSmpFdU1SRE1vWnlGVUNNZ1ZHRFBhWm9uQlp3UkdEcjVSaXUweWs3TnJvMUhfQ1dMUjl3WTVLMGVWWS1jeTBmcWxPellOYzMzaFlaZWtaWTV6UVV1bk5VMFA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOU0c4QlVSb1p4TzhubGwyWDZqYkZRZEtrMmZCSmliS3g5ZDZYS3pyay1LNFZpRENKZ2E2Z2pSR3IxRThONmg5RDlEUk1sNy1MeHdDRUdLRHY2ODRUZFdRSVdISzZfd2drMjBDai1wb2o1QlhuQ0JMUFpDS0I2djhBZUE4M0piam1aODc4SndLUzhFWlBGRHlnaktPZ1czWnJTZkNKOU1DR3oxcDhlOFdDc0ZRbjltNjMwRTZxaTVRWFNfTEU1T2hKV1RsMG94ajA2Sk94bDcwQkY?oc=5</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2550,52 +2550,52 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K39" s="1" t="n">
-        <v>46085.95877314815</v>
+        <v>46086.57835648148</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Kitzingen: Herrenlose nasse Tüte und drei Unbekannte beschäftigen Polizei - Radio Gong Würzburg</t>
+          <t>Grandbrothers verenigen klassiek en elektronisch in Brussel en Hasselt - whathappens.be</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Kitzingen: Abandoned wet bag and three unknown people employ the police - Radio Gong Würzburg</t>
+          <t>Grandbrothers unite classical and electronic in Brussels and Hasselt - whathappens.be</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 13:15:00 GMT</t>
+          <t>Thu, 05 Mar 2026 09:29:52 GMT</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPay1CSjA4VWZzbnZsRjhMZXVram52bGlHeWY3ZUJ0NjhGc19HMWlYNFFWVnNTcEc5X0NvbWtNVGQ5dTBBQWN4WnVZb09lbHY1QzhrSTNmWWtrUzFIZDBNY01fM0ZCR1VtWVRlQVFLWGNBWExlQTJITkQxNzg0T3ZkQXFSZXNhaGt0TXVZYlg5Ymp1X2FpeWoxNnRjNlFJRXJQVWQwdDF2dDJPMDFk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOdWJwR01POUpWUDlVMXFpM05EMlRTdlBEYXNDV2NPOHctc1pKR2I3M0tLemYyRHhBYmFmck42ODBsU09pbzRqaE9kNXZSOG9LM0pTRVlRREN1bW10WXk4V3R2NXZSNlRFUFNueUlZREdBMUl2OThNYU04X3NrbjZJczlubEJ2VDdKdTdjUkxSeTFCOTVGaFlMOEFIczA5UzJfeEE?oc=5</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2605,52 +2605,52 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K40" s="1" t="n">
-        <v>46085.55208333334</v>
+        <v>46086.39574074074</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+          <t>RESTOTIP. Gezellig tafelen tussen de bedrijven bij Het Cordaat op de Corda Campus in Hasselt - HLN</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+          <t>RESTORATION TIP. Pleasant dining between the companies at Het Cordaat on the Corda Campus in Hasselt - HLN</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 03:02:51 GMT</t>
+          <t>Thu, 05 Mar 2026 10:03:19 GMT</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE03RUZJdVVWTG5jTlA1R0dmc2YyQ3Z2S1ExYmhkN0FENFJGamUwenJsSFFPWGpKc3B2aFBaeHRYVDR3aWM1SXg0YWZFVDk0N3d4a0Jz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQNURtcTYxd0E1ZU93alAtNUNMYVozS1pqTl9JdzMzZU0zUkdkVEtBeWNPM2F0d2Fzclc2UktPUXVpSTVTWkxFRUhadHNhbDNpaUo2NUVkdnVIWmNsV2hucVNtMjI2RVl6Rk0zNXNDVmtsX3FMOVJDRmNkN2NzU2pzb1NRdFdSQXFYb1BDVFhGRHhDZWZRc05KdVFSYXgzYzJvNVZweHRsR1k5cXFERG1uNjNCcmh2R2JFTGNpNEpaME5zcVVXcW5z?oc=5</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2660,52 +2660,52 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K41" s="1" t="n">
-        <v>46086.12697916666</v>
+        <v>46086.4189699074</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Hundebiss und mehrere Sachbeschädigungen in Würzburg - SW1.News</t>
+          <t>OPROEP: Zit jij morgen op repatriëringsvlucht vanuit het Midden-Oosten? - HBVL</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Dog bite and multiple property damage in Würzburg - SW1.News</t>
+          <t>CALL: Are you on a repatriation flight from the Middle East tomorrow? - HBVL</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 12:35:01 GMT</t>
+          <t>Thu, 05 Mar 2026 13:53:20 GMT</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxObndrOEIwTm5pWjU4b25EaHRKRThqRGU1WUFTdldNa0UzQ043ZGEySnFnX0JYVkppSDlSbEc2Zkp4RWhuQmg5SDk1Y2NQOW91YnM2NjJRTXpFNDd2LVM3RU9kVGhYVUEtSjA5Ml85UGYzTXZHblh5V0UwRmJNRFBPN2lsNWtmT0QzQmt3SzRNVFBFa0w3SXRB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxPSXh5ejNOS1Z3STRIM2lvcnk1QVFTZmNHSlJhQjJ4aTRTVmRZMnNXVXdaLWtWZWhXUFZnUWdZTm5qWE9KMWlMOWdYeHdaUHQ0eUUtcDNtQ1ZCWGtlTDJ6STY0S25WdHNmZm9mQ3lpQzV2QzVobTFTcktUaG9xWjNJSk9fVVFYaE13WDNwUFhBcHBxamk4ZjRCVms3YlRaN1VtbkhucWR1NHkyMzBad2lIdkJCU0ZqUUxSSUVaUXdMMEl6M1hT?oc=5</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2715,52 +2715,52 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K42" s="1" t="n">
-        <v>46085.52431712963</v>
+        <v>46086.5787037037</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Wiesthal: 13-Jährige vermisst - Radio Gong Würzburg</t>
+          <t>Niemand draaide voor Genkenaar Aron in ‘The voice’, maar nu mag hij optreden op Het Schlagerfestival - Nieuwsblad</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Wiesthal: 13-year-old missing - Radio Gong Würzburg</t>
+          <t>Nobody played for Genkenaar Aron in 'The voice', but now he can perform at the Schlagerfestival - Nieuwsblad</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 14:10:00 GMT</t>
+          <t>Thu, 05 Mar 2026 12:00:00 GMT</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE9QWEtqdUh5RG9WRjQ1OFFtR0FtTC1lUlhSaXl1Uk5fdUVtWW1RN0VOY2c5ckxIZTdoNWYxNmVxRGZJTEQxd2lLdzRkZ1AtMmVSSHpia3NqSWNtNTktLVFQVFZ0U0NVWWZpcHJuQXRua3E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxQN1NCWUFhWDE3VlY0V1g4OUNxcHRVaV9kOXk2bVdBU2JrYTBOcUJrNUlON21WM1h3eXZ2NEVQUVBXWkI0UGwxZ0JyM3FDNnFuckdQZ0RibVVGajlNSi1MUjVIUDZWWkx4RTRCTF9ZWGJBUGl2XzhLd0xHODdYMGs4N1NDMTBiLWZUZDdWbEhWUnQ0ekxyd3NBdXlSQXRQOE5LTEFLRW5pVmVldzdaM1hjX1Qtd0ZreDFORjR4YTNQRzNmVThpdEdNeFNrSWRrNEp5QUxXMFBmUzhaVmxFemVvaE5pcDFWQWQ5V0IzbUpn?oc=5</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2770,52 +2770,52 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K43" s="1" t="n">
-        <v>46085.59027777778</v>
+        <v>46086.5</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Polizeibericht: Heimbuchenthal | Navigationsgerät sowie eine Dashcam entwendet - meine-news.de</t>
+          <t>Zestiger lichtgewond na botsing in Tongeren - HBVL</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Police report: Heimbuchenthal | Navigation device and a dashcam stolen - meine-news.de</t>
+          <t>Sixty-something slightly injured after collision in Tongeren - HBVL</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 10:48:36 GMT</t>
+          <t>Thu, 05 Mar 2026 13:42:58 GMT</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxOeC12WEU5ZjFwOWhJT18xck40MWZvNnU3bElqYlhJbkJ4X21pMDV6bk9udkgwUFdiT3dmdE9qNnlkM0ZNQm1iQVF3NlcxRm0tRXJsM015SUJiRE1yTzFMdFRuVUpLSVZKM3RMZFlZOC1uMWNWUUU0Q2FNUjNNSGoyeG1SUTQyNkhvUldFU1ZxTjE2Vm5VdlY3U3k0dXBsX2VqLXZiaGxRaWpINm9DUjdOUDd5QUlMOVZ0NVBtakpKaw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxNUjhnZ1pBc3VTQkFvbDJDWlU2aGgzWEJtS3dQQVZaQ0NsbE03ckcyU1JXcnJ5NVZhWG12ZTk3VnZtZEpoQU5vd1J0THBodXlub3o2a0R0MGJJTTUtblhoY21nbXZVX0NqUXNCVHBvR3o5dFV2WUhvSVVnQWlPaVpJd2I0dlkyekdHc2ZkOVptUzRJQUdpajNUQlBCLVBVem4xNEFJTVZ6WjJkVFBQbkl3?oc=5</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2825,52 +2825,52 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K44" s="1" t="n">
-        <v>46085.45041666667</v>
+        <v>46086.57150462963</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Village Wertheim (fallback)</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Tennis Channel streaming service joins Amazon Prime Video Channels - Awful Announcing</t>
+          <t>Na horrorcrash met 160 km/u doet topwaterskiër Tim Lisens voor het eerst verhaal: “Mijn hoofd zat alleen nog vast dankzij mijn wervelkolom” - HLN</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Tennis Channel streaming service joins Amazon Prime Video Channels - Awful Announcing</t>
+          <t>After a horror crash at 160 km/h, top water skier Tim Lisens tells his story for the first time: “My head was only stuck thanks to my spine” - HLN</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 00:36:38 GMT</t>
+          <t>Thu, 05 Mar 2026 13:28:14 GMT</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxOT1pDcFJQYmRXUy1YTEQxbTBlUF9Nc0FlUlZZUXlJeVlmTFZwTG5fRzZkemZzVld5RlpicnlHd2hUWjBDaFpybUNRYnZCMGh0WDdQd3hGbjhydTVYRGt1Sk9fcDN5QjVUaUR4bk5nRU4xYVJxSFNGaXo2UEhPLTN6TmMyRk5UTmlUN3VUbTk1T29qQ1Ff0gGaAUFVX3lxTE4wck1ja1E1aXNybXhseUxOSkM4SjJ0OUp3VjI5ZWpJdTdLY0ItWTJncDl5ZTRoYmk4dnZJcDlMR05sQ1dubmJSNkk1Nm85RnpRcG1mTGVISXliVmxlekwtVGRtWlloNjM3ZWptbEF4SHo2d0s0di0yYkhhQjhZRGwxSllhMGRsOWhSY19zMHB3WVhaTGF0TXhtWEE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigwJBVV95cUxQSVI3MzBISm1mWHdRNzJJam1FTVBITjBpX0VCRDNmQ2RRNVl0RVVwbG5ZeTJLWjBva1FmSXRPdXhSSHV4c2p1cmpoT3dfQTNqenVheXZSUkJndEdXTEhUQW9EQlZkbmpYUDRWYWRXVmNtbDlzZC1oVGtBaWN0ekhFVzljWHhZTm54Yk05U2VJcnAtMUFkM2U0Qy1aX0NpV0JZR1NiOVhDb1Q3c2VrT3AtWXRUekw4YVMyYmlEQnhYSXNDQkw2VE1fazN5YnBoT0FSdUxEYjBod3o1UmNtNzJiblFjcVZxTlp4WHFJY0N6bmNDY013OER4eHNCM25IbjQyMGZ3?oc=5</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2880,52 +2880,52 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K45" s="1" t="n">
-        <v>46086.02543981482</v>
+        <v>46086.56127314815</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Village Wertheim (fallback)</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Election night photos from Tuesday's primary in Abilene - Abilene Reporter-News</t>
+          <t>Dertiger lokt meisje (11) op spelplatform Roblox en vraagt naaktbeelden in ruil voor virtueel geld - HBVL</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Election night photos from Tuesday's primary in Abilene - Abilene Reporter-News</t>
+          <t>Thirty-something lures girl (11) to gaming platform Roblox and asks for nude images in exchange for virtual money - HBVL</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 15:49:00 GMT</t>
+          <t>Thu, 05 Mar 2026 11:47:18 GMT</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9gFBVV95cUxNb1VDSzBHTEE1SkVOSUJhTk8wMGYyaGNXX0kwVkYyQzNDX2YydFhhb2RJdFIwYUo3Ym9YMG85WnRtcVlNekY0aURSelRCZ18wTHNXSGtsLWFsNHhyVzNtUTNTdHRjUVdZWGlnQy1keUFxalM5S2lCMEVMR1BrQXNBb1JYSWVwNVU4MldnaUFvWjU2VkRFWUdyRTRuMFlRQlJCbmZMcG1waUZWZUlGZjRvbTR0N0p0U1lINFVrU29mNVBLUlJmU0JfNTBtV2VXY2hTd1RRTnZ3M0lmenFOMVYwcU04VjF4dEdZZmtHYnl4MmNYYWdzWFE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7wFBVV95cUxQR1BXTWZLVUpBenZ2REFtOVowekVzOEEyOTc1bmk1NGl2ZXhUUmFFeG1hUFlETk1LM2pvOVRTXy14ZzA4c2RwUmNJTWRrRktkVGVmdm5UWTBaY1pCYlJyckt5bGtmSG9qcGZIT3BQdUFmbWtGOXBPZTFSYTBlN2pYUkRuVjMwV2JjTHBwMWE2RFZLZFU4UkZ2aG1ETG4zTkVaOG1Vd2NvdFdmQnZCREUxWTFkLTNnQVlpMEJxR09YdkdYVDZ0LW1JY0czVFEyeS1lT01TOFV1WVpxanBMQWRIMkN2bXJtdjhyd1AyRVJPUQ?oc=5</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2935,52 +2935,52 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K46" s="1" t="n">
-        <v>46085.65902777778</v>
+        <v>46086.49118055555</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Lebensgefährliche Verletzungen: Motorrad-Fahrer (21) verunglückt bei Ingolstadt - Pfaffenhofen Today</t>
+          <t>Ontvoerder van 13-jarige tiener uit Genk werd voor zijn assisenproces maar liefst vier keer uit het verkeer geplukt voor gevaarlijk rijgedrag: “Ik gebruik geen drugs, mevrouw” - HLN</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Life-threatening injuries: Motorcycle driver (21) has an accident near Ingolstadt - Pfaffenhofen Today</t>
+          <t>Kidnapper of a 13-year-old teenager from Genk was picked up from traffic no fewer than four times before his assize trial for dangerous driving: “I don't use drugs, madam” - HLN</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 13:35:11 GMT</t>
+          <t>Thu, 05 Mar 2026 11:53:20 GMT</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiZEFVX3lxTE1mc3FhTmxyanVMeFB6YU1hNjFXWjdZOTJEaFBSS0ZOX1poR3NhanQ0Z3gwMHEwN0p0MHVsTnRYQWJDbTl6LUVQRW9xenlpZy1RMXpOSllRb3hUUGtWQVhLN0gzUEY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisgJBVV95cUxNYnVMZFRaSXRiOXBFdGlyeDBUUHFkYUJ5Z0ZZanlUWDdaTkFLdXRpWE8xUVFGOWhkX3BYNGp6a2NpbVlGNnZDNkY3ckxzUlM5aHAyWFNoZ05NTktuUUNHQktQUjZiWXBQaGJBcG1jdFFTZHlQdkdkOFp5QkFKZ2RvbFNfOTFRVW92U3V0Uk9zczhqRnlsR2JxdkhKbEQ1ekp0RVpzRUZFbE1LX2FaamZ2a1hDbXdLdF9fY0s2YmtHVmlFN0dEMXpNTzhvQVQ1RnBTWllMaC1LRVpjYjFJVHNFdXVfWHMyZTRFQ24wSXVqSUhRZ3h3blJRcGtIM3hXU1pGRkMyaDNkYlZneGo4NUg3bkV0MjNXallTS0E3WS1pMm5ScklnQThrdVhhYXQydlVWdWc?oc=5</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2990,52 +2990,52 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K47" s="1" t="n">
-        <v>46085.56609953703</v>
+        <v>46086.49537037037</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Village Ingolstadt (fallback)</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Audi: New Supercar Could Happen 'Someday' - inkl</t>
+          <t>Nieuw skatepark in Sint-Lambrechts-Herk officieel geopend: “Toegankelijk voor beginners, uitdagend voor ervaren skaters” - HLN</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Audi: New Supercar Could Happen 'Someday' - inkl</t>
+          <t>New skate park in Sint-Lambrechts-Herk officially opened: “Accessible for beginners, challenging for experienced skaters” - HLN</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 10:54:24 GMT</t>
+          <t>Thu, 05 Mar 2026 10:28:19 GMT</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxNcDFiaGtUYkRPWFR3TExMelFqR01CZ1dEVzVmTGhIMk5fOV8zUHlyZU5iRVhQNXQxcEtObjNscG1sNm1POXlXOGtkZHdvXzJBMmhkWUY3ajJDZzlWa1pLR2t1VUczVjhCOUkwVDJLS1Z4LW9QTDJEa3l1R0pLalE1UVBmR1p0OUU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxOUXU3Qlc4ajRYM2pYTngwMHV5aDIwQ21aU2xYSkIxWnpRWUluM2FCc3VaQ0E1UDJ2Ukhyc1ZBbmQ2dl9LZVE2UzN1ME03ZExFS01HOE0tVF9fRy1WQkVwNUFMdXNEbXFzbmF0UHVhR0R4Z2Rrc0p4Z3FQY1pxVFl1SGVWbnhkbzRjeEFjTnozdVQ0dGZ0R0o5ZVJaekxjdlFfWEtvME1NMS1xODBqQXBXRmRlaGZKVmIxaXpXeHZCWHQxXzRfY09FNkZkZnlCdWZjMy1FTUtEaERuUHNjZ1dZSXlrWHNsbVBv?oc=5</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3045,52 +3045,52 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K48" s="1" t="n">
-        <v>46085.45444444445</v>
+        <v>46086.43633101852</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Village Ingolstadt (fallback)</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Audi Becomes The Latest To Want A Luxury 4x4 Off Roader - Auto Spies</t>
+          <t>Nieuw postgraduaat bij PXL: “Directe impact op miljarden aan publieke middelen” - HBVL</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Audi Becomes The Latest To Want A Luxury 4x4 Off Roader - Auto Spies</t>
+          <t>New postgraduate degree at PXL: “Direct impact on billions in public resources” - HBVL</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 13:44:58 GMT</t>
+          <t>Thu, 05 Mar 2026 12:42:36 GMT</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxObkhCRHRUSVdoZDZYcFZydkZnXzNFQ0J3UklhamtodXRuM1VGaEZPR2N6VHl2c0NhblJZbmdfZGlvcXNtVFRJTDRhUC1NcXBZWUVRRVFoSVNoT3M5bWt4a1ViSElHVkZ6c2dXeUZaMGNwSnhrMnFMdUxEbVR2TXItQkppSzFiNU1weW9QdnFHU1d4ZDdfNVN0OHVR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxPRUdyV1F6VUExZi0zZGliejJLWXQwR0FjX2NSc1ZhcThtY0ViT21VMzA1bXY5RkFGZ19IZ2tPQkxydjZ4dFkteG1rTHprX2g4VmtiUXpTTEgzM3JyTHZER3kzTUd0TF9ZRmNiR3ZnODhzNGMzYXBOMHl3anNnS0I5ZDFDZ2FQaFRWTVdJdG83WFVoYkNMMjZwZVphZkN3TXFSUnkzaWlNNFg2YWtqZl9mcG9HbzhuazdmWEFLeHBJZXhkYV8xMjZQWklYbUlMZw?oc=5</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -3100,52 +3100,52 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K49" s="1" t="n">
-        <v>46085.57289351852</v>
+        <v>46086.52958333334</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Village Las Rozas La Roca (fallback)</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>("Las Rozas Village" OR "La Roca Village" OR "Las Rozas" OR "La Roca") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Captain Fresh completes acquisition of Frime to expand tuna presence in Europe - WEAREAQUACULTURE</t>
+          <t>Obligatiehouders vangen bot in Triamant-zaak: rechter wijst eis van 16 miljoen euro af - HLN</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Captain Fresh completes acquisition of Frime to expand tuna presence in Europe - WEAREAQUACULTURE</t>
+          <t>Bondholders are caught in the Triamant case: judge rejects demand for 16 million euros - HLN</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 10:06:37 GMT</t>
+          <t>Thu, 05 Mar 2026 09:31:07 GMT</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOTndjdnR6NEdJQlVUV0xKNm1lUFVlbUxIOHdOaHhRYXIzSmdKUjM3eTNLTWU2VmNDVHg3NVNVRXFHTEdPM2RLVFYwSnAzRDlMT0NFei1mbkNJVHJfdVBNTEpxWGUyODhXNDZSczlzT3VvU2k3UTcyTFRfQWx3QXJUZHFCRW8zRHdmd3lYWWpjUzVrcjFqNDkxUlNoYzZ2OUJnbjIxNHFKOGNZRUZqQVFPbzJ3RWF1MFNyenlqWNIBygFBVV95cUxPTzdBRVQ0VWlkcUowZzBaVF9Fa05DWDM4U0hsN0N1eHFsWHo4clBwODNmcEJzdkhZczJjR001SGtzSFhTaXljYkNtbDM2ZHhaNVN1dDdQWGtfTi1VbFVhbWZwRXhiS2d3a1Y3NUZibFdReUZ0enhaZ3NoN0p1S0ZDMk1aMkVSNXBETjQ2VWcxUVlWYi10WlNzMjJqa19hdE51YUVBRlk5SWh6cWVsQjh2S0pyQ1lFOGNyRzNVUmZiNm5LVVBjUW1SVWVB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxOenl6dm0tQjZodVlvUVJHRFNoUE1HSXJoSHZUMEM4ZkJpUHBvM2kxa0ozMnh4a19OMVJkUEdsSzhvUlN3bVVlTFV6ZEw4X2VMLXgyVGtPQ1VpTXR1OXFpTTN0Rm5rM3NWZ3JtZDQ1WHBDY1l4eFQycW5KY3RLY1F3emVBNFpuQktjTThXLTZyOVljamJMZFI4MG83bnZ0VVFHVlVvSUsxQmY5Rm03bnQ3YXc5QWlhLWpNOTVZZUZvMA?oc=5</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3155,52 +3155,52 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K50" s="1" t="n">
-        <v>46085.42126157408</v>
+        <v>46086.3966087963</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester outlet" OR "Kildare outlet")</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Public complaints lead to six motorists being caught speeding in Kildare village - The Irish Independent</t>
+          <t>Marie-Joël Kessen, 64 jaar - HBVL</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Public complaints lead to six motorists being caught speeding in Kildare village - The Irish Independent</t>
+          <t>Marie-Joël Kessen, 64 years old - HBVL</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 16:40:00 GMT</t>
+          <t>Thu, 05 Mar 2026 10:02:57 GMT</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxQX1ExLVJIVGNBWU5xOFJyVUt4bDNWVGtMRWVvaVdUYk1GM3NkSnktWk1Va3NxUjg5bVNRUHM4OGhmeTB4aWtlQlhMUW10a2h6OFdlNmI1NzU3SEk5ZkNJWVRIb05JblFPUUtVbkZJMU42YWlKdG1ZV3BHc1ZTdEdRUW5DbGRhZDJ6dlM4S1p2MnVjdnh1Q1dYTHVNd0w5TTBCNGUyMDhKQ0R6djUtM2VOeVpGbGVoWkJxam1tMzg4bDhucGp5VW5pQTFzbkZGdUdVQXQ4R1BEckZMWjR4YzFsUg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxORnpMTHYtWTN4YnFrU1B3dkh0TkV0cllraW1nY053czlPRzFObThaQS1JcTB3cktiN0R2a3hpX3RBeWltMGlFWVpnQURaWDMzbl92VUZNMkp4ODBPSG41NmFNZlhMOGp4dm0tdTAtTG0wNE9JLURzc1pJSzNkd0ZFa2xmUQ?oc=5</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3210,52 +3210,52 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K51" s="1" t="n">
-        <v>46085.69444444445</v>
+        <v>46086.41871527778</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>High Level City France English</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>("Paris" OR "Île-de-France") AND "France" AND ("bomb threat" OR "suspicious package" OR "shooting" OR "stabbing" OR "terror attack" OR "police operation" OR evacuation) AND -Texas AND -"Paris, Texas" AND -film AND -movie AND -football AND -transfer</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>France/Middle East • Paris deploys evacuation plans in face of Iran crisis - Intelligence Online</t>
+          <t>Zware klap tussen twee auto’s op N74 in Zonhoven - HBVL</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>France/Middle East • Paris deploys evacuation plans in face of Iran crisis - Intelligence Online</t>
+          <t>Heavy impact between two cars on N74 in Zonhoven - HBVL</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 13:41:12 GMT</t>
+          <t>Thu, 05 Mar 2026 11:54:25 GMT</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxPWm5obXRPM0Z0MFdvbmJvdW1zbndDcEFvLTBKa0EzQ05lUm41THFUREFMWUNfUnhHai1ic1k2RVFYM1EzX096NVFRdlZKQ0JQUVdhNWg3SngwMUVIN1N5dDdmOC1wODF3eUJpbGZlOWVZV0hySjBlam9zeHdmbzNDcUZiakF4MXh4RjU1V3dYV2xVbjJuTHAxbThBVG94ck5BRHF3emZId3k4MFpycm4wbGtWRVY3dF9WcG9aTHZQalYxYVNTMUdyZy1rMFREeUlUY3c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxQUUdXNUV2OEJCREs1MkpwMTVsLUplVWxRVTh5X05xVmFUZXRfR1ZJeWU4MVVjU2hVel9UUjdPbjlpUW5RNFZ0amlmVzh0YmFrZXJiWGhISFpHLVhLeVpveVd6aS1SeC0yc1lKQXRnSjVIb2Y3VWVGV1ZzZEd2U0tuUzNZa2lTaGFRSTJiUXdPRWpkVGh6bXQ5NTVEcVFJWHhNMU8wNFBqWjY?oc=5</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -3265,52 +3265,52 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>FR:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K52" s="1" t="n">
-        <v>46085.57027777778</v>
+        <v>46086.49612268519</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>High Level City Italy Italian</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Sciopero trasporti marzo 2026: quando si fermano treni, aerei e mezzi pubblici locali - ItaliaOggi</t>
+          <t>107 obligatiehouders vroegen samen 16 miljoen euro na faillissement Triamant, maar krijgen ongelijk: geen schadevergoeding en zélf opdraaien voor kosten - HLN</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Transport strike March 2026: when trains, planes and local public transport stop - ItaliaOggi</t>
+          <t>107 bondholders together asked for 16 million euros after Triamant bankruptcy, but were wrong: no compensation and had to pay costs themselves - HLN</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 04:46:52 GMT</t>
+          <t>Thu, 05 Mar 2026 09:19:59 GMT</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOQzJqcF85TU9pOVRPcWoyYzFJYzJYRGx2X3I0QnI0cVJNRG05UUZCNl93YlEtUEpKZFZ1WnhXSlUyTm1ZbTMxQ0xKdURUaVNvd1RiaVFVUWdSWXpGNm10MzB3Vmp5WlcwSTY1czhaQUZoQXg1OHVHUDFmallBNEhmdWdLc0hpbmNzR1QwbGNxSUhjU29VS2huUnVKcjQ3dnNmby1MMENEOFV5MjVBRkJYLUgyeUxoZlE4ai0tY2ZQdzZ4cUtPTWlhc3hJNFVBUmZQYUdNbk5xV1ktRG5QdjZJSnJ3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgJBVV95cUxOQXlsb3RhUHhjR0JoZDNnNnY1eE9LZk4zWjNoaFI3dm41dWt3MjFmdGUxT3Fzd0lUYnNrWlVsZ3FQcF9aMHVtM3FjSmUtM3hNRGVPV3kxbDhTU1ZKd3M1NnY3Q2k5REk1WmQxUnU3bk82OUxQVzFqUjZseDBvTHVhdERyWUdwUEU3dkNadDRxcHJLR3l0X0lTNlhJWjF0QnZqYnNPVVlhUUVET3ZUbUY4M0JHUnQ1TUVYUHY2cWNRbTFRQ2RlTHdpQU1TRmppc0hvZDY0c2UxUUxBcHBwWkl2OUpSLWlfWE1TVFdqOTRYWE94Y1NVSFU3cFBueUhfdmk3bEhKNjFqc3RaLUlWVEg1YXdIVlhjZw?oc=5</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3320,52 +3320,52 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>it</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>IT:it</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K53" s="1" t="n">
-        <v>46086.19921296297</v>
+        <v>46086.38887731481</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>High Level City Italy Italian</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Protesta contro il Muba. Tornano liberi i tre fermati. Nessuna misura cautelare - Il Resto del Carlino</t>
+          <t>Futsal Benfica Auderghem - Anderlecht</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Protest against Muba. The three arrested are freed. No precautionary measures - Il Resto del Carlino</t>
+          <t>Futsal Benfica Auderghem - Anderlecht</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 05:13:20 GMT</t>
+          <t>Thu, 05 Mar 2026 14:09:11 GMT</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxOY3EwLXVoaHVxRDdHeFg4RmNwWWV3QXVuM3NSdHNWZ2RJSlJfOTBKYUJKYzNLOE5jM3pCSmtjMFkyYjZIN2t3RUJMME50N1hrZmJKVk4xeFpySS1qZkpTQV9XM3hxS3Y0T0dvU1N2X1dIU3FiUWp3cGl5VmR5eFZjYVVuWkdpVHBKVDB6bUpzeURDc0U?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiUkFVX3lxTE5scURuclV0anR4NDRjYWFCWU9Ea0wtSG9JYTNEdTU5Z2NxdTlpQ2Zjcl9XOGRLZEFFcTVhVHZxTzdiUDVoeFpYaUZfWS1ZNFdKcFE?oc=5</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -3375,52 +3375,52 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>it</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>IT:it</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K54" s="1" t="n">
-        <v>46086.21759259259</v>
+        <v>46086.58971064815</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>High Level City Italy Italian</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Manifestazioni, mostre e visite gratuite: il programma completo delle iniziative per la Giornata della Donna 2026 a Milano - Secret Milano</t>
+          <t>Polizeibericht: Raum Aschaffenburg | Küchenbrand - Keine Verletzten, Pkws angefahren - Unfallflucht - meine-news.de</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Events, exhibitions and free visits: the complete program of initiatives for Women's Day 2026 in Milan - Secret Milano</t>
+          <t>Police report: Aschaffenburg area | Kitchen fire - no injuries, cars hit - hit and run - meine-news.de</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 15:27:35 GMT</t>
+          <t>Thu, 05 Mar 2026 13:32:07 GMT</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE0zNG9wSnU3bzNFOFdoSXB3dU02ZGxVQVdkSm55d3lveGNYUnZBcHZhSTZfanBzbkRuN196ZnNHMHFNNU4zMEdvd3hrY2ItVklrZkNqSFBOWGZfN19vemx5WUN0UDgyeWdwaE5IcFlScGI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxQNjdBaHdqMl9NT0d2UUhqUzRZVHBYaFVadWRnUzE3S0p5Vm9VT1FTZWZyaWdHZWx4VUtReTVUbThlSDdEd1RKTFlycFFjTEpDbzBhUGRjUmhDai14NnE4bEttc1RiT1FkNVhKZURQUWpMa053WldacVdvVEVFRmZKWWdwREpaU1l0UXJiOGtRZEVJNTRrcW8zNDZlbzhnd3ZVMV81Tl9WT2x6X2hYcXIxUUV4bjBqeUpCZ3BQejFnNndPa3BTVkZsY0tvd3dQT1V4Tk4tWlFkZFZodmdIWE9Ocw?oc=5</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -3430,52 +3430,52 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>it</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>IT:it</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K55" s="1" t="n">
-        <v>46085.6441550926</v>
+        <v>46086.56396990741</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>High Level City Italy Italian</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>BOLOGNA: Sgombero presidio ambientalista, Procura chiede 3 divieti di dimora - Teleromagna</t>
+          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>BOLOGNA: Clearance of environmentalist garrison, Prosecutor's office asks for 3 residence bans - Teleromagna</t>
+          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 10:10:37 GMT</t>
+          <t>Thu, 05 Mar 2026 09:23:17 GMT</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNWGVEX2lmQWdMX1doZ3Npci1MR2lOYmdpdnhXR1RlT2UyVC1lNGZ0Z0xlZ1dnbGNSd201QWpKU1lnNlJIS0puVGpYXzRPVEY5WVRBSXJmM2FzZHVCeVFUb3N6TXlGYjBxYy1nM3pidGltcVJ0cE5ZSDZTalhoNndHSEJVNGY5TW1BaFU1QnBRNnFZQU1QcXl5SXlCOUc4VDVKdjYwR3JmbXpoZnlOVjNVTFZKY1dGZHhsSExJYUtn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE03RUZJdVVWTG5jTlA1R0dmc2YyQ3Z2S1ExYmhkN0FENFJGamUwenJsSFFPWGpKc3B2aFBaeHRYVDR3aWM1SXg0YWZFVDk0N3d4a0Jz?oc=5</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -3485,52 +3485,52 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>it</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>IT:it</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K56" s="1" t="n">
-        <v>46085.42403935185</v>
+        <v>46086.39116898148</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>High Level City Italy Italian</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Scontri nel cantiere del MuBa, scarcerati i tre attivisti. E la protesta smonta | FOTO - BolognaToday</t>
+          <t>Schweinfurt: Neue Polizeikameras in der Innenstadt offiziell vorgestellt - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Clashes at the MuBa construction site, the three activists released from prison. And the protest disintegrates | PHOTO - BolognaToday</t>
+          <t>Schweinfurt: New police cameras officially presented in the city center - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 12:53:15 GMT</t>
+          <t>Thu, 05 Mar 2026 14:30:00 GMT</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNZ1JDbDhhczRJQUxYaGNzdVNfcHdfblFzWUttcG12bTd3cjlGeFVOZGczRy1Gb1BIVXdGdnlmTy1vWFpXRGtfN2wtN2lSQUZNeDZvQXh3T2dTTk5sc2JzU0dDaTlkbWJqb21PbWNTWldUZXlsMUM4ZDlpcENMLVowaTRTYkgtSEdLRzRGc3JZTzRIazFRblE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxNZ3RZa1V5ZmJlTWZzTk83QzNjRmRpWGxaelpwSFBxTElkTC1pQUhiSTVWbGR3akxqQU5sTVBxaGI1eGVXV1c4NnZibE9Pd3I2VTJDNDVHVWp6RVRIVzhSV19CNkVCeENocXpLSHpHVFdsVV91VHZia2Z1d2hUTUF3N2ZtQkZtdF9XUVVGNGs5RFFfNElpbDkzaG5OY0Jqbm84WUdOZ1ZEQTg?oc=5</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -3540,52 +3540,52 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>it</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>IT:it</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K57" s="1" t="n">
-        <v>46085.53697916667</v>
+        <v>46086.60416666666</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>High Level City Italy Italian</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Scatta il decreto sicurezza a Bologna, multe fino a 10mila euro agli attivisti del Pilastro dopo i tafferugli - Il Resto del Carlino</t>
+          <t>Tod von Messerangreifer aus Würzburg: Keine Hinweise auf Verbrechen - Joyn</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>The security decree comes into force in Bologna, fines of up to 10 thousand euros for Pilastro activists after the riots - Il Resto del Carlino</t>
+          <t>Death of knife attacker from Würzburg: No evidence of crime - Joyn</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 02:03:41 GMT</t>
+          <t>Thu, 05 Mar 2026 11:08:26 GMT</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxOYTdJZHk2eFNnOUdGQk45Yl9tTThzd0phTDV4VzVsb2FNcjFxTDhzbmRBWGJza1RjUzRuZ2NkNlFLZV9nZXIzZlVGU19ocHk1M1NQa3JpMldGbjY5Um02cm5DVkMta3hmNDc2bFpkOWpqbjlUUDJZcXNZaE0tVVhkSEU5a2ZXQmJ4M1J3Wm0ySnd6ekJuVm9XTkl0M2JZZ0syeDI2LVhMbk14ZUQxNExvVTVyYVk0ckhaMlVVN2JOTi1DUVNtMGln?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQV2RSWFRMaUpHNWlYYm5ON3U3QUN6UEFhZWRiUWZWYzY4RGhNYWo5TWJlLVNNMThIVU9qZTV0NFpqM3BuUTlidVYtQW9ENXdCUlF4Ul9vaEk5Q3RWbmU3Y3FHOU1Zc05CTFh3LWVQdzk3RTlhR2xhc1ZBMFdjWFg4UEJFb2YtbWxVOVcyVDFlMGJ4eHQwZ3AybEJRU1hkQXhwcm1MNXpTVGhhRFNUbzhwWVVTVkR2aHdB?oc=5</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -3595,52 +3595,52 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>it</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>IT:it</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K58" s="1" t="n">
-        <v>46086.0858912037</v>
+        <v>46086.46418981482</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>High Level City Italy Italian</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Per un no sociale al Referendum: dibattito a Milano lunedì 9 marzo, verso la manifestazione nazionale di Sabato 14 - Usb Pubblico Impiego</t>
+          <t>POL-LB: Großbottwar: auf offener Straße geschlagen und beleidigt – Zeugen gesucht - BlickLokal</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>For a social no to the Referendum: debate in Milan on Monday 9 March, towards the national demonstration on Saturday 14 - Usb Pubblico Impiego</t>
+          <t>POL-LB: Großbottwar: beaten and insulted on the street - witnesses wanted - BlickLokal</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 10:26:00 GMT</t>
+          <t>Thu, 05 Mar 2026 10:59:19 GMT</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxNOWJEOTNhaENHN3J1M2JDVUtmMVdicTEwd1BYWEx6NTJtQTAzOTBJTUQtRzF5TTE1Vi16UDhzSDNGZGJNbjc2WlBudk5qc3RrYzJwVXVwSmpnMnNadWhxcVJoTjNDdk92S01sTzFaMEhGUEhiRHdVQU9zdF9wU2xPTnBsMzVLUnhRcVRNWWhrOEF1Y0x3QWdLaTFDYVhzbGRENTRnSy1QUGk4RE4zWUpaWGtOVkZOR2xWenN5c093M1kyV3Frb3JpMnMxemFNbGdzSE5uSzd0YW5kcU5ZZWhiYVlZcC1WU1p6UENzY1YtOXltamFhMWFWSWFuYw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNaE0ybnFYUTY4b25kNkIyNjBhbmlaWk1wUmQxaTdGMERNRXVybEtXYldaS1NoYXltQ0dyeGpvcXBSUzBDRnZxMnFvVzJZdXFDeXlCX2Z1RlRjYkxmcmFpbmVZU0UzTGNmTm11bFVZNkFiQ0l6cTVvR2UzbmdPSGI3LWV3NDd4UTc2dFNEWEpnR2NOT3BZNWFlVE5nX0Q4NWVZS2w4cVVGS3psWEJKSGlOR01B0gGyAUFVX3lxTE1oTTJucVhRNjhvbmQ2QjI2MGFuaVpaTXBSZDFpN0YwRE1FdXJsS1diV1pLU2hheW1DR3J4am9xcFJTMENGdnEycW9XMll1cUN5eUJfZnVGVGNiTGZyYWluZVlTRTNMY2ZObXVsVVk2QWJDSXpxNW9HZTNuZ09IYjctZXc0N3hRNzZ0U0RYSmdHY05PcFk1YWVUTmdfRDg1ZVlLbDhxVUZLemxYQkpIaU5HTUE?oc=5</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -3650,52 +3650,52 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>it</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>IT:it</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K59" s="1" t="n">
-        <v>46085.43472222222</v>
+        <v>46086.4578587963</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>High Level City Italy Italian</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>BOLOGNA: QUESTA MATTINA UDIENZA DI CONVALIDA PER LE TRE PERSONE ARRESTATE. MIGLIAIA DI EURO DI MULTA AI RESIDENTI DEL PILASTRO - Radio Onda d`Urto</t>
+          <t>Blitzer in Blankenbach aktuell am Donnerstag: Hier nimmt die Polizei am 05.03.2026 Raser ins Visier - News.de</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>BOLOGNA: VALIDATION HEARING THIS MORNING FOR THE THREE ARRESTED PEOPLE. THOUSANDS OF EUROS IN FINE FOR PILLAR RESIDENTS - Radio Onda d`Urto</t>
+          <t>Speed ​​cameras in Blankenbach currently on Thursday: Here the police are targeting speeders on March 5th, 2026 - News.de</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 12:50:00 GMT</t>
+          <t>Thu, 05 Mar 2026 13:15:39 GMT</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-gFBVV95cUxPYUJXS3J1dlFKdTdaLXNGZUZYWFVhMWhnb3lPVUdveTNpdjl4TDR2Z1hRRkM0SGpoSGd2N0xueEthZ2tudHNGRExTanltMEZ3TlAwaTVoVnFjRGZqNDZWUnp3YmpvMkhtS1A0MU14TkcyNGN6aDVfcDg3RFp2aGdtTFZobGxsb1lxRUx2Y2pKaWtZNEI3bUNDelhkM2t2ZmpDNDNzWGdQbHU2d3J0Wk1wd1ZKZWJaVU54OU5pX2FXbmYwUHZMejBpazhCaVJwWV90TGNhSk1uM25PeDdRRmdEQkt6bm9OSzNHSGZjVXNhd3hKeEowNFZrT3hB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwJBVV95cUxNT3dZVW1WQzJkMWU4NV9lNTdWT3ZKdjhQWlJVSi1FSXZianZmYVpHUWZKMWx3LVVUSnFXSWlEUmJHREJLdVV4UVRoSUtSS3JfSUpLdGRwUHhsZ1J1bF9uVlQ4UEVYVE0zSTB1bzJJWnZYcm43T2p4LTdQekg1Vk9jaUJfVFItNGZYZkVycFZhT3h5UjBudkJYSmxMZDFYLThvVGFZLWtOOXFtVnRqOVVpVzNWTmlqSWhtQjBhamZXSUw2TUpmLXQ0eGRGaDQzYmtyRzhhQVlhaUpJVEZiRk5rQ2NKc0s4Y1ljWUw4TFVvMHhzMkhNT2QxNDZfYUtLTm4xZzFpT0xDSkI3bGQ5cXhTb0ZnSHdiUW_SAZwCQVVfeXFMTWgybGRuOHJFRHpxcWVON0NYZW9NSjdFY1phYV9mZm84NDFpcGF6Nk1tY3hNS0ZXb1JtNzNGOTdhMUpxeDRMQUR5akdOZUVKMU5FOTE4MWRJYXlWRXgxM0dKTDJabVBpdGk3aF9DVkJDZmRtV2dELUZSbWtaOGRCNDVLZWxmS284T3RGcGoyR2c1U0ZpZnNoMEduUmZLOHRweFFFTWJ1ZE9wQjh1NVVZTXM4dGRNTjIxaFFMTkQ0N2UwTk5Pd0RkWUJkMVVZV2N1T0hQQmRqZ0VzOHBkajU5d0hvYnczSkFMRjRmcTlPUUVEVFhHb1Jwb2dpUVhnS1c0cjREX3ZQdktKMVNDdlJ2NlJ1LUgtMDJGNEVkOFQ?oc=5</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -3705,76 +3705,351 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>it</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>IT:it</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K60" s="1" t="n">
-        <v>46085.53472222222</v>
+        <v>46086.55253472222</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Golfcart als Fluchtauto: Polizei sucht nach Einbrechern - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Golf cart as a getaway car: Police looking for burglars - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Thu, 05 Mar 2026 11:58:55 GMT</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQcF9qT1l3cEVrUDlCWUxhaEZRV3F3VFBCOUdXejUwNVdCZ1hLOFBpa2pUX2c4R3EzWV9PMGJPU2VYTHFmUHBfbkxyYWhPUzlIS05LNjdIamJvVDRTWFlwMmt0ZEVXM0FLU0Q5ZWpoN3kxVzRQUkRaUVl0aDc5WWRraGozWFFhLXhQTy11NFlBbGlFM0FyemRDN21CdUtTRTdMSWtuNDc4bjFMbW5Ia25iRVRPWDkxcjdWQWhsd3BOdUNOejFucGhr?oc=5</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K61" s="1" t="n">
+        <v>46086.49924768518</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Schüler gegen Wehrpflicht: Auch in Ingolstadt wollen Schüler heute demonstriereren - HITRADIO RT1</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Students against conscription: Students also want to demonstrate in Ingolstadt today - HITRADIO RT1</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Thu, 05 Mar 2026 09:34:00 GMT</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOT0dXeC0yU2RmcTNoWDM2dWJzZ0doZHN3OTNFSXNPWlF6YW84VGVWX1Vob2ptVXdVcGVLQ29GaUJjOWdaQllpYU1IYU9Ia3hiNWVGYjA4RUR2SGx2NUh3Nll6Z01JVlI2MTg3U0dXS1hZSEZxbHJnYXdyZ2dRX0duamF0RTQyaWU1SDY5WGcxT2FseFQ4TzlaRkdvaUttN3pCR0ppeGRid21PSUxMcjY5ek5Qb3psUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K62" s="1" t="n">
+        <v>46086.39861111111</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>30-Jähriger aus Manching verletzt sich bei Moped-Unglück in Ingolstadt - Pfaffenhofen Today</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>30-year-old from Manching is injured in a moped accident in Ingolstadt - Pfaffenhofen Today</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Thu, 05 Mar 2026 13:25:11 GMT</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFBSa1pzbUFsOWxJUk1UdXVwZjF2VkVlOGtMS0JMMjJGcUw4SVhSd2NzS25KYkU2NnNoRmFmeHJYcGN6UHFILVBmVm4tOFJoeHFDWkV1LXNiczJKZw?oc=5</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K63" s="1" t="n">
+        <v>46086.55915509259</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Fußgänger stößt mit einem Bus zusammen: Fahrtgast verletzt sich - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Pedestrian collides with a bus: passenger is injured - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Thu, 05 Mar 2026 13:57:30 GMT</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxQX3VTMjFDSE5HLURMWEpVNGpfdkJvMTJZVkpib1dLdGQ3b2g3cnhCcmZyeGNZN0JlUXNNZXdpMDg4RUlwbWhtalVyb0JEM0g5My05QUJxRl9OUnZ4eXdLOXI4aUtJNGRvUUxfTktOOU1VNVROX1FWdzZaOWliVUtzejNMTDBBNHVVOXE3ZUt4bVFMdDRsdEVZY1ZMX3V4c3luSEM2bWl3STNFU29LcWNyOEpXYW1lZ3Y4dHNhUFc1bmlvYTB5bTFIb2k2RDdwdWdTaVpWcFd3SFRHcmtOZkN2RG0zci0?oc=5</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K64" s="1" t="n">
+        <v>46086.58159722222</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester outlet" OR "Kildare outlet")</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Sugar Plum Sweetery To Represent Westmeath At National Enterprise Awards - Midlands 103</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Sugar Plum Sweetery To Represent Westmeath At National Enterprise Awards - Midlands 103</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Thu, 05 Mar 2026 10:19:43 GMT</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQS1dwX0x2SDQ2ejY1OFVvTGJzNGpfUTdjdThEZDhGQXBsWHJTeWwwMzgwUDlaLVFUZERvSVlrandHUC02WFlrZC1lZE1nYkFTV2k2eVJaR0xfSVdPZ1ZPeFlud1hfb3BtQ3lyUzZuX0p2NkdYeDFpS25wNEpaRnhaV3NYcmJxMVBiajJFSS1XQnpQNDE0d2VEUkhWbmpKcERjbnZWeVBxOUxSUVdKSXpWNXByOGZBak94T1IwMQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K65" s="1" t="n">
+        <v>46086.43035879629</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
           <t>High Level City Italy Italian</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Guerriglia al Pilastro, smantellato il presidio degli attivisti contro il Museo dei Bambini - Il Resto del Carlino</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>Guerrilla at the Pilastro, the garrison of activists against the Children's Museum dismantled - Il Resto del Carlino</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>Wed, 04 Mar 2026 12:03:30 GMT</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQR3loRFFSTDJhSHRHUGRoazVaR2FWdnlMRUlha0pST0FQRFZFdEFLemJoOGVuNnpTaEZVZ2laUmsyV0V5a2ZkZHZpcVYyWHh0OG50S0VPWFZYWURlTF83bnZ5WHZDTzBOVWwzUDJDWXhVTjdCLWZfQjdISm1HSWdBcnRR?oc=5</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND ("minaccia bomba" OR "pacco sospetto" OR "pacco esplosivo" OR sparatoria OR accoltellamento OR "attentato" OR "operazione di polizia" OR esplosione OR evacuazione) AND -Olimpiadi AND -pattinaggio AND -sci AND -Cortina AND -calcio AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Milano, brutale accoltellamento per una battuta: arrestati quattro minorenni per tentato omicidio - Affaritaliani</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Milan, brutal stabbing over a joke: four minors arrested for attempted murder - Affaritaliani</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Thu, 05 Mar 2026 12:05:39 GMT</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxPc3Q5NXBQa0xPYXUxMnpyQzFYRVNrTEZUTm1MTVQ3NUNkaTFnVi1HVjQ0Qy1xQWdQaXNYMDZfRW52M0swVTJodnB3ZHhmOWVQUFBPT0JUTnJKX3Y5Vklkc0o0MjhfZUV5MVRnNTRHNFdQSC1DbnQxeENJd1ZtOExZcW55eHlHYTVsbXBJb0ltZnBFQ0FyZjZaNm5oYUJMMnBlT0hQbllQMHlUYVB3dnFDSTBlZEVoRnRnWFpZei1qX084cmEwbFFvVVpvZmRxUDdQelE?oc=5</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
         <is>
           <t>it</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr">
+      <c r="I66" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="J61" t="inlineStr">
+      <c r="J66" t="inlineStr">
         <is>
           <t>IT:it</t>
         </is>
       </c>
-      <c r="K61" s="1" t="n">
-        <v>46085.50243055556</v>
+      <c r="K66" s="1" t="n">
+        <v>46086.50392361111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-03-06 14:39 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K77"/>
+  <dimension ref="A1:K58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,32 +480,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Value Retail Brand</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>B&amp;M European Value Retail (LON:BME) Share Price Passes Below 200 Day Moving Average – Here’s What Happened - Defense World</t>
+          <t>Replacement for huge empty Bullring shop confirmed as massive signs go up in Birmingham - Birmingham Live</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>B&amp;M European Value Retail (LON:BME) Share Price Passes Below 200 Day Moving Average – Here’s What Happened - Defense World</t>
+          <t>Replacement for huge empty Bullring shop confirmed as massive signs go up in Birmingham - Birmingham Live</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 02:49:13 GMT</t>
+          <t>Fri, 06 Mar 2026 10:54:00 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxOUGVTblc3d1ZLQ0tXZnRxT2NmNjd4QWpYaUtDTVJ5R3lPRVFBaDhQV05Hb0syVHJYRHNaT0Q2ZEpCM19WbHptNXR5TTZoRVRtTzhLa2pUSkc3YjlGX2J6QmlmV3lpOWktdTZ3SHhsVlNpSlFkMnJFQ2pSN3lscTJPQzIwQklrNHVVcHVQSFVvWGcyNzFwYi1BUzdMVGlnQ3dvMWppVVQ2Ul9NNHF4NzREVUR0Sm5udlN2QTY4ZVFwa1p5VEdKTG16aEhBSjYxSTEzQU1vTGJvV2hab1R2?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOc0pNTWdGR05qWkRub1RaOHo2dXhzVDdNWncyckxsSTlsZGVqSjJjXy1nbDU2VHFvZmtINXU5X2lDaUFhVWZQVTB5TGZjaFFIS1hPdm9yYzJpVlp0NFY5bGNOWWZWcmxiQXdSc3phT0ZCTHdudUlrR196OW1MQzM5dVU0SFR5Y3A4N2sySkhvelYzSGRuMXBrcUJOWHpmT2I0eEtTUzNaQnXSAagBQVVfeXFMTnNKTU1nRkdOalpEbm9UWjh6NnV4c1Q3TVp3MnJMbEk5bGRlakoyY18tZ2w1NlRxb2ZrSDV1OV9pQ2lBYVVmUFUweUxmY2hRSEtYT3ZvcmMyaVZadDRWOWxjTllmVnJsYkF3UnN6YU9GQkx3bnVJa0dfejltTEMzOXVVNEhUeWNwODdrMkpIb3pWM0hkbjFwa3FCTlh6Zk9iNHhLU1MzWkJ1?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -529,38 +529,38 @@
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46087.11751157408</v>
+        <v>46087.45416666667</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>'I make between £800 and £2,000 a month on zero-hours contracts. There's no consistency' - AOL.com</t>
+          <t>Prinses Kate stuurt ‘zeer bewuste’ verborgen boodschap met haar kleding na arrestatie van Andrew - HLN</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>'I make between £800 and £2,000 a month on zero-hours contracts. There's no consistency' - AOL.com</t>
+          <t>Princess Kate sends 'very deliberate' hidden message with her clothing after Andrew's arrest - HLN</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 15:33:05 GMT</t>
+          <t>Fri, 06 Mar 2026 12:15:26 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE84UkdzeExGN2xLSUh5VnBiUlNFTkI1ZWl1bVo2RFVEeVUwdnZaSjNuS2hrOVhlam9pamJzUTRGRWZsOER6Y0hXRFpxTGs4bXZzdTZ4YXNxVlVaNXpCUTVuT3pHeXVlOHA5V3FLZHVUa3ZtYVV4aXNVUDZEek4?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxPeUk2U3lTdVlQOFJteENNWnA0R1JYcG1rallxYnNZMFlvS0UxcVQxRU94WTdNUVZmZkdQaHhHWUlOdzFLNjJzb1ZpU3paWnNZd09URlJZblo3ZlFHZlNXM0ctSDQ4WG5UWmtTbzV5YjJHZ1I2UEx5c0ZuS3Vkd2Zxd2thNllCbnpzQXE0OHdfWWoxOFpILV9KYkw1ZEdWX3VIaldaak9BdEYtQlgxai1rcC0zajg5dHZzUGpUQ3M3Wm1QUVRYN1ktTzRQbw?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -570,52 +570,52 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46086.64797453704</v>
+        <v>46087.5107175926</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>London Marylebone Incident</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>("London Marylebone" OR "Marylebone station") AND (incident OR disruption OR closure OR police OR bomb OR explosion OR stabbing OR shooting OR "suspicious package")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>All lines blocked at London Marylebone – here’s what you need to know - London Now</t>
+          <t>Zonen ontfermen zich over Britney Spears na haar arrestatie voor rijden onder invloed: “Willen haar op het juiste pad zetten” - GVA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>All lines blocked at London Marylebone – here’s what you need to know - London Now</t>
+          <t>Sons take care of Britney Spears after her arrest for driving under the influence: “Want to put her on the right path” - GVA</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 08:40:35 GMT</t>
+          <t>Fri, 06 Mar 2026 12:50:25 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNWTRrdVIxT2VyazRBVXhDWnlBYnNsbkk0TDNucEdrLXJYczMxeXlGN3d2OWZlS1F5NGRYVFIzMXhnQ3RwSERERldwVTlrcGtkeWdUVF9YQl81SHdpdnNDMmtSZTZyRVF1VHpjajFQeHhqVnV4SWJ3Y0c4NHlUX3NZTXNzdWpMVGFIMkw2MGJMVlZaem5hYW80aFpqdEg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijwJBVV95cUxPSnVOeS0tbmNuQWhBakFpbndab2RmWHdiUWV3bE9Vcm1fRVpLV0o2ZTJNbGNPOXhDaE5idW53elJoamRGcmN1anBpYU16Z2RuNHhTbExmcmRLX3ZYWXlFeVJHOVFtTXRreG8wdUpWcmZMVVdsenRURlQ1MDJLNFRqRjdYTmViSDUzOURETEhmNENyWlZzUFVfaC1SLWNiYVNVUFBFeG12RDRQMjV3ZFRIVmxfeHRKT0hQYm5GY3E0eGVCYlIzMVlGMzN6RTdwXzB6MWZsdmVhTUZ4d25qQ1hqZWlXa2FHSHVsN0Iyb2VVYjQyWkl2U3JjcFhUcENwbF96Z2dMUkZOc2x4RTVUNTZJ?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -625,52 +625,52 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46086.3615162037</v>
+        <v>46087.53501157407</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>London Marylebone Incident</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("London Marylebone" OR "Marylebone station") AND (incident OR disruption OR closure OR police OR bomb OR explosion OR stabbing OR shooting OR "suspicious package")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Major disruption continues at Marylebone as delays extended - London Now</t>
+          <t>Diefstal uit auto leidt kort nadien tot arrestatie aan andere kant van land - Nieuwsblad</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Major disruption continues at Marylebone as delays extended - London Now</t>
+          <t>Theft from car shortly afterwards leads to arrest on the other side of the country - Nieuwsblad</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 09:26:57 GMT</t>
+          <t>Fri, 06 Mar 2026 14:35:23 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxNNEZOak9CQmlPMkdrRFNILVpCa0c0QTdGenJiMmhZUVdWWWFfbDZQRkVmMDNmT2ZsUTE3VGdtUDRORVpIYWYyU2dSRTNpcUhNYWZZXzFYczF5c1B1SnJ5T0phUGwtT05QVjhDdXdTbEpwUWo2bjBfVS13X3NhWHdsNzJxcXUyVFJvQjd1WklaRXp6QllOdy12T2t2TUpfR2RrMFFr?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxPMEE3ZGkxQnVpREZyRHdvWnRyamY2OERYWm5iN0F6NnFTaVlkUThvdXJBM3VObkFFY2NBdHBhYS14R2JYUzAzNHZxUGo0d1FRdXF1VzY4YjdaSi1sY0Fwd2ZhVkQ0d3IxMlpyS3BEVXNrcENkdE13NnhIVFk0M0tUek13MkVJMjBvaWwxTGV1eXFSWDllOXJuVEFaS3o4aGd5Z0oxMGlWdUZhNEhuSGo5RkhGNkQ4WnBGaTVoaTlvemVWNVN4MlQ5N1NVN2F4NVFGUnhiVnFySl9ZRWM?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -680,52 +680,52 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46086.39371527778</v>
+        <v>46087.60790509259</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>London Marylebone Incident</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>("London Marylebone" OR "Marylebone station") AND (incident OR disruption OR closure OR police OR bomb OR explosion OR stabbing OR shooting OR "suspicious package")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>‘Casey 2’ inquiry launched into Met’s overhaul since Sarah Everard murder - London Evening Standard</t>
+          <t>Jessy Mackenzie getuigt na MeToo-bom in muziekwereld: “Ik werd als 18-jarige zelf gemanipuleerd” - HLN</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>‘Casey 2’ inquiry launched into Met’s overhaul since Sarah Everard murder - London Evening Standard</t>
+          <t>Jessy Mackenzie testifies after MeToo bomb in the music world: “I was manipulated as an 18-year-old” - HLN</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 14:04:44 GMT</t>
+          <t>Fri, 06 Mar 2026 10:08:11 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQRGRYNEt2RkxuTUpFLWlULUNkTzU0LV9zTUgzRkZ6dEt6aUNZWk9uMGJYOTlYeHNHd2JjZm9mUk15aUxNWVh2VFNMWDUtMExNdFp4X0x6N2RCak5iNHp3V2hvVW13LXlqRmNNalFDcXM2S2NOM29xNzFHdjBPZ3d1MzlWaGdPVVNuVTdwYm5oOGc0SHozWU5NdURJRGk4SEJzbmtRME1SSXNFTmh6WlJKdlI5V1B2Y2xhbWNvQk5tWElGNm5Pek9Cb1hqTzY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxNbmFXaGpuakhNRHo4c0pwWUNiV2laTWk2V3RSMWlWdXJlTnljZ2dSWnBHOGd1SmlaSnZEV1o0dzBaVUpoMjRWUzRmWnk3MFpyVEhuSzFMX0VYbDNiZkdxTVpnWXNhZVMzb2ZEZExnU1ZKMTkxaTFZcHR5dk94UHJRVXB1U0lEYUoyYTBxR2k5TEd6cmpBZGROcTdoX0owOWNieUtTX0k4WF9La3NWbHNtVU5kRmJVUVAxR0E5Vl9SZGFZc0QwY3Q4N05aQQ?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -735,52 +735,52 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46086.58662037037</v>
+        <v>46087.42234953704</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>London Marylebone Incident</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>("London Marylebone" OR "Marylebone station") AND (incident OR disruption OR closure OR police OR bomb OR explosion OR stabbing OR shooting OR "suspicious package")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Husband of Labour MP questioned after arrest on suspicion of spying for China - London Evening Standard</t>
+          <t>Woonhaven Antwerpen verkoopt samen met gemeente vijf bescheiden woningen in Maria-ter-Heide - HLN</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Husband of Labour MP questioned after arrest on suspicion of spying for China - London Evening Standard</t>
+          <t>Woonhaven Antwerp, together with the municipality, sells five modest homes in Maria-ter-Heide - HLN</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 10:13:35 GMT</t>
+          <t>Fri, 06 Mar 2026 13:24:38 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxORUVZbnJyTFJnaHFvMEs3M1ZPdVhfMFE3RGIwMXlhQ1pZOGd2WXI2elB5Wl9tZThnZFlaLWN5Zms5ZENfa1JKcmM1a2Y0SXZUS0w1bng5UmxCSkE1d2NIRWdEc1Q2emlMSV9sQjRMRnRZdG5nMkVyMUhmRTVndG0zWnRqcWp3dmdQN2tIY0llc25aZnlZdnE4VjFOZFdkZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxQM3ZMdWR4aFQ5RzZzZExEcDEyNXVLVmVqWVpvUmxJaTBoNG16U1duT21BbE95ZjVwOWh6OS1icVdrNXBnRXhJbWRUOTZLTTFVN3VJM0Z4ajQ2V1g3ZDRaQk9HejItelZaX1N0a2tLRWM3OHZJaDVxZjBHaFdIVDBoTVlnUUZjR3I1T1luM3ZQRkFIcjd6Rzhjcmw2dXhfSjlzRGJ3QWh5TXFzLXFwRlI5cGNPUlF6T3lXVmlGMHgxcFZiTFpVRTNCclRyaw?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -790,52 +790,52 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46086.42609953704</v>
+        <v>46087.55877314815</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>London Marylebone Incident</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>("London Marylebone" OR "Marylebone station") AND (incident OR disruption OR closure OR police OR bomb OR explosion OR stabbing OR shooting OR "suspicious package")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Raver nicknamed Nasty guilty of killing deaf woman with single punch - London Evening Standard</t>
+          <t>20 minuten file op de E313 naar Antwerpen door defect voertuig in Wommelgem - HLN</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Raver nicknamed Nasty guilty of killing deaf woman with single punch - London Evening Standard</t>
+          <t>20 minutes of traffic jam on the E313 to Antwerp due to defective vehicle in Wommelgem - HLN</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 13:22:34 GMT</t>
+          <t>Fri, 06 Mar 2026 13:28:27 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNYkpSTEpxbHo2QjFzS0l5RUtCeXpaS0huMzhYQ01oS2NoYTdweHR5cnJtM3M4eXVZZmhWLVdFWlF2eWUwbXZvTHNVVF95TFN3ckh5SURGV1U3WmRVQVhSWDdUZFY5MXdpZnBNMHlCdFZyLTZVTlJVd3owNUtyNG1VcTlPNWdqbS1Ea1RaR3pRVFl2bk90dEZJaDNBM25UcUU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxPZ1k4Y3pub0dQVVFhVTU4MEtqZDdBX29GcHBPWnNmcnlpdnhnbVp6WFZjYXZCTGlTNFBkWnlia2hJN1c1akZjZE5QNk1VVzVYRGNsMVVwV2M3TUxDbWYzQi05VkdRX3RzUm9ReGJiTjEwenpvQlNiZXBmVER0c1pnVjU1aXA0eEJQWktoN252RDZMbVFISEc4VllvS0tqblItUFJLYml3TjhqYnpoS1ZCQ2FucnM?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -845,52 +845,52 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46086.55733796296</v>
+        <v>46087.56142361111</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>London Marylebone Incident</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>("London Marylebone" OR "Marylebone station") AND (incident OR disruption OR closure OR police OR bomb OR explosion OR stabbing OR shooting OR "suspicious package")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Risks from Chinese spying ‘not receding’, Speaker warns parliamentary staff - London Evening Standard</t>
+          <t>Nederlanders vinden oplossing die Antwerpen ontziet tijdens werken Westerscheldetunnel - HLN</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Risks from Chinese spying ‘not receding’, Speaker warns parliamentary staff - London Evening Standard</t>
+          <t>Dutch find solution that spares Antwerp during Western Scheldt tunnel works - HLN</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 11:48:45 GMT</t>
+          <t>Fri, 06 Mar 2026 07:41:46 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxNLTlsTzJZS3lUWUl5Z2lfRjEwZDFkaHVXTWdFUzhtRFZINmVYUnpYQ21XdklOM3MzMlhLYmsxRW5URWk1UFViUENZaElPUkNiUXZlc2pndFdtWjdtVGtrTzVYRnFmNmNuY2tLelhiRm5Uemh3NnRSdGxSN0REVFVMRmdpbmVSZnJSY1ZvRkZJTG5qbFJZUnpGTFZvZlBnOFg4cy1ici11eDVfNXJfWi1BVw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxQY2FuVjljTWlhclhUU3hibHBRZW1lN3RwaDlHSkMySkpmSzFicjVhRHdfdnU4V2tjd0VISHVVRWxFeFdkTmNoYWI0QTZYa0ZhMWtiZmM4aTk2UzF5ZlpCSmNGWG5YTlo3YzZZcGN5TDJfSGRMOFVWWEpKaTFOQXpEX1BKM2VZYVdFT1Z3U0s0LU5ueHNfYWIya3RwTGRGLUZ3NGJ0clNnTWI4dEk1R3FQWHk2RURrSTJoWUtWdHhwZFphRE0?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -900,21 +900,21 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46086.4921875</v>
+        <v>46087.32067129629</v>
       </c>
     </row>
     <row r="10">
@@ -930,22 +930,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Gewonde bij steekpartij in centrum Antwerpen: geen levensgevaar - VRT</t>
+          <t>Stad Brussel lanceert plan tegen straatintimidatie - HLN</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Injured in stabbing in the center of Antwerp: no danger to life - VRT</t>
+          <t>City of Brussels launches plan against street intimidation - HLN</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 17:04:04 GMT</t>
+          <t>Fri, 06 Mar 2026 13:58:01 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxPVXFjb09feVVNLUtDRS1FYWNmQ19ZMmFST0VvOXZuNlhTVFBPSjVSUlgwZ2ZrTTZJMGkzSV85aXFWb2lQa1dUTlA4ckNBLUNsbWFVSnJ2NkZNc04yNS01MjVuU0tPTTV6SVFMR0dHMS1fYlNrS2VtdzlvVjF6aTNxY1hfazJOUDFMMjNmZE1aTm82QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxQcmNKSnprMTA5OEpvR0wyVVNTUTY2SnNnQy1pSlhlbGJ5TzNyS0c5bWFoUHk1Wi1BY1BCQTJrc0U1aF9HSFVvVUMzdFpxa09TS0ttc2Z3aFh6X29zdDN2ZDNCYW5nVHd4RGhjTFhvYktGTHNicnZxWGt4MUZtM2s5NTAxLXdEUE1EQUVqY0x1dmY?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46086.71115740741</v>
+        <v>46087.58195601852</v>
       </c>
     </row>
     <row r="11">
@@ -985,22 +985,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Jessy Mackenzie getuigt na MeToo-bom in muziekwereld: “Ik werd als 18-jarige zelf gemanipuleerd” - HLN</t>
+          <t>Bewoners ontwerpen eigen carnavalsmaskers in residentie La Cambre - HLN</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Jessy Mackenzie testifies after MeToo bomb in the music world: “I was manipulated as an 18-year-old” - HLN</t>
+          <t>Residents design their own carnival masks in the La Cambre residence - HLN</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 05:49:43 GMT</t>
+          <t>Fri, 06 Mar 2026 13:38:19 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxNbmFXaGpuakhNRHo4c0pwWUNiV2laTWk2V3RSMWlWdXJlTnljZ2dSWnBHOGd1SmlaSnZEV1o0dzBaVUpoMjRWUzRmWnk3MFpyVEhuSzFMX0VYbDNiZkdxTVpnWXNhZVMzb2ZEZExnU1ZKMTkxaTFZcHR5dk94UHJRVXB1U0lEYUoyYTBxR2k5TEd6cmpBZGROcTdoX0owOWNieUtTX0k4WF9La3NWbHNtVU5kRmJVUVAxR0E5Vl9SZGFZc0QwY3Q4N05aQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOUFhQUFl2Z1pkN21IR204TWFLcWhzS1pvUWxfeFVuTDlaem9mMi1fdDhNZXNYNWp2aEhRcHVDZzdPQTdRbDBDNkFyVmw5aG16cTdVdHB4XzFzUU9KTlhCdUdYSHhUbTFIMnAwaFJTQ3ZvSDkzNk5hdnVjdXc2dzBZU2pZSERrVVVDZ044QzNxcHA1Q09qTTRGbFh1eWdOY085bGZ4Qg?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1024,7 +1024,7 @@
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46087.24285879629</v>
+        <v>46087.56827546296</v>
       </c>
     </row>
     <row r="12">
@@ -1040,22 +1040,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Hij fraudeerde voor miljarden, zit nu vast in Antwerpen en wil absoluut niet uitgeleverd worden: wie is Mehul Choski? ‘Sinds zijn arrestatie worden we gestalkt door een leger journalisten uit India’ - Humo: The Wild Site</t>
+          <t>Groen wil “volwaardige fietsboulevard’ tussen Antwerpen-Centraal en Berchem - HLN</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>He committed billions in fraud, is now stuck in Antwerp and absolutely does not want to be extradited: who is Mehul Choski? 'Since his arrest we have been stalked by an army of journalists from India' - Humo: The Wild Site</t>
+          <t>Groen wants a “full-fledged bicycle boulevard” between Antwerp Central and Berchem - HLN</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 14:42:00 GMT</t>
+          <t>Fri, 06 Mar 2026 13:33:18 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizwJBVV95cUxQYk0wNDFJbHNnMUp3VF9MU1ZfZkttOGkyM1FCbWlUNUNKZUtoOGN5UG5jRnNibjFJczlXNWFIYlVWS2drUkFtUlg3Z290UWtaVDFob19TOUFHZUQ0bS1pZ09SSTBjVTRwN3gzSFBoR1A5SllEcGEtR2FRTERqTDBhZHE2eTh4eHJuZzJfUGZadGg5cFlWWFNMa19vOWRRS1FLQ043dWJ1ZkRxRVR3ZTZGUjlzNGFaMDJKSndSNTliR2ZncXUxM1U5dkwtVTA4NFZuUVpFR29NWF9DOFJxcDBaenNGUGNwOGloYXpPRGY4SFFlYnRLZy1iVkRnLW1LUjdDTjF1QmVIeTBCQU5XRFVWeVhGY3I5aHkwbEFJX1JSTDNaaWk4UHhyWUtkMWlKd1hSeW5CdHZoX3o0OTlzR05Lbk5kNnZsSjUxLXRJZWNSYw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxQU0JQLUFteWVoYmFtc0pjSEFuanNraXVGRzJFSzRuSFI1bHdydVRObDhEVWFZTXBJbm9TQlBXTk1VRGtCSjI3OWpHMEtpbXVtQU1ja28wMHFUMmo2OGUtQTYwT0dMT3cydk41U09jRE5HSFA1Vll4aU15cWhGVjJpVjBUbkZ6bnZneG5DYXNDQlFVeFNNU3ZrdGtUaGo4Nl84eFdsZl80QU5wV0tYMW9JODV3?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1079,7 +1079,7 @@
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46086.6125</v>
+        <v>46087.56479166666</v>
       </c>
     </row>
     <row r="13">
@@ -1095,22 +1095,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Britney Spears slingerde over de weg voor arrestatie: zangeres “extreem emotioneel” en naar ziekenhuis gebracht - HLN</t>
+          <t>Drie voorbijgangers redden persoon uit kanaal aan metrostation Delacroix in Anderlecht - HLN</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Britney Spears swung across the road for arrest: singer “extremely emotional” and taken to hospital - HLN</t>
+          <t>Three passers-by rescue a person from the canal at Delacroix metro station in Anderlecht - HLN</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 05:52:43 GMT</t>
+          <t>Fri, 06 Mar 2026 12:23:01 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxNcnpOSEFlSGJZeUZqQ0JuUl9TZVJ5cnU1eGJTeTJDUEVIc1F3RDhXQ2xydWdRcVdRVHM1WGx0djYwdmhBckRzWXBoWVdCbUtyRTlxR3pZeWtNZEJQMlZYbjY5alQxRmVPRTBydnpMNmVDNC13dUhkOXRtZHd1RkIxR0VURUcxYUpaNFVJdFREQ2hzMHRKZGVXejgteEtLZDlNTzUwcnRaWE5TdmF5WFBBeEQ2WEhic1RIZWVTMk9SbGZRUkllY3QxNzVGOUtSNFlrMWdEdGFrWTZCeGM3a2RMRnNFNA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxPREw1UUFQNllDVUFZMEhGeW8tal9Mdk1nZTNWUkRwQklLTXhNTFltWjZtZUdIUkx5T3JQaGkxUFBsNi0ybE1qQU1lUVdTOHh4TDFvSm94QUxieFNtMmdBUWx6eXc0YTBnX0NwWWlNM1NTQ3VPTzdvQktsMFhFMTlBSzh1QmpsN1d3WXY0aGg0Yi1aU2V5OTFxV0x0VGNSSEQ4TUJIeXJ2TkxZS1o2NC14bDJzVTJHUnNKYkszeDQ4VGU?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1134,38 +1134,38 @@
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46087.24494212963</v>
+        <v>46087.51598379629</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Jente Bogaerts (Chocolatjeeke) is ‘Strafste Onderneemster’ van Antwerpen: “Ik wil vooral niet te groot worden zodat de kwaliteit blijft behouden” - GVA</t>
+          <t>Exclusive-NATO’s Rutte does not see need to invoke Art. 5 after missile incident - WTAQ</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Jente Bogaerts (Chocolatjeeke) is 'Toughest Entrepreneur' in Antwerp: "I especially don't want to grow too big so that the quality is maintained" - GVA</t>
+          <t>Exclusive-NATO’s Rutte does not see need to invoke Art. 5 after missile incident - WTAQ</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 04:59:09 GMT</t>
+          <t>Fri, 06 Mar 2026 09:45:20 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgJBVV95cUxQX0plWHRybDFBTHViUF8tM3h1eWpYaG4tTFVNYllTSkdVdG9nTEpHb0M0cVp3eDcwN2FTckU2UWZVZkFiSHk3cVJic2I2Vmdid19XZ2RNZFRwYTBBZWFGMkNKRVFOZFFORG5aTExfc1NzYnR2U2lPTmlnWlRfYWgxRnAwSFFDUGpZLWN5UFAwMkpzdEs2Y3E1VVQ3bFlKOFVwV0p1VVRhUDBFOGxHYTM1TVNlblVhX1lwdk9WV2FqRjdHSlpVYVMwQjFycHRoQWQ1QlMyLTNRUlZmanhlWGRQVzVVV280TFJkNHhvd3dvLXBPS2pKZEFEUGNkc3pneVJHLUh0WHRtaFFHMEpQbkF2dHBuWUZhT3dFZHZaN3FpeVFEc2s2ZmdXQ2lfQjVjODl1RzhVa0xn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQeE1KT2p0eEJXTmw4TlRFVG9zc0dOZ3FXdEFOLWxTRmdvcWx4bVcwaXVGUXdPdWJoLXB0aGx1VjczNVVEb09xVnhGSHNrampDMkJNc0ZGMDNoVHVzcDdhVHRoQ1pwMXk2TWlqbVE4WHJmWnNOcm82NXVxVDJsMXVHMHpvdnZCdUtyR001cHdfOXB4WUJSa2haRUU0NHZnbnVxeHBNTWNJR1kwNUk?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1185,42 +1185,42 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46087.20774305556</v>
+        <v>46087.40648148148</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Wat te doen dit weekend in Antwerpen? Van drumspektakel tot boekenzoektocht - HLN</t>
+          <t>"J'ai atteint une paix intérieure": une rescapée du 22 mars a rencontré l'un des condamnés des attentats de Bruxelles - BruxellesToday</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>What to do this weekend in Antwerp? From drum spectacle to book search - HLN</t>
+          <t>“I achieved inner peace”: a survivor of March 22 met one of those convicted of the Brussels attacks - BruxellesToday</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 05:01:12 GMT</t>
+          <t>Fri, 06 Mar 2026 11:00:00 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNcmZkUkVvOC1fc2s1QkowTDFlNTE4aXMwUkMzVzhHa3BhNkVPZ1did284S0tDYmNzaGY2Y0tTd2RITjdwalFVNUxwQV9oNEhWT21kaU1wU1NhQWxELWk4SjJBTjRkYmpMOWU3Slg3eGJEc1kta0dVaVdJaE0xMFFfUkNyblcyZkhfcGxYUy05WVQ2VnpNb0dvdTRKNm5MeU8tTlVFTmVDNjBOaDJkN0JFX2Frcw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxPZlFlWXNkRmZlZXZnTGFYeTFld1JleUNiaXVsMTgyMDdGSE8tS3J0WUhLZ0loTU43ZkVCaEo3cmNteUlaZnh5dS1zVGllZllMU0JxTThFZWtOUHp3N3JkNTlOQnVkVkZLOWZFRGpvS28wLUR3aC1NQ3VJem1FeTVHQ0lkRUxDSjNNTXc?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1240,42 +1240,42 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46087.20916666667</v>
+        <v>46087.45833333334</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Iraans-Antwerpse Wali Sediqi stapt uit N-VA door partijstandpunt over oorlog: “Uitspraken van Francken doen pijn” - GVA</t>
+          <t>Hammam de Schaerbeek : Comment un simple conflit de voisinage a viré au procès pour meurtre - Bladi.net</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Iranian-Antwerp Wali Sediqi leaves N-VA due to party position on war: “Francken's statements hurt” - GVA</t>
+          <t>Schaerbeek hammam: How a simple neighborhood conflict turned into a murder trial - Bladi.net</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 19:39:31 GMT</t>
+          <t>Fri, 06 Mar 2026 12:00:00 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxOZEY2SjEzVTlJdlF4Z3dWQzlacGlnTUg0bnFEbENtMVNLWWpncmM4ZXBQMDV0c1ZqY1NEOU82Z09jSHZreHg1QXdCRVhOdDNJUmIxMW1hNDZnMnVEYWs1bHBFSnhtc0RFdkctYjI2bHAwMDZKa1hKWHYwWFpreVY1OHczS0prRmQ3R1pkcGRqdlFQVDlUMmhRU3lDNGdndkFIOGV5ei1LQ3l3Qm9iQmxJbHNiTjNRbDNzSHJmdDc4N3RfbkY1Zk9WbkZtWUtER0hkem5CWjIzd0dmQU52SU5jNm1kbkdSTXN6VlN2LXVjWWtHaWNyWE96eGNjQWJSZ3JsZVBQYQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQWnFXYmRyakhQdVhWTnJZUXFqcWhNanNPeHQ4MGZpQnk4YVlabFRzT0l2Z1Q3X1JYNkt4X0hFYXJoekFIRUJCMHZVS3pNeV9HU2s2NGVEUTNuV3Y5M3o5RjR1allhTjFiNUFlcVZvWWdLRTdlQnpxX2ZCOFJiYkZuRXJER2JuOHVEVzJEVEJ3MDBPdw?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1295,42 +1295,42 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46086.8191087963</v>
+        <v>46087.5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Drie kwartier file op E313 naar Antwerpen door ongeval bij Antwerpen-Oost - HLN</t>
+          <t>Luchtvaartbedrijf ASL uit Hasselt evacueert Belgen met privévluchten uit Midden-Oosten: "Situatie verandert permanent" - VRT</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Three quarters of an hour traffic jam on E313 to Antwerp due to accident near Antwerp East - HLN</t>
+          <t>Aviation company ASL from Hasselt evacuates Belgians with private flights from the Middle East: "Situation changes permanently" - VRT</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 23:16:55 GMT</t>
+          <t>Fri, 06 Mar 2026 08:12:09 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxOZlpocl92Q1c2ZVdZbnY5RWlpeVBaai1MeDl2d0FvLVd5ai00Y3h3c2RBQzQzN29lOGtDV1lPTmJPME5KZlRUTWpDbHlrVnF3RWl4M1JfYnlCVGl0X1pTWmlzNDVLVVFaYy1FMWZiZTgtZXZpTWVrT05SQ1A2V1hjU0lQS0tLYXY3MFVGb0JrcHk4clZNaFEweDRwVnQ4YXBVN1ZGWVlIQXRZeEtzLTNBMGZn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPTVQxZGFRNVE2TnFOVkMwYkpfdnc3THk2S3BBQ196NnFmRDFuak0tbWluYVhSRGtXcEthUkRjQUw0SlptWHV6a3RIVzNERmtGZEhVbmhOQ3VpaWVtYml3ejBiMnFuSTJUdUUzSTdfU2pMLXh0Y1hGVGJWVGE4dXJZLVhCX3NFN3NHRXVpWE9SekpaWkZvSFJEMXptQ0NISXJXZEpN?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1354,38 +1354,38 @@
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46086.97008101852</v>
+        <v>46087.34177083334</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Leerlingen van het Stella Matutinacollege ontdekken de Belgische politiek in Brussel - HLN</t>
+          <t>Drie verdachten opgepakt voor brute woningoverval in Breezand - rodi.nl</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Students from the Stella Matutina College discover Belgian politics in Brussels - HLN</t>
+          <t>Three suspects arrested for brutal home invasion in Breezand - rodi.nl</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 10:18:10 GMT</t>
+          <t>Fri, 06 Mar 2026 12:34:22 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxQaWNBS3NPQjk2TC1WNmJmd3A3bEV3N283bFQxbjFkQWU5WTRmbmljTHBEQ1ZmUEw4TjNCMnNuaUxKOGlGSzA2Nm9fNllzeTc2R0hWMDhJdVhfeDNHLUFxbFJhdEZXblRrQ2trVGxzcWdfS2tOTFpUWjNzT3BNSUtsLTRZV0Mzd0Myd0k0ZHdXNXFua1NwRlJkbjM1SDIwV3htM082TVFiMkFjOWxwQUlUc1c2MC15N2lqdFE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOX2Z6Y1lGOGNaMi1Db21SeWdLS1hGOWRidDB0aVJTd3JZNzZPRVJQb2dYN2ttcUNreFROTFZiZkdiaGtoYXZlUS1Ea0hqbWJFRzZLSE1ma1hwS0E1SWRpRGlSN0haR19HSWkxcHZPdzRCREVmUVZsTF9EV2VOZ29maU8wNm9TcHFmZFJrMGh4anhfSkpYa2drTEt6ZFdRWXRReUdrVk1pZ25UX0xXQXpmWEl2OA?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1409,38 +1409,38 @@
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46086.42928240741</v>
+        <v>46087.52386574074</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Local Town Maasmechelen French</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Mondriaan sommeerde skaeve huse-adviseur kritiek terug te nemen onder dreiging van kort geding - De Limburger</t>
+          <t>Des passants sauvent une personne du canal à Anderlecht - BruxellesToday</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Mondriaan ordered Skaeve Huse advisor to take back criticism under threat of summary proceedings - De Limburger</t>
+          <t>Passersby save a person from the canal in Anderlecht - BruxellesToday</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 20:15:00 GMT</t>
+          <t>Fri, 06 Mar 2026 11:49:32 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxPa3N3Snc4WVhFOGlOcHdmbWdIQ3ViN1RJRjE2VzJpczNqYk9QYXdfbWpqVmNsMGlxNmVTOGRXOWhFRGhEeVVzUEZ1azM0c0libUZOSlFyZi1JZDE0Yk9lbHVDc2RjemlubTR1WTlucUJnYThSQ0lxdklSaWhFUHdjcHpVbndkV2hFNzh4cUFwTllXcHBFLXQ5d1ZYbmxKZjRPNkVoSVBLbHdoQ3FlYTdncGtBNUs5QUFTVFB2RE9IdXVuY1dzZ3VrcE0xQ2VkY0lWRzRlREdiTHJfUWc1d0xEdHdn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxNejRST0xJNUQtcHVzOENZSE5LRmJFdDE5bklaWjJPS3NpMDVvVkNJcmJ5eVljR3ltSWVEaGR4bXgzM19FZXc5ZzgtSDAzZ3NRazJIQUE2dkJCRnRVaGhJSDdQcWhIU21XdmhRMlk2ODdQa2NqczVfbmJ2OGw3YnUwa201SUc?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1450,7 +1450,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,42 +1460,42 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46086.84375</v>
+        <v>46087.49273148148</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Simulator in Brusselse Beurs laat je straatintimidatie door de ogen van een vrouw voelen - VRT</t>
+          <t>Herrmann würdigt zum Weltfrauentag am 8. März das Engagement von Frauen bei der Bayerischen Polizei - aschaffenburg.news</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Simulator in Brussels Stock Exchange lets you feel street harassment through the eyes of a woman - VRT</t>
+          <t>Herrmann honors the commitment of women in the Bavarian Police on International Women's Day on March 8th - aschaffenburg.news</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 06:46:18 GMT</t>
+          <t>Fri, 06 Mar 2026 11:24:25 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxQeVl0ZVFCeUFqOEM1MFU4ekVhWDI5Q29iYXdRSXpyZHVCeTdIVjVrektHc2dLOW1hcFA1Yk9aTEo3WEFYdU1KdjdudFFKOWlIQ3FvcTFWcFVYM1dUZEJmOXBJUFpYbFpkcWt1eVl2Z3h3N1JsNlhTSlpKYXlHbGlaSklmV2huZ19KWl9LNGRtd3Zsdlp3SFBlUVlXTzk0XzdD?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOYmk2SzhsLUhkdFEtSE9LMEJFT3FiMGJvdks5dVhQOVRta3YzZUVUektCQWs5Yl9HT3JreUZuSWJTRzg2ZjNxWWEzZktmcDMzUDlnVWNNMGhfb1NhMm9NLWhFVmNPS3lCY2pJNjhJYnVlUEVLd2N5MTBnTDBJZE5NMEtPdHpTek1nNGdFR2NyZWpPTGxJV3NjZFpBWkVGMlp3em50QjFkQ2pmU25UeEs0N3otbE82X0dvWXBLb2VrRFZFNm9rTlZWa2lMeEUyWl84NmNzY2M3SUdWNVdvYW5sUEV3?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1505,52 +1505,52 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46087.28215277778</v>
+        <v>46087.47528935185</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Overleven­de van aanslag in metrostati­on Maalbeek ontmoet ‘man met het hoedje’: “Als je oog in oog staat, kan je de mens niet negeren” - HLN</t>
+          <t>Polizei sucht nach Zeugen: 34 Jahre alte Frau wird in der Würzburger Straßenbahn verbal bedroht - Mainfranken News</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Survivor of attack in Maalbeek metro station meets 'man with the hat': “When you are face to face, you cannot ignore the person” - HLN</t>
+          <t>Police are looking for witnesses: 34-year-old woman is verbally threatened on the Würzburg tram - Mainfranken News</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 06:59:50 GMT</t>
+          <t>Fri, 06 Mar 2026 09:33:01 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxNTWlGV2dfLTlIYjVXS1Byc091SVUxSWc3VWttSS1KTld1ZGRsN1FtQWFXSFV4QUtqMGNBcEtuVVZlUjh1UFNxUlkxSXFxZ0Izc2hwZVRjSGNBMEk0LThwNlV2S1UyX25PaFo3Z0JoWDNTenNfb0ZPTV9rTm9XYmpZWDRIUmdfdW1LSmp2MUVFY1Z6dUZJNmd2WGNxamEyc0hlUjYzVEtpMDJUUnROdWJmMWVLUmxUQ3pXUlVyTXdpREI1c1pNWVdVdU9QY1lBazlyVWQ3SEZHVFE2TF9NcTJieUcyYjFIb1pzNXZOeE8zdi1TRjNFMlp5eUhQOA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxONlRuRjRFcHlqR2Q5SkJaUUdWcEhsNGFjOUJJRExDOG1adVRqemN2R1hDS3BsTDdYTGpZQmZaYkhaOG9JdXphMk5KVFduTjdfeUtVUzQ3ZXlXeDZrUjdPMDhybHpRVW1jUm4zRWpTcTNxMUwyaE5iSHlybVJaMlpFTndvUFp2QTYydFFyVDRiamNQUVJyc1QxYl9kMUpzUk1oNkx6NndJVDhVNF9xRXVObGd5ZjMtdzljdE02eEdxUHVMOEdmTkVXbWtyU004dw?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1560,52 +1560,52 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46087.29155092593</v>
+        <v>46087.39792824074</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>'BouwBoost' moet meer betaalbare woningen opleveren: zoveel leegstaande bedrijfspanden telt Antwerpen - HLN</t>
+          <t>Kreis Würzburg: Betrunkener stürzt mehrfach - Zeugen verhindern Fahrt - inFranken.de</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>'BouwBoost' must deliver more affordable housing: there are so many vacant business premises in Antwerp - HLN</t>
+          <t>Würzburg district: Drunk man falls several times - witnesses prevent ride - inFranken.de</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 07:31:45 GMT</t>
+          <t>Fri, 06 Mar 2026 10:00:00 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxOdnJvT3piSUQ0Q3RhelFYQzg5U1NzNE9wdGxWMVhHbkpxOWJZY2FnWFFxeXRQcGFvV1hOS20zMTI2SmphMDk4anNxQW13dm5haWtTWHBjSWNZcTVnbUpGNEEtdnl2Z3dtRkRCUi04R2xDZDNXbUZYUEFzbE1DeGotajlhSmVnVHFRVExCYnJZRk1KWjRVNi1hem5yNWxpQVpNNWtVamk4dXVjUW9vdjYzbURyak1rUjZjcTdwNHlZYzMyVkdEVS1GeHkySGloZW5JS2Q0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxPVzJONWxZUFVNZXZIR0FudGxqVnRiQWxRbzdnUTI2WWhjNTdnUmVBR3FPWkp1eWozSGVLVno3RlY3eDkzcDZERjJSZ1BiS19NM1Q0V2swdG1kZEtldTNMdkg3Tzc1T2VhUG91YUdIM0RRbFZxajQ5aGhaNER0b1Bsal80b0NoYUlfVUoyX1VIR01UY0lDai12cTZjTW9Ic2NXRi1rNExLT3VCRUxCWXBnLUxTNGtpZ2xlZTM1QS1EbTFmbjlpaGc40gHHAUFVX3lxTE9XMk41bFlQVU1ldkhHQW50bGpWdGJBbFFvN2dRMjZZaGM1N2dSZUFHcU9aSnV5ajNIZUtWejdGVjd4OTNwNkRGMlJnUGJLX00zVDRXazB0bWRkS2V1M0x2SDdPNzVPZWFQb3VhR0gzRFFsVnFqNDloaFo0RHRvUGxqXzRvQ2hhSV9VSjJfVUhHTVRjSUNqLXZxNmNNb0hzY1dGLWs0TEtPdUJFTEJZcGctTFM0a2lnbGVlMzVBLURtMWZuOWloZzg?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1615,52 +1615,52 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46087.31371527778</v>
+        <v>46087.41666666666</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Politieagent redt man uit kanaal in Molenbeek: slachtoffer moet gereanimeerd worden - HLN</t>
+          <t>Neustadt: Vier Personen bewusstlos in Einfamilienhaus aufgefunden - aschaffenburg.news</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Police officer rescues man from canal in Molenbeek: victim must be resuscitated - HLN</t>
+          <t>Neustadt: Four people found unconscious in a single-family home - aschaffenburg.news</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 16:33:12 GMT</t>
+          <t>Fri, 06 Mar 2026 10:51:28 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxON19odDlPTDZMTFgtUnZlS2I1UXRSSFY0dkxoYlBvYnM4bktJOW5Vd2dXbEhueWlXZjlfaGlSc0Y3cDRvR1JoLW1MNkstZWdVazFYdHc2ODFvZVpzMC0ybFlGLVFDOWRkanZXM1k4U0xLcWhjdWtValZPY0Z4RElwS3QzM1RoT1Vhc2trRGRQQ2Y2Q1FObVo1ZUktYUp1MjlTYkJGazBBdUZvTWdkMUxNNU5ka0VkZ0hvSW1v?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPNFE0eTdvUU1yc1V4SW5UVXBUMkxPcnpPelN3d0JGYmhlc3RVcjNGbnJTam42cXRuamtIM3dQOEtzTjBVVzUzS1NGdXRSSVg2bkZJLXRvSFVGRGhGbkJRRjA2VDZjUnNOaTloZWRfOWhRYWYxaG96TGhKR29HSnZaUEpQSkNIR0RmTVNfWk9hMHRDR3EyNkpJSHNKYkJTSksyZktEUThaNzNOUUtyaUVj?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1670,52 +1670,52 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46086.68972222223</v>
+        <v>46087.45240740741</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Centrum Jean Gol vecht uitsluiting van Brusselse Boekenbeurs aan voor de rechtbank - HLN</t>
+          <t>Wahlplakat in der Steubenstraße entzündet - aschaffenburg.news</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Centrum Jean Gol challenges exclusion from the Brussels Book Fair in court - HLN</t>
+          <t>Election poster lit on Steubenstrasse - aschaffenburg.news</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 17:07:58 GMT</t>
+          <t>Fri, 06 Mar 2026 11:14:03 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQZ2FYLTBWSDlvdnVGbEY2QjhMNUdmR2xRMHU1OE4xRVVoS3pZU1BxOGlCRUdXNnVYRjd3WnJaR19MRkhOUTlUMVNYczQ3SVZFVkFkdHhCc3QydEVMcHRPMHRQclpENTIzcG1ReEtqME1jZThjNWw0MlRDSk9JTVY3TlJEMG1Pci1HUVYyMHRxSDkwX0doRkxXek16NU03NFBVSVl4SVRmYUpITG5pZGUyU2pFNUY0ZXlJanZZ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxQZTVUWFlCb3VqU3d5aEwySllNbTYyVEdJS09CeXdsSXNpRWd2bXpIdHZDVkhWZkM5UGp5U3VqRUNjWWNOdDk3VmlIb0Zxb1JTNXFEdTNlQnoyM2tuaW5rbW9FV1ZyX1VtM204SjdWOVAyVkJrcnRHVlpBWHZTQTNKbVNycDh1emJKSDZpQ1V2dFRmVERQYjhYeDdtODFJbFVCX0dMU1dsQzUxR2Vha1p6d1FCbUF5ak1ZZlBGQnQyalFMREJI?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1725,52 +1725,52 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46086.71386574074</v>
+        <v>46087.46809027778</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Bromfiets vlucht weg voor politie tijdens controleactie - HLN</t>
+          <t>Mit drei Promille am Steuer: Polizei stoppt mehrere berauschte Fahrer - Augsburger Allgemeine</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Moped flees from police during inspection - HLN</t>
+          <t>Driving with a blood alcohol level of three per mille: Police stop several intoxicated drivers - Augsburger Allgemeine</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 15:41:23 GMT</t>
+          <t>Fri, 06 Mar 2026 11:44:40 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOT29PMkZtem9ORktTUXF6b29naHlGVy03bXJvOGVkcm1uTlFWbjdpVUFfRDZmV0QyejZOS3c3b3laTldQYmhTd2Z3endZNGhNd0JMc2JtbU55LTlhUU02cEJTWGcybzlvUWtGZ2pJdlhUR2dsWklGS1hxcE5JQThqWkVYajd3OTFzVjZXeGw1MERHWFkxVmlJZTl3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxQZ3VfT2V3bXgyVERNTFF5b1pYZGtMdmZvRl9sTy01YnZJVmVCQTN2YWpyRTl3bXNWSVpNTkZyWWdnRE5WNXJhMjBYM3N2X3MxVExMbmVrUm1sbExGdUczUm0xSVgwQU5UTElsTTh4SU9XOFRxT0tHNVcxV25xcy1OaTBueFhXZHFOc2FSem91Y05waXFlWGtYc18zZ0ZHSUtsUFZId3Qzb0hLQ21meDRSUnc1OVJWcER4cWFoWERXZ18?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1780,52 +1780,52 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46086.65373842593</v>
+        <v>46087.48935185185</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>7-jarige Enzo verliest been na busongeval in Sint-Gillis - HLN</t>
+          <t>20-Jähriger aus Manching ausgeraubt: Kripo ermittelt nach Tat in Zuchering - Pfaffenhofen Today</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>7-year-old Enzo loses leg after bus accident in Sint-Gillis - HLN</t>
+          <t>20-year-old from Manching robbed: Police investigate the crime in Zuchering - Pfaffenhofen Today</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 09:53:07 GMT</t>
+          <t>Fri, 06 Mar 2026 12:49:52 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQQUxRNVFaYkM2dVN1NG56YWw4OHZaQnQ1aWJZRlp1cmNrbVpEM0ZQVlVsTWs0LV9yemctZkwxWmY1Yk1kWDM3ZGo4RGlmT1oyb19iUS1uY1FmYWFBT2FRRkZ6X1BmdmJlUERaQUdNNmNQYXVrdG1kTUlucExSR0J3d2NLYjBmaUFOalpmcGluUnFnbjRuZnFSNA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTFAzcVd0aGpEd3UwTTZUdUZpdElqRlVTRUZUYWJBWXVMU0UyZVZRSy14SnEwWXdWYzhObFk4bkZaNmdvcmlaVS14N2JlZThieVlfMFpxSmhFTHE3a1RWLUJ5b0lhQkNSQ3hxYVE?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1835,52 +1835,52 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46086.41188657407</v>
+        <v>46087.53462962963</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Dutch suspect denies firing gun that killed Antwerp girl, 11; Will fight extradition - NL Times</t>
+          <t>E-Bike-Fahrer kreuzt Straße und verursacht Unfall mit Motorrad - Augsburger Allgemeine</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Dutch suspect denies firing gun that killed Antwerp girl, 11; Will fight extradition - NL Times</t>
+          <t>E-bike driver crosses street and causes accident with motorcycle - Augsburger Allgemeine</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 18:30:00 GMT</t>
+          <t>Fri, 06 Mar 2026 10:02:28 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQR0V5WXBFM2Rfckp3d0xhd1dKYWVlcVNqTF9IeWROV0hrUzdlekM1SmtSSTN1NVYwd25TSlNxYzRrSWJHS3JzVmJMelRqaW4xSDVRNk1wcVpFVWI4dEh2aDgtUUc3ZlBVMVVvQjRyU3lCRkFrN1A0UUlubnpndHBZeldFREwxY3B4RGNHTnhQUUtNWU1kbFR1NXdTX1JxVk1LU2VLOGg2czZLVUk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxNV2R0NnFpN0VnRG9YVFFLYXY5b1F0TzcxdlVvQ19DaW9BRFJaUVpDdXdtNkhPVnJRN21rVTRTb1JLamZNU1VFNlFVNTRQNWYtZXNzSFV1ei1La29WOU5lbW5oQ1pIOEJJLUlEMjRLakppNzJUbjlsdkNmdVlrcHlQUmVOd0tNU1ZHd3E2T3Y5bGRUZjZzbVR4NEJ4dVpQSTdoamtIYXlQNGlWVlB2eGl3SU5oeDdkdG5NMkNj?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1890,52 +1890,52 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46086.77083333334</v>
+        <v>46087.41837962963</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Village Ingolstadt (fallback)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Exclusive-NATO’s Rutte does not see need to invoke Art. 5 after missile incident - WKZO</t>
+          <t>Pioneering Ingolstadt coach Sabrina Wittmann signs new deal - Bulinews</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Exclusive-NATO’s Rutte does not see need to invoke Art. 5 after missile incident - WKZO</t>
+          <t>Pioneering Ingolstadt coach Sabrina Wittmann signs new deal - Bulinews</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 12:58:54 GMT</t>
+          <t>Fri, 06 Mar 2026 13:32:00 GMT</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxNM0FqSFEtMzdndE01OU1VandUNm04Um1fM2l1MWlfQzh0WlllWEY2dzNBYnJOdF9FSllVUW90R2Rjd0xfYllXaGhmZlBnTmEtVlVjcUFPcmNMOEhTYi03UFhrZlo0SEZKOV9iWmE2OUV5ZGZlV1ZZVmZzQ2ZqLVR2T3JZNWR0VHo5S252emwtVE5nY2dXMTFFOWxPR3ZqckRJZkF4SVlCRlBTWXc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxPY2VLWkxyVmV0aUdUdm0tUU1iNS1uUmxFVVJyT1J5dGlhaEttbjd0UTVZUWdUbjdsX1FDZ3NGak12T25VM2lyenQzQ2kzTTJCc043YWF3cmotQTNkOGh1T0xYNkNuU0F0dUw1V3kzcGtoZWRWN3hQbDRpal85bm1nTVBUbms2b0E?oc=5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1950,47 +1950,47 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K28" s="1" t="n">
-        <v>46086.54090277778</v>
+        <v>46087.56388888889</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Village Ingolstadt (fallback)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>‘Chinese Starbucks’ where you can buy a €1 coffee is coming to Brussels - The Brussels Times</t>
+          <t>Audi Stops Accepting A8 Orders After Chasing BMW And Mercedes For 37 Years - Auto Spies</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>‘Chinese Starbucks’ where you can buy a €1 coffee is coming to Brussels - The Brussels Times</t>
+          <t>Audi Stops Accepting A8 Orders After Chasing BMW And Mercedes For 37 Years - Auto Spies</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 05:07:55 GMT</t>
+          <t>Fri, 06 Mar 2026 13:22:17 GMT</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQT0xCRlFwRl9uV0t3alMwcVBmenFzcHEzdEFjRHRzUXR0eWlNeVdsWXJrMGRCc1JQdVFRT0hUNUlzelV5RXllODBsZktoZlZRczluLWZsMXJoM3RLeFZYRTF3bjBpSnRIb0J4eGVfcnlGaU1CcE9JS1Q0NjZRUGluN09uTjVUUUJqdXhBM2JIN2NqZURnd0t6UWVZV2V6WVhtSDQ1QXEyeGR3c3N2WHFKczdXd0hlemM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTE51SklIQ2xIOVZJekNkaGhrekVRdS04MVZfVWpwdnlvZmxYSThZMXYxcUNfeG1YVHJKa203bXFHejFYQ01PYll5T001TUJ3Sl84dW9UOWxlaDBHamhPZUJ4QXNKeGVKU0hqT01XUFpn?oc=5</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2005,47 +2005,47 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K29" s="1" t="n">
-        <v>46087.21383101852</v>
+        <v>46087.5571412037</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Iranian regime “conservative”? Never, the mullahs are like 19th century Bolsheviks - Brussels Signal</t>
+          <t>Claim that Kildare-based company is engaging in oil price gouging - Kildare Now</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Iranian regime “conservative”? Never, the mullahs are like 19th century Bolsheviks - Brussels Signal</t>
+          <t>Claim that Kildare-based company is engaging in oil price gouging - Kildare Now</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 11:03:11 GMT</t>
+          <t>Fri, 06 Mar 2026 11:05:00 GMT</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOWWFncXVOemxxYm1qOXpycnVRQmRza0Y1NlByR0ZRY0ZQVmVBTlJoTEpoV1dxMENHekJVeE4ySWJSZXBvdTVZeFN1SVZVbERnLVBuZFV1R0syNHNEMThfamlVcUlZNnIzYXZsV185NXdINjhMU1VaWVg2YklRU2U4dXhERHRlMm9hWldXbWpZRVotNTZwUmpaQVFGWi1wM1I3bjlpNTJLQUY2NEpoaDNZU0RQNA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNaUxOb3Q2emczcGFQbXpaSnBRUGhORW5jUjgxRVlYODlEVDNKU0hmMG00ck5VcC13QklvUjY3cldiSzY0czJaNk1JZW16LVBBMFhaS2d0ZTM4U2tDTnlnaXRfNXRZSUFjZ1pwS05VeDRSN1RMUzBNR1B4QVk1Vk1pVzUzcXE1ek1aTkJRSkJJTEFuOUdyMkUzdjd6LUY4TFhrb21Jc3dnVTVEOXFfYkFLekdLUm9pQl9TM3BZcldB?oc=5</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2060,47 +2060,47 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K30" s="1" t="n">
-        <v>46086.46054398148</v>
+        <v>46087.46180555555</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>NATO’s Rutte backs Macron’s nuclear revamp but says US umbrella is ultimate guarantee - The Straits Times</t>
+          <t>Gardaí in Kildare make urgent appeal for information on missing teenager (14) - The Irish Independent</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>NATO’s Rutte backs Macron’s nuclear revamp but says US umbrella is ultimate guarantee - The Straits Times</t>
+          <t>Gardaí in Kildare make urgent appeal for information on missing teenager (14) - The Irish Independent</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 13:24:02 GMT</t>
+          <t>Fri, 06 Mar 2026 09:58:47 GMT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxPaFRaS05qcUN5akFOdXlYTDdtQW5LSE9uMTQ0TUUwc3IxT3hkYmtPdW5PLWtYMGRhaGNCNy1qcFl2NWhJZkw1REljbVdoNTZEMlVtN3R2czE4Vi1GYmt5eEFzN1FmaW9FY0ZtNlBJSWdDdkNvYVhobkpwX3FRVnBfbXEyV01IZGUtQzVRQTBRM1FCNjZlZW81M3hkSHVCUUpRR3lHUlNfaENSTmNTS29aa3dpUXh5RngzNkc3Zm0tWGQ4VGhJUk8wUXNnUzFSaU1ldlE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxNTXktWTNyZnoyVVhOZm9BTTlGa0RsbDBFRFZ6cDJMbDRKQXVqTkhnNVM1ZDlEeEFlXy1uQWZmNVJlUTNSQWl4Yktfa1NMbS1zM0FrX2dTTnVOME9vYWFja1BuTWxpVEwzZ1hoWmtoWjJOcGJFZ1l0QzhFUzktRDNNRi05ZjQtd2RQUS16YWdwNUFqa0lKcUJGaDgwNXNqMEpaa21ZQ0Qwc3hKampDRkhlT0tFSlR3VWRIQWdaZ2huV0VMMERoWWdtakc2bGEyRU1pZE9LZlVfVGthUQ?oc=5</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2115,47 +2115,47 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K31" s="1" t="n">
-        <v>46086.55835648148</v>
+        <v>46087.41582175926</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Antony Blinken warns US can't sustain shooting down '$20,000 Iranian drones' with costly interceptors as markets, munition pressure builds - MSN</t>
+          <t>Kildare eateries win big at regional restaurant awards - kildare-nationalist.ie</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Antony Blinken warns US can't sustain shooting down '$20,000 Iranian drones' with costly interceptors as markets, munition pressure builds - MSN</t>
+          <t>Kildare eateries win big at regional restaurant awards - kildare-nationalist.ie</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 02:58:21 GMT</t>
+          <t>Fri, 06 Mar 2026 12:31:20 GMT</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitwJBVV95cUxPa1d5QUF1VUpDajQwWDM1ZXhBNFBBWDhXbUtBSmR4WDFrVkw2dl9wY3pDWmUzdkNtSXVuaUdlM0ZiQjlTeVhqRFhuZ053Yjd5Nm45aVgzYTBaZlJheFA0eFVFaVJNVENOSXREMnVSQXVkaTIxeFhOUWViaVYyblpkRG1reG54b1lXZlpOV29Mb2ZoU0NiTENCdUlPc0V6UUFOSjFIUjJKZVhBT2lYaHFZNU1nRE9OZVpqQ09GZzAxcWlNV1dabmFrbkt3amtDNVk2azBONFlOZmMtX1NzaUF3RHFISnhpUEhtTnJUMlE0b1JHbVlpZjhtbzBtcjA1elpZeWlMZ2JZNEYxOXg1Q1J1MVgyVnFMcXJ6aWZMcjl0eG9LVDlqZktSdmZKSjctbk1NdER0bHNjYw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxQQ1BUeG9EdGdfdktIMXZwX2RXMEVPZ1YwMVB6MG8wRFZ3b1NObEJzT3dZNFI0aHVuQ3QxSGdZYmdlWHRXTDVLdjRnMWF6N0ZZTEF5T2h1TlY1LXdyeHdYdTdPOTVEQzBmNkFzczZib0t1bC1uWVltMUNGaHNMdmdnc3lhZ2N1NTF0Y3NUZEVyWXFqdS1DX0xzZ0FjVVZnVkRvU0F1a2JpZ1dkZw?oc=5</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2170,47 +2170,47 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K32" s="1" t="n">
-        <v>46087.12385416667</v>
+        <v>46087.52175925926</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>French appeals court lowers charges against police officer facing trial for killing of teenager - The Straits Times</t>
+          <t>Nearly 200 apartments get green light beside Canal in Kildare - Kildare Now</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>French appeals court lowers charges against police officer facing trial for killing of teenager - The Straits Times</t>
+          <t>Nearly 200 apartments get green light beside Canal in Kildare - Kildare Now</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 12:39:02 GMT</t>
+          <t>Fri, 06 Mar 2026 11:47:00 GMT</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxNWFlaQXR6UWFyUDVwVkdLaE42OENlcnNpb3lmZXhYeTdTQmtQUmRaMnVLcy1ETXVoQm1BVFBQTEdrQktpWnB4YnZRQkxYZHNGXzhtV3JjOHFtelVlcVZpck5HMXBIUm1pQVdzUEFqeEJtaHpKeElISDhyMFVhY005ZWFoN3ZWRnI0S3d6OVpmSHZnaHloZTBFbWt6RkhQaXZUOXlHN09mRHN3bDU2alFyd0o3MU81UHZIN0J4ZkFrSHZoSjhXbC1JZUR0RkZWbzd1WWw5QTczVHd6VmpJNUVqeVF3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQdTUwNVF3aUFxSFgweWNwU2pWR2J2YTFHZjVRT0x3b3pvcnVCUWYwVFZUS3BkT2Vpdi11WERSQm5yRkJONjNnYlVmbnNOVEE2UzJUM0lnaG5TRERCRkRSbzNOUVpfU3JMb1lqRUtVU0tkWlJ1X3ZTZTdLdEdoZ3o1OHVJbFVfMFh4c3ByZWZ1c09HU1lJNXdJd05lWVZCM3dTckFnYm1SUzBERlN5clRxRXFGcVJINy0x?oc=5</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2225,47 +2225,47 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K33" s="1" t="n">
-        <v>46086.52710648148</v>
+        <v>46087.49097222222</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Hristanov on the ITN action in the Ministry of Agriculture: A dirty and muddy war, whose main target is me - fakti.bg</t>
+          <t>LATEST: Meet the Kildare firefighter balancing 'dream job' and life as a young dad - Kildare Now</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Hristanov on the ITN action in the Ministry of Agriculture: A dirty and muddy war, whose main target is me - fakti.bg</t>
+          <t>LATEST: Meet the Kildare firefighter balancing 'dream job' and life as a young dad - Kildare Now</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 16:10:00 GMT</t>
+          <t>Fri, 06 Mar 2026 11:21:00 GMT</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxOb3NNdllQNmZUbjRpeElOdUczdm1WQTh1U0VpSFNETnF5OTVNQ3BHRHBVX2hodmtDR0djR2dfNllJeGMwN19GMVE5cDdkS3N5NEZIQUxhbjhSVjhYYVVBbDhrV0VoT0tUSVZQWHVvQWs5ekpVWVZObGQ1ODZ3ZFpKZVlDQ0JaamFra3R1aHl6eHBrSUEyZDBHcWpVZlozaVlkQmNqSURrUURxQUhTUzlFZ3ljdkhLYnYxSkU4ODYxd3hDYkxTRmRtSTFkMEE4dEhfVl8ydA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxOSEtpd3ZYUEJvdHc1YU9IOGxoRUZhS21XUkxXcGg3cVpfUnlqZ3RmdnZZYzE3M3hTNW9NYWI1MVFJZ3k1M0R2QV82RzlaQUtkOG82eTRoYWc1Q25fUUxzLVIwMWtZQUtHQ2kzN1ByOXY5WkZ1eEo0R2hwWTBWZWIzZzNhcm84TTNzVHNLN2VDaFRuRXhocGpienZEQkpIX3lQLWRXWWtKMnhNQXFJdHg4blZ5NFNFeXlwdHRhcXBzMHN1M1ZJdnNncU1WMzdUVDVW?oc=5</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2280,47 +2280,47 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K34" s="1" t="n">
-        <v>46086.67361111111</v>
+        <v>46087.47291666667</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Highlights of NATO chief's interview with Reuters - The Straits Times</t>
+          <t>Kildare-based art group expresses delight as extension granted to free exhibition - Kildare Now</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Highlights of NATO chief's interview with Reuters - The Straits Times</t>
+          <t>Kildare-based art group expresses delight as extension granted to free exhibition - Kildare Now</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 13:34:14 GMT</t>
+          <t>Fri, 06 Mar 2026 12:35:00 GMT</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPTS04RHVLWjdNWW10NTdRM0V2ZUtvYnllbUJYSW9laTRoNmdvbWpqSXBnaGpfOWR3RHBjWXo2TGdzZXpKalB5YmxOWGtJWjJ5TzJBM0NoWTJXSlBVc21hVGlGbjB2MERwRkJ6UGJ5SzRaUWZWT0ZmZ25aeGJTMEZNeENVTXMyN1l1cDVTWTFzMnlmRGRmdmZFQXQ2b00xcldxejN3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxPUGNhM2lnTlRKYzVpLVZ2U25mMnVFOTRudVJJZkFzSm9KMU9YWk5semg4U0FGT3VGd0NuTWU4dUxfNlFOOGFSS0QtWjNlS0x5Zk1GUWVCWFdoUjlYRkU2cEtQcmNSOHRsT1gyUGVCT2dkdEs2c2ZUSWZIR3pyNXJVamFXdm5TVkh2N00xVmpqWkF3OHl6LXNEOS03WThVZjMzLTUzT0JnRlNTREhzeXNFWFJHZWs3Y2RuV0FPeEs4TDhkakF6SUZIMTZaMGtVOFZRRjk0?oc=5</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2335,47 +2335,47 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K35" s="1" t="n">
-        <v>46086.56543981482</v>
+        <v>46087.52430555555</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>“La démocratie ne s’impose pas par les bombes”: manifestation à Bruxelles pour dénoncer la “guerre d’agression” contre l’Iran - 7sur7.be</t>
+          <t>'Transformative': Praise heaped on blueprint for this Kildare town's future - Kildare Now</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>“Democracy cannot be imposed by bombs”: demonstration in Brussels to denounce the “war of aggression” against Iran - 7sur7.be</t>
+          <t>'Transformative': Praise heaped on blueprint for this Kildare town's future - Kildare Now</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 21:02:00 GMT</t>
+          <t>Fri, 06 Mar 2026 14:05:00 GMT</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxQMFZCRXc2MnpLUDlGenZIb000SVd6eC1nSnZ4YVZwNkNrelN1TU1mRU9NZ3FDTUJwQTRXZmlLeUlOUGlVU3JNbzdFRHhLVDF0VjhvNDZhb2JpVWpPQVg1aklaWnQ3NEJQMWRoWndsZnJGMlBEN2NuU05CR3BIb1RPRXUtV2NPQmZjMHFvc0Z1YmlVNzhtRXdFV2dha3NrTVBNc21VOE5GMnF5Tm1HeS0zZlR0LUJ6eHdLTlhsMW1YWVhVTHlqTlc0bk5PS2ROX2xOODVhZGVmX3FJLWRiTGZtTngwcmh5Y0tBRE5Kakln?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxNYW9uRGIwbkZmVmxiaHc3WVdhbGhhajhheG5HYndpTDNFdE8zNXBiZlMxaTEyZ0w0bG5WWE9DNEMtX1VyNzI5WUpNQUNleENaWUZ3RF9hM3lIeTh6a19tWVg5NHE0dGowaGFkeHZha3pSWTJ4eTFxZ25BZGdXN25uNzFYQm9oZnZ3X3VyQ3ZSZl9FYWsyQ1VCUTdhSWNsMnk3SEVjdS11eVZDWXQwQ0xNbi1UYkhuaHN0QllPNy1VOG9hWWFxam1F?oc=5</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2385,52 +2385,52 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K36" s="1" t="n">
-        <v>46086.87638888889</v>
+        <v>46087.58680555555</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Face au retard et à l'explosion du budget, le projet de stade national de hockey à Uccle ne sera pas poursuivi - BX1</t>
+          <t>Kildare man advocates with Taoiseach for Down Syndrome supports - kildare-nationalist.ie</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Faced with the delay and the explosion of the budget, the national hockey stadium project in Uccle will not be continued - BX1</t>
+          <t>Kildare man advocates with Taoiseach for Down Syndrome supports - kildare-nationalist.ie</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 14:03:00 GMT</t>
+          <t>Fri, 06 Mar 2026 14:01:23 GMT</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxNLXkxaU1WSE5WbkJ1cVNYbGhFXy11VkpRUjdnaGJlZkhxdnk1YmpjT2JTOHVySkNnN243UkpZT19rSDRmQmdGd0ZkeUdaM2JWS050b3BUWlpjS3RkV0FLNEhjemM5SlZGdFZzNldMdmstVEVla0ZfZ3NQTVdUYUN4bGRHZFdPUTlIS3NCQ1ljUnZmeE85X2hHVGM0d2VJWTh1RWNpVTAxWnZuVGZSN0x3ZXVlZm9KZkZndUx0TW5Nd1B3RlhKS3RNaklPZy1GQS1wbDNmLWxGbw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQN0Y4a2VwWkJ0RWpuRklobVR5N09zc0czQlQzZmI4MmZ5N0tid1czWkd2QTR0V1RuUklsb2pLMDlPejJZZGpIUG5fUDV4VTJ2RXUyaElxNHZ1b2dlN0pyNU8zcWJKMERRMUdERlB4aTdkbGpHMmI4bHl4SHI3aUhCeVVYbWZUR3hrb0NTMjZEbExyYnp0WGhQRTRhdnVMRzlWaml4dE9ULTBGLXAwblZjZnY4RjhJSk5YajY4?oc=5</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2440,52 +2440,52 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K37" s="1" t="n">
-        <v>46086.58541666667</v>
+        <v>46087.58429398148</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City France English (fallback)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Paris" OR "Île-de-France")</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Jeux paralympiques 2026. « Je n’y serais pas allé » : Maxime Montaggioni réagit à la cérémonie d’ouverture sans athlète - Ouest-France</t>
+          <t>All the Stars On the Front Row at Paris Fashion Week - vogue.com</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2026 Paralympic Games. “I wouldn’t have gone”: Maxime Montaggioni reacts to the opening ceremony without an athlete - Ouest-France</t>
+          <t>All the Stars On the Front Row at Paris Fashion Week - vogue.com</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 05:34:02 GMT</t>
+          <t>Fri, 06 Mar 2026 14:10:26 GMT</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimwJBVV95cUxNcHFOLVZ3VElQa2s0UXRnTFRaeS1ERkl2dlpBcmwyVTE3SGo5M3h0Y2NzQWJyazFkaUdYR0FXSlFNVTR6RzlvR1B6ako4VzFHNUxFeFdRMzRpdEFtbkVEWHhwQkx3WVc0MGN1amtQTF9SV1JYb3FRNTRrVkwtVUw4THpTVFloWDVrZlVxYnNnVDNJZlVudVhVNGtTWWFTY29SSUt5OV9rWjhIRkVrYTlhSVRsS0RHN0lHNF9PQ1JNRW5SOHEtSkxsdzc0aDZCemM0NXdvdWo5Q2haYVp4a0dWZHMtUjVqQlZiTTMtdDFBVml1S3E4NFJic1pHcm9mMDZ6XzlRU19BQkhuX1MwS183R3dKUGZDQzd3SXhN?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxNY1FpMzZfYjVyc29DRGUxcGN2aHU0aHFOcXR1Yk1iNzBodnJCazJPdlhCcTU4cmdPYmVjSF8zdjhaYURvQVkxa0VXcEFuaUVITktTQVVWaFVwendiaHRORjJrVUdscEdJZTdNSzhFcXhIcDFncWtBMWhJWHlWTnRnblpsa25DcmpTY0E?oc=5</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2495,52 +2495,52 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>FR:en</t>
         </is>
       </c>
       <c r="K38" s="1" t="n">
-        <v>46087.23196759259</v>
+        <v>46087.5905787037</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City France English (fallback)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Paris" OR "Île-de-France")</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Futsal Benfica Auderghem - Anderlecht</t>
+          <t>She had a vision of herself living in Paris. Now this American woman calls it home - AOL.com</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Futsal Benfica Auderghem - Anderlecht</t>
+          <t>She had a vision of herself living in Paris. Now this American woman calls it home - AOL.com</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 14:09:11 GMT</t>
+          <t>Fri, 06 Mar 2026 10:29:53 GMT</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiUkFVX3lxTE5scURuclV0anR4NDRjYWFCWU9Ea0wtSG9JYTNEdTU5Z2NxdTlpQ2Zjcl9XOGRLZEFFcTVhVHZxTzdiUDVoeFpYaUZfWS1ZNFdKcFE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE9GS0tVWXg1d3NuV3VfQTM2eU5hM0JxbFZ4bHBaeng0TFY4UE9seTNYSUhBZzRxNE9HOVQyMjNiampLSFQ4STN2dXd3c0tSWkthb0FyV01RdDZLaEsxQjhsdUVuenMtSUFoaWdjbzdyTzJvbExUbG1pSkRNblhLQQ?oc=5</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2550,52 +2550,52 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>FR:en</t>
         </is>
       </c>
       <c r="K39" s="1" t="n">
-        <v>46086.58971064815</v>
+        <v>46087.43741898148</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City France English (fallback)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Paris" OR "Île-de-France")</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>"Panique et peur" : les prisonniers politiques iraniens sous le feu des bombes israélo-américaines - France 24</t>
+          <t>NBA YoungBoy Pops Out at Paris Fashion Week for Rick Owens FW26 Show - Complex</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>“Panic and fear”: Iranian political prisoners under fire from Israeli-American bombs - France 24</t>
+          <t>NBA YoungBoy Pops Out at Paris Fashion Week for Rick Owens FW26 Show - Complex</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 17:51:50 GMT</t>
+          <t>Fri, 06 Mar 2026 10:59:13 GMT</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxPQ0Jad1J6Z212Z1psd3ZsZmFRVG5VV3NpMjVDWjlVTy14U2NIRVgwa1NiTU9STTNzS0JiTW9YdG91d3JwLWtyNnRLMUJpVkdfYU5qZWNJMlQ2RXQ5M1pLQzNiNzZZNUdDNzEybW9vMEkxUmlZR29xblBHUm8zamE1WWdhM21UWTJ4VnZIdjZFRmhBcWJKNzhiNTY5bnRTVGUxOE1BQ0phYVN4MUVHZW16d2NuTEk2LXVhMlhkTFRvX1VRdzJQMWhfQTJXVXp4d1NRU0FuX3ByY2VBaUlJTll5S3VieHlYNXh4R2Vubg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOaFZiV0NKYk10emtXdnJlMzI5NXNjT3lvRDBBZnJMQV9yUmxwNFp4TlpYX3JwVEdaUC04dlBIMDVlMGRuOTJnRXEzdlBMYUh6anV4dTcySWxHUEg4bmIxbGg5RV9PZWJaVm10ai1NVmtWZUl6WGVpTkktYXZyWE0tcTN4c2xiN2NMRE1RNHM5TQ?oc=5</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2605,52 +2605,52 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>FR:en</t>
         </is>
       </c>
       <c r="K40" s="1" t="n">
-        <v>46086.7443287037</v>
+        <v>46087.45778935185</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City France English (fallback)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Paris" OR "Île-de-France")</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>À León, vivre l’Europe autrement : une mobilité EURECA-PRO au cœur de l’Espagne - Université de Lorraine</t>
+          <t>News | Roka targets large-scale operations in Paris and London - CoStar</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>In León, experience Europe differently: EURECA-PRO mobility in the heart of Spain - University of Lorraine</t>
+          <t>News | Roka targets large-scale operations in Paris and London - CoStar</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 07:04:28 GMT</t>
+          <t>Fri, 06 Mar 2026 10:50:23 GMT</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQdURSV1JodjJHTkx5VnRNNkhKZ3prQmUtbXVTcFgtUlVnSHM1VjFEUkVJanFWRjBhZ2dOTlE2bGdLTTRkY3QwYXlMY0dvNE83aDFHbWhuSWl5Qk5pUzFiZ3JkdlRsZ0RXVUJfVDFlWDdHVTB5NWZNN2pCVVFyUy1obDdKUTU5OWp5WGxVYUlFS3FQcEd2YnRha08wNGR2TUp6OHVhY1VVX1VhaEhFdERXM0JhN0VrU2RG?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxNcDMtLVhaZGIxa3pQVzBPVzhHRFU5dTAyMzE4UnJfR01VX0M4UkM4V19rMVNMLXQ0QVdKM181RGMxUF9sdjl3dGU5M2hwVllfTGJKUXBnMy1QdTFTcS1nQndMZXZtTU4xdDhDVG0wY19TSWZsai00X1VzcTY2bHlISDg5M2VIcElUYUdYckFn?oc=5</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2660,52 +2660,52 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>FR:en</t>
         </is>
       </c>
       <c r="K41" s="1" t="n">
-        <v>46087.29476851852</v>
+        <v>46087.45165509259</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City France English (fallback)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Paris" OR "Île-de-France")</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Pressemeldungen des Polizeipräsidiums Unterfranken vom 05.03.2026 - Polizei Bayern</t>
+          <t>5 Strange Discoveries Hidden Under the Streets of Paris - WorldAtlas</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Press releases from the Lower Franconia Police Headquarters from March 5th, 2026 - Bavaria Police</t>
+          <t>5 Strange Discoveries Hidden Under the Streets of Paris - WorldAtlas</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 19:39:06 GMT</t>
+          <t>Fri, 06 Mar 2026 10:30:00 GMT</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxNQ1NITk0yV3NhWm53dEx4eDBjQXU5N2NKckJfeFZEcXlybjYwbk01dFcwSW80eFctUzFadlNxYUhZRUNNaW5FNm9ITFF2bHRBX3owNnVaa1MtLXR3a21lUnh3Z21QRXdHUEM0WEV3VS1Qc1I5Z3h6eFlGdFEyUzdpa0hB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxPZVhmeC1BdllfS3Y4T291RVNabU5mSjlKaTl5MFg4LUt1STVSVFBkR01ldnBSNjdpSC1MNU8yRWNyTnNHdHNqOHN1eFlydThxSFE2VjJnZmJvYzZkSnBzXy1VUzBzalpoNDdqeGZIUmNpSHBVdXYtQTBrWDE1MVZuNXNHWllpMHNjNVh5dUh3bEY2dkhkaEl4cXdjQ09IQQ?oc=5</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2715,52 +2715,52 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>FR:en</t>
         </is>
       </c>
       <c r="K42" s="1" t="n">
-        <v>46086.81881944444</v>
+        <v>46087.4375</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City France English (fallback)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Paris" OR "Île-de-France")</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Einsatz von Polizei und Feuerwehr am Hauptbahnhof in Würzburg: Das steckt dahinter - Main-Post</t>
+          <t>Mbappé’s Paris trip raises hope – but the clock is ticking - Diario AS</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Deployment of the police and fire brigade at the main train station in Würzburg: That's what's behind it - Main-Post</t>
+          <t>Mbappé’s Paris trip raises hope – but the clock is ticking - Diario AS</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 14:30:00 GMT</t>
+          <t>Fri, 06 Mar 2026 09:57:13 GMT</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxNYkdBVUxTOWF6bzYwenRRN01oVXNFNE5DR0hXeVZzalpxOC1tdnM1dG1RT0JZRnFvdDV2QlY2bm84MzZTUWFvR0MzNHBPQ29sN0hZVWlqRjBfTHB0UnBEOTJYaFBieFlyQ3NKYTA5OTVNNzdvV2wzcUhYY1pKTWZWTjFPbHBUY1BucXJzZXo2ZUFYS2pZbmVjWWNVWkZEdTl3S3dRX0VsVkhTVkxpbmVKVkJhN3NGdFF6T2c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPbngtTVI5TUNLdjZsM3JVYUhaTy15cjZ2S3Zvc3J5cU85ZXRzbWRNM0w0OG4xQkpqNURTRllOYnRqeTZ3ZXQ4Z3RlVUNObEwzdDlSN1FNLWVBbkhfOGdxY0VzWFpTSWItSmZhUVBEZjlUdjI2eEtFdUVZRkVTMTV3M2lHYUdmblJyRmptYklNdnA3Yi1DYWfSAaoBQVVfeXFMTVJaY0dpNmdqUmE2amhhazNwRHlKcXliNlF6MDB2dXpqMkpQNVJ6UENpVzFQQ0t5cGVIcVgyLWlfSkZyZlJkQkFrV1VNenpRVnRYQjJxckRHYlZidERlWDNFM0M5V0dSVzdOTkUyV2d1Y2tjOTh2SWE3cExzTWpiMF92T2o5OEpYVGpvakw3T2VNaUZ0YW9QUzRXYURIM1JWVGU0VG1hTTUwWUE?oc=5</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2770,52 +2770,52 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>FR:en</t>
         </is>
       </c>
       <c r="K43" s="1" t="n">
-        <v>46086.60416666666</v>
+        <v>46087.41473379629</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City France English (fallback)</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Paris" OR "Île-de-France")</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Nach schwerer Attacke auf Mann in Waldaschaff: Polizei sucht nach mutmaßlicher Tatwaffe | Foto: Stephanie Renger - main-echo.de</t>
+          <t>Paris’ Tour Montparnasse Observatory to Close in March 2026 as Redevelopment Plans Move Forward - ArchDaily</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>After a serious attack on a man in Waldaschaff: Police search for suspected murder weapon | Photo: Stephanie Renger - main-echo.de</t>
+          <t>Paris’ Tour Montparnasse Observatory to Close in March 2026 as Redevelopment Plans Move Forward - ArchDaily</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 11:08:46 GMT</t>
+          <t>Fri, 06 Mar 2026 11:30:00 GMT</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxPaDJ2TlE2U0ZLVURRWjZfaEdCZTd0OE1pZGI4WUs2YXg3NVQyeDkxNjdIYTFRLUhacWxJZUhHdzF5alJDbGltNUdwSFpfLWNMb2NWSDBJMEFqUGZPd1lKcWNFVjFTSEFfSGZ5aUxIVWM1VWVMaHMyVGx5QjhPdVphRnUxTnQzSGJEM0djcVJFUlJhU2lwb3JVV0x3emxJZ0o1V2JRWWFpRmRGaVBGR3VDanRuYjc2a3FkZ09ISHJ2TVlSY0ZERGo0RVVnUURVQllrSlpwTl9QYVJfVEk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxOQkozVlM1c0RqM1JYZnNNZms5cUhpUmxUWUtwMjJQdklWc196ckVmcTY3XzJMM21lRWZGcTRqM1JqODQ4NHl2VjBHc3Rod2YzNHR5XzRGTlNVMnVlNHlUN1VrSFNzNFEtdG9PNEU4Nlc5ZHN3NzMtV2hCTDczN0xXM004NTh0cXE0d0RVbEFPMzRhVnc5dWpwQTV3Z3JqNEJ1X280dDZKVXZNTktJTzJ3S2NTOUVqSEZGZE96Q05PMHlVbDVkTWpB?oc=5</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2825,52 +2825,52 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>FR:en</t>
         </is>
       </c>
       <c r="K44" s="1" t="n">
-        <v>46086.4644212963</v>
+        <v>46087.47916666666</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City France English (fallback)</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Paris" OR "Île-de-France")</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Mellrichstadt: Polizei nimmt falsche Spendensammler fest - Radio Gong Würzburg</t>
+          <t>UAE Team Emirates-XRG all set for double-header of Paris-Nice and Tirreno-Adriatico - UAE Team Emirates</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Mellrichstadt: Police arrest fake fundraisers - Radio Gong Würzburg</t>
+          <t>UAE Team Emirates-XRG all set for double-header of Paris-Nice and Tirreno-Adriatico - UAE Team Emirates</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 17:00:00 GMT</t>
+          <t>Fri, 06 Mar 2026 12:03:38 GMT</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxQNVpjWXJISUZrLS1kaVU1UzVKV3Y3RVJhZ2wyOVRmOEwzaVB2QkhqMnRRVWpYNldnam1iUlRoel84YWpZZGRXdHktc3B1dmNqcHZncWNlY0hpRDJuRzAtbWlPNENJU1FDSmZ0anJPcEtZajIwVl90TU9JUXlVZnFESHgxaE03a1JzaEcwYTNzenVmRjQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPTXJBUmpqUlQ3VEJtbmhUajZrMWNFU3BIVVhIdmJPRERsb0NvdzN6YjdNVktGOXotRG5JcVVLTWdxb3p4RDF5SGNzc0VrNmstSlZ6a19XZXBieXNuUTFuc0tuakVDWUVjQU5lZEhNZmlrZmxfUjdIUVZaSmxDZy1Cb2pBSnBrb09pWDZSRklMTExYcWR4dzhOa3JtdElkMkw5dU1F?oc=5</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2880,52 +2880,52 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>FR:en</t>
         </is>
       </c>
       <c r="K45" s="1" t="n">
-        <v>46086.70833333334</v>
+        <v>46087.50252314815</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City France English (fallback)</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Paris" OR "Île-de-France")</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Blitzer in Blankenbach aktuell am Donnerstag: Hier nimmt die Polizei am 05.03.2026 Raser ins Visier - News.de</t>
+          <t>COSRX and Courrèges Reunite Backstage at Paris Fashion Week FW26, Introducing a Limited-Edition Collaboration Kit | Corporate - EQS News</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Speed ​​cameras in Blankenbach currently on Thursday: Here the police are targeting speeders on March 5th, 2026 - News.de</t>
+          <t>COSRX and Courrèges Reunite Backstage at Paris Fashion Week FW26, Introducing a Limited-Edition Collaboration Kit | Corporate - EQS News</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 13:15:39 GMT</t>
+          <t>Fri, 06 Mar 2026 10:06:21 GMT</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwJBVV95cUxNT3dZVW1WQzJkMWU4NV9lNTdWT3ZKdjhQWlJVSi1FSXZianZmYVpHUWZKMWx3LVVUSnFXSWlEUmJHREJLdVV4UVRoSUtSS3JfSUpLdGRwUHhsZ1J1bF9uVlQ4UEVYVE0zSTB1bzJJWnZYcm43T2p4LTdQekg1Vk9jaUJfVFItNGZYZkVycFZhT3h5UjBudkJYSmxMZDFYLThvVGFZLWtOOXFtVnRqOVVpVzNWTmlqSWhtQjBhamZXSUw2TUpmLXQ0eGRGaDQzYmtyRzhhQVlhaUpJVEZiRk5rQ2NKc0s4Y1ljWUw4TFVvMHhzMkhNT2QxNDZfYUtLTm4xZzFpT0xDSkI3bGQ5cXhTb0ZnSHdiUW_SAZwCQVVfeXFMTWgybGRuOHJFRHpxcWVON0NYZW9NSjdFY1phYV9mZm84NDFpcGF6Nk1tY3hNS0ZXb1JtNzNGOTdhMUpxeDRMQUR5akdOZUVKMU5FOTE4MWRJYXlWRXgxM0dKTDJabVBpdGk3aF9DVkJDZmRtV2dELUZSbWtaOGRCNDVLZWxmS284T3RGcGoyR2c1U0ZpZnNoMEduUmZLOHRweFFFTWJ1ZE9wQjh1NVVZTXM4dGRNTjIxaFFMTkQ0N2UwTk5Pd0RkWUJkMVVZV2N1T0hQQmRqZ0VzOHBkajU5d0hvYnczSkFMRjRmcTlPUUVEVFhHb1Jwb2dpUVhnS1c0cjREX3ZQdktKMVNDdlJ2NlJ1LUgtMDJGNEVkOFQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowJBVV95cUxPZU8yblQ0TVRHMm5NQ1ZDbThDMk9YZzZhRTh2VmtFWktKbkt2cTd4V1BZLXdqdmhoTk9qWU9ZN2V2amdVdVloUTJDTzNQcFh2NFVFN19Hb00zaTc0SVV1RjBBT3B2U1JyWVRSMXI1ZkVjN1kzVDkyRkF0dHptZ21YUDVRLWRfRXg2UGFhYU9mVmZ3STE1MHRvUGM2ekdSUzVyVFNUYjRuTWx6SW96UG92N0F0TGNmOWwwMFktbXkyMlB5bTA3M3NMbVQ4N2pteElLOUswY284bjJxbVVXSUNCeG9qYW02T0pIel9CUFRVOWVaUjE2QnlkS3h2UzRnRnVjbWhRM2ktSnRPbV9BbnZnbXhMTVVaalZ3bHNfTjNhU002NkU?oc=5</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2935,52 +2935,52 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>FR:en</t>
         </is>
       </c>
       <c r="K46" s="1" t="n">
-        <v>46086.55253472222</v>
+        <v>46087.42107638889</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Village Wertheim (fallback)</t>
+          <t>High Level City France English (fallback)</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Paris" OR "Île-de-France")</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Opinion | Of Course Trump Bombed Iran - The New York Times</t>
+          <t>Paris Jackson embraces boho-chic in sheer dress - HELLO! Magazine</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Opinion | Of Course Trump Bombed Iran - The New York Times</t>
+          <t>Paris Jackson embraces boho-chic in sheer dress - HELLO! Magazine</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 10:03:00 GMT</t>
+          <t>Fri, 06 Mar 2026 12:36:46 GMT</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxNbmhEOW1POGNRa3YxZXAwb2Y1dzVzNW1NWW5VUWp6MGxPdEZMS1l5RGo5c1JISHNNYlFaY1kyS1p3VjFKam5hRWpMV1NuU1hVcm4wTTNLTlhhRG8tcy04cko2TnlHc1FIbzJ5WTl1ZHVCTkRvbTBKNVhHczhpX3pHWEcwQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxNVjJrbndndTJfcHpEdHNqOUdvVWRuWl9kWXM5SU1YdmQ0eXlxQm04Q1dVOGplV0RtUW1lVlJmekFkcEZGOHFkUTlXbWhMdFJMM0tEa25aUll3Y0xSVktINks2bmprc0hyZkdzYnB5OVdQWlQ3WF8zRzA5S3FIWVUtcXFJT0wyX01NZlRpNjBiSEJUUQ?oc=5</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2995,47 +2995,47 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>FR:en</t>
         </is>
       </c>
       <c r="K47" s="1" t="n">
-        <v>46086.41875</v>
+        <v>46087.52553240741</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Village Wertheim (fallback)</t>
+          <t>High Level City France English (fallback)</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Paris" OR "Île-de-France")</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>FIU Medicine Earns Full LCME Accreditation Through 2033 - FIU Herbert Wertheim College of Medicine</t>
+          <t>I Went Shopping at the Paris Flea Markets with Top Designers. Here’s What They Taught Me - AOL.com</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>FIU Medicine Earns Full LCME Accreditation Through 2033 - FIU Herbert Wertheim College of Medicine</t>
+          <t>I Went Shopping at the Paris Flea Markets with Top Designers. Here’s What They Taught Me - AOL.com</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 15:27:30 GMT</t>
+          <t>Fri, 06 Mar 2026 13:22:24 GMT</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxPaV9PT2tESnE4NVdQZTdxVkt4RTg5T2dmUHQ3cDBsUnRTSWZfSWxsUDZrYkFWcUt1RVpsak9hTVYyaldJMjljQm8tQ2JKM1RCS096ZDVKN0d6MkNjRm9penNFRDZ6Q3VoZEdBRlZxYzN0SUs1YWlMMUR5R2J4N1RYNFNXMUVoRVJyZGtIdzdSRGROMmpfalRvNUdtUm1UZnJNTVE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQU3RZT3NGYkgxNVROaFdPU1Zsa2J4WGxJUU9sUjR5RHBSTHI1YWJzWnllWWFaQ0ZTWnJNVmFRMFVSMUtNOEh5LTRTRjBSNlFCeFF1WUZMc2U4Y05GYWtMTlZPX19xYk5mUndmalRtWkU3Q2NTOVlpUEcycURJcDd4YWJn?oc=5</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3050,47 +3050,47 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>FR:en</t>
         </is>
       </c>
       <c r="K48" s="1" t="n">
-        <v>46086.64409722222</v>
+        <v>46087.55722222223</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Village Wertheim (fallback)</t>
+          <t>High Level City France English (fallback)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Paris" OR "Île-de-France")</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Government lists Hizb ut-Tahrir as banned hate group - The Australian Jewish News</t>
+          <t>The Best Backstage Photos From the Fall 2026 Shows in Paris - vogue.com</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Government lists Hizb ut-Tahrir as banned hate group - The Australian Jewish News</t>
+          <t>The Best Backstage Photos From the Fall 2026 Shows in Paris - vogue.com</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 22:36:59 GMT</t>
+          <t>Fri, 06 Mar 2026 09:46:04 GMT</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPNWpUdWdpZEJfdEZFZW1xYXBYRjJHMEJId3lkU1E0cnZjVTFOOHlrbnRlcDNfdWFXLU9zZVZXVnpnaWJKUzM5eFFBMUtOdWdUVWM1TGdfZ3ZOdGtYdWZ5a3FtSU52cXgySEFNWXVESzVRcXJZYWFwYkxvejZXYVpLRlhWWWxuLV9mZVdyN1NabVQzMFJsVkRRWHBR0gGfAUFVX3lxTE9NMlVoTWxBbWRINW9WMlVnU0xLcHQzMy10eUlha3FoZWFxQXZ5dVFJR0o0c1VEU3I0Z2pwUGtoV05LVGxmOVYzVnd5MnJlV3VUWkVDRjc3elUtYkp1ZUVhLUhRbU1ka0FPUGsxTFVRTjh0eDVBQXR1ZEF0M0Z4U0hCbmhXeWsyNF9uV1pucGk4UVJSSXYzSXo2Z1NDT1lZNA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPTTlqZjVILWlLa0I1aDJyTGNhNEtXV2VRM2NDczFIalFVcG1zY3JDZ0lJa3V2SGtiN3o1UmtSbG5RYXhJT3VoWTlubnlCbmV3UzdZbW5kY0RBcm1wd2dVemFZS1VWd3FNOWpZZ01TTndpTlF2cWtJV25sSHVNanQ1cFgzcGpRX0tGTHVfNnNDck14RHgwUUE?oc=5</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -3105,47 +3105,47 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>FR:en</t>
         </is>
       </c>
       <c r="K49" s="1" t="n">
-        <v>46086.94234953704</v>
+        <v>46087.40699074074</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>High Level City France English (fallback)</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Paris" OR "Île-de-France")</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>1,6 Promille: Polizei stoppt Autofahrer auf Münchner Straße - Augsburger Allgemeine</t>
+          <t>Sofia Vergara Embraces Bold Strapless Corset Look While in Paris - Reality Tea</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>1.6 per mille: Police stop drivers on Münchner Straße - Augsburger Allgemeine</t>
+          <t>Sofia Vergara Embraces Bold Strapless Corset Look While in Paris - Reality Tea</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 07:09:38 GMT</t>
+          <t>Fri, 06 Mar 2026 14:04:00 GMT</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOS2VjakpKWkFXaW84T043bWJBSHFSNDlZX3BTTUYtU2Vfb3JUQnZlTVFFeDRHRFNJcEJhVGw3OFphaUg5eWNLTUtmUlZ2M0xBQWVwQ3ZtNXVTSDU5djVpWWo3QTFTVWpIenE5MGtmS0NndWFRejVLQTJLTEZKWlY3QVVjUFdiaFEybHFhZ3N5NWZ3S0JBQjJGejVqeVgxdHMwUFZiZWtSTjBtYi1iLVVSQzJEemdxUTh5MlVETDctTUZtV0RDTUo1RmJGaw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNckNrLTRsckFPLWJzcmYtZEdkdnFXQkJuME1XODV4NEd4SUtCa09CQzAyT3JVeUEwdkNqZHJzR2lfaWkzejNIWWxlOXRobklOdXdTOGpLdWx3UzJMcVRmREJYUDE4VnlkX2NLWVhZUWg3dzhqMVdZQ1ZfMmtEV3lXZWZZSzluVEQ3VEgtc1hrS01uLXl0QVVzdE1UbEg2T1XSAaQBQVVfeXFMUHN3UnA2clZTQVFGTEZ3S2NwVVJucWtWYWdiRmlsTlJjNHlLR1NFcExCbGxEWnNuOVNybzUyQnhIblpSUndGRjBzREpJT0JuckFvN2NRQVdQOVk2ekNUWk8yYWV3dGF6VUVnaVdpaWQtdTdxSHc3anFxOGl4dGM3U2ZpQjZwanVtMVRicTIyU3o1NkFnZTRXaDBKTnliMGkzcmM2Q2w?oc=5</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3155,52 +3155,52 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>FR:en</t>
         </is>
       </c>
       <c r="K50" s="1" t="n">
-        <v>46087.29835648148</v>
+        <v>46087.58611111111</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>High Level City France English (fallback)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Paris" OR "Île-de-France")</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Schüler gegen Wehrpflicht: Auch in Ingolstadt wollen Schüler heute demonstriereren - HITRADIO RT1</t>
+          <t>Paris Jackson’s Tattoos Show Through Unbuttoned Shirt at Mugler Show - Reality Tea</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Students against conscription: Students also want to demonstrate in Ingolstadt today - HITRADIO RT1</t>
+          <t>Paris Jackson’s Tattoos Show Through Unbuttoned Shirt at Mugler Show - Reality Tea</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 09:34:00 GMT</t>
+          <t>Fri, 06 Mar 2026 12:35:40 GMT</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOT0dXeC0yU2RmcTNoWDM2dWJzZ0doZHN3OTNFSXNPWlF6YW84VGVWX1Vob2ptVXdVcGVLQ29GaUJjOWdaQllpYU1IYU9Ia3hiNWVGYjA4RUR2SGx2NUh3Nll6Z01JVlI2MTg3U0dXS1hZSEZxbHJnYXdyZ2dRX0duamF0RTQyaWU1SDY5WGcxT2FseFQ4TzlaRkdvaUttN3pCR0ppeGRid21PSUxMcjY5ek5Qb3psUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxPa2ZZVXVDcWpmOHlGNV9oaG1WVlEzQm1ZRVRuUjFoSFhITlluX3lsaGs1UXNWRWtaQUxwSVQtanFYV2wtOXZiSW83MlVqeUNVYU1KQjB0b0hEOE9wbmhHeURWTzNkc0c0MWxlMWlQOVBnZlZ3Y01ybUtCMjcwclI2ZHR2WjRBTXdsMlVyWDlpUdIBlAFBVV95cUxNVTNVZTZ5Nkh3M1hxLXg4TjRqMVFmX2liM245Z3d1NXBrei1haWxwUzNuckJseFdIZExDVTR6S1BTR3NucFlGdUtvd0I3aWI5ZEVuVVFpMkFySzJWWHUzWjhNS0h3Y2tMNjVQVlF3SFdUNE1FbG96U1ZieGlWSEJrM3VSYlJCQ0hiQWc1dTBWSm9YZ2JH?oc=5</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3210,52 +3210,52 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>FR:en</t>
         </is>
       </c>
       <c r="K51" s="1" t="n">
-        <v>46086.39861111111</v>
+        <v>46087.52476851852</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>High Level City France English (fallback)</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Paris" OR "Île-de-France")</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Ingolstadt: Unbekannte brechen in Golf-Club ein und flüchten mit Golf-Mobil - Pfaffenhofen Today</t>
+          <t>Paris-Nice 2026 | Vingegaard and Ayuso’s Tour ambitions go on the scales for the first time - IDLprocycling.com</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Ingolstadt: Unknown people break into the golf club and escape in a golf cart - Pfaffenhofen Today</t>
+          <t>Paris-Nice 2026 | Vingegaard and Ayuso’s Tour ambitions go on the scales for the first time - IDLprocycling.com</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 11:52:22 GMT</t>
+          <t>Fri, 06 Mar 2026 13:22:58 GMT</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTFBudV94ay1OLWFZclZ4QkUxX1IwczJvN1NQQ0wxWDd4N3lIS2o4akd0cHRWVm5uZ19zeEhsTWhyT0tpOFQzeHNxNlRzWE5tbjVicHhjTml1N1NnMm1wbG9kM3pLR19hTWlSb2VZaHJR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxPOVNRc1V4N1JYeGtnOS1lN0ZXNm9SZW1XMnRKWEhneXE4MzBqX3cyZzY4SzhrQ3d6NTBXdjNmdHgtTXZLaDBxY0s0aWhpLWM2MmpELURRdFBSNEN0U3Z0ZnVUZklZOXZKSlNfaUlvQWdVU1N0eFNNMU83UmtsS2lHOHlkcUZwMldCZzU3S1VacHNHZjBPZ2NzQU0wbUFFbC1YcDdTMGZzbWVXaEJIdG5VYXhMbkpVaEZ1YVNlX0ZLWWEzU3BW?oc=5</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -3265,52 +3265,52 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>FR:en</t>
         </is>
       </c>
       <c r="K52" s="1" t="n">
-        <v>46086.49469907407</v>
+        <v>46087.55761574074</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>High Level City France English (fallback)</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Paris" OR "Île-de-France")</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>30-Jähriger aus Manching verletzt sich bei Moped-Unglück in Ingolstadt - Pfaffenhofen Today</t>
+          <t>Rick Owens Injects Love and Light Into FW26 - Hypebae</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>30-year-old from Manching is injured in a moped accident in Ingolstadt - Pfaffenhofen Today</t>
+          <t>Rick Owens Injects Love and Light Into FW26 - Hypebae</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 13:25:11 GMT</t>
+          <t>Fri, 06 Mar 2026 13:26:12 GMT</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFBSa1pzbUFsOWxJUk1UdXVwZjF2VkVlOGtMS0JMMjJGcUw4SVhSd2NzS25KYkU2NnNoRmFmeHJYcGN6UHFILVBmVm4tOFJoeHFDWkV1LXNiczJKZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxObU9NY3RNN0xEbDM4ZkNtOXJUOVl3elNJMTU5eDBSMFFaeWY5Q0NrRTdoSk5PWnJqbnJBZDRNMHc3MUU0LW10amVPRm4ybXBBczYtdjNqYkEyNC1MVzBQWTJ3dFZiajlFRXBMbWx0SzhUVkdjWGxpd1ZvZDh4NFVZYw?oc=5</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3320,52 +3320,52 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>FR:en</t>
         </is>
       </c>
       <c r="K53" s="1" t="n">
-        <v>46086.55915509259</v>
+        <v>46087.55986111111</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>High Level City France English (fallback)</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Paris" OR "Île-de-France")</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Fußgänger stößt mit einem Bus zusammen: Fahrtgast verletzt sich - Augsburger Allgemeine</t>
+          <t>Comexposium puts Serres in charge of Paris tradeshows Siec and NRF Retail’s Big Show Europe - FashionNetwork - The World's Fashion Business News</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Pedestrian collides with a bus: passenger is injured - Augsburger Allgemeine</t>
+          <t>Comexposium puts Serres in charge of Paris tradeshows Siec and NRF Retail’s Big Show Europe - FashionNetwork - The World's Fashion Business News</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 13:57:30 GMT</t>
+          <t>Fri, 06 Mar 2026 14:23:44 GMT</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxQX3VTMjFDSE5HLURMWEpVNGpfdkJvMTJZVkpib1dLdGQ3b2g3cnhCcmZyeGNZN0JlUXNNZXdpMDg4RUlwbWhtalVyb0JEM0g5My05QUJxRl9OUnZ4eXdLOXI4aUtJNGRvUUxfTktOOU1VNVROX1FWdzZaOWliVUtzejNMTDBBNHVVOXE3ZUt4bVFMdDRsdEVZY1ZMX3V4c3luSEM2bWl3STNFU29LcWNyOEpXYW1lZ3Y4dHNhUFc1bmlvYTB5bTFIb2k2RDdwdWdTaVpWcFd3SFRHcmtOZkN2RG0zci0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxPTHd5VTlWc05ZWk9DaDFWV1c5OGkxSkRpYmxqNUxXbEhKVmJTRlloLWcxY3JVVldDWnlBYmF0eVNkeE44eFktdEs2OUZsZWNYRUJHb0ZMWHRFTGZ1dWdqWmRiNkJhZlRhenR6OWhHTXN6emRlaEdhRkpMUUdoZXpGR005cDY4MlNiQ203NUNRMXF6UzJ3bUFnVEI4aHZ6MDByYTFTZHRxV1QyT2NBNnM4ZEJpb1ZwaTAzTndaWW1kU25vaWtJQmFTamVOOFJIMDBHVkVBZ1Nn?oc=5</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -3375,52 +3375,52 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>FR:en</t>
         </is>
       </c>
       <c r="K54" s="1" t="n">
-        <v>46086.58159722222</v>
+        <v>46087.59981481481</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Village Ingolstadt (fallback)</t>
+          <t>High Level City France English (fallback)</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Paris" OR "Île-de-France")</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Here are the best-selling new luxury cars ᐉ News from Fakti.bg - Auto - fakti.bg</t>
+          <t>Viktor &amp; Rolf Fall 2026 Ready-to-Wear Collection [PHOTO] - wwd.com</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Here are the best-selling new luxury cars ᐉ News from Fakti.bg - Auto - fakti.bg</t>
+          <t>Viktor &amp; Rolf Fall 2026 Ready-to-Wear Collection [PHOTO] - wwd.com</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 07:27:00 GMT</t>
+          <t>Fri, 06 Mar 2026 09:09:17 GMT</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE9XeUtoeU1qYk9ZanR4MEJhUXhwUEpTUVliNVlJSFdtNml0WFdqdmJRRlBfajJyYXdoT3RkUUJfWWFtb3hXSXNadGpWcVVqTDZ1MGdtOWJXZHBPRm9HVXQ4eUhMRkpMSlk3cHJMZm1MX01IVm1aNlM1dTVSTDBEZXc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNeWYxYWlKUU5BT01jeTRDVVBvenExYlpqMkotTFA1VU9qWlJ0VFkyNVFiZG93cnQ4VGdseXd6MnNEb09UamZBLU5Ba3NrSGlsbW5DSTU3M2dZMmp5am8zUFF2eEIxMEdzNjZoMEhUZWgtTDJtVEhEODNzcDlLR1BiZU9ncU1fYk5rN1NRR1dZUTNoUEFkaXpJc3dsSFZmUU05TTJWbXBoLWlNWS1ONWc?oc=5</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -3435,47 +3435,47 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>FR:en</t>
         </is>
       </c>
       <c r="K55" s="1" t="n">
-        <v>46087.31041666667</v>
+        <v>46087.38144675926</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare</t>
+          <t>High Level City France English (fallback)</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester outlet" OR "Kildare outlet")</t>
+          <t>("Paris" OR "Île-de-France")</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Sugar Plum Sweetery Win Westmeath Enterprise Award - Midlands 103</t>
+          <t>Chappell Roan’s Dramatic Hair Makeover Continues in Paris - AOL.com</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Sugar Plum Sweetery Win Westmeath Enterprise Award - Midlands 103</t>
+          <t>Chappell Roan’s Dramatic Hair Makeover Continues in Paris - AOL.com</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 10:19:43 GMT</t>
+          <t>Fri, 06 Mar 2026 12:23:37 GMT</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQS1dwX0x2SDQ2ejY1OFVvTGJzNGpfUTdjdThEZDhGQXBsWHJTeWwwMzgwUDlaLVFUZERvSVlrandHUC02WFlrZC1lZE1nYkFTV2k2eVJaR0xfSVdPZ1ZPeFlud1hfb3BtQ3lyUzZuX0p2NkdYeDFpS25wNEpaRnhaV3NYcmJxMVBiajJFSS1XQnpQNDE0d2VEUkhWbmpKcERjbnZWeVBxOUxSUVdKSXpWNXByOGZBak94T1IwMQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxQZTd5MkZ4TXFNdjlkOGEteW1OZFVvXzI2QU55MTZidkFhYjdYUDZmeGQ5eURnbGtGX0RiN29lUV8zT3QxVjJEaVFvamEwUU8tMFZDQU9vd195RC1MaVRkSUVoeGJYZUdFWTNHRURsQTVyUUdtaUZ5X2xCa3Fudk9NR05COHFKLU0?oc=5</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -3490,16 +3490,16 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>FR:en</t>
         </is>
       </c>
       <c r="K56" s="1" t="n">
-        <v>46086.43035879629</v>
+        <v>46087.51640046296</v>
       </c>
     </row>
     <row r="57">
@@ -3515,22 +3515,22 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Milano, brutale accoltellamento per una battuta: arrestati quattro minorenni per tentato omicidio - Affaritaliani.it</t>
+          <t>Allarme bomba al tribunale di Milano, evacuazione di alcune parti dell’edificio. Udienze interrotte - Il Fatto Quotidiano</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Milan, brutal stabbing over a joke: four minors arrested for attempted murder - Affaritaliani.it</t>
+          <t>Bomb alert at the Milan courthouse, evacuation of some parts of the building. Hearings interrupted - Il Fatto Quotidiano</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 12:05:39 GMT</t>
+          <t>Fri, 06 Mar 2026 09:03:46 GMT</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxPc3Q5NXBQa0xPYXUxMnpyQzFYRVNrTEZUTm1MTVQ3NUNkaTFnVi1HVjQ0Qy1xQWdQaXNYMDZfRW52M0swVTJodnB3ZHhmOWVQUFBPT0JUTnJKX3Y5Vklkc0o0MjhfZUV5MVRnNTRHNFdQSC1DbnQxeENJd1ZtOExZcW55eHlHYTVsbXBJb0ltZnBFQ0FyZjZaNm5oYUJMMnBlT0hQbllQMHlUYVB3dnFDSTBlZEVoRnRnWFpZei1qX084cmEwbFFvVVpvZmRxUDdQelE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxPY0lRRjFENHdzWGpoYkh3UTBmS01pRldYZG5Yd0xUS3otYWZ4bF9GcktlWDd3aVp5ZGI0bXJSVElhMmhDeEk5T2JMVy05MXUwZkJVbGVUMFNlYVR5aVd3V21kc3RSa2FVUHFBeVphSGdUNS1sejNhUHVoUUM2V3JMbWk3YUttTkVvdzlRMHEzcFFpUlFiUzNXdFpEVGVQUU9rcXpON1VR?oc=5</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -3554,38 +3554,38 @@
         </is>
       </c>
       <c r="K57" s="1" t="n">
-        <v>46086.50392361111</v>
+        <v>46087.37761574074</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>High Level City Italy Italian</t>
+          <t>Local Town Fidenza Italian</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+          <t>("Fidenza" OR "Parma" OR "Piacenza" OR "Cremona") AND (protesta OR "minaccia bomba" OR esplosione OR sparatoria OR accoltellamento OR evacuazione OR "operazione di polizia" OR arresto) AND -calcio AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Lagarde contestata a Bologna: lancio di uova contro i fantocci e tensioni con la polizia | VIDEO - BolognaToday</t>
+          <t>Nas Parma. Primario arrestato per peculato: avrebbe incassato in contanti prestazioni intramoenia senza registrarle - Quotidiano Sanità</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Lagarde contested in Bologna: throwing eggs at the puppets and tensions with the police | VIDEO - BolognaToday</t>
+          <t>Nas Parma. Head doctor arrested for embezzlement: he allegedly collected intramoenia benefits in cash without registering them - Quotidiano Sanità</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 19:35:08 GMT</t>
+          <t>Fri, 06 Mar 2026 11:45:59 GMT</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxQWEZZN0poc2JXa0ZpR2FmdWtlcjhLQjNIWG5maUZDbnMycEYteHJsU0RuVTZsZjl3MF9jRUxlR25lX3VXelVtdlFqNmJLLTRzQ29DMWprVGpGNTdTcWVrUFRzcjZyZlFsMC1lOWlKdzd6VjltWEpzQ0tMaHVzMDBnT1hFbWxSdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxOY0dRUnd5aXhXYWVaOE02eUthYnNHRmIyWHByaEVwVjlLN2cyVWdoMHNkcHhzTlQ0eHBQOHpUbjQxemFGUVR3bldXWDhBZDFCM3RFcUx2WENBbHBSY2EwNEo5cW82ZGlaamVaOU92UE5qNGV6Wlo3QU1YTERXVEdjMENIOHQ4ZlNyZkI0cnRMa2NndXBWY2t0bVRWcFZxSERKNHRoZHZTUXd0ZzZXaExnWU9ULWE1N01ydUk5LU9QM0tCYURtTE0zSEtTdTFvX3JiVVByRTlEU3M5SVJHNzBWNjJxYmdUc3BubjA0?oc=5</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -3609,1052 +3609,7 @@
         </is>
       </c>
       <c r="K58" s="1" t="n">
-        <v>46086.81606481481</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Manifestazione contro Lagarde, un centinaio in corteo - RaiNews</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>Demonstration against Lagarde, around a hundred in procession - RaiNews</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>Thu, 05 Mar 2026 16:26:00 GMT</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxQS3NiTEpkdkJTbUxBSkxjNVM3LVR1dDdrWlk0Mm45ZWFuMUkwUGMycDV2V2N0N3BlVVYwZzZVdnB0YmtnSHVpZzVWY0NaOW1nOVRJRk95ZGRZcGlpazJSOWEtR253dV9IdEdsdVExOVBKLW1JWjZnRXNGakozTVRsc3J4TkwxRzhUSE9ZQzZYQUEtQnBzZlhOeURmY2dqYjZzMk84OVJZRjVaREVUMnhNR21KaUZ6elh0dW0zM1pVWk1peHhNNGViYTROTFVGVTJ5ZDJIRjhQSTVpN3dERkxYdm44eUc5Vlc30gHuAUFVX3lxTFA3eHpsXzhzaTdlQTcwNi1NVjB5aXl6VFVTQXlTWXlTLU1JWTEyZDNndjdqeDI2WjRBaFhPcHFaMzRRSXN4UHBfRWpLYV91X3pqN1lfclBhSkU2S2JIekdVNEVqalNmNml3UUVWdkN0XzJFSktObXBaS3gyMmlUZUFTRTdwQW02ZlQ5Y3Q3NEt0al9ZdTV1Umkzc2xhd21QZHFNVkRWVVA3WDVFOFVoY1N2a09BTVZnSVJyc19LeXdEd21wREFEOGtQQWptdkZHQW8weVRxRExnZjhicm1aRUE1N2h2V01haC1oVjA1X3c?oc=5</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K59" s="1" t="n">
-        <v>46086.68472222222</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>La protesta contro Christine Lagarde alla Johns Hopkins a Bologna, foto imbrattate di sangue e fantocci: contestate anche Meloni e Schlein - Il Resto del Carlino</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>The protest against Christine Lagarde at Johns Hopkins in Bologna, photos smeared with blood and puppets: Meloni and Schlein also protested - Il Resto del Carlino</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>Thu, 05 Mar 2026 20:03:11 GMT</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOb0xhNC1rT0cwTEY2anRVZ29LVkRqYUROS1ItWFJZWnd6WktZNTRQY3RYYkcwTEo4dVUtRTJIUWtXbVVPT1lYRjhfdk43MGlZWGl3QzhubXlNUFFGNWpTQWhzc0RZbFJnQ2VETHZQUTZWQzA4VF9LWkNIQTdSeDZNZDEzdkRleW9nandhWERVUUlReHo3SnpHSGU3WW1vZw?oc=5</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K60" s="1" t="n">
-        <v>46086.83554398148</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Sciopero generale, aerei e ATM: marzo di passione a Milano - Milano Weekend</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>General strike, planes and ATM: march of passion in Milan - Milan Weekend</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>Thu, 05 Mar 2026 18:37:46 GMT</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFB6cHBiM2lyVlRvcDBibW1wZzE4NnV4SXJad0NVbW82dDJCUkt3aml4LUx3OWtWc09DNl9PbmZUbDhjRGZpeWxQdEliOERkSU1fT0JnUFFXVGs4czI4T0Z3Vlh0ZnJnb2FXejU5eUpzUmR4QkhUQWc?oc=5</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K61" s="1" t="n">
-        <v>46086.77622685185</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Bologna, manifestazione contro presidente BCE Lagarde a Bologna - Local Team</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>Bologna, demonstration against ECB president Lagarde in Bologna - Local Team</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>Thu, 05 Mar 2026 19:02:46 GMT</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOcS16d3UtZjJBd0xCU0oxUENYQXZEMXBBWHVqRDg1ZEZsaFBDWlZPdzdCZGcyT25pUmd6UmltNkhmOWhHZUVxQWQzcmJrYjB6SmU2N3JKRWxvRy1TbllVMXN5R0hlTVBiWjlOd19ld282R04zTkVpMkFCZ2t4b2RWd2RVckhhdzQwaDBZZU5uNnFDeHZGcVlRZmI0T2ZjRXl1WUFLcnNuVnZkM1E?oc=5</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K62" s="1" t="n">
-        <v>46086.79358796297</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Milano. Giù le mani dal Medio Oriente, corteo - Contropiano</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>Milan. Hands off the Middle East, march - Counterpiano</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>Fri, 06 Mar 2026 05:35:45 GMT</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE9iQWdVLUdzdUtOSi02Vkd1SXRLV1Z6RjYteFROY1NLeHVwcmsyY0ZlaUJrZl9jU2tMakhrMkhyV0dtam1CdmtYdlRMdE9DcDI2VDBrOGg2ejhac1Ywek9SRFhGdTBwN1hFd3BvY1dKTHp2UjZMMHNpMzU4R3ZjdTQ?oc=5</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K63" s="1" t="n">
-        <v>46087.23315972222</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Il presidio degli studenti davanti alla Prefettura di Milano - Il Giorno</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>The student demonstration in front of the Prefecture of Milan - Il Giorno</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>Thu, 05 Mar 2026 17:30:39 GMT</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxQZDNOUlJVSGtBeklfME5NUHM4bGVyamNmLXVYLTROalIwZ0ltSU15SkxoRGNGVTg5QmZGVnAteEFqaFFyNEVQUVEydUNlNkdmcGZGdmdSczJQV1h0TEZrZzh0eklQUEZVYVFYYXI5eEZkUm5Vb182RXVub3NUMnkySzVITml4dk1wdHFpMjgxLVpGWUZ5SWN6WW1WejNOcmxy?oc=5</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K64" s="1" t="n">
-        <v>46086.72961805556</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Lagarde a Bologna, la contestazione contro la guerra e la presidente della Bce - Radio Città Fujiko</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>Lagarde in Bologna, the anti-war protest and the president of the ECB - Radio Città Fujiko</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>Thu, 05 Mar 2026 10:40:36 GMT</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOSGV6dU5VcXRBQXJleXZ4SWNGNHA3eFVhOXNVMDItMkw0WU5zc3NHa1FlTmhFcTFqbHc5SjBudU01cXhvS3NVNE9NZktCZUVUWElPZjFmZmlzZmV4S0F0LUMxWDUyLWEtMHRycFAwVXJhLXJSSFdycS1KeFRSeUczT0xtMFA3cTFjbUtHZWdFN2p2S0ZkQUtCWVRFRUJveFJOazM0UmdHNHplWHd0a1I0?oc=5</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K65" s="1" t="n">
-        <v>46086.44486111111</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>8 marzo 2026 a Milano: manifestazioni ed iniziative in città - Secret Milano</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>8 March 2026 in Milan: events and initiatives in the city - Secret Milano</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>Thu, 05 Mar 2026 11:35:18 GMT</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE0zNG9wSnU3bzNFOFdoSXB3dU02ZGxVQVdkSm55d3lveGNYUnZBcHZhSTZfanBzbkRuN196ZnNHMHFNNU4zMEdvd3hrY2ItVklrZkNqSFBOWGZfN19vemx5WUN0UDgyeWdwaE5IcFlScGI?oc=5</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K66" s="1" t="n">
-        <v>46086.48284722222</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>Sciopero generale e corteo: stop a scuole, sanità e uffici pubblici - BolognaToday</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>General strike and march: stop in schools, healthcare and public offices - BolognaToday</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>Thu, 05 Mar 2026 08:10:00 GMT</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE9LRk82di1uN2ZNLXJCbjJ5Zld4X2NvbzdVOS1mZEdwcEdFcGhUT0w3LVpWR29sdS1ZQ2RDSTNBSGpFWDY0S1NYQ1EzRW5ZUTNNcjNJelhLS2FKVl80eS1WLThWNlRpN1BJNThfMWV5TFluZ3lGSDlvQTRzbjlyZw?oc=5</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K67" s="1" t="n">
-        <v>46086.34027777778</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>A Milano come a Berlino e Torino la protesta degli studenti contro la guerra, nel mirino il ministro Crosetto: “No alla leva obbligatoria e a politiche guerrafondaie” - Il Giorno</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>In Milan, as in Berlin and Turin, the student protest against the war, with Minister Crosetto in the crosshairs: "No to compulsory military service and warmongering policies" - Il Giorno</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>Thu, 05 Mar 2026 17:40:08 GMT</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOckxLdjYzSkI3YXV6WFdReEd4eUZ0emc3V0NXYjJpaVJ3YVZUSUFEUWhMZlNlMDVXVHFzSUR2dUhWdWFtdkNXUGpjNHZ4amwyU3l1R1hwMWtzUGFneVk4SHFLV3ZSNlJtQmJBMnJtcGdtY2lPc3FrOHZPRFRUM0kyZ1pEQnZtS3p5OE50RXRCSlM2c19iTFFVUDBsZ1ZNSlVVY1paaEhkS2QtbGpUd1FCZS0xM2dxRG1VaTlHXw?oc=5</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K68" s="1" t="n">
-        <v>46086.7362037037</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>Esprime solidarietà alla Palestina, salta la liberazione anticipata - il manifesto</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>Expresses solidarity with Palestine, skips early release - the manifesto</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>Thu, 05 Mar 2026 23:15:15 GMT</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxNQkt2Z1VuakNxejFXYlU0dWZGQmZWbnZremVlbFRuLVhqU3M0OUdBRDRPaFR3RnNURkxiSGUyc3U4ajg3X0tOSGRhdXhqSTFXQ0ZNbG9SWl9lLTZaR0JtNlZFRVZaSnRKREFJSzM4Zi1aNWNrcG5USFN4OUhoWVp2MWpJZERpY2ZKVFowTXpXNW55Ulk?oc=5</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H69" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J69" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K69" s="1" t="n">
-        <v>46086.96892361111</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>Bologna, spintoni tra Digos e i manifestanti contro la Lagarde - RaiNews</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>Bologna, shoving between Digos and protesters against Lagarde - RaiNews</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>Thu, 05 Mar 2026 18:59:03 GMT</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxQaE81ai1nMXNqTFE4N3pIcV9zMkpqMlRkazlHcWpEQ19TZnZRSWdxYlNNN1FGclVBRW9zQ1o1bU1YcHNkaFF6ZDZUUV9ubDNUUFVzYjhvc3lKOWVrbkROLW03bXJ1TkUxQkF0QjNMTDhpV0Jnd1NFQXBva1hyTDhEemFkQVQ2RzY3RHdVNjI0blYyeGVBUllDRW9JenlFem5INlVlM29jcGVsX0hPWHRzYUdVQVBQeTh5WnZack52UmFHV3diWEl0cEcyT1Fwd3VYYXRtc3VUNy1lOXF10gHcAUFVX3lxTFBoTzVqLWcxc2pMUTg3ekhxX3MySmoyVGRrOUdxakRDX1NmdlFJZ3FiU003UUZyVUFFb3NDWjVtTVhwc2RoUXpkNlRRX25sM1RQVXNiOG9zeUo5ZWtuRE4tbTdtcnVORTFCQXRCM0xMOGlXQmd3U0VBcG9rWHJMOER6YWRBVDZHNjdEd1U2MjRuVjJ4ZUFSWUNFb0l6eUV6bkg2VWUzb2NwZWxfSE9YdHNhR1VBUFB5OHladlpyTnZSYUdXd2JYSXRwRzJPUXB3dVhhdG1zdVQ3LWU5cXU?oc=5</t>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H70" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J70" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K70" s="1" t="n">
-        <v>46086.79100694445</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>La “Milano-Meda” a pagamento? Scattano tre flashmob: "No al ticket" - Il Giorno</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>The “Milano-Meda” for a fee? Three flashmobs break out: "No to tickets" - Il Giorno</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>Fri, 06 Mar 2026 03:50:15 GMT</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxOazU0bFcyZnBuLVZvbXpESl9SY2xwdV9JajZBcFFGVHhOQ2xQV2tFNUVRZFZESUNRVmN1UkFZWlNMb0tUQWpyRWg1VTRUY0d6SzRTNkR6TDdQeV9Jb1NNRGp4U1N6cWhTWXB3dmVZUTZSWFktRGI0dS1FU2N3TGhjTE5FUUtEV3pBNWxr?oc=5</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J71" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K71" s="1" t="n">
-        <v>46087.15989583333</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>Sciopero generale del 9 marzo, si fermano anche i mezzi pubblici? Chi aderisce e chi no - Moveo by Telepass</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>General strike on March 9th, will public transport also stop? Who joins and who doesn't - Moveo by Telepass</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>Thu, 05 Mar 2026 09:02:48 GMT</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMickFVX3lxTFBOOFg4aFJ1RXNfSmpYTUJoRDBiazE1WXB3alBabWhpQTVFa2MwbG5qUmFSQVJaQzU5RVJyU1FZLUV1Y2h6RmN5RXB2dWNvZ2FrTUoyX1VCSW1xS3lNT0IwS0VVclhLUFZ4Z196dndCYnpadw?oc=5</t>
-        </is>
-      </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J72" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K72" s="1" t="n">
-        <v>46086.37694444445</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>Pilastro, presidio smantellato. Maxi-multe della Digos a tre attivisti. Applicato il nuovo decreto sicurezza - Il Resto del Carlino</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>Pillar, garrison dismantled. Maxi fines from Digos to three activists. The new safety decree has been applied - Il Resto del Carlino</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>Thu, 05 Mar 2026 12:00:34 GMT</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxNdk9YZlR2TXl2eFF2dC1ia245VjR4VkhvVnFHYk1SYmZ4a3I3LTZ3dUczNTRCdDVXMnlXMDRvWkVQOEdlZTZEeTNJckRobHBqUjY3aVdmV0VZWEFHaDdMeXhvNEhkamlFZnJHOEVpSEgtaUVQTzRkTlhiZWhpcW9DWWV0TTg4RVRuX3BQRXVlTE9oVkxrYkZFZ1lKMEI3dmJZNUg3XzIwVQ?oc=5</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J73" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K73" s="1" t="n">
-        <v>46086.50039351852</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>Anci: "La scuola è il presidio di comunità, di inclusione e di relazione con il territorio" - NewTuscia</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>Anci: "The school is the garrison of community, inclusion and relationship with the territory" - NewTuscia</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>Thu, 05 Mar 2026 15:04:05 GMT</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPY3NzMGlUZmtfb2NzX216VUxCUzZCUVNja29NbGk0ZDhfUFhvdTd4NnZ6aHc4b1hzaV9tOFM1SUprZ2E0eVhUWWVVTF96TW1uZlhhU0oyaGhkNkQ0UXoxSXIzZEV4U05VZXBwTG1Va3ZjM3BFVnE2VkdEWG00azA0ZURJal8xWV9yQ0NhWTJONWpEOW4wMldEU2NDQ2JaQXZIU183RXhqYm5JVnZNN1lXa2ktLWMyOWg0YW5qUkVCbXVoQQ?oc=5</t>
-        </is>
-      </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K74" s="1" t="n">
-        <v>46086.62783564815</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>Local Town Fidenza Italian</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>("Fidenza" OR "Parma" OR "Piacenza" OR "Cremona") AND (protesta OR "minaccia bomba" OR esplosione OR sparatoria OR accoltellamento OR evacuazione OR "operazione di polizia" OR arresto) AND -calcio AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>Morto dopo essere stato accoltellato al torace a Parma, fidanzata di Cristopher Gaston Ogando indagata - Virgilio</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>Christopher Gaston Ogando's girlfriend died after being stabbed in the chest in Parma - Virgilio</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>Thu, 05 Mar 2026 19:13:00 GMT</t>
-        </is>
-      </c>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxPSHFvaWdSMlRmMDdVZzFfY0x2MmFqTTFabHNWVTRmWlBVcFpHdlVBQ2JJM0l4dVhKNWQtTHY3WG1XT1JBeVdiemhKdThJY2xqU3FGYUlTNFA0dHNyLVNzQTR3Z0h2X3ZzQTYyRlZHUEhMSl82WXZkaHhPMnpGbXpIaVhjRjdCT0g2bm56R1BqQ3YyaWl5NmxVMmotR0o2U1JIazV3aUVvRXp1M1ZGc0Z1Ry15WHN6bUF3UlVSSUE5TFZabjFheG1LSzhKdG5wbGhiRDgzU3I5TmfSAd4BQVVfeXFMT3k2aVBGajNUYWdGZTBRUHlkZmxmcEs5NmFYYjhJWEZkNldGemRCbER5Y3ZhZGx1blN4OHNTeEtzN0VnODJ2eXMtenhYT2oxbFpFZXVHdDlualZJMG02SFVhRThwY3VOcjNVY2NrTDE0bl9nMlh4X0ZVdzg1SnQ4VFZmeW5rMnJBaG1xZFNQTGY5OUJsb3VrTGd3S3FWZjMwMzFMTURsQlpxeU1kY3A1ZzdVaDZrd0pFcVBKZkpxUzZoNzJYTWhWMUhCR09qWmR6SlBhMG41cmtqb0RSQlZR?oc=5</t>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H75" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J75" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K75" s="1" t="n">
-        <v>46086.80069444444</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>Local Town Fidenza Italian</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>("Fidenza" OR "Parma" OR "Piacenza" OR "Cremona") AND (protesta OR "minaccia bomba" OR esplosione OR sparatoria OR accoltellamento OR evacuazione OR "operazione di polizia" OR arresto) AND -calcio AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>Parma, giovane accoltellato e ucciso dopo una lite. Indagata la fidanzata - la Repubblica</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>Parma, young man stabbed and killed after an argument. Girlfriend investigated - la Repubblica</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>Thu, 05 Mar 2026 09:52:47 GMT</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQN1l6dGtNYjF6NU1iblhlUW9ZalhKb3ZnS3REMEZfakZ4MUJyd2piYlFKcjcxUmNqNk9WZ0ZCMEFRejlxY1VtRktQbm12cVB4aXFhTFBNMUtyT29ZX3VfTUdNUDgzbHNVazVxVElXTWg0VnhZSFN2X0dsUkhDVnNyS3BsSXAxZGwtZTg0eXFIbDItNjk3eTdTc1pnLU5CTGZyNkt5VXBpYlJiVU1STTR4Sm5ZZkR0cHAxNVA0?oc=5</t>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I76" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J76" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K76" s="1" t="n">
-        <v>46086.41165509259</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>Local Town Fidenza Italian</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>("Fidenza" OR "Parma" OR "Piacenza" OR "Cremona") AND (protesta OR "minaccia bomba" OR esplosione OR sparatoria OR accoltellamento OR evacuazione OR "operazione di polizia" OR arresto) AND -calcio AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>"Visite private pagate in contanti": medico primario arrestato dai Nas di Parma - ParmaToday</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>"Private visits paid in cash": primary doctor arrested by the Parma NAS - ParmaToday</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>Thu, 05 Mar 2026 08:04:08 GMT</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPWmtETkZER3RWclhUT0dfWHRFMjZSR0wwOGQ2LTRWOFVlVWMwTFR0Q2pHMm10TmZoVHN6LVlQZWxITTU2RVB1OFRvWjdxQlpVZmN5V0xjSkVqcGdXUUllX2RoaS1Ua0haRWs0M2dDX19XbU03LXRxZGxEakZmTUYzVUU3ZlJhZE9YdGlreDZpdl9wOFE3OEE?oc=5</t>
-        </is>
-      </c>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H77" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J77" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K77" s="1" t="n">
-        <v>46086.3362037037</v>
+        <v>46087.49026620371</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-03-07 07:38 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K58"/>
+  <dimension ref="A1:K66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,32 +480,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Replacement for huge empty Bullring shop confirmed as massive signs go up in Birmingham - Birmingham Live</t>
+          <t>Woolworth March 6: 1,000th Germany Store Marks Value Retail Surge - Meyka</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Replacement for huge empty Bullring shop confirmed as massive signs go up in Birmingham - Birmingham Live</t>
+          <t>Woolworth March 6: 1,000th Germany Store Marks Value Retail Surge - Meyka</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 10:54:00 GMT</t>
+          <t>Fri, 06 Mar 2026 16:54:37 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOc0pNTWdGR05qWkRub1RaOHo2dXhzVDdNWncyckxsSTlsZGVqSjJjXy1nbDU2VHFvZmtINXU5X2lDaUFhVWZQVTB5TGZjaFFIS1hPdm9yYzJpVlp0NFY5bGNOWWZWcmxiQXdSc3phT0ZCTHdudUlrR196OW1MQzM5dVU0SFR5Y3A4N2sySkhvelYzSGRuMXBrcUJOWHpmT2I0eEtTUzNaQnXSAagBQVVfeXFMTnNKTU1nRkdOalpEbm9UWjh6NnV4c1Q3TVp3MnJMbEk5bGRlakoyY18tZ2w1NlRxb2ZrSDV1OV9pQ2lBYVVmUFUweUxmY2hRSEtYT3ZvcmMyaVZadDRWOWxjTllmVnJsYkF3UnN6YU9GQkx3bnVJa0dfejltTEMzOXVVNEhUeWNwODdrMkpIb3pWM0hkbjFwa3FCTlh6Zk9iNHhLU1MzWkJ1?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxNdkJJUk5LQjUzRUNNNy0wQ0dzQTAtcndDUm1tY0RUY0lPRTJsMmZ5b2ZKZ0FIQ1JVaV81N1dYZjg4X0dlOWcwZlo4N1VHOHM2ZmNyTWFGU1VaUnZrelVQRWV1Y2hPd05lbk9LMVJMa3lDbDB5WWt1VllSOEhwS3ItZXkwYlJHd0NEajYyTUZUQmZiZUMwOFB3?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -529,38 +529,38 @@
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46087.45416666667</v>
+        <v>46087.70459490741</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Prinses Kate stuurt ‘zeer bewuste’ verborgen boodschap met haar kleding na arrestatie van Andrew - HLN</t>
+          <t>The Efficiency Machine: A Deep Dive into Williams-Sonoma’s Profitability Renaissance - FinancialContent</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Princess Kate sends 'very deliberate' hidden message with her clothing after Andrew's arrest - HLN</t>
+          <t>The Efficiency Machine: A Deep Dive into Williams-Sonoma’s Profitability Renaissance - FinancialContent</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 12:15:26 GMT</t>
+          <t>Fri, 06 Mar 2026 14:48:00 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxPeUk2U3lTdVlQOFJteENNWnA0R1JYcG1rallxYnNZMFlvS0UxcVQxRU94WTdNUVZmZkdQaHhHWUlOdzFLNjJzb1ZpU3paWnNZd09URlJZblo3ZlFHZlNXM0ctSDQ4WG5UWmtTbzV5YjJHZ1I2UEx5c0ZuS3Vkd2Zxd2thNllCbnpzQXE0OHdfWWoxOFpILV9KYkw1ZEdWX3VIaldaak9BdEYtQlgxai1rcC0zajg5dHZzUGpUQ3M3Wm1QUVRYN1ktTzRQbw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxPYXRFbVNZWTR1VDFnVTk5cTZrcWNETm1PSE9wTFNMaUhFZEFHYVZHS2dHTlN3aEJDX0ZLYVlsOFRTT1Q1WEd2ZWVTYW9zV295ZVlOSWp5TkktREVBd2Y5eWl1Wkc5bHdxRTBKcEE5TlNYdFB1bUltYjd4ZFBqSTlUNUhjMjdlRVBoOHlXZGo3cnZheEtFd1h5Zm53RGFsNjMyM0xxUGlhMmhMWURqMmlOMmVvMS1HcHFWaHM0c2RQRC1qN1A2UndXMTVIQ1lDQTkyQmxuRGpYaC0xaE1oMDlhbnZBZ0E2MG8?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -570,52 +570,52 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46087.5107175926</v>
+        <v>46087.61666666667</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Zonen ontfermen zich over Britney Spears na haar arrestatie voor rijden onder invloed: “Willen haar op het juiste pad zetten” - GVA</t>
+          <t>Customers warned ‘check before you travel’ ahead of key London Marylebone upgrades - Chiltern Railways News</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Sons take care of Britney Spears after her arrest for driving under the influence: “Want to put her on the right path” - GVA</t>
+          <t>Customers warned ‘check before you travel’ ahead of key London Marylebone upgrades - Chiltern Railways News</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 12:50:25 GMT</t>
+          <t>Fri, 06 Mar 2026 17:51:40 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijwJBVV95cUxPSnVOeS0tbmNuQWhBakFpbndab2RmWHdiUWV3bE9Vcm1fRVpLV0o2ZTJNbGNPOXhDaE5idW53elJoamRGcmN1anBpYU16Z2RuNHhTbExmcmRLX3ZYWXlFeVJHOVFtTXRreG8wdUpWcmZMVVdsenRURlQ1MDJLNFRqRjdYTmViSDUzOURETEhmNENyWlZzUFVfaC1SLWNiYVNVUFBFeG12RDRQMjV3ZFRIVmxfeHRKT0hQYm5GY3E0eGVCYlIzMVlGMzN6RTdwXzB6MWZsdmVhTUZ4d25qQ1hqZWlXa2FHSHVsN0Iyb2VVYjQyWkl2U3JjcFhUcENwbF96Z2dMUkZOc2x4RTVUNTZJ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxNTmdHd29YbDRwTnNrNlZYVnlyR3R5T3JMcmFPUHYwRHJ0WTduTXVDV1VYdUFXbzhDbXBkcURibGpTblBzVmUyMm9DUUhJeHVqYWo4SHJNWlR4V2FmOTNFQnBpR2s5VDY5clNHWTBYcXQ0Yl8yVjJKQTRvbXNoaVNYSzhiR2RZQjl4dk94MFRLSkRJUHFYeUZxbF9WRUlxMHNBLUFYeHB0cVM1MGF5MUZyRnJnbDFtN3JNb2NXTEgzWQ?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -625,52 +625,52 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46087.53501157407</v>
+        <v>46087.74421296296</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Diefstal uit auto leidt kort nadien tot arrestatie aan andere kant van land - Nieuwsblad</t>
+          <t>Plans for 41 later living homes in village refused by council - This Is Oxfordshire</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Theft from car shortly afterwards leads to arrest on the other side of the country - Nieuwsblad</t>
+          <t>Plans for 41 later living homes in village refused by council - This Is Oxfordshire</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 14:35:23 GMT</t>
+          <t>Sat, 07 Mar 2026 05:00:00 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxPMEE3ZGkxQnVpREZyRHdvWnRyamY2OERYWm5iN0F6NnFTaVlkUThvdXJBM3VObkFFY2NBdHBhYS14R2JYUzAzNHZxUGo0d1FRdXF1VzY4YjdaSi1sY0Fwd2ZhVkQ0d3IxMlpyS3BEVXNrcENkdE13NnhIVFk0M0tUek13MkVJMjBvaWwxTGV1eXFSWDllOXJuVEFaS3o4aGd5Z0oxMGlWdUZhNEhuSGo5RkhGNkQ4WnBGaTVoaTlvemVWNVN4MlQ5N1NVN2F4NVFGUnhiVnFySl9ZRWM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOVGlDUk02OVRSQ2FpcGV6VVltTXMtTzFzNFlnZW1SaXdHZGtVUEY3b2JNSWxuSGRNODFFV2VBQ1pfems2Z1BmSmpLem5XLXlzSlU3NmlDSm9xWndoRWtJS1hVMGhOUnc3MWpVZm04dlUtNXlmVUFvX0loT2Q0WGplR0ZRQjljSklUUWFFOV9VQU5oZzRyelRyc0tpR2J6NFFRcXRF?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -680,52 +680,52 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46087.60790509259</v>
+        <v>46088.20833333334</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Jessy Mackenzie getuigt na MeToo-bom in muziekwereld: “Ik werd als 18-jarige zelf gemanipuleerd” - HLN</t>
+          <t>Replacement for huge empty Bullring shop confirmed as massive signs go up in Birmingham - Birmingham Live</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Jessy Mackenzie testifies after MeToo bomb in the music world: “I was manipulated as an 18-year-old” - HLN</t>
+          <t>Replacement for huge empty Bullring shop confirmed as massive signs go up in Birmingham - Birmingham Live</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 10:08:11 GMT</t>
+          <t>Fri, 06 Mar 2026 10:54:00 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxNbmFXaGpuakhNRHo4c0pwWUNiV2laTWk2V3RSMWlWdXJlTnljZ2dSWnBHOGd1SmlaSnZEV1o0dzBaVUpoMjRWUzRmWnk3MFpyVEhuSzFMX0VYbDNiZkdxTVpnWXNhZVMzb2ZEZExnU1ZKMTkxaTFZcHR5dk94UHJRVXB1U0lEYUoyYTBxR2k5TEd6cmpBZGROcTdoX0owOWNieUtTX0k4WF9La3NWbHNtVU5kRmJVUVAxR0E5Vl9SZGFZc0QwY3Q4N05aQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOc0pNTWdGR05qWkRub1RaOHo2dXhzVDdNWncyckxsSTlsZGVqSjJjXy1nbDU2VHFvZmtINXU5X2lDaUFhVWZQVTB5TGZjaFFIS1hPdm9yYzJpVlp0NFY5bGNOWWZWcmxiQXdSc3phT0ZCTHdudUlrR196OW1MQzM5dVU0SFR5Y3A4N2sySkhvelYzSGRuMXBrcUJOWHpmT2I0eEtTUzNaQnXSAagBQVVfeXFMTnNKTU1nRkdOalpEbm9UWjh6NnV4c1Q3TVp3MnJMbEk5bGRlakoyY18tZ2w1NlRxb2ZrSDV1OV9pQ2lBYVVmUFUweUxmY2hRSEtYT3ZvcmMyaVZadDRWOWxjTllmVnJsYkF3UnN6YU9GQkx3bnVJa0dfejltTEMzOXVVNEhUeWNwODdrMkpIb3pWM0hkbjFwa3FCTlh6Zk9iNHhLU1MzWkJ1?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -735,52 +735,52 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46087.42234953704</v>
+        <v>46087.45416666667</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>London Marylebone Incident</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("London Marylebone" OR "Marylebone station") AND (incident OR disruption OR closure OR police OR bomb OR explosion OR stabbing OR shooting OR "suspicious package")</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Woonhaven Antwerpen verkoopt samen met gemeente vijf bescheiden woningen in Maria-ter-Heide - HLN</t>
+          <t>Tube lines still hit by delays after rush hour disruption - MSN</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Woonhaven Antwerp, together with the municipality, sells five modest homes in Maria-ter-Heide - HLN</t>
+          <t>Tube lines still hit by delays after rush hour disruption - MSN</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 13:24:38 GMT</t>
+          <t>Fri, 06 Mar 2026 12:41:03 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxQM3ZMdWR4aFQ5RzZzZExEcDEyNXVLVmVqWVpvUmxJaTBoNG16U1duT21BbE95ZjVwOWh6OS1icVdrNXBnRXhJbWRUOTZLTTFVN3VJM0Z4ajQ2V1g3ZDRaQk9HejItelZaX1N0a2tLRWM3OHZJaDVxZjBHaFdIVDBoTVlnUUZjR3I1T1luM3ZQRkFIcjd6Rzhjcmw2dXhfSjlzRGJ3QWh5TXFzLXFwRlI5cGNPUlF6T3lXVmlGMHgxcFZiTFpVRTNCclRyaw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxNZzJ6T2htT1lZdndMdmVtQ0FUWmFRZE1hME9iSkM1a3hmZEQ1cnUydFE3QmFzU0hBbFM1N1RrY29ySm5PaXdMeTFXcEttTndCbzRXN2lIUi0xeVJkYThCb2o1VHR2Y2dSeVlxQ190cHJxeWNVRXhOSnVtZ1NNNElJT2lWRlBJRERKdkVBc1lmZ1FkUFNCd1E4WEU5RnRoQ1dDTjdkY1UwbHh1ZTQ?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -790,21 +790,21 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46087.55877314815</v>
+        <v>46087.52850694444</v>
       </c>
     </row>
     <row r="8">
@@ -820,22 +820,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>20 minuten file op de E313 naar Antwerpen door defect voertuig in Wommelgem - HLN</t>
+          <t>Politie treft zwaargewonde man aan na steekpartij in Borgerhout - HLN</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>20 minutes of traffic jam on the E313 to Antwerp due to defective vehicle in Wommelgem - HLN</t>
+          <t>Police find seriously injured man after stabbing in Borgerhout - HLN</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 13:28:27 GMT</t>
+          <t>Sat, 07 Mar 2026 07:05:40 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxPZ1k4Y3pub0dQVVFhVTU4MEtqZDdBX29GcHBPWnNmcnlpdnhnbVp6WFZjYXZCTGlTNFBkWnlia2hJN1c1akZjZE5QNk1VVzVYRGNsMVVwV2M3TUxDbWYzQi05VkdRX3RzUm9ReGJiTjEwenpvQlNiZXBmVER0c1pnVjU1aXA0eEJQWktoN252RDZMbVFISEc4VllvS0tqblItUFJLYml3TjhqYnpoS1ZCQ2FucnM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPZ2FydjNGYm5aakN4Rm1zU1M4U1RmbUlha25JWlVlU1VnQTFVX1pZNGFWc3hEai1CcENUeUFfbGtpa0NlMUJ3eUdLT0ViMXRjVXdQVmQxTHd2eUxvRXpna0hTRHFVN18yXzJPMGo2cmlsTndyZ004LVhDb0llTWdnV0YtcF9nZzJTM3BxWER6SXAwVnBlQ2g3Si1CWm00a0dEY2xkZg?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46087.56142361111</v>
+        <v>46088.29560185185</v>
       </c>
     </row>
     <row r="9">
@@ -875,22 +875,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Nederlanders vinden oplossing die Antwerpen ontziet tijdens werken Westerscheldetunnel - HLN</t>
+          <t>Antwerpse politie sluit parking van Decathlon af om tuners tegen te houden - GVA</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Dutch find solution that spares Antwerp during Western Scheldt tunnel works - HLN</t>
+          <t>Antwerp police close Decathlon parking lot to stop tuners - GVA</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 07:41:46 GMT</t>
+          <t>Sat, 07 Mar 2026 05:06:50 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxQY2FuVjljTWlhclhUU3hibHBRZW1lN3RwaDlHSkMySkpmSzFicjVhRHdfdnU4V2tjd0VISHVVRWxFeFdkTmNoYWI0QTZYa0ZhMWtiZmM4aTk2UzF5ZlpCSmNGWG5YTlo3YzZZcGN5TDJfSGRMOFVWWEpKaTFOQXpEX1BKM2VZYVdFT1Z3U0s0LU5ueHNfYWIya3RwTGRGLUZ3NGJ0clNnTWI4dEk1R3FQWHk2RURrSTJoWUtWdHhwZFphRE0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxPTHI5TmJyMWdRcmdFc3ZCV04xX0lYa2NfdkUtOGN1bTZyU2tlNmV3dEVSSU5uU2NfNEhxTy10TXotR3QyMDNXWlVsRVVpa0tySzBnWHQ3UGFyVWZWM1dzajFkdjNnQWpfbGtmZzFWLXdEWVV6N200ZFJWMl9qOXFFdmlzNGZ5R3RnOG9rd1N1U21XZWY4OWkwVlN4VGxlMUhnbno5MUZfWnJSU0pnQl9uOVF1Nm1wdnIzNnNySnc1d1cxQ2tkZjhkOC1iREpiTFJaakQzQ2k5T1dXTmZNYUdmOXlublM?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -914,7 +914,7 @@
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46087.32067129629</v>
+        <v>46088.2130787037</v>
       </c>
     </row>
     <row r="10">
@@ -930,22 +930,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Stad Brussel lanceert plan tegen straatintimidatie - HLN</t>
+          <t>Voortvluchtige Antwerpenaar (22) gearresteerd op Franse luchthaven - GVA</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>City of Brussels launches plan against street intimidation - HLN</t>
+          <t>Fugitive Antwerp resident (22) arrested at French airport - GVA</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 13:58:01 GMT</t>
+          <t>Fri, 06 Mar 2026 17:15:15 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxQcmNKSnprMTA5OEpvR0wyVVNTUTY2SnNnQy1pSlhlbGJ5TzNyS0c5bWFoUHk1Wi1BY1BCQTJrc0U1aF9HSFVvVUMzdFpxa09TS0ttc2Z3aFh6X29zdDN2ZDNCYW5nVHd4RGhjTFhvYktGTHNicnZxWGt4MUZtM2s5NTAxLXdEUE1EQUVqY0x1dmY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQSVRINHFTbG9tenlTZGRvQVViUmo4MTFMQWlvRGpjcHRPVkN6WmlpQ2cyendBQlhBQmVkLVFuSmtESFZlaUg5cHZ3WW1UU0xCVWNjWkdXU2R1OU1pdDN3NGs5MGYxMHdTZW5kOWV4STc0bmpvUGpGQVdTMFBNR3BaU2N3cEthQk40ZUs3OVZudHY5R1Z3ZzR2bE5LNFd4Nl9NYkNOenJkSzhzUERwTktXOHFYaGdoeTBldlU3UVpwRGllZXhoaXRJZHJUcE1DYUNBRXVQb0JhMA?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46087.58195601852</v>
+        <v>46087.71892361111</v>
       </c>
     </row>
     <row r="11">
@@ -985,22 +985,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Bewoners ontwerpen eigen carnavalsmaskers in residentie La Cambre - HLN</t>
+          <t>Treinverkeer van en naar Brussel grondig verstoord door werken in weekend van 7 en 8 maart - Nieuwsblad</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Residents design their own carnival masks in the La Cambre residence - HLN</t>
+          <t>Train traffic to and from Brussels thoroughly disrupted by works during the weekend of March 7 and 8 - Nieuwsblad</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 13:38:19 GMT</t>
+          <t>Fri, 06 Mar 2026 13:22:08 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOUFhQUFl2Z1pkN21IR204TWFLcWhzS1pvUWxfeFVuTDlaem9mMi1fdDhNZXNYNWp2aEhRcHVDZzdPQTdRbDBDNkFyVmw5aG16cTdVdHB4XzFzUU9KTlhCdUdYSHhUbTFIMnAwaFJTQ3ZvSDkzNk5hdnVjdXc2dzBZU2pZSERrVVVDZ044QzNxcHA1Q09qTTRGbFh1eWdOY085bGZ4Qg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxPY1ZRVXY1a2lvTFY2MGdpODk1eXhQdjJ5eklxdElDOHFVdWNSU2VPbTIwMUtlUGNlVGtyRjV3dWtGVTh1T1hjQVNDWkw0U1pfYlpXUFFlcmxrZTFMSGhPTHp6eGNNUjFOcENGcDNVODk5WWJzbXl1dzg3VWRqcmMzRDg3Mm5LLWhzVHhKRk5jTWJTbnJCT3NFVWRxaHY3Z1YtN3pYMDBTUVVreTRrZnoyNEpNNWZMNzlLWWJKZEx5NTRST1ZFckdOMzZnQ190NlRiZjE0UQ?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1024,7 +1024,7 @@
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46087.56827546296</v>
+        <v>46087.55703703704</v>
       </c>
     </row>
     <row r="12">
@@ -1040,22 +1040,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Groen wil “volwaardige fietsboulevard’ tussen Antwerpen-Centraal en Berchem - HLN</t>
+          <t>Jozef Van den Nieuwenhuizen, 97 jaar - GVA</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Groen wants a “full-fledged bicycle boulevard” between Antwerp Central and Berchem - HLN</t>
+          <t>Jozef Van den Nieuwenhuizen, 97 years old - GVA</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 13:33:18 GMT</t>
+          <t>Sat, 07 Mar 2026 04:13:56 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxQU0JQLUFteWVoYmFtc0pjSEFuanNraXVGRzJFSzRuSFI1bHdydVRObDhEVWFZTXBJbm9TQlBXTk1VRGtCSjI3OWpHMEtpbXVtQU1ja28wMHFUMmo2OGUtQTYwT0dMT3cydk41U09jRE5HSFA1Vll4aU15cWhGVjJpVjBUbkZ6bnZneG5DYXNDQlFVeFNNU3ZrdGtUaGo4Nl84eFdsZl80QU5wV0tYMW9JODV3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxQMGM0YXFoRWtOMmExOEw2Y1MtSDJ5d3p3OUdVWEVqUzF6MVplZU83QzlkYnhMV0VzRXlJeF96Y0JKazhLeHpEendUUVEyRzJaRWNlRUl4VnFyNjMwcUdLSkZBek4tNGJRZmlKQlFQMzhLU1pvME5GQmduaXppOGhOYVRvaW1xS0VvdnUteU5MWQ?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1079,7 +1079,7 @@
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46087.56479166666</v>
+        <v>46088.17634259259</v>
       </c>
     </row>
     <row r="13">
@@ -1095,22 +1095,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Drie voorbijgangers redden persoon uit kanaal aan metrostation Delacroix in Anderlecht - HLN</t>
+          <t>Diefstal uit auto leidt kort nadien tot arrestatie aan andere kant van land - Nieuwsblad</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Three passers-by rescue a person from the canal at Delacroix metro station in Anderlecht - HLN</t>
+          <t>Theft from car shortly afterwards leads to arrest on the other side of the country - Nieuwsblad</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 12:23:01 GMT</t>
+          <t>Fri, 06 Mar 2026 14:35:23 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxPREw1UUFQNllDVUFZMEhGeW8tal9Mdk1nZTNWUkRwQklLTXhNTFltWjZtZUdIUkx5T3JQaGkxUFBsNi0ybE1qQU1lUVdTOHh4TDFvSm94QUxieFNtMmdBUWx6eXc0YTBnX0NwWWlNM1NTQ3VPTzdvQktsMFhFMTlBSzh1QmpsN1d3WXY0aGg0Yi1aU2V5OTFxV0x0VGNSSEQ4TUJIeXJ2TkxZS1o2NC14bDJzVTJHUnNKYkszeDQ4VGU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxPMEE3ZGkxQnVpREZyRHdvWnRyamY2OERYWm5iN0F6NnFTaVlkUThvdXJBM3VObkFFY2NBdHBhYS14R2JYUzAzNHZxUGo0d1FRdXF1VzY4YjdaSi1sY0Fwd2ZhVkQ0d3IxMlpyS3BEVXNrcENkdE13NnhIVFk0M0tUek13MkVJMjBvaWwxTGV1eXFSWDllOXJuVEFaS3o4aGd5Z0oxMGlWdUZhNEhuSGo5RkhGNkQ4WnBGaTVoaTlvemVWNVN4MlQ5N1NVN2F4NVFGUnhiVnFySl9ZRWM?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1134,38 +1134,38 @@
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46087.51598379629</v>
+        <v>46087.60790509259</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Exclusive-NATO’s Rutte does not see need to invoke Art. 5 after missile incident - WTAQ</t>
+          <t>Melding van explosie Roermond - De Limburger</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Exclusive-NATO’s Rutte does not see need to invoke Art. 5 after missile incident - WTAQ</t>
+          <t>Report of explosion Roermond - De Limburger</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 09:45:20 GMT</t>
+          <t>Fri, 06 Mar 2026 22:59:57 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQeE1KT2p0eEJXTmw4TlRFVG9zc0dOZ3FXdEFOLWxTRmdvcWx4bVcwaXVGUXdPdWJoLXB0aGx1VjczNVVEb09xVnhGSHNrampDMkJNc0ZGMDNoVHVzcDdhVHRoQ1pwMXk2TWlqbVE4WHJmWnNOcm82NXVxVDJsMXVHMHpvdnZCdUtyR001cHdfOXB4WUJSa2haRUU0NHZnbnVxeHBNTWNJR1kwNUk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNQzdkWmxjOHJ0NVF0VkFWdXEweDdYaDlONEVHZXBPUzFJRUd4Qzk1U2liZHhYaTFDdkV0eTJqWmJQZWtTMW0wWVBjMmZaWmxGbnFrWEZfMHdjWHNDcjU0ZTNhTF9Ea1NsVzQ3OF83cUUwNGlnTkFEVmxCbzlNYUxMdG5BM0ZVcU5h?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1185,42 +1185,42 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46087.40648148148</v>
+        <v>46087.95829861111</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>"J'ai atteint une paix intérieure": une rescapée du 22 mars a rencontré l'un des condamnés des attentats de Bruxelles - BruxellesToday</t>
+          <t>Amper treinverkeer in Brussel-Noord en Brussel-Centraal dit weekend - HLN</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>“I achieved inner peace”: a survivor of March 22 met one of those convicted of the Brussels attacks - BruxellesToday</t>
+          <t>Hardly any train traffic in Brussels North and Brussels Central this weekend - HLN</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 11:00:00 GMT</t>
+          <t>Sat, 07 Mar 2026 07:03:20 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxPZlFlWXNkRmZlZXZnTGFYeTFld1JleUNiaXVsMTgyMDdGSE8tS3J0WUhLZ0loTU43ZkVCaEo3cmNteUlaZnh5dS1zVGllZllMU0JxTThFZWtOUHp3N3JkNTlOQnVkVkZLOWZFRGpvS28wLUR3aC1NQ3VJem1FeTVHQ0lkRUxDSjNNTXc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxQb1lZYUlhQWw1Y0QzQkRmdkRVWGFnYzdJQjlkZUdacGtVZWVoVWVCQU5NNkhhUEVOOTFfSTJEN1pfeFFPanJ2VFo1ZHZyck5YVjZJcTdtOWJ0d2h6bUlwdkFKVHFlWWc4S1U5QTBBcWZySFdqcTFoMGh2WFlzZk9HRG1YT1lpUzVzWmVVLThjd04wSExXZWlFdU95Zl9WWGVZR1VQQk1jcw?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1240,42 +1240,42 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46087.45833333334</v>
+        <v>46088.29398148148</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Hammam de Schaerbeek : Comment un simple conflit de voisinage a viré au procès pour meurtre - Bladi.net</t>
+          <t>Prinses Kate stuurt ‘zeer bewuste’ verborgen boodschap met haar kleding na arrestatie van Andrew - HLN</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Schaerbeek hammam: How a simple neighborhood conflict turned into a murder trial - Bladi.net</t>
+          <t>Princess Kate sends 'very deliberate' hidden message with her clothing after Andrew's arrest - HLN</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 12:00:00 GMT</t>
+          <t>Fri, 06 Mar 2026 12:15:26 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQWnFXYmRyakhQdVhWTnJZUXFqcWhNanNPeHQ4MGZpQnk4YVlabFRzT0l2Z1Q3X1JYNkt4X0hFYXJoekFIRUJCMHZVS3pNeV9HU2s2NGVEUTNuV3Y5M3o5RjR1allhTjFiNUFlcVZvWWdLRTdlQnpxX2ZCOFJiYkZuRXJER2JuOHVEVzJEVEJ3MDBPdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxPeUk2U3lTdVlQOFJteENNWnA0R1JYcG1rallxYnNZMFlvS0UxcVQxRU94WTdNUVZmZkdQaHhHWUlOdzFLNjJzb1ZpU3paWnNZd09URlJZblo3ZlFHZlNXM0ctSDQ4WG5UWmtTbzV5YjJHZ1I2UEx5c0ZuS3Vkd2Zxd2thNllCbnpzQXE0OHdfWWoxOFpILV9KYkw1ZEdWX3VIaldaak9BdEYtQlgxai1rcC0zajg5dHZzUGpUQ3M3Wm1QUVRYN1ktTzRQbw?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1295,42 +1295,42 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46087.5</v>
+        <v>46087.5107175926</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Luchtvaartbedrijf ASL uit Hasselt evacueert Belgen met privévluchten uit Midden-Oosten: "Situatie verandert permanent" - VRT</t>
+          <t>The Buena Vista Orchestra, Cymande en meer voor Jazz Middelheim - HLN</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Aviation company ASL from Hasselt evacuates Belgians with private flights from the Middle East: "Situation changes permanently" - VRT</t>
+          <t>The Buena Vista Orchestra, Cymande and more for Jazz Middelheim - HLN</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 08:12:09 GMT</t>
+          <t>Sat, 07 Mar 2026 06:02:39 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPTVQxZGFRNVE2TnFOVkMwYkpfdnc3THk2S3BBQ196NnFmRDFuak0tbWluYVhSRGtXcEthUkRjQUw0SlptWHV6a3RIVzNERmtGZEhVbmhOQ3VpaWVtYml3ejBiMnFuSTJUdUUzSTdfU2pMLXh0Y1hGVGJWVGE4dXJZLVhCX3NFN3NHRXVpWE9SekpaWkZvSFJEMXptQ0NISXJXZEpN?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxQaUNjX3RxamZnWmJidF9mcDRLRnZnLWlXMjN0b01GaE11enNPZFkwNno3NU9UbVNNY2FiaWlkZEplQjRqMW1ibFhzQW5UUFhTQmtIOWJlVTdNRDlsOHFPVTFJRjlxT05yQWVKcHV6cDVRamx6U3FaNlM1ZkdOdWpXQjZMM0JUZFByN1NkMDlqZHBpMkk3QzRQYzliSmlHUjNaNUZN?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1354,38 +1354,38 @@
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46087.34177083334</v>
+        <v>46088.25184027778</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Drie verdachten opgepakt voor brute woningoverval in Breezand - rodi.nl</t>
+          <t>Jessy Mackenzie getuigt na MeToo-bom in muziekwereld: “Ik werd als 18-jarige zelf gemanipuleerd” - HLN</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Three suspects arrested for brutal home invasion in Breezand - rodi.nl</t>
+          <t>Jessy Mackenzie testifies after MeToo bomb in the music world: “I was manipulated as an 18-year-old” - HLN</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 12:34:22 GMT</t>
+          <t>Fri, 06 Mar 2026 13:05:26 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOX2Z6Y1lGOGNaMi1Db21SeWdLS1hGOWRidDB0aVJTd3JZNzZPRVJQb2dYN2ttcUNreFROTFZiZkdiaGtoYXZlUS1Ea0hqbWJFRzZLSE1ma1hwS0E1SWRpRGlSN0haR19HSWkxcHZPdzRCREVmUVZsTF9EV2VOZ29maU8wNm9TcHFmZFJrMGh4anhfSkpYa2drTEt6ZFdRWXRReUdrVk1pZ25UX0xXQXpmWEl2OA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxNbmFXaGpuakhNRHo4c0pwWUNiV2laTWk2V3RSMWlWdXJlTnljZ2dSWnBHOGd1SmlaSnZEV1o0dzBaVUpoMjRWUzRmWnk3MFpyVEhuSzFMX0VYbDNiZkdxTVpnWXNhZVMzb2ZEZExnU1ZKMTkxaTFZcHR5dk94UHJRVXB1U0lEYUoyYTBxR2k5TEd6cmpBZGROcTdoX0owOWNieUtTX0k4WF9La3NWbHNtVU5kRmJVUVAxR0E5Vl9SZGFZc0QwY3Q4N05aQQ?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1409,38 +1409,38 @@
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46087.52386574074</v>
+        <v>46087.54543981481</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Des passants sauvent une personne du canal à Anderlecht - BruxellesToday</t>
+          <t>Stad Brussel lanceert plan tegen straatintimidatie - HLN</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Passersby save a person from the canal in Anderlecht - BruxellesToday</t>
+          <t>City of Brussels launches plan against street intimidation - HLN</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 11:49:32 GMT</t>
+          <t>Fri, 06 Mar 2026 13:58:01 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxNejRST0xJNUQtcHVzOENZSE5LRmJFdDE5bklaWjJPS3NpMDVvVkNJcmJ5eVljR3ltSWVEaGR4bXgzM19FZXc5ZzgtSDAzZ3NRazJIQUE2dkJCRnRVaGhJSDdQcWhIU21XdmhRMlk2ODdQa2NqczVfbmJ2OGw3YnUwa201SUc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxQcmNKSnprMTA5OEpvR0wyVVNTUTY2SnNnQy1pSlhlbGJ5TzNyS0c5bWFoUHk1Wi1BY1BCQTJrc0U1aF9HSFVvVUMzdFpxa09TS0ttc2Z3aFh6X29zdDN2ZDNCYW5nVHd4RGhjTFhvYktGTHNicnZxWGt4MUZtM2s5NTAxLXdEUE1EQUVqY0x1dmY?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1450,7 +1450,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,42 +1460,42 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46087.49273148148</v>
+        <v>46087.58195601852</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Herrmann würdigt zum Weltfrauentag am 8. März das Engagement von Frauen bei der Bayerischen Polizei - aschaffenburg.news</t>
+          <t>Voorwaardelijke celstraf voor zeventiger die zich bijzonder hevig verzette tijdens arrestatie: “Het was een paniekreactie” - HLN</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Herrmann honors the commitment of women in the Bavarian Police on International Women's Day on March 8th - aschaffenburg.news</t>
+          <t>Conditional prison sentence for a man in his seventies who resisted particularly fiercely during arrest: “It was a panic reaction” - HLN</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 11:24:25 GMT</t>
+          <t>Fri, 06 Mar 2026 11:17:36 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOYmk2SzhsLUhkdFEtSE9LMEJFT3FiMGJvdks5dVhQOVRta3YzZUVUektCQWs5Yl9HT3JreUZuSWJTRzg2ZjNxWWEzZktmcDMzUDlnVWNNMGhfb1NhMm9NLWhFVmNPS3lCY2pJNjhJYnVlUEVLd2N5MTBnTDBJZE5NMEtPdHpTek1nNGdFR2NyZWpPTGxJV3NjZFpBWkVGMlp3em50QjFkQ2pmU25UeEs0N3otbE82X0dvWXBLb2VrRFZFNm9rTlZWa2lMeEUyWl84NmNzY2M3SUdWNVdvYW5sUEV3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxOcW9id3phUHdQTDRZcGNGbzVJcG9sSW1YaFNxbDhFRjRwMU5QVjNDZkRGWEotaVRhazBUendYVjk1dTJWNEJFaHFWSWIyMjE0NHBESWZvUWdnS2FxR0hBUlh4dU9iUFZHbUdHeHpuTnJ6Q0pKSHVfcTZBSWlRQUxldTRKQmpoU0VGNW1sUG5Lc3VWQlEzVjZuQkY5b0VGSFk4cThBZ1oyRWhZTUtYSnptQ1dmOThyamRXVVI2aXliSmdJdHVXRVZCOS1DVkFzLWdaVmgteUpoYUFZLS1yNGxURkItWnJwX1BPV1RWaW5tU3Y?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1505,52 +1505,52 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46087.47528935185</v>
+        <v>46087.47055555556</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Polizei sucht nach Zeugen: 34 Jahre alte Frau wird in der Würzburger Straßenbahn verbal bedroht - Mainfranken News</t>
+          <t>Ruim uur file op Antwerpse ring richting Nederland door ongeval in Antwerpen-Oost: twee rijstroken versperd - HLN</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Police are looking for witnesses: 34-year-old woman is verbally threatened on the Würzburg tram - Mainfranken News</t>
+          <t>More than an hour of traffic jam on the Antwerp ring road towards the Netherlands due to an accident in Antwerp East: two lanes blocked - HLN</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 09:33:01 GMT</t>
+          <t>Fri, 06 Mar 2026 14:55:34 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxONlRuRjRFcHlqR2Q5SkJaUUdWcEhsNGFjOUJJRExDOG1adVRqemN2R1hDS3BsTDdYTGpZQmZaYkhaOG9JdXphMk5KVFduTjdfeUtVUzQ3ZXlXeDZrUjdPMDhybHpRVW1jUm4zRWpTcTNxMUwyaE5iSHlybVJaMlpFTndvUFp2QTYydFFyVDRiamNQUVJyc1QxYl9kMUpzUk1oNkx6NndJVDhVNF9xRXVObGd5ZjMtdzljdE02eEdxUHVMOEdmTkVXbWtyU004dw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxQbE5obThYMlQ0M04tMVYtalVRT01mWFJmQUIzYW44WC1PcllxbEJERG9iZ0R3MGR5a2R5QU1FdEMtUjF4NHp6ckd6ODFyNDFpSGVuZ3BXN21XQm9wY0JWczB2MHJPU1d1aEJIR3cyMnlaR0lpaGhBVTNtdnh2MGpqNzhCTkJHdjRUaUNSTTZoNEUzdldjcGFyN25JUlVtdkw1N1NlSk1HY21Sckl2enZOTnctbDF5MDNxMC1Sd1VkRDFBaEpfazNWMmZZRmkxeG1SZ2FEcnFCTUJKdWJIbVE?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1560,52 +1560,52 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46087.39792824074</v>
+        <v>46087.6219212963</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Kreis Würzburg: Betrunkener stürzt mehrfach - Zeugen verhindern Fahrt - inFranken.de</t>
+          <t>Zonen gaan voor Britney Spears zorgen na haar aanhouding voor rijden onder invloed: “Willen haar op het juiste pad zetten” - HLN</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Würzburg district: Drunk man falls several times - witnesses prevent ride - inFranken.de</t>
+          <t>Sons will care for Britney Spears after her arrest for driving under the influence: “We want to put her on the right path” - HLN</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 10:00:00 GMT</t>
+          <t>Fri, 06 Mar 2026 11:53:15 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxPVzJONWxZUFVNZXZIR0FudGxqVnRiQWxRbzdnUTI2WWhjNTdnUmVBR3FPWkp1eWozSGVLVno3RlY3eDkzcDZERjJSZ1BiS19NM1Q0V2swdG1kZEtldTNMdkg3Tzc1T2VhUG91YUdIM0RRbFZxajQ5aGhaNER0b1Bsal80b0NoYUlfVUoyX1VIR01UY0lDai12cTZjTW9Ic2NXRi1rNExLT3VCRUxCWXBnLUxTNGtpZ2xlZTM1QS1EbTFmbjlpaGc40gHHAUFVX3lxTE9XMk41bFlQVU1ldkhHQW50bGpWdGJBbFFvN2dRMjZZaGM1N2dSZUFHcU9aSnV5ajNIZUtWejdGVjd4OTNwNkRGMlJnUGJLX00zVDRXazB0bWRkS2V1M0x2SDdPNzVPZWFQb3VhR0gzRFFsVnFqNDloaFo0RHRvUGxqXzRvQ2hhSV9VSjJfVUhHTVRjSUNqLXZxNmNNb0hzY1dGLWs0TEtPdUJFTEJZcGctTFM0a2lnbGVlMzVBLURtMWZuOWloZzg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxNRnBhLTNhd0R5RW41V1BRdnRWeVVQT1JvblI0enBoR09KcGthSWtWTFFRV3JFS1ZMaWRUN1UwN0JDYzkwMjhFSmxtYXR5RWE2cUZoekVQOVNLVElSRVZacWFRenZkRmJhSTk3NWp5d3NqVTdILU5XNTByaEF1bGk1TjFCYmpFNzNDWjdCLUpxWldqajIzd2VvdkNmd3ZwZFJ2LWtTcXRMcTJ0c084YWMwZ0FkVXB1dkxhWVpWM0JiN0VFOVlkUXZ4RFVlaHl4a0tHT0s0MXMxR1VWSHhrcm41WEZ5VlFDaVhaOFNDczl6WDdEQQ?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1615,52 +1615,52 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46087.41666666666</v>
+        <v>46087.4953125</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Neustadt: Vier Personen bewusstlos in Einfamilienhaus aufgefunden - aschaffenburg.news</t>
+          <t>Exclusive-NATO’s Rutte does not see need to invoke Art. 5 after missile incident - WTAQ</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Neustadt: Four people found unconscious in a single-family home - aschaffenburg.news</t>
+          <t>Exclusive-NATO’s Rutte does not see need to invoke Art. 5 after missile incident - WTAQ</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 10:51:28 GMT</t>
+          <t>Fri, 06 Mar 2026 09:45:20 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPNFE0eTdvUU1yc1V4SW5UVXBUMkxPcnpPelN3d0JGYmhlc3RVcjNGbnJTam42cXRuamtIM3dQOEtzTjBVVzUzS1NGdXRSSVg2bkZJLXRvSFVGRGhGbkJRRjA2VDZjUnNOaTloZWRfOWhRYWYxaG96TGhKR29HSnZaUEpQSkNIR0RmTVNfWk9hMHRDR3EyNkpJSHNKYkJTSksyZktEUThaNzNOUUtyaUVj?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQeE1KT2p0eEJXTmw4TlRFVG9zc0dOZ3FXdEFOLWxTRmdvcWx4bVcwaXVGUXdPdWJoLXB0aGx1VjczNVVEb09xVnhGSHNrampDMkJNc0ZGMDNoVHVzcDdhVHRoQ1pwMXk2TWlqbVE4WHJmWnNOcm82NXVxVDJsMXVHMHpvdnZCdUtyR001cHdfOXB4WUJSa2haRUU0NHZnbnVxeHBNTWNJR1kwNUk?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1670,52 +1670,52 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46087.45240740741</v>
+        <v>46087.40648148148</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Wahlplakat in der Steubenstraße entzündet - aschaffenburg.news</t>
+          <t>She ate 22 meals and walked away without paying. Now a judge has had enough - The Brussels Times</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Election poster lit on Steubenstrasse - aschaffenburg.news</t>
+          <t>She ate 22 meals and walked away without paying. Now a judge has had enough - The Brussels Times</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 11:14:03 GMT</t>
+          <t>Fri, 06 Mar 2026 17:47:08 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxQZTVUWFlCb3VqU3d5aEwySllNbTYyVEdJS09CeXdsSXNpRWd2bXpIdHZDVkhWZkM5UGp5U3VqRUNjWWNOdDk3VmlIb0Zxb1JTNXFEdTNlQnoyM2tuaW5rbW9FV1ZyX1VtM204SjdWOVAyVkJrcnRHVlpBWHZTQTNKbVNycDh1emJKSDZpQ1V2dFRmVERQYjhYeDdtODFJbFVCX0dMU1dsQzUxR2Vha1p6d1FCbUF5ak1ZZlBGQnQyalFMREJI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxPMVFqZzZXako4aVZJUWZ2dk5XanJqakVsX2NIdEYzcTI2YWhwV0hsZE9lUGtZZ3diZndMbTZXc05LNkZSUVJVelF2eGFxSDBSSkpjZmQ4enE3SGNBdDRIT0RrQVBnWVNtYmZQMGtMbGJDbmliUEVWMTJuZWhzdGJuY2xuNEF0Y29NeGRHNDdRQnZnSFBHdXpFd0NKRHdPWU9TSzVURTVrd2YxX2hVVmFRMDFyTWNaa0lj?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1725,52 +1725,52 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46087.46809027778</v>
+        <v>46087.74106481481</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Mit drei Promille am Steuer: Polizei stoppt mehrere berauschte Fahrer - Augsburger Allgemeine</t>
+          <t>Three Polish Armaments Group companies took part in the round-table talks in Brussels - MILMAG</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Driving with a blood alcohol level of three per mille: Police stop several intoxicated drivers - Augsburger Allgemeine</t>
+          <t>Three Polish Armaments Group companies took part in the round-table talks in Brussels - MILMAG</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 11:44:40 GMT</t>
+          <t>Fri, 06 Mar 2026 09:10:30 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxQZ3VfT2V3bXgyVERNTFF5b1pYZGtMdmZvRl9sTy01YnZJVmVCQTN2YWpyRTl3bXNWSVpNTkZyWWdnRE5WNXJhMjBYM3N2X3MxVExMbmVrUm1sbExGdUczUm0xSVgwQU5UTElsTTh4SU9XOFRxT0tHNVcxV25xcy1OaTBueFhXZHFOc2FSem91Y05waXFlWGtYc18zZ0ZHSUtsUFZId3Qzb0hLQ21meDRSUnc1OVJWcER4cWFoWERXZ18?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQbzhFYkd2Z0ZuRElRVVpSa2d5NVFqdFBnZm1td1VyNGZZUGl2bkJzYWxyYVRsWHdzdThYUEE0TUMzS3MtN202X21BeWdlU0t3bFZjOU1ub1Fqb2NhWlFoTHVHYVJYRThwdjBJd2R3ckppOW9oZDQ4MVNmWnF4ZjQ5bnNfOXRBZUpJYW41MjhKSHJnWXhRX2x3MVNVOW02dXpmeHpVNXUwc1p4TDg?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1780,52 +1780,52 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46087.48935185185</v>
+        <v>46087.38229166667</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>20-Jähriger aus Manching ausgeraubt: Kripo ermittelt nach Tat in Zuchering - Pfaffenhofen Today</t>
+          <t>"Je voulais comprendre": 10 ans après les attentats de Bruxelles, une survivante parle au terroriste Mohamed Abrini - VRT</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>20-year-old from Manching robbed: Police investigate the crime in Zuchering - Pfaffenhofen Today</t>
+          <t>“I wanted to understand”: 10 years after the Brussels attacks, a survivor speaks to terrorist Mohamed Abrini - VRT</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 12:49:52 GMT</t>
+          <t>Fri, 06 Mar 2026 16:13:00 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTFAzcVd0aGpEd3UwTTZUdUZpdElqRlVTRUZUYWJBWXVMU0UyZVZRSy14SnEwWXdWYzhObFk4bkZaNmdvcmlaVS14N2JlZThieVlfMFpxSmhFTHE3a1RWLUJ5b0lhQkNSQ3hxYVE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOLTZvQm0wdDdNTDFvb0VWRlloZzNJQVdpSHlJdi1ILXJlTUYzSUlRT1Y0NkJWX2Nfa1ZGM21TZUdGZEZrbERSZDAxQ3JQd1dzcm9hTVpwdlVqX2RUNndfNVVjUlJ1X3AyRmFtdHdpWFltX1RnenFGMWFxTWNyOHhreDJHOFN1dWsyNWFFYjBMWGh0X1VPN1hRRU5WVU9XQzJQZHVmVw?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1835,52 +1835,52 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46087.53462962963</v>
+        <v>46087.67569444444</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>E-Bike-Fahrer kreuzt Straße und verursacht Unfall mit Motorrad - Augsburger Allgemeine</t>
+          <t>Coup de couteau dans une mosquée en Allemagne, le suspect recherché - 7sur7.be</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>E-bike driver crosses street and causes accident with motorcycle - Augsburger Allgemeine</t>
+          <t>Stabbing in a mosque in Germany, the suspect sought - 7sur7.be</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 10:02:28 GMT</t>
+          <t>Fri, 06 Mar 2026 17:20:00 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxNV2R0NnFpN0VnRG9YVFFLYXY5b1F0TzcxdlVvQ19DaW9BRFJaUVpDdXdtNkhPVnJRN21rVTRTb1JLamZNU1VFNlFVNTRQNWYtZXNzSFV1ei1La29WOU5lbW5oQ1pIOEJJLUlEMjRLakppNzJUbjlsdkNmdVlrcHlQUmVOd0tNU1ZHd3E2T3Y5bGRUZjZzbVR4NEJ4dVpQSTdoamtIYXlQNGlWVlB2eGl3SU5oeDdkdG5NMkNj?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQNnJrTVdzeThmbEJXY3NiWURHTHAxa0oySHBHdXFXYkJ0VkNyLXNWVWJZZkM3bW9Dc055NTFyN0F4dlpxWklGUk5OZWI1SnFFUldQNV83aTZacTRGWDdTOHpoS3RSaGRpRUcxcnVoNHFJWUhuLXVqWFczQ0ppR0h1M1dtMWRUdXVtekFZeFgzd3k3aFVTcS1HOG5JS0w0OFNpM0RoejREZi0yRjJ2eXNn?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1890,52 +1890,52 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46087.41837962963</v>
+        <v>46087.72222222222</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Village Ingolstadt (fallback)</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Pioneering Ingolstadt coach Sabrina Wittmann signs new deal - Bulinews</t>
+          <t>Prix ​​du gaz record en Europe suite à l'agression israélo-américaine contre l'Iran - www.saba.ye</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Pioneering Ingolstadt coach Sabrina Wittmann signs new deal - Bulinews</t>
+          <t>Record gas prices in Europe following Israeli-American aggression against Iran - www.saba.ye</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 13:32:00 GMT</t>
+          <t>Fri, 06 Mar 2026 08:15:42 GMT</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxPY2VLWkxyVmV0aUdUdm0tUU1iNS1uUmxFVVJyT1J5dGlhaEttbjd0UTVZUWdUbjdsX1FDZ3NGak12T25VM2lyenQzQ2kzTTJCc043YWF3cmotQTNkOGh1T0xYNkNuU0F0dUw1V3kzcGtoZWRWN3hQbDRpal85bm1nTVBUbms2b0E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiT0FVX3lxTFBweUpxS1RKamU0QUZia2tBNXV6dnQ0ODBsOWlBcHJNZzZvV1FGX2tKUWZoQUYtVE9MUkpEcTlDMGZoTGpyc19ZQ0pCekFSS3M?oc=5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1945,52 +1945,52 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K28" s="1" t="n">
-        <v>46087.56388888889</v>
+        <v>46087.34423611111</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Village Ingolstadt (fallback)</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Audi Stops Accepting A8 Orders After Chasing BMW And Mercedes For 37 Years - Auto Spies</t>
+          <t>Hammam de Schaerbeek : Comment un simple conflit de voisinage a viré au procès pour meurtre - Bladi.net</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Audi Stops Accepting A8 Orders After Chasing BMW And Mercedes For 37 Years - Auto Spies</t>
+          <t>Schaerbeek hammam: How a simple neighborhood conflict turned into a murder trial - Bladi.net</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 13:22:17 GMT</t>
+          <t>Fri, 06 Mar 2026 12:00:00 GMT</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTE51SklIQ2xIOVZJekNkaGhrekVRdS04MVZfVWpwdnlvZmxYSThZMXYxcUNfeG1YVHJKa203bXFHejFYQ01PYll5T001TUJ3Sl84dW9UOWxlaDBHamhPZUJ4QXNKeGVKU0hqT01XUFpn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQWnFXYmRyakhQdVhWTnJZUXFqcWhNanNPeHQ4MGZpQnk4YVlabFRzT0l2Z1Q3X1JYNkt4X0hFYXJoekFIRUJCMHZVS3pNeV9HU2s2NGVEUTNuV3Y5M3o5RjR1allhTjFiNUFlcVZvWWdLRTdlQnpxX2ZCOFJiYkZuRXJER2JuOHVEVzJEVEJ3MDBPdw?oc=5</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2000,52 +2000,52 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K29" s="1" t="n">
-        <v>46087.5571412037</v>
+        <v>46087.5</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Claim that Kildare-based company is engaging in oil price gouging - Kildare Now</t>
+          <t>Luchtvaartbedrijf ASL uit Hasselt evacueert Belgen met privévluchten uit Midden-Oosten: "Situatie verandert permanent" - VRT</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Claim that Kildare-based company is engaging in oil price gouging - Kildare Now</t>
+          <t>Aviation company ASL from Hasselt evacuates Belgians with private flights from the Middle East: "Situation changes permanently" - VRT</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 11:05:00 GMT</t>
+          <t>Fri, 06 Mar 2026 08:12:09 GMT</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNaUxOb3Q2emczcGFQbXpaSnBRUGhORW5jUjgxRVlYODlEVDNKU0hmMG00ck5VcC13QklvUjY3cldiSzY0czJaNk1JZW16LVBBMFhaS2d0ZTM4U2tDTnlnaXRfNXRZSUFjZ1pwS05VeDRSN1RMUzBNR1B4QVk1Vk1pVzUzcXE1ek1aTkJRSkJJTEFuOUdyMkUzdjd6LUY4TFhrb21Jc3dnVTVEOXFfYkFLekdLUm9pQl9TM3BZcldB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPTVQxZGFRNVE2TnFOVkMwYkpfdnc3THk2S3BBQ196NnFmRDFuak0tbWluYVhSRGtXcEthUkRjQUw0SlptWHV6a3RIVzNERmtGZEhVbmhOQ3VpaWVtYml3ejBiMnFuSTJUdUUzSTdfU2pMLXh0Y1hGVGJWVGE4dXJZLVhCX3NFN3NHRXVpWE9SekpaWkZvSFJEMXptQ0NISXJXZEpN?oc=5</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2055,52 +2055,52 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K30" s="1" t="n">
-        <v>46087.46180555555</v>
+        <v>46087.34177083334</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Gardaí in Kildare make urgent appeal for information on missing teenager (14) - The Irish Independent</t>
+          <t>Meer dan 400 leerlingen van basisschool in Rapertingen even geëvacueerd door gasgeur, blijkt vals alarm - VRT</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Gardaí in Kildare make urgent appeal for information on missing teenager (14) - The Irish Independent</t>
+          <t>More than 400 pupils from primary school in Rapertingen briefly evacuated due to the smell of gas, turns out to be a false alarm - VRT</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 09:58:47 GMT</t>
+          <t>Fri, 06 Mar 2026 15:16:55 GMT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxNTXktWTNyZnoyVVhOZm9BTTlGa0RsbDBFRFZ6cDJMbDRKQXVqTkhnNVM1ZDlEeEFlXy1uQWZmNVJlUTNSQWl4Yktfa1NMbS1zM0FrX2dTTnVOME9vYWFja1BuTWxpVEwzZ1hoWmtoWjJOcGJFZ1l0QzhFUzktRDNNRi05ZjQtd2RQUS16YWdwNUFqa0lKcUJGaDgwNXNqMEpaa21ZQ0Qwc3hKampDRkhlT0tFSlR3VWRIQWdaZ2huV0VMMERoWWdtakc2bGEyRU1pZE9LZlVfVGthUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxNT0E0aEQ5a0V2MWRMWjB0WllKZThQcHBySGhyMG1yLVltNU43eWRaRTdHTUdsODluYVFXaUJ0Qnc1SU1haDdSQ2h5ZFpQUEtlNFFtdlNwRDdQbzM3MFVqXzBacXlfTWp0REpKMFBtSk9SeWxsUGl6dzEyRV9JNmIwUTFiMA?oc=5</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2110,52 +2110,52 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K31" s="1" t="n">
-        <v>46087.41582175926</v>
+        <v>46087.63674768519</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Kildare eateries win big at regional restaurant awards - kildare-nationalist.ie</t>
+          <t>Drie verdachten opgepakt voor brute woningoverval in Breezand - rodi.nl</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Kildare eateries win big at regional restaurant awards - kildare-nationalist.ie</t>
+          <t>Three suspects arrested for brutal home invasion in Breezand - rodi.nl</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 12:31:20 GMT</t>
+          <t>Fri, 06 Mar 2026 12:34:22 GMT</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxQQ1BUeG9EdGdfdktIMXZwX2RXMEVPZ1YwMVB6MG8wRFZ3b1NObEJzT3dZNFI0aHVuQ3QxSGdZYmdlWHRXTDVLdjRnMWF6N0ZZTEF5T2h1TlY1LXdyeHdYdTdPOTVEQzBmNkFzczZib0t1bC1uWVltMUNGaHNMdmdnc3lhZ2N1NTF0Y3NUZEVyWXFqdS1DX0xzZ0FjVVZnVkRvU0F1a2JpZ1dkZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOX2Z6Y1lGOGNaMi1Db21SeWdLS1hGOWRidDB0aVJTd3JZNzZPRVJQb2dYN2ttcUNreFROTFZiZkdiaGtoYXZlUS1Ea0hqbWJFRzZLSE1ma1hwS0E1SWRpRGlSN0haR19HSWkxcHZPdzRCREVmUVZsTF9EV2VOZ29maU8wNm9TcHFmZFJrMGh4anhfSkpYa2drTEt6ZFdRWXRReUdrVk1pZ25UX0xXQXpmWEl2OA?oc=5</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2165,52 +2165,52 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K32" s="1" t="n">
-        <v>46087.52175925926</v>
+        <v>46087.52386574074</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Maasmechelen French</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Nearly 200 apartments get green light beside Canal in Kildare - Kildare Now</t>
+          <t>Des passants sauvent une personne du canal à Anderlecht - BruxellesToday</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Nearly 200 apartments get green light beside Canal in Kildare - Kildare Now</t>
+          <t>Passersby save a person from the canal in Anderlecht - BruxellesToday</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 11:47:00 GMT</t>
+          <t>Fri, 06 Mar 2026 11:49:32 GMT</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQdTUwNVF3aUFxSFgweWNwU2pWR2J2YTFHZjVRT0x3b3pvcnVCUWYwVFZUS3BkT2Vpdi11WERSQm5yRkJONjNnYlVmbnNOVEE2UzJUM0lnaG5TRERCRkRSbzNOUVpfU3JMb1lqRUtVU0tkWlJ1X3ZTZTdLdEdoZ3o1OHVJbFVfMFh4c3ByZWZ1c09HU1lJNXdJd05lWVZCM3dTckFnYm1SUzBERlN5clRxRXFGcVJINy0x?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxNejRST0xJNUQtcHVzOENZSE5LRmJFdDE5bklaWjJPS3NpMDVvVkNJcmJ5eVljR3ltSWVEaGR4bXgzM19FZXc5ZzgtSDAzZ3NRazJIQUE2dkJCRnRVaGhJSDdQcWhIU21XdmhRMlk2ODdQa2NqczVfbmJ2OGw3YnUwa201SUc?oc=5</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2220,52 +2220,52 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K33" s="1" t="n">
-        <v>46087.49097222222</v>
+        <v>46087.49273148148</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>LATEST: Meet the Kildare firefighter balancing 'dream job' and life as a young dad - Kildare Now</t>
+          <t>Smart combinations of antibiotics can slow down resistance - Medical Xpress</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>LATEST: Meet the Kildare firefighter balancing 'dream job' and life as a young dad - Kildare Now</t>
+          <t>Smart combinations of antibiotics can slow down resistance - Medical Xpress</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 11:21:00 GMT</t>
+          <t>Fri, 06 Mar 2026 16:00:02 GMT</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxOSEtpd3ZYUEJvdHc1YU9IOGxoRUZhS21XUkxXcGg3cVpfUnlqZ3RmdnZZYzE3M3hTNW9NYWI1MVFJZ3k1M0R2QV82RzlaQUtkOG82eTRoYWc1Q25fUUxzLVIwMWtZQUtHQ2kzN1ByOXY5WkZ1eEo0R2hwWTBWZWIzZzNhcm84TTNzVHNLN2VDaFRuRXhocGpienZEQkpIX3lQLWRXWWtKMnhNQXFJdHg4blZ5NFNFeXlwdHRhcXBzMHN1M1ZJdnNncU1WMzdUVDVW?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxQN0NqRzNUZDJGRzZaY0dJT3AyRTZ2aC13M3FMTGVRNXFlcklpeVNNdFlyQ0hLempqVFNyR2R1bUZtYk9lVDg5NjlWeUVLSlB1ZGhnSmFqOWtDRUhzQVZPcmlKU2stY3hHcWRlX2VETXI3djRtS2RVU0JuUFdmNjhYQWYxcXdXNUM2bFRHWDVB?oc=5</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2289,38 +2289,38 @@
         </is>
       </c>
       <c r="K34" s="1" t="n">
-        <v>46087.47291666667</v>
+        <v>46087.66668981482</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Kildare-based art group expresses delight as extension granted to free exhibition - Kildare Now</t>
+          <t>New Flemish FTI technology festival spread across eight cities this autumn - belganewsagency.eu</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Kildare-based art group expresses delight as extension granted to free exhibition - Kildare Now</t>
+          <t>New Flemish FTI technology festival spread across eight cities this autumn - belganewsagency.eu</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 12:35:00 GMT</t>
+          <t>Fri, 06 Mar 2026 15:30:00 GMT</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxPUGNhM2lnTlRKYzVpLVZ2U25mMnVFOTRudVJJZkFzSm9KMU9YWk5semg4U0FGT3VGd0NuTWU4dUxfNlFOOGFSS0QtWjNlS0x5Zk1GUWVCWFdoUjlYRkU2cEtQcmNSOHRsT1gyUGVCT2dkdEs2c2ZUSWZIR3pyNXJVamFXdm5TVkh2N00xVmpqWkF3OHl6LXNEOS03WThVZjMzLTUzT0JnRlNTREhzeXNFWFJHZWs3Y2RuV0FPeEs4TDhkakF6SUZIMTZaMGtVOFZRRjk0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOMUJHVWdLWHlaeHF0MVZZVWJpcXdpMS1McTg3X2diTGlxUmh6RG1ISHdWclZhOEIyWHZkMHQxMnpZbDZBa1VmT1BDRlhZNG9fb1BfRUVDc29GNkpCb2NtZ21yajQwRGNPTTV2eTd4UzAyWmhOSllmU2RnWXREN0VWcDUzYlNENGVkRWRhd09zTDExeEM0V3g1cGdjVEc2WGpmZkFuWURHY1M?oc=5</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2344,38 +2344,38 @@
         </is>
       </c>
       <c r="K35" s="1" t="n">
-        <v>46087.52430555555</v>
+        <v>46087.64583333334</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>'Transformative': Praise heaped on blueprint for this Kildare town's future - Kildare Now</t>
+          <t>Why PSG's victory over Marseille will send shock waves across Europe? - MSN</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>'Transformative': Praise heaped on blueprint for this Kildare town's future - Kildare Now</t>
+          <t>Why PSG's victory over Marseille will send shock waves across Europe? - MSN</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 14:05:00 GMT</t>
+          <t>Sat, 07 Mar 2026 02:09:59 GMT</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxNYW9uRGIwbkZmVmxiaHc3WVdhbGhhajhheG5HYndpTDNFdE8zNXBiZlMxaTEyZ0w0bG5WWE9DNEMtX1VyNzI5WUpNQUNleENaWUZ3RF9hM3lIeTh6a19tWVg5NHE0dGowaGFkeHZha3pSWTJ4eTFxZ25BZGdXN25uNzFYQm9oZnZ3X3VyQ3ZSZl9FYWsyQ1VCUTdhSWNsMnk3SEVjdS11eVZDWXQwQ0xNbi1UYkhuaHN0QllPNy1VOG9hWWFxam1F?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwNBVV95cUxNWEh6WjI3M0ZIVmJScU91Q1FZMDFpUnluT3RncHRZZlI3VHU0V2tQT1ptZXNERDM4b3JKNm10Y00ydjhGQUc3Q2lpZmllODRDR3lsbGdFSllQcVFBUzV2dU1VRlpRcUgydVJYWGFfNlc2TVRiUEJaRDd1UmdHcWZJZm43TkZNNm5FS18wQm1HaTNJTFI0dVJueUR1N0oyU1FaQndXdzBPVWZIRGFxSDRBLW9rM1htS3ptR0ZHcnNNaHlSaWw5aEUtbkQxSVA4ZVZUZmdSQU53WFJQejZhWXBlTHNUZ1RqUEtEbm9jWnFEMjcwMklfWVBjSUJscXo4bWVFdWw2UW9ic3lnRWo1YmdwRWtnQURyR0U1QzJQQ0ZUNlhHbEZxMFF3ZlpDOGQ4bFYta3ZQSHJzOUpJTzlPZE1lRkY5NG1vZTFGSTZKb3M0NUpGaFdPRlNFSlVYX3FOUk1pam5QWVVMNkI5bS1yeThrNHVRakItS256ZUE1aWFRYm85dG93b0s1ZG53NG5NQVM4SFk0UVVBYml0TWNBYnBF?oc=5</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2399,38 +2399,38 @@
         </is>
       </c>
       <c r="K36" s="1" t="n">
-        <v>46087.58680555555</v>
+        <v>46088.0902662037</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Kildare man advocates with Taoiseach for Down Syndrome supports - kildare-nationalist.ie</t>
+          <t>41-jährige Frau vermisst – Intensive Suchmaßnahmen – Wer kann Hinweise geben? - Polizei Bayern</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Kildare man advocates with Taoiseach for Down Syndrome supports - kildare-nationalist.ie</t>
+          <t>41-year-old woman missing – Intensive search measures – Who can provide information? - Bavaria Police</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 14:01:23 GMT</t>
+          <t>Fri, 06 Mar 2026 20:49:50 GMT</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQN0Y4a2VwWkJ0RWpuRklobVR5N09zc0czQlQzZmI4MmZ5N0tid1czWkd2QTR0V1RuUklsb2pLMDlPejJZZGpIUG5fUDV4VTJ2RXUyaElxNHZ1b2dlN0pyNU8zcWJKMERRMUdERlB4aTdkbGpHMmI4bHl4SHI3aUhCeVVYbWZUR3hrb0NTMjZEbExyYnp0WGhQRTRhdnVMRzlWaml4dE9ULTBGLXAwblZjZnY4RjhJSk5YajY4?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxOS0RyZmllN3RtZ2ZjaUxROWJxUEhiOFFaeFdGNmp0bm8xS0dsMkJKXzZuaVgxRjYtOVVDNDNaVER4UW5iTzVkeXZQcGx3U2hkUzJ5ZXljRVJjR05JM3czaE1yQXE2cE11YmVrc2NxNTJoNjZacTlqNnZ3QmJDWl9Ud1h3?oc=5</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2440,52 +2440,52 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K37" s="1" t="n">
-        <v>46087.58429398148</v>
+        <v>46087.86793981482</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>High Level City France English (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>("Paris" OR "Île-de-France")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>All the Stars On the Front Row at Paris Fashion Week - vogue.com</t>
+          <t>Einsatz von Polizei und Feuerwehr am Hauptbahnhof in Würzburg: Das steckt dahinter - Main-Post</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>All the Stars On the Front Row at Paris Fashion Week - vogue.com</t>
+          <t>Deployment of the police and fire brigade at the main train station in Würzburg: That's what's behind it - Main-Post</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 14:10:26 GMT</t>
+          <t>Fri, 06 Mar 2026 16:17:08 GMT</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxNY1FpMzZfYjVyc29DRGUxcGN2aHU0aHFOcXR1Yk1iNzBodnJCazJPdlhCcTU4cmdPYmVjSF8zdjhaYURvQVkxa0VXcEFuaUVITktTQVVWaFVwendiaHRORjJrVUdscEdJZTdNSzhFcXhIcDFncWtBMWhJWHlWTnRnblpsa25DcmpTY0E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxNYkdBVUxTOWF6bzYwenRRN01oVXNFNE5DR0hXeVZzalpxOC1tdnM1dG1RT0JZRnFvdDV2QlY2bm84MzZTUWFvR0MzNHBPQ29sN0hZVWlqRjBfTHB0UnBEOTJYaFBieFlyQ3NKYTA5OTVNNzdvV2wzcUhYY1pKTWZWTjFPbHBUY1BucXJzZXo2ZUFYS2pZbmVjWWNVWkZEdTl3S3dRX0VsVkhTVkxpbmVKVkJhN3NGdFF6T2c?oc=5</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2495,52 +2495,52 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>FR:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K38" s="1" t="n">
-        <v>46087.5905787037</v>
+        <v>46087.67856481481</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>High Level City France English (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>("Paris" OR "Île-de-France")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>She had a vision of herself living in Paris. Now this American woman calls it home - AOL.com</t>
+          <t>Urteil in Aschaffenburg: Rocker-Chef mit Drogen versorgt - Polizei hörte mit - main-echo.de</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>She had a vision of herself living in Paris. Now this American woman calls it home - AOL.com</t>
+          <t>Verdict in Aschaffenburg: Rocker boss supplied with drugs - police listened in - main-echo.de</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 10:29:53 GMT</t>
+          <t>Fri, 06 Mar 2026 13:47:00 GMT</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE9GS0tVWXg1d3NuV3VfQTM2eU5hM0JxbFZ4bHBaeng0TFY4UE9seTNYSUhBZzRxNE9HOVQyMjNiampLSFQ4STN2dXd3c0tSWkthb0FyV01RdDZLaEsxQjhsdUVuenMtSUFoaWdjbzdyTzJvbExUbG1pSkRNblhLQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxNSzJoeC04cUhzcjlQam42ejNXZ0MyMnhHT2NDa1hyUElpLTZIVGNjbjhlUUtIZWxMd1ExakF0ZjVoZEVHTGNHOTNFb0FhSHRSNk1RQTc2UlJSQVlNVm1yeXo0ZVd5NkFRQW9sU3JJWlNLa21MSVVkLVlXWlRSaVhqYkpVanZFeVZObkZOYUVXQ2lFRkQ2MFpJVzVWczlPaEs3czlvbVFRUk5BZFV5QnhrNXNBWS1hNTNrTl9uZG4zcXdiYno5T1Nj?oc=5</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2550,52 +2550,52 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>FR:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K39" s="1" t="n">
-        <v>46087.43741898148</v>
+        <v>46087.57430555556</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>High Level City France English (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>("Paris" OR "Île-de-France")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>NBA YoungBoy Pops Out at Paris Fashion Week for Rick Owens FW26 Show - Complex</t>
+          <t>Herrmann würdigt zum Weltfrauentag am 8. März das Engagement von Frauen bei der Bayerischen Polizei - aschaffenburg.news</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>NBA YoungBoy Pops Out at Paris Fashion Week for Rick Owens FW26 Show - Complex</t>
+          <t>Herrmann honors the commitment of women in the Bavarian Police on International Women's Day on March 8th - aschaffenburg.news</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 10:59:13 GMT</t>
+          <t>Fri, 06 Mar 2026 11:24:25 GMT</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOaFZiV0NKYk10emtXdnJlMzI5NXNjT3lvRDBBZnJMQV9yUmxwNFp4TlpYX3JwVEdaUC04dlBIMDVlMGRuOTJnRXEzdlBMYUh6anV4dTcySWxHUEg4bmIxbGg5RV9PZWJaVm10ai1NVmtWZUl6WGVpTkktYXZyWE0tcTN4c2xiN2NMRE1RNHM5TQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOYmk2SzhsLUhkdFEtSE9LMEJFT3FiMGJvdks5dVhQOVRta3YzZUVUektCQWs5Yl9HT3JreUZuSWJTRzg2ZjNxWWEzZktmcDMzUDlnVWNNMGhfb1NhMm9NLWhFVmNPS3lCY2pJNjhJYnVlUEVLd2N5MTBnTDBJZE5NMEtPdHpTek1nNGdFR2NyZWpPTGxJV3NjZFpBWkVGMlp3em50QjFkQ2pmU25UeEs0N3otbE82X0dvWXBLb2VrRFZFNm9rTlZWa2lMeEUyWl84NmNzY2M3SUdWNVdvYW5sUEV3?oc=5</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2605,52 +2605,52 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>FR:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K40" s="1" t="n">
-        <v>46087.45778935185</v>
+        <v>46087.47528935185</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>High Level City France English (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>("Paris" OR "Île-de-France")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>News | Roka targets large-scale operations in Paris and London - CoStar</t>
+          <t>Würzburg: Nach Sprung in den Main, um die Tasche zu retten: Wer zahlt die Kosten für den Einsatz in Würzburg? - Main-Post</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>News | Roka targets large-scale operations in Paris and London - CoStar</t>
+          <t>Würzburg: After jumping into the Main to save the bag: Who pays the costs for the operation in Würzburg? - Main post</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 10:50:23 GMT</t>
+          <t>Fri, 06 Mar 2026 16:00:00 GMT</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxNcDMtLVhaZGIxa3pQVzBPVzhHRFU5dTAyMzE4UnJfR01VX0M4UkM4V19rMVNMLXQ0QVdKM181RGMxUF9sdjl3dGU5M2hwVllfTGJKUXBnMy1QdTFTcS1nQndMZXZtTU4xdDhDVG0wY19TSWZsai00X1VzcTY2bHlISDg5M2VIcElUYUdYckFn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxQdGhFSEw2a0FMcElUSjhVMFlXV1VpbGo3azktMHV5M2dQMnZPVHhCUG5ReE5LQ0lzMVYxX21QdjFIdklrZE9pbzFJNzVsZFpNSl9Pa1lnam1BVHZGQmdpTnBzRkFCQkdCem9TT3lLb1JCVDdBc0I2MnVoaU1rVUc1Rmx1RjMzTXI0WmVHM0NfQk91Q2x5T29VOEVmU0ZBTFRPVmt3ZmdKUVY4SWd5UVJYRXZwM1h0aGhBd3AtanNVcTVTSlA0cTRKSVRCOTBnd19tMkFRYXk4a0NVT00zZVZ3YkZEZ29JWnlCV2RVMFlmV3VpMW9LTnhrR3Zqaw?oc=5</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2660,52 +2660,52 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>FR:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K41" s="1" t="n">
-        <v>46087.45165509259</v>
+        <v>46087.66666666666</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>High Level City France English (fallback)</t>
+          <t>Village Wertheim (fallback)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>("Paris" OR "Île-de-France")</t>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>5 Strange Discoveries Hidden Under the Streets of Paris - WorldAtlas</t>
+          <t>How to survive Daylight Saving Time: FIU sleep expert shares tips before we spring forward - Florida International University</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>5 Strange Discoveries Hidden Under the Streets of Paris - WorldAtlas</t>
+          <t>How to survive Daylight Saving Time: FIU sleep expert shares tips before we spring forward - Florida International University</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 10:30:00 GMT</t>
+          <t>Fri, 06 Mar 2026 16:33:00 GMT</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxPZVhmeC1BdllfS3Y4T291RVNabU5mSjlKaTl5MFg4LUt1STVSVFBkR01ldnBSNjdpSC1MNU8yRWNyTnNHdHNqOHN1eFlydThxSFE2VjJnZmJvYzZkSnBzXy1VUzBzalpoNDdqeGZIUmNpSHBVdXYtQTBrWDE1MVZuNXNHWllpMHNjNVh5dUh3bEY2dkhkaEl4cXdjQ09IQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOd185VUQzWXVaZms2Q0E5OVVkaDVLOExlUHNuVGQ5al9XMnJDWE5pYnp3NHdzTFpiT0ZPOTZ1WGs1ZEdUaU5xa1d5eElNVWNFamdzTDhiM0xuZ20yN0lLYWc2b3M5UXo3dG1HRTRKSUNWQTFKMEFwMnJneFdjVUowOUc5c3M5cFBIcGh1bVFNNmlySUdZVmZ3SWFHdzFMTm40RnB4N2JlOFVhRXYxb0dNalRRNDRNQQ?oc=5</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2720,47 +2720,47 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>FR:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K42" s="1" t="n">
-        <v>46087.4375</v>
+        <v>46087.68958333333</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>High Level City France English (fallback)</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>("Paris" OR "Île-de-France")</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Mbappé’s Paris trip raises hope – but the clock is ticking - Diario AS</t>
+          <t>Mit drei Promille am Steuer: Polizei stoppt mehrere berauschte Fahrer - Augsburger Allgemeine</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Mbappé’s Paris trip raises hope – but the clock is ticking - Diario AS</t>
+          <t>Driving with a blood alcohol level of three per mille: Police stop several intoxicated drivers - Augsburger Allgemeine</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 09:57:13 GMT</t>
+          <t>Fri, 06 Mar 2026 11:44:40 GMT</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPbngtTVI5TUNLdjZsM3JVYUhaTy15cjZ2S3Zvc3J5cU85ZXRzbWRNM0w0OG4xQkpqNURTRllOYnRqeTZ3ZXQ4Z3RlVUNObEwzdDlSN1FNLWVBbkhfOGdxY0VzWFpTSWItSmZhUVBEZjlUdjI2eEtFdUVZRkVTMTV3M2lHYUdmblJyRmptYklNdnA3Yi1DYWfSAaoBQVVfeXFMTVJaY0dpNmdqUmE2amhhazNwRHlKcXliNlF6MDB2dXpqMkpQNVJ6UENpVzFQQ0t5cGVIcVgyLWlfSkZyZlJkQkFrV1VNenpRVnRYQjJxckRHYlZidERlWDNFM0M5V0dSVzdOTkUyV2d1Y2tjOTh2SWE3cExzTWpiMF92T2o5OEpYVGpvakw3T2VNaUZ0YW9QUzRXYURIM1JWVGU0VG1hTTUwWUE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxQZ3VfT2V3bXgyVERNTFF5b1pYZGtMdmZvRl9sTy01YnZJVmVCQTN2YWpyRTl3bXNWSVpNTkZyWWdnRE5WNXJhMjBYM3N2X3MxVExMbmVrUm1sbExGdUczUm0xSVgwQU5UTElsTTh4SU9XOFRxT0tHNVcxV25xcy1OaTBueFhXZHFOc2FSem91Y05waXFlWGtYc18zZ0ZHSUtsUFZId3Qzb0hLQ21meDRSUnc1OVJWcER4cWFoWERXZ18?oc=5</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2770,52 +2770,52 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>FR:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K43" s="1" t="n">
-        <v>46087.41473379629</v>
+        <v>46087.48935185185</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>High Level City France English (fallback)</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>("Paris" OR "Île-de-France")</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Paris’ Tour Montparnasse Observatory to Close in March 2026 as Redevelopment Plans Move Forward - ArchDaily</t>
+          <t>E-Bike-Fahrer kreuzt Straße und verursacht Unfall mit Motorrad - Augsburger Allgemeine</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Paris’ Tour Montparnasse Observatory to Close in March 2026 as Redevelopment Plans Move Forward - ArchDaily</t>
+          <t>E-bike driver crosses street and causes accident with motorcycle - Augsburger Allgemeine</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 11:30:00 GMT</t>
+          <t>Fri, 06 Mar 2026 10:02:28 GMT</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxOQkozVlM1c0RqM1JYZnNNZms5cUhpUmxUWUtwMjJQdklWc196ckVmcTY3XzJMM21lRWZGcTRqM1JqODQ4NHl2VjBHc3Rod2YzNHR5XzRGTlNVMnVlNHlUN1VrSFNzNFEtdG9PNEU4Nlc5ZHN3NzMtV2hCTDczN0xXM004NTh0cXE0d0RVbEFPMzRhVnc5dWpwQTV3Z3JqNEJ1X280dDZKVXZNTktJTzJ3S2NTOUVqSEZGZE96Q05PMHlVbDVkTWpB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxNV2R0NnFpN0VnRG9YVFFLYXY5b1F0TzcxdlVvQ19DaW9BRFJaUVpDdXdtNkhPVnJRN21rVTRTb1JLamZNU1VFNlFVNTRQNWYtZXNzSFV1ei1La29WOU5lbW5oQ1pIOEJJLUlEMjRLakppNzJUbjlsdkNmdVlrcHlQUmVOd0tNU1ZHd3E2T3Y5bGRUZjZzbVR4NEJ4dVpQSTdoamtIYXlQNGlWVlB2eGl3SU5oeDdkdG5NMkNj?oc=5</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2825,52 +2825,52 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>FR:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K44" s="1" t="n">
-        <v>46087.47916666666</v>
+        <v>46087.41837962963</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>High Level City France English (fallback)</t>
+          <t>Village Ingolstadt (fallback)</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>("Paris" OR "Île-de-France")</t>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>UAE Team Emirates-XRG all set for double-header of Paris-Nice and Tirreno-Adriatico - UAE Team Emirates</t>
+          <t>Official | Ingolstadt confirm contract extension for trailblazing and record-nearing female head coach Sabrina Wittmann - Get German Football News</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>UAE Team Emirates-XRG all set for double-header of Paris-Nice and Tirreno-Adriatico - UAE Team Emirates</t>
+          <t>Official | Ingolstadt confirm contract extension for trailblazing and record-nearing female head coach Sabrina Wittmann - Get German Football News</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 12:03:38 GMT</t>
+          <t>Fri, 06 Mar 2026 19:26:19 GMT</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPTXJBUmpqUlQ3VEJtbmhUajZrMWNFU3BIVVhIdmJPRERsb0NvdzN6YjdNVktGOXotRG5JcVVLTWdxb3p4RDF5SGNzc0VrNmstSlZ6a19XZXBieXNuUTFuc0tuakVDWUVjQU5lZEhNZmlrZmxfUjdIUVZaSmxDZy1Cb2pBSnBrb09pWDZSRklMTExYcWR4dzhOa3JtdElkMkw5dU1F?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE9fcm43TkxTUkNUc0VMQVF3ajc3WE52bmlvMHlvcVdtM19sMkFhS25NaTV3anQ3djBXaVpXQnhBaHp5MXdUYUIzNk9QaVd1Yy01TzE1NFBSbzFmdFlCaUp0X2RYellyaklRVGRvUHpZaXd5WGhKVm1xRUY0RnE?oc=5</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2885,47 +2885,47 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>FR:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K45" s="1" t="n">
-        <v>46087.50252314815</v>
+        <v>46087.80994212963</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>High Level City France English (fallback)</t>
+          <t>Village Ingolstadt (fallback)</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>("Paris" OR "Île-de-France")</t>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>COSRX and Courrèges Reunite Backstage at Paris Fashion Week FW26, Introducing a Limited-Edition Collaboration Kit | Corporate - EQS News</t>
+          <t>Trailblazer Wittmann extends deal as first woman coach in German men's football | Football News - Hindustan Times</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>COSRX and Courrèges Reunite Backstage at Paris Fashion Week FW26, Introducing a Limited-Edition Collaboration Kit | Corporate - EQS News</t>
+          <t>Trailblazer Wittmann extends deal as first woman coach in German men's football | Football News - Hindustan Times</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 10:06:21 GMT</t>
+          <t>Fri, 06 Mar 2026 20:36:14 GMT</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowJBVV95cUxPZU8yblQ0TVRHMm5NQ1ZDbThDMk9YZzZhRTh2VmtFWktKbkt2cTd4V1BZLXdqdmhoTk9qWU9ZN2V2amdVdVloUTJDTzNQcFh2NFVFN19Hb00zaTc0SVV1RjBBT3B2U1JyWVRSMXI1ZkVjN1kzVDkyRkF0dHptZ21YUDVRLWRfRXg2UGFhYU9mVmZ3STE1MHRvUGM2ekdSUzVyVFNUYjRuTWx6SW96UG92N0F0TGNmOWwwMFktbXkyMlB5bTA3M3NMbVQ4N2pteElLOUswY284bjJxbVVXSUNCeG9qYW02T0pIel9CUFRVOWVaUjE2QnlkS3h2UzRnRnVjbWhRM2ktSnRPbV9BbnZnbXhMTVVaalZ3bHNfTjNhU002NkU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5gFBVV95cUxOeVh5amxSUWwtWFg0clhDNHhpTXBZeENHempuM3F0MWZjSWROVHJNX3VYSlBjYURrTk9vVUh4NjNyckFQWm1rakMyUWc1Sl9jRmllSmVDd0ZOdlp3TC1ET1AxYjN2dG5xeE9RdUdfTGNpUGVCNXNzRTU3cWVEVEppQmZTcU85R3E2WmYySGhjanB3SlZZajEzaTZtLVFDblJodTB5TFhNb3l1T2hZaExiM3pRSjM1LXZqbTVxUmJiTzcwQ29WWkhValBUNmhwNFd2RXJNN1hPZy04VmJ3TG51OEotODFDUdIB5gFBVV95cUxOeVh5amxSUWwtWFg0clhDNHhpTXBZeENHempuM3F0MWZjSWROVHJNX3VYSlBjYURrTk9vVUh4NjNyckFQWm1rakMyUWc1Sl9jRmllSmVDd0ZOdlp3TC1ET1AxYjN2dG5xeE9RdUdfTGNpUGVCNXNzRTU3cWVEVEppQmZTcU85R3E2WmYySGhjanB3SlZZajEzaTZtLVFDblJodTB5TFhNb3l1T2hZaExiM3pRSjM1LXZqbTVxUmJiTzcwQ29WWkhValBUNmhwNFd2RXJNN1hPZy04VmJ3TG51OEotODFDUQ?oc=5</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2940,47 +2940,47 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>FR:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K46" s="1" t="n">
-        <v>46087.42107638889</v>
+        <v>46087.85849537037</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>High Level City France English (fallback)</t>
+          <t>Local Town La Vallee French</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>("Paris" OR "Île-de-France")</t>
+          <t>("Serris" OR "Chessy" OR "Bailly-Romainvilliers" OR "Magny-le-Hongre" OR "Seine-et-Marne") AND (manifestation OR "alerte à la bombe" OR "colis suspect" OR bombe OR fusillade OR couteau OR protestation OR évacuation OR attentat OR "opération de police")</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Paris Jackson embraces boho-chic in sheer dress - HELLO! Magazine</t>
+          <t>Seine-et-Marne. « On est passé à côté du drame absolu ! » : un homme attaqué au couteau dans une laverie - Actu.fr</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Paris Jackson embraces boho-chic in sheer dress - HELLO! Magazine</t>
+          <t>Seine-et-Marne. “We missed the absolute drama! »: a man attacked with a knife in a laundromat - Actu.fr</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 12:36:46 GMT</t>
+          <t>Fri, 06 Mar 2026 14:52:43 GMT</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxNVjJrbndndTJfcHpEdHNqOUdvVWRuWl9kWXM5SU1YdmQ0eXlxQm04Q1dVOGplV0RtUW1lVlJmekFkcEZGOHFkUTlXbWhMdFJMM0tEa25aUll3Y0xSVktINks2bmprc0hyZkdzYnB5OVdQWlQ3WF8zRzA5S3FIWVUtcXFJT0wyX01NZlRpNjBiSEJUUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxNZ2N0TDJLZmNLN0kwdkc1aXktYk1OeWlYR1ZmVWR6c3Jxa0F1dzZGZ3dmY2xLVURldFk4cmwtY3RiU255c0VHM0V5SEoxZ0F4dkxhRlJXNHFYRVphM2MwUEZCT19OSElvQjJxRlN4Y2JIRFJkZ3VNUU4yZVZJMXdlaWtpRW90Z1RQRTMwQnVybzlyTmdBY1NoSEVTTHVXdi1OVjlzQlFLVHo3T1k0VFc4ZWt3VnE0ZEtldXluT0dWeXc3VjQtRVVHS0VBeXdJc2FGVmhXZHlad2tzcXRuLXplMllJdl9ONFE?oc=5</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2990,7 +2990,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3000,42 +3000,42 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>FR:en</t>
+          <t>FR:fr</t>
         </is>
       </c>
       <c r="K47" s="1" t="n">
-        <v>46087.52553240741</v>
+        <v>46087.61994212963</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>High Level City France English (fallback)</t>
+          <t>Village La Vallee (fallback)</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>("Paris" OR "Île-de-France")</t>
+          <t>("La Vallee Village" OR "La Vallée Village" OR "Serris" OR "Chessy") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>I Went Shopping at the Paris Flea Markets with Top Designers. Here’s What They Taught Me - AOL.com</t>
+          <t>Crufts 2026 winners so far as competition nears end of second day - Birmingham Live</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>I Went Shopping at the Paris Flea Markets with Top Designers. Here’s What They Taught Me - AOL.com</t>
+          <t>Crufts 2026 winners so far as competition nears end of second day - Birmingham Live</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 13:22:24 GMT</t>
+          <t>Fri, 06 Mar 2026 19:21:00 GMT</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQU3RZT3NGYkgxNVROaFdPU1Zsa2J4WGxJUU9sUjR5RHBSTHI1YWJzWnllWWFaQ0ZTWnJNVmFRMFVSMUtNOEh5LTRTRjBSNlFCeFF1WUZMc2U4Y05GYWtMTlZPX19xYk5mUndmalRtWkU3Q2NTOVlpUEcycURJcDd4YWJn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxOMkZLRmFJZzVEVk8yUTF1UVZMZE94ZHExTDV3MkZqR3NQemdEYzFrbDRnNENfbXB6VUFTWUE5QXJmczllT3dJM1JSU1NVN1EtVHdkWG43bjU5aGV0enVIVDdGYXh5dzFlYUxYX0ZTcnJqUUxGaTNZX2JzaWhGM0NzOXlCN1ExbmZzajZvVHdZVjNHN1JBeWhNZtIBngFBVV95cUxPakJXanpjMmpLOGpIclh5TzhLM2JEdVFjZW1xMmhnOXZqRHhXTFZ6azZnMjFhWmw1SnlUeGhyT0l1S3g1QThhbWpQUnFzd1BDTlVrWjZTRjhUNngwUzlFR0NxNWNvdWJ0NnVuT1g3M2VhWlhUNjRONWxPVTB0WVZ1LWhHWFhqNXJaZ2NrR2t6dnotZEJCcmJGWWR5cDZYUQ?oc=5</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3050,47 +3050,47 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>FR:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K48" s="1" t="n">
-        <v>46087.55722222223</v>
+        <v>46087.80625</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>High Level City France English (fallback)</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>("Paris" OR "Île-de-France")</t>
+          <t>("Milano" OR "Bologna") AND ("minaccia bomba" OR "pacco sospetto" OR "pacco esplosivo" OR sparatoria OR accoltellamento OR "attentato" OR "operazione di polizia" OR esplosione OR evacuazione) AND -Olimpiadi AND -pattinaggio AND -sci AND -Cortina AND -calcio AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>The Best Backstage Photos From the Fall 2026 Shows in Paris - vogue.com</t>
+          <t>Allarme bomba al tribunale di Milano, evacuazione in corso da Palazzo di Giustizia. Più chiamate arrivate in Questura - L'Espresso</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>The Best Backstage Photos From the Fall 2026 Shows in Paris - vogue.com</t>
+          <t>Bomb alert at the Milan courthouse, evacuation underway from the Palace of Justice. More calls arrived at the police station - L'Espresso</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 09:46:04 GMT</t>
+          <t>Fri, 06 Mar 2026 21:22:30 GMT</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPTTlqZjVILWlLa0I1aDJyTGNhNEtXV2VRM2NDczFIalFVcG1zY3JDZ0lJa3V2SGtiN3o1UmtSbG5RYXhJT3VoWTlubnlCbmV3UzdZbW5kY0RBcm1wd2dVemFZS1VWd3FNOWpZZ01TTndpTlF2cWtJV25sSHVNanQ1cFgzcGpRX0tGTHVfNnNDck14RHgwUUE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxPUWtxbVlUUTl4OTZaalJjWG1KcGNyM0JkRzRYTDRrSk9vc05aclF3NWJIaUNsVjFBV2F5RVczNjktOFZiTkhqS2tPcEtVOFdmdjludjdzakxfTXFETlhmSlhSQmR2ZW1BUlBUMmE5Ukhmb3lyeVZsd25KWFVQVlA1RElma3o?oc=5</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -3100,52 +3100,52 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>FR:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K49" s="1" t="n">
-        <v>46087.40699074074</v>
+        <v>46087.890625</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>High Level City France English (fallback)</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>("Paris" OR "Île-de-France")</t>
+          <t>("Milano" OR "Bologna") AND ("minaccia bomba" OR "pacco sospetto" OR "pacco esplosivo" OR sparatoria OR accoltellamento OR "attentato" OR "operazione di polizia" OR esplosione OR evacuazione) AND -Olimpiadi AND -pattinaggio AND -sci AND -Cortina AND -calcio AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Sofia Vergara Embraces Bold Strapless Corset Look While in Paris - Reality Tea</t>
+          <t>Giovane accoltellato a Milano, 4 minorenni in carcere - ANSA</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Sofia Vergara Embraces Bold Strapless Corset Look While in Paris - Reality Tea</t>
+          <t>Young man stabbed in Milan, 4 minors in prison - ANSA</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 14:04:00 GMT</t>
+          <t>Fri, 06 Mar 2026 07:55:00 GMT</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNckNrLTRsckFPLWJzcmYtZEdkdnFXQkJuME1XODV4NEd4SUtCa09CQzAyT3JVeUEwdkNqZHJzR2lfaWkzejNIWWxlOXRobklOdXdTOGpLdWx3UzJMcVRmREJYUDE4VnlkX2NLWVhZUWg3dzhqMVdZQ1ZfMmtEV3lXZWZZSzluVEQ3VEgtc1hrS01uLXl0QVVzdE1UbEg2T1XSAaQBQVVfeXFMUHN3UnA2clZTQVFGTEZ3S2NwVVJucWtWYWdiRmlsTlJjNHlLR1NFcExCbGxEWnNuOVNybzUyQnhIblpSUndGRjBzREpJT0JuckFvN2NRQVdQOVk2ekNUWk8yYWV3dGF6VUVnaVdpaWQtdTdxSHc3anFxOGl4dGM3U2ZpQjZwanVtMVRicTIyU3o1NkFnZTRXaDBKTnliMGkzcmM2Q2w?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-AFBVV95cUxONC1NaHJqNHl0czFpQy1IWXg3akJ0ZjUwTGFCQjVvejlBeUc3elc0cnhuWndsRGpveVlUU3JPM3k5MWg3WTF4RXlWWTFPYnVWZXU3QjhTUmUweU9zdmhHN3pnck5HU1U5STFNLXNaWFV4ZEt0SGI2S0ZKaEJWMjBDUkpTQTR5THBQTVlNQ1VVcEZEVk9la0pVbHJXTVJZeHh2cEZ4UHpfeHhDVXNXU1N5UnQ1LTcyTW85cjJaUlhvVHlsVngzYUdMRmdmTUFudDJvOG5vanBoQ1luY1ZaOVNvX2t3UEVyMjFRY2gxN19fVldWRzc1VjdnMtIB_gFBVV95cUxNOWl1VlFkZVdpWWdxbGIyOC1yc0lDUEp5UzdScUhsUW12RGoxaXdlalVvYldNTmNfT3d3Y1NMdGNKeHBwbzhXQkxzVTdXa2hYN2t4Z0UtcmhXNnFNSGh6Y1pYVURLa2dOeTVYVnYyU3B3NXdGQ3FPMFF3WTJTV29vYUVPZkRXcG1iMWowRkp1d3poZVlldjlQMUNDQ2hjRGdYYnpqNnNyemR4dWIwNjFwZzM4OVNyYlBsWVoxbHZVVlB6ZlllU3NjeE1GT25US21WbmQ1QUJ3SWlwUUxwWUMzZnU1NF9iS0drUE5Ma0c0OU9MX2lmdXd2SlRzaXl1QQ?oc=5</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3155,52 +3155,52 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>FR:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K50" s="1" t="n">
-        <v>46087.58611111111</v>
+        <v>46087.32986111111</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>High Level City France English (fallback)</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>("Paris" OR "Île-de-France")</t>
+          <t>("Milano" OR "Bologna") AND ("minaccia bomba" OR "pacco sospetto" OR "pacco esplosivo" OR sparatoria OR accoltellamento OR "attentato" OR "operazione di polizia" OR esplosione OR evacuazione) AND -Olimpiadi AND -pattinaggio AND -sci AND -Cortina AND -calcio AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Paris Jackson’s Tattoos Show Through Unbuttoned Shirt at Mugler Show - Reality Tea</t>
+          <t>Allarme bomba in Tribunale a Milano: le 4 telefonate, i controlli e l’evacuazione. Ispezioni con i cani in ogni stanza - Il Giorno</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Paris Jackson’s Tattoos Show Through Unbuttoned Shirt at Mugler Show - Reality Tea</t>
+          <t>Bomb alert in the Court of Milan: the 4 phone calls, the checks and the evacuation. Inspections with dogs in every room - The Day</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 12:35:40 GMT</t>
+          <t>Fri, 06 Mar 2026 12:37:12 GMT</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxPa2ZZVXVDcWpmOHlGNV9oaG1WVlEzQm1ZRVRuUjFoSFhITlluX3lsaGs1UXNWRWtaQUxwSVQtanFYV2wtOXZiSW83MlVqeUNVYU1KQjB0b0hEOE9wbmhHeURWTzNkc0c0MWxlMWlQOVBnZlZ3Y01ybUtCMjcwclI2ZHR2WjRBTXdsMlVyWDlpUdIBlAFBVV95cUxNVTNVZTZ5Nkh3M1hxLXg4TjRqMVFmX2liM245Z3d1NXBrei1haWxwUzNuckJseFdIZExDVTR6S1BTR3NucFlGdUtvd0I3aWI5ZEVuVVFpMkFySzJWWHUzWjhNS0h3Y2tMNjVQVlF3SFdUNE1FbG96U1ZieGlWSEJrM3VSYlJCQ0hiQWc1dTBWSm9YZ2JH?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE1FTnFKa1VwVlBXLWZkSGdLamE3U20wYUdLcEpqRF9DdVAtal91ZTl1M043YWZvTlppWFF3X1p6amRBcUl3RjJMdXRtbFRfZHJ4QVBvZktFblZ2eWxTRVZDeGVGTHVfQzhhTWtVTC1ZbTQxZHFvQWx0RE9sRQ?oc=5</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3210,52 +3210,52 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>FR:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K51" s="1" t="n">
-        <v>46087.52476851852</v>
+        <v>46087.52583333333</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>High Level City France English (fallback)</t>
+          <t>High Level City Italy English</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>("Paris" OR "Île-de-France")</t>
+          <t>("Milan" OR "Milano" OR "Bologna") AND ("Italy" OR "Italian") AND (protest OR demonstration OR rally OR "civil unrest" OR strike OR blockade OR march) AND -football AND -transfer AND -Serie AND -"fashion week" AND -catwalk AND -runway</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Paris-Nice 2026 | Vingegaard and Ayuso’s Tour ambitions go on the scales for the first time - IDLprocycling.com</t>
+          <t>Demonstration Alert – U.S. Consulate Milan, Italy, March 8, 2026 - U.S. Embassy and Consulates in Italy (.gov)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Paris-Nice 2026 | Vingegaard and Ayuso’s Tour ambitions go on the scales for the first time - IDLprocycling.com</t>
+          <t>Demonstration Alert – U.S. Consulate Milan, Italy, March 8, 2026 - U.S. Embassy and Consulates in Italy (.gov)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 13:22:58 GMT</t>
+          <t>Fri, 06 Mar 2026 19:57:10 GMT</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxPOVNRc1V4N1JYeGtnOS1lN0ZXNm9SZW1XMnRKWEhneXE4MzBqX3cyZzY4SzhrQ3d6NTBXdjNmdHgtTXZLaDBxY0s0aWhpLWM2MmpELURRdFBSNEN0U3Z0ZnVUZklZOXZKSlNfaUlvQWdVU1N0eFNNMU83UmtsS2lHOHlkcUZwMldCZzU3S1VacHNHZjBPZ2NzQU0wbUFFbC1YcDdTMGZzbWVXaEJIdG5VYXhMbkpVaEZ1YVNlX0ZLWWEzU3BW?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNSFRscWZHVnBqbkJ3S1JTSDJZcUZGV184blhoMFIyVEZPVXRxRkxJNEdfWXJpaDZ3ZGVfeHJqRlhoNzlPVWc5X3pCY0NvZ2lBbm91eHluUzdZR09ac2xkeHBUTGN2UUk3V2dVcGx1aG5aZE5QWUNtZWhfUUtfa2IwOV9yeGtxbVNmSjloaA?oc=5</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -3270,47 +3270,47 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>FR:en</t>
+          <t>IT:en</t>
         </is>
       </c>
       <c r="K52" s="1" t="n">
-        <v>46087.55761574074</v>
+        <v>46087.83136574074</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>High Level City France English (fallback)</t>
+          <t>High Level City Italy English</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>("Paris" OR "Île-de-France")</t>
+          <t>("Milan" OR "Milano" OR "Bologna") AND ("Italy" OR "Italian") AND (protest OR demonstration OR rally OR "civil unrest" OR strike OR blockade OR march) AND -football AND -transfer AND -Serie AND -"fashion week" AND -catwalk AND -runway</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Rick Owens Injects Love and Light Into FW26 - Hypebae</t>
+          <t>Milano Cortina 2026: Opening Ceremony sparkles in Verona Arena to inaugurate Winter Paralympics - olympics.com</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Rick Owens Injects Love and Light Into FW26 - Hypebae</t>
+          <t>Milano Cortina 2026: Opening Ceremony sparkles in Verona Arena to inaugurate Winter Paralympics - olympics.com</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 13:26:12 GMT</t>
+          <t>Fri, 06 Mar 2026 21:15:00 GMT</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxObU9NY3RNN0xEbDM4ZkNtOXJUOVl3elNJMTU5eDBSMFFaeWY5Q0NrRTdoSk5PWnJqbnJBZDRNMHc3MUU0LW10amVPRm4ybXBBczYtdjNqYkEyNC1MVzBQWTJ3dFZiajlFRXBMbWx0SzhUVkdjWGxpd1ZvZDh4NFVZYw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxOaThsQjFwLUJ5Wl9UVEVQai01ZGhNeHVMRFJiQXo1Ui0tZmZvcnlsWjQ4YUN6d0ZyeDJjVWQ3MzEwOXhVRlMwbXNDU1BIaGhVUFREMGh4bGlEa09IU0tFa3FleWtYT3g5bTU0cXJ5TWJMbVVSM1ZaZUdRd01yR1cxZEtnZUFwUnhVQU12aS1jQThFQ3pZYzBFUzVKdFEwbFM4RGt2QllubmdBS1IwZmJ0X1BsWDNXNnhWcDhxSmhNRVJFdjMyVUJSX01VckFRTUsyM1NRbWp3?oc=5</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3325,47 +3325,47 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>FR:en</t>
+          <t>IT:en</t>
         </is>
       </c>
       <c r="K53" s="1" t="n">
-        <v>46087.55986111111</v>
+        <v>46087.88541666666</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>High Level City France English (fallback)</t>
+          <t>High Level City Italy English</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>("Paris" OR "Île-de-France")</t>
+          <t>("Milan" OR "Milano" OR "Bologna") AND ("Italy" OR "Italian") AND (protest OR demonstration OR rally OR "civil unrest" OR strike OR blockade OR march) AND -football AND -transfer AND -Serie AND -"fashion week" AND -catwalk AND -runway</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Comexposium puts Serres in charge of Paris tradeshows Siec and NRF Retail’s Big Show Europe - FashionNetwork - The World's Fashion Business News</t>
+          <t>2026 Winter Paralympics: How to watch and stream - The Edwardsville Intelligencer</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Comexposium puts Serres in charge of Paris tradeshows Siec and NRF Retail’s Big Show Europe - FashionNetwork - The World's Fashion Business News</t>
+          <t>2026 Winter Paralympics: How to watch and stream - The Edwardsville Intelligencer</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 14:23:44 GMT</t>
+          <t>Fri, 06 Mar 2026 20:07:55 GMT</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxPTHd5VTlWc05ZWk9DaDFWV1c5OGkxSkRpYmxqNUxXbEhKVmJTRlloLWcxY3JVVldDWnlBYmF0eVNkeE44eFktdEs2OUZsZWNYRUJHb0ZMWHRFTGZ1dWdqWmRiNkJhZlRhenR6OWhHTXN6emRlaEdhRkpMUUdoZXpGR005cDY4MlNiQ203NUNRMXF6UzJ3bUFnVEI4aHZ6MDByYTFTZHRxV1QyT2NBNnM4ZEJpb1ZwaTAzTndaWW1kU25vaWtJQmFTamVOOFJIMDBHVkVBZ1Nn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxNaFk0Nm9UWkVTWEZWdVdnbGlYblRUM2lydm9Vd3RmX2dhSEZzcWFGS08yblJaZFZhRTJXZXZ1WkhlS1N6UVdBUnpVb1REQngtY2hjWE0wVE1BNF94a0ZYUjRPcVdyczkyYjlBRHZoYlE5TUxhUmhSd0JqTTNZaktoNWg3R3A2bmRObjZoR2hKT2s?oc=5</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -3380,47 +3380,47 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>FR:en</t>
+          <t>IT:en</t>
         </is>
       </c>
       <c r="K54" s="1" t="n">
-        <v>46087.59981481481</v>
+        <v>46087.83883101852</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>High Level City France English (fallback)</t>
+          <t>High Level City Italy English</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>("Paris" OR "Île-de-France")</t>
+          <t>("Milan" OR "Milano" OR "Bologna") AND ("Italy" OR "Italian") AND (protest OR demonstration OR rally OR "civil unrest" OR strike OR blockade OR march) AND -football AND -transfer AND -Serie AND -"fashion week" AND -catwalk AND -runway</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Viktor &amp; Rolf Fall 2026 Ready-to-Wear Collection [PHOTO] - wwd.com</t>
+          <t>La Bella Vita: A new Milan-Brussels sleeper train and March events in Italy - The Local Italy</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Viktor &amp; Rolf Fall 2026 Ready-to-Wear Collection [PHOTO] - wwd.com</t>
+          <t>La Bella Vita: A new Milan-Brussels sleeper train and March events in Italy - The Local Italy</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 09:09:17 GMT</t>
+          <t>Fri, 06 Mar 2026 13:23:58 GMT</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNeWYxYWlKUU5BT01jeTRDVVBvenExYlpqMkotTFA1VU9qWlJ0VFkyNVFiZG93cnQ4VGdseXd6MnNEb09UamZBLU5Ba3NrSGlsbW5DSTU3M2dZMmp5am8zUFF2eEIxMEdzNjZoMEhUZWgtTDJtVEhEODNzcDlLR1BiZU9ncU1fYk5rN1NRR1dZUTNoUEFkaXpJc3dsSFZmUU05TTJWbXBoLWlNWS1ONWc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQaGZpMUZfSWlubkZTTm5lbEkyY1dxLVB1OUhSYVRETVFwSUk2LVdpa0tMR3NXNWhxYzhhZzZyNVUzZVZEV05LazR5SnZzWkFIaGExdkJZSDNSTnl6bHI2S2c2VTdpeFpVcEkzS0RnTlpFa0lsR01jMEo3VUVhQUppa0x1RUNYdlp6U2luNS1KSWx4RDY0dTQyMDVESGE4WExFUnlfdnVJUFVkVEE?oc=5</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -3435,47 +3435,47 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>FR:en</t>
+          <t>IT:en</t>
         </is>
       </c>
       <c r="K55" s="1" t="n">
-        <v>46087.38144675926</v>
+        <v>46087.55831018519</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>High Level City France English (fallback)</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>("Paris" OR "Île-de-France")</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Chappell Roan’s Dramatic Hair Makeover Continues in Paris - AOL.com</t>
+          <t>Sciopero transfemminista dell'8 marzo 2026 a Milano: percorso, strade chiuse e programma della manifestazione - Mentelocale</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Chappell Roan’s Dramatic Hair Makeover Continues in Paris - AOL.com</t>
+          <t>Transfeminist strike of 8 March 2026 in Milan: route, closed streets and program of the demonstration - Mentelocale</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 12:23:37 GMT</t>
+          <t>Sat, 07 Mar 2026 02:48:26 GMT</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxQZTd5MkZ4TXFNdjlkOGEteW1OZFVvXzI2QU55MTZidkFhYjdYUDZmeGQ5eURnbGtGX0RiN29lUV8zT3QxVjJEaVFvamEwUU8tMFZDQU9vd195RC1MaVRkSUVoeGJYZUdFWTNHRURsQTVyUUdtaUZ5X2xCa3Fudk9NR05COHFKLU0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxPaEpKdVBXd2lZU3IyZ0hYb19fNmN5TEloWlZ1M1VaZi1Bc3I5RHFWOFhnYnhRa085QnRBSGpoVjUwM0dSNEVBX0Q1UzFUNjhnSWhzWmNkdkRnaEtEOWdsS05ZZ0dKWExTb1RJN1FpSlFWa0FacXlsSTFuc0s4ODBIR0twdUpDeEVkNDdnNDRjQ0pMX2hCaEZFT0JtdzdWa1FhRVNXM0l2UmkxZkVGR3dTcjdJYUdLR0NVeDg0QmlaN1VHWUVocGNpN0M4OTJNdk5TTENxeE5UdDczbnp6TkV6c0xGOGpGQ00?oc=5</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -3485,21 +3485,21 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>FR:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K56" s="1" t="n">
-        <v>46087.51640046296</v>
+        <v>46088.11696759259</v>
       </c>
     </row>
     <row r="57">
@@ -3510,27 +3510,27 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>("Milano" OR "Bologna") AND ("minaccia bomba" OR "pacco sospetto" OR "pacco esplosivo" OR sparatoria OR accoltellamento OR "attentato" OR "operazione di polizia" OR esplosione OR evacuazione) AND -Olimpiadi AND -pattinaggio AND -sci AND -Cortina AND -calcio AND -Serie AND -mercato</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Allarme bomba al tribunale di Milano, evacuazione di alcune parti dell’edificio. Udienze interrotte - Il Fatto Quotidiano</t>
+          <t>Lagarde contestata a Bologna: lancio di uova contro i fantocci e tensioni con la polizia | VIDEO - BolognaToday</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Bomb alert at the Milan courthouse, evacuation of some parts of the building. Hearings interrupted - Il Fatto Quotidiano</t>
+          <t>Lagarde contested in Bologna: throwing eggs at the puppets and tensions with the police | VIDEO - BolognaToday</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 09:03:46 GMT</t>
+          <t>Fri, 06 Mar 2026 19:19:08 GMT</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxPY0lRRjFENHdzWGpoYkh3UTBmS01pRldYZG5Yd0xUS3otYWZ4bF9GcktlWDd3aVp5ZGI0bXJSVElhMmhDeEk5T2JMVy05MXUwZkJVbGVUMFNlYVR5aVd3V21kc3RSa2FVUHFBeVphSGdUNS1sejNhUHVoUUM2V3JMbWk3YUttTkVvdzlRMHEzcFFpUlFiUzNXdFpEVGVQUU9rcXpON1VR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxQWEZZN0poc2JXa0ZpR2FmdWtlcjhLQjNIWG5maUZDbnMycEYteHJsU0RuVTZsZjl3MF9jRUxlR25lX3VXelVtdlFqNmJLLTRzQ29DMWprVGpGNTdTcWVrUFRzcjZyZlFsMC1lOWlKdzd6VjltWEpzQ0tMaHVzMDBnT1hFbWxSdw?oc=5</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -3554,38 +3554,38 @@
         </is>
       </c>
       <c r="K57" s="1" t="n">
-        <v>46087.37761574074</v>
+        <v>46087.8049537037</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Local Town Fidenza Italian</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>("Fidenza" OR "Parma" OR "Piacenza" OR "Cremona") AND (protesta OR "minaccia bomba" OR esplosione OR sparatoria OR accoltellamento OR evacuazione OR "operazione di polizia" OR arresto) AND -calcio AND -Serie AND -mercato</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Nas Parma. Primario arrestato per peculato: avrebbe incassato in contanti prestazioni intramoenia senza registrarle - Quotidiano Sanità</t>
+          <t>Sciopero 9 marzo 2026, treni, bus, scuola e sanità: chi aderisce (e chi no) a Bologna - Il Resto del Carlino</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Nas Parma. Head doctor arrested for embezzlement: he allegedly collected intramoenia benefits in cash without registering them - Quotidiano Sanità</t>
+          <t>Strike 9 March 2026, trains, buses, schools and healthcare: who joins (and who doesn't) in Bologna - Il Resto del Carlino</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Fri, 06 Mar 2026 11:45:59 GMT</t>
+          <t>Fri, 06 Mar 2026 17:24:12 GMT</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxOY0dRUnd5aXhXYWVaOE02eUthYnNHRmIyWHByaEVwVjlLN2cyVWdoMHNkcHhzTlQ0eHBQOHpUbjQxemFGUVR3bldXWDhBZDFCM3RFcUx2WENBbHBSY2EwNEo5cW82ZGlaamVaOU92UE5qNGV6Wlo3QU1YTERXVEdjMENIOHQ4ZlNyZkI0cnRMa2NndXBWY2t0bVRWcFZxSERKNHRoZHZTUXd0ZzZXaExnWU9ULWE1N01ydUk5LU9QM0tCYURtTE0zSEtTdTFvX3JiVVByRTlEU3M5SVJHNzBWNjJxYmdUc3BubjA0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxPMzJRaTg2bWRHR2dsZ0lxSjRKd3puZ2lLaVprMFFRcVdEc0txNGJXUHk3WTVMenFuOVl1dl9SeFJQWXNIdmVGUlBsUS02Q1YxZjJXMmx0TnQtUmlWV0RYeF8zYUtqNzB1NWJVc216VmZ6VkpsdTltbHNRak9aRDlWX01YVE9YaEE?oc=5</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -3609,7 +3609,447 @@
         </is>
       </c>
       <c r="K58" s="1" t="n">
-        <v>46087.49026620371</v>
+        <v>46087.72513888889</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Giochi paralimpici di Milano e Cortina, 12 Paesi disertano l'Arena di Verona: cresce la protesta contro la Russia - Corriere del Veneto</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Paralympic Games in Milan and Cortina, 12 countries desert the Verona Arena: protest against Russia grows - Corriere del Veneto</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Fri, 06 Mar 2026 15:50:00 GMT</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirgJBVV95cUxOQmVGQ1FBTWNWczVBSEVQMWNwXzFCd0RZcFd5ZXM5c3dQMXBzZU1MU1Q3eDRBSjlKVXBnTnlWekE0U25zQU1MUmx6Y1lCMWFvSkNSeFVvemNRRW82Q19jUzNsNGh2cTNKaDhHSG5VVWVoblNJODlSYW05UVBLY09Wa3loaEdwN0xRcmN3dGZtbFk1YVE4MEJaYVN4UHFIV3AwR2s0NENzVzNzLUFrUjZ4azdZWmZWbVBxR3BpUEk5bUpkYy1JQlVpajE3bWpRVDZXWmV5YklUYUF5d2J6cDNZZVppejFnWTlHX19IOU1IZUJ1ZlBIRnU2MXVhcXBCRlYxN0I3R3FtYnRYZmZiZ2liVGRwemJHV0JETzVfakZOd1pMQzV1OHN5LVlUSkVUUdIBswJBVV95cUxQZ1dKdUZ6VHRGaDgtM0hXUFFUM2ZrM09WOTZualRtbFdBNk9reENjV29yM285N1NTM2czdEZLSlk3VFlwT0RhT1h5ekJLcjVmZUJQTjBIc2JTenpNdWczc3AxSlVCd3p4QzlPdlM0cldrMzBLbFdxTTdYQVhDWGx2UjB1VVV6UC1YZkp3aTlxQklnbmo1SU8xRmxTUkxweVpLSHVoZmVVQU9vQUFFR3I4TWxTZ2RscTNmQjZlT253VVNMY1ptWGwxSUtwMTZwZHZ2UjBqZXNBVWhGSWNock9rV1pWdklaNy1UUTVSdThudlhpM1hfdDlSS3F5TFB0UXZZUFR0Z1NTWEN4OG5nSEo2a2ZRTDRmdVFJVk50cXRJWFRKRERTQmgwdEFmUktKVGZseHZj?oc=5</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K59" s="1" t="n">
+        <v>46087.65972222222</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Quando ci sarà il prossimo sciopero dei mezzi a Milano - Virgilio</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>When will there be the next transport strike in Milan - Virgilio</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Fri, 06 Mar 2026 16:00:04 GMT</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPRXAyc01GREdsaWswNnE0MjlxMExqSVA0QWYyU1VpX1VrUVVXdFdXSm44WXozVm1rZzlNdE1pMWZNdFlkU1dKRXE5dEVMeldkNXM1MkNydFVHLUhrSG5SQmN1enowVUlyNU90MXBLczQ5NnVMZ1ZjZHRGUGZncFFKOWdVNTRrSmhVZXhqX1pjMnZPbGdYTnNTZlF5NzBrNkhGMTRtSEx4cWJ4NzdPMXNVNVp2RVpyNnljTGVV0gHAAUFVX3lxTE9sZkZqM2NaWGY5VTlWS3NpNmgySE12dTdoSTlqS3o0Zm9zYk5IWGNKc1E1VG1XRFlITnoxdEhlWnBGZ1hnbkhMOGlYSTRzVUY1SUZDajJuM3pyaWFFdzR4b0pNOTl0STZ6YUdaVTB1ZUo0ZjFTTHN1RjVNN0wwRFpPbkx1NVhpdWFCb1dzYm1VOWRCNFRkODQ0UmczdUVibEI5TEp1UTItYlRIb1hPUFhCX3ZQVVhEUXNMSTRIWU12RA?oc=5</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K60" s="1" t="n">
+        <v>46087.66671296296</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Scontri nel cantiere del MuBa, scarcerati i tre attivisti. E la protesta smonta | FOTO - BolognaToday</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Clashes at the MuBa construction site, the three activists released from prison. And the protest disintegrates | PHOTO - BolognaToday</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Fri, 06 Mar 2026 15:51:00 GMT</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNZ1JDbDhhczRJQUxYaGNzdVNfcHdfblFzWUttcG12bTd3cjlGeFVOZGczRy1Gb1BIVXdGdnlmTy1vWFpXRGtfN2wtN2lSQUZNeDZvQXh3T2dTTk5sc2JzU0dDaTlkbWJqb21PbWNTWldUZXlsMUM4ZDlpcENMLVowaTRTYkgtSEdLRzRGc3JZTzRIazFRblE?oc=5</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K61" s="1" t="n">
+        <v>46087.66041666667</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>8 marzo 2026 a Milano: manifestazioni ed iniziative in città - Secret Milano</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>8 March 2026 in Milan: events and initiatives in the city - Secret Milano</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Fri, 06 Mar 2026 10:15:42 GMT</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE0zNG9wSnU3bzNFOFdoSXB3dU02ZGxVQVdkSm55d3lveGNYUnZBcHZhSTZfanBzbkRuN196ZnNHMHFNNU4zMEdvd3hrY2ItVklrZkNqSFBOWGZfN19vemx5WUN0UDgyeWdwaE5IcFlScGI?oc=5</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K62" s="1" t="n">
+        <v>46087.42756944444</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Il 9 marzo sciopero generale: il costo delle mobilitazioni per l’economia italiana supera i 5 miliardi l’anno - Capitalist.it</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>General strike on March 9th: the cost of the protests for the Italian economy exceeds 5 billion a year - Capitalist.it</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Fri, 06 Mar 2026 14:54:57 GMT</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxPbUJZZk5HWERKXzBJakNxd2h0anBTNFhLblc2WWtySlozVnVITE5EV01aSjlpUWFxZzZzek5vMVZKWGhvSV93SFEzaU1YWVFZb3EyWl9nRUNzRUFtaEQzc252TzE2bl9jQ0szZFFhNV9NdEtFWTVZZ3FvNzZyU21vcXFzcw?oc=5</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K63" s="1" t="n">
+        <v>46087.62149305556</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Sciopero lunedì 9 marzo, dalla scuola ai trasporti pubblici: ecco chi si ferma - Tgcom24</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Strike on Monday 9 March, from schools to public transport: here's who's stopping - Tgcom24</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Fri, 06 Mar 2026 11:37:05 GMT</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxOXzlnVUtVU1hfYkFHSkZnc2lYNERMNEFmdDlvNFBaQnRPeFRCWlpxNmJ1RTlkeEplc2tnTnk4a2VjdXAyTzVWQWI2MWp5VGo2c0tSbS1NcUZabGpqUmxJSFFqTVlGeEduSXU0ZVVjcEF5eHo0enAyOUtOeXFTR081Y25pQlZ4MGFiNGlnY3B4TmLSAWhBVV95cUxPbUdmeVBMOW03bUFoeE1PQnN1ZE52OVdkNV9GYkt3OWRtalRNNTE0d2ZHQWM1NTczTFp4OGRYbDBrZGNlQ2RUUDNKQlVNMU5RSFZGbVFzbkZ3TGNOQlI0S0pSZGFkYTRnbQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K64" s="1" t="n">
+        <v>46087.48408564815</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Licenziamenti in arrivo, all'Unilever scatta la protesta dei lavoratori - Virgilio</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Layoffs are coming, workers protest at Unilever - Virgilio</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Fri, 06 Mar 2026 22:30:42 GMT</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxQZHJWU3VwSUUxRHB6YUJJUGdtZXhxbjV2UU8xZEU5SlZWNzF1ZHBvYllLUXJIalJJSjM0MkVpcmNObDVUZVFWTEpWM2NQSGFjSWtNRG9hbEVXOEgyaks1WlBEQ1lKOWptLXU0U3MwcVhYMER3UFRiNE0wRTlvSDRNbXc0UFdDb1VSeGJxWXFURjVuT293R2ctdjZneXIzYkw2cWUxd20zV1pPUVUxME5KVTlUZ2g1QXZ1MzdTTWR0REd2RUEzY3EtTkxqNDRIODQzbGfSAdcBQVVfeXFMTVFHT1FncTZ0a3F5anYxa0lzRERBMFlYWFd0bWlQNXFROU9aVmxTVzNNTV9aZ3hNUl9fdXlEX0l3WFJSeDVSOUZXdUduZFZWQi1zQ2xmNnNOR2c3SVJHcU84ZDk5QlRpQ2c4TE8xUXhUVXJvWXZjM3dMRW1vd2c4UTRGZXlYWWtlaFRWR3JaNWNQeVpTai1rdmZoa2t1bG9fUHVjeFBlWHJ6U1ZTNW1kc0xTbmpWR2VoRTBhdW16eHdFMjZJcndIRXY4NDhIQi15d19lMVlMa00?oc=5</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K65" s="1" t="n">
+        <v>46087.93798611111</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Sit-in degli alluvionati in difesa delle querce - Il Resto del Carlino</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Sit-in of flood victims in defense of oaks - Il Resto del Carlino</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Fri, 06 Mar 2026 19:44:11 GMT</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxNUDRGTlRaQkxzSENMcTJrNFFUWEk4Z25pdm1nc09vQ0ZsODF4Y2ZxV2VDMTQ3THpZci03SzI2UlQ0dkhZektqdUp2aWx2Y05yejlWZDZaNjczY1AxLU56UGlSYTdmdDAtR0pwbkhCWFRadEFBdmpROGxkSmoxR0VGM0RYZkFTQ2ZCb0liWHZ3bXpxTjQ0?oc=5</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K66" s="1" t="n">
+        <v>46087.82234953704</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-03-08 07:38 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,32 +480,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Verdachte opgepakt voor steekpartij Terloplein: “Man kwam verhaal halen na verkeersruzie” - HLN</t>
+          <t>Incredible new £169m ‘shopping village’ opening beside busy UK motorway - Express.co.uk</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Suspect arrested for stabbing Terloplein: “Man came to seek redress after traffic dispute” - HLN</t>
+          <t>Incredible new £169m ‘shopping village’ opening beside busy UK motorway - Express.co.uk</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 09:04:34 GMT</t>
+          <t>Sat, 07 Mar 2026 19:56:00 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxOT0kwX3FxUTVISFdHSGdsNURaa3VidHdCd1J6Y3pwQzB2cHBORG14NjBNREp4S05abWdBcTRkcWVxazcyQ1dJYVFpdm5qYlpySVNlZHIxb1pmVzF3OURYQjl1LVdyaFh3bE9QTUExSmlFeG9maWlGcGpTWElLRUkyRlhLZmJvSU1HTmRpU0FFMUlNV2I1ZE1RSF9TbGNJbDYzR0V4MlZTNGJhWjBqV0tGa05MT1JYZGlrM29reEVZOEJKd1k?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxPd05JNm1DTmZkYVFPRlNDaEc4Y19ELTlaN3dLRElrMU1KeTJiNHlUQkpiRkR5UXoxRi12Y0ZKcThxcF9xQlNRVThqc2JhbjRKdlBfeXd1RVE1WkNFMEpheWx3V0lHdl95dXRNeUk4T2VlMWlNUVVud3FLRXB3cElESGFOX3fSAYoBQVVfeXFMT3BlY3hHQ01hLUZnZDhZSlJ4dnlhNDJMSV9KeHhfWEJ2eGZScnlGMUNkTU9halBuSUM1WC1KM3lkZjRYZ0pYelpMX3JnbUhab3A3ZXB2TlREVDFKRDJRaW5sWXFOSUlKRDZVWGxiVkU2eVFXZWF3Y1hRYmViXzEtSWM3NUh4MUVTUGZB?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -515,21 +515,21 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46088.3781712963</v>
+        <v>46088.83055555556</v>
       </c>
     </row>
     <row r="3">
@@ -545,22 +545,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Verkeersdispuut mondt uit in steekpartij op Terloplein: verdachte (29) opgepakt - GVA</t>
+          <t>Tieners aangeklaagd voor moord na dodelijke steekpartij bij treinstation in Melbourne - GVA</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Traffic dispute results in stabbing on Terloplein: suspect (29) arrested - GVA</t>
+          <t>Teenagers charged with murder after fatal stabbing at Melbourne train station - GVA</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 10:16:00 GMT</t>
+          <t>Sun, 08 Mar 2026 05:17:35 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9gFBVV95cUxQTlk2RmlvN3RneWVzY2RmTFo1SzktZlVwWXF1amprVENvbUhma2F3TTZsNzBGZnl5VFRFdWNadUlnMDhZTG01ODFWS0RJX2lUNlRSdXQyaEFuQUJCcTRYXzJtQ1BrbWcwNjRpb2F1aFZnSVR3OUF5c1MxbVJjc25aZ2tzUkZPLWVRb2xYaHlJbzVoTHRPQWhhUkNRTURFNFhjYko3bzZiSE9RSnVKYXA2ZG1pUDd2OTVfMXVYbDRObFk3cUFmQV9DemNqbTFDdlQzR3ZkU3Z1eHNIb1NYS2NBcDU3OEtNVV9zN3pFNVcxVGQ1OVZmVnc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxQTmNoa2NsaEswUWJBWDZkeFl0bWMyVHJwYXNobzV0c3Y5MmY4M0I2N1djS3VsWWcwSzJBLUxLVnAxZnNxa3JsMm1CS1hqdWtkQkZLR3ZlaXF2dUl6VVRFNm9zRGp1ZGlTNmFRaFlQMXBSQW9EY2YtU0M0Y0EzLXZVTF9yZklVRTcwTUNwZGJkM0RKdmVSYTlrYW9ZSWkyWkJZS3VUa1dKTjZ5VjEwcTNIWVc4ZHNJNzRaWmdfQmk4TW53N2JEUENicHdB?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46088.42777777778</v>
+        <v>46089.22054398148</v>
       </c>
     </row>
     <row r="4">
@@ -600,22 +600,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Moeder (44) in shock en dochter (15) lichtgewond na explosie in woning in Zulte: “In overleg met familie en sociale dienst voor opvang komende weken” - HLN</t>
+          <t>Verdachte opgepakt voor steekpartij Terloplein: “Man kwam verhaal halen na verkeersruzie” - HLN</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Mother (44) in shock and daughter (15) slightly injured after explosion in home in Zulte: “In consultation with family and social services for care in the coming weeks” - HLN</t>
+          <t>Suspect arrested for stabbing Terloplein: “Man came to seek redress after traffic dispute” - HLN</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 11:01:40 GMT</t>
+          <t>Sat, 07 Mar 2026 14:13:39 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxPSVplVU5ibFVPNVdRdU9jT2Z5Vm9BZGtkQjZtVFNuQ1Z3Slhhb3V4bUVUUkl5Zzl6c2J6LUN2czhLUTgxM3RuMUlubk1tckdtLU1yU2FOemFsVG0zTHJjcE9OWE0wR2taUk1CRFVQTlZhUGxPczhET1cyV051MFZ5Skp0MVdHb0p5dm1kSko5M3hjLTF5VXVKc0tmQVFYWS1XaTYwRWpyYlNEbW1FODNUbEg2elAxX1NId0FaNGdhZHV1SEVXYnpvTllCMk84dVUzb00xX1ZqVUttNDdjTEFTNGV6c2FqNVJ0ZGc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxOT0kwX3FxUTVISFdHSGdsNURaa3VidHdCd1J6Y3pwQzB2cHBORG14NjBNREp4S05abWdBcTRkcWVxazcyQ1dJYVFpdm5qYlpySVNlZHIxb1pmVzF3OURYQjl1LVdyaFh3bE9QTUExSmlFeG9maWlGcGpTWElLRUkyRlhLZmJvSU1HTmRpU0FFMUlNV2I1ZE1RSF9TbGNJbDYzR0V4MlZTNGJhWjBqV0tGa05MT1JYZGlrM29reEVZOEJKd1k?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46088.45949074074</v>
+        <v>46088.5928125</v>
       </c>
     </row>
     <row r="5">
@@ -655,22 +655,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Amper treinverkeer in Brussel-Noord en Brussel-Centraal dit weekend - HLN</t>
+          <t>Man (30) neergestoken in Borgerhout na verkeersdispuut, verdachte (29) opgepakt - VRT</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Hardly any train traffic in Brussels North and Brussels Central this weekend - HLN</t>
+          <t>Man (30) stabbed in Borgerhout after traffic dispute, suspect (29) arrested - VRT</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 12:37:57 GMT</t>
+          <t>Sat, 07 Mar 2026 10:27:22 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxQb1lZYUlhQWw1Y0QzQkRmdkRVWGFnYzdJQjlkZUdacGtVZWVoVWVCQU5NNkhhUEVOOTFfSTJEN1pfeFFPanJ2VFo1ZHZyck5YVjZJcTdtOWJ0d2h6bUlwdkFKVHFlWWc4S1U5QTBBcWZySFdqcTFoMGh2WFlzZk9HRG1YT1lpUzVzWmVVLThjd04wSExXZWlFdU95Zl9WWGVZR1VQQk1jcw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxOcXhOWUdkdFVzc0ZIbl8wbzdteFAzZF9WcC1vYXZZWVFkaVZhbVdKOUZha2Vodk92MzhvMXE2OGoxd3B2UHBWdlFicVJia0tFUTQ1ZUs2al8wSGdQMWVad1pybm12V01ObUpESHBlcHpzV3VYVnlsZ1JqWGhaUkRWSTFlcTBRVERGTWl4Tw?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46088.52635416666</v>
+        <v>46088.4356712963</v>
       </c>
     </row>
     <row r="6">
@@ -710,22 +710,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Eerste militaire vlucht met 185 Belgen vliegt vanavond vanuit Oman naar Brussel - Vlaamse Wout (20) boekte zelf ticket en wacht nu op luchthaven Dubai - HLN</t>
+          <t>The Kids vieren vijftigste verjaardag op Left Festival - Nieuwsblad</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>First military flight with 185 Belgians flies from Oman to Brussels tonight - Flemish Wout (20) booked his own ticket and is now waiting at Dubai airport - HLN</t>
+          <t>The Kids celebrate their fiftieth anniversary at Left Festival - Nieuwsblad</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 10:38:12 GMT</t>
+          <t>Sun, 08 Mar 2026 02:27:03 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilAJBVV95cUxNUHVCejdUOFk3ek4wMk9McVhpRlM3Vmt1ZXVqT2txbkdOQWZieDY5Z2tmREg1a1E4RXd1eWp0VGNxU3VsTkR6Z3gwUVJnOFVqNk12eUQ1Ti12aWV0bTVnMHFPbFpsR21teENsQTVrUDcySjljUTgyUXNZR1RRekE5aUJpbXlVa1hEX0hNelA3Z1JDcHRjdlNkeUdndFFVdkhwUjNvbXhPb1RxekZublg0Rkt6V2FhY3ZrXzNEYWIxQmt3aE9oUWhTaDlwWDZtclN5WVo4N0Z3dDlPVTREUVZhYnV2N1lZZUswZUROaE5uMGNwWFUwMl9SaGZKaExlSlZNR0Utc3pxNWE2SlZqRzVSTkptSXo?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxOYVkyNjBBZTZWSFU0ek1pMGN6cWVnZ1ZoRTJPM2QtZFlTa2kzczFiTjV3NWloUUZPTlczX1dzMkFiMVVQenRVVjh2cUFPcmF2MERBZWhMNzZyZGFYano3T2R0OE5Qa2psV0p3Zk1IT2dxZzlFM3hhVmxraVRncmNFWC1lb1VwSTlfWF9nLVljS1pocU9RcEJRajJWUkhfMnE2aWNMcDUwTU13MW5qRWdaaTlyUzBIaXJJYkV0NkZxUUpzc0ZrTnZDb3hEQUhIdlNXeVgw?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46088.44319444444</v>
+        <v>46089.10211805555</v>
       </c>
     </row>
     <row r="7">
@@ -765,22 +765,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Voortvluchtige Antwerpenaar opgepakt op luchthaven in Frankrijk - HLN</t>
+          <t>Moeder (44) in shock en dochter (15) lichtgewond na explosie in woning in Zulte: “In overleg met familie en sociale dienst voor opvang komende weken” - HLN</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Fugitive Antwerp citizen arrested at airport in France - HLN</t>
+          <t>Mother (44) in shock and daughter (15) slightly injured after explosion in home in Zulte: “In consultation with family and social services for care in the coming weeks” - HLN</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 14:11:39 GMT</t>
+          <t>Sat, 07 Mar 2026 11:01:40 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOTW5KMzYxbllHYlVfcjZQaUthZ0tkbV90QUxEOXBTdkZmRzBNZ0N2UWFuZnpUMEs5eWNJXzdMcnJhTmhEX3dzNmVUc2VNLUVPem00UmhydG1ndmlOc0tOVzd4bzFSYUdsUnJ2eHdIXy1qdUVxLXVGdmwySlpINW5jVnJlX0xWbXlLMEpDWkRiVlhTcktfb3dLVlhwUDVjc2s4UVBVWg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxPSVplVU5ibFVPNVdRdU9jT2Z5Vm9BZGtkQjZtVFNuQ1Z3Slhhb3V4bUVUUkl5Zzl6c2J6LUN2czhLUTgxM3RuMUlubk1tckdtLU1yU2FOemFsVG0zTHJjcE9OWE0wR2taUk1CRFVQTlZhUGxPczhET1cyV051MFZ5Skp0MVdHb0p5dm1kSko5M3hjLTF5VXVKc0tmQVFYWS1XaTYwRWpyYlNEbW1FODNUbEg2elAxX1NId0FaNGdhZHV1SEVXYnpvTllCMk84dVUzb00xX1ZqVUttNDdjTEFTNGV6c2FqNVJ0ZGc?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46088.59142361111</v>
+        <v>46088.45949074074</v>
       </c>
     </row>
     <row r="8">
@@ -820,22 +820,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Dit was Kuurne-Brussel-Kuurne van 2026 met Matthew Brennan die won en Jasper Philipsen die niet tot sprinten kwam: “Geen frisse benen meer” - HLN</t>
+          <t>Eerste militaire vlucht met 185 Belgen vliegt vanavond vanuit Oman naar Brussel - Vlaamse Wout (20) boekte zelf ticket en wacht nu op luchthaven Dubai - HLN</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>This was Kuurne-Brussels-Kuurne of 2026 with Matthew Brennan who won and Jasper Philipsen who failed to sprint: “No fresh legs anymore” - HLN</t>
+          <t>First military flight with 185 Belgians flies from Oman to Brussels tonight - Flemish Wout (20) booked his own ticket and is now waiting at Dubai airport - HLN</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 11:54:28 GMT</t>
+          <t>Sat, 07 Mar 2026 10:38:12 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwJBVV95cUxQcFp6Wm5HRzJxXzMzY0dwUGc1bEZSbkV4YzhtamNRRFJpcjg0X1hFMnNxMU9NSXNNREwycEx6Y3NvSUNqSmRPT2x4S3lYa3lnNlYxMEhhMTlwTm82MXpxTE1Eb2NUWWtJT1NyRkNMRTZhSFRTdHg3and0VnZKV1l6a0F0ZDFURGZzNTIyTUVjT0hLRUdmRDY1SVVxUXpwYzBfNUxPUDcyYUF5NmxqY090Ry11NldmT1BtVkhLaldnZVZOT2Y4MW10RXR5V0VUYVJmWDgzUnBoS2p5VlRMSEFzY2JSZmp0VFVCVnoxMXZEalE4Qk1VMXlLanhaSlJXZHlhWnJUemNsaw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilAJBVV95cUxNUHVCejdUOFk3ek4wMk9McVhpRlM3Vmt1ZXVqT2txbkdOQWZieDY5Z2tmREg1a1E4RXd1eWp0VGNxU3VsTkR6Z3gwUVJnOFVqNk12eUQ1Ti12aWV0bTVnMHFPbFpsR21teENsQTVrUDcySjljUTgyUXNZR1RRekE5aUJpbXlVa1hEX0hNelA3Z1JDcHRjdlNkeUdndFFVdkhwUjNvbXhPb1RxekZublg0Rkt6V2FhY3ZrXzNEYWIxQmt3aE9oUWhTaDlwWDZtclN5WVo4N0Z3dDlPVTREUVZhYnV2N1lZZUswZUROaE5uMGNwWFUwMl9SaGZKaExlSlZNR0Utc3pxNWE2SlZqRzVSTkptSXo?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46088.4961574074</v>
+        <v>46088.44319444444</v>
       </c>
     </row>
     <row r="9">
@@ -875,22 +875,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Medewerkers van bouwhandel redden zestiger uit kanaal Brussel-Charleroi in Halle - HLN</t>
+          <t>Voortvluchtige Antwerpenaar opgepakt op luchthaven in Frankrijk - HLN</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Construction trade employees rescue sixties from the Brussels-Charleroi canal in Halle - HLN</t>
+          <t>Fugitive Antwerp citizen arrested at airport in France - HLN</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 12:43:15 GMT</t>
+          <t>Sat, 07 Mar 2026 14:11:39 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQeDlXb0lTSmZZbU1ucXM4V01GcHRKUzVRSkNsR2lXVGt1emlSMlJ4SDQwY0RZeVF4ZnNlLURReTZEeWpkc2JHbEU3ZlpURm5YVW5VdlVheG83clQ5X0ItUVhWeExBNlNoUzh2M3FndXpabDdvSnREVzE5Wjh3OHRUcUFqTmpDTWZxVFRJdVB6QmVwbi16dDAwVWtuNl9RUUZYN2Q2WUxiVmNWeUVtSDI2VjhSTC1sUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOTW5KMzYxbllHYlVfcjZQaUthZ0tkbV90QUxEOXBTdkZmRzBNZ0N2UWFuZnpUMEs5eWNJXzdMcnJhTmhEX3dzNmVUc2VNLUVPem00UmhydG1ndmlOc0tOVzd4bzFSYUdsUnJ2eHdIXy1qdUVxLXVGdmwySlpINW5jVnJlX0xWbXlLMEpDWkRiVlhTcktfb3dLVlhwUDVjc2s4UVBVWg?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -914,38 +914,38 @@
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46088.53003472222</v>
+        <v>46088.59142361111</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Le mari d'une serveuse licenciée tire à deux reprises sur son patron et de son père avant d'être poignardé - BruxellesToday</t>
+          <t>Medewerkers van bouwhandel redden zestiger uit kanaal Brussel-Charleroi - HLN</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>The husband of a fired waitress shoots his boss and his father twice before being stabbed - BruxellesToday</t>
+          <t>Construction trade employees rescue sixties from Brussels-Charleroi canal - HLN</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 10:41:00 GMT</t>
+          <t>Sat, 07 Mar 2026 12:38:06 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxPaEhQMlJhS2NaV05lbEUySUg3aEo5OW93NFRpeEVRTTdFODVTNXRVRVRWeHFZWnc4ekRyWFFpWEpFdkFuOWZsRHpNdnZmTExoRi1FdmI3RldKcjA2OFBxWnRsZmJFRmxvQTAxamdocC1HZ2ZKcjAtTkFfNzNYOHQ3WnVPX0V3UkQzcUNBUTlsME1KemVDNlV4TQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxNUTZQTHNldFVteXIyeTFSTnZkMXlKZVBxeFV0UDItTTNLLVR0U1VTWHM0SmI1S1NJajhuQnFDVjFOR0F1akI2SmUwOTg4czRuODY0VS1KUmpYNUVkMWp1WjMwTWFEbGFXV1BvUFJTRlo3STBVYTFvdG10VmNISGVuUUo1ZjJ0a2xWT190X1FlR29IWEF5dnVRMTdYdktpRURIeUhwN083X2RFUQ?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -955,7 +955,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -965,42 +965,42 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46088.44513888889</v>
+        <v>46088.52645833333</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Politie waarschuwt voor valse biljetten van 50 euro: hier duiken ze op - Nieuws365</t>
+          <t>Foreign Minister Ferit Hoxha: For Albania, all roads lead to Brussels - cna.al</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Police warn about counterfeit 50 euro notes: this is where they appear - Nieuws365</t>
+          <t>Foreign Minister Ferit Hoxha: For Albania, all roads lead to Brussels - cna.al</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 12:00:14 GMT</t>
+          <t>Sat, 07 Mar 2026 12:08:00 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxQZE9YQUpIYWg2NUctMG5oM3VrWHJxcVJ2T0t1clFRVy1TemUwVHpwemZjaGVuZnFkVFZKMnd0a1o2Q0pyMzNZOEFBRnNTVHFjVU1DNUVWLWY3REZMTjhLVFJNRlV5LXZxcFJOOUl1NXlZbVVsWkFQOF9ybEttZ3h2cEJlMnN0SHh0R0MyY291VEdGWTc4aGM5cmVJdks3UkZpYlpFY05kd1A?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPWEZlaTZVelVnQlZ6SWlTS2VvNVNBVVJYMUFMeUJXSm9hcDdOSmFvRzBOOEhyd25kX2UwckFXX1pMVHhfX0xMZ2d2Y3BORzczV3ZyTWJEXzl6cEV0OWVTNkVFeDVYWWZsbDE1Wi16Si1QdFNoOU5VYUlWMTRicTZSQzZTN2tzbXVETDBrNFRLeU80ZkU2LUJZa1M1Q2NDZWNaaWhQR3VDMkVRSnRid0VyQVpYSHRPQQ?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1020,42 +1020,42 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46088.50016203704</v>
+        <v>46088.50555555556</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Cross Car et Rallycross prennent leur envol à Maasmechelen ce dimanche... - SpeedactionTV.be</t>
+          <t>Le mari d'une serveuse licenciée tire à deux reprises sur son patron et son père avant d'être poignardé - BruxellesToday</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Cross Car and Rallycross take off in Maasmechelen this Sunday... - SpeedactionTV.be</t>
+          <t>Husband of fired waitress shoots boss and father twice before being stabbed - BruxellesToday</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 08:59:13 GMT</t>
+          <t>Sat, 07 Mar 2026 10:41:00 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNQ1JPUElCTTdzSjFhSWpjSGpkX1pXTEd1dHJnVmZJa2h0Mjc4VnMyTi1PVGVRYzlJOXB6aVdpRVg5TEUtUVJZTU1Jdjd1VHlrZ3o2bUM4STJRWjNVWF9hN3JLQWlRWm1LR05tM1JaOTZTTEpSR3YtXzRjNUdzSnlWamIwbUJZbU9URnZMRm55SGFrckUzQzZvajczVmRHYlRxaFFDWk1OUUZtNWthcTZjTmt3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxPaEhQMlJhS2NaV05lbEUySUg3aEo5OW93NFRpeEVRTTdFODVTNXRVRVRWeHFZWnc4ekRyWFFpWEpFdkFuOWZsRHpNdnZmTExoRi1FdmI3RldKcjA2OFBxWnRsZmJFRmxvQTAxamdocC1HZ2ZKcjAtTkFfNzNYOHQ3WnVPX0V3UkQzcUNBUTlsME1KemVDNlV4TQ?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1079,38 +1079,38 @@
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46088.37445601852</v>
+        <v>46088.44513888889</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Highlights: RealDev Vilvoorde 2-6 RSCA Futsal (F. League) - Anderlecht</t>
+          <t>Agression contre l’Iran : Après l’Espagne la « rébellion » gagne la Belgique - La patrie news</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Highlights: RealDev Vilvoorde 2-6 RSCA Futsal (F. League) - Anderlecht</t>
+          <t>Aggression against Iran: After Spain the “rebellion” reaches Belgium - La Patrie news</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 11:19:56 GMT</t>
+          <t>Sat, 07 Mar 2026 18:13:18 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxPVTZsQy1aUFRtbVpXOFRvdV9VaG0tOGhPckpiT1lKci1kb1REYVYzY3ZQVFdBbXJPajhiQmhzYkpLdmZPVFhBaFRIbVpNeU9oRXF2QXV3bDF1OU5iUU9NZGxqdmg0OXBlVnNFaEdzNklwdURtNmNyODYySkF4ek1RVV92TGdvSDVJ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxPSGtpZjFtVldEdU5ycFNtamRwaWpNVXJXelRubkh0dFAxb1phWUhGODVfU0tUSWRhRDRyb25HZ1ZOTEd3RTFLY0owaXJnU0lNZVpjaTF0bXRUZFJMLTdUY0xHMkZEV1Y5dHRwWHhnZ0tFdU1NaXdETVNnTU9od3FUZ3lyanJXaTlrd1FmcXlDNWhzZUptcUFJbA?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1134,38 +1134,38 @@
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46088.47217592593</v>
+        <v>46088.75923611111</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Toulouse FC - OM : Les blessés, les compos probables et nos prédictions pour ce match de Ligue 1 - MSN</t>
+          <t>Politie waarschuwt voor valse biljetten van 50 euro: hier duiken ze op - Nieuws365</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Toulouse FC - OM: Injuries, probable lineups and our predictions for this Ligue 1 match - MSN</t>
+          <t>Police warn about counterfeit 50 euro notes: this is where they appear - Nieuws365</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 10:18:45 GMT</t>
+          <t>Sat, 07 Mar 2026 12:00:14 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxPT0phODJ0NUVPX1pIQXRZNG5tMHpFOTl5czVxM3JVakZva1dINmtwemdZXy16bndsOG13RGFoSFVoemdUVGFUal9xWUN5VEVJdmxkVWZYQ1NFbVBqSmU5UGRqRHR3bTY0T0FHY3lUX2t5TTRqaVdURXlISEF2LUl0TDYzMS10SVFjUThJY3gyVHlXZ2E3WWFFWEp1ZFZGTl9hSjdCYjU0dVpUaWthTEI0c01rN0g2a2RqMVREdkRpcDVKQ3ZXQUM5Y2VMaldoZXJYM1RVZzljVHZyME9seUk4N2tzQnFpdkFydlE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxQZE9YQUpIYWg2NUctMG5oM3VrWHJxcVJ2T0t1clFRVy1TemUwVHpwemZjaGVuZnFkVFZKMnd0a1o2Q0pyMzNZOEFBRnNTVHFjVU1DNUVWLWY3REZMTjhLVFJNRlV5LXZxcFJOOUl1NXlZbVVsWkFQOF9ybEttZ3h2cEJlMnN0SHh0R0MyY291VEdGWTc4aGM5cmVJdks3UkZpYlpFY05kd1A?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1185,42 +1185,42 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46088.4296875</v>
+        <v>46088.50016203704</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+          <t>France pick uncapped Brau-Boirie in new centre pairing for Wales - MSN</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+          <t>France pick uncapped Brau-Boirie in new centre pairing for Wales - MSN</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 09:29:58 GMT</t>
+          <t>Sat, 07 Mar 2026 17:11:30 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE03RUZJdVVWTG5jTlA1R0dmc2YyQ3Z2S1ExYmhkN0FENFJGamUwenJsSFFPWGpKc3B2aFBaeHRYVDR3aWM1SXg0YWZFVDk0N3d4a0Jz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPb2h2dUtROE9VZnBqUHRjTlJ3SUs4bzVNTkN2ZlNRWmw5NVdhcXlja3UyMXVOY1ZtS3VkcXRoZUszd21LQ3U4WC03TmY2X3VlaDhpaklGc19wUERhUDhEQ0ZxUWNVS1o1N1FzbTUyVVRmaTAtaEJpak5pRkdJQ0dtTDVCNjVOMmdzZHFBLVZ0XzZZR1dlVXRGWE1yUkJNSkdLYjNYdnpfQlU3b2Jp?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1230,52 +1230,52 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46088.39581018518</v>
+        <v>46088.71631944444</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Auffahrunfall zwischen zwei Linienbussen – Polizei sucht verletzte Fahrgäste - SW1.News</t>
+          <t>Why PSG's victory over Marseille will send shock waves across Europe? - MSN</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Rear-end collision between two buses – police are looking for injured passengers - SW1.News</t>
+          <t>Why PSG's victory over Marseille will send shock waves across Europe? - MSN</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 10:20:01 GMT</t>
+          <t>Sat, 07 Mar 2026 12:49:43 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNMTZTQ0Q0MDVhUGJOV2hXQ2tGaUZPYTRUUWlGOWxOV0xWa01nQTY3UUFVUlNnNDRhWjh2VTIxdXdFYW11ekVrN2ZjQ0hBMXE4T0pHeFRwNFZ4NUwwVDMzbXZqeWc2b2JsQ3dtNkJNaG8yUi00Z0pwUGpFSzZNVW1JWU1ZTUtzMjJlTVFWdnlIRW9XblczRjNEX0dwUDJrWG1obVlQVzhlRmpBV1d6cFU5X1o0UQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimANBVV95cUxNcjBtWDRxbnJObHg5UGptOUNOZnRXNHhRVUFKdlhOUWE0Z2FvNjZIWVd4eWhjclJUc182eV9xenpEZUl1cHhsOUoxY055RUlJSjRhNFQyVGxGcDJFd2Y3S2hDYXpXcXc5ODNmMkJfbUl2dnFWRVFUT2pNbTZsY1dsRkNHV3p0VVhOQ0dKSE55SGhBUXpVazRGbGRkWi1XRHc2cEp5dWpiaS1jcWw3TUFCOHZDbVV3TU9kblR2cEFQazNaOGxQTkdLSWY5aWFsa0NoaWJ0RXg2NUhFNGduOHBWVXZoVTF3ODFBdmhrSF9EM1dCbVVhX3RRUkZyQ1p4QURjbG9vMmJvSEJPcWs1b3NJZHRrMFhRUnJMVzJtRHFXaGdBbHNqRGd1WWx2VEVrM3lHb2NPXzRpQTN1WW1nNThRRl81ZkxKZng0SjctakE1LUtULUl0cFJXX1Q5eWZjbWM1b1U1YnFkYk80WkxCZWFDV2d5OXhDbVV3c3h6dTJWNHVGMERtNGduXzBPNzNNM0Q4YUMxRnYydmc?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1285,52 +1285,52 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46088.43056712963</v>
+        <v>46088.53452546296</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>72 Jahre nach der Hochzeit: Polizei schlichtet Streit bei hochbetagtem Paar - Augsburger Allgemeine</t>
+          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>72 years after the wedding: Police settle dispute between elderly couple - Augsburger Allgemeine</t>
+          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 10:08:15 GMT</t>
+          <t>Sun, 08 Mar 2026 02:22:42 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxOa25iNHQ2OTFnbGw2QTlJNlB3dTBFZUpZR1VrUnUzSUlPYVRTT0NOVDEtNlRZdzNTUHNCM2NrWkhYRHZRM19sVFppZTR4TVZUQzVIaTEzZGxzMld4cEZoLS1VbDFqN3VnS2M4bXl6eUhqcnM4ZWZWX3B2THB1Wl9oelY3cTlkU3RTMmQ4YlctdW5ZbG5RcEp0dzJQcWpFdmI4clV4QTRMWmZTWFM3TGozTktYaHZqNWVkYXpOdHFDSXplcDUxRGFIS21ia3ZnbVphTkRj?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE03RUZJdVVWTG5jTlA1R0dmc2YyQ3Z2S1ExYmhkN0FENFJGamUwenJsSFFPWGpKc3B2aFBaeHRYVDR3aWM1SXg0YWZFVDk0N3d4a0Jz?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1354,38 +1354,38 @@
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46088.42239583333</v>
+        <v>46089.09909722222</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Einsatz in Bayern wird zur Paarberatung: Hochbetagtes Paar ruft nach Streit im 72. Ehejahr die Polizei - Nordbayern</t>
+          <t>Mehrere Mülleimer in Brand gesteckt – Polizei sucht nach Zeugen - Newsallianz.de</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Mission in Bavaria turns into couples counseling: Elderly couple calls the police after an argument in their 72nd year of marriage - Northern Bavaria</t>
+          <t>Several trash cans set on fire – police are looking for witnesses - Newsallianz.de</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 11:00:00 GMT</t>
+          <t>Sat, 07 Mar 2026 08:29:54 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxOaVdMSGFfczY2dVM2T19tQTgxZFhVT3loaXYzVThscHppN3BVYkxRdExCbUlwTEY2Q1lWTV9GUmFTdzRuWGNoVWhmQkFzcnFtcWhZamM1dFc1ZHBUak5JUWR0bVQ3RVd5X0ZrTm5tNVRibUlBRXBvb19SejViNnJSOTE1azUyMXdVcGFRVHdua21qTzZhSlhoT3NBalM1OGRZYkh5T1J2anpmWlhLVVpOMGJ3NllGNmVHWlVHUEd5MWlmdlpyTVJhSGtTNUtDNGZfd3B4Um14UQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxPNWV0SFhZUGRDZWVlUzhBZ2tpQ0VJZkVwQTQ0SG16bFc3ZklkVXR6VnZTbFhaVlVaMG5QQXBGYWhxbXRjOU1JUGxLeVc2LXFzNEpjUUtvYS1XVy1kZVdWZkFJendUak9yTXdjdjV4VWZKWlBSOXYyLTY4aHJGMzYzdkdtUmJZOFp1b2ZBTGFTZGZZMHlFZ0FoRk5zU1Z5dw?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1409,38 +1409,38 @@
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46088.45833333334</v>
+        <v>46088.35409722223</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Polizeieinsatz bei Ehestreit: Versöhnung nach 72 Jahren Ehe in Ingolstadt - RegionalReporter</t>
+          <t>20-Jährige springt in Würzburg ihrer Tasche hinterher in den Main – dann wird die Strömung zu stark - Main-Post</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Police intervention in marital dispute: Reconciliation after 72 years of marriage in Ingolstadt - RegionalReporter</t>
+          <t>20-year-old jumps into the Main in Würzburg after her bag - then the current becomes too strong - Main-Post</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 09:32:41 GMT</t>
+          <t>Sun, 08 Mar 2026 07:35:20 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQZEdfd0otNGJRcjB0OVczeXl3UnF5cDVjUXZMWkgyZkhJeG9xNkt4M243ZzRaS25YeEtqN1hJWlRWbWJxNkpzb3FoTGNDTzlWM19tS1M5QlVOTkpDNlJjNHZOMXhQRnozUTZRM1I2a20yV09wdC1JTHNPWTJBclU0UHZ5MU96alhtcFptNlRYR0hUX1dOWDh6ajRMam0tY1QwY211SW9GcUtkN1ItakRjVkFNSDRicGNycVlhbFl3X1o3RG5GcGRJMGpRdnQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-gFBVV95cUxOaFEtcS03Qm9lb2ljMW9BdjRHMzYzai0tSkl3X1NSRkNtcGRVUFljakdCakJjcVhIM1dsalRtRXZteWsyallqTkllcHBaV0ZOQU1lbzRKMFU0WGdKcG5XdGoyQTJlQU5IVWRkRHluT08wdkhxLUhkc0R3cC1sTHNuajE2TmtXYWktUFQ5R2VDTXpsZHdDdjA5M1ZnN1JkZ0VnR1Z0UENhcmNFVERCUGlXSl9FbGJmcElFZm5NWFRMQnRXZGpTNVU3eGhNUWN0em5qQ0ZSOFRLYy1yS1NzVUV1dUZ1ZUIxVXBUYWVOc1BSR2psOTZpMWtZQV9n?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1464,62 +1464,1162 @@
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46088.39769675926</v>
+        <v>46089.3162037037</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Auffahrunfall zwischen zwei Linienbussen – Polizei sucht verletzte Fahrgäste - SW1.News</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Rear-end collision between two buses – police are looking for injured passengers - SW1.News</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Sat, 07 Mar 2026 10:20:01 GMT</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNMTZTQ0Q0MDVhUGJOV2hXQ2tGaUZPYTRUUWlGOWxOV0xWa01nQTY3UUFVUlNnNDRhWjh2VTIxdXdFYW11ekVrN2ZjQ0hBMXE4T0pHeFRwNFZ4NUwwVDMzbXZqeWc2b2JsQ3dtNkJNaG8yUi00Z0pwUGpFSzZNVW1JWU1ZTUtzMjJlTVFWdnlIRW9XblczRjNEX0dwUDJrWG1obVlQVzhlRmpBV1d6cFU5X1o0UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K20" s="1" t="n">
+        <v>46088.43056712963</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>Local Town Ingolstadt German</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Zeuge verpetzt Motocross-Fahrer (16) ohne Führerschein - RegionalReporter</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Witness rats out motocross driver (16) without a driver's license - RegionalReporter</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Sat, 07 Mar 2026 08:27:16 GMT</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNTU1PYzVOZVdQR2tZV0s1VjJHZTRpVXA3c2lqVFBwUFROVl9hYXl2NDgwNFVKV3hRUVpTSlJhRUl2VFpobVppT3NmZklZSmtkc2g1d3NmTGlmWHh1OVE2NjhTdGdYOTk0b2t6d3RzeXk4NjhSbHNkdHJqMVlXd3dNWG1TdlpFNFlLWVFlLWZpbklOQXdZX3pXZElZSjR0RXhDNEhfTzVjZzhoQnhUaHduUFB6ekg?oc=5</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>72 Jahre nach der Hochzeit: Polizei schlichtet Streit bei hochbetagtem Paar - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>72 years after the wedding: Police settle dispute between elderly couple - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Sat, 07 Mar 2026 10:08:15 GMT</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxOa25iNHQ2OTFnbGw2QTlJNlB3dTBFZUpZR1VrUnUzSUlPYVRTT0NOVDEtNlRZdzNTUHNCM2NrWkhYRHZRM19sVFppZTR4TVZUQzVIaTEzZGxzMld4cEZoLS1VbDFqN3VnS2M4bXl6eUhqcnM4ZWZWX3B2THB1Wl9oelY3cTlkU3RTMmQ4YlctdW5ZbG5RcEp0dzJQcWpFdmI4clV4QTRMWmZTWFM3TGozTktYaHZqNWVkYXpOdHFDSXplcDUxRGFIS21ia3ZnbVphTkRj?oc=5</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
         <is>
           <t>de</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>DE:de</t>
         </is>
       </c>
-      <c r="K20" s="1" t="n">
-        <v>46088.35226851852</v>
+      <c r="K21" s="1" t="n">
+        <v>46088.42239583333</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Polizeieinsatz bei Ehestreit: Versöhnung nach 72 Jahren Ehe in Ingolstadt - RegionalReporter</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Police intervention in marital dispute: Reconciliation after 72 years of marriage in Ingolstadt - RegionalReporter</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Sat, 07 Mar 2026 09:32:41 GMT</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQZEdfd0otNGJRcjB0OVczeXl3UnF5cDVjUXZMWkgyZkhJeG9xNkt4M243ZzRaS25YeEtqN1hJWlRWbWJxNkpzb3FoTGNDTzlWM19tS1M5QlVOTkpDNlJjNHZOMXhQRnozUTZRM1I2a20yV09wdC1JTHNPWTJBclU0UHZ5MU96alhtcFptNlRYR0hUX1dOWDh6ajRMam0tY1QwY211SW9GcUtkN1ItakRjVkFNSDRicGNycVlhbFl3X1o3RG5GcGRJMGpRdnQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K22" s="1" t="n">
+        <v>46088.39769675926</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Einsatz in Bayern wird zur Paarberatung: Hochbetagtes Paar ruft nach Streit im 72. Ehejahr die Polizei - Nordbayern</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Mission in Bavaria turns into couples counseling: Elderly couple calls the police after an argument in their 72nd year of marriage - Northern Bavaria</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Sat, 07 Mar 2026 11:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxOaVdMSGFfczY2dVM2T19tQTgxZFhVT3loaXYzVThscHppN3BVYkxRdExCbUlwTEY2Q1lWTV9GUmFTdzRuWGNoVWhmQkFzcnFtcWhZamM1dFc1ZHBUak5JUWR0bVQ3RVd5X0ZrTm5tNVRibUlBRXBvb19SejViNnJSOTE1azUyMXdVcGFRVHdua21qTzZhSlhoT3NBalM1OGRZYkh5T1J2anpmWlhLVVpOMGJ3NllGNmVHWlVHUEd5MWlmdlpyTVJhSGtTNUtDNGZfd3B4Um14UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K23" s="1" t="n">
+        <v>46088.45833333334</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Streit in Ingolstadt endet mit Polizeieingriff - lomazoma.com</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Dispute in Ingolstadt ends with police intervention - lomazoma.com</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Sat, 07 Mar 2026 18:53:04 GMT</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTFB3SFMxM2k4WW5HMHd1b2hVdHZQMDQ5ZkliRmozVnJmclNpejVqZ0lhdjR1RF9kY3VJSjUtTWhtbWxub1dmUnU1aXRHN2VCeFYxZ0JCcF9odTM1N1A5c2NnS3Fsd3VNU3ExN04xdVNmVFgxeGw3bjZJ?oc=5</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K24" s="1" t="n">
+        <v>46088.78685185185</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Village Ingolstadt (fallback)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Female coach Sabrina Wittmann blazing a lonely trail in men’s soccer in Germany - AP News</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Female coach Sabrina Wittmann blazing a lonely trail in men’s soccer in Germany - AP News</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Sat, 07 Mar 2026 16:53:00 GMT</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxQYmRQQUxtSm82aFlWRmlZZjBObFBrT0czblkwSUNvR2xBU0RxdVhVemdyQTU3SlByLWpkNkZaT2hjeEQ3QnZQVzBDNEEyRE5qVVdENFRlQVpzckt6VWw1X1M0NDU0SnhWTnlQWm1PSWM2MzczMHM0bG1BUEx4NGtHY1p5SHBIUU8tdzdleTNTMENCaUFjRk5Zcnk5YW51Zi1YTTAwcEpoMDJ2Zw?oc=5</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K25" s="1" t="n">
+        <v>46088.70347222222</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Village Las Rozas La Roca (fallback)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>("Las Rozas Village" OR "La Roca Village" OR "Las Rozas" OR "La Roca") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Las Rozas vs AD Parla: predictions, odds, head to head, where to watch, and more! - APWin</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Las Rozas vs AD Parla: predictions, odds, head to head, where to watch, and more! - APWin</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Sun, 08 Mar 2026 03:00:45 GMT</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOcW55RHBXb3VjTG1odktKSHp1WVhkOHNqc2V2cGhtTzBSZWpMSzRIMkxjalV5RHJ2amdKejA3WGphNzNJX0RZakZzcUlBaGdabnlrYWpIZjFFZ2JCYmpCQzRzNWhmczlpT1JQLWEybmp5aFVWdlJidVY4enhEdTdCZzIySVNFTmNxamVUTUVrVVpzV001MERBSW53?oc=5</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K26" s="1" t="n">
+        <v>46089.12552083333</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Sciopero generale lunedì 9 marzo 2026 - Comune di Bologna</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>General strike Monday 9 March 2026 - Municipality of Bologna</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Sat, 07 Mar 2026 23:20:46 GMT</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE5kOVNmT3ljRmJxNVZSLTFydDRJUmZRd2pBbkUyRmM2eEI0UmNTS0taVXdNZm9FNlFLTXhYZnRselFETmF6a1BEQkVjQ0UtRmN0VXpfZ2hfRm82N242U2Foc3JEbzh6OVFnbnlxNQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K27" s="1" t="n">
+        <v>46088.97275462963</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>8 marzo, desiderio rabbia e conflitto - il manifesto</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>March 8, desire, anger and conflict - the manifesto</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Sat, 07 Mar 2026 23:15:39 GMT</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMia0FVX3lxTE1OLUN1endkdkNhQ3o2ZHJpcEg1eHdvZmJLaXpXQUtiQjBudk43SUZPTjlvaG5GQVRucnFXTkVPbk1QNURWcGVJQkRUcDhlekZGNFZrX1oyeXJZMmJ6RE1yUm9IY2VMRmY4TVBj?oc=5</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K28" s="1" t="n">
+        <v>46088.96920138889</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Pilastro, circa 700 in corteo contro il Museo dei bambini: “Questa è una lotta”. Piantedosi: “Le proteste? La polizia serve altrove” - Il Resto del Carlino</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Pilastro, around 700 in procession against the Children's Museum: "This is a fight". Piantedosi: "The protests? The police are needed elsewhere" - Il Resto del Carlino</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Sat, 07 Mar 2026 20:44:02 GMT</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxQZzhVVElZR3ZkZHpNa3VYV3dhS21tRUQzVkVsU2dkczJKaEROak9qX3c4VHpyRzJYU2VFZHdBM1dXaF9BYlFOWUw1eU9OU3lhdFh3Uk41bEI0aXBHXzhtZVR6UlRuTnNtQTRKNXdPSW5YVVpkdEZCN1hpSDlCSllaT0p0RzlSUzhvT1lBYjZOUTRCaDRQN0R6MXJISUtoY053bkxrZjBvUlkzdw?oc=5</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K29" s="1" t="n">
+        <v>46088.86391203704</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>BOLOGNA: IN CENTINAIA AL CORTEO RIONALE PER DIFENDERE IL PARCO PUBBLICO DEL PILASTRO - Radio Onda d`Urto</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>BOLOGNA: HUNDREDS AT THE LOCAL PROCESSION TO DEFEND THE PILASTRO PUBLIC PARK - Radio Onda d`Urto</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Sat, 07 Mar 2026 17:21:00 GMT</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPWHRNZ0tDekxmcy1rdzd6WHZJVW1DdEluTlN3eEE4X1RITUFJcENFSWhTVWhsNGJZR0VZbGxKTWU2X2dlbm92TmxXVVJFeU9Kdl84MmtZSnRRMkdmblNsRkcxbXMzdThGSVQ5RWhZNjhEc2ZvczY2dzV5bHRrSW04cUtORktSZ1k3TDE3Ri1MOVpMOGZJX3JWeFBMZmNHd2NwWGJNcFQ4M1lxOEc3YThOcUpxRlZURlJqNHUwLWlxUmpTd1U?oc=5</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K30" s="1" t="n">
+        <v>46088.72291666667</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Milano, corteo pro Pal: sventolata bandiera repubblica islamica Iran - Local Team</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Milan, pro Pal procession: Islamic Republic of Iran flag waved - Local Team</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Sat, 07 Mar 2026 20:23:09 GMT</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxOZVNvX0lXNWY3REpHTUIwM2haNTFmRllkU3FCbUFfT01OSDl3RDI3SXh4LS1FWmlVb2I2cHV2UWlvY19kcGk5dkhiQVFZQ1ZsS1lKY1M5NnRzNE43WHNKRGdSeHg4ZzFvbE1qb3lsenlnSEVVcUw5akY2T244SFZNNnMySWtzU0lZaE42azBzZWxBal94eDAtZlFPWW9TYkJEbHRiYmFrdS1FRk5hbTlVbg?oc=5</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K31" s="1" t="n">
+        <v>46088.84940972222</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Milano, corteo 8 marzo ‘Non Una di Meno’ per i diritti delle donne: percorso e strade chiuse - Il Giorno</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Milan, 8 March 'Non Una di Meno' procession for women's rights: route and closed roads - Il Giorno</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Sat, 07 Mar 2026 18:54:56 GMT</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTE9DcGRSQ0FGYWlMT0w0UnI1dGxxbWdXT3pTUE15WFdmdEtjSHI2cFlIVzFDbnJFODJpUVJ6WlJlckpuZUFaanVzZ2pPU2ZBMGxxQXZ6RmRrMEhnUS1VVDRwYU5SZHhtM251eVJUZmhjSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K32" s="1" t="n">
+        <v>46088.78814814815</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Milano. Giù le mani dal Medio Oriente, corteo - Contropiano</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Milan. Hands off the Middle East, march - Counterpiano</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Sat, 07 Mar 2026 19:43:44 GMT</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE9iQWdVLUdzdUtOSi02Vkd1SXRLV1Z6RjYteFROY1NLeHVwcmsyY0ZlaUJrZl9jU2tMakhrMkhyV0dtam1CdmtYdlRMdE9DcDI2VDBrOGg2ejhac1Ywek9SRFhGdTBwN1hFd3BvY1dKTHp2UjZMMHNpMzU4R3ZjdTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K33" s="1" t="n">
+        <v>46088.82203703704</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Milano, corteo pro Palestina giunge al consolato USA - Local Team</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Milan, pro-Palestine march reaches the US consulate - Local Team</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Sat, 07 Mar 2026 17:03:07 GMT</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQMEJkU1BBNFFZb1IwekI5Y3h3bkxaTFdRZmYxSFBPeEEwUW9PTEc5N2FmVmxuc2dLQ1o0TXd0VFA2Z2lhRng5cHFzWTYyN3ZvNWdxSFZFS2Z1MGJCWmc2bFhvQ0RITVozMjkwQjNjSjFodW9jeU9Ya2VZa01mTzVfLUNFcTZOUG56UWdxazItX3VSV0RWSmwxVGpuWTg?oc=5</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K34" s="1" t="n">
+        <v>46088.71049768518</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Prato, estremisti di destra in corteo per la Remigrazione - Local Team</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Prato, right-wing extremists in the procession for Remigration - Local Team</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Sat, 07 Mar 2026 15:18:06 GMT</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxQdEF5aDd5aE1YQ01QREJXTXFja3dNdy1pN3lmd3dURU9IT1BqSVdBVFY4QkNHbGdFbnh0d2hTVXpKdDdEUlBaV0p2cjk2eVJRV3VjNUZENWFBelhidllNUTZhTGdNZDJQVDNYcXFzLUhyV1dXc0tfZUhXWGlOdk5nMlRMRHkzMFZTRUxkdWVvR3lJaUNmaURlWEpmQlR4V3YxeTVZ?oc=5</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K35" s="1" t="n">
+        <v>46088.63756944444</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>La situazione in Medio Oriente e le tre piazze di protesta a Milano - RaiNews</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>The situation in the Middle East and the three protest squares in Milan - RaiNews</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Sat, 07 Mar 2026 17:04:00 GMT</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxQX19CRmlLbTktdTJLdW9QNDdUOUFEbzhhek1BU3V2eHhRbGU4WTg5WW9GR1YzTk96dHpVQmV3cFVpZERRTXJ4ZDBuZUVlc2dpYUFWTmZQd3FiWU8waUNEekVlRFZmcmJFTU13cHBSNFE0RWRxU2VOQWd2VW1rZjhpZVBScl9uUS1haU9NaHl3UUIybkNvUG9wN3JFaWU1TUdhM0ZIbl9heVZ6ZkpOQ2NudWh1Y3U4aFRNOWpaUGtaejZHdEtVazB1TlhCZ3VQZjRnYWE5c1Q2RE9ZNW5Hdk94aEZrMmRXaU5q0gHoAUFVX3lxTFBfX0JGaUttOS11Mkt1b1A0N1Q5QURvOGF6TUFTdXZ4eFFsZThZODlZb0ZHVjNOT3p0elVCZXdwVWlkRFFNcnhkMG5lRWVzZ2lhQVZOZlB3cWJZTzBpQ0R6RWVEVmZyYkVNTXdwcFI0UTRFZHFTZU5BZ3ZVbWtmOGllUFJyX25RLWFpT01oeXdRQjJuQ29Qb3A3ckVpZTVNR2EzRkhuX2F5VnpmSk5DY251aHVjdThoVE05alpQa1p6Nkd0S1VrMHVOWEJndVBmNGdhYTlzVDZET1k1bkd2T3hoRmsyZFdpTmo?oc=5</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K36" s="1" t="n">
+        <v>46088.71111111111</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Pilastro, in marcia il corteo contro il Museo dei bambini nel parco bolognese - RaiNews</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Pilastro, the march against the Children's Museum in the Bolognese park - RaiNews</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Sat, 07 Mar 2026 16:19:00 GMT</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihwJBVV95cUxOVnU1SnhCUXIwenFmQUloRHhxdDFFalpGZ2d0TDV0UWlRTGVBajkxYUxESzdOeEZhUGd2ZW5HT2lEamZUZ2FORWROOU1Kd29JbWpadDhQeVZYSjlmYzFmVXJmdlE0NUV2RWVvcnF0dVI4UGlvSFc5cG55MUJvTndWVU43NXBnV09ERFJMblVacmhQNFRUYVNhdXdLTGNuODFtNVhmLXE0d2JWQmRKSlpHcUtNcm8xY1FiQm5xTE8tYnM4Qk81RDIzaENMSVBIQVlnQm9LYnhoX29sN3RraWtFaDRpd3Rja3FPa3o2Y2E0Z0JYb2lJRkdOUHB0Umh1WHhweTM4dE5ESdIBjAJBVV95cUxONXVGRTZnclZmaUp6alpreTkyaGJOVWJubWNGT0VsRkdwbk1hU0MySzFuZlYtNU96a253ZC1HbDVYLU14MEhfeVNIaXJsZHpscUpFS0ZDM1NRak1XY0FjcEZzSnllNlpLMUpMNEd0eHVZeTRoVUhCRmQ5VkR1MDFIeDd6Wk9DaEZGNWVIWHJHU2tHQ0RHR3FUdUhkeG1IVUMtU195WDV4MklUc3FaSS1kSndFMExMWVVHNS1XTldQU0FtVlF0Vzl0QndZUEd6MEtuWklNMGExem8wbVhtNTd2UWhlcmN2OHdIcmtOekJJOUxuYm9yc0ltbWNCUmtZX0hsb2pBVFBmRnc0S2wt?oc=5</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K37" s="1" t="n">
+        <v>46088.67986111111</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Sciopero generale del 9 marzo, si fermano anche i mezzi pubblici? Chi aderisce e chi no - Moveo by Telepass</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>General strike on March 9th, will public transport also stop? Who joins and who doesn't - Moveo by Telepass</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Sun, 08 Mar 2026 06:05:18 GMT</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTFBOOFg4aFJ1RXNfSmpYTUJoRDBiazE1WXB3alBabWhpQTVFa2MwbG5qUmFSQVJaQzU5RVJyU1FZLUV1Y2h6RmN5RXB2dWNvZ2FrTUoyX1VCSW1xS3lNT0IwS0VVclhLUFZ4Z196dndCYnpadw?oc=5</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K38" s="1" t="n">
+        <v>46089.25368055556</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Il Museo del Patriarcato apre a Milano, una mostra per raccontare le origini e l'attualità della violenza di genere - Il Giorno</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>The Patriarchate Museum opens in Milan, an exhibition to tell the origins and current events of gender violence - Il Giorno</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Sat, 07 Mar 2026 18:48:58 GMT</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE14Z1VZWXJtaUZBQWtHVmIwbFo0aVRvdnVFY2NPQnE0VkRsZ3doWGktR1l5U2twY0V1cXdLaUpnelh0VFZWN19yVnNJTFlNbjlXWW13czlyMDNjMUkwcE1BbU5Od0VSSjBzZlFEM1VqcXRCQXNfWHc?oc=5</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K39" s="1" t="n">
+        <v>46088.78400462963</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Iran, presidio a Milano per commemorare Ali Khamenei: "Fermate la guerra" - Rete Chiara</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Iran, protest in Milan to commemorate Ali Khamenei: "Stop the war" - Rete Chiara</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Sat, 07 Mar 2026 15:08:56 GMT</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxQelFSaS1jaDIwR0pPTkZYSjdvYXQ1SGtVSlVqSGx1NHZJcmNPWnJZel9UUm16aEs3aHBLTU5fZDVrV2NCTXl5X3BiV1l6QmV4N1NTTzZPa0NfSXFlYzBWMDlfT3FHQXhnbGhtaDNzRGVUYW1qTXNiWFlRNloxamZnbHhIRzNoSHczVUxuSktWdktjQlpDemtqT0ptcw?oc=5</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K40" s="1" t="n">
+        <v>46088.63120370371</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-03-08 14:25 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K40"/>
+  <dimension ref="A1:K64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -490,22 +490,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Incredible new £169m ‘shopping village’ opening beside busy UK motorway - Express.co.uk</t>
+          <t>No Trains to London Marylebone During Major Chiltern Line Engineering Works - DPSimulation</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Incredible new £169m ‘shopping village’ opening beside busy UK motorway - Express.co.uk</t>
+          <t>No Trains to London Marylebone During Major Chiltern Line Engineering Works - DPSimulation</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 19:56:00 GMT</t>
+          <t>Sun, 08 Mar 2026 10:38:17 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxPd05JNm1DTmZkYVFPRlNDaEc4Y19ELTlaN3dLRElrMU1KeTJiNHlUQkpiRkR5UXoxRi12Y0ZKcThxcF9xQlNRVThqc2JhbjRKdlBfeXd1RVE1WkNFMEpheWx3V0lHdl95dXRNeUk4T2VlMWlNUVVud3FLRXB3cElESGFOX3fSAYoBQVVfeXFMT3BlY3hHQ01hLUZnZDhZSlJ4dnlhNDJMSV9KeHhfWEJ2eGZScnlGMUNkTU9halBuSUM1WC1KM3lkZjRYZ0pYelpMX3JnbUhab3A3ZXB2TlREVDFKRDJRaW5sWXFOSUlKRDZVWGxiVkU2eVFXZWF3Y1hRYmViXzEtSWM3NUh4MUVTUGZB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxPQjFrMkIwSVljVmZEMWZHWkRVVHJtSUdKbGh1R1k3QWdHTTgtcE5XOHRUU2pEUVNueHBheGtFbk5yRGxnWEZmOE5kU013YlhsMlQ5c1pib0llN0NNTTVpSmhULVVMN2NEUHRYN2NFRUZqVFEyUmQ2ZXdGQlZwaUwyenR3R1EzQ0paVTNNeGpDRDJudnQxYVhXeHg1THZCMlBQbGsxa1Rvdm95WjR5NUdGZUgwS1VxV1RUc1M1dk5WRVo?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -529,38 +529,38 @@
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46088.83055555556</v>
+        <v>46089.44325231481</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>London Marylebone Incident</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("London Marylebone" OR "Marylebone station") AND (incident OR disruption OR closure OR police OR bomb OR explosion OR stabbing OR shooting OR "suspicious package")</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Tieners aangeklaagd voor moord na dodelijke steekpartij bij treinstation in Melbourne - GVA</t>
+          <t>Tunnel Safety Issue Triggers Rail Delays Between Blackburn and Bolton - DPSimulation</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Teenagers charged with murder after fatal stabbing at Melbourne train station - GVA</t>
+          <t>Tunnel Safety Issue Triggers Rail Delays Between Blackburn and Bolton - DPSimulation</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Sun, 08 Mar 2026 05:17:35 GMT</t>
+          <t>Sun, 08 Mar 2026 12:30:57 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxQTmNoa2NsaEswUWJBWDZkeFl0bWMyVHJwYXNobzV0c3Y5MmY4M0I2N1djS3VsWWcwSzJBLUxLVnAxZnNxa3JsMm1CS1hqdWtkQkZLR3ZlaXF2dUl6VVRFNm9zRGp1ZGlTNmFRaFlQMXBSQW9EY2YtU0M0Y0EzLXZVTF9yZklVRTcwTUNwZGJkM0RKdmVSYTlrYW9ZSWkyWkJZS3VUa1dKTjZ5VjEwcTNIWVc4ZHNJNzRaWmdfQmk4TW53N2JEUENicHdB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNcUtVY2hULS1tRTlqemtiOV9ERi1sQkJXNF9Zc2Vmek1TY19WaU1MZ1FXVVhBT2UxYjQwbktleHlaNFRHTW5mSnVTZUxDZWFZb3Z1eFRQekpiMURmQi1PYUd3RlJRZFhpbDJqRWE5TDJpRFprdE9sMkE4eFNpa2lSWWpFY0VuU3p6SFdNeE83Wm50SzB5RHhOY21uUnVuaFJJNWlNNVdVTDVqMUZDNHB1dnIyMkx4ZVAz?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -570,21 +570,21 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46089.22054398148</v>
+        <v>46089.52149305555</v>
       </c>
     </row>
     <row r="4">
@@ -600,22 +600,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Verdachte opgepakt voor steekpartij Terloplein: “Man kwam verhaal halen na verkeersruzie” - HLN</t>
+          <t>Tieners aangeklaagd voor moord na dodelijke steekpartij bij treinstation in Melbourne - GVA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Suspect arrested for stabbing Terloplein: “Man came to seek redress after traffic dispute” - HLN</t>
+          <t>Teenagers charged with murder after fatal stabbing at Melbourne train station - GVA</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 14:13:39 GMT</t>
+          <t>Sun, 08 Mar 2026 09:46:50 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxOT0kwX3FxUTVISFdHSGdsNURaa3VidHdCd1J6Y3pwQzB2cHBORG14NjBNREp4S05abWdBcTRkcWVxazcyQ1dJYVFpdm5qYlpySVNlZHIxb1pmVzF3OURYQjl1LVdyaFh3bE9QTUExSmlFeG9maWlGcGpTWElLRUkyRlhLZmJvSU1HTmRpU0FFMUlNV2I1ZE1RSF9TbGNJbDYzR0V4MlZTNGJhWjBqV0tGa05MT1JYZGlrM29reEVZOEJKd1k?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxQTmNoa2NsaEswUWJBWDZkeFl0bWMyVHJwYXNobzV0c3Y5MmY4M0I2N1djS3VsWWcwSzJBLUxLVnAxZnNxa3JsMm1CS1hqdWtkQkZLR3ZlaXF2dUl6VVRFNm9zRGp1ZGlTNmFRaFlQMXBSQW9EY2YtU0M0Y0EzLXZVTF9yZklVRTcwTUNwZGJkM0RKdmVSYTlrYW9ZSWkyWkJZS3VUa1dKTjZ5VjEwcTNIWVc4ZHNJNzRaWmdfQmk4TW53N2JEUENicHdB?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46088.5928125</v>
+        <v>46089.40752314815</v>
       </c>
     </row>
     <row r="5">
@@ -655,22 +655,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Man (30) neergestoken in Borgerhout na verkeersdispuut, verdachte (29) opgepakt - VRT</t>
+          <t>Vijftig jaar The Kids, Belgian Asociality en Wahwahsda op Left Festival - HLN</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Man (30) stabbed in Borgerhout after traffic dispute, suspect (29) arrested - VRT</t>
+          <t>Vijftig jaar The Kids, Belgian Asociality en Wahwahsda op Left Festival - HLN</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 10:27:22 GMT</t>
+          <t>Sun, 08 Mar 2026 12:47:27 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxOcXhOWUdkdFVzc0ZIbl8wbzdteFAzZF9WcC1vYXZZWVFkaVZhbVdKOUZha2Vodk92MzhvMXE2OGoxd3B2UHBWdlFicVJia0tFUTQ1ZUs2al8wSGdQMWVad1pybm12V01ObUpESHBlcHpzV3VYVnlsZ1JqWGhaUkRWSTFlcTBRVERGTWl4Tw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxQVUpIby0ycXZRN0lpa1JvaXFDMVVkTEUyVVVmU2FxcDQtUW1URTI3eFhaZkQ3Q3ZaYk1MRWFNYnAzbHlGamJOTE80bGJMZUVxU0M0eFZGVUJDTXdlbUhvRDNRY0xmbVptNVVhQ25XemYtRWY3cC1PTWl2Y3Q1ZlJYOVZPMjBUTktYbnVIS1hjOTZMREo2S0s2Vjk5RkhOcThpX2hEenA3dUxyVnBXbHc?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46088.4356712963</v>
+        <v>46089.53295138889</v>
       </c>
     </row>
     <row r="6">
@@ -710,22 +710,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>The Kids vieren vijftigste verjaardag op Left Festival - Nieuwsblad</t>
+          <t>Man opgepakt na knokpartij voor Manneken Pis - HLN</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>The Kids celebrate their fiftieth anniversary at Left Festival - Nieuwsblad</t>
+          <t>Man arrested after brawl in front of Manneken Pis - HLN</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Sun, 08 Mar 2026 02:27:03 GMT</t>
+          <t>Sun, 08 Mar 2026 12:13:05 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxOYVkyNjBBZTZWSFU0ek1pMGN6cWVnZ1ZoRTJPM2QtZFlTa2kzczFiTjV3NWloUUZPTlczX1dzMkFiMVVQenRVVjh2cUFPcmF2MERBZWhMNzZyZGFYano3T2R0OE5Qa2psV0p3Zk1IT2dxZzlFM3hhVmxraVRncmNFWC1lb1VwSTlfWF9nLVljS1pocU9RcEJRajJWUkhfMnE2aWNMcDUwTU13MW5qRWdaaTlyUzBIaXJJYkV0NkZxUUpzc0ZrTnZDb3hEQUhIdlNXeVgw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxQZ0RyODNhTHF1Vy1rSWFqajNhR2ZhSzhQSFhWYjBCZHZEOE5UYUhONkpuQmNOWnFLZC1tYlplM0Y3VFI0WjRxZUEtdkJ0OGppMnotenA3M04tUDdmQ3hDLUZnX2U3LUcxQmhQYjZEdTlObkdvaE9LeWtRU1Z0S3lDOVhITW1CVHE3?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46089.10211805555</v>
+        <v>46089.50908564815</v>
       </c>
     </row>
     <row r="7">
@@ -765,22 +765,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Moeder (44) in shock en dochter (15) lichtgewond na explosie in woning in Zulte: “In overleg met familie en sociale dienst voor opvang komende weken” - HLN</t>
+          <t>Explosie bij Amerikaanse ambassade in Oslo, politie komt massaal ter plaatse - GVA</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Mother (44) in shock and daughter (15) slightly injured after explosion in home in Zulte: “In consultation with family and social services for care in the coming weeks” - HLN</t>
+          <t>Explosion at American embassy in Oslo, police arrive en masse - GVA</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 11:01:40 GMT</t>
+          <t>Sun, 08 Mar 2026 07:41:05 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxPSVplVU5ibFVPNVdRdU9jT2Z5Vm9BZGtkQjZtVFNuQ1Z3Slhhb3V4bUVUUkl5Zzl6c2J6LUN2czhLUTgxM3RuMUlubk1tckdtLU1yU2FOemFsVG0zTHJjcE9OWE0wR2taUk1CRFVQTlZhUGxPczhET1cyV051MFZ5Skp0MVdHb0p5dm1kSko5M3hjLTF5VXVKc0tmQVFYWS1XaTYwRWpyYlNEbW1FODNUbEg2elAxX1NId0FaNGdhZHV1SEVXYnpvTllCMk84dVUzb00xX1ZqVUttNDdjTEFTNGV6c2FqNVJ0ZGc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxQczlaLWRqOWFWdFpJb0huTUp0MkhQSGo2WG1qRWZrN0Y2NDlCSUZ5Y3RCeV9lQU5PV3JsRkVLdnNMX0JWMVM1Y3pVZGFyaTBOaUtHYjZEejV4bWV6cWxXUnBZZDJqV3ZzMHlMOWUySFZ0bGc4UU5keV9wbVBpUi1iTVZUM2hjSDBzT0lGdHVUNHBBamprX2ZHSm84U2lTT2pUV3FJ?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46088.45949074074</v>
+        <v>46089.32019675926</v>
       </c>
     </row>
     <row r="8">
@@ -820,22 +820,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Eerste militaire vlucht met 185 Belgen vliegt vanavond vanuit Oman naar Brussel - Vlaamse Wout (20) boekte zelf ticket en wacht nu op luchthaven Dubai - HLN</t>
+          <t>“Overeenstemming over nieuwe hoogste leider Iran” - Eerste repatriëringsvlucht met Belgen geland in Brussel - HLN</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>First military flight with 185 Belgians flies from Oman to Brussels tonight - Flemish Wout (20) booked his own ticket and is now waiting at Dubai airport - HLN</t>
+          <t>“Agreement on Iran's new supreme leader” - First repatriation flight with Belgians landed in Brussels - HLN</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 10:38:12 GMT</t>
+          <t>Sun, 08 Mar 2026 09:54:18 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilAJBVV95cUxNUHVCejdUOFk3ek4wMk9McVhpRlM3Vmt1ZXVqT2txbkdOQWZieDY5Z2tmREg1a1E4RXd1eWp0VGNxU3VsTkR6Z3gwUVJnOFVqNk12eUQ1Ti12aWV0bTVnMHFPbFpsR21teENsQTVrUDcySjljUTgyUXNZR1RRekE5aUJpbXlVa1hEX0hNelA3Z1JDcHRjdlNkeUdndFFVdkhwUjNvbXhPb1RxekZublg0Rkt6V2FhY3ZrXzNEYWIxQmt3aE9oUWhTaDlwWDZtclN5WVo4N0Z3dDlPVTREUVZhYnV2N1lZZUswZUROaE5uMGNwWFUwMl9SaGZKaExlSlZNR0Utc3pxNWE2SlZqRzVSTkptSXo?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMia0FVX3lxTE0ySkZQOW9rcXdkZUZ6Smt0VE5zLW5NVVQ1b1E0akNSQV84dDVfRi1aMFEzeUQ3dFc3RlJNeXpmS1hmdE5WbWlxUzdXeExvaDNsZ29rMGFPMGl4aHFUc0Rtdi1mWXFSQmxNTEV3?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46088.44319444444</v>
+        <v>46089.41270833334</v>
       </c>
     </row>
     <row r="9">
@@ -875,22 +875,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Voortvluchtige Antwerpenaar opgepakt op luchthaven in Frankrijk - HLN</t>
+          <t>Bomaanslag in Peruviaanse nachtclub maakt 33 gewonden onder wie minstens drie minderjarigen - GVA</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Fugitive Antwerp citizen arrested at airport in France - HLN</t>
+          <t>Bomb attack in Peruvian nightclub leaves 33 injured, including at least three minors - GVA</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 14:11:39 GMT</t>
+          <t>Sun, 08 Mar 2026 10:17:54 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOTW5KMzYxbllHYlVfcjZQaUthZ0tkbV90QUxEOXBTdkZmRzBNZ0N2UWFuZnpUMEs5eWNJXzdMcnJhTmhEX3dzNmVUc2VNLUVPem00UmhydG1ndmlOc0tOVzd4bzFSYUdsUnJ2eHdIXy1qdUVxLXVGdmwySlpINW5jVnJlX0xWbXlLMEpDWkRiVlhTcktfb3dLVlhwUDVjc2s4UVBVWg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxOa1cySW1NT2JMdVhKazRyV29HWk9WTGdUUG9EN1BJa0tGLXVlTUlscm9BRlM2cGhGQzV2Y0h5VktudUxMajhYRENFZWVENE1Xb3hKZjNyLVdZOTdvbjYtSmtocEo1TmFia1FtWVVBaGREVWplVTNzY2c1MklaT2VkLUhDS3AtQjRrZnpXaldHQXU2eHFSTVcxaUtuRnNEaVBXRWo4eW9tRjJHbzZPZ3A2bTlwZDZvZk1waE1lcWRBdTVCTDRGcTMzR3RzdjBPMlMxMnc?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -914,7 +914,7 @@
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46088.59142361111</v>
+        <v>46089.42909722222</v>
       </c>
     </row>
     <row r="10">
@@ -930,22 +930,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Medewerkers van bouwhandel redden zestiger uit kanaal Brussel-Charleroi - HLN</t>
+          <t>Ondanks hoge woningnood zit nieuwbouw op laagste punt: zoveel huizen kwamen erbij in Antwerpen - HLN</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Construction trade employees rescue sixties from Brussels-Charleroi canal - HLN</t>
+          <t>Despite a high housing shortage, new construction is at its lowest point: so many houses were added in Antwerp - HLN</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 12:38:06 GMT</t>
+          <t>Sun, 08 Mar 2026 07:32:54 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxNUTZQTHNldFVteXIyeTFSTnZkMXlKZVBxeFV0UDItTTNLLVR0U1VTWHM0SmI1S1NJajhuQnFDVjFOR0F1akI2SmUwOTg4czRuODY0VS1KUmpYNUVkMWp1WjMwTWFEbGFXV1BvUFJTRlo3STBVYTFvdG10VmNISGVuUUo1ZjJ0a2xWT190X1FlR29IWEF5dnVRMTdYdktpRURIeUhwN083X2RFUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxQdGR6TzBSVG5fb1had2xZMGlUWUUybEZhLVNkX3dpeEZjTGx1ejVxTGRfZDVpNHg4WWx1T1VBb196c3VMRWJZX3RPYWdIRVVIeWJwZTM0TjFDdlRGUS0zU2tVZFJqaEpnb3NZdWdGekpVbDNzRGhaWkNfTTc1T3MyQlVFQmxydkdqVmxjblczb3I1V1RZVjNzdDdtckN2b0VMSjR3T19NbFltQkZBZUZtYzViMzBCODg5S0pweDA4YXFoZlFnZWUxLXdVZGZUQQ?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -969,38 +969,38 @@
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46088.52645833333</v>
+        <v>46089.31451388889</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Foreign Minister Ferit Hoxha: For Albania, all roads lead to Brussels - cna.al</t>
+          <t>Fietser raakt levensgevaarlijk gewond bij botsing - GVA</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Foreign Minister Ferit Hoxha: For Albania, all roads lead to Brussels - cna.al</t>
+          <t>Cyclist suffers life-threatening injuries in collision - GVA</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 12:08:00 GMT</t>
+          <t>Sun, 08 Mar 2026 11:39:17 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPWEZlaTZVelVnQlZ6SWlTS2VvNVNBVVJYMUFMeUJXSm9hcDdOSmFvRzBOOEhyd25kX2UwckFXX1pMVHhfX0xMZ2d2Y3BORzczV3ZyTWJEXzl6cEV0OWVTNkVFeDVYWWZsbDE1Wi16Si1QdFNoOU5VYUlWMTRicTZSQzZTN2tzbXVETDBrNFRLeU80ZkU2LUJZa1M1Q2NDZWNaaWhQR3VDMkVRSnRid0VyQVpYSHRPQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNcnF5Y1hSZWdoWXA0UVcyc2N2UFRDa0ZTSVRUVURJbEtvbG9EMmZFTUV4WnpzMkNNQzAzWVRxb2ppUzR5U2JVLUdQWldRZnJtZFlZQmpwZTNZTl81bm9qQ0RDUFRLVlU0ZDhrNXdEd2dEUVFZQVU1ZUYwT1pLNHI1Wk82NTRtNENtU1lFTWtTRWk3bk0wU0ZYMjI1OWJkSVRNUHRDcmpqRlYyWE12ZURXN2Nn?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1020,42 +1020,42 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46088.50555555556</v>
+        <v>46089.48561342592</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Le mari d'une serveuse licenciée tire à deux reprises sur son patron et son père avant d'être poignardé - BruxellesToday</t>
+          <t>Explosie in klokkentoren tijdens Spaans dorpsfeest: 14 gewonden - HLN</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Husband of fired waitress shoots boss and father twice before being stabbed - BruxellesToday</t>
+          <t>Explosion in bell tower during Spanish village festival: 14 injured - HLN</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 10:41:00 GMT</t>
+          <t>Sun, 08 Mar 2026 10:18:19 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxPaEhQMlJhS2NaV05lbEUySUg3aEo5OW93NFRpeEVRTTdFODVTNXRVRVRWeHFZWnc4ekRyWFFpWEpFdkFuOWZsRHpNdnZmTExoRi1FdmI3RldKcjA2OFBxWnRsZmJFRmxvQTAxamdocC1HZ2ZKcjAtTkFfNzNYOHQ3WnVPX0V3UkQzcUNBUTlsME1KemVDNlV4TQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxQVlo3NGhuYlc1WXJVQ2VONTA1SnhfV2VwR0RQNXltbHg2NWtxajdJQm1GQnlka3lHV0RjLXdILVF5QUg2bkVJRWRVTGNfMkszREJIQWhzdHhVSDZhX25kay1XSGVyNXdBSkMwVFoxaHQzY2IySkRWTmMxaWJIX2k0TFBZWXJYOFp2Qm9MdVN4dXZmcFBqMzZIdjlFSGVBY2Vxd1J0QjI3d3Z1WXQ1NHZaMXJLa1NqWFVINEF4eHI0XzFxS2RZbGFmTlNmWlVsbW1JOHhDRmJpQTZaT1NkZFR2R0FwVVNraVpGWU9hc0NR?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1075,42 +1075,42 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46088.44513888889</v>
+        <v>46089.42938657408</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Agression contre l’Iran : Après l’Espagne la « rébellion » gagne la Belgique - La patrie news</t>
+          <t>Ben Stiller vraagt Witte Huis om fragment van ‘Tropic Thunder’ uit propaganda-filmpje te halen: “Oorlog is geen film” - GVA</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Aggression against Iran: After Spain the “rebellion” reaches Belgium - La Patrie news</t>
+          <t>Ben Stiller asks White House to remove fragment of 'Tropic Thunder' from propaganda video: “War is not a movie” - GVA</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 18:13:18 GMT</t>
+          <t>Sun, 08 Mar 2026 10:00:00 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxPSGtpZjFtVldEdU5ycFNtamRwaWpNVXJXelRubkh0dFAxb1phWUhGODVfU0tUSWRhRDRyb25HZ1ZOTEd3RTFLY0owaXJnU0lNZVpjaTF0bXRUZFJMLTdUY0xHMkZEV1Y5dHRwWHhnZ0tFdU1NaXdETVNnTU9od3FUZ3lyanJXaTlrd1FmcXlDNWhzZUptcUFJbA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxNVm1NQU5NWE8tV2tsZExiNWl0OTU0dldEVzZsa2p2bzcwYmstZnBSeERVUFp5bU1JYkwxZFVIYUd1VWl5V2RjajhHdFlhbWotdmNvVmNvRy0yUHY3MzhVYUp0NGdKbzhuNG00NzN5V1M2dkR4OExoUTBZc0ZwOUp2WGIzVDhuQXgzbk9IUkFBYzl6RGQtRWoxd0RDa2lKTGkwUTV0TXdqbk5VY3IzZlhhT3lUaFJfenc5bm1HaC1uWFdRNm9pVW1ic1pFc1VEX1NKVnVZdDVEYVdzSzFYdUlBSWVBUWtyOWlYa05tNDhR?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1130,42 +1130,42 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46088.75923611111</v>
+        <v>46089.41666666666</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Politie waarschuwt voor valse biljetten van 50 euro: hier duiken ze op - Nieuws365</t>
+          <t>KMI waarschuwt voor dikke mist: “Zichtbaarheid lokaal minder dan 100 meter” - GVA</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Police warn about counterfeit 50 euro notes: this is where they appear - Nieuws365</t>
+          <t>KMI warns of thick fog: “Visibility locally less than 100 meters” - GVA</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 12:00:14 GMT</t>
+          <t>Sun, 08 Mar 2026 08:34:11 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxQZE9YQUpIYWg2NUctMG5oM3VrWHJxcVJ2T0t1clFRVy1TemUwVHpwemZjaGVuZnFkVFZKMnd0a1o2Q0pyMzNZOEFBRnNTVHFjVU1DNUVWLWY3REZMTjhLVFJNRlV5LXZxcFJOOUl1NXlZbVVsWkFQOF9ybEttZ3h2cEJlMnN0SHh0R0MyY291VEdGWTc4aGM5cmVJdks3UkZpYlpFY05kd1A?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNaFZ1Y3FDWVVPWExvQ1RDRm5jZWVSTlhXbDZVOGZsM3VoM0NRX1ZYMFdWS3Rob09fdmI4ek5TR08tTkRnblRvTUlVTUlwS29uRHRmNXBvN2FpYXY5NVJSUDk5STlpYnBaQlpmTFE4dDMwblJ1b1UxdWFpSnZpMDlNSllpZUVYbEV1akpFekJmemE2WTN2TGZVLXlkaG55bW1hTXlUZGVBSlJHRGs3QVAtdVJDX0NEaXNR?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1189,38 +1189,38 @@
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46088.50016203704</v>
+        <v>46089.35707175926</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>France pick uncapped Brau-Boirie in new centre pairing for Wales - MSN</t>
+          <t>Norway US Embassy Explosion 2026 Warning for Europe? - Brussels Morning Newspaper</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>France pick uncapped Brau-Boirie in new centre pairing for Wales - MSN</t>
+          <t>Norway US Embassy Explosion 2026 Warning for Europe? - Brussels Morning Newspaper</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 17:11:30 GMT</t>
+          <t>Sun, 08 Mar 2026 12:50:59 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPb2h2dUtROE9VZnBqUHRjTlJ3SUs4bzVNTkN2ZlNRWmw5NVdhcXlja3UyMXVOY1ZtS3VkcXRoZUszd21LQ3U4WC03TmY2X3VlaDhpaklGc19wUERhUDhEQ0ZxUWNVS1o1N1FzbTUyVVRmaTAtaEJpak5pRkdJQ0dtTDVCNjVOMmdzZHFBLVZ0XzZZR1dlVXRGWE1yUkJNSkdLYjNYdnpfQlU3b2Jp?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTE1aSUlLdmMxc0N4X201UmNnN2VpU3I1aVJ0ODlva2NaSWJFLUpfc3UtNlpVWU41bDhnOEEzYzA5NFBaZTR4anBXNzJsb2VnZ2J1Q1BiU1VyVDhSUDVBNnhKNEhBZkp3VU9EajFXZ1ljVQ?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1235,47 +1235,47 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46088.71631944444</v>
+        <v>46089.5354050926</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Why PSG's victory over Marseille will send shock waves across Europe? - MSN</t>
+          <t>Un jeune homme roué de coups devant la gare de Vilvorde, quatre adolescents interpellés (VIDEO) - BruxellesToday</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Why PSG's victory over Marseille will send shock waves across Europe? - MSN</t>
+          <t>A young man severely beaten in front of Vilvoorde station, four teenagers arrested (VIDEO) - BruxellesToday</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 12:49:43 GMT</t>
+          <t>Sun, 08 Mar 2026 12:15:00 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimANBVV95cUxNcjBtWDRxbnJObHg5UGptOUNOZnRXNHhRVUFKdlhOUWE0Z2FvNjZIWVd4eWhjclJUc182eV9xenpEZUl1cHhsOUoxY055RUlJSjRhNFQyVGxGcDJFd2Y3S2hDYXpXcXc5ODNmMkJfbUl2dnFWRVFUT2pNbTZsY1dsRkNHV3p0VVhOQ0dKSE55SGhBUXpVazRGbGRkWi1XRHc2cEp5dWpiaS1jcWw3TUFCOHZDbVV3TU9kblR2cEFQazNaOGxQTkdLSWY5aWFsa0NoaWJ0RXg2NUhFNGduOHBWVXZoVTF3ODFBdmhrSF9EM1dCbVVhX3RRUkZyQ1p4QURjbG9vMmJvSEJPcWs1b3NJZHRrMFhRUnJMVzJtRHFXaGdBbHNqRGd1WWx2VEVrM3lHb2NPXzRpQTN1WW1nNThRRl81ZkxKZng0SjctakE1LUtULUl0cFJXX1Q5eWZjbWM1b1U1YnFkYk80WkxCZWFDV2d5OXhDbVV3c3h6dTJWNHVGMERtNGduXzBPNzNNM0Q4YUMxRnYydmc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxNMmpYVXlpRnlRRVNSWlNORURIQW5XOVBmc1JpNTNrZmxra0dDTHRhUHhGN2YyOVVFWjJBZVZTejZEZWo5ckxCemp3S0FwQW1qLTVPNVBBc3ZfcnkxN0ZtNG5Ud0NlTjZfc0kzVEpGclpBQ1h1ZWdCczRYNWtZTFhhb05RRlQ0VnlrUk8w?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1285,52 +1285,52 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46088.53452546296</v>
+        <v>46089.51041666666</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+          <t>Un homme arrêté après avoir déclenché une bagarre devant le Manneken Pis - BruxellesToday</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+          <t>Man arrested after starting a fight in front of Manneken Pis - BruxellesToday</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Sun, 08 Mar 2026 02:22:42 GMT</t>
+          <t>Sun, 08 Mar 2026 10:08:48 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE03RUZJdVVWTG5jTlA1R0dmc2YyQ3Z2S1ExYmhkN0FENFJGamUwenJsSFFPWGpKc3B2aFBaeHRYVDR3aWM1SXg0YWZFVDk0N3d4a0Jz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxOQXJiSXdHTTYzSDJaVDE4R2pHVnh2RGRKX19aWVJUXzhJdlBQUzAyRWo0cHltcl9JdWdrSEZzdzJMcy1aVEU5ZFFZZHFsM2YyY1JvWnlXb09mZUZVeHBHcXFnVk5BRW9DZEtKVHZnS08tS3VBRzA5TTdZWldmS1p2OTdleDdtZk44?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1340,52 +1340,52 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46089.09909722222</v>
+        <v>46089.42277777778</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Mehrere Mülleimer in Brand gesteckt – Polizei sucht nach Zeugen - Newsallianz.de</t>
+          <t>Alles wat je moet weten over de jeugdstoet en internationale carnavalstoet in Maasmechelen - HLN</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Several trash cans set on fire – police are looking for witnesses - Newsallianz.de</t>
+          <t>Everything you need to know about the youth parade and international carnival parade in Maasmechelen - HLN</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 08:29:54 GMT</t>
+          <t>Sun, 08 Mar 2026 10:13:03 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxPNWV0SFhZUGRDZWVlUzhBZ2tpQ0VJZkVwQTQ0SG16bFc3ZklkVXR6VnZTbFhaVlVaMG5QQXBGYWhxbXRjOU1JUGxLeVc2LXFzNEpjUUtvYS1XVy1kZVdWZkFJendUak9yTXdjdjV4VWZKWlBSOXYyLTY4aHJGMzYzdkdtUmJZOFp1b2ZBTGFTZGZZMHlFZ0FoRk5zU1Z5dw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxNZG5yNkNZZTUzSWpBeGp0alZoMWVrUzN5QXllVmdBNzFxUFB5RFV5ODRyaDBBYnhXMGV6YTdKRy1hTG9Zb3NlSnN2SlB2U1dlMDd0c2JFZ2w3TU9id0VhYzhtLWZjVHVORnM4NkF3bXEwaEpwYTMtbUFiMkRmNnc3RjcyaWNzSFQtU05TM0FNOUhoaXNGOFhaa09XUl9Sczd4bFJKSkd5aGNTaXVDUUNJbHJ3OUJWcDdyMHd2SjZ0MlZmUXNFN3lIekk0dFM?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1395,52 +1395,52 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46088.35409722223</v>
+        <v>46089.42572916667</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>20-Jährige springt in Würzburg ihrer Tasche hinterher in den Main – dann wird die Strömung zu stark - Main-Post</t>
+          <t>“We blijven in hetzelfde bedje ziek”: Sporting Hasselt morst ook met punten tegen rode lantaarn - HBVL</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>20-year-old jumps into the Main in Würzburg after her bag - then the current becomes too strong - Main-Post</t>
+          <t>“We remain sick in the same bed”: Sporting Hasselt also loses points against the red lantern - HBVL</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Sun, 08 Mar 2026 07:35:20 GMT</t>
+          <t>Sun, 08 Mar 2026 12:32:01 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-gFBVV95cUxOaFEtcS03Qm9lb2ljMW9BdjRHMzYzai0tSkl3X1NSRkNtcGRVUFljakdCakJjcVhIM1dsalRtRXZteWsyallqTkllcHBaV0ZOQU1lbzRKMFU0WGdKcG5XdGoyQTJlQU5IVWRkRHluT08wdkhxLUhkc0R3cC1sTHNuajE2TmtXYWktUFQ5R2VDTXpsZHdDdjA5M1ZnN1JkZ0VnR1Z0UENhcmNFVERCUGlXSl9FbGJmcElFZm5NWFRMQnRXZGpTNVU3eGhNUWN0em5qQ0ZSOFRLYy1yS1NzVUV1dUZ1ZUIxVXBUYWVOc1BSR2psOTZpMWtZQV9n?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOUmpxdVBGOXJpOHZZM0swRGxBRFJrSUFmRzJkZkFTSjVBTXg2cmJVbEw0ODNnbGZ2UGZPaHNkNG9jZjVUUEd3aE1MdWZIUTYzU0RJcDBjUk82MS1WZFN6eV8wWWVYQ0VpR19tUDVzenE2RDNZNlJ4d0VsNDk0eTBiQWNZdUppMW5YOFpHOTJ4LXdvYWFjNEJaUXQ3a29yQkRmei1RYm9VSFBQUzlSYWk0Y09RNVB4NjAxMDktbnBBeWwtTVRMM0tsSW9JU3RmdElXRXdOV0dVeHE?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1450,52 +1450,52 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46089.3162037037</v>
+        <v>46089.5222337963</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Auffahrunfall zwischen zwei Linienbussen – Polizei sucht verletzte Fahrgäste - SW1.News</t>
+          <t>E313 in Olen volledig versperd in de richting van Hasselt na ongeval - rtv.be</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Rear-end collision between two buses – police are looking for injured passengers - SW1.News</t>
+          <t>E313 in Olen completely blocked in the direction of Hasselt after accident - rtv.be</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 10:20:01 GMT</t>
+          <t>Sun, 08 Mar 2026 14:06:56 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNMTZTQ0Q0MDVhUGJOV2hXQ2tGaUZPYTRUUWlGOWxOV0xWa01nQTY3UUFVUlNnNDRhWjh2VTIxdXdFYW11ekVrN2ZjQ0hBMXE4T0pHeFRwNFZ4NUwwVDMzbXZqeWc2b2JsQ3dtNkJNaG8yUi00Z0pwUGpFSzZNVW1JWU1ZTUtzMjJlTVFWdnlIRW9XblczRjNEX0dwUDJrWG1obVlQVzhlRmpBV1d6cFU5X1o0UQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxObHh0WGcxOXRtQVlfWmdCbmdNQUxsR2VxeXFZdWFzcER5WS1QSXFiQ2Raa2xkbktOOUVUSEtaMGNqeG9ZT1BlZGNpb0hKZzU5c0QwTEpfa0YyN2dlNkhSbnlQd0lHQVRVLV9SS25Mc1EwQkFFQzVqdXRyVEVOUmlhaFBKR2JHWjNWWlR1OC1fc1YyRGRCLTlaeDJpeG85TUJ5NC1uZkRn?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1505,52 +1505,52 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46088.43056712963</v>
+        <v>46089.58814814815</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>72 Jahre nach der Hochzeit: Polizei schlichtet Streit bei hochbetagtem Paar - Augsburger Allgemeine</t>
+          <t>Henri Van Marcke nadert met SK Roeselare na spektakelrijke zege tot op drie punten van leider Hasselt: “Dit is mooi maar doet ons nog niet dromen” - Nieuwsblad</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>72 years after the wedding: Police settle dispute between elderly couple - Augsburger Allgemeine</t>
+          <t>Henri Van Marcke comes within three points of leader Hasselt with SK Roeselare after a spectacular victory: “This is nice but does not make us dream yet” - Nieuwsblad</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 10:08:15 GMT</t>
+          <t>Sun, 08 Mar 2026 10:13:47 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxOa25iNHQ2OTFnbGw2QTlJNlB3dTBFZUpZR1VrUnUzSUlPYVRTT0NOVDEtNlRZdzNTUHNCM2NrWkhYRHZRM19sVFppZTR4TVZUQzVIaTEzZGxzMld4cEZoLS1VbDFqN3VnS2M4bXl6eUhqcnM4ZWZWX3B2THB1Wl9oelY3cTlkU3RTMmQ4YlctdW5ZbG5RcEp0dzJQcWpFdmI4clV4QTRMWmZTWFM3TGozTktYaHZqNWVkYXpOdHFDSXplcDUxRGFIS21ia3ZnbVphTkRj?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAJBVV95cUxOT3ZDc3Nkak03bDFmVzl2eEY1OWI3N2t0N0FRamhZVjdoS1B5S1RtUHlwcm1aYmpLcGp0aVFHTHFYSkRlSDg5R25vb2ZJdHlxTk9VN3pMa0xXNFRtaTRJek5sTzZ6N3BLUWpfN1RIeFdoNzhmd3ByeVNiV1U3eERuVktxODZQODNScXN2dzI1NFo3UTFsR1d4RkEyNld5WXA4ZGZVVGJncmhNZkl2SXl1ZHppMjMwX3RkRWlQY1BjdERxb3llbGxQMzFseUdxMnhnVl9wVXVMdkpnc0xvenh1S3VJSTl6ek5CRzZySUdhczlKYVY5NDZUd0hPNUlreW4zUE8wZ1p3bmxtMHBid2hnZmx2TlhXRFhKbEN2bkR0NGN0T1ltcjQxYg?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1560,52 +1560,52 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46088.42239583333</v>
+        <v>46089.42623842593</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Polizeieinsatz bei Ehestreit: Versöhnung nach 72 Jahren Ehe in Ingolstadt - RegionalReporter</t>
+          <t>Zwaar ongeval op E313 bij Herentals-Oost: snelweg naar Hasselt volledig versperd - HLN</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Police intervention in marital dispute: Reconciliation after 72 years of marriage in Ingolstadt - RegionalReporter</t>
+          <t>Serious accident on E313 near Herentals-Oost: highway to Hasselt completely blocked - HLN</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 09:32:41 GMT</t>
+          <t>Sun, 08 Mar 2026 14:03:45 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQZEdfd0otNGJRcjB0OVczeXl3UnF5cDVjUXZMWkgyZkhJeG9xNkt4M243ZzRaS25YeEtqN1hJWlRWbWJxNkpzb3FoTGNDTzlWM19tS1M5QlVOTkpDNlJjNHZOMXhQRnozUTZRM1I2a20yV09wdC1JTHNPWTJBclU0UHZ5MU96alhtcFptNlRYR0hUX1dOWDh6ajRMam0tY1QwY211SW9GcUtkN1ItakRjVkFNSDRicGNycVlhbFl3X1o3RG5GcGRJMGpRdnQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxQT0VGZ1NOZkI2SmlEWHdtRWJheWotVDAtYmRyakVDZmI0YTk0ZVhrR09uR01aQkZnOTR6LXZ6WjB0eUJ2LXRvTEtBTVQzQkJWMml4MjdoNUpnWkR4VkpPWEtLbHJwRmtYa3VvbFlFaXRZNzZGU1R0dnFOczZaVEdYaExWLVk5Nkc4RkxuYXBuREFNTmlvalRKWklzRWJ2REo0NVJHN3R4RHFTNXZTdGw1Ynh1MnRfTUZNLUE?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1615,52 +1615,52 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46088.39769675926</v>
+        <v>46089.5859375</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Einsatz in Bayern wird zur Paarberatung: Hochbetagtes Paar ruft nach Streit im 72. Ehejahr die Polizei - Nordbayern</t>
+          <t>Doelman Roofthoofd bezorgt Hasselt winst in derby die niemand wilde verliezen - HBVL</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Mission in Bavaria turns into couples counseling: Elderly couple calls the police after an argument in their 72nd year of marriage - Northern Bavaria</t>
+          <t>Goalkeeper Roofthoofd gives Hasselt a win in the derby that no one wanted to lose - HBVL</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Sat, 07 Mar 2026 11:00:00 GMT</t>
+          <t>Sun, 08 Mar 2026 14:00:31 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxOaVdMSGFfczY2dVM2T19tQTgxZFhVT3loaXYzVThscHppN3BVYkxRdExCbUlwTEY2Q1lWTV9GUmFTdzRuWGNoVWhmQkFzcnFtcWhZamM1dFc1ZHBUak5JUWR0bVQ3RVd5X0ZrTm5tNVRibUlBRXBvb19SejViNnJSOTE1azUyMXdVcGFRVHdua21qTzZhSlhoT3NBalM1OGRZYkh5T1J2anpmWlhLVVpOMGJ3NllGNmVHWlVHUEd5MWlmdlpyTVJhSGtTNUtDNGZfd3B4Um14UQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxPQl83c3lrWTgteFhQa3J1OFNVbWFvNVQ5QmRXcTI3enBCTzNZWWNVVURCT1hqVjNzWGxfa1NRcnNoYXFpejBFR1hTU2ZEVlZ0eVFTbFk4Rl9wTGdidmJoLTVnY0VKZW5RQl9LLW9yQ0prTUlCb29kRXE4UFVSLWVMV3dkNTBVaDJoc21ZZm1TLUtRY0Z2bkx1RjhrRWJubkhtLUlyQkFHa2xsaDNnODlQRUlicUpoTEVfSjFFUUw4dkNJTWdIVHdwaUd3?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1670,52 +1670,52 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46088.45833333334</v>
+        <v>46089.58369212963</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Streit in Ingolstadt endet mit Polizeieingriff - lomazoma.com</t>
+          <t>FULL Hasselt kroont zich tot grote winnaar van het weekend: “Deze thriller was niet goed voor mijn hart” - H